<commit_message>
Daily portfolio update 2026-09-13
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-12 06:50 IST</t>
+          <t>Generated: 2026-09-13 07:08 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-12</t>
+          <t>Last snapshot: 2026-09-13</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DY19"/>
+  <dimension ref="A1:DZ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -748,6 +748,7 @@
     <col width="21" customWidth="1" min="127" max="127"/>
     <col width="21" customWidth="1" min="128" max="128"/>
     <col width="21" customWidth="1" min="129" max="129"/>
+    <col width="21" customWidth="1" min="130" max="130"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1396,6 +1397,11 @@
           <t>2026-09-12</t>
         </is>
       </c>
+      <c r="DZ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1786,6 +1792,9 @@
       <c r="DY2" s="3" t="n">
         <v>590.5999755859375</v>
       </c>
+      <c r="DZ2" s="3" t="n">
+        <v>590.5999755859375</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2206,6 +2215,9 @@
       <c r="DY4" s="3" t="n">
         <v>1411.400024414062</v>
       </c>
+      <c r="DZ4" s="3" t="n">
+        <v>1411.400024414062</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2599,6 +2611,9 @@
       <c r="DY5" s="3" t="n">
         <v>548.25</v>
       </c>
+      <c r="DZ5" s="3" t="n">
+        <v>548.25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2992,6 +3007,9 @@
       <c r="DY6" s="3" t="n">
         <v>332.7999877929688</v>
       </c>
+      <c r="DZ6" s="3" t="n">
+        <v>332.7999877929688</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3385,6 +3403,9 @@
       <c r="DY7" s="3" t="n">
         <v>268.9500122070312</v>
       </c>
+      <c r="DZ7" s="3" t="n">
+        <v>268.9500122070312</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3805,6 +3826,9 @@
       <c r="DY9" s="3" t="n">
         <v>16.02000045776367</v>
       </c>
+      <c r="DZ9" s="3" t="n">
+        <v>16.02000045776367</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4198,6 +4222,9 @@
       <c r="DY10" s="3" t="n">
         <v>489.7999877929688</v>
       </c>
+      <c r="DZ10" s="3" t="n">
+        <v>489.7999877929688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4591,6 +4618,9 @@
       <c r="DY11" s="3" t="n">
         <v>13.69999980926514</v>
       </c>
+      <c r="DZ11" s="3" t="n">
+        <v>13.69999980926514</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4984,6 +5014,9 @@
       <c r="DY12" s="3" t="n">
         <v>2811.39990234375</v>
       </c>
+      <c r="DZ12" s="3" t="n">
+        <v>2811.39990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5377,6 +5410,9 @@
       <c r="DY13" s="3" t="n">
         <v>44.11999893188477</v>
       </c>
+      <c r="DZ13" s="3" t="n">
+        <v>44.11999893188477</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5770,6 +5806,9 @@
       <c r="DY14" s="3" t="n">
         <v>612.4500122070312</v>
       </c>
+      <c r="DZ14" s="3" t="n">
+        <v>612.4500122070312</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6217,6 +6256,9 @@
       <c r="DY17" s="3" t="n">
         <v>552.6500244140625</v>
       </c>
+      <c r="DZ17" s="3" t="n">
+        <v>552.6500244140625</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6608,6 +6650,9 @@
         <v>364.75</v>
       </c>
       <c r="DY18" s="3" t="n">
+        <v>364.6499938964844</v>
+      </c>
+      <c r="DZ18" s="3" t="n">
         <v>364.6499938964844</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-14
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-13 07:08 IST</t>
+          <t>Generated: 2026-09-14 07:31 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-13</t>
+          <t>Last snapshot: 2026-09-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-15
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-14 07:31 IST</t>
+          <t>Generated: 2026-09-15 07:09 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>544434.4981460571</v>
+        <v>546619.50182724</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-46347.52185394289</v>
+        <v>-44162.51817276003</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07845113812695736</v>
+        <v>-0.07475264425406858</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5699428.822658957</v>
+        <v>5701613.82634014</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>638646.8026589574</v>
+        <v>640831.8063401403</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1261952797285186</v>
+        <v>0.1266270319107995</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-14</t>
+          <t>Last snapshot: 2026-09-15</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DZ19"/>
+  <dimension ref="A1:EA19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -749,6 +749,7 @@
     <col width="21" customWidth="1" min="128" max="128"/>
     <col width="21" customWidth="1" min="129" max="129"/>
     <col width="21" customWidth="1" min="130" max="130"/>
+    <col width="21" customWidth="1" min="131" max="131"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1402,6 +1403,11 @@
           <t>2026-09-13</t>
         </is>
       </c>
+      <c r="EA1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1421,13 +1427,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>590.5999755859375</v>
+        <v>592.5999755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47247.998046875</v>
+        <v>47407.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3430.488046874998</v>
+        <v>3590.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1794,6 +1800,9 @@
       </c>
       <c r="DZ2" s="3" t="n">
         <v>590.5999755859375</v>
+      </c>
+      <c r="EA2" s="3" t="n">
+        <v>592.5999755859375</v>
       </c>
     </row>
     <row r="3">
@@ -1841,13 +1850,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1411.400024414062</v>
+        <v>1384.900024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28228.00048828125</v>
+        <v>27698.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3876.579511718752</v>
+        <v>-4406.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2217,6 +2226,9 @@
       </c>
       <c r="DZ4" s="3" t="n">
         <v>1411.400024414062</v>
+      </c>
+      <c r="EA4" s="3" t="n">
+        <v>1384.900024414062</v>
       </c>
     </row>
     <row r="5">
@@ -2237,13 +2249,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>548.25</v>
+        <v>543.7000122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>10965</v>
+        <v>10874.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-3248.1</v>
+        <v>-3339.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2613,6 +2625,9 @@
       </c>
       <c r="DZ5" s="3" t="n">
         <v>548.25</v>
+      </c>
+      <c r="EA5" s="3" t="n">
+        <v>543.7000122070312</v>
       </c>
     </row>
     <row r="6">
@@ -2633,13 +2648,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>332.7999877929688</v>
+        <v>331.4500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13311.99951171875</v>
+        <v>13258.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4190.240488281252</v>
+        <v>-4244.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3009,6 +3024,9 @@
       </c>
       <c r="DZ6" s="3" t="n">
         <v>332.7999877929688</v>
+      </c>
+      <c r="EA6" s="3" t="n">
+        <v>331.4500122070312</v>
       </c>
     </row>
     <row r="7">
@@ -3029,13 +3047,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>268.9500122070312</v>
+        <v>265.0499877929688</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>26895.00122070312</v>
+        <v>26504.99877929688</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>461.1812207031253</v>
+        <v>71.17877929687529</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3405,6 +3423,9 @@
       </c>
       <c r="DZ7" s="3" t="n">
         <v>268.9500122070312</v>
+      </c>
+      <c r="EA7" s="3" t="n">
+        <v>265.0499877929688</v>
       </c>
     </row>
     <row r="8">
@@ -3452,13 +3473,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>16.02000045776367</v>
+        <v>15.77999973297119</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>24030.00068664551</v>
+        <v>23669.99959945679</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7020.16931335449</v>
+        <v>-7380.170400543211</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -3828,6 +3849,9 @@
       </c>
       <c r="DZ9" s="3" t="n">
         <v>16.02000045776367</v>
+      </c>
+      <c r="EA9" s="3" t="n">
+        <v>15.77999973297119</v>
       </c>
     </row>
     <row r="10">
@@ -3848,13 +3872,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>489.7999877929688</v>
+        <v>488.4500122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48979.99877929688</v>
+        <v>48845.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2518.481220703128</v>
+        <v>-2653.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4224,6 +4248,9 @@
       </c>
       <c r="DZ10" s="3" t="n">
         <v>489.7999877929688</v>
+      </c>
+      <c r="EA10" s="3" t="n">
+        <v>488.4500122070312</v>
       </c>
     </row>
     <row r="11">
@@ -4244,13 +4271,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>13.69999980926514</v>
+        <v>13.25</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>13699.99980926514</v>
+        <v>13250</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3858.789809265138</v>
+        <v>3408.790000000001</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4620,6 +4647,9 @@
       </c>
       <c r="DZ11" s="3" t="n">
         <v>13.69999980926514</v>
+      </c>
+      <c r="EA11" s="3" t="n">
+        <v>13.25</v>
       </c>
     </row>
     <row r="12">
@@ -4640,13 +4670,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2811.39990234375</v>
+        <v>2744.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>28113.9990234375</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>390.7490234375</v>
+        <v>27445</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>-278.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5016,6 +5046,9 @@
       </c>
       <c r="DZ12" s="3" t="n">
         <v>2811.39990234375</v>
+      </c>
+      <c r="EA12" s="3" t="n">
+        <v>2744.5</v>
       </c>
     </row>
     <row r="13">
@@ -5036,13 +5069,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>44.11999893188477</v>
+        <v>43.65999984741211</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>26471.99935913086</v>
+        <v>26195.99990844727</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-8559.760640869143</v>
+        <v>-8835.760091552736</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5412,6 +5445,9 @@
       </c>
       <c r="DZ13" s="3" t="n">
         <v>44.11999893188477</v>
+      </c>
+      <c r="EA13" s="3" t="n">
+        <v>43.65999984741211</v>
       </c>
     </row>
     <row r="14">
@@ -5432,13 +5468,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>612.4500122070312</v>
+        <v>734.9000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>30622.50061035156</v>
+        <v>36745.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11840.00938964844</v>
+        <v>-5717.508779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -5808,6 +5844,9 @@
       </c>
       <c r="DZ14" s="3" t="n">
         <v>612.4500122070312</v>
+      </c>
+      <c r="EA14" s="3" t="n">
+        <v>734.9000244140625</v>
       </c>
     </row>
     <row r="15">
@@ -5882,13 +5921,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>552.6500244140625</v>
+        <v>525.9000244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>27632.50122070312</v>
+        <v>26295.00122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>5877.971220703126</v>
+        <v>4540.471220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6258,6 +6297,9 @@
       </c>
       <c r="DZ17" s="3" t="n">
         <v>552.6500244140625</v>
+      </c>
+      <c r="EA17" s="3" t="n">
+        <v>525.9000244140625</v>
       </c>
     </row>
     <row r="18">
@@ -6278,13 +6320,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>364.6499938964844</v>
+        <v>366.6000061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36464.99938964844</v>
+        <v>36660.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-10175.82061035156</v>
+        <v>-9980.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -6654,6 +6696,9 @@
       </c>
       <c r="DZ18" s="3" t="n">
         <v>364.6499938964844</v>
+      </c>
+      <c r="EA18" s="3" t="n">
+        <v>366.6000061035156</v>
       </c>
     </row>
     <row r="19">
@@ -6666,10 +6711,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>544434.4981460571</v>
+        <v>546619.50182724</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-46347.52185394288</v>
+        <v>-44162.51817276002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-16
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-15 07:09 IST</t>
+          <t>Generated: 2026-09-16 07:10 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>546619.50182724</v>
+        <v>540595.4997138977</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-44162.51817276003</v>
+        <v>-50186.52028610231</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07475264425406858</v>
+        <v>-0.08494930208963081</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5701613.82634014</v>
+        <v>5695589.824226798</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>640831.8063401403</v>
+        <v>634807.804226798</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1266270319107995</v>
+        <v>0.1254367016239909</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-15</t>
+          <t>Last snapshot: 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EA19"/>
+  <dimension ref="A1:EB19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -750,6 +750,7 @@
     <col width="21" customWidth="1" min="129" max="129"/>
     <col width="21" customWidth="1" min="130" max="130"/>
     <col width="21" customWidth="1" min="131" max="131"/>
+    <col width="21" customWidth="1" min="132" max="132"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1408,6 +1409,11 @@
           <t>2026-09-15</t>
         </is>
       </c>
+      <c r="EB1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1427,13 +1433,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>592.5999755859375</v>
+        <v>564.3499755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47407.998046875</v>
+        <v>45147.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3590.488046874998</v>
+        <v>1330.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1803,6 +1809,9 @@
       </c>
       <c r="EA2" s="3" t="n">
         <v>592.5999755859375</v>
+      </c>
+      <c r="EB2" s="3" t="n">
+        <v>564.3499755859375</v>
       </c>
     </row>
     <row r="3">
@@ -1850,13 +1859,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1384.900024414062</v>
+        <v>1379.300048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27698.00048828125</v>
+        <v>27586.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4406.579511718752</v>
+        <v>-4518.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2229,6 +2238,9 @@
       </c>
       <c r="EA4" s="3" t="n">
         <v>1384.900024414062</v>
+      </c>
+      <c r="EB4" s="3" t="n">
+        <v>1379.300048828125</v>
       </c>
     </row>
     <row r="5">
@@ -2249,13 +2261,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>543.7000122070312</v>
+        <v>542.6500244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>10874.00024414062</v>
+        <v>10853.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-3339.099755859375</v>
+        <v>-3360.09951171875</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2628,6 +2640,9 @@
       </c>
       <c r="EA5" s="3" t="n">
         <v>543.7000122070312</v>
+      </c>
+      <c r="EB5" s="3" t="n">
+        <v>542.6500244140625</v>
       </c>
     </row>
     <row r="6">
@@ -2648,13 +2663,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>331.4500122070312</v>
+        <v>325.5499877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13258.00048828125</v>
+        <v>13021.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4244.239511718752</v>
+        <v>-4480.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3027,6 +3042,9 @@
       </c>
       <c r="EA6" s="3" t="n">
         <v>331.4500122070312</v>
+      </c>
+      <c r="EB6" s="3" t="n">
+        <v>325.5499877929688</v>
       </c>
     </row>
     <row r="7">
@@ -3047,13 +3065,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>265.0499877929688</v>
+        <v>258.8999938964844</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>26504.99877929688</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>71.17877929687529</v>
+        <v>25889.99938964844</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>-543.8206103515622</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3426,6 +3444,9 @@
       </c>
       <c r="EA7" s="3" t="n">
         <v>265.0499877929688</v>
+      </c>
+      <c r="EB7" s="3" t="n">
+        <v>258.8999938964844</v>
       </c>
     </row>
     <row r="8">
@@ -3473,13 +3494,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.77999973297119</v>
+        <v>15.4399995803833</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23669.99959945679</v>
+        <v>23159.99937057495</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7380.170400543211</v>
+        <v>-7890.170629425047</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -3852,6 +3873,9 @@
       </c>
       <c r="EA9" s="3" t="n">
         <v>15.77999973297119</v>
+      </c>
+      <c r="EB9" s="3" t="n">
+        <v>15.4399995803833</v>
       </c>
     </row>
     <row r="10">
@@ -3872,13 +3896,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>488.4500122070312</v>
+        <v>485</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48845.00122070312</v>
+        <v>48500</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2653.478779296878</v>
+        <v>-2998.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4251,6 +4275,9 @@
       </c>
       <c r="EA10" s="3" t="n">
         <v>488.4500122070312</v>
+      </c>
+      <c r="EB10" s="3" t="n">
+        <v>485</v>
       </c>
     </row>
     <row r="11">
@@ -4271,13 +4298,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>13.25</v>
+        <v>12.21000003814697</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>13250</v>
+        <v>12210.00003814697</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3408.790000000001</v>
+        <v>2368.790038146974</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4650,6 +4677,9 @@
       </c>
       <c r="EA11" s="3" t="n">
         <v>13.25</v>
+      </c>
+      <c r="EB11" s="3" t="n">
+        <v>12.21000003814697</v>
       </c>
     </row>
     <row r="12">
@@ -4670,13 +4700,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2744.5</v>
+        <v>2686.60009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27445</v>
+        <v>26866.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-278.25</v>
+        <v>-857.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5049,6 +5079,9 @@
       </c>
       <c r="EA12" s="3" t="n">
         <v>2744.5</v>
+      </c>
+      <c r="EB12" s="3" t="n">
+        <v>2686.60009765625</v>
       </c>
     </row>
     <row r="13">
@@ -5069,13 +5102,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>43.65999984741211</v>
+        <v>42.40000152587891</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>26195.99990844727</v>
+        <v>25440.00091552734</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-8835.760091552736</v>
+        <v>-9591.759084472658</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5448,6 +5481,9 @@
       </c>
       <c r="EA13" s="3" t="n">
         <v>43.65999984741211</v>
+      </c>
+      <c r="EB13" s="3" t="n">
+        <v>42.40000152587891</v>
       </c>
     </row>
     <row r="14">
@@ -5468,13 +5504,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>734.9000244140625</v>
+        <v>761</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36745.00122070312</v>
+        <v>38050</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5717.508779296877</v>
+        <v>-4412.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -5847,6 +5883,9 @@
       </c>
       <c r="EA14" s="3" t="n">
         <v>734.9000244140625</v>
+      </c>
+      <c r="EB14" s="3" t="n">
+        <v>761</v>
       </c>
     </row>
     <row r="15">
@@ -5921,13 +5960,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>525.9000244140625</v>
+        <v>516.4000244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>26295.00122070312</v>
+        <v>25820.00122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4540.471220703126</v>
+        <v>4065.471220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6300,6 +6339,9 @@
       </c>
       <c r="EA17" s="3" t="n">
         <v>525.9000244140625</v>
+      </c>
+      <c r="EB17" s="3" t="n">
+        <v>516.4000244140625</v>
       </c>
     </row>
     <row r="18">
@@ -6320,13 +6362,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>366.6000061035156</v>
+        <v>362.7999877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36660.00061035156</v>
+        <v>36279.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9980.819389648437</v>
+        <v>-10360.82122070312</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -6699,6 +6741,9 @@
       </c>
       <c r="EA18" s="3" t="n">
         <v>366.6000061035156</v>
+      </c>
+      <c r="EB18" s="3" t="n">
+        <v>362.7999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -6711,10 +6756,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>546619.50182724</v>
+        <v>540595.4997138977</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-44162.51817276002</v>
+        <v>-50186.52028610231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-17
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-16 07:10 IST</t>
+          <t>Generated: 2026-09-17 07:07 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>540595.4997138977</v>
+        <v>541591.4985733032</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-50186.52028610231</v>
+        <v>-49190.5214266968</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08494930208963081</v>
+        <v>-0.0832634030174053</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5695589.824226798</v>
+        <v>5696585.823086203</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>634807.804226798</v>
+        <v>635803.8030862035</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1254367016239909</v>
+        <v>0.1256335089267891</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-16</t>
+          <t>Last snapshot: 2026-09-17</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EB19"/>
+  <dimension ref="A1:EC19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -751,6 +751,7 @@
     <col width="21" customWidth="1" min="130" max="130"/>
     <col width="21" customWidth="1" min="131" max="131"/>
     <col width="21" customWidth="1" min="132" max="132"/>
+    <col width="21" customWidth="1" min="133" max="133"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1414,6 +1415,11 @@
           <t>2026-09-16</t>
         </is>
       </c>
+      <c r="EC1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1433,13 +1439,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>564.3499755859375</v>
+        <v>570.1500244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45147.998046875</v>
+        <v>45612.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1330.488046874998</v>
+        <v>1794.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1812,6 +1818,9 @@
       </c>
       <c r="EB2" s="3" t="n">
         <v>564.3499755859375</v>
+      </c>
+      <c r="EC2" s="3" t="n">
+        <v>570.1500244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1859,13 +1868,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1379.300048828125</v>
+        <v>1393.699951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27586.0009765625</v>
+        <v>27873.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4518.579023437502</v>
+        <v>-4230.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2241,6 +2250,9 @@
       </c>
       <c r="EB4" s="3" t="n">
         <v>1379.300048828125</v>
+      </c>
+      <c r="EC4" s="3" t="n">
+        <v>1393.699951171875</v>
       </c>
     </row>
     <row r="5">
@@ -2261,13 +2273,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>542.6500244140625</v>
+        <v>552.2999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>10853.00048828125</v>
+        <v>11045.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-3360.09951171875</v>
+        <v>-3167.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2643,6 +2655,9 @@
       </c>
       <c r="EB5" s="3" t="n">
         <v>542.6500244140625</v>
+      </c>
+      <c r="EC5" s="3" t="n">
+        <v>552.2999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -2663,13 +2678,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>325.5499877929688</v>
+        <v>330.1499938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13021.99951171875</v>
+        <v>13205.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4480.240488281252</v>
+        <v>-4296.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3045,6 +3060,9 @@
       </c>
       <c r="EB6" s="3" t="n">
         <v>325.5499877929688</v>
+      </c>
+      <c r="EC6" s="3" t="n">
+        <v>330.1499938964844</v>
       </c>
     </row>
     <row r="7">
@@ -3065,13 +3083,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>258.8999938964844</v>
+        <v>265.4500122070312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25889.99938964844</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>-543.8206103515622</v>
+        <v>26545.00122070312</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>111.1812207031253</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3447,6 +3465,9 @@
       </c>
       <c r="EB7" s="3" t="n">
         <v>258.8999938964844</v>
+      </c>
+      <c r="EC7" s="3" t="n">
+        <v>265.4500122070312</v>
       </c>
     </row>
     <row r="8">
@@ -3494,13 +3515,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.4399995803833</v>
+        <v>15.52000045776367</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23159.99937057495</v>
+        <v>23280.00068664551</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7890.170629425047</v>
+        <v>-7770.16931335449</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -3876,6 +3897,9 @@
       </c>
       <c r="EB9" s="3" t="n">
         <v>15.4399995803833</v>
+      </c>
+      <c r="EC9" s="3" t="n">
+        <v>15.52000045776367</v>
       </c>
     </row>
     <row r="10">
@@ -3896,13 +3920,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>485</v>
+        <v>478.5499877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48500</v>
+        <v>47854.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2998.480000000003</v>
+        <v>-3643.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4278,6 +4302,9 @@
       </c>
       <c r="EB10" s="3" t="n">
         <v>485</v>
+      </c>
+      <c r="EC10" s="3" t="n">
+        <v>478.5499877929688</v>
       </c>
     </row>
     <row r="11">
@@ -4298,13 +4325,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12.21000003814697</v>
+        <v>12.5600004196167</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>12210.00003814697</v>
+        <v>12560.0004196167</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2368.790038146974</v>
+        <v>2718.7904196167</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4680,6 +4707,9 @@
       </c>
       <c r="EB11" s="3" t="n">
         <v>12.21000003814697</v>
+      </c>
+      <c r="EC11" s="3" t="n">
+        <v>12.5600004196167</v>
       </c>
     </row>
     <row r="12">
@@ -4700,13 +4730,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2686.60009765625</v>
+        <v>2692.39990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26866.0009765625</v>
+        <v>26923.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-857.2490234375</v>
+        <v>-799.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5082,6 +5112,9 @@
       </c>
       <c r="EB12" s="3" t="n">
         <v>2686.60009765625</v>
+      </c>
+      <c r="EC12" s="3" t="n">
+        <v>2692.39990234375</v>
       </c>
     </row>
     <row r="13">
@@ -5102,13 +5135,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>42.40000152587891</v>
+        <v>42.68999862670898</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>25440.00091552734</v>
+        <v>25613.99917602539</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-9591.759084472658</v>
+        <v>-9417.760823974611</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5484,6 +5517,9 @@
       </c>
       <c r="EB13" s="3" t="n">
         <v>42.40000152587891</v>
+      </c>
+      <c r="EC13" s="3" t="n">
+        <v>42.68999862670898</v>
       </c>
     </row>
     <row r="14">
@@ -5504,13 +5540,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>761</v>
+        <v>737.5</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38050</v>
+        <v>36875</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-4412.510000000002</v>
+        <v>-5587.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -5886,6 +5922,9 @@
       </c>
       <c r="EB14" s="3" t="n">
         <v>761</v>
+      </c>
+      <c r="EC14" s="3" t="n">
+        <v>737.5</v>
       </c>
     </row>
     <row r="15">
@@ -5960,13 +5999,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>516.4000244140625</v>
+        <v>518.0999755859375</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25820.00122070312</v>
+        <v>25904.99877929688</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4065.471220703126</v>
+        <v>4150.468779296876</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6342,6 +6381,9 @@
       </c>
       <c r="EB17" s="3" t="n">
         <v>516.4000244140625</v>
+      </c>
+      <c r="EC17" s="3" t="n">
+        <v>518.0999755859375</v>
       </c>
     </row>
     <row r="18">
@@ -6362,13 +6404,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>362.7999877929688</v>
+        <v>365.25</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36279.99877929688</v>
+        <v>36525</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-10360.82122070312</v>
+        <v>-10115.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -6744,6 +6786,9 @@
       </c>
       <c r="EB18" s="3" t="n">
         <v>362.7999877929688</v>
+      </c>
+      <c r="EC18" s="3" t="n">
+        <v>365.25</v>
       </c>
     </row>
     <row r="19">
@@ -6756,10 +6801,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>540595.4997138977</v>
+        <v>541591.4985733032</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-50186.52028610231</v>
+        <v>-49190.52142669679</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-18
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-17 07:07 IST</t>
+          <t>Generated: 2026-09-18 07:00 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>541591.4985733032</v>
+        <v>540243.5030822754</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-49190.5214266968</v>
+        <v>-50538.51691772463</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.0832634030174053</v>
+        <v>-0.08554511682282516</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5696585.823086203</v>
+        <v>5695237.827595175</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>635803.8030862035</v>
+        <v>634455.8075951757</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1256335089267891</v>
+        <v>0.1253671478217858</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-17</t>
+          <t>Last snapshot: 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EC19"/>
+  <dimension ref="A1:ED19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -752,6 +752,7 @@
     <col width="21" customWidth="1" min="131" max="131"/>
     <col width="21" customWidth="1" min="132" max="132"/>
     <col width="21" customWidth="1" min="133" max="133"/>
+    <col width="21" customWidth="1" min="134" max="134"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1420,6 +1421,11 @@
           <t>2026-09-17</t>
         </is>
       </c>
+      <c r="ED1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1439,13 +1445,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>570.1500244140625</v>
+        <v>561.9500122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45612.001953125</v>
+        <v>44956.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1794.491953124998</v>
+        <v>1138.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1821,6 +1827,9 @@
       </c>
       <c r="EC2" s="3" t="n">
         <v>570.1500244140625</v>
+      </c>
+      <c r="ED2" s="3" t="n">
+        <v>561.9500122070312</v>
       </c>
     </row>
     <row r="3">
@@ -1868,13 +1877,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1393.699951171875</v>
+        <v>1407.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27873.9990234375</v>
+        <v>28151.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4230.580976562502</v>
+        <v>-3952.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2253,6 +2262,9 @@
       </c>
       <c r="EC4" s="3" t="n">
         <v>1393.699951171875</v>
+      </c>
+      <c r="ED4" s="3" t="n">
+        <v>1407.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -2273,13 +2285,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>552.2999877929688</v>
+        <v>552.7999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11045.99975585938</v>
+        <v>11055.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-3167.100244140625</v>
+        <v>-3157.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2658,6 +2670,9 @@
       </c>
       <c r="EC5" s="3" t="n">
         <v>552.2999877929688</v>
+      </c>
+      <c r="ED5" s="3" t="n">
+        <v>552.7999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -2678,13 +2693,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>330.1499938964844</v>
+        <v>324.3999938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13205.99975585938</v>
+        <v>12975.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4296.240244140627</v>
+        <v>-4526.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3063,6 +3078,9 @@
       </c>
       <c r="EC6" s="3" t="n">
         <v>330.1499938964844</v>
+      </c>
+      <c r="ED6" s="3" t="n">
+        <v>324.3999938964844</v>
       </c>
     </row>
     <row r="7">
@@ -3083,13 +3101,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>265.4500122070312</v>
+        <v>266.3500061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>26545.00122070312</v>
+        <v>26635.00061035156</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>111.1812207031253</v>
+        <v>201.1806103515628</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3468,6 +3486,9 @@
       </c>
       <c r="EC7" s="3" t="n">
         <v>265.4500122070312</v>
+      </c>
+      <c r="ED7" s="3" t="n">
+        <v>266.3500061035156</v>
       </c>
     </row>
     <row r="8">
@@ -3515,13 +3536,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.52000045776367</v>
+        <v>15.31999969482422</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23280.00068664551</v>
+        <v>22979.99954223633</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7770.16931335449</v>
+        <v>-8070.17045776367</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -3900,6 +3921,9 @@
       </c>
       <c r="EC9" s="3" t="n">
         <v>15.52000045776367</v>
+      </c>
+      <c r="ED9" s="3" t="n">
+        <v>15.31999969482422</v>
       </c>
     </row>
     <row r="10">
@@ -3920,13 +3944,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>478.5499877929688</v>
+        <v>475</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47854.99877929688</v>
+        <v>47500</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3643.481220703128</v>
+        <v>-3998.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4305,6 +4329,9 @@
       </c>
       <c r="EC10" s="3" t="n">
         <v>478.5499877929688</v>
+      </c>
+      <c r="ED10" s="3" t="n">
+        <v>475</v>
       </c>
     </row>
     <row r="11">
@@ -4325,13 +4352,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12.5600004196167</v>
+        <v>12.68000030517578</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>12560.0004196167</v>
+        <v>12680.00030517578</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2718.7904196167</v>
+        <v>2838.790305175782</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4710,6 +4737,9 @@
       </c>
       <c r="EC11" s="3" t="n">
         <v>12.5600004196167</v>
+      </c>
+      <c r="ED11" s="3" t="n">
+        <v>12.68000030517578</v>
       </c>
     </row>
     <row r="12">
@@ -4730,13 +4760,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2692.39990234375</v>
+        <v>2757.800048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26923.9990234375</v>
+        <v>27578.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-799.2509765625</v>
+        <v>-145.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5115,6 +5145,9 @@
       </c>
       <c r="EC12" s="3" t="n">
         <v>2692.39990234375</v>
+      </c>
+      <c r="ED12" s="3" t="n">
+        <v>2757.800048828125</v>
       </c>
     </row>
     <row r="13">
@@ -5135,13 +5168,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>42.68999862670898</v>
+        <v>43.40000152587891</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>25613.99917602539</v>
+        <v>26040.00091552734</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-9417.760823974611</v>
+        <v>-8991.759084472658</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5520,6 +5553,9 @@
       </c>
       <c r="EC13" s="3" t="n">
         <v>42.68999862670898</v>
+      </c>
+      <c r="ED13" s="3" t="n">
+        <v>43.40000152587891</v>
       </c>
     </row>
     <row r="14">
@@ -5540,13 +5576,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>737.5</v>
+        <v>705.2000122070312</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36875</v>
+        <v>35260.00061035156</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5587.510000000002</v>
+        <v>-7202.50938964844</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -5925,6 +5961,9 @@
       </c>
       <c r="EC14" s="3" t="n">
         <v>737.5</v>
+      </c>
+      <c r="ED14" s="3" t="n">
+        <v>705.2000122070312</v>
       </c>
     </row>
     <row r="15">
@@ -5999,13 +6038,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>518.0999755859375</v>
+        <v>516.4000244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25904.99877929688</v>
+        <v>25820.00122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4150.468779296876</v>
+        <v>4065.471220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6384,6 +6423,9 @@
       </c>
       <c r="EC17" s="3" t="n">
         <v>518.0999755859375</v>
+      </c>
+      <c r="ED17" s="3" t="n">
+        <v>516.4000244140625</v>
       </c>
     </row>
     <row r="18">
@@ -6404,13 +6446,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>365.25</v>
+        <v>368.3999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36525</v>
+        <v>36839.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-10115.82</v>
+        <v>-9800.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -6789,6 +6831,9 @@
       </c>
       <c r="EC18" s="3" t="n">
         <v>365.25</v>
+      </c>
+      <c r="ED18" s="3" t="n">
+        <v>368.3999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -6801,10 +6846,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>541591.4985733032</v>
+        <v>540243.5030822754</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-49190.52142669679</v>
+        <v>-50538.51691772462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-19
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-18 07:00 IST</t>
+          <t>Generated: 2026-09-19 07:00 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>540243.5030822754</v>
+        <v>542120.0002174377</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-50538.51691772463</v>
+        <v>-48662.01978256227</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08554511682282516</v>
+        <v>-0.08236882324645269</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5695237.827595175</v>
+        <v>5697114.324730338</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>634455.8075951757</v>
+        <v>636332.304730338</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1253671478217858</v>
+        <v>0.1257379397523109</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-18</t>
+          <t>Last snapshot: 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:ED19"/>
+  <dimension ref="A1:EE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -753,6 +753,7 @@
     <col width="21" customWidth="1" min="132" max="132"/>
     <col width="21" customWidth="1" min="133" max="133"/>
     <col width="21" customWidth="1" min="134" max="134"/>
+    <col width="21" customWidth="1" min="135" max="135"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1426,6 +1427,11 @@
           <t>2026-09-18</t>
         </is>
       </c>
+      <c r="EE1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1445,13 +1451,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>561.9500122070312</v>
+        <v>559.75</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44956.0009765625</v>
+        <v>44780</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1138.490976562498</v>
+        <v>962.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1830,6 +1836,9 @@
       </c>
       <c r="ED2" s="3" t="n">
         <v>561.9500122070312</v>
+      </c>
+      <c r="EE2" s="3" t="n">
+        <v>559.75</v>
       </c>
     </row>
     <row r="3">
@@ -1877,13 +1886,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1407.599975585938</v>
+        <v>1427.699951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28151.99951171875</v>
+        <v>28553.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3952.580488281252</v>
+        <v>-3550.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2265,6 +2274,9 @@
       </c>
       <c r="ED4" s="3" t="n">
         <v>1407.599975585938</v>
+      </c>
+      <c r="EE4" s="3" t="n">
+        <v>1427.699951171875</v>
       </c>
     </row>
     <row r="5">
@@ -2285,13 +2297,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>552.7999877929688</v>
+        <v>580.25</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11055.99975585938</v>
+        <v>11605</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-3157.100244140625</v>
+        <v>-2608.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2673,6 +2685,9 @@
       </c>
       <c r="ED5" s="3" t="n">
         <v>552.7999877929688</v>
+      </c>
+      <c r="EE5" s="3" t="n">
+        <v>580.25</v>
       </c>
     </row>
     <row r="6">
@@ -2693,13 +2708,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>324.3999938964844</v>
+        <v>322.4500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12975.99975585938</v>
+        <v>12898.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4526.240244140627</v>
+        <v>-4604.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3081,6 +3096,9 @@
       </c>
       <c r="ED6" s="3" t="n">
         <v>324.3999938964844</v>
+      </c>
+      <c r="EE6" s="3" t="n">
+        <v>322.4500122070312</v>
       </c>
     </row>
     <row r="7">
@@ -3490,6 +3508,9 @@
       <c r="ED7" s="3" t="n">
         <v>266.3500061035156</v>
       </c>
+      <c r="EE7" s="3" t="n">
+        <v>266.3500061035156</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3536,13 +3557,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.31999969482422</v>
+        <v>15.36999988555908</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22979.99954223633</v>
+        <v>23054.99982833862</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8070.17045776367</v>
+        <v>-7995.170171661375</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -3924,6 +3945,9 @@
       </c>
       <c r="ED9" s="3" t="n">
         <v>15.31999969482422</v>
+      </c>
+      <c r="EE9" s="3" t="n">
+        <v>15.36999988555908</v>
       </c>
     </row>
     <row r="10">
@@ -3944,13 +3968,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>475</v>
+        <v>475.7000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47500</v>
+        <v>47570.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3998.480000000003</v>
+        <v>-3928.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4332,6 +4356,9 @@
       </c>
       <c r="ED10" s="3" t="n">
         <v>475</v>
+      </c>
+      <c r="EE10" s="3" t="n">
+        <v>475.7000122070312</v>
       </c>
     </row>
     <row r="11">
@@ -4352,13 +4379,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12.68000030517578</v>
+        <v>12.72000026702881</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>12680.00030517578</v>
+        <v>12720.00026702881</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2838.790305175782</v>
+        <v>2878.790267028809</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4740,6 +4767,9 @@
       </c>
       <c r="ED11" s="3" t="n">
         <v>12.68000030517578</v>
+      </c>
+      <c r="EE11" s="3" t="n">
+        <v>12.72000026702881</v>
       </c>
     </row>
     <row r="12">
@@ -4760,13 +4790,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2757.800048828125</v>
+        <v>2859.10009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27578.00048828125</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>-145.24951171875</v>
+        <v>28591.0009765625</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>867.7509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5148,6 +5178,9 @@
       </c>
       <c r="ED12" s="3" t="n">
         <v>2757.800048828125</v>
+      </c>
+      <c r="EE12" s="3" t="n">
+        <v>2859.10009765625</v>
       </c>
     </row>
     <row r="13">
@@ -5168,13 +5201,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>43.40000152587891</v>
+        <v>43.13999938964844</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>26040.00091552734</v>
+        <v>25883.99963378906</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-8991.759084472658</v>
+        <v>-9147.76036621094</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5556,6 +5589,9 @@
       </c>
       <c r="ED13" s="3" t="n">
         <v>43.40000152587891</v>
+      </c>
+      <c r="EE13" s="3" t="n">
+        <v>43.13999938964844</v>
       </c>
     </row>
     <row r="14">
@@ -5576,13 +5612,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>705.2000122070312</v>
+        <v>693.25</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35260.00061035156</v>
+        <v>34662.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7202.50938964844</v>
+        <v>-7800.010000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -5964,6 +6000,9 @@
       </c>
       <c r="ED14" s="3" t="n">
         <v>705.2000122070312</v>
+      </c>
+      <c r="EE14" s="3" t="n">
+        <v>693.25</v>
       </c>
     </row>
     <row r="15">
@@ -6038,13 +6077,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>516.4000244140625</v>
+        <v>518.2999877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25820.00122070312</v>
+        <v>25914.99938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4065.471220703126</v>
+        <v>4160.469389648439</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6426,6 +6465,9 @@
       </c>
       <c r="ED17" s="3" t="n">
         <v>516.4000244140625</v>
+      </c>
+      <c r="EE17" s="3" t="n">
+        <v>518.2999877929688</v>
       </c>
     </row>
     <row r="18">
@@ -6446,13 +6488,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>368.3999938964844</v>
+        <v>374.7999877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36839.99938964844</v>
+        <v>37479.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9800.820610351562</v>
+        <v>-9160.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -6834,6 +6876,9 @@
       </c>
       <c r="ED18" s="3" t="n">
         <v>368.3999938964844</v>
+      </c>
+      <c r="EE18" s="3" t="n">
+        <v>374.7999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -6846,10 +6891,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>540243.5030822754</v>
+        <v>542120.0002174377</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-50538.51691772462</v>
+        <v>-48662.01978256227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-20
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-19 07:00 IST</t>
+          <t>Generated: 2026-09-20 07:24 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-19</t>
+          <t>Last snapshot: 2026-09-20</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EE19"/>
+  <dimension ref="A1:EF19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -754,6 +754,7 @@
     <col width="21" customWidth="1" min="133" max="133"/>
     <col width="21" customWidth="1" min="134" max="134"/>
     <col width="21" customWidth="1" min="135" max="135"/>
+    <col width="21" customWidth="1" min="136" max="136"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1432,6 +1433,11 @@
           <t>2026-09-19</t>
         </is>
       </c>
+      <c r="EF1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1840,6 +1846,9 @@
       <c r="EE2" s="3" t="n">
         <v>559.75</v>
       </c>
+      <c r="EF2" s="3" t="n">
+        <v>559.75</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2278,6 +2287,9 @@
       <c r="EE4" s="3" t="n">
         <v>1427.699951171875</v>
       </c>
+      <c r="EF4" s="3" t="n">
+        <v>1427.699951171875</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2689,6 +2701,9 @@
       <c r="EE5" s="3" t="n">
         <v>580.25</v>
       </c>
+      <c r="EF5" s="3" t="n">
+        <v>580.25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3100,6 +3115,9 @@
       <c r="EE6" s="3" t="n">
         <v>322.4500122070312</v>
       </c>
+      <c r="EF6" s="3" t="n">
+        <v>322.4500122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3511,6 +3529,9 @@
       <c r="EE7" s="3" t="n">
         <v>266.3500061035156</v>
       </c>
+      <c r="EF7" s="3" t="n">
+        <v>266.3500061035156</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3949,6 +3970,9 @@
       <c r="EE9" s="3" t="n">
         <v>15.36999988555908</v>
       </c>
+      <c r="EF9" s="3" t="n">
+        <v>15.36999988555908</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4360,6 +4384,9 @@
       <c r="EE10" s="3" t="n">
         <v>475.7000122070312</v>
       </c>
+      <c r="EF10" s="3" t="n">
+        <v>475.7000122070312</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4771,6 +4798,9 @@
       <c r="EE11" s="3" t="n">
         <v>12.72000026702881</v>
       </c>
+      <c r="EF11" s="3" t="n">
+        <v>12.72000026702881</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5182,6 +5212,9 @@
       <c r="EE12" s="3" t="n">
         <v>2859.10009765625</v>
       </c>
+      <c r="EF12" s="3" t="n">
+        <v>2859.10009765625</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5593,6 +5626,9 @@
       <c r="EE13" s="3" t="n">
         <v>43.13999938964844</v>
       </c>
+      <c r="EF13" s="3" t="n">
+        <v>43.13999938964844</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6004,6 +6040,9 @@
       <c r="EE14" s="3" t="n">
         <v>693.25</v>
       </c>
+      <c r="EF14" s="3" t="n">
+        <v>693.25</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6469,6 +6508,9 @@
       <c r="EE17" s="3" t="n">
         <v>518.2999877929688</v>
       </c>
+      <c r="EF17" s="3" t="n">
+        <v>518.2999877929688</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6878,6 +6920,9 @@
         <v>368.3999938964844</v>
       </c>
       <c r="EE18" s="3" t="n">
+        <v>374.7999877929688</v>
+      </c>
+      <c r="EF18" s="3" t="n">
         <v>374.7999877929688</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-21
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-20 07:24 IST</t>
+          <t>Generated: 2026-09-21 07:35 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5154994.3245129</v>
+        <v>5116603.6715003</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>684994.3245128999</v>
+        <v>646603.6715003001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1532425781908053</v>
+        <v>0.1446540652125951</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>542120.0002174377</v>
+        <v>545504.5062713623</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-48662.01978256227</v>
+        <v>-45277.51372863771</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08236882324645269</v>
+        <v>-0.07663996566557275</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5697114.324730338</v>
+        <v>5662108.177771662</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>636332.304730338</v>
+        <v>601326.1577716628</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1257379397523109</v>
+        <v>0.11882079793108</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-20</t>
+          <t>Last snapshot: 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EF19"/>
+  <dimension ref="A1:EG19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -755,6 +755,7 @@
     <col width="21" customWidth="1" min="134" max="134"/>
     <col width="21" customWidth="1" min="135" max="135"/>
     <col width="21" customWidth="1" min="136" max="136"/>
+    <col width="21" customWidth="1" min="137" max="137"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1438,6 +1439,11 @@
           <t>2026-09-20</t>
         </is>
       </c>
+      <c r="EG1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1457,13 +1463,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>559.75</v>
+        <v>567.4000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44780</v>
+        <v>45392.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>962.489999999998</v>
+        <v>1574.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1848,6 +1854,9 @@
       </c>
       <c r="EF2" s="3" t="n">
         <v>559.75</v>
+      </c>
+      <c r="EG2" s="3" t="n">
+        <v>567.4000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1895,13 +1904,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1427.699951171875</v>
+        <v>1406.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28553.9990234375</v>
+        <v>28123.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3550.580976562502</v>
+        <v>-3980.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2289,6 +2298,9 @@
       </c>
       <c r="EF4" s="3" t="n">
         <v>1427.699951171875</v>
+      </c>
+      <c r="EG4" s="3" t="n">
+        <v>1406.199951171875</v>
       </c>
     </row>
     <row r="5">
@@ -2309,13 +2321,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>580.25</v>
+        <v>562.1500244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11605</v>
+        <v>11243.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-2608.1</v>
+        <v>-2970.09951171875</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2703,6 +2715,9 @@
       </c>
       <c r="EF5" s="3" t="n">
         <v>580.25</v>
+      </c>
+      <c r="EG5" s="3" t="n">
+        <v>562.1500244140625</v>
       </c>
     </row>
     <row r="6">
@@ -2723,13 +2738,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>322.4500122070312</v>
+        <v>323.25</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12898.00048828125</v>
+        <v>12930</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4604.239511718752</v>
+        <v>-4572.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3117,6 +3132,9 @@
       </c>
       <c r="EF6" s="3" t="n">
         <v>322.4500122070312</v>
+      </c>
+      <c r="EG6" s="3" t="n">
+        <v>323.25</v>
       </c>
     </row>
     <row r="7">
@@ -3137,13 +3155,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>266.3500061035156</v>
+        <v>284.2000122070312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>26635.00061035156</v>
+        <v>28420.00122070312</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>201.1806103515628</v>
+        <v>1986.181220703125</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3531,6 +3549,9 @@
       </c>
       <c r="EF7" s="3" t="n">
         <v>266.3500061035156</v>
+      </c>
+      <c r="EG7" s="3" t="n">
+        <v>284.2000122070312</v>
       </c>
     </row>
     <row r="8">
@@ -3578,13 +3599,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.36999988555908</v>
+        <v>16.90999984741211</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23054.99982833862</v>
+        <v>25364.99977111816</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7995.170171661375</v>
+        <v>-5685.170228881834</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -3972,6 +3993,9 @@
       </c>
       <c r="EF9" s="3" t="n">
         <v>15.36999988555908</v>
+      </c>
+      <c r="EG9" s="3" t="n">
+        <v>16.90999984741211</v>
       </c>
     </row>
     <row r="10">
@@ -3992,13 +4016,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>475.7000122070312</v>
+        <v>481.7000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47570.00122070312</v>
+        <v>48170.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3928.478779296878</v>
+        <v>-3328.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4386,6 +4410,9 @@
       </c>
       <c r="EF10" s="3" t="n">
         <v>475.7000122070312</v>
+      </c>
+      <c r="EG10" s="3" t="n">
+        <v>481.7000122070312</v>
       </c>
     </row>
     <row r="11">
@@ -4406,13 +4433,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12.72000026702881</v>
+        <v>12.81999969482422</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>12720.00026702881</v>
+        <v>12819.99969482422</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2878.790267028809</v>
+        <v>2978.78969482422</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4800,6 +4827,9 @@
       </c>
       <c r="EF11" s="3" t="n">
         <v>12.72000026702881</v>
+      </c>
+      <c r="EG11" s="3" t="n">
+        <v>12.81999969482422</v>
       </c>
     </row>
     <row r="12">
@@ -4820,13 +4850,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2859.10009765625</v>
+        <v>2792.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>28591.0009765625</v>
+        <v>27923.00048828125</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>867.7509765625</v>
+        <v>199.75048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5214,6 +5244,9 @@
       </c>
       <c r="EF12" s="3" t="n">
         <v>2859.10009765625</v>
+      </c>
+      <c r="EG12" s="3" t="n">
+        <v>2792.300048828125</v>
       </c>
     </row>
     <row r="13">
@@ -5234,13 +5267,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>43.13999938964844</v>
+        <v>43.36999893188477</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>25883.99963378906</v>
+        <v>26021.99935913086</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-9147.76036621094</v>
+        <v>-9009.760640869143</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5628,6 +5661,9 @@
       </c>
       <c r="EF13" s="3" t="n">
         <v>43.13999938964844</v>
+      </c>
+      <c r="EG13" s="3" t="n">
+        <v>43.36999893188477</v>
       </c>
     </row>
     <row r="14">
@@ -5648,13 +5684,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>693.25</v>
+        <v>690.9000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34662.5</v>
+        <v>34545.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7800.010000000002</v>
+        <v>-7917.508779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6042,6 +6078,9 @@
       </c>
       <c r="EF14" s="3" t="n">
         <v>693.25</v>
+      </c>
+      <c r="EG14" s="3" t="n">
+        <v>690.9000244140625</v>
       </c>
     </row>
     <row r="15">
@@ -6116,13 +6155,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>518.2999877929688</v>
+        <v>520.4000244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25914.99938964844</v>
+        <v>26020.00122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4160.469389648439</v>
+        <v>4265.471220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6510,6 +6549,9 @@
       </c>
       <c r="EF17" s="3" t="n">
         <v>518.2999877929688</v>
+      </c>
+      <c r="EG17" s="3" t="n">
+        <v>520.4000244140625</v>
       </c>
     </row>
     <row r="18">
@@ -6530,13 +6572,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>374.7999877929688</v>
+        <v>367.6000061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>37479.99877929688</v>
+        <v>36760.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9160.821220703125</v>
+        <v>-9880.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -6924,6 +6966,9 @@
       </c>
       <c r="EF18" s="3" t="n">
         <v>374.7999877929688</v>
+      </c>
+      <c r="EG18" s="3" t="n">
+        <v>367.6000061035156</v>
       </c>
     </row>
     <row r="19">
@@ -6936,10 +6981,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>542120.0002174377</v>
+        <v>545504.5062713623</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-48662.01978256227</v>
+        <v>-45277.51372863771</v>
       </c>
     </row>
   </sheetData>
@@ -6953,7 +6998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DB41"/>
+  <dimension ref="A1:DC41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6963,7 +7008,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
@@ -7062,6 +7107,7 @@
     <col width="13" customWidth="1" min="104" max="104"/>
     <col width="13" customWidth="1" min="105" max="105"/>
     <col width="13" customWidth="1" min="106" max="106"/>
+    <col width="13" customWidth="1" min="107" max="107"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7595,6 +7641,11 @@
           <t>2026-08-19</t>
         </is>
       </c>
+      <c r="DC1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7619,16 +7670,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.8323</v>
+        <v>57.4332</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64915.71576859999</v>
+        <v>64467.7332024</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14915.71576859999</v>
+        <v>14467.7332024</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2983143153719998</v>
+        <v>0.289354664048</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -7920,6 +7971,9 @@
       </c>
       <c r="DB2" s="3" t="n">
         <v>57.8323</v>
+      </c>
+      <c r="DC2" s="3" t="n">
+        <v>57.4332</v>
       </c>
     </row>
     <row r="3">
@@ -7945,16 +7999,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>27.1975</v>
+        <v>26.4646</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>66775.65556750001</v>
+        <v>64976.22995980001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>6775.655567500013</v>
+        <v>4976.22995980001</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.1129275927916669</v>
+        <v>0.08293716599666684</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8240,6 +8294,9 @@
       </c>
       <c r="DB3" s="3" t="n">
         <v>27.1975</v>
+      </c>
+      <c r="DC3" s="3" t="n">
+        <v>26.4646</v>
       </c>
     </row>
     <row r="4">
@@ -8265,16 +8322,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.81</v>
+        <v>12.64</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>246030.05133</v>
+        <v>242765.01552</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>66030.05133000002</v>
+        <v>62765.01552000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3668336185000001</v>
+        <v>0.3486945306666668</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -8560,6 +8617,9 @@
       </c>
       <c r="DB4" s="3" t="n">
         <v>12.81</v>
+      </c>
+      <c r="DC4" s="3" t="n">
+        <v>12.64</v>
       </c>
     </row>
     <row r="5">
@@ -8585,16 +8645,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.774699999999999</v>
+        <v>9.3049</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>179405.7039736</v>
+        <v>170782.9534312</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-30594.29602640003</v>
+        <v>-39217.0465688</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1456871239352382</v>
+        <v>-0.1867478408038095</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -8880,6 +8940,9 @@
       </c>
       <c r="DB5" s="3" t="n">
         <v>9.774699999999999</v>
+      </c>
+      <c r="DC5" s="3" t="n">
+        <v>9.3049</v>
       </c>
     </row>
     <row r="6">
@@ -8905,16 +8968,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.9871</v>
+        <v>11.6863</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>50693.1701967</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>693.1701966999972</v>
-      </c>
-      <c r="I6" s="12" t="n">
-        <v>0.01386340393399994</v>
+        <v>49421.0939151</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>-578.9060849000016</v>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>-0.01157812169800003</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9206,6 +9269,9 @@
       </c>
       <c r="DB6" s="3" t="n">
         <v>11.9871</v>
+      </c>
+      <c r="DC6" s="3" t="n">
+        <v>11.6863</v>
       </c>
     </row>
     <row r="7">
@@ -9231,16 +9297,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>35.7207</v>
+        <v>34.2716</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>78801.293028</v>
+        <v>75604.520464</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>18801.293028</v>
+        <v>15604.520464</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.3133548838</v>
+        <v>0.2600753410666667</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -9526,6 +9592,9 @@
       </c>
       <c r="DB7" s="3" t="n">
         <v>35.7207</v>
+      </c>
+      <c r="DC7" s="3" t="n">
+        <v>34.2716</v>
       </c>
     </row>
     <row r="8">
@@ -9551,16 +9620,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.2472</v>
+        <v>35.9613</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>56557.4103896</v>
+        <v>57703.2502509</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6557.410389600002</v>
+        <v>7703.250250900004</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.131148207792</v>
+        <v>0.1540650050180001</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -9852,6 +9921,9 @@
       </c>
       <c r="DB8" s="3" t="n">
         <v>35.2472</v>
+      </c>
+      <c r="DC8" s="3" t="n">
+        <v>35.9613</v>
       </c>
     </row>
     <row r="9">
@@ -9877,16 +9949,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.4458</v>
+        <v>40.407</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>133430.3183994</v>
+        <v>130086.012951</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>33430.31839939998</v>
+        <v>30086.012951</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3343031839939998</v>
+        <v>0.30086012951</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10172,6 +10244,9 @@
       </c>
       <c r="DB9" s="3" t="n">
         <v>41.4458</v>
+      </c>
+      <c r="DC9" s="3" t="n">
+        <v>40.407</v>
       </c>
     </row>
     <row r="10">
@@ -10197,16 +10272,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>50.0037</v>
+        <v>48.5568</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>142343.4826383</v>
+        <v>138224.6517312</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>42343.48263830002</v>
+        <v>38224.65173120002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.4234348263830002</v>
+        <v>0.3822465173120002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -10492,6 +10567,9 @@
       </c>
       <c r="DB10" s="3" t="n">
         <v>50.0037</v>
+      </c>
+      <c r="DC10" s="3" t="n">
+        <v>48.5568</v>
       </c>
     </row>
     <row r="11">
@@ -10517,16 +10595,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.5377</v>
+        <v>105.1674</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32360.1371463</v>
+        <v>31646.8688406</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2360.1371463</v>
+        <v>1646.8688406</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07867123820999998</v>
+        <v>0.05489562802</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -10812,6 +10890,9 @@
       </c>
       <c r="DB11" s="3" t="n">
         <v>107.5377</v>
+      </c>
+      <c r="DC11" s="3" t="n">
+        <v>105.1674</v>
       </c>
     </row>
     <row r="12">
@@ -10837,16 +10918,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>235.873</v>
+        <v>231.413</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>109804.070706</v>
+        <v>107727.842586</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>9804.070705999999</v>
+        <v>7727.842585999999</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.09804070705999998</v>
+        <v>0.07727842585999999</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -11138,6 +11219,9 @@
       </c>
       <c r="DB12" s="3" t="n">
         <v>235.873</v>
+      </c>
+      <c r="DC12" s="3" t="n">
+        <v>231.413</v>
       </c>
     </row>
     <row r="13">
@@ -11163,16 +11247,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22.3</v>
+        <v>22.803</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>258403.5915</v>
+        <v>264232.156815</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>58403.59150000001</v>
+        <v>64232.15681499999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2920179575</v>
+        <v>0.321160784075</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -11464,6 +11548,9 @@
       </c>
       <c r="DB13" s="3" t="n">
         <v>22.3</v>
+      </c>
+      <c r="DC13" s="3" t="n">
+        <v>22.803</v>
       </c>
     </row>
     <row r="14">
@@ -11489,16 +11576,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.3768</v>
+        <v>38.0967</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>138448.3739408</v>
+        <v>137437.8835002</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>38448.37394080003</v>
+        <v>37437.8835002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3844837394080002</v>
+        <v>0.374378835002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -11784,6 +11871,9 @@
       </c>
       <c r="DB14" s="3" t="n">
         <v>38.3768</v>
+      </c>
+      <c r="DC14" s="3" t="n">
+        <v>38.0967</v>
       </c>
     </row>
     <row r="15">
@@ -11809,16 +11899,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.92</v>
+        <v>11.75</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>116147.84824</v>
+        <v>114491.37725</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>16147.84824000001</v>
+        <v>14491.37725000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1614784824000001</v>
+        <v>0.1449137725</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -12110,6 +12200,9 @@
       </c>
       <c r="DB15" s="3" t="n">
         <v>11.92</v>
+      </c>
+      <c r="DC15" s="3" t="n">
+        <v>11.75</v>
       </c>
     </row>
     <row r="16">
@@ -12135,16 +12228,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.9385</v>
+        <v>24.6909</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>142721.239928</v>
+        <v>141304.2429552</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>42721.239928</v>
+        <v>41304.2429552</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4272123992799999</v>
+        <v>0.4130424295519999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -12430,6 +12523,9 @@
       </c>
       <c r="DB16" s="3" t="n">
         <v>24.9385</v>
+      </c>
+      <c r="DC16" s="3" t="n">
+        <v>24.6909</v>
       </c>
     </row>
     <row r="17">
@@ -12455,16 +12551,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>17.2323</v>
+        <v>16.9784</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>56970.96604109999</v>
+        <v>56131.5581688</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>6970.966041099993</v>
+        <v>6131.558168800002</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1394193208219999</v>
+        <v>0.122631163376</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -12750,6 +12846,9 @@
       </c>
       <c r="DB17" s="3" t="n">
         <v>17.2323</v>
+      </c>
+      <c r="DC17" s="3" t="n">
+        <v>16.9784</v>
       </c>
     </row>
     <row r="18">
@@ -12775,16 +12874,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.2</v>
+        <v>46.86</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>89039.7792</v>
+        <v>88398.39095999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>9039.779200000004</v>
+        <v>8398.39095999999</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1129972400000001</v>
+        <v>0.1049798869999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -13076,6 +13175,9 @@
       </c>
       <c r="DB18" s="3" t="n">
         <v>47.2</v>
+      </c>
+      <c r="DC18" s="3" t="n">
+        <v>46.86</v>
       </c>
     </row>
     <row r="19">
@@ -13101,16 +13203,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.8481</v>
+        <v>12.9538</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>200337.2222446</v>
+        <v>187399.5934108</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>50337.22224460001</v>
+        <v>37399.59341079998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3355814816306667</v>
+        <v>0.2493306227386665</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -13396,6 +13498,9 @@
       </c>
       <c r="DB19" s="3" t="n">
         <v>13.8481</v>
+      </c>
+      <c r="DC19" s="3" t="n">
+        <v>12.9538</v>
       </c>
     </row>
     <row r="20">
@@ -13421,16 +13526,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.14</v>
+        <v>9.99</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>266233.84242</v>
+        <v>262295.47197</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>16233.84242</v>
+        <v>12295.47197000001</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.06493536968000001</v>
+        <v>0.04918188788000005</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -13722,6 +13827,9 @@
       </c>
       <c r="DB20" s="3" t="n">
         <v>10.14</v>
+      </c>
+      <c r="DC20" s="3" t="n">
+        <v>9.99</v>
       </c>
     </row>
     <row r="21">
@@ -13747,16 +13855,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>116.165</v>
+        <v>114.9258</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>176484.721735</v>
+        <v>174602.0559822</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>6484.721734999999</v>
+        <v>4602.055982199992</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.03814542197058823</v>
+        <v>0.0270709175423529</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -14048,6 +14156,9 @@
       </c>
       <c r="DB21" s="3" t="n">
         <v>116.165</v>
+      </c>
+      <c r="DC21" s="3" t="n">
+        <v>114.9258</v>
       </c>
     </row>
     <row r="22">
@@ -14073,16 +14184,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.606</v>
+        <v>43.696</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>66911.66276000001</v>
+        <v>67049.76415999999</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>6911.662760000007</v>
+        <v>7049.764159999992</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1151943793333334</v>
+        <v>0.1174960693333332</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -14368,6 +14479,9 @@
       </c>
       <c r="DB22" s="3" t="n">
         <v>43.606</v>
+      </c>
+      <c r="DC22" s="3" t="n">
+        <v>43.696</v>
       </c>
     </row>
     <row r="23">
@@ -14393,16 +14507,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>64.49890000000001</v>
+        <v>63.1453</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>175209.1333863</v>
+        <v>171532.1236551</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>25209.13338630003</v>
+        <v>21532.1236551</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1680608892420002</v>
+        <v>0.143547491034</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -14694,6 +14808,9 @@
       </c>
       <c r="DB23" s="3" t="n">
         <v>64.49890000000001</v>
+      </c>
+      <c r="DC23" s="3" t="n">
+        <v>63.1453</v>
       </c>
     </row>
     <row r="24">
@@ -14719,16 +14836,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.5495</v>
+        <v>26.8474</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>100097.967607</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>97.96760699999868</v>
-      </c>
-      <c r="I24" s="12" t="n">
-        <v>0.0009796760699999868</v>
+        <v>97546.96729640001</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>-2453.032703599994</v>
+      </c>
+      <c r="I24" s="13" t="n">
+        <v>-0.02453032703599994</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -15014,6 +15131,9 @@
       </c>
       <c r="DB24" s="3" t="n">
         <v>27.5495</v>
+      </c>
+      <c r="DC24" s="3" t="n">
+        <v>26.8474</v>
       </c>
     </row>
     <row r="25">
@@ -15039,16 +15159,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.9123</v>
+        <v>13.2104</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>212041.5811902</v>
+        <v>216936.8822096</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>12041.5811902</v>
+        <v>16936.88220959998</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.06020790595099999</v>
+        <v>0.0846844110479999</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -15337,6 +15457,9 @@
       </c>
       <c r="DB25" s="3" t="n">
         <v>12.9123</v>
+      </c>
+      <c r="DC25" s="3" t="n">
+        <v>13.2104</v>
       </c>
     </row>
     <row r="26">
@@ -15362,16 +15485,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.1408</v>
+        <v>11.4804</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>121098.543472</v>
+        <v>137095.664886</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>11098.543472</v>
+        <v>27095.66488599998</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1008958497454546</v>
+        <v>0.2463242262363635</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -15660,6 +15783,9 @@
       </c>
       <c r="DB26" s="3" t="n">
         <v>10.1408</v>
+      </c>
+      <c r="DC26" s="3" t="n">
+        <v>11.4804</v>
       </c>
     </row>
     <row r="27">
@@ -15685,16 +15811,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>70.88339999999999</v>
+        <v>70.78400000000001</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>114183.233724</v>
+        <v>114023.11424</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>4183.233723999991</v>
+        <v>4023.11424000001</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.03802939749090901</v>
+        <v>0.03657376581818191</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -15986,6 +16112,9 @@
       </c>
       <c r="DB27" s="3" t="n">
         <v>70.88339999999999</v>
+      </c>
+      <c r="DC27" s="3" t="n">
+        <v>70.78400000000001</v>
       </c>
     </row>
     <row r="28">
@@ -16011,16 +16140,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>120.0094</v>
+        <v>120.0335</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>396829.9225758</v>
+        <v>396909.6130095</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>16829.92257580004</v>
+        <v>16909.61300950003</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.04428926993631589</v>
+        <v>0.04449898160394744</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -16312,6 +16441,9 @@
       </c>
       <c r="DB28" s="3" t="n">
         <v>120.0094</v>
+      </c>
+      <c r="DC28" s="3" t="n">
+        <v>120.0335</v>
       </c>
     </row>
     <row r="29">
@@ -16337,16 +16469,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>13.0713</v>
+        <v>12.2624</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>125532.8830239</v>
+        <v>117764.4476672</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>25532.88302389999</v>
+        <v>17764.44766719999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.2553288302389999</v>
+        <v>0.1776444766719999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -16632,6 +16764,9 @@
       </c>
       <c r="DB29" s="3" t="n">
         <v>13.0713</v>
+      </c>
+      <c r="DC29" s="3" t="n">
+        <v>12.2624</v>
       </c>
     </row>
     <row r="30">
@@ -16657,16 +16792,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.6294</v>
+        <v>17.6516</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>130384.5919134</v>
+        <v>130548.7800276</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>30384.5919134</v>
+        <v>30548.78002759999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.303845919134</v>
+        <v>0.3054878002759999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -16952,6 +17087,9 @@
       </c>
       <c r="DB30" s="3" t="n">
         <v>17.6294</v>
+      </c>
+      <c r="DC30" s="3" t="n">
+        <v>17.6516</v>
       </c>
     </row>
     <row r="31">
@@ -16977,16 +17115,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>423.8435</v>
+        <v>411.6581</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>112776.27848</v>
+        <v>109533.987248</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>12776.27847999999</v>
+        <v>9533.98724799999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1277627847999999</v>
+        <v>0.09533987247999991</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -17275,6 +17413,9 @@
       </c>
       <c r="DB31" s="3" t="n">
         <v>423.8435</v>
+      </c>
+      <c r="DC31" s="3" t="n">
+        <v>411.6581</v>
       </c>
     </row>
     <row r="32">
@@ -17300,16 +17441,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>11.14</v>
+        <v>10.98</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>235499.1544</v>
+        <v>232116.7608</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>35499.1544</v>
+        <v>32116.76079999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.177495772</v>
+        <v>0.1605838039999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -17601,6 +17742,9 @@
       </c>
       <c r="DB32" s="3" t="n">
         <v>11.14</v>
+      </c>
+      <c r="DC32" s="3" t="n">
+        <v>10.98</v>
       </c>
     </row>
     <row r="33">
@@ -17626,16 +17770,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>20.24</v>
+        <v>20.33</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>72532.87359999999</v>
+        <v>72855.40119999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>12532.87359999999</v>
+        <v>12855.40119999999</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.2088812266666665</v>
+        <v>0.2142566866666666</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -17921,6 +18065,9 @@
       </c>
       <c r="DB33" s="3" t="n">
         <v>20.24</v>
+      </c>
+      <c r="DC33" s="3" t="n">
+        <v>20.33</v>
       </c>
     </row>
     <row r="34">
@@ -17946,16 +18093,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>232.4809</v>
+        <v>229.8675</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>81724.2432579</v>
+        <v>80805.5521425</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>1724.243257900001</v>
+        <v>805.5521425000043</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.02155304072375002</v>
+        <v>0.01006940178125005</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -18244,6 +18391,9 @@
       </c>
       <c r="DB34" s="3" t="n">
         <v>232.4809</v>
+      </c>
+      <c r="DC34" s="3" t="n">
+        <v>229.8675</v>
       </c>
     </row>
     <row r="35">
@@ -18269,16 +18419,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.71</v>
+        <v>16.29</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>112097.49533</v>
+        <v>116236.04067</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>12097.49533000001</v>
+        <v>16236.04066999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1209749533</v>
+        <v>0.1623604066999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -18567,6 +18717,9 @@
       </c>
       <c r="DB35" s="3" t="n">
         <v>15.71</v>
+      </c>
+      <c r="DC35" s="3" t="n">
+        <v>16.29</v>
       </c>
     </row>
     <row r="36">
@@ -18592,16 +18745,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>388.4546</v>
+        <v>392.0411</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>180905.6379476</v>
+        <v>182575.8925166</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>30905.63794760001</v>
+        <v>32575.8925166</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.2060375863173334</v>
+        <v>0.2171726167773333</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -18890,6 +19043,9 @@
       </c>
       <c r="DB36" s="3" t="n">
         <v>388.4546</v>
+      </c>
+      <c r="DC36" s="3" t="n">
+        <v>392.0411</v>
       </c>
     </row>
     <row r="37">
@@ -18915,16 +19071,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.579</v>
+        <v>17.79</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>66147.825731</v>
+        <v>66941.79531</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>16147.825731</v>
+        <v>16941.79531</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.3229565146200001</v>
+        <v>0.3388359062</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -19213,6 +19369,9 @@
       </c>
       <c r="DB37" s="3" t="n">
         <v>17.579</v>
+      </c>
+      <c r="DC37" s="3" t="n">
+        <v>17.79</v>
       </c>
     </row>
     <row r="38">
@@ -19238,16 +19397,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.5869</v>
+        <v>14.2118</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>87236.6928858</v>
+        <v>84993.4140876</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>7236.692885800003</v>
+        <v>4993.414087600002</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.09045866107250003</v>
+        <v>0.06241767609500003</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -19533,6 +19692,9 @@
       </c>
       <c r="DB38" s="3" t="n">
         <v>14.5869</v>
+      </c>
+      <c r="DC38" s="3" t="n">
+        <v>14.2118</v>
       </c>
     </row>
     <row r="39">
@@ -19558,16 +19720,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1028.0858</v>
+        <v>1028.1888</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51281.9477898</v>
+        <v>51287.0855328</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1281.947789800004</v>
+        <v>1287.085532799996</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02563895579600008</v>
+        <v>0.02574171065599992</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -19853,6 +20015,9 @@
       </c>
       <c r="DB39" s="3" t="n">
         <v>1028.0858</v>
+      </c>
+      <c r="DC39" s="3" t="n">
+        <v>1028.1888</v>
       </c>
     </row>
     <row r="40">
@@ -19878,16 +20043,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.1461</v>
+        <v>21.851</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>106598.0610447</v>
+        <v>110151.480977</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>6598.061044700007</v>
+        <v>10151.480977</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.06598061044700007</v>
+        <v>0.10151480977</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -20176,6 +20341,9 @@
       </c>
       <c r="DB40" s="3" t="n">
         <v>21.1461</v>
+      </c>
+      <c r="DC40" s="3" t="n">
+        <v>21.851</v>
       </c>
     </row>
     <row r="41">
@@ -20188,13 +20356,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5154994.3245129</v>
+        <v>5116603.6715003</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>684994.3245129001</v>
+        <v>646603.6715002999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1532425781908054</v>
+        <v>0.1446540652125951</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-22
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-21 07:35 IST</t>
+          <t>Generated: 2026-09-22 07:15 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5116603.6715003</v>
+        <v>5145636.5629507</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>646603.6715003001</v>
+        <v>675636.5629506996</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1446540652125951</v>
+        <v>0.1511491192283444</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>545504.5062713623</v>
+        <v>543316.4980773926</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-45277.51372863771</v>
+        <v>-47465.52192260744</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07663996566557275</v>
+        <v>-0.08034354519219701</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5662108.177771662</v>
+        <v>5688953.061028092</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>601326.1577716628</v>
+        <v>628171.0410280926</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.11882079793108</v>
+        <v>0.1241252910213455</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-21</t>
+          <t>Last snapshot: 2026-09-22</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EG19"/>
+  <dimension ref="A1:EH19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -756,6 +756,7 @@
     <col width="21" customWidth="1" min="135" max="135"/>
     <col width="21" customWidth="1" min="136" max="136"/>
     <col width="21" customWidth="1" min="137" max="137"/>
+    <col width="21" customWidth="1" min="138" max="138"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1444,6 +1445,11 @@
           <t>2026-09-21</t>
         </is>
       </c>
+      <c r="EH1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1463,13 +1469,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>567.4000244140625</v>
+        <v>567.5</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45392.001953125</v>
+        <v>45400</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1574.491953124998</v>
+        <v>1582.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1857,6 +1863,9 @@
       </c>
       <c r="EG2" s="3" t="n">
         <v>567.4000244140625</v>
+      </c>
+      <c r="EH2" s="3" t="n">
+        <v>567.5</v>
       </c>
     </row>
     <row r="3">
@@ -1904,13 +1913,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1406.199951171875</v>
+        <v>1396.400024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28123.9990234375</v>
+        <v>27928.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3980.580976562502</v>
+        <v>-4176.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2301,6 +2310,9 @@
       </c>
       <c r="EG4" s="3" t="n">
         <v>1406.199951171875</v>
+      </c>
+      <c r="EH4" s="3" t="n">
+        <v>1396.400024414062</v>
       </c>
     </row>
     <row r="5">
@@ -2321,13 +2333,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>562.1500244140625</v>
+        <v>555.5</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11243.00048828125</v>
+        <v>11110</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-2970.09951171875</v>
+        <v>-3103.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2718,6 +2730,9 @@
       </c>
       <c r="EG5" s="3" t="n">
         <v>562.1500244140625</v>
+      </c>
+      <c r="EH5" s="3" t="n">
+        <v>555.5</v>
       </c>
     </row>
     <row r="6">
@@ -2738,13 +2753,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>323.25</v>
+        <v>322.25</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12930</v>
+        <v>12890</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4572.240000000002</v>
+        <v>-4612.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3135,6 +3150,9 @@
       </c>
       <c r="EG6" s="3" t="n">
         <v>323.25</v>
+      </c>
+      <c r="EH6" s="3" t="n">
+        <v>322.25</v>
       </c>
     </row>
     <row r="7">
@@ -3155,13 +3173,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>284.2000122070312</v>
+        <v>291.2000122070312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>28420.00122070312</v>
+        <v>29120.00122070312</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1986.181220703125</v>
+        <v>2686.181220703125</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3552,6 +3570,9 @@
       </c>
       <c r="EG7" s="3" t="n">
         <v>284.2000122070312</v>
+      </c>
+      <c r="EH7" s="3" t="n">
+        <v>291.2000122070312</v>
       </c>
     </row>
     <row r="8">
@@ -3599,13 +3620,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>16.90999984741211</v>
+        <v>16.17000007629395</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>25364.99977111816</v>
+        <v>24255.00011444092</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-5685.170228881834</v>
+        <v>-6795.16988555908</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -3996,6 +4017,9 @@
       </c>
       <c r="EG9" s="3" t="n">
         <v>16.90999984741211</v>
+      </c>
+      <c r="EH9" s="3" t="n">
+        <v>16.17000007629395</v>
       </c>
     </row>
     <row r="10">
@@ -4016,13 +4040,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>481.7000122070312</v>
+        <v>471.5</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48170.00122070312</v>
+        <v>47150</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3328.478779296878</v>
+        <v>-4348.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4413,6 +4437,9 @@
       </c>
       <c r="EG10" s="3" t="n">
         <v>481.7000122070312</v>
+      </c>
+      <c r="EH10" s="3" t="n">
+        <v>471.5</v>
       </c>
     </row>
     <row r="11">
@@ -4433,13 +4460,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12.81999969482422</v>
+        <v>13.21000003814697</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>12819.99969482422</v>
+        <v>13210.00003814697</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2978.78969482422</v>
+        <v>3368.790038146974</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4830,6 +4857,9 @@
       </c>
       <c r="EG11" s="3" t="n">
         <v>12.81999969482422</v>
+      </c>
+      <c r="EH11" s="3" t="n">
+        <v>13.21000003814697</v>
       </c>
     </row>
     <row r="12">
@@ -4850,13 +4880,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2792.300048828125</v>
+        <v>2793.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27923.00048828125</v>
+        <v>27938.9990234375</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>199.75048828125</v>
+        <v>215.7490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5247,6 +5277,9 @@
       </c>
       <c r="EG12" s="3" t="n">
         <v>2792.300048828125</v>
+      </c>
+      <c r="EH12" s="3" t="n">
+        <v>2793.89990234375</v>
       </c>
     </row>
     <row r="13">
@@ -5267,13 +5300,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>43.36999893188477</v>
+        <v>43.13999938964844</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>26021.99935913086</v>
+        <v>25883.99963378906</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-9009.760640869143</v>
+        <v>-9147.76036621094</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5664,6 +5697,9 @@
       </c>
       <c r="EG13" s="3" t="n">
         <v>43.36999893188477</v>
+      </c>
+      <c r="EH13" s="3" t="n">
+        <v>43.13999938964844</v>
       </c>
     </row>
     <row r="14">
@@ -5684,13 +5720,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>690.9000244140625</v>
+        <v>678.8499755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34545.00122070312</v>
+        <v>33942.49877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7917.508779296877</v>
+        <v>-8520.011220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6081,6 +6117,9 @@
       </c>
       <c r="EG14" s="3" t="n">
         <v>690.9000244140625</v>
+      </c>
+      <c r="EH14" s="3" t="n">
+        <v>678.8499755859375</v>
       </c>
     </row>
     <row r="15">
@@ -6155,13 +6194,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>520.4000244140625</v>
+        <v>518.75</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>26020.00122070312</v>
+        <v>25937.5</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4265.471220703126</v>
+        <v>4182.970000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6552,6 +6591,9 @@
       </c>
       <c r="EG17" s="3" t="n">
         <v>520.4000244140625</v>
+      </c>
+      <c r="EH17" s="3" t="n">
+        <v>518.75</v>
       </c>
     </row>
     <row r="18">
@@ -6572,13 +6614,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>367.6000061035156</v>
+        <v>367.7999877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36760.00061035156</v>
+        <v>36779.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9880.819389648437</v>
+        <v>-9860.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -6969,6 +7011,9 @@
       </c>
       <c r="EG18" s="3" t="n">
         <v>367.6000061035156</v>
+      </c>
+      <c r="EH18" s="3" t="n">
+        <v>367.7999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -6981,10 +7026,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>545504.5062713623</v>
+        <v>543316.4980773926</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-45277.51372863771</v>
+        <v>-47465.52192260743</v>
       </c>
     </row>
   </sheetData>
@@ -6998,7 +7043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DC41"/>
+  <dimension ref="A1:DD41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7008,8 +7053,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -7108,6 +7153,7 @@
     <col width="13" customWidth="1" min="105" max="105"/>
     <col width="13" customWidth="1" min="106" max="106"/>
     <col width="13" customWidth="1" min="107" max="107"/>
+    <col width="13" customWidth="1" min="108" max="108"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7646,6 +7692,11 @@
           <t>2026-09-21</t>
         </is>
       </c>
+      <c r="DD1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7670,16 +7721,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.4332</v>
+        <v>58.1047</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64467.7332024</v>
+        <v>65221.4798654</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14467.7332024</v>
+        <v>15221.4798654</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.289354664048</v>
+        <v>0.304429597308</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -7974,6 +8025,9 @@
       </c>
       <c r="DC2" s="3" t="n">
         <v>57.4332</v>
+      </c>
+      <c r="DD2" s="3" t="n">
+        <v>58.1047</v>
       </c>
     </row>
     <row r="3">
@@ -7999,16 +8053,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.4646</v>
+        <v>26.6665</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>64976.22995980001</v>
+        <v>65471.93746450001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4976.22995980001</v>
+        <v>5471.937464500006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.08293716599666684</v>
+        <v>0.09119895774166677</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8297,6 +8351,9 @@
       </c>
       <c r="DC3" s="3" t="n">
         <v>26.4646</v>
+      </c>
+      <c r="DD3" s="3" t="n">
+        <v>26.6665</v>
       </c>
     </row>
     <row r="4">
@@ -8322,16 +8379,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.64</v>
+        <v>12.98</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>242765.01552</v>
+        <v>249295.08714</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>62765.01552000002</v>
+        <v>69295.08714000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3486945306666668</v>
+        <v>0.3849727063333334</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -8620,6 +8677,9 @@
       </c>
       <c r="DC4" s="3" t="n">
         <v>12.64</v>
+      </c>
+      <c r="DD4" s="3" t="n">
+        <v>12.98</v>
       </c>
     </row>
     <row r="5">
@@ -8645,16 +8705,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.3049</v>
+        <v>9.3466</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>170782.9534312</v>
+        <v>171548.3189008</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-39217.0465688</v>
+        <v>-38451.68109919998</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1867478408038095</v>
+        <v>-0.1831032433295237</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -8943,6 +9003,9 @@
       </c>
       <c r="DC5" s="3" t="n">
         <v>9.3049</v>
+      </c>
+      <c r="DD5" s="3" t="n">
+        <v>9.3466</v>
       </c>
     </row>
     <row r="6">
@@ -8968,16 +9031,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.6863</v>
+        <v>11.6666</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>49421.0939151</v>
+        <v>49337.7830682</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-578.9060849000016</v>
+        <v>-662.2169318000015</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.01157812169800003</v>
+        <v>-0.01324433863600003</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9272,6 +9335,9 @@
       </c>
       <c r="DC6" s="3" t="n">
         <v>11.6863</v>
+      </c>
+      <c r="DD6" s="3" t="n">
+        <v>11.6666</v>
       </c>
     </row>
     <row r="7">
@@ -9297,16 +9363,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.2716</v>
+        <v>34.6408</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75604.520464</v>
+        <v>76418.99043199999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15604.520464</v>
+        <v>16418.99043199999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2600753410666667</v>
+        <v>0.2736498405333332</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -9595,6 +9661,9 @@
       </c>
       <c r="DC7" s="3" t="n">
         <v>34.2716</v>
+      </c>
+      <c r="DD7" s="3" t="n">
+        <v>34.6408</v>
       </c>
     </row>
     <row r="8">
@@ -9620,16 +9689,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.9613</v>
+        <v>36.0099</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57703.2502509</v>
+        <v>57781.2334707</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7703.250250900004</v>
+        <v>7781.233470700005</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1540650050180001</v>
+        <v>0.1556246694140001</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -9924,6 +9993,9 @@
       </c>
       <c r="DC8" s="3" t="n">
         <v>35.9613</v>
+      </c>
+      <c r="DD8" s="3" t="n">
+        <v>36.0099</v>
       </c>
     </row>
     <row r="9">
@@ -9949,16 +10021,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.407</v>
+        <v>41.4204</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>130086.012951</v>
+        <v>133348.5458172</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>30086.012951</v>
+        <v>33348.54581720001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.30086012951</v>
+        <v>0.3334854581720001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10247,6 +10319,9 @@
       </c>
       <c r="DC9" s="3" t="n">
         <v>40.407</v>
+      </c>
+      <c r="DD9" s="3" t="n">
+        <v>41.4204</v>
       </c>
     </row>
     <row r="10">
@@ -10272,16 +10347,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.5568</v>
+        <v>48.7334</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138224.6517312</v>
+        <v>138727.3717106</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38224.65173120002</v>
+        <v>38727.37171060001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3822465173120002</v>
+        <v>0.3872737171060001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -10570,6 +10645,9 @@
       </c>
       <c r="DC10" s="3" t="n">
         <v>48.5568</v>
+      </c>
+      <c r="DD10" s="3" t="n">
+        <v>48.7334</v>
       </c>
     </row>
     <row r="11">
@@ -10595,16 +10673,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>105.1674</v>
+        <v>107.3221</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31646.8688406</v>
+        <v>32295.2590099</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1646.8688406</v>
+        <v>2295.259009900001</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.05489562802</v>
+        <v>0.07650863366333337</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -10893,6 +10971,9 @@
       </c>
       <c r="DC11" s="3" t="n">
         <v>105.1674</v>
+      </c>
+      <c r="DD11" s="3" t="n">
+        <v>107.3221</v>
       </c>
     </row>
     <row r="12">
@@ -10918,16 +10999,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>231.413</v>
+        <v>230.669</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>107727.842586</v>
+        <v>107381.494218</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>7727.842585999999</v>
+        <v>7381.494218000007</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.07727842585999999</v>
+        <v>0.07381494218000006</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -11222,6 +11303,9 @@
       </c>
       <c r="DC12" s="3" t="n">
         <v>231.413</v>
+      </c>
+      <c r="DD12" s="3" t="n">
+        <v>230.669</v>
       </c>
     </row>
     <row r="13">
@@ -11247,16 +11331,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22.803</v>
+        <v>22.892</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>264232.156815</v>
+        <v>265263.45366</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>64232.15681499999</v>
+        <v>65263.45366</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.321160784075</v>
+        <v>0.3263172683</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -11551,6 +11635,9 @@
       </c>
       <c r="DC13" s="3" t="n">
         <v>22.803</v>
+      </c>
+      <c r="DD13" s="3" t="n">
+        <v>22.892</v>
       </c>
     </row>
     <row r="14">
@@ -11576,16 +11663,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.0967</v>
+        <v>38.6079</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>137437.8835002</v>
+        <v>139282.0916874</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>37437.8835002</v>
+        <v>39282.09168740001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.374378835002</v>
+        <v>0.3928209168740001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -11874,6 +11961,9 @@
       </c>
       <c r="DC14" s="3" t="n">
         <v>38.0967</v>
+      </c>
+      <c r="DD14" s="3" t="n">
+        <v>38.6079</v>
       </c>
     </row>
     <row r="15">
@@ -11899,16 +11989,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.75</v>
+        <v>11.78</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114491.37725</v>
+        <v>114783.69566</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14491.37725000001</v>
+        <v>14783.69566</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1449137725</v>
+        <v>0.1478369566</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -12203,6 +12293,9 @@
       </c>
       <c r="DC15" s="3" t="n">
         <v>11.75</v>
+      </c>
+      <c r="DD15" s="3" t="n">
+        <v>11.78</v>
       </c>
     </row>
     <row r="16">
@@ -12228,16 +12321,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.6909</v>
+        <v>25.3905</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>141304.2429552</v>
+        <v>145308.003384</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>41304.2429552</v>
+        <v>45308.00338399998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4130424295519999</v>
+        <v>0.4530800338399998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -12526,6 +12619,9 @@
       </c>
       <c r="DC16" s="3" t="n">
         <v>24.6909</v>
+      </c>
+      <c r="DD16" s="3" t="n">
+        <v>25.3905</v>
       </c>
     </row>
     <row r="17">
@@ -12551,16 +12647,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.9784</v>
+        <v>17.0253</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>56131.5581688</v>
+        <v>56286.6122421</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>6131.558168800002</v>
+        <v>6286.612242100004</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.122631163376</v>
+        <v>0.1257322448420001</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -12849,6 +12945,9 @@
       </c>
       <c r="DC17" s="3" t="n">
         <v>16.9784</v>
+      </c>
+      <c r="DD17" s="3" t="n">
+        <v>17.0253</v>
       </c>
     </row>
     <row r="18">
@@ -12874,16 +12973,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.86</v>
+        <v>47.41</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>88398.39095999999</v>
+        <v>89435.93075999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8398.39095999999</v>
+        <v>9435.930759999988</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1049798869999999</v>
+        <v>0.1179491344999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -13178,6 +13277,9 @@
       </c>
       <c r="DC18" s="3" t="n">
         <v>46.86</v>
+      </c>
+      <c r="DD18" s="3" t="n">
+        <v>47.41</v>
       </c>
     </row>
     <row r="19">
@@ -13203,16 +13305,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>12.9538</v>
+        <v>13.2202</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>187399.5934108</v>
+        <v>191253.5398732</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>37399.59341079998</v>
+        <v>41253.5398732</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2493306227386665</v>
+        <v>0.2750235991546667</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -13501,6 +13603,9 @@
       </c>
       <c r="DC19" s="3" t="n">
         <v>12.9538</v>
+      </c>
+      <c r="DD19" s="3" t="n">
+        <v>13.2202</v>
       </c>
     </row>
     <row r="20">
@@ -13526,16 +13631,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.99</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>262295.47197</v>
+        <v>261770.35591</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>12295.47197000001</v>
+        <v>11770.35591000001</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.04918188788000005</v>
+        <v>0.04708142364000005</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -13830,6 +13935,9 @@
       </c>
       <c r="DC20" s="3" t="n">
         <v>9.99</v>
+      </c>
+      <c r="DD20" s="3" t="n">
+        <v>9.970000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -13855,16 +13963,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>114.9258</v>
+        <v>114.6398</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>174602.0559822</v>
+        <v>174167.5479082</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>4602.055982199992</v>
+        <v>4167.54790819998</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.0270709175423529</v>
+        <v>0.024514987695294</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -14159,6 +14267,9 @@
       </c>
       <c r="DC21" s="3" t="n">
         <v>114.9258</v>
+      </c>
+      <c r="DD21" s="3" t="n">
+        <v>114.6398</v>
       </c>
     </row>
     <row r="22">
@@ -14184,16 +14295,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.696</v>
+        <v>44.345</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67049.76415999999</v>
+        <v>68045.6287</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7049.764159999992</v>
+        <v>8045.628700000001</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1174960693333332</v>
+        <v>0.1340938116666667</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -14482,6 +14593,9 @@
       </c>
       <c r="DC22" s="3" t="n">
         <v>43.696</v>
+      </c>
+      <c r="DD22" s="3" t="n">
+        <v>44.345</v>
       </c>
     </row>
     <row r="23">
@@ -14507,16 +14621,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.1453</v>
+        <v>63.19</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>171532.1236551</v>
+        <v>171653.54973</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>21532.1236551</v>
+        <v>21653.54973</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.143547491034</v>
+        <v>0.1443569982</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -14811,6 +14925,9 @@
       </c>
       <c r="DC23" s="3" t="n">
         <v>63.1453</v>
+      </c>
+      <c r="DD23" s="3" t="n">
+        <v>63.19</v>
       </c>
     </row>
     <row r="24">
@@ -14836,16 +14953,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>26.8474</v>
+        <v>26.8692</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>97546.96729640001</v>
+        <v>97626.17511119999</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-2453.032703599994</v>
+        <v>-2373.824888800009</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.02453032703599994</v>
+        <v>-0.02373824888800009</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -15134,6 +15251,9 @@
       </c>
       <c r="DC24" s="3" t="n">
         <v>26.8474</v>
+      </c>
+      <c r="DD24" s="3" t="n">
+        <v>26.8692</v>
       </c>
     </row>
     <row r="25">
@@ -15159,16 +15279,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>13.2104</v>
+        <v>13.215</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>216936.8822096</v>
+        <v>217012.42191</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>16936.88220959998</v>
+        <v>17012.42190999998</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.0846844110479999</v>
+        <v>0.08506210954999988</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -15460,6 +15580,9 @@
       </c>
       <c r="DC25" s="3" t="n">
         <v>13.2104</v>
+      </c>
+      <c r="DD25" s="3" t="n">
+        <v>13.215</v>
       </c>
     </row>
     <row r="26">
@@ -15485,16 +15608,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.4804</v>
+        <v>11.5991</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>137095.664886</v>
+        <v>138513.1464565</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>27095.66488599998</v>
+        <v>28513.14645649999</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.2463242262363635</v>
+        <v>0.2592104223318181</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -15786,6 +15909,9 @@
       </c>
       <c r="DC26" s="3" t="n">
         <v>11.4804</v>
+      </c>
+      <c r="DD26" s="3" t="n">
+        <v>11.5991</v>
       </c>
     </row>
     <row r="27">
@@ -15811,16 +15937,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>70.78400000000001</v>
+        <v>70.8528</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>114023.11424</v>
+        <v>114133.941408</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>4023.11424000001</v>
+        <v>4133.941407999999</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.03657376581818191</v>
+        <v>0.03758128552727272</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -16115,6 +16241,9 @@
       </c>
       <c r="DC27" s="3" t="n">
         <v>70.78400000000001</v>
+      </c>
+      <c r="DD27" s="3" t="n">
+        <v>70.8528</v>
       </c>
     </row>
     <row r="28">
@@ -16140,16 +16269,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>120.0335</v>
+        <v>119.7221</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>396909.6130095</v>
+        <v>395879.9200197</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>16909.61300950003</v>
+        <v>15879.92001970002</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.04449898160394744</v>
+        <v>0.04178926320973689</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -16444,6 +16573,9 @@
       </c>
       <c r="DC28" s="3" t="n">
         <v>120.0335</v>
+      </c>
+      <c r="DD28" s="3" t="n">
+        <v>119.7221</v>
       </c>
     </row>
     <row r="29">
@@ -16469,16 +16601,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.2624</v>
+        <v>12.3476</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>117764.4476672</v>
+        <v>118582.6831628</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>17764.44766719999</v>
+        <v>18582.68316279999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1776444766719999</v>
+        <v>0.1858268316279999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -16767,6 +16899,9 @@
       </c>
       <c r="DC29" s="3" t="n">
         <v>12.2624</v>
+      </c>
+      <c r="DD29" s="3" t="n">
+        <v>12.3476</v>
       </c>
     </row>
     <row r="30">
@@ -16792,16 +16927,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.6516</v>
+        <v>17.6661</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>130548.7800276</v>
+        <v>130656.0200121</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>30548.78002759999</v>
+        <v>30656.02001209999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.3054878002759999</v>
+        <v>0.3065602001209999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -17090,6 +17225,9 @@
       </c>
       <c r="DC30" s="3" t="n">
         <v>17.6516</v>
+      </c>
+      <c r="DD30" s="3" t="n">
+        <v>17.6661</v>
       </c>
     </row>
     <row r="31">
@@ -17115,16 +17253,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>411.6581</v>
+        <v>412.984</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109533.987248</v>
+        <v>109886.78272</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9533.98724799999</v>
+        <v>9886.782719999988</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09533987247999991</v>
+        <v>0.09886782719999988</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -17416,6 +17554,9 @@
       </c>
       <c r="DC31" s="3" t="n">
         <v>411.6581</v>
+      </c>
+      <c r="DD31" s="3" t="n">
+        <v>412.984</v>
       </c>
     </row>
     <row r="32">
@@ -17441,16 +17582,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.98</v>
+        <v>11.02</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>232116.7608</v>
+        <v>232962.3592</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>32116.76079999999</v>
+        <v>32962.35919999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1605838039999999</v>
+        <v>0.1648117959999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -17745,6 +17886,9 @@
       </c>
       <c r="DC32" s="3" t="n">
         <v>10.98</v>
+      </c>
+      <c r="DD32" s="3" t="n">
+        <v>11.02</v>
       </c>
     </row>
     <row r="33">
@@ -17770,16 +17914,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>20.33</v>
+        <v>20.28</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>72855.40119999999</v>
+        <v>72676.21920000001</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>12855.40119999999</v>
+        <v>12676.21920000001</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.2142566866666666</v>
+        <v>0.2112703200000001</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -18068,6 +18212,9 @@
       </c>
       <c r="DC33" s="3" t="n">
         <v>20.33</v>
+      </c>
+      <c r="DD33" s="3" t="n">
+        <v>20.28</v>
       </c>
     </row>
     <row r="34">
@@ -18093,16 +18240,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>229.8675</v>
+        <v>229.2492</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>80805.5521425</v>
+        <v>80588.20052520001</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>805.5521425000043</v>
+        <v>588.200525200009</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.01006940178125005</v>
+        <v>0.007352506565000113</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -18394,6 +18541,9 @@
       </c>
       <c r="DC34" s="3" t="n">
         <v>229.8675</v>
+      </c>
+      <c r="DD34" s="3" t="n">
+        <v>229.2492</v>
       </c>
     </row>
     <row r="35">
@@ -18419,16 +18569,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.29</v>
+        <v>16.27</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>116236.04067</v>
+        <v>116093.33221</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>16236.04066999999</v>
+        <v>16093.33220999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1623604066999999</v>
+        <v>0.1609333220999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -18720,6 +18870,9 @@
       </c>
       <c r="DC35" s="3" t="n">
         <v>16.29</v>
+      </c>
+      <c r="DD35" s="3" t="n">
+        <v>16.27</v>
       </c>
     </row>
     <row r="36">
@@ -18745,16 +18898,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>392.0411</v>
+        <v>394.1051</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>182575.8925166</v>
+        <v>183537.1097006</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>32575.8925166</v>
+        <v>33537.10970060001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.2171726167773333</v>
+        <v>0.2235807313373334</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -19046,6 +19199,9 @@
       </c>
       <c r="DC36" s="3" t="n">
         <v>392.0411</v>
+      </c>
+      <c r="DD36" s="3" t="n">
+        <v>394.1051</v>
       </c>
     </row>
     <row r="37">
@@ -19071,16 +19227,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.79</v>
+        <v>17.906</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>66941.79531</v>
+        <v>67378.290434</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>16941.79531</v>
+        <v>17378.290434</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.3388359062</v>
+        <v>0.3475658086799999</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -19372,6 +19528,9 @@
       </c>
       <c r="DC37" s="3" t="n">
         <v>17.79</v>
+      </c>
+      <c r="DD37" s="3" t="n">
+        <v>17.906</v>
       </c>
     </row>
     <row r="38">
@@ -19397,16 +19556,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2118</v>
+        <v>14.2034</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>84993.4140876</v>
+        <v>84943.1780388</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>4993.414087600002</v>
+        <v>4943.178038800004</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06241767609500003</v>
+        <v>0.06178972548500005</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -19695,6 +19854,9 @@
       </c>
       <c r="DC38" s="3" t="n">
         <v>14.2118</v>
+      </c>
+      <c r="DD38" s="3" t="n">
+        <v>14.2034</v>
       </c>
     </row>
     <row r="39">
@@ -19720,16 +19882,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1028.1888</v>
+        <v>1028.0807</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51287.0855328</v>
+        <v>51281.6933967</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1287.085532799996</v>
+        <v>1281.6933967</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02574171065599992</v>
+        <v>0.02563386793400001</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -20018,6 +20180,9 @@
       </c>
       <c r="DC39" s="3" t="n">
         <v>1028.1888</v>
+      </c>
+      <c r="DD39" s="3" t="n">
+        <v>1028.0807</v>
       </c>
     </row>
     <row r="40">
@@ -20043,16 +20208,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.851</v>
+        <v>21.7827</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>110151.480977</v>
+        <v>109807.1788329</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>10151.480977</v>
+        <v>9807.178832899997</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.10151480977</v>
+        <v>0.09807178832899997</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -20344,6 +20509,9 @@
       </c>
       <c r="DC40" s="3" t="n">
         <v>21.851</v>
+      </c>
+      <c r="DD40" s="3" t="n">
+        <v>21.7827</v>
       </c>
     </row>
     <row r="41">
@@ -20356,13 +20524,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5116603.6715003</v>
+        <v>5145636.5629507</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>646603.6715002999</v>
+        <v>675636.5629506999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1446540652125951</v>
+        <v>0.1511491192283445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-23
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-22 07:15 IST</t>
+          <t>Generated: 2026-09-23 07:17 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5145636.5629507</v>
+        <v>5155761.0299865</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>675636.5629506996</v>
+        <v>685761.0299864998</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1511491192283444</v>
+        <v>0.1534141006681208</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>543316.4980773926</v>
+        <v>545908.9930801392</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-47465.52192260744</v>
+        <v>-44873.02691986086</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08034354519219701</v>
+        <v>-0.07595530229552494</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5688953.061028092</v>
+        <v>5701670.023066639</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>628171.0410280926</v>
+        <v>640888.0030666394</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1241252910213455</v>
+        <v>0.1266381362670585</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-22</t>
+          <t>Last snapshot: 2026-09-23</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EH19"/>
+  <dimension ref="A1:EI19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -757,6 +757,7 @@
     <col width="21" customWidth="1" min="136" max="136"/>
     <col width="21" customWidth="1" min="137" max="137"/>
     <col width="21" customWidth="1" min="138" max="138"/>
+    <col width="21" customWidth="1" min="139" max="139"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1450,6 +1451,11 @@
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="EI1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1469,13 +1475,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>567.5</v>
+        <v>564.0999755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45400</v>
+        <v>45127.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1582.489999999998</v>
+        <v>1310.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1866,6 +1872,9 @@
       </c>
       <c r="EH2" s="3" t="n">
         <v>567.5</v>
+      </c>
+      <c r="EI2" s="3" t="n">
+        <v>564.0999755859375</v>
       </c>
     </row>
     <row r="3">
@@ -1913,13 +1922,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1396.400024414062</v>
+        <v>1401.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27928.00048828125</v>
+        <v>28023.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4176.579511718752</v>
+        <v>-4080.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2313,6 +2322,9 @@
       </c>
       <c r="EH4" s="3" t="n">
         <v>1396.400024414062</v>
+      </c>
+      <c r="EI4" s="3" t="n">
+        <v>1401.199951171875</v>
       </c>
     </row>
     <row r="5">
@@ -2333,13 +2345,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>555.5</v>
+        <v>599.2000122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11110</v>
+        <v>11984.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-3103.1</v>
+        <v>-2229.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2733,6 +2745,9 @@
       </c>
       <c r="EH5" s="3" t="n">
         <v>555.5</v>
+      </c>
+      <c r="EI5" s="3" t="n">
+        <v>599.2000122070312</v>
       </c>
     </row>
     <row r="6">
@@ -2753,13 +2768,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>322.25</v>
+        <v>324.4500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12890</v>
+        <v>12978.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4612.240000000002</v>
+        <v>-4524.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3153,6 +3168,9 @@
       </c>
       <c r="EH6" s="3" t="n">
         <v>322.25</v>
+      </c>
+      <c r="EI6" s="3" t="n">
+        <v>324.4500122070312</v>
       </c>
     </row>
     <row r="7">
@@ -3173,13 +3191,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>291.2000122070312</v>
+        <v>304.7999877929688</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>29120.00122070312</v>
+        <v>30479.99877929688</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>2686.181220703125</v>
+        <v>4046.178779296875</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3573,6 +3591,9 @@
       </c>
       <c r="EH7" s="3" t="n">
         <v>291.2000122070312</v>
+      </c>
+      <c r="EI7" s="3" t="n">
+        <v>304.7999877929688</v>
       </c>
     </row>
     <row r="8">
@@ -3620,13 +3641,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>16.17000007629395</v>
+        <v>16.1299991607666</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>24255.00011444092</v>
+        <v>24194.9987411499</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-6795.16988555908</v>
+        <v>-6855.171258850096</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4020,6 +4041,9 @@
       </c>
       <c r="EH9" s="3" t="n">
         <v>16.17000007629395</v>
+      </c>
+      <c r="EI9" s="3" t="n">
+        <v>16.1299991607666</v>
       </c>
     </row>
     <row r="10">
@@ -4040,13 +4064,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>471.5</v>
+        <v>468.75</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47150</v>
+        <v>46875</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-4348.480000000003</v>
+        <v>-4623.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4440,6 +4464,9 @@
       </c>
       <c r="EH10" s="3" t="n">
         <v>471.5</v>
+      </c>
+      <c r="EI10" s="3" t="n">
+        <v>468.75</v>
       </c>
     </row>
     <row r="11">
@@ -4460,13 +4487,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>13.21000003814697</v>
+        <v>14.42000007629395</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>13210.00003814697</v>
+        <v>14420.00007629395</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3368.790038146974</v>
+        <v>4578.790076293946</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4860,6 +4887,9 @@
       </c>
       <c r="EH11" s="3" t="n">
         <v>13.21000003814697</v>
+      </c>
+      <c r="EI11" s="3" t="n">
+        <v>14.42000007629395</v>
       </c>
     </row>
     <row r="12">
@@ -4880,13 +4910,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2793.89990234375</v>
+        <v>2836</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27938.9990234375</v>
+        <v>28360</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>215.7490234375</v>
+        <v>636.75</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5280,6 +5310,9 @@
       </c>
       <c r="EH12" s="3" t="n">
         <v>2793.89990234375</v>
+      </c>
+      <c r="EI12" s="3" t="n">
+        <v>2836</v>
       </c>
     </row>
     <row r="13">
@@ -5300,13 +5333,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>43.13999938964844</v>
+        <v>42.16999816894531</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>25883.99963378906</v>
+        <v>25301.99890136719</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-9147.76036621094</v>
+        <v>-9729.761098632815</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5700,6 +5733,9 @@
       </c>
       <c r="EH13" s="3" t="n">
         <v>43.13999938964844</v>
+      </c>
+      <c r="EI13" s="3" t="n">
+        <v>42.16999816894531</v>
       </c>
     </row>
     <row r="14">
@@ -5720,13 +5756,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>678.8499755859375</v>
+        <v>669.5999755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>33942.49877929688</v>
+        <v>33479.99877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-8520.011220703127</v>
+        <v>-8982.511220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6120,6 +6156,9 @@
       </c>
       <c r="EH14" s="3" t="n">
         <v>678.8499755859375</v>
+      </c>
+      <c r="EI14" s="3" t="n">
+        <v>669.5999755859375</v>
       </c>
     </row>
     <row r="15">
@@ -6194,13 +6233,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>518.75</v>
+        <v>519.0499877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25937.5</v>
+        <v>25952.49938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4182.970000000001</v>
+        <v>4197.969389648439</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6594,6 +6633,9 @@
       </c>
       <c r="EH17" s="3" t="n">
         <v>518.75</v>
+      </c>
+      <c r="EI17" s="3" t="n">
+        <v>519.0499877929688</v>
       </c>
     </row>
     <row r="18">
@@ -6614,13 +6656,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>367.7999877929688</v>
+        <v>369.6000061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36779.99877929688</v>
+        <v>36960.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9860.821220703125</v>
+        <v>-9680.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7014,6 +7056,9 @@
       </c>
       <c r="EH18" s="3" t="n">
         <v>367.7999877929688</v>
+      </c>
+      <c r="EI18" s="3" t="n">
+        <v>369.6000061035156</v>
       </c>
     </row>
     <row r="19">
@@ -7026,10 +7071,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>543316.4980773926</v>
+        <v>545908.9930801392</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-47465.52192260743</v>
+        <v>-44873.02691986085</v>
       </c>
     </row>
   </sheetData>
@@ -7043,7 +7088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DD41"/>
+  <dimension ref="A1:DE41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7053,8 +7098,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -7154,6 +7199,7 @@
     <col width="13" customWidth="1" min="106" max="106"/>
     <col width="13" customWidth="1" min="107" max="107"/>
     <col width="13" customWidth="1" min="108" max="108"/>
+    <col width="13" customWidth="1" min="109" max="109"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7697,6 +7743,11 @@
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="DE1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7721,16 +7772,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>58.1047</v>
+        <v>58.0646</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>65221.4798654</v>
+        <v>65176.4683372</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>15221.4798654</v>
+        <v>15176.4683372</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.304429597308</v>
+        <v>0.303529366744</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8028,6 +8079,9 @@
       </c>
       <c r="DD2" s="3" t="n">
         <v>58.1047</v>
+      </c>
+      <c r="DE2" s="3" t="n">
+        <v>58.0646</v>
       </c>
     </row>
     <row r="3">
@@ -8053,16 +8107,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.6665</v>
+        <v>26.9104</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65471.93746450001</v>
+        <v>66070.7639152</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5471.937464500006</v>
+        <v>6070.763915200005</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09119895774166677</v>
+        <v>0.1011793985866667</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8354,6 +8408,9 @@
       </c>
       <c r="DD3" s="3" t="n">
         <v>26.6665</v>
+      </c>
+      <c r="DE3" s="3" t="n">
+        <v>26.9104</v>
       </c>
     </row>
     <row r="4">
@@ -8379,16 +8436,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.98</v>
+        <v>13.07</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>249295.08714</v>
+        <v>251023.63551</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>69295.08714000002</v>
+        <v>71023.63551000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3849727063333334</v>
+        <v>0.3945757528333335</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -8680,6 +8737,9 @@
       </c>
       <c r="DD4" s="3" t="n">
         <v>12.98</v>
+      </c>
+      <c r="DE4" s="3" t="n">
+        <v>13.07</v>
       </c>
     </row>
     <row r="5">
@@ -8705,16 +8765,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.3466</v>
+        <v>9.2996</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>171548.3189008</v>
+        <v>170685.6767648</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-38451.68109919998</v>
+        <v>-39314.32323519999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1831032433295237</v>
+        <v>-0.1872110630247619</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9006,6 +9066,9 @@
       </c>
       <c r="DD5" s="3" t="n">
         <v>9.3466</v>
+      </c>
+      <c r="DE5" s="3" t="n">
+        <v>9.2996</v>
       </c>
     </row>
     <row r="6">
@@ -9031,16 +9094,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.6666</v>
+        <v>11.6363</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>49337.7830682</v>
+        <v>49209.6450651</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-662.2169318000015</v>
+        <v>-790.3549349000023</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.01324433863600003</v>
+        <v>-0.01580709869800005</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9338,6 +9401,9 @@
       </c>
       <c r="DD6" s="3" t="n">
         <v>11.6666</v>
+      </c>
+      <c r="DE6" s="3" t="n">
+        <v>11.6363</v>
       </c>
     </row>
     <row r="7">
@@ -9363,16 +9429,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.6408</v>
+        <v>34.8275</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>76418.99043199999</v>
+        <v>76830.8581</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>16418.99043199999</v>
+        <v>16830.8581</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2736498405333332</v>
+        <v>0.2805143016666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -9664,6 +9730,9 @@
       </c>
       <c r="DD7" s="3" t="n">
         <v>34.6408</v>
+      </c>
+      <c r="DE7" s="3" t="n">
+        <v>34.8275</v>
       </c>
     </row>
     <row r="8">
@@ -9689,16 +9758,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>36.0099</v>
+        <v>36.297</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57781.2334707</v>
+        <v>58241.912121</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7781.233470700005</v>
+        <v>8241.912121000001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1556246694140001</v>
+        <v>0.16483824242</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -9996,6 +10065,9 @@
       </c>
       <c r="DD8" s="3" t="n">
         <v>36.0099</v>
+      </c>
+      <c r="DE8" s="3" t="n">
+        <v>36.297</v>
       </c>
     </row>
     <row r="9">
@@ -10021,16 +10093,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.4204</v>
+        <v>42.1878</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>133348.5458172</v>
+        <v>135819.1080054</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>33348.54581720001</v>
+        <v>35819.10800540002</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3334854581720001</v>
+        <v>0.3581910800540002</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10322,6 +10394,9 @@
       </c>
       <c r="DD9" s="3" t="n">
         <v>41.4204</v>
+      </c>
+      <c r="DE9" s="3" t="n">
+        <v>42.1878</v>
       </c>
     </row>
     <row r="10">
@@ -10347,16 +10422,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.7334</v>
+        <v>48.8786</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138727.3717106</v>
+        <v>139140.7065974</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38727.37171060001</v>
+        <v>39140.70659740001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3872737171060001</v>
+        <v>0.3914070659740002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -10648,6 +10723,9 @@
       </c>
       <c r="DD10" s="3" t="n">
         <v>48.7334</v>
+      </c>
+      <c r="DE10" s="3" t="n">
+        <v>48.8786</v>
       </c>
     </row>
     <row r="11">
@@ -10673,16 +10751,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.3221</v>
+        <v>107.8955</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32295.2590099</v>
+        <v>32467.8059645</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2295.259009900001</v>
+        <v>2467.805964499999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07650863366333337</v>
+        <v>0.08226019881666664</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -10974,6 +11052,9 @@
       </c>
       <c r="DD11" s="3" t="n">
         <v>107.3221</v>
+      </c>
+      <c r="DE11" s="3" t="n">
+        <v>107.8955</v>
       </c>
     </row>
     <row r="12">
@@ -10999,16 +11080,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>230.669</v>
+        <v>229.926</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>107381.494218</v>
+        <v>107035.611372</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>7381.494218000007</v>
+        <v>7035.611371999999</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.07381494218000006</v>
+        <v>0.07035611371999999</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -11306,6 +11387,9 @@
       </c>
       <c r="DD12" s="3" t="n">
         <v>230.669</v>
+      </c>
+      <c r="DE12" s="3" t="n">
+        <v>229.926</v>
       </c>
     </row>
     <row r="13">
@@ -11331,16 +11415,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22.892</v>
+        <v>22.689</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>265263.45366</v>
+        <v>262911.169845</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>65263.45366</v>
+        <v>62911.16984499997</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.3263172683</v>
+        <v>0.3145558492249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -11638,6 +11722,9 @@
       </c>
       <c r="DD13" s="3" t="n">
         <v>22.892</v>
+      </c>
+      <c r="DE13" s="3" t="n">
+        <v>22.689</v>
       </c>
     </row>
     <row r="14">
@@ -11663,16 +11750,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.6079</v>
+        <v>39.0148</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>139282.0916874</v>
+        <v>140750.0265688</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>39282.09168740001</v>
+        <v>40750.02656880001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3928209168740001</v>
+        <v>0.4075002656880001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -11964,6 +12051,9 @@
       </c>
       <c r="DD14" s="3" t="n">
         <v>38.6079</v>
+      </c>
+      <c r="DE14" s="3" t="n">
+        <v>39.0148</v>
       </c>
     </row>
     <row r="15">
@@ -11989,16 +12079,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.78</v>
+        <v>11.75</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114783.69566</v>
+        <v>114491.37725</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14783.69566</v>
+        <v>14491.37725000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1478369566</v>
+        <v>0.1449137725</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -12296,6 +12386,9 @@
       </c>
       <c r="DD15" s="3" t="n">
         <v>11.78</v>
+      </c>
+      <c r="DE15" s="3" t="n">
+        <v>11.75</v>
       </c>
     </row>
     <row r="16">
@@ -12321,16 +12414,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.3905</v>
+        <v>25.6033</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>145308.003384</v>
+        <v>146525.8424624</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>45308.00338399998</v>
+        <v>46525.8424624</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4530800338399998</v>
+        <v>0.465258424624</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -12622,6 +12715,9 @@
       </c>
       <c r="DD16" s="3" t="n">
         <v>25.3905</v>
+      </c>
+      <c r="DE16" s="3" t="n">
+        <v>25.6033</v>
       </c>
     </row>
     <row r="17">
@@ -12647,16 +12743,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>17.0253</v>
+        <v>17.0425</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>56286.6122421</v>
+        <v>56343.4764225</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>6286.612242100004</v>
+        <v>6343.476422499996</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1257322448420001</v>
+        <v>0.1268695284499999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -12948,6 +13044,9 @@
       </c>
       <c r="DD17" s="3" t="n">
         <v>17.0253</v>
+      </c>
+      <c r="DE17" s="3" t="n">
+        <v>17.0425</v>
       </c>
     </row>
     <row r="18">
@@ -12973,16 +13072,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.41</v>
+        <v>47.22</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>89435.93075999999</v>
+        <v>89077.50791999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>9435.930759999988</v>
+        <v>9077.507919999989</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1179491344999999</v>
+        <v>0.1134688489999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -13280,6 +13379,9 @@
       </c>
       <c r="DD18" s="3" t="n">
         <v>47.41</v>
+      </c>
+      <c r="DE18" s="3" t="n">
+        <v>47.22</v>
       </c>
     </row>
     <row r="19">
@@ -13305,16 +13407,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.2202</v>
+        <v>13.4049</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>191253.5398732</v>
+        <v>193925.5515534</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>41253.5398732</v>
+        <v>43925.5515534</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2750235991546667</v>
+        <v>0.292837010356</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -13606,6 +13708,9 @@
       </c>
       <c r="DD19" s="3" t="n">
         <v>13.2202</v>
+      </c>
+      <c r="DE19" s="3" t="n">
+        <v>13.4049</v>
       </c>
     </row>
     <row r="20">
@@ -13631,16 +13736,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.970000000000001</v>
+        <v>10</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>261770.35591</v>
+        <v>262558.03</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>11770.35591000001</v>
+        <v>12558.03000000003</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.04708142364000005</v>
+        <v>0.05023212000000011</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -13938,6 +14043,9 @@
       </c>
       <c r="DD20" s="3" t="n">
         <v>9.970000000000001</v>
+      </c>
+      <c r="DE20" s="3" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -13963,16 +14071,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>114.6398</v>
+        <v>114.7061</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>174167.5479082</v>
+        <v>174268.2747799</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>4167.54790819998</v>
+        <v>4268.274779900006</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.024514987695294</v>
+        <v>0.02510749870529416</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -14270,6 +14378,9 @@
       </c>
       <c r="DD21" s="3" t="n">
         <v>114.6398</v>
+      </c>
+      <c r="DE21" s="3" t="n">
+        <v>114.7061</v>
       </c>
     </row>
     <row r="22">
@@ -14295,16 +14406,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.345</v>
+        <v>44.764</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68045.6287</v>
+        <v>68688.56744</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8045.628700000001</v>
+        <v>8688.567439999999</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1340938116666667</v>
+        <v>0.1448094573333333</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -14596,6 +14707,9 @@
       </c>
       <c r="DD22" s="3" t="n">
         <v>44.345</v>
+      </c>
+      <c r="DE22" s="3" t="n">
+        <v>44.764</v>
       </c>
     </row>
     <row r="23">
@@ -14621,16 +14735,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.19</v>
+        <v>63.4874</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>171653.54973</v>
+        <v>172461.4270158</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>21653.54973</v>
+        <v>22461.4270158</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1443569982</v>
+        <v>0.149742846772</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -14928,6 +15042,9 @@
       </c>
       <c r="DD23" s="3" t="n">
         <v>63.19</v>
+      </c>
+      <c r="DE23" s="3" t="n">
+        <v>63.4874</v>
       </c>
     </row>
     <row r="24">
@@ -14953,16 +15070,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>26.8692</v>
+        <v>26.8557</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>97626.17511119999</v>
+        <v>97577.12440019999</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-2373.824888800009</v>
+        <v>-2422.875599800012</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.02373824888800009</v>
+        <v>-0.02422875599800012</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -15254,6 +15371,9 @@
       </c>
       <c r="DD24" s="3" t="n">
         <v>26.8692</v>
+      </c>
+      <c r="DE24" s="3" t="n">
+        <v>26.8557</v>
       </c>
     </row>
     <row r="25">
@@ -15279,16 +15399,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>13.215</v>
+        <v>13.1893</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>217012.42191</v>
+        <v>216590.3848882</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>17012.42190999998</v>
+        <v>16590.38488819997</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.08506210954999988</v>
+        <v>0.08295192444099986</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -15583,6 +15703,9 @@
       </c>
       <c r="DD25" s="3" t="n">
         <v>13.215</v>
+      </c>
+      <c r="DE25" s="3" t="n">
+        <v>13.1893</v>
       </c>
     </row>
     <row r="26">
@@ -15608,16 +15731,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.5991</v>
+        <v>11.7355</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>138513.1464565</v>
+        <v>140141.9963825</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>28513.14645649999</v>
+        <v>30141.99638250002</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.2592104223318181</v>
+        <v>0.2740181489318183</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -15912,6 +16035,9 @@
       </c>
       <c r="DD26" s="3" t="n">
         <v>11.5991</v>
+      </c>
+      <c r="DE26" s="3" t="n">
+        <v>11.7355</v>
       </c>
     </row>
     <row r="27">
@@ -15937,16 +16063,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>70.8528</v>
+        <v>70.792</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>114133.941408</v>
+        <v>114036.00112</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>4133.941407999999</v>
+        <v>4036.001120000001</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.03758128552727272</v>
+        <v>0.03669091927272728</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -16244,6 +16370,9 @@
       </c>
       <c r="DD27" s="3" t="n">
         <v>70.8528</v>
+      </c>
+      <c r="DE27" s="3" t="n">
+        <v>70.792</v>
       </c>
     </row>
     <row r="28">
@@ -16269,16 +16398,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>119.7221</v>
+        <v>119.7578</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>395879.9200197</v>
+        <v>395997.9676746</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>15879.92001970002</v>
+        <v>15997.96767460002</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.04178926320973689</v>
+        <v>0.04209991493315794</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -16576,6 +16705,9 @@
       </c>
       <c r="DD28" s="3" t="n">
         <v>119.7221</v>
+      </c>
+      <c r="DE28" s="3" t="n">
+        <v>119.7578</v>
       </c>
     </row>
     <row r="29">
@@ -16601,16 +16733,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.3476</v>
+        <v>12.4206</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>118582.6831628</v>
+        <v>119283.7534818</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>18582.68316279999</v>
+        <v>19283.7534818</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1858268316279999</v>
+        <v>0.192837534818</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -16902,6 +17034,9 @@
       </c>
       <c r="DD29" s="3" t="n">
         <v>12.3476</v>
+      </c>
+      <c r="DE29" s="3" t="n">
+        <v>12.4206</v>
       </c>
     </row>
     <row r="30">
@@ -16927,16 +17062,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.6661</v>
+        <v>17.6535</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>130656.0200121</v>
+        <v>130562.8321635</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>30656.02001209999</v>
+        <v>30562.8321635</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.3065602001209999</v>
+        <v>0.305628321635</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -17228,6 +17363,9 @@
       </c>
       <c r="DD30" s="3" t="n">
         <v>17.6661</v>
+      </c>
+      <c r="DE30" s="3" t="n">
+        <v>17.6535</v>
       </c>
     </row>
     <row r="31">
@@ -17253,16 +17391,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>412.984</v>
+        <v>412.6503</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109886.78272</v>
+        <v>109797.991824</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9886.782719999988</v>
+        <v>9797.991823999997</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09886782719999988</v>
+        <v>0.09797991823999996</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -17557,6 +17695,9 @@
       </c>
       <c r="DD31" s="3" t="n">
         <v>412.984</v>
+      </c>
+      <c r="DE31" s="3" t="n">
+        <v>412.6503</v>
       </c>
     </row>
     <row r="32">
@@ -17582,16 +17723,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>11.02</v>
+        <v>11.03</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>232962.3592</v>
+        <v>233173.7588</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>32962.35919999998</v>
+        <v>33173.75879999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1648117959999999</v>
+        <v>0.1658687939999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -17889,6 +18030,9 @@
       </c>
       <c r="DD32" s="3" t="n">
         <v>11.02</v>
+      </c>
+      <c r="DE32" s="3" t="n">
+        <v>11.03</v>
       </c>
     </row>
     <row r="33">
@@ -17914,16 +18058,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>20.28</v>
+        <v>20.35</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>72676.21920000001</v>
+        <v>72927.07400000001</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>12676.21920000001</v>
+        <v>12927.07400000001</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.2112703200000001</v>
+        <v>0.2154512333333335</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -18215,6 +18359,9 @@
       </c>
       <c r="DD33" s="3" t="n">
         <v>20.28</v>
+      </c>
+      <c r="DE33" s="3" t="n">
+        <v>20.35</v>
       </c>
     </row>
     <row r="34">
@@ -18240,16 +18387,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>229.2492</v>
+        <v>228.6807</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>80588.20052520001</v>
+        <v>80388.3551517</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>588.200525200009</v>
+        <v>388.3551517000014</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.007352506565000113</v>
+        <v>0.004854439396250018</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -18544,6 +18691,9 @@
       </c>
       <c r="DD34" s="3" t="n">
         <v>229.2492</v>
+      </c>
+      <c r="DE34" s="3" t="n">
+        <v>228.6807</v>
       </c>
     </row>
     <row r="35">
@@ -18569,16 +18719,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.27</v>
+        <v>16.28</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>116093.33221</v>
+        <v>116164.68644</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>16093.33220999999</v>
+        <v>16164.68644</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1609333220999999</v>
+        <v>0.1616468644000001</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -18873,6 +19023,9 @@
       </c>
       <c r="DD35" s="3" t="n">
         <v>16.27</v>
+      </c>
+      <c r="DE35" s="3" t="n">
+        <v>16.28</v>
       </c>
     </row>
     <row r="36">
@@ -18898,16 +19051,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>394.1051</v>
+        <v>392.2582</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>183537.1097006</v>
+        <v>182676.9972892</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>33537.10970060001</v>
+        <v>32676.99728919999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.2235807313373334</v>
+        <v>0.2178466485946666</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -19202,6 +19355,9 @@
       </c>
       <c r="DD36" s="3" t="n">
         <v>394.1051</v>
+      </c>
+      <c r="DE36" s="3" t="n">
+        <v>392.2582</v>
       </c>
     </row>
     <row r="37">
@@ -19227,16 +19383,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.906</v>
+        <v>17.791</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>67378.290434</v>
+        <v>66945.55819900001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>17378.290434</v>
+        <v>16945.55819900001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.3475658086799999</v>
+        <v>0.3389111639800002</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -19531,6 +19687,9 @@
       </c>
       <c r="DD37" s="3" t="n">
         <v>17.906</v>
+      </c>
+      <c r="DE37" s="3" t="n">
+        <v>17.791</v>
       </c>
     </row>
     <row r="38">
@@ -19556,16 +19715,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2034</v>
+        <v>14.1685</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>84943.1780388</v>
+        <v>84734.459217</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>4943.178038800004</v>
+        <v>4734.459216999996</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06178972548500005</v>
+        <v>0.05918074021249995</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -19857,6 +20016,9 @@
       </c>
       <c r="DD38" s="3" t="n">
         <v>14.2034</v>
+      </c>
+      <c r="DE38" s="3" t="n">
+        <v>14.1685</v>
       </c>
     </row>
     <row r="39">
@@ -19882,16 +20044,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1028.0807</v>
+        <v>1028.4146</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51281.6933967</v>
+        <v>51298.3486626</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1281.6933967</v>
+        <v>1298.348662600001</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02563386793400001</v>
+        <v>0.02596697325200003</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -20183,6 +20345,9 @@
       </c>
       <c r="DD39" s="3" t="n">
         <v>1028.0807</v>
+      </c>
+      <c r="DE39" s="3" t="n">
+        <v>1028.4146</v>
       </c>
     </row>
     <row r="40">
@@ -20208,16 +20373,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.7827</v>
+        <v>21.7734</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>109807.1788329</v>
+        <v>109760.2972818</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>9807.178832899997</v>
+        <v>9760.297281799998</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.09807178832899997</v>
+        <v>0.09760297281799998</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -20512,6 +20677,9 @@
       </c>
       <c r="DD40" s="3" t="n">
         <v>21.7827</v>
+      </c>
+      <c r="DE40" s="3" t="n">
+        <v>21.7734</v>
       </c>
     </row>
     <row r="41">
@@ -20524,13 +20692,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5145636.5629507</v>
+        <v>5155761.0299865</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>675636.5629506999</v>
+        <v>685761.0299865</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1511491192283445</v>
+        <v>0.1534141006681208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-24
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-23 07:17 IST</t>
+          <t>Generated: 2026-09-24 07:07 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5155761.0299865</v>
+        <v>5167781.2049771</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>685761.0299864998</v>
+        <v>697781.2049770998</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1534141006681208</v>
+        <v>0.1561031778472259</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>545908.9930801392</v>
+        <v>543811.5040092468</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-44873.02691986086</v>
+        <v>-46970.51599075319</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07595530229552494</v>
+        <v>-0.07950566266514542</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5701670.023066639</v>
+        <v>5711592.708986347</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>640888.0030666394</v>
+        <v>650810.6889863471</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1266381362670585</v>
+        <v>0.1285988383641837</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-23</t>
+          <t>Last snapshot: 2026-09-24</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EI19"/>
+  <dimension ref="A1:EJ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -758,6 +758,7 @@
     <col width="21" customWidth="1" min="137" max="137"/>
     <col width="21" customWidth="1" min="138" max="138"/>
     <col width="21" customWidth="1" min="139" max="139"/>
+    <col width="21" customWidth="1" min="140" max="140"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1456,6 +1457,11 @@
           <t>2026-09-23</t>
         </is>
       </c>
+      <c r="EJ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1475,13 +1481,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>564.0999755859375</v>
+        <v>573.6500244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45127.998046875</v>
+        <v>45892.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1310.488046874998</v>
+        <v>2074.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1875,6 +1881,9 @@
       </c>
       <c r="EI2" s="3" t="n">
         <v>564.0999755859375</v>
+      </c>
+      <c r="EJ2" s="3" t="n">
+        <v>573.6500244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1922,13 +1931,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1401.199951171875</v>
+        <v>1400</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28023.9990234375</v>
+        <v>28000</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4080.580976562502</v>
+        <v>-4104.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2325,6 +2334,9 @@
       </c>
       <c r="EI4" s="3" t="n">
         <v>1401.199951171875</v>
+      </c>
+      <c r="EJ4" s="3" t="n">
+        <v>1400</v>
       </c>
     </row>
     <row r="5">
@@ -2345,13 +2357,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>599.2000122070312</v>
+        <v>581.6500244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11984.00024414062</v>
+        <v>11633.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-2229.099755859375</v>
+        <v>-2580.09951171875</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2748,6 +2760,9 @@
       </c>
       <c r="EI5" s="3" t="n">
         <v>599.2000122070312</v>
+      </c>
+      <c r="EJ5" s="3" t="n">
+        <v>581.6500244140625</v>
       </c>
     </row>
     <row r="6">
@@ -2768,13 +2783,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>324.4500122070312</v>
+        <v>334.75</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12978.00048828125</v>
+        <v>13390</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4524.239511718752</v>
+        <v>-4112.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3171,6 +3186,9 @@
       </c>
       <c r="EI6" s="3" t="n">
         <v>324.4500122070312</v>
+      </c>
+      <c r="EJ6" s="3" t="n">
+        <v>334.75</v>
       </c>
     </row>
     <row r="7">
@@ -3191,13 +3209,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>304.7999877929688</v>
+        <v>299.6000061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>30479.99877929688</v>
+        <v>29960.00061035156</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4046.178779296875</v>
+        <v>3526.180610351563</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3594,6 +3612,9 @@
       </c>
       <c r="EI7" s="3" t="n">
         <v>304.7999877929688</v>
+      </c>
+      <c r="EJ7" s="3" t="n">
+        <v>299.6000061035156</v>
       </c>
     </row>
     <row r="8">
@@ -3641,13 +3662,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>16.1299991607666</v>
+        <v>15.86999988555908</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>24194.9987411499</v>
+        <v>23804.99982833862</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-6855.171258850096</v>
+        <v>-7245.170171661375</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4044,6 +4065,9 @@
       </c>
       <c r="EI9" s="3" t="n">
         <v>16.1299991607666</v>
+      </c>
+      <c r="EJ9" s="3" t="n">
+        <v>15.86999988555908</v>
       </c>
     </row>
     <row r="10">
@@ -4064,13 +4088,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>468.75</v>
+        <v>471.5</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46875</v>
+        <v>47150</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-4623.480000000003</v>
+        <v>-4348.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4467,6 +4491,9 @@
       </c>
       <c r="EI10" s="3" t="n">
         <v>468.75</v>
+      </c>
+      <c r="EJ10" s="3" t="n">
+        <v>471.5</v>
       </c>
     </row>
     <row r="11">
@@ -4487,13 +4514,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>14.42000007629395</v>
+        <v>14.22999954223633</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14420.00007629395</v>
+        <v>14229.99954223633</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4578.790076293946</v>
+        <v>4388.789542236329</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4890,6 +4917,9 @@
       </c>
       <c r="EI11" s="3" t="n">
         <v>14.42000007629395</v>
+      </c>
+      <c r="EJ11" s="3" t="n">
+        <v>14.22999954223633</v>
       </c>
     </row>
     <row r="12">
@@ -4910,13 +4940,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2836</v>
+        <v>2822.10009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>28360</v>
+        <v>28221.0009765625</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>636.75</v>
+        <v>497.7509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5313,6 +5343,9 @@
       </c>
       <c r="EI12" s="3" t="n">
         <v>2836</v>
+      </c>
+      <c r="EJ12" s="3" t="n">
+        <v>2822.10009765625</v>
       </c>
     </row>
     <row r="13">
@@ -5333,13 +5366,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>42.16999816894531</v>
+        <v>41</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>25301.99890136719</v>
+        <v>24600</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-9729.761098632815</v>
+        <v>-10431.76</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5736,6 +5769,9 @@
       </c>
       <c r="EI13" s="3" t="n">
         <v>42.16999816894531</v>
+      </c>
+      <c r="EJ13" s="3" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="14">
@@ -5756,13 +5792,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>669.5999755859375</v>
+        <v>662</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>33479.99877929688</v>
+        <v>33100</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-8982.511220703127</v>
+        <v>-9362.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6159,6 +6195,9 @@
       </c>
       <c r="EI14" s="3" t="n">
         <v>669.5999755859375</v>
+      </c>
+      <c r="EJ14" s="3" t="n">
+        <v>662</v>
       </c>
     </row>
     <row r="15">
@@ -6233,13 +6272,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>519.0499877929688</v>
+        <v>510</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25952.49938964844</v>
+        <v>25500</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4197.969389648439</v>
+        <v>3745.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6636,6 +6675,9 @@
       </c>
       <c r="EI17" s="3" t="n">
         <v>519.0499877929688</v>
+      </c>
+      <c r="EJ17" s="3" t="n">
+        <v>510</v>
       </c>
     </row>
     <row r="18">
@@ -6656,13 +6698,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>369.6000061035156</v>
+        <v>365.6000061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36960.00061035156</v>
+        <v>36560.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9680.819389648437</v>
+        <v>-10080.81938964844</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7059,6 +7101,9 @@
       </c>
       <c r="EI18" s="3" t="n">
         <v>369.6000061035156</v>
+      </c>
+      <c r="EJ18" s="3" t="n">
+        <v>365.6000061035156</v>
       </c>
     </row>
     <row r="19">
@@ -7071,10 +7116,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>545908.9930801392</v>
+        <v>543811.5040092468</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-44873.02691986085</v>
+        <v>-46970.51599075319</v>
       </c>
     </row>
   </sheetData>
@@ -7088,7 +7133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DE41"/>
+  <dimension ref="A1:DF41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7200,6 +7245,7 @@
     <col width="13" customWidth="1" min="107" max="107"/>
     <col width="13" customWidth="1" min="108" max="108"/>
     <col width="13" customWidth="1" min="109" max="109"/>
+    <col width="13" customWidth="1" min="110" max="110"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7748,6 +7794,11 @@
           <t>2026-09-23</t>
         </is>
       </c>
+      <c r="DF1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7772,16 +7823,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>58.0646</v>
+        <v>57.6847</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>65176.4683372</v>
+        <v>64750.0374254</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>15176.4683372</v>
+        <v>14750.0374254</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.303529366744</v>
+        <v>0.295000748508</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8082,6 +8133,9 @@
       </c>
       <c r="DE2" s="3" t="n">
         <v>58.0646</v>
+      </c>
+      <c r="DF2" s="3" t="n">
+        <v>57.6847</v>
       </c>
     </row>
     <row r="3">
@@ -8107,16 +8161,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.9104</v>
+        <v>26.7849</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>66070.7639152</v>
+        <v>65762.6346837</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>6070.763915200005</v>
+        <v>5762.634683700002</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.1011793985866667</v>
+        <v>0.09604391139500003</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8411,6 +8465,9 @@
       </c>
       <c r="DE3" s="3" t="n">
         <v>26.9104</v>
+      </c>
+      <c r="DF3" s="3" t="n">
+        <v>26.7849</v>
       </c>
     </row>
     <row r="4">
@@ -8436,16 +8493,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>13.07</v>
+        <v>12.92</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>251023.63551</v>
+        <v>248142.72156</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>71023.63551000002</v>
+        <v>68142.72156000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3945757528333335</v>
+        <v>0.3785706753333334</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -8740,6 +8797,9 @@
       </c>
       <c r="DE4" s="3" t="n">
         <v>13.07</v>
+      </c>
+      <c r="DF4" s="3" t="n">
+        <v>12.92</v>
       </c>
     </row>
     <row r="5">
@@ -8765,16 +8825,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.2996</v>
+        <v>9.3133</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>170685.6767648</v>
+        <v>170937.1277704</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-39314.32323519999</v>
+        <v>-39062.87222960001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1872110630247619</v>
+        <v>-0.1860136772838095</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9069,6 +9129,9 @@
       </c>
       <c r="DE5" s="3" t="n">
         <v>9.2996</v>
+      </c>
+      <c r="DF5" s="3" t="n">
+        <v>9.3133</v>
       </c>
     </row>
     <row r="6">
@@ -9094,16 +9157,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.6363</v>
+        <v>11.6984</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>49209.6450651</v>
+        <v>49472.26453679999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-790.3549349000023</v>
+        <v>-527.7354632000061</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.01580709869800005</v>
+        <v>-0.01055470926400012</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9404,6 +9467,9 @@
       </c>
       <c r="DE6" s="3" t="n">
         <v>11.6363</v>
+      </c>
+      <c r="DF6" s="3" t="n">
+        <v>11.6984</v>
       </c>
     </row>
     <row r="7">
@@ -9429,16 +9495,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.8275</v>
+        <v>34.4836</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>76830.8581</v>
+        <v>76072.20094400001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>16830.8581</v>
+        <v>16072.20094400001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2805143016666666</v>
+        <v>0.2678700157333335</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -9733,6 +9799,9 @@
       </c>
       <c r="DE7" s="3" t="n">
         <v>34.8275</v>
+      </c>
+      <c r="DF7" s="3" t="n">
+        <v>34.4836</v>
       </c>
     </row>
     <row r="8">
@@ -9758,16 +9827,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>36.297</v>
+        <v>36.3955</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>58241.912121</v>
+        <v>58399.9645315</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>8241.912121000001</v>
+        <v>8399.964531500002</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.16483824242</v>
+        <v>0.16799929063</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -10068,6 +10137,9 @@
       </c>
       <c r="DE8" s="3" t="n">
         <v>36.297</v>
+      </c>
+      <c r="DF8" s="3" t="n">
+        <v>36.3955</v>
       </c>
     </row>
     <row r="9">
@@ -10093,16 +10165,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.1878</v>
+        <v>42.3429</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>135819.1080054</v>
+        <v>136318.4358597</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>35819.10800540002</v>
+        <v>36318.4358597</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3581910800540002</v>
+        <v>0.3631843585969999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10397,6 +10469,9 @@
       </c>
       <c r="DE9" s="3" t="n">
         <v>42.1878</v>
+      </c>
+      <c r="DF9" s="3" t="n">
+        <v>42.3429</v>
       </c>
     </row>
     <row r="10">
@@ -10422,16 +10497,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.8786</v>
+        <v>48.6196</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>139140.7065974</v>
+        <v>138403.4219164</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>39140.70659740001</v>
+        <v>38403.4219164</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3914070659740002</v>
+        <v>0.3840342191639999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -10726,6 +10801,9 @@
       </c>
       <c r="DE10" s="3" t="n">
         <v>48.8786</v>
+      </c>
+      <c r="DF10" s="3" t="n">
+        <v>48.6196</v>
       </c>
     </row>
     <row r="11">
@@ -10751,16 +10829,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.8955</v>
+        <v>106.9125</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32467.8059645</v>
+        <v>32172.0025875</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2467.805964499999</v>
+        <v>2172.002587499996</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.08226019881666664</v>
+        <v>0.07240008624999986</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -11055,6 +11133,9 @@
       </c>
       <c r="DE11" s="3" t="n">
         <v>107.8955</v>
+      </c>
+      <c r="DF11" s="3" t="n">
+        <v>106.9125</v>
       </c>
     </row>
     <row r="12">
@@ -11080,16 +11161,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>229.926</v>
+        <v>231.07</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>107035.611372</v>
+        <v>107568.16854</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>7035.611371999999</v>
+        <v>7568.168539999999</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.07035611371999999</v>
+        <v>0.07568168539999999</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -11390,6 +11471,9 @@
       </c>
       <c r="DE12" s="3" t="n">
         <v>229.926</v>
+      </c>
+      <c r="DF12" s="3" t="n">
+        <v>231.07</v>
       </c>
     </row>
     <row r="13">
@@ -11415,16 +11499,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22.689</v>
+        <v>22.873</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>262911.169845</v>
+        <v>265043.289165</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>62911.16984499997</v>
+        <v>65043.28916500002</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.3145558492249999</v>
+        <v>0.3252164458250001</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -11725,6 +11809,9 @@
       </c>
       <c r="DE13" s="3" t="n">
         <v>22.689</v>
+      </c>
+      <c r="DF13" s="3" t="n">
+        <v>22.873</v>
       </c>
     </row>
     <row r="14">
@@ -11750,16 +11837,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.0148</v>
+        <v>38.9279</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>140750.0265688</v>
+        <v>140436.5256074</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>40750.02656880001</v>
+        <v>40436.52560740002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4075002656880001</v>
+        <v>0.4043652560740002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -12054,6 +12141,9 @@
       </c>
       <c r="DE14" s="3" t="n">
         <v>39.0148</v>
+      </c>
+      <c r="DF14" s="3" t="n">
+        <v>38.9279</v>
       </c>
     </row>
     <row r="15">
@@ -12079,16 +12169,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.75</v>
+        <v>11.81</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114491.37725</v>
+        <v>115076.01407</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14491.37725000001</v>
+        <v>15076.01407</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1449137725</v>
+        <v>0.1507601407</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -12389,6 +12479,9 @@
       </c>
       <c r="DE15" s="3" t="n">
         <v>11.75</v>
+      </c>
+      <c r="DF15" s="3" t="n">
+        <v>11.81</v>
       </c>
     </row>
     <row r="16">
@@ -12414,16 +12507,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.6033</v>
+        <v>25.362</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>146525.8424624</v>
+        <v>145144.899936</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>46525.8424624</v>
+        <v>45144.899936</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.465258424624</v>
+        <v>0.45144899936</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -12718,6 +12811,9 @@
       </c>
       <c r="DE16" s="3" t="n">
         <v>25.6033</v>
+      </c>
+      <c r="DF16" s="3" t="n">
+        <v>25.362</v>
       </c>
     </row>
     <row r="17">
@@ -12743,16 +12839,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>17.0425</v>
+        <v>16.9752</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>56343.4764225</v>
+        <v>56120.9787864</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>6343.476422499996</v>
+        <v>6120.978786400003</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1268695284499999</v>
+        <v>0.1224195757280001</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -13047,6 +13143,9 @@
       </c>
       <c r="DE17" s="3" t="n">
         <v>17.0425</v>
+      </c>
+      <c r="DF17" s="3" t="n">
+        <v>16.9752</v>
       </c>
     </row>
     <row r="18">
@@ -13072,16 +13171,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.22</v>
+        <v>47.48</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>89077.50791999999</v>
+        <v>89567.98127999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>9077.507919999989</v>
+        <v>9567.981279999993</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1134688489999999</v>
+        <v>0.1195997659999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -13382,6 +13481,9 @@
       </c>
       <c r="DE18" s="3" t="n">
         <v>47.22</v>
+      </c>
+      <c r="DF18" s="3" t="n">
+        <v>47.48</v>
       </c>
     </row>
     <row r="19">
@@ -13407,16 +13509,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.4049</v>
+        <v>13.4111</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>193925.5515534</v>
+        <v>194015.2455026</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>43925.5515534</v>
+        <v>44015.24550259998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.292837010356</v>
+        <v>0.2934349700173332</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -13711,6 +13813,9 @@
       </c>
       <c r="DE19" s="3" t="n">
         <v>13.4049</v>
+      </c>
+      <c r="DF19" s="3" t="n">
+        <v>13.4111</v>
       </c>
     </row>
     <row r="20">
@@ -13736,16 +13841,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10</v>
+        <v>9.98</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>262558.03</v>
+        <v>262032.91394</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>12558.03000000003</v>
+        <v>12032.91394</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.05023212000000011</v>
+        <v>0.04813165576</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -14046,6 +14151,9 @@
       </c>
       <c r="DE20" s="3" t="n">
         <v>10</v>
+      </c>
+      <c r="DF20" s="3" t="n">
+        <v>9.98</v>
       </c>
     </row>
     <row r="21">
@@ -14071,16 +14179,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>114.7061</v>
+        <v>115.6828</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>174268.2747799</v>
+        <v>175752.1350452</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>4268.274779900006</v>
+        <v>5752.135045200004</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.02510749870529416</v>
+        <v>0.0338360885011765</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -14381,6 +14489,9 @@
       </c>
       <c r="DE21" s="3" t="n">
         <v>114.7061</v>
+      </c>
+      <c r="DF21" s="3" t="n">
+        <v>115.6828</v>
       </c>
     </row>
     <row r="22">
@@ -14406,16 +14517,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.764</v>
+        <v>44.652</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68688.56744</v>
+        <v>68516.70792</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8688.567439999999</v>
+        <v>8516.707920000001</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1448094573333333</v>
+        <v>0.141945132</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -14710,6 +14821,9 @@
       </c>
       <c r="DE22" s="3" t="n">
         <v>44.764</v>
+      </c>
+      <c r="DF22" s="3" t="n">
+        <v>44.652</v>
       </c>
     </row>
     <row r="23">
@@ -14735,16 +14849,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.4874</v>
+        <v>63.9074</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>172461.4270158</v>
+        <v>173602.3431558</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>22461.4270158</v>
+        <v>23602.34315580002</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.149742846772</v>
+        <v>0.1573489543720001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -15045,6 +15159,9 @@
       </c>
       <c r="DE23" s="3" t="n">
         <v>63.4874</v>
+      </c>
+      <c r="DF23" s="3" t="n">
+        <v>63.9074</v>
       </c>
     </row>
     <row r="24">
@@ -15070,16 +15187,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>26.8557</v>
+        <v>27.1255</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>97577.12440019999</v>
+        <v>98557.411943</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-2422.875599800012</v>
+        <v>-1442.588057000001</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.02422875599800012</v>
+        <v>-0.01442588057000001</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -15374,6 +15491,9 @@
       </c>
       <c r="DE24" s="3" t="n">
         <v>26.8557</v>
+      </c>
+      <c r="DF24" s="3" t="n">
+        <v>27.1255</v>
       </c>
     </row>
     <row r="25">
@@ -15399,16 +15519,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>13.1893</v>
+        <v>13.2439</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>216590.3848882</v>
+        <v>217487.0082886</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>16590.38488819997</v>
+        <v>17487.00828859999</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.08295192444099986</v>
+        <v>0.08743504144299993</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -15706,6 +15826,9 @@
       </c>
       <c r="DE25" s="3" t="n">
         <v>13.1893</v>
+      </c>
+      <c r="DF25" s="3" t="n">
+        <v>13.2439</v>
       </c>
     </row>
     <row r="26">
@@ -15731,16 +15854,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.7355</v>
+        <v>11.7709</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>140141.9963825</v>
+        <v>140564.7330935</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>30141.99638250002</v>
+        <v>30564.73309349999</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.2740181489318183</v>
+        <v>0.277861209940909</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -16038,6 +16161,9 @@
       </c>
       <c r="DE26" s="3" t="n">
         <v>11.7355</v>
+      </c>
+      <c r="DF26" s="3" t="n">
+        <v>11.7709</v>
       </c>
     </row>
     <row r="27">
@@ -16063,16 +16189,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>70.792</v>
+        <v>71.459</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>114036.00112</v>
+        <v>115110.44474</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>4036.001120000001</v>
+        <v>5110.444739999992</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.03669091927272728</v>
+        <v>0.04645858854545447</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -16373,6 +16499,9 @@
       </c>
       <c r="DE27" s="3" t="n">
         <v>70.792</v>
+      </c>
+      <c r="DF27" s="3" t="n">
+        <v>71.459</v>
       </c>
     </row>
     <row r="28">
@@ -16398,16 +16527,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>119.7578</v>
+        <v>120.2786</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>395997.9676746</v>
+        <v>397720.0746402</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>15997.96767460002</v>
+        <v>17720.07464020001</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.04209991493315794</v>
+        <v>0.04663177536894739</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -16708,6 +16837,9 @@
       </c>
       <c r="DE28" s="3" t="n">
         <v>119.7578</v>
+      </c>
+      <c r="DF28" s="3" t="n">
+        <v>120.2786</v>
       </c>
     </row>
     <row r="29">
@@ -16733,16 +16865,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.4206</v>
+        <v>12.4073</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>119283.7534818</v>
+        <v>119156.0242319</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>19283.7534818</v>
+        <v>19156.02423189998</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.192837534818</v>
+        <v>0.1915602423189998</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -17037,6 +17169,9 @@
       </c>
       <c r="DE29" s="3" t="n">
         <v>12.4206</v>
+      </c>
+      <c r="DF29" s="3" t="n">
+        <v>12.4073</v>
       </c>
     </row>
     <row r="30">
@@ -17062,16 +17197,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.6535</v>
+        <v>17.7452</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>130562.8321635</v>
+        <v>131241.0326172</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>30562.8321635</v>
+        <v>31241.03261719999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.305628321635</v>
+        <v>0.3124103261719999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -17366,6 +17501,9 @@
       </c>
       <c r="DE30" s="3" t="n">
         <v>17.6535</v>
+      </c>
+      <c r="DF30" s="3" t="n">
+        <v>17.7452</v>
       </c>
     </row>
     <row r="31">
@@ -17391,16 +17529,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>412.6503</v>
+        <v>416.3455</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109797.991824</v>
+        <v>110781.21064</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9797.991823999997</v>
+        <v>10781.21063999999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09797991823999996</v>
+        <v>0.1078121063999999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -17698,6 +17836,9 @@
       </c>
       <c r="DE31" s="3" t="n">
         <v>412.6503</v>
+      </c>
+      <c r="DF31" s="3" t="n">
+        <v>416.3455</v>
       </c>
     </row>
     <row r="32">
@@ -17723,16 +17864,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>11.03</v>
+        <v>11.1</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>233173.7588</v>
+        <v>234653.556</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>33173.75879999998</v>
+        <v>34653.55599999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1658687939999999</v>
+        <v>0.1732677799999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -18033,6 +18174,9 @@
       </c>
       <c r="DE32" s="3" t="n">
         <v>11.03</v>
+      </c>
+      <c r="DF32" s="3" t="n">
+        <v>11.1</v>
       </c>
     </row>
     <row r="33">
@@ -18058,16 +18202,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>20.35</v>
+        <v>20.47</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>72927.07400000001</v>
+        <v>73357.11079999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>12927.07400000001</v>
+        <v>13357.11079999999</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.2154512333333335</v>
+        <v>0.2226185133333332</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -18362,6 +18506,9 @@
       </c>
       <c r="DE33" s="3" t="n">
         <v>20.35</v>
+      </c>
+      <c r="DF33" s="3" t="n">
+        <v>20.47</v>
       </c>
     </row>
     <row r="34">
@@ -18387,16 +18534,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>228.6807</v>
+        <v>227.9414</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>80388.3551517</v>
+        <v>80128.4682834</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>388.3551517000014</v>
+        <v>128.4682833999977</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.004854439396250018</v>
+        <v>0.001605853542499972</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -18694,6 +18841,9 @@
       </c>
       <c r="DE34" s="3" t="n">
         <v>228.6807</v>
+      </c>
+      <c r="DF34" s="3" t="n">
+        <v>227.9414</v>
       </c>
     </row>
     <row r="35">
@@ -18719,16 +18869,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.28</v>
+        <v>16.41</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>116164.68644</v>
+        <v>117092.29143</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>16164.68644</v>
+        <v>17092.29143</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1616468644000001</v>
+        <v>0.1709229143</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -19026,6 +19176,9 @@
       </c>
       <c r="DE35" s="3" t="n">
         <v>16.28</v>
+      </c>
+      <c r="DF35" s="3" t="n">
+        <v>16.41</v>
       </c>
     </row>
     <row r="36">
@@ -19051,16 +19204,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>392.2582</v>
+        <v>394.9941</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>182676.9972892</v>
+        <v>183951.1223346</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>32676.99728919999</v>
+        <v>33951.12233460002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.2178466485946666</v>
+        <v>0.2263408155640001</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -19358,6 +19511,9 @@
       </c>
       <c r="DE36" s="3" t="n">
         <v>392.2582</v>
+      </c>
+      <c r="DF36" s="3" t="n">
+        <v>394.9941</v>
       </c>
     </row>
     <row r="37">
@@ -19383,16 +19539,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.791</v>
+        <v>17.971</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>66945.55819900001</v>
+        <v>67622.87821900001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>16945.55819900001</v>
+        <v>17622.87821900001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.3389111639800002</v>
+        <v>0.3524575643800001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -19690,6 +19846,9 @@
       </c>
       <c r="DE37" s="3" t="n">
         <v>17.791</v>
+      </c>
+      <c r="DF37" s="3" t="n">
+        <v>17.971</v>
       </c>
     </row>
     <row r="38">
@@ -19715,16 +19874,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.1685</v>
+        <v>14.2541</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>84734.459217</v>
+        <v>85246.38847619999</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>4734.459216999996</v>
+        <v>5246.388476199994</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.05918074021249995</v>
+        <v>0.06557985595249993</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -20019,6 +20178,9 @@
       </c>
       <c r="DE38" s="3" t="n">
         <v>14.1685</v>
+      </c>
+      <c r="DF38" s="3" t="n">
+        <v>14.2541</v>
       </c>
     </row>
     <row r="39">
@@ -20044,16 +20206,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1028.4146</v>
+        <v>1028.4394</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51298.3486626</v>
+        <v>51299.5857114</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1298.348662600001</v>
+        <v>1299.585711399995</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02596697325200003</v>
+        <v>0.02599171422799991</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -20348,6 +20510,9 @@
       </c>
       <c r="DE39" s="3" t="n">
         <v>1028.4146</v>
+      </c>
+      <c r="DF39" s="3" t="n">
+        <v>1028.4394</v>
       </c>
     </row>
     <row r="40">
@@ -20373,16 +20538,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.7734</v>
+        <v>21.9209</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>109760.2972818</v>
+        <v>110503.8487643</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>9760.297281799998</v>
+        <v>10503.8487643</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.09760297281799998</v>
+        <v>0.105038487643</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -20680,6 +20845,9 @@
       </c>
       <c r="DE40" s="3" t="n">
         <v>21.7734</v>
+      </c>
+      <c r="DF40" s="3" t="n">
+        <v>21.9209</v>
       </c>
     </row>
     <row r="41">
@@ -20692,13 +20860,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5155761.0299865</v>
+        <v>5167781.2049771</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>685761.0299865</v>
+        <v>697781.2049771</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1534141006681208</v>
+        <v>0.156103177847226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-25
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-24 07:07 IST</t>
+          <t>Generated: 2026-09-25 07:05 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5167781.2049771</v>
+        <v>5100610.7657169</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>697781.2049770998</v>
+        <v>630610.7657169001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1561031778472259</v>
+        <v>0.141076233941141</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>543811.5040092468</v>
+        <v>544502.9979782104</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-46970.51599075319</v>
+        <v>-46279.02202178957</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07950566266514542</v>
+        <v>-0.07833519040032662</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5711592.708986347</v>
+        <v>5645113.763695111</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>650810.6889863471</v>
+        <v>584331.743695111</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1285988383641837</v>
+        <v>0.1154627370603706</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-24</t>
+          <t>Last snapshot: 2026-09-25</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EJ19"/>
+  <dimension ref="A1:EK19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -759,6 +759,7 @@
     <col width="21" customWidth="1" min="138" max="138"/>
     <col width="21" customWidth="1" min="139" max="139"/>
     <col width="21" customWidth="1" min="140" max="140"/>
+    <col width="21" customWidth="1" min="141" max="141"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1462,6 +1463,11 @@
           <t>2026-09-24</t>
         </is>
       </c>
+      <c r="EK1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1481,13 +1487,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>573.6500244140625</v>
+        <v>608.0999755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45892.001953125</v>
+        <v>48647.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2074.491953124998</v>
+        <v>4830.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1884,6 +1890,9 @@
       </c>
       <c r="EJ2" s="3" t="n">
         <v>573.6500244140625</v>
+      </c>
+      <c r="EK2" s="3" t="n">
+        <v>608.0999755859375</v>
       </c>
     </row>
     <row r="3">
@@ -1931,13 +1940,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1400</v>
+        <v>1391.099975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28000</v>
+        <v>27821.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4104.580000000002</v>
+        <v>-4282.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2337,6 +2346,9 @@
       </c>
       <c r="EJ4" s="3" t="n">
         <v>1400</v>
+      </c>
+      <c r="EK4" s="3" t="n">
+        <v>1391.099975585938</v>
       </c>
     </row>
     <row r="5">
@@ -2357,13 +2369,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>581.6500244140625</v>
+        <v>569.75</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11633.00048828125</v>
+        <v>11395</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-2580.09951171875</v>
+        <v>-2818.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2763,6 +2775,9 @@
       </c>
       <c r="EJ5" s="3" t="n">
         <v>581.6500244140625</v>
+      </c>
+      <c r="EK5" s="3" t="n">
+        <v>569.75</v>
       </c>
     </row>
     <row r="6">
@@ -2783,13 +2798,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>334.75</v>
+        <v>336.7999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13390</v>
+        <v>13471.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4112.240000000002</v>
+        <v>-4030.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3189,6 +3204,9 @@
       </c>
       <c r="EJ6" s="3" t="n">
         <v>334.75</v>
+      </c>
+      <c r="EK6" s="3" t="n">
+        <v>336.7999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -3209,13 +3227,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>299.6000061035156</v>
+        <v>304.2000122070312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>29960.00061035156</v>
+        <v>30420.00122070312</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>3526.180610351563</v>
+        <v>3986.181220703125</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3615,6 +3633,9 @@
       </c>
       <c r="EJ7" s="3" t="n">
         <v>299.6000061035156</v>
+      </c>
+      <c r="EK7" s="3" t="n">
+        <v>304.2000122070312</v>
       </c>
     </row>
     <row r="8">
@@ -3662,13 +3683,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.86999988555908</v>
+        <v>15.77000045776367</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23804.99982833862</v>
+        <v>23655.00068664551</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7245.170171661375</v>
+        <v>-7395.16931335449</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4068,6 +4089,9 @@
       </c>
       <c r="EJ9" s="3" t="n">
         <v>15.86999988555908</v>
+      </c>
+      <c r="EK9" s="3" t="n">
+        <v>15.77000045776367</v>
       </c>
     </row>
     <row r="10">
@@ -4088,13 +4112,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>471.5</v>
+        <v>471.75</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47150</v>
+        <v>47175</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-4348.480000000003</v>
+        <v>-4323.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4494,6 +4518,9 @@
       </c>
       <c r="EJ10" s="3" t="n">
         <v>471.5</v>
+      </c>
+      <c r="EK10" s="3" t="n">
+        <v>471.75</v>
       </c>
     </row>
     <row r="11">
@@ -4514,13 +4541,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>14.22999954223633</v>
+        <v>14.30000019073486</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14229.99954223633</v>
+        <v>14300.00019073486</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4388.789542236329</v>
+        <v>4458.790190734864</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4920,6 +4947,9 @@
       </c>
       <c r="EJ11" s="3" t="n">
         <v>14.22999954223633</v>
+      </c>
+      <c r="EK11" s="3" t="n">
+        <v>14.30000019073486</v>
       </c>
     </row>
     <row r="12">
@@ -4940,13 +4970,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2822.10009765625</v>
+        <v>2781</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>28221.0009765625</v>
+        <v>27810</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>497.7509765625</v>
+        <v>86.75</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5346,6 +5376,9 @@
       </c>
       <c r="EJ12" s="3" t="n">
         <v>2822.10009765625</v>
+      </c>
+      <c r="EK12" s="3" t="n">
+        <v>2781</v>
       </c>
     </row>
     <row r="13">
@@ -5366,13 +5399,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>41</v>
+        <v>40.22999954223633</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>24600</v>
+        <v>24137.9997253418</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-10431.76</v>
+        <v>-10893.76027465821</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5772,6 +5805,9 @@
       </c>
       <c r="EJ13" s="3" t="n">
         <v>41</v>
+      </c>
+      <c r="EK13" s="3" t="n">
+        <v>40.22999954223633</v>
       </c>
     </row>
     <row r="14">
@@ -5792,13 +5828,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>662</v>
+        <v>640.0999755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>33100</v>
+        <v>32004.99877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-9362.510000000002</v>
+        <v>-10457.51122070313</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6198,6 +6234,9 @@
       </c>
       <c r="EJ14" s="3" t="n">
         <v>662</v>
+      </c>
+      <c r="EK14" s="3" t="n">
+        <v>640.0999755859375</v>
       </c>
     </row>
     <row r="15">
@@ -6272,13 +6311,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>510</v>
+        <v>505.8500061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25500</v>
+        <v>25292.50030517578</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>3745.470000000001</v>
+        <v>3537.970305175782</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6678,6 +6717,9 @@
       </c>
       <c r="EJ17" s="3" t="n">
         <v>510</v>
+      </c>
+      <c r="EK17" s="3" t="n">
+        <v>505.8500061035156</v>
       </c>
     </row>
     <row r="18">
@@ -6698,13 +6740,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>365.6000061035156</v>
+        <v>366</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36560.00061035156</v>
+        <v>36600</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-10080.81938964844</v>
+        <v>-10040.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7104,6 +7146,9 @@
       </c>
       <c r="EJ18" s="3" t="n">
         <v>365.6000061035156</v>
+      </c>
+      <c r="EK18" s="3" t="n">
+        <v>366</v>
       </c>
     </row>
     <row r="19">
@@ -7116,10 +7161,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>543811.5040092468</v>
+        <v>544502.9979782104</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-46970.51599075319</v>
+        <v>-46279.02202178956</v>
       </c>
     </row>
   </sheetData>
@@ -7133,7 +7178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DF41"/>
+  <dimension ref="A1:DG41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7246,6 +7291,7 @@
     <col width="13" customWidth="1" min="108" max="108"/>
     <col width="13" customWidth="1" min="109" max="109"/>
     <col width="13" customWidth="1" min="110" max="110"/>
+    <col width="13" customWidth="1" min="111" max="111"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7799,6 +7845,11 @@
           <t>2026-09-24</t>
         </is>
       </c>
+      <c r="DG1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7823,16 +7874,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.6847</v>
+        <v>57.7341</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64750.0374254</v>
+        <v>64805.4880362</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14750.0374254</v>
+        <v>14805.4880362</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.295000748508</v>
+        <v>0.2961097607239999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8136,6 +8187,9 @@
       </c>
       <c r="DF2" s="3" t="n">
         <v>57.6847</v>
+      </c>
+      <c r="DG2" s="3" t="n">
+        <v>57.7341</v>
       </c>
     </row>
     <row r="3">
@@ -8161,16 +8215,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.7849</v>
+        <v>26.5259</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65762.6346837</v>
+        <v>65126.7345167</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5762.634683700002</v>
+        <v>5126.734516700002</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09604391139500003</v>
+        <v>0.08544557527833337</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8468,6 +8522,9 @@
       </c>
       <c r="DF3" s="3" t="n">
         <v>26.7849</v>
+      </c>
+      <c r="DG3" s="3" t="n">
+        <v>26.5259</v>
       </c>
     </row>
     <row r="4">
@@ -8493,16 +8550,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.92</v>
+        <v>12.83</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>248142.72156</v>
+        <v>246414.17319</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>68142.72156000001</v>
+        <v>66414.17319</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3785706753333334</v>
+        <v>0.3689676288333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -8800,6 +8857,9 @@
       </c>
       <c r="DF4" s="3" t="n">
         <v>12.92</v>
+      </c>
+      <c r="DG4" s="3" t="n">
+        <v>12.83</v>
       </c>
     </row>
     <row r="5">
@@ -8825,16 +8885,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.3133</v>
+        <v>9.2141</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>170937.1277704</v>
+        <v>169116.4022408</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-39062.87222960001</v>
+        <v>-40883.5977592</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1860136772838095</v>
+        <v>-0.1946837988533333</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9132,6 +9192,9 @@
       </c>
       <c r="DF5" s="3" t="n">
         <v>9.3133</v>
+      </c>
+      <c r="DG5" s="3" t="n">
+        <v>9.2141</v>
       </c>
     </row>
     <row r="6">
@@ -9157,16 +9220,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.6984</v>
+        <v>11.5738</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>49472.26453679999</v>
+        <v>48945.3340026</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-527.7354632000061</v>
+        <v>-1054.665997399999</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.01055470926400012</v>
+        <v>-0.02109331994799999</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9470,6 +9533,9 @@
       </c>
       <c r="DF6" s="3" t="n">
         <v>11.6984</v>
+      </c>
+      <c r="DG6" s="3" t="n">
+        <v>11.5738</v>
       </c>
     </row>
     <row r="7">
@@ -9495,16 +9561,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.4836</v>
+        <v>34.3524</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>76072.20094400001</v>
+        <v>75782.768496</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>16072.20094400001</v>
+        <v>15782.768496</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2678700157333335</v>
+        <v>0.2630461416000001</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -9802,6 +9868,9 @@
       </c>
       <c r="DF7" s="3" t="n">
         <v>34.4836</v>
+      </c>
+      <c r="DG7" s="3" t="n">
+        <v>34.3524</v>
       </c>
     </row>
     <row r="8">
@@ -9827,16 +9896,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>36.3955</v>
+        <v>35.77</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>58399.9645315</v>
+        <v>57396.29161000001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>8399.964531500002</v>
+        <v>7396.291610000007</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.16799929063</v>
+        <v>0.1479258322000002</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -10140,6 +10209,9 @@
       </c>
       <c r="DF8" s="3" t="n">
         <v>36.3955</v>
+      </c>
+      <c r="DG8" s="3" t="n">
+        <v>35.77</v>
       </c>
     </row>
     <row r="9">
@@ -10165,16 +10237,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.3429</v>
+        <v>42.0279</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>136318.4358597</v>
+        <v>135304.3270647</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>36318.4358597</v>
+        <v>35304.32706470002</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3631843585969999</v>
+        <v>0.3530432706470002</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10472,6 +10544,9 @@
       </c>
       <c r="DF9" s="3" t="n">
         <v>42.3429</v>
+      </c>
+      <c r="DG9" s="3" t="n">
+        <v>42.0279</v>
       </c>
     </row>
     <row r="10">
@@ -10497,16 +10572,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.6196</v>
+        <v>48.5491</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138403.4219164</v>
+        <v>138202.7324569</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38403.4219164</v>
+        <v>38202.7324569</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3840342191639999</v>
+        <v>0.3820273245690001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -10804,6 +10879,9 @@
       </c>
       <c r="DF10" s="3" t="n">
         <v>48.6196</v>
+      </c>
+      <c r="DG10" s="3" t="n">
+        <v>48.5491</v>
       </c>
     </row>
     <row r="11">
@@ -10829,16 +10907,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>106.9125</v>
+        <v>107.4933</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32172.0025875</v>
+        <v>32346.7763427</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2172.002587499996</v>
+        <v>2346.776342699999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07240008624999986</v>
+        <v>0.07822587808999996</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -11136,6 +11214,9 @@
       </c>
       <c r="DF11" s="3" t="n">
         <v>106.9125</v>
+      </c>
+      <c r="DG11" s="3" t="n">
+        <v>107.4933</v>
       </c>
     </row>
     <row r="12">
@@ -11161,16 +11242,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>231.07</v>
+        <v>226.836</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>107568.16854</v>
+        <v>105597.148392</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>7568.168539999999</v>
+        <v>5597.148392000003</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.07568168539999999</v>
+        <v>0.05597148392000003</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -11474,6 +11555,9 @@
       </c>
       <c r="DF12" s="3" t="n">
         <v>231.07</v>
+      </c>
+      <c r="DG12" s="3" t="n">
+        <v>226.836</v>
       </c>
     </row>
     <row r="13">
@@ -11499,16 +11583,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22.873</v>
+        <v>22.702</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>265043.289165</v>
+        <v>263061.80871</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>65043.28916500002</v>
+        <v>63061.80871000001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.3252164458250001</v>
+        <v>0.3153090435500001</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -11812,6 +11896,9 @@
       </c>
       <c r="DF13" s="3" t="n">
         <v>22.873</v>
+      </c>
+      <c r="DG13" s="3" t="n">
+        <v>22.702</v>
       </c>
     </row>
     <row r="14">
@@ -11837,16 +11924,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.9279</v>
+        <v>38.5918</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>140436.5256074</v>
+        <v>139224.0092308</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>40436.52560740002</v>
+        <v>39224.0092308</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4043652560740002</v>
+        <v>0.392240092308</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -12144,6 +12231,9 @@
       </c>
       <c r="DF14" s="3" t="n">
         <v>38.9279</v>
+      </c>
+      <c r="DG14" s="3" t="n">
+        <v>38.5918</v>
       </c>
     </row>
     <row r="15">
@@ -12169,16 +12259,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.81</v>
+        <v>11.69</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>115076.01407</v>
+        <v>113906.74043</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>15076.01407</v>
+        <v>13906.74042999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1507601407</v>
+        <v>0.1390674042999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -12482,6 +12572,9 @@
       </c>
       <c r="DF15" s="3" t="n">
         <v>11.81</v>
+      </c>
+      <c r="DG15" s="3" t="n">
+        <v>11.69</v>
       </c>
     </row>
     <row r="16">
@@ -12507,16 +12600,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.362</v>
+        <v>25.4163</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>145144.899936</v>
+        <v>145455.6549264</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>45144.899936</v>
+        <v>45455.65492639999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.45144899936</v>
+        <v>0.4545565492639999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -12814,6 +12907,9 @@
       </c>
       <c r="DF16" s="3" t="n">
         <v>25.362</v>
+      </c>
+      <c r="DG16" s="3" t="n">
+        <v>25.4163</v>
       </c>
     </row>
     <row r="17">
@@ -12839,16 +12935,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.9752</v>
+        <v>16.8585</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>56120.9787864</v>
+        <v>55735.16193449999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>6120.978786400003</v>
+        <v>5735.161934499993</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1224195757280001</v>
+        <v>0.1147032386899998</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -13146,6 +13242,9 @@
       </c>
       <c r="DF17" s="3" t="n">
         <v>16.9752</v>
+      </c>
+      <c r="DG17" s="3" t="n">
+        <v>16.8585</v>
       </c>
     </row>
     <row r="18">
@@ -13171,16 +13270,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.48</v>
+        <v>47.17</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>89567.98127999999</v>
+        <v>88983.18612</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>9567.981279999993</v>
+        <v>8983.186119999998</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1195997659999999</v>
+        <v>0.1122898265</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -13484,6 +13583,9 @@
       </c>
       <c r="DF18" s="3" t="n">
         <v>47.48</v>
+      </c>
+      <c r="DG18" s="3" t="n">
+        <v>47.17</v>
       </c>
     </row>
     <row r="19">
@@ -13509,16 +13611,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.4111</v>
+        <v>13.027</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>194015.2455026</v>
+        <v>188458.560682</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>44015.24550259998</v>
+        <v>38458.56068199998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2934349700173332</v>
+        <v>0.2563904045466666</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -13816,6 +13918,9 @@
       </c>
       <c r="DF19" s="3" t="n">
         <v>13.4111</v>
+      </c>
+      <c r="DG19" s="3" t="n">
+        <v>13.027</v>
       </c>
     </row>
     <row r="20">
@@ -13841,16 +13946,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.98</v>
+        <v>9.81</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>262032.91394</v>
+        <v>257569.42743</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>12032.91394</v>
+        <v>7569.427430000011</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.04813165576</v>
+        <v>0.03027770972000004</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -14154,6 +14259,9 @@
       </c>
       <c r="DF20" s="3" t="n">
         <v>9.98</v>
+      </c>
+      <c r="DG20" s="3" t="n">
+        <v>9.81</v>
       </c>
     </row>
     <row r="21">
@@ -14179,16 +14287,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>115.6828</v>
+        <v>113.9381</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>175752.1350452</v>
+        <v>173101.4838679</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>5752.135045200004</v>
+        <v>3101.483867900009</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.0338360885011765</v>
+        <v>0.018244022752353</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -14492,6 +14600,9 @@
       </c>
       <c r="DF21" s="3" t="n">
         <v>115.6828</v>
+      </c>
+      <c r="DG21" s="3" t="n">
+        <v>113.9381</v>
       </c>
     </row>
     <row r="22">
@@ -14517,16 +14628,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.652</v>
+        <v>44.244</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68516.70792</v>
+        <v>67890.64823999999</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8516.707920000001</v>
+        <v>7890.648239999995</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.141945132</v>
+        <v>0.1315108039999999</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -14824,6 +14935,9 @@
       </c>
       <c r="DF22" s="3" t="n">
         <v>44.652</v>
+      </c>
+      <c r="DG22" s="3" t="n">
+        <v>44.244</v>
       </c>
     </row>
     <row r="23">
@@ -14849,16 +14963,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.9074</v>
+        <v>63.3089</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>173602.3431558</v>
+        <v>171976.5376563</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>23602.34315580002</v>
+        <v>21976.5376563</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1573489543720001</v>
+        <v>0.146510251042</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -15162,6 +15276,9 @@
       </c>
       <c r="DF23" s="3" t="n">
         <v>63.9074</v>
+      </c>
+      <c r="DG23" s="3" t="n">
+        <v>63.3089</v>
       </c>
     </row>
     <row r="24">
@@ -15187,16 +15304,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.1255</v>
+        <v>26.847</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>98557.411943</v>
+        <v>97545.51394200001</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-1442.588057000001</v>
+        <v>-2454.486057999995</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.01442588057000001</v>
+        <v>-0.02454486057999995</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -15494,6 +15611,9 @@
       </c>
       <c r="DF24" s="3" t="n">
         <v>27.1255</v>
+      </c>
+      <c r="DG24" s="3" t="n">
+        <v>26.847</v>
       </c>
     </row>
     <row r="25">
@@ -15519,16 +15639,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>13.2439</v>
+        <v>13.0166</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>217487.0082886</v>
+        <v>213754.3617884</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>17487.00828859999</v>
+        <v>13754.36178839998</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.08743504144299993</v>
+        <v>0.06877180894199991</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -15829,6 +15949,9 @@
       </c>
       <c r="DF25" s="3" t="n">
         <v>13.2439</v>
+      </c>
+      <c r="DG25" s="3" t="n">
+        <v>13.0166</v>
       </c>
     </row>
     <row r="26">
@@ -15854,16 +15977,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.7709</v>
+        <v>11.4086</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>140564.7330935</v>
+        <v>136238.249749</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>30564.73309349999</v>
+        <v>26238.24974900001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.277861209940909</v>
+        <v>0.2385295431727274</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -16164,6 +16287,9 @@
       </c>
       <c r="DF26" s="3" t="n">
         <v>11.7709</v>
+      </c>
+      <c r="DG26" s="3" t="n">
+        <v>11.4086</v>
       </c>
     </row>
     <row r="27">
@@ -16189,16 +16315,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>71.459</v>
+        <v>70.4213</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>115110.44474</v>
+        <v>113438.855318</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>5110.444739999992</v>
+        <v>3438.855318000002</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.04645858854545447</v>
+        <v>0.03126232107272729</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -16502,6 +16628,9 @@
       </c>
       <c r="DF27" s="3" t="n">
         <v>71.459</v>
+      </c>
+      <c r="DG27" s="3" t="n">
+        <v>70.4213</v>
       </c>
     </row>
     <row r="28">
@@ -16527,16 +16656,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>120.2786</v>
+        <v>116.9959</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>397720.0746402</v>
+        <v>386865.3117063</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>17720.07464020001</v>
+        <v>6865.31170630001</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.04663177536894739</v>
+        <v>0.01806660975342108</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -16840,6 +16969,9 @@
       </c>
       <c r="DF28" s="3" t="n">
         <v>120.2786</v>
+      </c>
+      <c r="DG28" s="3" t="n">
+        <v>116.9959</v>
       </c>
     </row>
     <row r="29">
@@ -16865,16 +16997,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.4073</v>
+        <v>12.2766</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>119156.0242319</v>
+        <v>117900.8202498</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>19156.02423189998</v>
+        <v>17900.8202498</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1915602423189998</v>
+        <v>0.179008202498</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -17172,6 +17304,9 @@
       </c>
       <c r="DF29" s="3" t="n">
         <v>12.4073</v>
+      </c>
+      <c r="DG29" s="3" t="n">
+        <v>12.2766</v>
       </c>
     </row>
     <row r="30">
@@ -17197,16 +17332,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.7452</v>
+        <v>17.565</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>131241.0326172</v>
+        <v>129908.298465</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>31241.03261719999</v>
+        <v>29908.29846500001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.3124103261719999</v>
+        <v>0.2990829846500002</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -17504,6 +17639,9 @@
       </c>
       <c r="DF30" s="3" t="n">
         <v>17.7452</v>
+      </c>
+      <c r="DG30" s="3" t="n">
+        <v>17.565</v>
       </c>
     </row>
     <row r="31">
@@ -17529,16 +17667,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>416.3455</v>
+        <v>410.8551</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>110781.21064</v>
+        <v>109320.325008</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>10781.21063999999</v>
+        <v>9320.325007999985</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1078121063999999</v>
+        <v>0.09320325007999986</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -17839,6 +17977,9 @@
       </c>
       <c r="DF31" s="3" t="n">
         <v>416.3455</v>
+      </c>
+      <c r="DG31" s="3" t="n">
+        <v>410.8551</v>
       </c>
     </row>
     <row r="32">
@@ -17864,16 +18005,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>11.1</v>
+        <v>10.98</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>234653.556</v>
+        <v>232116.7608</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>34653.55599999998</v>
+        <v>32116.76079999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1732677799999999</v>
+        <v>0.1605838039999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -18177,6 +18318,9 @@
       </c>
       <c r="DF32" s="3" t="n">
         <v>11.1</v>
+      </c>
+      <c r="DG32" s="3" t="n">
+        <v>10.98</v>
       </c>
     </row>
     <row r="33">
@@ -18202,16 +18346,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>20.47</v>
+        <v>20.21</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>73357.11079999999</v>
+        <v>72425.36440000001</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>13357.11079999999</v>
+        <v>12425.36440000001</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.2226185133333332</v>
+        <v>0.2070894066666668</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -18509,6 +18653,9 @@
       </c>
       <c r="DF33" s="3" t="n">
         <v>20.47</v>
+      </c>
+      <c r="DG33" s="3" t="n">
+        <v>20.21</v>
       </c>
     </row>
     <row r="34">
@@ -18534,16 +18681,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>227.9414</v>
+        <v>222.7199</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>80128.4682834</v>
-      </c>
-      <c r="H34" s="4" t="n">
-        <v>128.4682833999977</v>
-      </c>
-      <c r="I34" s="12" t="n">
-        <v>0.001605853542499972</v>
+        <v>78292.9491669</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>-1707.050833100002</v>
+      </c>
+      <c r="I34" s="13" t="n">
+        <v>-0.02133813541375002</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -18844,6 +18991,9 @@
       </c>
       <c r="DF34" s="3" t="n">
         <v>227.9414</v>
+      </c>
+      <c r="DG34" s="3" t="n">
+        <v>222.7199</v>
       </c>
     </row>
     <row r="35">
@@ -18869,16 +19019,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.41</v>
+        <v>16.08</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>117092.29143</v>
+        <v>114737.60184</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>17092.29143</v>
+        <v>14737.60183999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1709229143</v>
+        <v>0.1473760183999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -19179,6 +19329,9 @@
       </c>
       <c r="DF35" s="3" t="n">
         <v>16.41</v>
+      </c>
+      <c r="DG35" s="3" t="n">
+        <v>16.08</v>
       </c>
     </row>
     <row r="36">
@@ -19204,16 +19357,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>394.9941</v>
+        <v>392.6752</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>183951.1223346</v>
+        <v>182871.1966912</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>33951.12233460002</v>
+        <v>32871.19669120002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.2263408155640001</v>
+        <v>0.2191413112746668</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -19514,6 +19667,9 @@
       </c>
       <c r="DF36" s="3" t="n">
         <v>394.9941</v>
+      </c>
+      <c r="DG36" s="3" t="n">
+        <v>392.6752</v>
       </c>
     </row>
     <row r="37">
@@ -19539,16 +19695,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.971</v>
+        <v>17.835</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>67622.87821900001</v>
+        <v>67111.12531500001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>17622.87821900001</v>
+        <v>17111.12531500001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.3524575643800001</v>
+        <v>0.3422225063000002</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -19849,6 +20005,9 @@
       </c>
       <c r="DF37" s="3" t="n">
         <v>17.971</v>
+      </c>
+      <c r="DG37" s="3" t="n">
+        <v>17.835</v>
       </c>
     </row>
     <row r="38">
@@ -19874,16 +20033,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2541</v>
+        <v>13.9965</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85246.38847619999</v>
+        <v>83705.81631299999</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5246.388476199994</v>
+        <v>3705.816312999988</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06557985595249993</v>
+        <v>0.04632270391249985</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -20181,6 +20340,9 @@
       </c>
       <c r="DF38" s="3" t="n">
         <v>14.2541</v>
+      </c>
+      <c r="DG38" s="3" t="n">
+        <v>13.9965</v>
       </c>
     </row>
     <row r="39">
@@ -20206,16 +20368,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1028.4394</v>
+        <v>1027.4945</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51299.5857114</v>
+        <v>51252.4531545</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1299.585711399995</v>
+        <v>1252.453154499999</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02599171422799991</v>
+        <v>0.02504906308999998</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -20513,6 +20675,9 @@
       </c>
       <c r="DF39" s="3" t="n">
         <v>1028.4394</v>
+      </c>
+      <c r="DG39" s="3" t="n">
+        <v>1027.4945</v>
       </c>
     </row>
     <row r="40">
@@ -20538,16 +20703,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.9209</v>
+        <v>21.5679</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>110503.8487643</v>
+        <v>108724.3662333</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>10503.8487643</v>
+        <v>8724.36623330001</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.105038487643</v>
+        <v>0.0872436623330001</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -20848,6 +21013,9 @@
       </c>
       <c r="DF40" s="3" t="n">
         <v>21.9209</v>
+      </c>
+      <c r="DG40" s="3" t="n">
+        <v>21.5679</v>
       </c>
     </row>
     <row r="41">
@@ -20860,13 +21028,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5167781.2049771</v>
+        <v>5100610.7657169</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>697781.2049771</v>
+        <v>630610.7657169</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.156103177847226</v>
+        <v>0.1410762339411409</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-26
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-25 07:05 IST</t>
+          <t>Generated: 2026-09-26 07:02 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5100610.7657169</v>
+        <v>5104310.4877042</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>630610.7657169001</v>
+        <v>634310.4877041997</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.141076233941141</v>
+        <v>0.141903912238076</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>544502.9979782104</v>
+        <v>546777.4988441467</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-46279.02202178957</v>
+        <v>-44004.52115585329</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07833519040032662</v>
+        <v>-0.07448520717650359</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5645113.763695111</v>
+        <v>5651087.986548346</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>584331.743695111</v>
+        <v>590305.9665483469</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1154627370603706</v>
+        <v>0.1166432310689301</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-25</t>
+          <t>Last snapshot: 2026-09-26</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EK19"/>
+  <dimension ref="A1:EL19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -760,6 +760,7 @@
     <col width="21" customWidth="1" min="139" max="139"/>
     <col width="21" customWidth="1" min="140" max="140"/>
     <col width="21" customWidth="1" min="141" max="141"/>
+    <col width="21" customWidth="1" min="142" max="142"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1468,6 +1469,11 @@
           <t>2026-09-25</t>
         </is>
       </c>
+      <c r="EL1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1487,13 +1493,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>608.0999755859375</v>
+        <v>607.75</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>48647.998046875</v>
+        <v>48620</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4830.488046874998</v>
+        <v>4802.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1893,6 +1899,9 @@
       </c>
       <c r="EK2" s="3" t="n">
         <v>608.0999755859375</v>
+      </c>
+      <c r="EL2" s="3" t="n">
+        <v>607.75</v>
       </c>
     </row>
     <row r="3">
@@ -1940,13 +1949,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1391.099975585938</v>
+        <v>1399</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27821.99951171875</v>
+        <v>27980</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4282.580488281252</v>
+        <v>-4124.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2349,6 +2358,9 @@
       </c>
       <c r="EK4" s="3" t="n">
         <v>1391.099975585938</v>
+      </c>
+      <c r="EL4" s="3" t="n">
+        <v>1399</v>
       </c>
     </row>
     <row r="5">
@@ -2369,13 +2381,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>569.75</v>
+        <v>573.9500122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11395</v>
+        <v>11479.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-2818.1</v>
+        <v>-2734.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2778,6 +2790,9 @@
       </c>
       <c r="EK5" s="3" t="n">
         <v>569.75</v>
+      </c>
+      <c r="EL5" s="3" t="n">
+        <v>573.9500122070312</v>
       </c>
     </row>
     <row r="6">
@@ -2798,13 +2813,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>336.7999877929688</v>
+        <v>338.5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13471.99951171875</v>
+        <v>13540</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4030.240488281252</v>
+        <v>-3962.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3207,6 +3222,9 @@
       </c>
       <c r="EK6" s="3" t="n">
         <v>336.7999877929688</v>
+      </c>
+      <c r="EL6" s="3" t="n">
+        <v>338.5</v>
       </c>
     </row>
     <row r="7">
@@ -3227,13 +3245,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>304.2000122070312</v>
+        <v>315.6499938964844</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>30420.00122070312</v>
+        <v>31564.99938964844</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>3986.181220703125</v>
+        <v>5131.179389648438</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3636,6 +3654,9 @@
       </c>
       <c r="EK7" s="3" t="n">
         <v>304.2000122070312</v>
+      </c>
+      <c r="EL7" s="3" t="n">
+        <v>315.6499938964844</v>
       </c>
     </row>
     <row r="8">
@@ -3683,13 +3704,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.77000045776367</v>
+        <v>15.86999988555908</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23655.00068664551</v>
+        <v>23804.99982833862</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7395.16931335449</v>
+        <v>-7245.170171661375</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4092,6 +4113,9 @@
       </c>
       <c r="EK9" s="3" t="n">
         <v>15.77000045776367</v>
+      </c>
+      <c r="EL9" s="3" t="n">
+        <v>15.86999988555908</v>
       </c>
     </row>
     <row r="10">
@@ -4112,13 +4136,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>471.75</v>
+        <v>475.1499938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47175</v>
+        <v>47514.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-4323.480000000003</v>
+        <v>-3983.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4521,6 +4545,9 @@
       </c>
       <c r="EK10" s="3" t="n">
         <v>471.75</v>
+      </c>
+      <c r="EL10" s="3" t="n">
+        <v>475.1499938964844</v>
       </c>
     </row>
     <row r="11">
@@ -4541,13 +4568,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>14.30000019073486</v>
+        <v>14.10999965667725</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14300.00019073486</v>
+        <v>14109.99965667725</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4458.790190734864</v>
+        <v>4268.789656677247</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -4950,6 +4977,9 @@
       </c>
       <c r="EK11" s="3" t="n">
         <v>14.30000019073486</v>
+      </c>
+      <c r="EL11" s="3" t="n">
+        <v>14.10999965667725</v>
       </c>
     </row>
     <row r="12">
@@ -4970,13 +5000,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2781</v>
+        <v>2778.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27810</v>
+        <v>27783.00048828125</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>86.75</v>
+        <v>59.75048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5379,6 +5409,9 @@
       </c>
       <c r="EK12" s="3" t="n">
         <v>2781</v>
+      </c>
+      <c r="EL12" s="3" t="n">
+        <v>2778.300048828125</v>
       </c>
     </row>
     <row r="13">
@@ -5399,13 +5432,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>40.22999954223633</v>
+        <v>40.79999923706055</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>24137.9997253418</v>
+        <v>24479.99954223633</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-10893.76027465821</v>
+        <v>-10551.76045776367</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5808,6 +5841,9 @@
       </c>
       <c r="EK13" s="3" t="n">
         <v>40.22999954223633</v>
+      </c>
+      <c r="EL13" s="3" t="n">
+        <v>40.79999923706055</v>
       </c>
     </row>
     <row r="14">
@@ -5828,13 +5864,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>640.0999755859375</v>
+        <v>643.75</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>32004.99877929688</v>
+        <v>32187.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-10457.51122070313</v>
+        <v>-10275.01</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6237,6 +6273,9 @@
       </c>
       <c r="EK14" s="3" t="n">
         <v>640.0999755859375</v>
+      </c>
+      <c r="EL14" s="3" t="n">
+        <v>643.75</v>
       </c>
     </row>
     <row r="15">
@@ -6311,13 +6350,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>505.8500061035156</v>
+        <v>503.8500061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25292.50030517578</v>
+        <v>25192.50030517578</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>3537.970305175782</v>
+        <v>3437.970305175782</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6720,6 +6759,9 @@
       </c>
       <c r="EK17" s="3" t="n">
         <v>505.8500061035156</v>
+      </c>
+      <c r="EL17" s="3" t="n">
+        <v>503.8500061035156</v>
       </c>
     </row>
     <row r="18">
@@ -6740,13 +6782,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>366</v>
+        <v>367.5</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36600</v>
+        <v>36750</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-10040.82</v>
+        <v>-9890.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7149,6 +7191,9 @@
       </c>
       <c r="EK18" s="3" t="n">
         <v>366</v>
+      </c>
+      <c r="EL18" s="3" t="n">
+        <v>367.5</v>
       </c>
     </row>
     <row r="19">
@@ -7161,10 +7206,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>544502.9979782104</v>
+        <v>546777.4988441467</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-46279.02202178956</v>
+        <v>-44004.52115585328</v>
       </c>
     </row>
   </sheetData>
@@ -7178,7 +7223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DG41"/>
+  <dimension ref="A1:DH41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7292,6 +7337,7 @@
     <col width="13" customWidth="1" min="109" max="109"/>
     <col width="13" customWidth="1" min="110" max="110"/>
     <col width="13" customWidth="1" min="111" max="111"/>
+    <col width="13" customWidth="1" min="112" max="112"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7850,6 +7896,11 @@
           <t>2026-09-25</t>
         </is>
       </c>
+      <c r="DH1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7874,16 +7925,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.7341</v>
+        <v>57.9132</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64805.4880362</v>
+        <v>65006.5245624</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14805.4880362</v>
+        <v>15006.5245624</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2961097607239999</v>
+        <v>0.300130491248</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8190,6 +8241,9 @@
       </c>
       <c r="DG2" s="3" t="n">
         <v>57.7341</v>
+      </c>
+      <c r="DH2" s="3" t="n">
+        <v>57.9132</v>
       </c>
     </row>
     <row r="3">
@@ -8215,16 +8269,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.5259</v>
+        <v>26.7854</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65126.7345167</v>
+        <v>65763.86229020001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5126.734516700002</v>
+        <v>5763.862290200006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.08544557527833337</v>
+        <v>0.09606437150333344</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8525,6 +8579,9 @@
       </c>
       <c r="DG3" s="3" t="n">
         <v>26.5259</v>
+      </c>
+      <c r="DH3" s="3" t="n">
+        <v>26.7854</v>
       </c>
     </row>
     <row r="4">
@@ -8550,16 +8607,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.83</v>
+        <v>12.85</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>246414.17319</v>
+        <v>246798.29505</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>66414.17319</v>
+        <v>66798.29505000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3689676288333333</v>
+        <v>0.3711016391666668</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -8860,6 +8917,9 @@
       </c>
       <c r="DG4" s="3" t="n">
         <v>12.83</v>
+      </c>
+      <c r="DH4" s="3" t="n">
+        <v>12.85</v>
       </c>
     </row>
     <row r="5">
@@ -8885,16 +8945,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.2141</v>
+        <v>9.253299999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>169116.4022408</v>
+        <v>169835.8824904</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-40883.5977592</v>
+        <v>-40164.11750960001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1946837988533333</v>
+        <v>-0.1912577024266667</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9195,6 +9255,9 @@
       </c>
       <c r="DG5" s="3" t="n">
         <v>9.2141</v>
+      </c>
+      <c r="DH5" s="3" t="n">
+        <v>9.253299999999999</v>
       </c>
     </row>
     <row r="6">
@@ -9220,16 +9283,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.5738</v>
+        <v>11.5949</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>48945.3340026</v>
+        <v>49034.5654173</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-1054.665997399999</v>
+        <v>-965.4345826999997</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.02109331994799999</v>
+        <v>-0.019308691654</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9536,6 +9599,9 @@
       </c>
       <c r="DG6" s="3" t="n">
         <v>11.5738</v>
+      </c>
+      <c r="DH6" s="3" t="n">
+        <v>11.5949</v>
       </c>
     </row>
     <row r="7">
@@ -9561,16 +9627,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.3524</v>
+        <v>34.4256</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75782.768496</v>
+        <v>75944.25062400001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15782.768496</v>
+        <v>15944.25062400001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2630461416000001</v>
+        <v>0.2657375104000001</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -9871,6 +9937,9 @@
       </c>
       <c r="DG7" s="3" t="n">
         <v>34.3524</v>
+      </c>
+      <c r="DH7" s="3" t="n">
+        <v>34.4256</v>
       </c>
     </row>
     <row r="8">
@@ -9896,16 +9965,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.77</v>
+        <v>35.6635</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57396.29161000001</v>
+        <v>57225.4024555</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7396.291610000007</v>
+        <v>7225.4024555</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1479258322000002</v>
+        <v>0.14450804911</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -10212,6 +10281,9 @@
       </c>
       <c r="DG8" s="3" t="n">
         <v>35.77</v>
+      </c>
+      <c r="DH8" s="3" t="n">
+        <v>35.6635</v>
       </c>
     </row>
     <row r="9">
@@ -10237,16 +10309,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.0279</v>
+        <v>42.5002</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>135304.3270647</v>
+        <v>136824.8463786</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>35304.32706470002</v>
+        <v>36824.84637859999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3530432706470002</v>
+        <v>0.3682484637859999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10547,6 +10619,9 @@
       </c>
       <c r="DG9" s="3" t="n">
         <v>42.0279</v>
+      </c>
+      <c r="DH9" s="3" t="n">
+        <v>42.5002</v>
       </c>
     </row>
     <row r="10">
@@ -10572,16 +10647,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.5491</v>
+        <v>48.5874</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138202.7324569</v>
+        <v>138311.7594966</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38202.7324569</v>
+        <v>38311.75949660002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3820273245690001</v>
+        <v>0.3831175949660002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -10882,6 +10957,9 @@
       </c>
       <c r="DG10" s="3" t="n">
         <v>48.5491</v>
+      </c>
+      <c r="DH10" s="3" t="n">
+        <v>48.5874</v>
       </c>
     </row>
     <row r="11">
@@ -10907,16 +10985,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.4933</v>
+        <v>107.8591</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32346.7763427</v>
+        <v>32456.8525129</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2346.776342699999</v>
+        <v>2456.852512899997</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07822587808999996</v>
+        <v>0.08189508376333324</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -11217,6 +11295,9 @@
       </c>
       <c r="DG11" s="3" t="n">
         <v>107.4933</v>
+      </c>
+      <c r="DH11" s="3" t="n">
+        <v>107.8591</v>
       </c>
     </row>
     <row r="12">
@@ -11242,16 +11323,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>226.836</v>
+        <v>226.38</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105597.148392</v>
+        <v>105384.87036</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5597.148392000003</v>
+        <v>5384.870360000001</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05597148392000003</v>
+        <v>0.05384870360000001</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -11558,6 +11639,9 @@
       </c>
       <c r="DG12" s="3" t="n">
         <v>226.836</v>
+      </c>
+      <c r="DH12" s="3" t="n">
+        <v>226.38</v>
       </c>
     </row>
     <row r="13">
@@ -11583,16 +11667,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22.702</v>
+        <v>22.61</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>263061.80871</v>
+        <v>261995.74905</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>63061.80871000001</v>
+        <v>61995.74904999998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.3153090435500001</v>
+        <v>0.3099787452499999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -11899,6 +11983,9 @@
       </c>
       <c r="DG13" s="3" t="n">
         <v>22.702</v>
+      </c>
+      <c r="DH13" s="3" t="n">
+        <v>22.61</v>
       </c>
     </row>
     <row r="14">
@@ -11924,16 +12011,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.5918</v>
+        <v>38.566</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>139224.0092308</v>
+        <v>139130.932996</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>39224.0092308</v>
+        <v>39130.93299600002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.392240092308</v>
+        <v>0.3913093299600002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -12234,6 +12321,9 @@
       </c>
       <c r="DG14" s="3" t="n">
         <v>38.5918</v>
+      </c>
+      <c r="DH14" s="3" t="n">
+        <v>38.566</v>
       </c>
     </row>
     <row r="15">
@@ -12259,16 +12349,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.69</v>
+        <v>11.71</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>113906.74043</v>
+        <v>114101.61937</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>13906.74042999999</v>
+        <v>14101.61937000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1390674042999999</v>
+        <v>0.1410161937000002</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -12575,6 +12665,9 @@
       </c>
       <c r="DG15" s="3" t="n">
         <v>11.69</v>
+      </c>
+      <c r="DH15" s="3" t="n">
+        <v>11.71</v>
       </c>
     </row>
     <row r="16">
@@ -12600,16 +12693,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.4163</v>
+        <v>25.5188</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>145455.6549264</v>
+        <v>146042.2550464</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>45455.65492639999</v>
+        <v>46042.25504639998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4545565492639999</v>
+        <v>0.4604225504639998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -12910,6 +13003,9 @@
       </c>
       <c r="DG16" s="3" t="n">
         <v>25.4163</v>
+      </c>
+      <c r="DH16" s="3" t="n">
+        <v>25.5188</v>
       </c>
     </row>
     <row r="17">
@@ -12935,16 +13031,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8585</v>
+        <v>16.8838</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55735.16193449999</v>
+        <v>55818.8051766</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5735.161934499993</v>
+        <v>5818.805176599999</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1147032386899998</v>
+        <v>0.116376103532</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -13245,6 +13341,9 @@
       </c>
       <c r="DG17" s="3" t="n">
         <v>16.8585</v>
+      </c>
+      <c r="DH17" s="3" t="n">
+        <v>16.8838</v>
       </c>
     </row>
     <row r="18">
@@ -13270,16 +13369,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.17</v>
+        <v>47.06</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>88983.18612</v>
+        <v>88775.67816</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8983.186119999998</v>
+        <v>8775.678159999996</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1122898265</v>
+        <v>0.1096959769999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -13586,6 +13685,9 @@
       </c>
       <c r="DG18" s="3" t="n">
         <v>47.17</v>
+      </c>
+      <c r="DH18" s="3" t="n">
+        <v>47.06</v>
       </c>
     </row>
     <row r="19">
@@ -13611,16 +13713,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.027</v>
+        <v>13.3412</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>188458.560682</v>
+        <v>193004.0185592</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>38458.56068199998</v>
+        <v>43004.01855919999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2563904045466666</v>
+        <v>0.2866934570613333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -13921,6 +14023,9 @@
       </c>
       <c r="DG19" s="3" t="n">
         <v>13.027</v>
+      </c>
+      <c r="DH19" s="3" t="n">
+        <v>13.3412</v>
       </c>
     </row>
     <row r="20">
@@ -13946,16 +14051,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.81</v>
+        <v>9.77</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>257569.42743</v>
+        <v>256519.19531</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>7569.427430000011</v>
+        <v>6519.195309999981</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.03027770972000004</v>
+        <v>0.02607678123999992</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -14262,6 +14367,9 @@
       </c>
       <c r="DG20" s="3" t="n">
         <v>9.81</v>
+      </c>
+      <c r="DH20" s="3" t="n">
+        <v>9.77</v>
       </c>
     </row>
     <row r="21">
@@ -14287,16 +14395,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>113.9381</v>
+        <v>114.1916</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>173101.4838679</v>
+        <v>173486.6160244</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>3101.483867900009</v>
+        <v>3486.616024399991</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.018244022752353</v>
+        <v>0.0205095060258823</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -14603,6 +14711,9 @@
       </c>
       <c r="DG21" s="3" t="n">
         <v>113.9381</v>
+      </c>
+      <c r="DH21" s="3" t="n">
+        <v>114.1916</v>
       </c>
     </row>
     <row r="22">
@@ -14628,16 +14739,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.244</v>
+        <v>44.385</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67890.64823999999</v>
+        <v>68107.0071</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7890.648239999995</v>
+        <v>8107.007100000003</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1315108039999999</v>
+        <v>0.135116785</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -14938,6 +15049,9 @@
       </c>
       <c r="DG22" s="3" t="n">
         <v>44.244</v>
+      </c>
+      <c r="DH22" s="3" t="n">
+        <v>44.385</v>
       </c>
     </row>
     <row r="23">
@@ -14963,16 +15077,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.3089</v>
+        <v>63.4064</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>171976.5376563</v>
+        <v>172241.3931888</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>21976.5376563</v>
+        <v>22241.39318879999</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.146510251042</v>
+        <v>0.148275954592</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -15279,6 +15393,9 @@
       </c>
       <c r="DG23" s="3" t="n">
         <v>63.3089</v>
+      </c>
+      <c r="DH23" s="3" t="n">
+        <v>63.4064</v>
       </c>
     </row>
     <row r="24">
@@ -15304,16 +15421,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>26.847</v>
+        <v>26.8183</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>97545.51394200001</v>
+        <v>97441.2357638</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-2454.486057999995</v>
+        <v>-2558.764236200004</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.02454486057999995</v>
+        <v>-0.02558764236200004</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -15614,6 +15731,9 @@
       </c>
       <c r="DG24" s="3" t="n">
         <v>26.847</v>
+      </c>
+      <c r="DH24" s="3" t="n">
+        <v>26.8183</v>
       </c>
     </row>
     <row r="25">
@@ -15639,16 +15759,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>13.0166</v>
+        <v>13.0033</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>213754.3617884</v>
+        <v>213535.9535242</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>13754.36178839998</v>
+        <v>13535.95352419998</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.06877180894199991</v>
+        <v>0.06767976762099992</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -15952,6 +16072,9 @@
       </c>
       <c r="DG25" s="3" t="n">
         <v>13.0166</v>
+      </c>
+      <c r="DH25" s="3" t="n">
+        <v>13.0033</v>
       </c>
     </row>
     <row r="26">
@@ -15977,16 +16100,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.4086</v>
+        <v>11.2512</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>136238.249749</v>
+        <v>134358.623808</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>26238.24974900001</v>
+        <v>24358.623808</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.2385295431727274</v>
+        <v>0.2214420346181818</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -16290,6 +16413,9 @@
       </c>
       <c r="DG26" s="3" t="n">
         <v>11.4086</v>
+      </c>
+      <c r="DH26" s="3" t="n">
+        <v>11.2512</v>
       </c>
     </row>
     <row r="27">
@@ -16315,16 +16441,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>70.4213</v>
+        <v>70.21899999999999</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>113438.855318</v>
+        <v>113112.97834</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>3438.855318000002</v>
+        <v>3112.978339999987</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.03126232107272729</v>
+        <v>0.02829980309090897</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -16631,6 +16757,9 @@
       </c>
       <c r="DG27" s="3" t="n">
         <v>70.4213</v>
+      </c>
+      <c r="DH27" s="3" t="n">
+        <v>70.21899999999999</v>
       </c>
     </row>
     <row r="28">
@@ -16656,16 +16785,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>116.9959</v>
+        <v>116.6964</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>386865.3117063</v>
+        <v>385874.9679348</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>6865.31170630001</v>
+        <v>5874.967934800021</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.01806660975342108</v>
+        <v>0.01546044193368427</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -16972,6 +17101,9 @@
       </c>
       <c r="DG28" s="3" t="n">
         <v>116.9959</v>
+      </c>
+      <c r="DH28" s="3" t="n">
+        <v>116.6964</v>
       </c>
     </row>
     <row r="29">
@@ -16997,16 +17129,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.2766</v>
+        <v>12.3288</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>117900.8202498</v>
+        <v>118402.1335464</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>17900.8202498</v>
+        <v>18402.13354639999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.179008202498</v>
+        <v>0.1840213354639998</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -17307,6 +17439,9 @@
       </c>
       <c r="DG29" s="3" t="n">
         <v>12.2766</v>
+      </c>
+      <c r="DH29" s="3" t="n">
+        <v>12.3288</v>
       </c>
     </row>
     <row r="30">
@@ -17332,16 +17467,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.565</v>
+        <v>17.5007</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>129908.298465</v>
+        <v>129432.7446027</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>29908.29846500001</v>
+        <v>29432.74460269998</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2990829846500002</v>
+        <v>0.2943274460269998</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -17642,6 +17777,9 @@
       </c>
       <c r="DG30" s="3" t="n">
         <v>17.565</v>
+      </c>
+      <c r="DH30" s="3" t="n">
+        <v>17.5007</v>
       </c>
     </row>
     <row r="31">
@@ -17667,16 +17805,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>410.8551</v>
+        <v>411.1217</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109320.325008</v>
+        <v>109391.261936</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9320.325007999985</v>
+        <v>9391.261935999981</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09320325007999986</v>
+        <v>0.09391261935999981</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -17980,6 +18118,9 @@
       </c>
       <c r="DG31" s="3" t="n">
         <v>410.8551</v>
+      </c>
+      <c r="DH31" s="3" t="n">
+        <v>411.1217</v>
       </c>
     </row>
     <row r="32">
@@ -18005,16 +18146,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.98</v>
+        <v>10.96</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>232116.7608</v>
+        <v>231693.9616</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>32116.76079999999</v>
+        <v>31693.96160000001</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1605838039999999</v>
+        <v>0.158469808</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -18321,6 +18462,9 @@
       </c>
       <c r="DG32" s="3" t="n">
         <v>10.98</v>
+      </c>
+      <c r="DH32" s="3" t="n">
+        <v>10.96</v>
       </c>
     </row>
     <row r="33">
@@ -18346,16 +18490,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>20.21</v>
+        <v>20.26</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>72425.36440000001</v>
+        <v>72604.54640000001</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>12425.36440000001</v>
+        <v>12604.54640000001</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.2070894066666668</v>
+        <v>0.2100757733333334</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -18656,6 +18800,9 @@
       </c>
       <c r="DG33" s="3" t="n">
         <v>20.21</v>
+      </c>
+      <c r="DH33" s="3" t="n">
+        <v>20.26</v>
       </c>
     </row>
     <row r="34">
@@ -18681,16 +18828,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>222.7199</v>
+        <v>223.1542</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>78292.9491669</v>
+        <v>78445.61908020001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-1707.050833100002</v>
+        <v>-1554.380919799994</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.02133813541375002</v>
+        <v>-0.01942976149749993</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -18994,6 +19141,9 @@
       </c>
       <c r="DG34" s="3" t="n">
         <v>222.7199</v>
+      </c>
+      <c r="DH34" s="3" t="n">
+        <v>223.1542</v>
       </c>
     </row>
     <row r="35">
@@ -19019,16 +19169,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.08</v>
+        <v>16.14</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>114737.60184</v>
+        <v>115165.72722</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>14737.60183999999</v>
+        <v>15165.72722</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1473760183999999</v>
+        <v>0.1516572722</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -19332,6 +19482,9 @@
       </c>
       <c r="DG35" s="3" t="n">
         <v>16.08</v>
+      </c>
+      <c r="DH35" s="3" t="n">
+        <v>16.14</v>
       </c>
     </row>
     <row r="36">
@@ -19357,16 +19510,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>392.6752</v>
+        <v>390.833</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>182871.1966912</v>
+        <v>182013.273098</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>32871.19669120002</v>
+        <v>32013.27309800001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.2191413112746668</v>
+        <v>0.2134218206533334</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -19670,6 +19823,9 @@
       </c>
       <c r="DG36" s="3" t="n">
         <v>392.6752</v>
+      </c>
+      <c r="DH36" s="3" t="n">
+        <v>390.833</v>
       </c>
     </row>
     <row r="37">
@@ -19695,16 +19851,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.835</v>
+        <v>17.815</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>67111.12531500001</v>
+        <v>67035.86753500001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>17111.12531500001</v>
+        <v>17035.86753500001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.3422225063000002</v>
+        <v>0.3407173507000003</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -20008,6 +20164,9 @@
       </c>
       <c r="DG37" s="3" t="n">
         <v>17.835</v>
+      </c>
+      <c r="DH37" s="3" t="n">
+        <v>17.815</v>
       </c>
     </row>
     <row r="38">
@@ -20033,16 +20192,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9965</v>
+        <v>14.0124</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83705.81631299999</v>
+        <v>83800.9059768</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3705.816312999988</v>
+        <v>3800.905976800001</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.04632270391249985</v>
+        <v>0.04751132471000001</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -20343,6 +20502,9 @@
       </c>
       <c r="DG38" s="3" t="n">
         <v>13.9965</v>
+      </c>
+      <c r="DH38" s="3" t="n">
+        <v>14.0124</v>
       </c>
     </row>
     <row r="39">
@@ -20368,16 +20530,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1027.4945</v>
+        <v>1026.9538</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51252.4531545</v>
+        <v>51225.4824978</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1252.453154499999</v>
+        <v>1225.482497800003</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02504906308999998</v>
+        <v>0.02450964995600007</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -20678,6 +20840,9 @@
       </c>
       <c r="DG39" s="3" t="n">
         <v>1027.4945</v>
+      </c>
+      <c r="DH39" s="3" t="n">
+        <v>1026.9538</v>
       </c>
     </row>
     <row r="40">
@@ -20703,16 +20868,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.5679</v>
+        <v>21.6156</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>108724.3662333</v>
+        <v>108964.8232212</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>8724.36623330001</v>
+        <v>8964.8232212</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.0872436623330001</v>
+        <v>0.08964823221200001</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -21016,6 +21181,9 @@
       </c>
       <c r="DG40" s="3" t="n">
         <v>21.5679</v>
+      </c>
+      <c r="DH40" s="3" t="n">
+        <v>21.6156</v>
       </c>
     </row>
     <row r="41">
@@ -21028,13 +21196,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5100610.7657169</v>
+        <v>5104310.4877042</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>630610.7657169</v>
+        <v>634310.4877042</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1410762339411409</v>
+        <v>0.1419039122380761</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-27
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-26 07:02 IST</t>
+          <t>Generated: 2026-09-27 07:33 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-26</t>
+          <t>Last snapshot: 2026-09-27</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL19"/>
+  <dimension ref="A1:EM19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -761,6 +761,7 @@
     <col width="21" customWidth="1" min="140" max="140"/>
     <col width="21" customWidth="1" min="141" max="141"/>
     <col width="21" customWidth="1" min="142" max="142"/>
+    <col width="21" customWidth="1" min="143" max="143"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1474,6 +1475,11 @@
           <t>2026-09-26</t>
         </is>
       </c>
+      <c r="EM1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1903,6 +1909,9 @@
       <c r="EL2" s="3" t="n">
         <v>607.75</v>
       </c>
+      <c r="EM2" s="3" t="n">
+        <v>607.75</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2362,6 +2371,9 @@
       <c r="EL4" s="3" t="n">
         <v>1399</v>
       </c>
+      <c r="EM4" s="3" t="n">
+        <v>1399</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2794,6 +2806,9 @@
       <c r="EL5" s="3" t="n">
         <v>573.9500122070312</v>
       </c>
+      <c r="EM5" s="3" t="n">
+        <v>573.9500122070312</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3226,6 +3241,9 @@
       <c r="EL6" s="3" t="n">
         <v>338.5</v>
       </c>
+      <c r="EM6" s="3" t="n">
+        <v>338.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3658,6 +3676,9 @@
       <c r="EL7" s="3" t="n">
         <v>315.6499938964844</v>
       </c>
+      <c r="EM7" s="3" t="n">
+        <v>315.6499938964844</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4117,6 +4138,9 @@
       <c r="EL9" s="3" t="n">
         <v>15.86999988555908</v>
       </c>
+      <c r="EM9" s="3" t="n">
+        <v>15.86999988555908</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4549,6 +4573,9 @@
       <c r="EL10" s="3" t="n">
         <v>475.1499938964844</v>
       </c>
+      <c r="EM10" s="3" t="n">
+        <v>475.1499938964844</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4981,6 +5008,9 @@
       <c r="EL11" s="3" t="n">
         <v>14.10999965667725</v>
       </c>
+      <c r="EM11" s="3" t="n">
+        <v>14.10999965667725</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5413,6 +5443,9 @@
       <c r="EL12" s="3" t="n">
         <v>2778.300048828125</v>
       </c>
+      <c r="EM12" s="3" t="n">
+        <v>2778.300048828125</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5845,6 +5878,9 @@
       <c r="EL13" s="3" t="n">
         <v>40.79999923706055</v>
       </c>
+      <c r="EM13" s="3" t="n">
+        <v>40.79999923706055</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6277,6 +6313,9 @@
       <c r="EL14" s="3" t="n">
         <v>643.75</v>
       </c>
+      <c r="EM14" s="3" t="n">
+        <v>643.75</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6763,6 +6802,9 @@
       <c r="EL17" s="3" t="n">
         <v>503.8500061035156</v>
       </c>
+      <c r="EM17" s="3" t="n">
+        <v>503.8500061035156</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7193,6 +7235,9 @@
         <v>366</v>
       </c>
       <c r="EL18" s="3" t="n">
+        <v>367.5</v>
+      </c>
+      <c r="EM18" s="3" t="n">
         <v>367.5</v>
       </c>
     </row>
@@ -7223,7 +7268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH41"/>
+  <dimension ref="A1:DI41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7338,6 +7383,7 @@
     <col width="13" customWidth="1" min="110" max="110"/>
     <col width="13" customWidth="1" min="111" max="111"/>
     <col width="13" customWidth="1" min="112" max="112"/>
+    <col width="13" customWidth="1" min="113" max="113"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7901,6 +7947,11 @@
           <t>2026-09-26</t>
         </is>
       </c>
+      <c r="DI1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8245,6 +8296,9 @@
       <c r="DH2" s="3" t="n">
         <v>57.9132</v>
       </c>
+      <c r="DI2" s="3" t="n">
+        <v>57.9132</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8583,6 +8637,9 @@
       <c r="DH3" s="3" t="n">
         <v>26.7854</v>
       </c>
+      <c r="DI3" s="3" t="n">
+        <v>26.7854</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8921,6 +8978,9 @@
       <c r="DH4" s="3" t="n">
         <v>12.85</v>
       </c>
+      <c r="DI4" s="3" t="n">
+        <v>12.85</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9259,6 +9319,9 @@
       <c r="DH5" s="3" t="n">
         <v>9.253299999999999</v>
       </c>
+      <c r="DI5" s="3" t="n">
+        <v>9.253299999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9603,6 +9666,9 @@
       <c r="DH6" s="3" t="n">
         <v>11.5949</v>
       </c>
+      <c r="DI6" s="3" t="n">
+        <v>11.5949</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9941,6 +10007,9 @@
       <c r="DH7" s="3" t="n">
         <v>34.4256</v>
       </c>
+      <c r="DI7" s="3" t="n">
+        <v>34.4256</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10285,6 +10354,9 @@
       <c r="DH8" s="3" t="n">
         <v>35.6635</v>
       </c>
+      <c r="DI8" s="3" t="n">
+        <v>35.6635</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -10623,6 +10695,9 @@
       <c r="DH9" s="3" t="n">
         <v>42.5002</v>
       </c>
+      <c r="DI9" s="3" t="n">
+        <v>42.5002</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -10961,6 +11036,9 @@
       <c r="DH10" s="3" t="n">
         <v>48.5874</v>
       </c>
+      <c r="DI10" s="3" t="n">
+        <v>48.5874</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11299,6 +11377,9 @@
       <c r="DH11" s="3" t="n">
         <v>107.8591</v>
       </c>
+      <c r="DI11" s="3" t="n">
+        <v>107.8591</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11643,6 +11724,9 @@
       <c r="DH12" s="3" t="n">
         <v>226.38</v>
       </c>
+      <c r="DI12" s="3" t="n">
+        <v>226.38</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11987,6 +12071,9 @@
       <c r="DH13" s="3" t="n">
         <v>22.61</v>
       </c>
+      <c r="DI13" s="3" t="n">
+        <v>22.61</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12325,6 +12412,9 @@
       <c r="DH14" s="3" t="n">
         <v>38.566</v>
       </c>
+      <c r="DI14" s="3" t="n">
+        <v>38.566</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12669,6 +12759,9 @@
       <c r="DH15" s="3" t="n">
         <v>11.71</v>
       </c>
+      <c r="DI15" s="3" t="n">
+        <v>11.71</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13007,6 +13100,9 @@
       <c r="DH16" s="3" t="n">
         <v>25.5188</v>
       </c>
+      <c r="DI16" s="3" t="n">
+        <v>25.5188</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13345,6 +13441,9 @@
       <c r="DH17" s="3" t="n">
         <v>16.8838</v>
       </c>
+      <c r="DI17" s="3" t="n">
+        <v>16.8838</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13689,6 +13788,9 @@
       <c r="DH18" s="3" t="n">
         <v>47.06</v>
       </c>
+      <c r="DI18" s="3" t="n">
+        <v>47.06</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14027,6 +14129,9 @@
       <c r="DH19" s="3" t="n">
         <v>13.3412</v>
       </c>
+      <c r="DI19" s="3" t="n">
+        <v>13.3412</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -14371,6 +14476,9 @@
       <c r="DH20" s="3" t="n">
         <v>9.77</v>
       </c>
+      <c r="DI20" s="3" t="n">
+        <v>9.77</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -14715,6 +14823,9 @@
       <c r="DH21" s="3" t="n">
         <v>114.1916</v>
       </c>
+      <c r="DI21" s="3" t="n">
+        <v>114.1916</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -15053,6 +15164,9 @@
       <c r="DH22" s="3" t="n">
         <v>44.385</v>
       </c>
+      <c r="DI22" s="3" t="n">
+        <v>44.385</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -15397,6 +15511,9 @@
       <c r="DH23" s="3" t="n">
         <v>63.4064</v>
       </c>
+      <c r="DI23" s="3" t="n">
+        <v>63.4064</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -15735,6 +15852,9 @@
       <c r="DH24" s="3" t="n">
         <v>26.8183</v>
       </c>
+      <c r="DI24" s="3" t="n">
+        <v>26.8183</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -16076,6 +16196,9 @@
       <c r="DH25" s="3" t="n">
         <v>13.0033</v>
       </c>
+      <c r="DI25" s="3" t="n">
+        <v>13.0033</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -16417,6 +16540,9 @@
       <c r="DH26" s="3" t="n">
         <v>11.2512</v>
       </c>
+      <c r="DI26" s="3" t="n">
+        <v>11.2512</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -16761,6 +16887,9 @@
       <c r="DH27" s="3" t="n">
         <v>70.21899999999999</v>
       </c>
+      <c r="DI27" s="3" t="n">
+        <v>70.21899999999999</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -17105,6 +17234,9 @@
       <c r="DH28" s="3" t="n">
         <v>116.6964</v>
       </c>
+      <c r="DI28" s="3" t="n">
+        <v>116.6964</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -17443,6 +17575,9 @@
       <c r="DH29" s="3" t="n">
         <v>12.3288</v>
       </c>
+      <c r="DI29" s="3" t="n">
+        <v>12.3288</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -17781,6 +17916,9 @@
       <c r="DH30" s="3" t="n">
         <v>17.5007</v>
       </c>
+      <c r="DI30" s="3" t="n">
+        <v>17.5007</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -18122,6 +18260,9 @@
       <c r="DH31" s="3" t="n">
         <v>411.1217</v>
       </c>
+      <c r="DI31" s="3" t="n">
+        <v>411.1217</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -18466,6 +18607,9 @@
       <c r="DH32" s="3" t="n">
         <v>10.96</v>
       </c>
+      <c r="DI32" s="3" t="n">
+        <v>10.96</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -18804,6 +18948,9 @@
       <c r="DH33" s="3" t="n">
         <v>20.26</v>
       </c>
+      <c r="DI33" s="3" t="n">
+        <v>20.26</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -19145,6 +19292,9 @@
       <c r="DH34" s="3" t="n">
         <v>223.1542</v>
       </c>
+      <c r="DI34" s="3" t="n">
+        <v>223.1542</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -19486,6 +19636,9 @@
       <c r="DH35" s="3" t="n">
         <v>16.14</v>
       </c>
+      <c r="DI35" s="3" t="n">
+        <v>16.14</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -19827,6 +19980,9 @@
       <c r="DH36" s="3" t="n">
         <v>390.833</v>
       </c>
+      <c r="DI36" s="3" t="n">
+        <v>390.833</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -20168,6 +20324,9 @@
       <c r="DH37" s="3" t="n">
         <v>17.815</v>
       </c>
+      <c r="DI37" s="3" t="n">
+        <v>17.815</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -20506,6 +20665,9 @@
       <c r="DH38" s="3" t="n">
         <v>14.0124</v>
       </c>
+      <c r="DI38" s="3" t="n">
+        <v>14.0124</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -20844,6 +21006,9 @@
       <c r="DH39" s="3" t="n">
         <v>1026.9538</v>
       </c>
+      <c r="DI39" s="3" t="n">
+        <v>1026.9538</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -21183,6 +21348,9 @@
         <v>21.5679</v>
       </c>
       <c r="DH40" s="3" t="n">
+        <v>21.6156</v>
+      </c>
+      <c r="DI40" s="3" t="n">
         <v>21.6156</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-28
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-27 07:33 IST</t>
+          <t>Generated: 2026-09-28 08:10 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>546777.4988441467</v>
+        <v>541164.4967918396</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-44004.52115585329</v>
+        <v>-49617.52320816042</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07448520717650359</v>
+        <v>-0.08398617684431293</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5651087.986548346</v>
+        <v>5645474.984496039</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>590305.9665483469</v>
+        <v>584692.9644960398</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1166432310689301</v>
+        <v>0.1155341135392431</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-27</t>
+          <t>Last snapshot: 2026-09-28</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EM19"/>
+  <dimension ref="A1:EN19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -762,6 +762,7 @@
     <col width="21" customWidth="1" min="141" max="141"/>
     <col width="21" customWidth="1" min="142" max="142"/>
     <col width="21" customWidth="1" min="143" max="143"/>
+    <col width="21" customWidth="1" min="144" max="144"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1480,6 +1481,11 @@
           <t>2026-09-27</t>
         </is>
       </c>
+      <c r="EN1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1499,13 +1505,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>607.75</v>
+        <v>593</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>48620</v>
+        <v>47440</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4802.489999999998</v>
+        <v>3622.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1911,6 +1917,9 @@
       </c>
       <c r="EM2" s="3" t="n">
         <v>607.75</v>
+      </c>
+      <c r="EN2" s="3" t="n">
+        <v>593</v>
       </c>
     </row>
     <row r="3">
@@ -1958,13 +1967,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1399</v>
+        <v>1373.699951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27980</v>
+        <v>27473.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4124.580000000002</v>
+        <v>-4630.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2373,6 +2382,9 @@
       </c>
       <c r="EM4" s="3" t="n">
         <v>1399</v>
+      </c>
+      <c r="EN4" s="3" t="n">
+        <v>1373.699951171875</v>
       </c>
     </row>
     <row r="5">
@@ -2393,13 +2405,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>573.9500122070312</v>
+        <v>565.25</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11479.00024414062</v>
+        <v>11305</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-2734.099755859375</v>
+        <v>-2908.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2808,6 +2820,9 @@
       </c>
       <c r="EM5" s="3" t="n">
         <v>573.9500122070312</v>
+      </c>
+      <c r="EN5" s="3" t="n">
+        <v>565.25</v>
       </c>
     </row>
     <row r="6">
@@ -2828,13 +2843,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>338.5</v>
+        <v>331.3999938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13540</v>
+        <v>13255.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-3962.240000000002</v>
+        <v>-4246.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3243,6 +3258,9 @@
       </c>
       <c r="EM6" s="3" t="n">
         <v>338.5</v>
+      </c>
+      <c r="EN6" s="3" t="n">
+        <v>331.3999938964844</v>
       </c>
     </row>
     <row r="7">
@@ -3263,13 +3281,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>315.6499938964844</v>
+        <v>313.2000122070312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>31564.99938964844</v>
+        <v>31320.00122070312</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>5131.179389648438</v>
+        <v>4886.181220703125</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3678,6 +3696,9 @@
       </c>
       <c r="EM7" s="3" t="n">
         <v>315.6499938964844</v>
+      </c>
+      <c r="EN7" s="3" t="n">
+        <v>313.2000122070312</v>
       </c>
     </row>
     <row r="8">
@@ -3725,13 +3746,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.86999988555908</v>
+        <v>15.60999965667725</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23804.99982833862</v>
+        <v>23414.99948501587</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7245.170171661375</v>
+        <v>-7635.170514984129</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4140,6 +4161,9 @@
       </c>
       <c r="EM9" s="3" t="n">
         <v>15.86999988555908</v>
+      </c>
+      <c r="EN9" s="3" t="n">
+        <v>15.60999965667725</v>
       </c>
     </row>
     <row r="10">
@@ -4160,13 +4184,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>475.1499938964844</v>
+        <v>466.1499938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47514.99938964844</v>
+        <v>46614.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3983.480610351566</v>
+        <v>-4883.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4575,6 +4599,9 @@
       </c>
       <c r="EM10" s="3" t="n">
         <v>475.1499938964844</v>
+      </c>
+      <c r="EN10" s="3" t="n">
+        <v>466.1499938964844</v>
       </c>
     </row>
     <row r="11">
@@ -4595,13 +4622,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>14.10999965667725</v>
+        <v>13.8100004196167</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14109.99965667725</v>
+        <v>13810.0004196167</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4268.789656677247</v>
+        <v>3968.7904196167</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5010,6 +5037,9 @@
       </c>
       <c r="EM11" s="3" t="n">
         <v>14.10999965667725</v>
+      </c>
+      <c r="EN11" s="3" t="n">
+        <v>13.8100004196167</v>
       </c>
     </row>
     <row r="12">
@@ -5030,13 +5060,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2778.300048828125</v>
+        <v>2759.699951171875</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27783.00048828125</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>59.75048828125</v>
+        <v>27596.99951171875</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>-126.25048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5445,6 +5475,9 @@
       </c>
       <c r="EM12" s="3" t="n">
         <v>2778.300048828125</v>
+      </c>
+      <c r="EN12" s="3" t="n">
+        <v>2759.699951171875</v>
       </c>
     </row>
     <row r="13">
@@ -5465,13 +5498,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>40.79999923706055</v>
+        <v>39.66999816894531</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>24479.99954223633</v>
+        <v>23801.99890136719</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-10551.76045776367</v>
+        <v>-11229.76109863281</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5880,6 +5913,9 @@
       </c>
       <c r="EM13" s="3" t="n">
         <v>40.79999923706055</v>
+      </c>
+      <c r="EN13" s="3" t="n">
+        <v>39.66999816894531</v>
       </c>
     </row>
     <row r="14">
@@ -5900,13 +5936,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>643.75</v>
+        <v>647.3499755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>32187.5</v>
+        <v>32367.49877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-10275.01</v>
+        <v>-10095.01122070313</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6315,6 +6351,9 @@
       </c>
       <c r="EM14" s="3" t="n">
         <v>643.75</v>
+      </c>
+      <c r="EN14" s="3" t="n">
+        <v>647.3499755859375</v>
       </c>
     </row>
     <row r="15">
@@ -6389,13 +6428,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>503.8500061035156</v>
+        <v>494.3500061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25192.50030517578</v>
+        <v>24717.50030517578</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>3437.970305175782</v>
+        <v>2962.970305175782</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6804,6 +6843,9 @@
       </c>
       <c r="EM17" s="3" t="n">
         <v>503.8500061035156</v>
+      </c>
+      <c r="EN17" s="3" t="n">
+        <v>494.3500061035156</v>
       </c>
     </row>
     <row r="18">
@@ -6824,13 +6866,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>367.5</v>
+        <v>362.75</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36750</v>
+        <v>36275</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9890.82</v>
+        <v>-10365.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7239,6 +7281,9 @@
       </c>
       <c r="EM18" s="3" t="n">
         <v>367.5</v>
+      </c>
+      <c r="EN18" s="3" t="n">
+        <v>362.75</v>
       </c>
     </row>
     <row r="19">
@@ -7251,10 +7296,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>546777.4988441467</v>
+        <v>541164.4967918396</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-44004.52115585328</v>
+        <v>-49617.52320816041</v>
       </c>
     </row>
   </sheetData>
@@ -7268,7 +7313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DI41"/>
+  <dimension ref="A1:DJ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7384,6 +7429,7 @@
     <col width="13" customWidth="1" min="111" max="111"/>
     <col width="13" customWidth="1" min="112" max="112"/>
     <col width="13" customWidth="1" min="113" max="113"/>
+    <col width="13" customWidth="1" min="114" max="114"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7952,6 +7998,11 @@
           <t>2026-09-27</t>
         </is>
       </c>
+      <c r="DJ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8299,6 +8350,9 @@
       <c r="DI2" s="3" t="n">
         <v>57.9132</v>
       </c>
+      <c r="DJ2" s="3" t="n">
+        <v>57.9132</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8640,6 +8694,9 @@
       <c r="DI3" s="3" t="n">
         <v>26.7854</v>
       </c>
+      <c r="DJ3" s="3" t="n">
+        <v>26.7854</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8981,6 +9038,9 @@
       <c r="DI4" s="3" t="n">
         <v>12.85</v>
       </c>
+      <c r="DJ4" s="3" t="n">
+        <v>12.85</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9322,6 +9382,9 @@
       <c r="DI5" s="3" t="n">
         <v>9.253299999999999</v>
       </c>
+      <c r="DJ5" s="3" t="n">
+        <v>9.253299999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9669,6 +9732,9 @@
       <c r="DI6" s="3" t="n">
         <v>11.5949</v>
       </c>
+      <c r="DJ6" s="3" t="n">
+        <v>11.5949</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10010,6 +10076,9 @@
       <c r="DI7" s="3" t="n">
         <v>34.4256</v>
       </c>
+      <c r="DJ7" s="3" t="n">
+        <v>34.4256</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10357,6 +10426,9 @@
       <c r="DI8" s="3" t="n">
         <v>35.6635</v>
       </c>
+      <c r="DJ8" s="3" t="n">
+        <v>35.6635</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -10698,6 +10770,9 @@
       <c r="DI9" s="3" t="n">
         <v>42.5002</v>
       </c>
+      <c r="DJ9" s="3" t="n">
+        <v>42.5002</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11039,6 +11114,9 @@
       <c r="DI10" s="3" t="n">
         <v>48.5874</v>
       </c>
+      <c r="DJ10" s="3" t="n">
+        <v>48.5874</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11380,6 +11458,9 @@
       <c r="DI11" s="3" t="n">
         <v>107.8591</v>
       </c>
+      <c r="DJ11" s="3" t="n">
+        <v>107.8591</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11727,6 +11808,9 @@
       <c r="DI12" s="3" t="n">
         <v>226.38</v>
       </c>
+      <c r="DJ12" s="3" t="n">
+        <v>226.38</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12074,6 +12158,9 @@
       <c r="DI13" s="3" t="n">
         <v>22.61</v>
       </c>
+      <c r="DJ13" s="3" t="n">
+        <v>22.61</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12415,6 +12502,9 @@
       <c r="DI14" s="3" t="n">
         <v>38.566</v>
       </c>
+      <c r="DJ14" s="3" t="n">
+        <v>38.566</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12762,6 +12852,9 @@
       <c r="DI15" s="3" t="n">
         <v>11.71</v>
       </c>
+      <c r="DJ15" s="3" t="n">
+        <v>11.71</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13103,6 +13196,9 @@
       <c r="DI16" s="3" t="n">
         <v>25.5188</v>
       </c>
+      <c r="DJ16" s="3" t="n">
+        <v>25.5188</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13444,6 +13540,9 @@
       <c r="DI17" s="3" t="n">
         <v>16.8838</v>
       </c>
+      <c r="DJ17" s="3" t="n">
+        <v>16.8838</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13791,6 +13890,9 @@
       <c r="DI18" s="3" t="n">
         <v>47.06</v>
       </c>
+      <c r="DJ18" s="3" t="n">
+        <v>47.06</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14132,6 +14234,9 @@
       <c r="DI19" s="3" t="n">
         <v>13.3412</v>
       </c>
+      <c r="DJ19" s="3" t="n">
+        <v>13.3412</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -14479,6 +14584,9 @@
       <c r="DI20" s="3" t="n">
         <v>9.77</v>
       </c>
+      <c r="DJ20" s="3" t="n">
+        <v>9.77</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -14826,6 +14934,9 @@
       <c r="DI21" s="3" t="n">
         <v>114.1916</v>
       </c>
+      <c r="DJ21" s="3" t="n">
+        <v>114.1916</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -15167,6 +15278,9 @@
       <c r="DI22" s="3" t="n">
         <v>44.385</v>
       </c>
+      <c r="DJ22" s="3" t="n">
+        <v>44.385</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -15514,6 +15628,9 @@
       <c r="DI23" s="3" t="n">
         <v>63.4064</v>
       </c>
+      <c r="DJ23" s="3" t="n">
+        <v>63.4064</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -15855,6 +15972,9 @@
       <c r="DI24" s="3" t="n">
         <v>26.8183</v>
       </c>
+      <c r="DJ24" s="3" t="n">
+        <v>26.8183</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -16199,6 +16319,9 @@
       <c r="DI25" s="3" t="n">
         <v>13.0033</v>
       </c>
+      <c r="DJ25" s="3" t="n">
+        <v>13.0033</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -16543,6 +16666,9 @@
       <c r="DI26" s="3" t="n">
         <v>11.2512</v>
       </c>
+      <c r="DJ26" s="3" t="n">
+        <v>11.2512</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -16890,6 +17016,9 @@
       <c r="DI27" s="3" t="n">
         <v>70.21899999999999</v>
       </c>
+      <c r="DJ27" s="3" t="n">
+        <v>70.21899999999999</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -17237,6 +17366,9 @@
       <c r="DI28" s="3" t="n">
         <v>116.6964</v>
       </c>
+      <c r="DJ28" s="3" t="n">
+        <v>116.6964</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -17578,6 +17710,9 @@
       <c r="DI29" s="3" t="n">
         <v>12.3288</v>
       </c>
+      <c r="DJ29" s="3" t="n">
+        <v>12.3288</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -17919,6 +18054,9 @@
       <c r="DI30" s="3" t="n">
         <v>17.5007</v>
       </c>
+      <c r="DJ30" s="3" t="n">
+        <v>17.5007</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -18263,6 +18401,9 @@
       <c r="DI31" s="3" t="n">
         <v>411.1217</v>
       </c>
+      <c r="DJ31" s="3" t="n">
+        <v>411.1217</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -18610,6 +18751,9 @@
       <c r="DI32" s="3" t="n">
         <v>10.96</v>
       </c>
+      <c r="DJ32" s="3" t="n">
+        <v>10.96</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -18951,6 +19095,9 @@
       <c r="DI33" s="3" t="n">
         <v>20.26</v>
       </c>
+      <c r="DJ33" s="3" t="n">
+        <v>20.26</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -19295,6 +19442,9 @@
       <c r="DI34" s="3" t="n">
         <v>223.1542</v>
       </c>
+      <c r="DJ34" s="3" t="n">
+        <v>223.1542</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -19639,6 +19789,9 @@
       <c r="DI35" s="3" t="n">
         <v>16.14</v>
       </c>
+      <c r="DJ35" s="3" t="n">
+        <v>16.14</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -19983,6 +20136,9 @@
       <c r="DI36" s="3" t="n">
         <v>390.833</v>
       </c>
+      <c r="DJ36" s="3" t="n">
+        <v>390.833</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -20327,6 +20483,9 @@
       <c r="DI37" s="3" t="n">
         <v>17.815</v>
       </c>
+      <c r="DJ37" s="3" t="n">
+        <v>17.815</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -20668,6 +20827,9 @@
       <c r="DI38" s="3" t="n">
         <v>14.0124</v>
       </c>
+      <c r="DJ38" s="3" t="n">
+        <v>14.0124</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -21009,6 +21171,9 @@
       <c r="DI39" s="3" t="n">
         <v>1026.9538</v>
       </c>
+      <c r="DJ39" s="3" t="n">
+        <v>1026.9538</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -21351,6 +21516,9 @@
         <v>21.6156</v>
       </c>
       <c r="DI40" s="3" t="n">
+        <v>21.6156</v>
+      </c>
+      <c r="DJ40" s="3" t="n">
         <v>21.6156</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-29
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-28 08:10 IST</t>
+          <t>Generated: 2026-09-29 07:51 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5104310.4877042</v>
+        <v>5036310.356807</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>634310.4877041997</v>
+        <v>566310.356807</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.141903912238076</v>
+        <v>0.1266913549903803</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>541164.4967918396</v>
+        <v>538662.5014190674</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-49617.52320816042</v>
+        <v>-52119.51858093264</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08398617684431293</v>
+        <v>-0.08822123357940487</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5645474.984496039</v>
+        <v>5574972.858226067</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>584692.9644960398</v>
+        <v>514190.8382260678</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1155341135392431</v>
+        <v>0.1016030400428248</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-28</t>
+          <t>Last snapshot: 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EN19"/>
+  <dimension ref="A1:EO19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -763,6 +763,7 @@
     <col width="21" customWidth="1" min="142" max="142"/>
     <col width="21" customWidth="1" min="143" max="143"/>
     <col width="21" customWidth="1" min="144" max="144"/>
+    <col width="21" customWidth="1" min="145" max="145"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1486,6 +1487,11 @@
           <t>2026-09-28</t>
         </is>
       </c>
+      <c r="EO1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1505,13 +1511,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>593</v>
+        <v>593.9000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47440</v>
+        <v>47512.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3622.489999999998</v>
+        <v>3694.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1920,6 +1926,9 @@
       </c>
       <c r="EN2" s="3" t="n">
         <v>593</v>
+      </c>
+      <c r="EO2" s="3" t="n">
+        <v>593.9000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1967,13 +1976,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1373.699951171875</v>
+        <v>1375.300048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27473.9990234375</v>
+        <v>27506.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4630.580976562502</v>
+        <v>-4598.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2385,6 +2394,9 @@
       </c>
       <c r="EN4" s="3" t="n">
         <v>1373.699951171875</v>
+      </c>
+      <c r="EO4" s="3" t="n">
+        <v>1375.300048828125</v>
       </c>
     </row>
     <row r="5">
@@ -2405,13 +2417,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>565.25</v>
+        <v>539.5</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11305</v>
+        <v>10790</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-2908.1</v>
+        <v>-3423.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2823,6 +2835,9 @@
       </c>
       <c r="EN5" s="3" t="n">
         <v>565.25</v>
+      </c>
+      <c r="EO5" s="3" t="n">
+        <v>539.5</v>
       </c>
     </row>
     <row r="6">
@@ -2843,13 +2858,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>331.3999938964844</v>
+        <v>332.7999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13255.99975585938</v>
+        <v>13311.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4246.240244140627</v>
+        <v>-4190.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3261,6 +3276,9 @@
       </c>
       <c r="EN6" s="3" t="n">
         <v>331.3999938964844</v>
+      </c>
+      <c r="EO6" s="3" t="n">
+        <v>332.7999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -3281,13 +3299,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>313.2000122070312</v>
+        <v>314.1499938964844</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>31320.00122070312</v>
+        <v>31414.99938964844</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4886.181220703125</v>
+        <v>4981.179389648438</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3699,6 +3717,9 @@
       </c>
       <c r="EN7" s="3" t="n">
         <v>313.2000122070312</v>
+      </c>
+      <c r="EO7" s="3" t="n">
+        <v>314.1499938964844</v>
       </c>
     </row>
     <row r="8">
@@ -3746,13 +3767,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.60999965667725</v>
+        <v>15.40999984741211</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23414.99948501587</v>
+        <v>23114.99977111816</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7635.170514984129</v>
+        <v>-7935.170228881834</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4164,6 +4185,9 @@
       </c>
       <c r="EN9" s="3" t="n">
         <v>15.60999965667725</v>
+      </c>
+      <c r="EO9" s="3" t="n">
+        <v>15.40999984741211</v>
       </c>
     </row>
     <row r="10">
@@ -4184,13 +4208,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>466.1499938964844</v>
+        <v>465.3999938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46614.99938964844</v>
+        <v>46539.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-4883.480610351566</v>
+        <v>-4958.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4602,6 +4626,9 @@
       </c>
       <c r="EN10" s="3" t="n">
         <v>466.1499938964844</v>
+      </c>
+      <c r="EO10" s="3" t="n">
+        <v>465.3999938964844</v>
       </c>
     </row>
     <row r="11">
@@ -4622,13 +4649,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>13.8100004196167</v>
+        <v>13.31999969482422</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>13810.0004196167</v>
+        <v>13319.99969482422</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3968.7904196167</v>
+        <v>3478.78969482422</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5040,6 +5067,9 @@
       </c>
       <c r="EN11" s="3" t="n">
         <v>13.8100004196167</v>
+      </c>
+      <c r="EO11" s="3" t="n">
+        <v>13.31999969482422</v>
       </c>
     </row>
     <row r="12">
@@ -5060,13 +5090,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2759.699951171875</v>
+        <v>2832.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27596.99951171875</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>-126.25048828125</v>
+        <v>28325</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>601.75</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5478,6 +5508,9 @@
       </c>
       <c r="EN12" s="3" t="n">
         <v>2759.699951171875</v>
+      </c>
+      <c r="EO12" s="3" t="n">
+        <v>2832.5</v>
       </c>
     </row>
     <row r="13">
@@ -5498,13 +5531,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>39.66999816894531</v>
+        <v>39.47000122070312</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23801.99890136719</v>
+        <v>23682.00073242188</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11229.76109863281</v>
+        <v>-11349.75926757813</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5916,6 +5949,9 @@
       </c>
       <c r="EN13" s="3" t="n">
         <v>39.66999816894531</v>
+      </c>
+      <c r="EO13" s="3" t="n">
+        <v>39.47000122070312</v>
       </c>
     </row>
     <row r="14">
@@ -5936,13 +5972,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>647.3499755859375</v>
+        <v>622.8499755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>32367.49877929688</v>
+        <v>31142.49877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-10095.01122070313</v>
+        <v>-11320.01122070313</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6354,6 +6390,9 @@
       </c>
       <c r="EN14" s="3" t="n">
         <v>647.3499755859375</v>
+      </c>
+      <c r="EO14" s="3" t="n">
+        <v>622.8499755859375</v>
       </c>
     </row>
     <row r="15">
@@ -6428,13 +6467,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>494.3500061035156</v>
+        <v>491.25</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>24717.50030517578</v>
+        <v>24562.5</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>2962.970305175782</v>
+        <v>2807.970000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6846,6 +6885,9 @@
       </c>
       <c r="EN17" s="3" t="n">
         <v>494.3500061035156</v>
+      </c>
+      <c r="EO17" s="3" t="n">
+        <v>491.25</v>
       </c>
     </row>
     <row r="18">
@@ -6866,13 +6908,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>362.75</v>
+        <v>356.7000122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36275</v>
+        <v>35670.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-10365.82</v>
+        <v>-10970.81877929687</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7284,6 +7326,9 @@
       </c>
       <c r="EN18" s="3" t="n">
         <v>362.75</v>
+      </c>
+      <c r="EO18" s="3" t="n">
+        <v>356.7000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -7296,10 +7341,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>541164.4967918396</v>
+        <v>538662.5014190674</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-49617.52320816041</v>
+        <v>-52119.51858093263</v>
       </c>
     </row>
   </sheetData>
@@ -7313,7 +7358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DJ41"/>
+  <dimension ref="A1:DK41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7324,7 +7369,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -7430,6 +7475,7 @@
     <col width="13" customWidth="1" min="112" max="112"/>
     <col width="13" customWidth="1" min="113" max="113"/>
     <col width="13" customWidth="1" min="114" max="114"/>
+    <col width="13" customWidth="1" min="115" max="115"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8003,6 +8049,11 @@
           <t>2026-09-28</t>
         </is>
       </c>
+      <c r="DK1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8027,16 +8078,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.9132</v>
+        <v>57.7781</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>65006.5245624</v>
+        <v>64854.8772442</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>15006.5245624</v>
+        <v>14854.8772442</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.300130491248</v>
+        <v>0.2970975448839999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8352,6 +8403,9 @@
       </c>
       <c r="DJ2" s="3" t="n">
         <v>57.9132</v>
+      </c>
+      <c r="DK2" s="3" t="n">
+        <v>57.7781</v>
       </c>
     </row>
     <row r="3">
@@ -8377,16 +8431,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.7854</v>
+        <v>26.8173</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65763.86229020001</v>
+        <v>65842.18358490001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5763.862290200006</v>
+        <v>5842.183584900005</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09606437150333344</v>
+        <v>0.09736972641500009</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8696,6 +8750,9 @@
       </c>
       <c r="DJ3" s="3" t="n">
         <v>26.7854</v>
+      </c>
+      <c r="DK3" s="3" t="n">
+        <v>26.8173</v>
       </c>
     </row>
     <row r="4">
@@ -8721,16 +8778,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.85</v>
+        <v>12.79</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>246798.29505</v>
+        <v>245645.92947</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>66798.29505000002</v>
+        <v>65645.92947</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3711016391666668</v>
+        <v>0.3646996081666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9040,6 +9097,9 @@
       </c>
       <c r="DJ4" s="3" t="n">
         <v>12.85</v>
+      </c>
+      <c r="DK4" s="3" t="n">
+        <v>12.79</v>
       </c>
     </row>
     <row r="5">
@@ -9065,16 +9125,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.253299999999999</v>
+        <v>9.154</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>169835.8824904</v>
+        <v>168013.321552</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-40164.11750960001</v>
+        <v>-41986.67844799999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1912577024266667</v>
+        <v>-0.1999365640380952</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9384,6 +9444,9 @@
       </c>
       <c r="DJ5" s="3" t="n">
         <v>9.253299999999999</v>
+      </c>
+      <c r="DK5" s="3" t="n">
+        <v>9.154</v>
       </c>
     </row>
     <row r="6">
@@ -9409,16 +9472,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.5949</v>
+        <v>11.3945</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>49034.5654173</v>
+        <v>48187.0784265</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-965.4345826999997</v>
+        <v>-1812.921573499996</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.019308691654</v>
+        <v>-0.03625843146999992</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9734,6 +9797,9 @@
       </c>
       <c r="DJ6" s="3" t="n">
         <v>11.5949</v>
+      </c>
+      <c r="DK6" s="3" t="n">
+        <v>11.3945</v>
       </c>
     </row>
     <row r="7">
@@ -9759,16 +9825,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.4256</v>
+        <v>34.5388</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75944.25062400001</v>
+        <v>76193.974352</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15944.25062400001</v>
+        <v>16193.974352</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2657375104000001</v>
+        <v>0.2698995725333334</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -10078,6 +10144,9 @@
       </c>
       <c r="DJ7" s="3" t="n">
         <v>34.4256</v>
+      </c>
+      <c r="DK7" s="3" t="n">
+        <v>34.5388</v>
       </c>
     </row>
     <row r="8">
@@ -10103,16 +10172,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.6635</v>
+        <v>35.1305</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57225.4024555</v>
+        <v>56370.1543865</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7225.4024555</v>
+        <v>6370.154386499999</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.14450804911</v>
+        <v>0.12740308773</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -10428,6 +10497,9 @@
       </c>
       <c r="DJ8" s="3" t="n">
         <v>35.6635</v>
+      </c>
+      <c r="DK8" s="3" t="n">
+        <v>35.1305</v>
       </c>
     </row>
     <row r="9">
@@ -10453,16 +10525,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.5002</v>
+        <v>41.5718</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>136824.8463786</v>
+        <v>133835.9619174</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>36824.84637859999</v>
+        <v>33835.96191740001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3682484637859999</v>
+        <v>0.3383596191740001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10772,6 +10844,9 @@
       </c>
       <c r="DJ9" s="3" t="n">
         <v>42.5002</v>
+      </c>
+      <c r="DK9" s="3" t="n">
+        <v>41.5718</v>
       </c>
     </row>
     <row r="10">
@@ -10797,16 +10872,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.5874</v>
+        <v>48.6105</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138311.7594966</v>
+        <v>138377.5173195</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38311.75949660002</v>
+        <v>38377.51731950001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3831175949660002</v>
+        <v>0.3837751731950001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -11116,6 +11191,9 @@
       </c>
       <c r="DJ10" s="3" t="n">
         <v>48.5874</v>
+      </c>
+      <c r="DK10" s="3" t="n">
+        <v>48.6105</v>
       </c>
     </row>
     <row r="11">
@@ -11141,16 +11219,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.8591</v>
+        <v>107.1497</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32456.8525129</v>
+        <v>32243.3805743</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2456.852512899997</v>
+        <v>2243.380574299998</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.08189508376333324</v>
+        <v>0.07477935247666659</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -11460,6 +11538,9 @@
       </c>
       <c r="DJ11" s="3" t="n">
         <v>107.8591</v>
+      </c>
+      <c r="DK11" s="3" t="n">
+        <v>107.1497</v>
       </c>
     </row>
     <row r="12">
@@ -11485,16 +11566,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>226.38</v>
+        <v>223.172</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105384.87036</v>
+        <v>103891.475784</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5384.870360000001</v>
+        <v>3891.475783999995</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05384870360000001</v>
+        <v>0.03891475783999995</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -11810,6 +11891,9 @@
       </c>
       <c r="DJ12" s="3" t="n">
         <v>226.38</v>
+      </c>
+      <c r="DK12" s="3" t="n">
+        <v>223.172</v>
       </c>
     </row>
     <row r="13">
@@ -11835,16 +11919,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22.61</v>
+        <v>22.315</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>261995.74905</v>
+        <v>258577.405575</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>61995.74904999998</v>
+        <v>58577.40557500001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.3099787452499999</v>
+        <v>0.292887027875</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -12160,6 +12244,9 @@
       </c>
       <c r="DJ13" s="3" t="n">
         <v>22.61</v>
+      </c>
+      <c r="DK13" s="3" t="n">
+        <v>22.315</v>
       </c>
     </row>
     <row r="14">
@@ -12185,16 +12272,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.566</v>
+        <v>38.0915</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>139130.932996</v>
+        <v>137419.123949</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>39130.93299600002</v>
+        <v>37419.12394900003</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3913093299600002</v>
+        <v>0.3741912394900003</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -12504,6 +12591,9 @@
       </c>
       <c r="DJ14" s="3" t="n">
         <v>38.566</v>
+      </c>
+      <c r="DK14" s="3" t="n">
+        <v>38.0915</v>
       </c>
     </row>
     <row r="15">
@@ -12529,16 +12619,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.71</v>
+        <v>11.51</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114101.61937</v>
+        <v>112152.82997</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14101.61937000001</v>
+        <v>12152.82997000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1410161937000002</v>
+        <v>0.1215282997000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -12854,6 +12944,9 @@
       </c>
       <c r="DJ15" s="3" t="n">
         <v>11.71</v>
+      </c>
+      <c r="DK15" s="3" t="n">
+        <v>11.51</v>
       </c>
     </row>
     <row r="16">
@@ -12879,16 +12972,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.5188</v>
+        <v>25.2619</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>146042.2550464</v>
+        <v>144572.0348432</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>46042.25504639998</v>
+        <v>44572.0348432</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4604225504639998</v>
+        <v>0.445720348432</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -13198,6 +13291,9 @@
       </c>
       <c r="DJ16" s="3" t="n">
         <v>25.5188</v>
+      </c>
+      <c r="DK16" s="3" t="n">
+        <v>25.2619</v>
       </c>
     </row>
     <row r="17">
@@ -13223,16 +13319,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8838</v>
+        <v>16.735</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55818.8051766</v>
+        <v>55326.86389499999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5818.805176599999</v>
+        <v>5326.863894999995</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.116376103532</v>
+        <v>0.1065372778999999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -13542,6 +13638,9 @@
       </c>
       <c r="DJ17" s="3" t="n">
         <v>16.8838</v>
+      </c>
+      <c r="DK17" s="3" t="n">
+        <v>16.735</v>
       </c>
     </row>
     <row r="18">
@@ -13567,16 +13666,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.06</v>
+        <v>46.66</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>88775.67816</v>
+        <v>88021.10375999998</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8775.678159999996</v>
+        <v>8021.103759999984</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1096959769999999</v>
+        <v>0.1002637969999998</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -13892,6 +13991,9 @@
       </c>
       <c r="DJ18" s="3" t="n">
         <v>47.06</v>
+      </c>
+      <c r="DK18" s="3" t="n">
+        <v>46.66</v>
       </c>
     </row>
     <row r="19">
@@ -13917,16 +14019,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.3412</v>
+        <v>13.0952</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>193004.0185592</v>
+        <v>189445.1941232</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>43004.01855919999</v>
+        <v>39445.1941232</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2866934570613333</v>
+        <v>0.2629679608213333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -14236,6 +14338,9 @@
       </c>
       <c r="DJ19" s="3" t="n">
         <v>13.3412</v>
+      </c>
+      <c r="DK19" s="3" t="n">
+        <v>13.0952</v>
       </c>
     </row>
     <row r="20">
@@ -14261,16 +14366,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.77</v>
+        <v>9.69</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>256519.19531</v>
+        <v>254418.73107</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>6519.195309999981</v>
+        <v>4418.73106999998</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.02607678123999992</v>
+        <v>0.01767492427999992</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -14586,6 +14691,9 @@
       </c>
       <c r="DJ20" s="3" t="n">
         <v>9.77</v>
+      </c>
+      <c r="DK20" s="3" t="n">
+        <v>9.69</v>
       </c>
     </row>
     <row r="21">
@@ -14611,16 +14719,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>114.1916</v>
+        <v>112.2782</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>173486.6160244</v>
+        <v>170579.6658538</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>3486.616024399991</v>
+        <v>579.6658537999901</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.0205095060258823</v>
+        <v>0.003409799139999942</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -14936,6 +15044,9 @@
       </c>
       <c r="DJ21" s="3" t="n">
         <v>114.1916</v>
+      </c>
+      <c r="DK21" s="3" t="n">
+        <v>112.2782</v>
       </c>
     </row>
     <row r="22">
@@ -14961,16 +15072,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.385</v>
+        <v>43.707</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68107.0071</v>
+        <v>67066.64322</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8107.007100000003</v>
+        <v>7066.643219999998</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.135116785</v>
+        <v>0.117777387</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -15280,6 +15391,9 @@
       </c>
       <c r="DJ22" s="3" t="n">
         <v>44.385</v>
+      </c>
+      <c r="DK22" s="3" t="n">
+        <v>43.707</v>
       </c>
     </row>
     <row r="23">
@@ -15305,16 +15419,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.4064</v>
+        <v>62.2613</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>172241.3931888</v>
+        <v>169130.7668271</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>22241.39318879999</v>
+        <v>19130.76682710001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.148275954592</v>
+        <v>0.1275384455140001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -15630,6 +15744,9 @@
       </c>
       <c r="DJ23" s="3" t="n">
         <v>63.4064</v>
+      </c>
+      <c r="DK23" s="3" t="n">
+        <v>62.2613</v>
       </c>
     </row>
     <row r="24">
@@ -15655,16 +15772,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>26.8183</v>
+        <v>26.2569</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>97441.2357638</v>
+        <v>95401.4528634</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-2558.764236200004</v>
+        <v>-4598.547136599998</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.02558764236200004</v>
+        <v>-0.04598547136599998</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -15974,6 +16091,9 @@
       </c>
       <c r="DJ24" s="3" t="n">
         <v>26.8183</v>
+      </c>
+      <c r="DK24" s="3" t="n">
+        <v>26.2569</v>
       </c>
     </row>
     <row r="25">
@@ -15999,16 +16119,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>13.0033</v>
+        <v>12.7622</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>213535.9535242</v>
+        <v>209576.6879228</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>13535.95352419998</v>
+        <v>9576.687922799989</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.06767976762099992</v>
+        <v>0.04788343961399994</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -16321,6 +16441,9 @@
       </c>
       <c r="DJ25" s="3" t="n">
         <v>13.0033</v>
+      </c>
+      <c r="DK25" s="3" t="n">
+        <v>12.7622</v>
       </c>
     </row>
     <row r="26">
@@ -16346,16 +16469,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.2512</v>
+        <v>11.0326</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>134358.623808</v>
+        <v>131748.164909</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>24358.623808</v>
+        <v>21748.16490900001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.2214420346181818</v>
+        <v>0.1977105900818183</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -16668,6 +16791,9 @@
       </c>
       <c r="DJ26" s="3" t="n">
         <v>11.2512</v>
+      </c>
+      <c r="DK26" s="3" t="n">
+        <v>11.0326</v>
       </c>
     </row>
     <row r="27">
@@ -16693,16 +16819,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>70.21899999999999</v>
+        <v>69.0719</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>113112.97834</v>
+        <v>111265.160834</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>3112.978339999987</v>
+        <v>1265.160833999995</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.02829980309090897</v>
+        <v>0.01150146212727268</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -17018,6 +17144,9 @@
       </c>
       <c r="DJ27" s="3" t="n">
         <v>70.21899999999999</v>
+      </c>
+      <c r="DK27" s="3" t="n">
+        <v>69.0719</v>
       </c>
     </row>
     <row r="28">
@@ -17043,16 +17172,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>116.6964</v>
+        <v>114.8816</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>385874.9679348</v>
-      </c>
-      <c r="H28" s="4" t="n">
-        <v>5874.967934800021</v>
-      </c>
-      <c r="I28" s="12" t="n">
-        <v>0.01546044193368427</v>
+        <v>379874.0468112</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>-125.9531887999619</v>
+      </c>
+      <c r="I28" s="13" t="n">
+        <v>-0.0003314557599998998</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -17368,6 +17497,9 @@
       </c>
       <c r="DJ28" s="3" t="n">
         <v>116.6964</v>
+      </c>
+      <c r="DK28" s="3" t="n">
+        <v>114.8816</v>
       </c>
     </row>
     <row r="29">
@@ -17393,16 +17525,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.3288</v>
+        <v>12.1049</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>118402.1335464</v>
+        <v>116251.8644447</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>18402.13354639999</v>
+        <v>16251.8644447</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1840213354639998</v>
+        <v>0.162518644447</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -17712,6 +17844,9 @@
       </c>
       <c r="DJ29" s="3" t="n">
         <v>12.3288</v>
+      </c>
+      <c r="DK29" s="3" t="n">
+        <v>12.1049</v>
       </c>
     </row>
     <row r="30">
@@ -17737,16 +17872,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.5007</v>
+        <v>17.3078</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>129432.7446027</v>
+        <v>128006.0830158</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>29432.74460269998</v>
+        <v>28006.0830158</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2943274460269998</v>
+        <v>0.280060830158</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -18056,6 +18191,9 @@
       </c>
       <c r="DJ30" s="3" t="n">
         <v>17.5007</v>
+      </c>
+      <c r="DK30" s="3" t="n">
+        <v>17.3078</v>
       </c>
     </row>
     <row r="31">
@@ -18081,16 +18219,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>411.1217</v>
+        <v>403.933</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109391.261936</v>
+        <v>107478.49264</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9391.261935999981</v>
+        <v>7478.492639999997</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09391261935999981</v>
+        <v>0.07478492639999997</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -18403,6 +18541,9 @@
       </c>
       <c r="DJ31" s="3" t="n">
         <v>411.1217</v>
+      </c>
+      <c r="DK31" s="3" t="n">
+        <v>403.933</v>
       </c>
     </row>
     <row r="32">
@@ -18428,16 +18569,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.96</v>
+        <v>10.76</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>231693.9616</v>
+        <v>227465.9696</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>31693.96160000001</v>
+        <v>27465.96959999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.158469808</v>
+        <v>0.1373298479999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -18753,6 +18894,9 @@
       </c>
       <c r="DJ32" s="3" t="n">
         <v>10.96</v>
+      </c>
+      <c r="DK32" s="3" t="n">
+        <v>10.76</v>
       </c>
     </row>
     <row r="33">
@@ -18778,16 +18922,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>20.26</v>
+        <v>19.87</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>72604.54640000001</v>
+        <v>71206.9268</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>12604.54640000001</v>
+        <v>11206.9268</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.2100757733333334</v>
+        <v>0.1867821133333334</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -19097,6 +19241,9 @@
       </c>
       <c r="DJ33" s="3" t="n">
         <v>20.26</v>
+      </c>
+      <c r="DK33" s="3" t="n">
+        <v>19.87</v>
       </c>
     </row>
     <row r="34">
@@ -19122,16 +19269,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>223.1542</v>
+        <v>221.2707</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>78445.61908020001</v>
+        <v>77783.5104417</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-1554.380919799994</v>
+        <v>-2216.489558300003</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.01942976149749993</v>
+        <v>-0.02770611947875004</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -19444,6 +19591,9 @@
       </c>
       <c r="DJ34" s="3" t="n">
         <v>223.1542</v>
+      </c>
+      <c r="DK34" s="3" t="n">
+        <v>221.2707</v>
       </c>
     </row>
     <row r="35">
@@ -19469,16 +19619,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.14</v>
+        <v>15.91</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>115165.72722</v>
+        <v>113524.57993</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>15165.72722</v>
+        <v>13524.57992999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1516572722</v>
+        <v>0.1352457992999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -19791,6 +19941,9 @@
       </c>
       <c r="DJ35" s="3" t="n">
         <v>16.14</v>
+      </c>
+      <c r="DK35" s="3" t="n">
+        <v>15.91</v>
       </c>
     </row>
     <row r="36">
@@ -19816,16 +19969,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>390.833</v>
+        <v>386.9382</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>182013.273098</v>
+        <v>180199.4413692</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>32013.27309800001</v>
+        <v>30199.44136920001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.2134218206533334</v>
+        <v>0.201329609128</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -20138,6 +20291,9 @@
       </c>
       <c r="DJ36" s="3" t="n">
         <v>390.833</v>
+      </c>
+      <c r="DK36" s="3" t="n">
+        <v>386.9382</v>
       </c>
     </row>
     <row r="37">
@@ -20163,16 +20319,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.815</v>
+        <v>17.582</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>67035.86753500001</v>
+        <v>66159.11439800001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>17035.86753500001</v>
+        <v>16159.11439800001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.3407173507000003</v>
+        <v>0.3231822879600001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -20485,6 +20641,9 @@
       </c>
       <c r="DJ37" s="3" t="n">
         <v>17.815</v>
+      </c>
+      <c r="DK37" s="3" t="n">
+        <v>17.582</v>
       </c>
     </row>
     <row r="38">
@@ -20510,16 +20669,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.0124</v>
+        <v>13.7834</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83800.9059768</v>
+        <v>82431.3755988</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3800.905976800001</v>
+        <v>2431.375598800005</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.04751132471000001</v>
+        <v>0.03039219498500006</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -20829,6 +20988,9 @@
       </c>
       <c r="DJ38" s="3" t="n">
         <v>14.0124</v>
+      </c>
+      <c r="DK38" s="3" t="n">
+        <v>13.7834</v>
       </c>
     </row>
     <row r="39">
@@ -20854,16 +21016,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1026.9538</v>
+        <v>1025.7643</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51225.4824978</v>
+        <v>51166.1490483</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1225.482497800003</v>
+        <v>1166.149048300002</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02450964995600007</v>
+        <v>0.02332298096600003</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -21173,6 +21335,9 @@
       </c>
       <c r="DJ39" s="3" t="n">
         <v>1026.9538</v>
+      </c>
+      <c r="DK39" s="3" t="n">
+        <v>1025.7643</v>
       </c>
     </row>
     <row r="40">
@@ -21198,16 +21363,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.6156</v>
+        <v>21.1475</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>108964.8232212</v>
+        <v>106605.1184825</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>8964.8232212</v>
+        <v>6605.118482500009</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.08964823221200001</v>
+        <v>0.06605118482500009</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -21520,6 +21685,9 @@
       </c>
       <c r="DJ40" s="3" t="n">
         <v>21.6156</v>
+      </c>
+      <c r="DK40" s="3" t="n">
+        <v>21.1475</v>
       </c>
     </row>
     <row r="41">
@@ -21532,13 +21700,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5104310.4877042</v>
+        <v>5036310.356807</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>634310.4877042</v>
+        <v>566310.3568070001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1419039122380761</v>
+        <v>0.1266913549903803</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-09-30
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,8 +483,8 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-29 07:51 IST</t>
+          <t>Generated: 2026-09-30 07:54 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5036310.356807</v>
+        <v>5016567.8105559</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>566310.356807</v>
+        <v>546567.8105558995</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1266913549903803</v>
+        <v>0.1222746779767113</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>538662.5014190674</v>
+        <v>536298.5044937134</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-52119.51858093264</v>
+        <v>-54483.51550628664</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08822123357940487</v>
+        <v>-0.09222270424933826</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5574972.858226067</v>
+        <v>5552866.315049613</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>514190.8382260678</v>
+        <v>492084.2950496133</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1016030400428248</v>
+        <v>0.0972348330959359</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-29</t>
+          <t>Last snapshot: 2026-09-30</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EO19"/>
+  <dimension ref="A1:EP19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -764,6 +764,7 @@
     <col width="21" customWidth="1" min="143" max="143"/>
     <col width="21" customWidth="1" min="144" max="144"/>
     <col width="21" customWidth="1" min="145" max="145"/>
+    <col width="21" customWidth="1" min="146" max="146"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1492,6 +1493,11 @@
           <t>2026-09-29</t>
         </is>
       </c>
+      <c r="EP1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1511,13 +1517,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>593.9000244140625</v>
+        <v>591.2000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47512.001953125</v>
+        <v>47296.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3694.491953124998</v>
+        <v>3478.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1929,6 +1935,9 @@
       </c>
       <c r="EO2" s="3" t="n">
         <v>593.9000244140625</v>
+      </c>
+      <c r="EP2" s="3" t="n">
+        <v>591.2000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -1976,13 +1985,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1375.300048828125</v>
+        <v>1379</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27506.0009765625</v>
+        <v>27580</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4598.579023437502</v>
+        <v>-4524.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2397,6 +2406,9 @@
       </c>
       <c r="EO4" s="3" t="n">
         <v>1375.300048828125</v>
+      </c>
+      <c r="EP4" s="3" t="n">
+        <v>1379</v>
       </c>
     </row>
     <row r="5">
@@ -2417,13 +2429,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>539.5</v>
+        <v>525.5</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>10790</v>
+        <v>10510</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-3423.1</v>
+        <v>-3703.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2838,6 +2850,9 @@
       </c>
       <c r="EO5" s="3" t="n">
         <v>539.5</v>
+      </c>
+      <c r="EP5" s="3" t="n">
+        <v>525.5</v>
       </c>
     </row>
     <row r="6">
@@ -2858,13 +2873,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>332.7999877929688</v>
+        <v>332.3500061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13311.99951171875</v>
+        <v>13294.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4190.240488281252</v>
+        <v>-4208.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3279,6 +3294,9 @@
       </c>
       <c r="EO6" s="3" t="n">
         <v>332.7999877929688</v>
+      </c>
+      <c r="EP6" s="3" t="n">
+        <v>332.3500061035156</v>
       </c>
     </row>
     <row r="7">
@@ -3299,13 +3317,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>314.1499938964844</v>
+        <v>312.25</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>31414.99938964844</v>
+        <v>31225</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4981.179389648438</v>
+        <v>4791.18</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3720,6 +3738,9 @@
       </c>
       <c r="EO7" s="3" t="n">
         <v>314.1499938964844</v>
+      </c>
+      <c r="EP7" s="3" t="n">
+        <v>312.25</v>
       </c>
     </row>
     <row r="8">
@@ -3767,13 +3788,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.40999984741211</v>
+        <v>15.34000015258789</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23114.99977111816</v>
+        <v>23010.00022888184</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-7935.170228881834</v>
+        <v>-8040.169771118162</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4188,6 +4209,9 @@
       </c>
       <c r="EO9" s="3" t="n">
         <v>15.40999984741211</v>
+      </c>
+      <c r="EP9" s="3" t="n">
+        <v>15.34000015258789</v>
       </c>
     </row>
     <row r="10">
@@ -4208,13 +4232,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>465.3999938964844</v>
+        <v>450.4500122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46539.99938964844</v>
+        <v>45045.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-4958.480610351566</v>
+        <v>-6453.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4629,6 +4653,9 @@
       </c>
       <c r="EO10" s="3" t="n">
         <v>465.3999938964844</v>
+      </c>
+      <c r="EP10" s="3" t="n">
+        <v>450.4500122070312</v>
       </c>
     </row>
     <row r="11">
@@ -4649,13 +4676,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>13.31999969482422</v>
+        <v>13.47000026702881</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>13319.99969482422</v>
+        <v>13470.00026702881</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3478.78969482422</v>
+        <v>3628.790267028809</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5070,6 +5097,9 @@
       </c>
       <c r="EO11" s="3" t="n">
         <v>13.31999969482422</v>
+      </c>
+      <c r="EP11" s="3" t="n">
+        <v>13.47000026702881</v>
       </c>
     </row>
     <row r="12">
@@ -5090,13 +5120,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2832.5</v>
+        <v>2760.60009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>28325</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>601.75</v>
+        <v>27606.0009765625</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>-117.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5511,6 +5541,9 @@
       </c>
       <c r="EO12" s="3" t="n">
         <v>2832.5</v>
+      </c>
+      <c r="EP12" s="3" t="n">
+        <v>2760.60009765625</v>
       </c>
     </row>
     <row r="13">
@@ -5531,13 +5564,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>39.47000122070312</v>
+        <v>39.77000045776367</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23682.00073242188</v>
+        <v>23862.0002746582</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11349.75926757813</v>
+        <v>-11169.7597253418</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5952,6 +5985,9 @@
       </c>
       <c r="EO13" s="3" t="n">
         <v>39.47000122070312</v>
+      </c>
+      <c r="EP13" s="3" t="n">
+        <v>39.77000045776367</v>
       </c>
     </row>
     <row r="14">
@@ -5972,13 +6008,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>622.8499755859375</v>
+        <v>617.9000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31142.49877929688</v>
+        <v>30895.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11320.01122070313</v>
+        <v>-11567.50877929688</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6393,6 +6429,9 @@
       </c>
       <c r="EO14" s="3" t="n">
         <v>622.8499755859375</v>
+      </c>
+      <c r="EP14" s="3" t="n">
+        <v>617.9000244140625</v>
       </c>
     </row>
     <row r="15">
@@ -6467,13 +6506,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>491.25</v>
+        <v>491.1000061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>24562.5</v>
+        <v>24555.00030517578</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>2807.970000000001</v>
+        <v>2800.470305175782</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6888,6 +6927,9 @@
       </c>
       <c r="EO17" s="3" t="n">
         <v>491.25</v>
+      </c>
+      <c r="EP17" s="3" t="n">
+        <v>491.1000061035156</v>
       </c>
     </row>
     <row r="18">
@@ -6908,13 +6950,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>356.7000122070312</v>
+        <v>361.7999877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35670.00122070312</v>
+        <v>36179.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-10970.81877929687</v>
+        <v>-10460.82122070312</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7329,6 +7371,9 @@
       </c>
       <c r="EO18" s="3" t="n">
         <v>356.7000122070312</v>
+      </c>
+      <c r="EP18" s="3" t="n">
+        <v>361.7999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -7341,10 +7386,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>538662.5014190674</v>
+        <v>536298.5044937134</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-52119.51858093263</v>
+        <v>-54483.51550628663</v>
       </c>
     </row>
   </sheetData>
@@ -7358,7 +7403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DK41"/>
+  <dimension ref="A1:DL41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7369,7 +7414,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -7476,6 +7521,7 @@
     <col width="13" customWidth="1" min="113" max="113"/>
     <col width="13" customWidth="1" min="114" max="114"/>
     <col width="13" customWidth="1" min="115" max="115"/>
+    <col width="13" customWidth="1" min="116" max="116"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8054,6 +8100,11 @@
           <t>2026-09-29</t>
         </is>
       </c>
+      <c r="DL1" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8078,16 +8129,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.7781</v>
+        <v>57.6679</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64854.8772442</v>
+        <v>64731.1797278</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14854.8772442</v>
+        <v>14731.1797278</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2970975448839999</v>
+        <v>0.294623594556</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8406,6 +8457,9 @@
       </c>
       <c r="DK2" s="3" t="n">
         <v>57.7781</v>
+      </c>
+      <c r="DL2" s="3" t="n">
+        <v>57.6679</v>
       </c>
     </row>
     <row r="3">
@@ -8431,16 +8485,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.8173</v>
+        <v>26.7769</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65842.18358490001</v>
+        <v>65742.99297970001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5842.183584900005</v>
+        <v>5742.992979700008</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09736972641500009</v>
+        <v>0.09571654966166679</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8753,6 +8807,9 @@
       </c>
       <c r="DK3" s="3" t="n">
         <v>26.8173</v>
+      </c>
+      <c r="DL3" s="3" t="n">
+        <v>26.7769</v>
       </c>
     </row>
     <row r="4">
@@ -8778,16 +8835,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.79</v>
+        <v>12.7</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>245645.92947</v>
+        <v>243917.3811</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>65645.92947</v>
+        <v>63917.3811</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3646996081666667</v>
+        <v>0.3550965616666666</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9100,6 +9157,9 @@
       </c>
       <c r="DK4" s="3" t="n">
         <v>12.79</v>
+      </c>
+      <c r="DL4" s="3" t="n">
+        <v>12.7</v>
       </c>
     </row>
     <row r="5">
@@ -9125,16 +9185,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.154</v>
+        <v>8.998799999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>168013.321552</v>
+        <v>165164.7670944</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-41986.67844799999</v>
+        <v>-44835.23290560002</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1999365640380952</v>
+        <v>-0.2135011090742858</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9447,6 +9507,9 @@
       </c>
       <c r="DK5" s="3" t="n">
         <v>9.154</v>
+      </c>
+      <c r="DL5" s="3" t="n">
+        <v>8.998799999999999</v>
       </c>
     </row>
     <row r="6">
@@ -9472,16 +9535,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.3945</v>
+        <v>11.3464</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>48187.0784265</v>
+        <v>47983.66463279999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-1812.921573499996</v>
+        <v>-2016.335367200008</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.03625843146999992</v>
+        <v>-0.04032670734400017</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9800,6 +9863,9 @@
       </c>
       <c r="DK6" s="3" t="n">
         <v>11.3945</v>
+      </c>
+      <c r="DL6" s="3" t="n">
+        <v>11.3464</v>
       </c>
     </row>
     <row r="7">
@@ -9825,16 +9891,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.5388</v>
+        <v>34.4078</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>76193.974352</v>
+        <v>75904.983112</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>16193.974352</v>
+        <v>15904.983112</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2698995725333334</v>
+        <v>0.2650830518666667</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -10147,6 +10213,9 @@
       </c>
       <c r="DK7" s="3" t="n">
         <v>34.5388</v>
+      </c>
+      <c r="DL7" s="3" t="n">
+        <v>34.4078</v>
       </c>
     </row>
     <row r="8">
@@ -10172,16 +10241,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.1305</v>
+        <v>35.5494</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>56370.1543865</v>
+        <v>57042.3183942</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6370.154386499999</v>
+        <v>7042.318394200003</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.12740308773</v>
+        <v>0.1408463678840001</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -10500,6 +10569,9 @@
       </c>
       <c r="DK8" s="3" t="n">
         <v>35.1305</v>
+      </c>
+      <c r="DL8" s="3" t="n">
+        <v>35.5494</v>
       </c>
     </row>
     <row r="9">
@@ -10525,16 +10597,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.5718</v>
+        <v>41.8901</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>133835.9619174</v>
+        <v>134860.6947093</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>33835.96191740001</v>
+        <v>34860.69470930001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3383596191740001</v>
+        <v>0.3486069470930001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10847,6 +10919,9 @@
       </c>
       <c r="DK9" s="3" t="n">
         <v>41.5718</v>
+      </c>
+      <c r="DL9" s="3" t="n">
+        <v>41.8901</v>
       </c>
     </row>
     <row r="10">
@@ -10872,16 +10947,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.6105</v>
+        <v>48.3434</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138377.5173195</v>
+        <v>137617.1747006</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38377.51731950001</v>
+        <v>37617.17470060001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3837751731950001</v>
+        <v>0.3761717470060001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -11194,6 +11269,9 @@
       </c>
       <c r="DK10" s="3" t="n">
         <v>48.6105</v>
+      </c>
+      <c r="DL10" s="3" t="n">
+        <v>48.3434</v>
       </c>
     </row>
     <row r="11">
@@ -11219,16 +11297,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.1497</v>
+        <v>107.326</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32243.3805743</v>
+        <v>32296.43259399999</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2243.380574299998</v>
+        <v>2296.432593999994</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07477935247666659</v>
+        <v>0.07654775313333315</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -11541,6 +11619,9 @@
       </c>
       <c r="DK11" s="3" t="n">
         <v>107.1497</v>
+      </c>
+      <c r="DL11" s="3" t="n">
+        <v>107.326</v>
       </c>
     </row>
     <row r="12">
@@ -11566,16 +11647,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>223.172</v>
+        <v>221.354</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>103891.475784</v>
+        <v>103045.156788</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3891.475783999995</v>
+        <v>3045.156788000008</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.03891475783999995</v>
+        <v>0.03045156788000008</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -11894,6 +11975,9 @@
       </c>
       <c r="DK12" s="3" t="n">
         <v>223.172</v>
+      </c>
+      <c r="DL12" s="3" t="n">
+        <v>221.354</v>
       </c>
     </row>
     <row r="13">
@@ -11919,16 +12003,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22.315</v>
+        <v>22.392</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>258577.405575</v>
+        <v>259469.65116</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>58577.40557500001</v>
+        <v>59469.65115999998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.292887027875</v>
+        <v>0.2973482557999999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -12247,6 +12331,9 @@
       </c>
       <c r="DK13" s="3" t="n">
         <v>22.315</v>
+      </c>
+      <c r="DL13" s="3" t="n">
+        <v>22.392</v>
       </c>
     </row>
     <row r="14">
@@ -12272,16 +12359,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.0915</v>
+        <v>37.8958</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>137419.123949</v>
+        <v>136713.1154548</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>37419.12394900003</v>
+        <v>36713.11545480002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3741912394900003</v>
+        <v>0.3671311545480002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -12594,6 +12681,9 @@
       </c>
       <c r="DK14" s="3" t="n">
         <v>38.0915</v>
+      </c>
+      <c r="DL14" s="3" t="n">
+        <v>37.8958</v>
       </c>
     </row>
     <row r="15">
@@ -12948,6 +13038,9 @@
       <c r="DK15" s="3" t="n">
         <v>11.51</v>
       </c>
+      <c r="DL15" s="3" t="n">
+        <v>11.51</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12972,16 +13065,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.2619</v>
+        <v>25.3304</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>144572.0348432</v>
+        <v>144964.0554112</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>44572.0348432</v>
+        <v>44964.05541120001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.445720348432</v>
+        <v>0.4496405541120001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -13294,6 +13387,9 @@
       </c>
       <c r="DK16" s="3" t="n">
         <v>25.2619</v>
+      </c>
+      <c r="DL16" s="3" t="n">
+        <v>25.3304</v>
       </c>
     </row>
     <row r="17">
@@ -13319,16 +13415,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.735</v>
+        <v>16.6951</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55326.86389499999</v>
+        <v>55194.9522207</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5326.863894999995</v>
+        <v>5194.952220699997</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1065372778999999</v>
+        <v>0.1038990444139999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -13641,6 +13737,9 @@
       </c>
       <c r="DK17" s="3" t="n">
         <v>16.735</v>
+      </c>
+      <c r="DL17" s="3" t="n">
+        <v>16.6951</v>
       </c>
     </row>
     <row r="18">
@@ -13666,16 +13765,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.66</v>
+        <v>46.98</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>88021.10375999998</v>
+        <v>88624.76327999998</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8021.103759999984</v>
+        <v>8624.763279999985</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1002637969999998</v>
+        <v>0.1078095409999998</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -13994,6 +14093,9 @@
       </c>
       <c r="DK18" s="3" t="n">
         <v>46.66</v>
+      </c>
+      <c r="DL18" s="3" t="n">
+        <v>46.98</v>
       </c>
     </row>
     <row r="19">
@@ -14019,16 +14121,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.0952</v>
+        <v>12.9141</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>189445.1941232</v>
+        <v>186825.2628006</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>39445.1941232</v>
+        <v>36825.2628006</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2629679608213333</v>
+        <v>0.245501752004</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -14341,6 +14443,9 @@
       </c>
       <c r="DK19" s="3" t="n">
         <v>13.0952</v>
+      </c>
+      <c r="DL19" s="3" t="n">
+        <v>12.9141</v>
       </c>
     </row>
     <row r="20">
@@ -14366,16 +14471,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.69</v>
+        <v>9.59</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>254418.73107</v>
+        <v>251793.15077</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>4418.73106999998</v>
+        <v>1793.150770000007</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.01767492427999992</v>
+        <v>0.00717260308000003</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -14694,6 +14799,9 @@
       </c>
       <c r="DK20" s="3" t="n">
         <v>9.69</v>
+      </c>
+      <c r="DL20" s="3" t="n">
+        <v>9.59</v>
       </c>
     </row>
     <row r="21">
@@ -14719,16 +14827,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>112.2782</v>
+        <v>112.015</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>170579.6658538</v>
+        <v>170179.796885</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>579.6658537999901</v>
+        <v>179.7968849999888</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.003409799139999942</v>
+        <v>0.001057628735294052</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -15047,6 +15155,9 @@
       </c>
       <c r="DK21" s="3" t="n">
         <v>112.2782</v>
+      </c>
+      <c r="DL21" s="3" t="n">
+        <v>112.015</v>
       </c>
     </row>
     <row r="22">
@@ -15072,16 +15183,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.707</v>
+        <v>43.607</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67066.64322</v>
+        <v>66913.19722</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7066.643219999998</v>
+        <v>6913.197220000002</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.117777387</v>
+        <v>0.1152199536666667</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -15394,6 +15505,9 @@
       </c>
       <c r="DK22" s="3" t="n">
         <v>43.707</v>
+      </c>
+      <c r="DL22" s="3" t="n">
+        <v>43.607</v>
       </c>
     </row>
     <row r="23">
@@ -15419,16 +15533,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.2613</v>
+        <v>62.4269</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>169130.7668271</v>
+        <v>169580.6137623</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>19130.76682710001</v>
+        <v>19580.61376230002</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1275384455140001</v>
+        <v>0.1305374250820002</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -15747,6 +15861,9 @@
       </c>
       <c r="DK23" s="3" t="n">
         <v>62.2613</v>
+      </c>
+      <c r="DL23" s="3" t="n">
+        <v>62.4269</v>
       </c>
     </row>
     <row r="24">
@@ -15772,16 +15889,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>26.2569</v>
+        <v>26.117</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>95401.4528634</v>
+        <v>94893.142162</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-4598.547136599998</v>
+        <v>-5106.857837999996</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.04598547136599998</v>
+        <v>-0.05106857837999997</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -16094,6 +16211,9 @@
       </c>
       <c r="DK24" s="3" t="n">
         <v>26.2569</v>
+      </c>
+      <c r="DL24" s="3" t="n">
+        <v>26.117</v>
       </c>
     </row>
     <row r="25">
@@ -16119,16 +16239,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.7622</v>
+        <v>12.6601</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>209576.6879228</v>
+        <v>207900.0350074</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>9576.687922799989</v>
+        <v>7900.035007399973</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.04788343961399994</v>
+        <v>0.03950017503699986</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -16444,6 +16564,9 @@
       </c>
       <c r="DK25" s="3" t="n">
         <v>12.7622</v>
+      </c>
+      <c r="DL25" s="3" t="n">
+        <v>12.6601</v>
       </c>
     </row>
     <row r="26">
@@ -16469,16 +16592,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.0326</v>
+        <v>10.8655</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>131748.164909</v>
+        <v>129752.7043325</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>21748.16490900001</v>
+        <v>19752.70433250001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1977105900818183</v>
+        <v>0.1795700393863638</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -16794,6 +16917,9 @@
       </c>
       <c r="DK26" s="3" t="n">
         <v>11.0326</v>
+      </c>
+      <c r="DL26" s="3" t="n">
+        <v>10.8655</v>
       </c>
     </row>
     <row r="27">
@@ -16819,16 +16945,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>69.0719</v>
+        <v>68.7615</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>111265.160834</v>
+        <v>110765.14989</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>1265.160833999995</v>
+        <v>765.149889999986</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.01150146212727268</v>
+        <v>0.006955908090908964</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -17147,6 +17273,9 @@
       </c>
       <c r="DK27" s="3" t="n">
         <v>69.0719</v>
+      </c>
+      <c r="DL27" s="3" t="n">
+        <v>68.7615</v>
       </c>
     </row>
     <row r="28">
@@ -17172,16 +17301,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>114.8816</v>
+        <v>114.3124</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>379874.0468112</v>
+        <v>377991.8976468</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-125.9531887999619</v>
+        <v>-2008.102353199967</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.0003314557599998998</v>
+        <v>-0.005284479876842019</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -17500,6 +17629,9 @@
       </c>
       <c r="DK28" s="3" t="n">
         <v>114.8816</v>
+      </c>
+      <c r="DL28" s="3" t="n">
+        <v>114.3124</v>
       </c>
     </row>
     <row r="29">
@@ -17525,16 +17657,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.1049</v>
+        <v>11.9835</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>116251.8644447</v>
+        <v>115085.9749005</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>16251.8644447</v>
+        <v>15085.97490049999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.162518644447</v>
+        <v>0.1508597490049999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -17847,6 +17979,9 @@
       </c>
       <c r="DK29" s="3" t="n">
         <v>12.1049</v>
+      </c>
+      <c r="DL29" s="3" t="n">
+        <v>11.9835</v>
       </c>
     </row>
     <row r="30">
@@ -17872,16 +18007,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.3078</v>
+        <v>17.2934</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>128006.0830158</v>
+        <v>127899.5826174</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>28006.0830158</v>
+        <v>27899.58261739998</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.280060830158</v>
+        <v>0.2789958261739998</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -18194,6 +18329,9 @@
       </c>
       <c r="DK30" s="3" t="n">
         <v>17.3078</v>
+      </c>
+      <c r="DL30" s="3" t="n">
+        <v>17.2934</v>
       </c>
     </row>
     <row r="31">
@@ -18219,16 +18357,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>403.933</v>
+        <v>401.5127</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>107478.49264</v>
+        <v>106834.499216</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>7478.492639999997</v>
+        <v>6834.499215999997</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.07478492639999997</v>
+        <v>0.06834499215999996</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -18544,6 +18682,9 @@
       </c>
       <c r="DK31" s="3" t="n">
         <v>403.933</v>
+      </c>
+      <c r="DL31" s="3" t="n">
+        <v>401.5127</v>
       </c>
     </row>
     <row r="32">
@@ -18569,16 +18710,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.76</v>
+        <v>10.69</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>227465.9696</v>
+        <v>225986.1724</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>27465.96959999998</v>
+        <v>25986.17239999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1373298479999999</v>
+        <v>0.1299308619999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -18897,6 +19038,9 @@
       </c>
       <c r="DK32" s="3" t="n">
         <v>10.76</v>
+      </c>
+      <c r="DL32" s="3" t="n">
+        <v>10.69</v>
       </c>
     </row>
     <row r="33">
@@ -18922,16 +19066,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.87</v>
+        <v>19.8</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>71206.9268</v>
+        <v>70956.072</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>11206.9268</v>
+        <v>10956.072</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1867821133333334</v>
+        <v>0.1826012</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -19244,6 +19388,9 @@
       </c>
       <c r="DK33" s="3" t="n">
         <v>19.87</v>
+      </c>
+      <c r="DL33" s="3" t="n">
+        <v>19.8</v>
       </c>
     </row>
     <row r="34">
@@ -19269,16 +19416,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>221.2707</v>
+        <v>219.4698</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>77783.5104417</v>
+        <v>77150.4382638</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-2216.489558300003</v>
+        <v>-2849.561736200005</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.02770611947875004</v>
+        <v>-0.03561952170250006</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -19594,6 +19741,9 @@
       </c>
       <c r="DK34" s="3" t="n">
         <v>221.2707</v>
+      </c>
+      <c r="DL34" s="3" t="n">
+        <v>219.4698</v>
       </c>
     </row>
     <row r="35">
@@ -19619,16 +19769,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.91</v>
+        <v>16.08</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>113524.57993</v>
+        <v>114737.60184</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>13524.57992999999</v>
+        <v>14737.60183999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1352457992999999</v>
+        <v>0.1473760183999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -19944,6 +20094,9 @@
       </c>
       <c r="DK35" s="3" t="n">
         <v>15.91</v>
+      </c>
+      <c r="DL35" s="3" t="n">
+        <v>16.08</v>
       </c>
     </row>
     <row r="36">
@@ -19969,16 +20122,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>386.9382</v>
+        <v>388.3981</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>180199.4413692</v>
+        <v>180879.3255586</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>30199.44136920001</v>
+        <v>30879.32555860002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.201329609128</v>
+        <v>0.2058621703906668</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -20294,6 +20447,9 @@
       </c>
       <c r="DK36" s="3" t="n">
         <v>386.9382</v>
+      </c>
+      <c r="DL36" s="3" t="n">
+        <v>388.3981</v>
       </c>
     </row>
     <row r="37">
@@ -20319,16 +20475,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.582</v>
+        <v>17.601</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>66159.11439800001</v>
+        <v>66230.609289</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>16159.11439800001</v>
+        <v>16230.609289</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.3231822879600001</v>
+        <v>0.32461218578</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -20644,6 +20800,9 @@
       </c>
       <c r="DK37" s="3" t="n">
         <v>17.582</v>
+      </c>
+      <c r="DL37" s="3" t="n">
+        <v>17.601</v>
       </c>
     </row>
     <row r="38">
@@ -20669,16 +20828,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.7834</v>
+        <v>13.6809</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>82431.3755988</v>
+        <v>81818.3761938</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>2431.375598800005</v>
+        <v>1818.376193799995</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.03039219498500006</v>
+        <v>0.02272970242249994</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -20991,6 +21150,9 @@
       </c>
       <c r="DK38" s="3" t="n">
         <v>13.7834</v>
+      </c>
+      <c r="DL38" s="3" t="n">
+        <v>13.6809</v>
       </c>
     </row>
     <row r="39">
@@ -21016,16 +21178,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.7643</v>
+        <v>1025.3573</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51166.1490483</v>
+        <v>51145.84748129999</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1166.149048300002</v>
+        <v>1145.847481299992</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02332298096600003</v>
+        <v>0.02291694962599984</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -21338,6 +21500,9 @@
       </c>
       <c r="DK39" s="3" t="n">
         <v>1025.7643</v>
+      </c>
+      <c r="DL39" s="3" t="n">
+        <v>1025.3573</v>
       </c>
     </row>
     <row r="40">
@@ -21363,16 +21528,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.1475</v>
+        <v>20.9922</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>106605.1184825</v>
+        <v>105822.2469894</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>6605.118482500009</v>
+        <v>5822.24698940001</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.06605118482500009</v>
+        <v>0.0582224698940001</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -21688,6 +21853,9 @@
       </c>
       <c r="DK40" s="3" t="n">
         <v>21.1475</v>
+      </c>
+      <c r="DL40" s="3" t="n">
+        <v>20.9922</v>
       </c>
     </row>
     <row r="41">
@@ -21700,13 +21868,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5036310.356807</v>
+        <v>5016567.8105559</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>566310.3568070001</v>
+        <v>546567.8105559</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1266913549903803</v>
+        <v>0.1222746779767114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-01
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-30 07:54 IST</t>
+          <t>Generated: 2026-10-01 08:16 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5016567.8105559</v>
+        <v>5009483.4415209</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>546567.8105558995</v>
+        <v>539483.4415208995</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1222746779767113</v>
+        <v>0.12068980794651</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>536298.5044937134</v>
+        <v>523712.0045166016</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-54483.51550628664</v>
+        <v>-67070.01548339846</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.09222270424933826</v>
+        <v>-0.1135275164322002</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5552866.315049613</v>
+        <v>5533195.446037501</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>492084.2950496133</v>
+        <v>472413.4260375015</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.0972348330959359</v>
+        <v>0.09334791029736973</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-09-30</t>
+          <t>Last snapshot: 2026-10-01</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EP19"/>
+  <dimension ref="A1:EQ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -765,6 +765,7 @@
     <col width="21" customWidth="1" min="144" max="144"/>
     <col width="21" customWidth="1" min="145" max="145"/>
     <col width="21" customWidth="1" min="146" max="146"/>
+    <col width="21" customWidth="1" min="147" max="147"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1498,6 +1499,11 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="EQ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1517,13 +1523,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>591.2000122070312</v>
+        <v>580.7000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47296.0009765625</v>
+        <v>46456.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3478.490976562498</v>
+        <v>2638.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1938,6 +1944,9 @@
       </c>
       <c r="EP2" s="3" t="n">
         <v>591.2000122070312</v>
+      </c>
+      <c r="EQ2" s="3" t="n">
+        <v>580.7000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -1985,13 +1994,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1379</v>
+        <v>1321.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27580</v>
+        <v>26436.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4524.580000000002</v>
+        <v>-5668.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2409,6 +2418,9 @@
       </c>
       <c r="EP4" s="3" t="n">
         <v>1379</v>
+      </c>
+      <c r="EQ4" s="3" t="n">
+        <v>1321.800048828125</v>
       </c>
     </row>
     <row r="5">
@@ -2429,13 +2441,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>525.5</v>
+        <v>500.6000061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>10510</v>
+        <v>10012.00012207031</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-3703.1</v>
+        <v>-4201.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2853,6 +2865,9 @@
       </c>
       <c r="EP5" s="3" t="n">
         <v>525.5</v>
+      </c>
+      <c r="EQ5" s="3" t="n">
+        <v>500.6000061035156</v>
       </c>
     </row>
     <row r="6">
@@ -2873,13 +2888,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>332.3500061035156</v>
+        <v>315</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13294.00024414062</v>
+        <v>12600</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4208.239755859377</v>
+        <v>-4902.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3297,6 +3312,9 @@
       </c>
       <c r="EP6" s="3" t="n">
         <v>332.3500061035156</v>
+      </c>
+      <c r="EQ6" s="3" t="n">
+        <v>315</v>
       </c>
     </row>
     <row r="7">
@@ -3317,13 +3335,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>312.25</v>
+        <v>306.5499877929688</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>31225</v>
+        <v>30654.99877929688</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4791.18</v>
+        <v>4221.178779296875</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3741,6 +3759,9 @@
       </c>
       <c r="EP7" s="3" t="n">
         <v>312.25</v>
+      </c>
+      <c r="EQ7" s="3" t="n">
+        <v>306.5499877929688</v>
       </c>
     </row>
     <row r="8">
@@ -3788,13 +3809,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.34000015258789</v>
+        <v>14.82999992370605</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23010.00022888184</v>
+        <v>22244.99988555908</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8040.169771118162</v>
+        <v>-8805.170114440916</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4212,6 +4233,9 @@
       </c>
       <c r="EP9" s="3" t="n">
         <v>15.34000015258789</v>
+      </c>
+      <c r="EQ9" s="3" t="n">
+        <v>14.82999992370605</v>
       </c>
     </row>
     <row r="10">
@@ -4232,13 +4256,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>450.4500122070312</v>
+        <v>437.2000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45045.00122070312</v>
+        <v>43720.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6453.478779296878</v>
+        <v>-7778.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4656,6 +4680,9 @@
       </c>
       <c r="EP10" s="3" t="n">
         <v>450.4500122070312</v>
+      </c>
+      <c r="EQ10" s="3" t="n">
+        <v>437.2000122070312</v>
       </c>
     </row>
     <row r="11">
@@ -4676,13 +4703,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>13.47000026702881</v>
+        <v>12.69999980926514</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>13470.00026702881</v>
+        <v>12699.99980926514</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3628.790267028809</v>
+        <v>2858.789809265138</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5100,6 +5127,9 @@
       </c>
       <c r="EP11" s="3" t="n">
         <v>13.47000026702881</v>
+      </c>
+      <c r="EQ11" s="3" t="n">
+        <v>12.69999980926514</v>
       </c>
     </row>
     <row r="12">
@@ -5120,13 +5150,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2760.60009765625</v>
+        <v>2591</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27606.0009765625</v>
+        <v>25910</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-117.2490234375</v>
+        <v>-1813.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5544,6 +5574,9 @@
       </c>
       <c r="EP12" s="3" t="n">
         <v>2760.60009765625</v>
+      </c>
+      <c r="EQ12" s="3" t="n">
+        <v>2591</v>
       </c>
     </row>
     <row r="13">
@@ -5564,13 +5597,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>39.77000045776367</v>
+        <v>38.5</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23862.0002746582</v>
+        <v>23100</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11169.7597253418</v>
+        <v>-11931.76</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -5988,6 +6021,9 @@
       </c>
       <c r="EP13" s="3" t="n">
         <v>39.77000045776367</v>
+      </c>
+      <c r="EQ13" s="3" t="n">
+        <v>38.5</v>
       </c>
     </row>
     <row r="14">
@@ -6008,13 +6044,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>617.9000244140625</v>
+        <v>602.4000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>30895.00122070312</v>
+        <v>30120.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11567.50877929688</v>
+        <v>-12342.50877929688</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6432,6 +6468,9 @@
       </c>
       <c r="EP14" s="3" t="n">
         <v>617.9000244140625</v>
+      </c>
+      <c r="EQ14" s="3" t="n">
+        <v>602.4000244140625</v>
       </c>
     </row>
     <row r="15">
@@ -6506,13 +6545,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>491.1000061035156</v>
+        <v>464.3500061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>24555.00030517578</v>
+        <v>23217.50030517578</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>2800.470305175782</v>
+        <v>1462.970305175782</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6930,6 +6969,9 @@
       </c>
       <c r="EP17" s="3" t="n">
         <v>491.1000061035156</v>
+      </c>
+      <c r="EQ17" s="3" t="n">
+        <v>464.3500061035156</v>
       </c>
     </row>
     <row r="18">
@@ -6950,13 +6992,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>361.7999877929688</v>
+        <v>347.7000122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>36179.99877929688</v>
+        <v>34770.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-10460.82122070312</v>
+        <v>-11870.81877929687</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7374,6 +7416,9 @@
       </c>
       <c r="EP18" s="3" t="n">
         <v>361.7999877929688</v>
+      </c>
+      <c r="EQ18" s="3" t="n">
+        <v>347.7000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -7386,10 +7431,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>536298.5044937134</v>
+        <v>523712.0045166016</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-54483.51550628663</v>
+        <v>-67070.01548339844</v>
       </c>
     </row>
   </sheetData>
@@ -7403,7 +7448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DL41"/>
+  <dimension ref="A1:DM41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7522,6 +7567,7 @@
     <col width="13" customWidth="1" min="114" max="114"/>
     <col width="13" customWidth="1" min="115" max="115"/>
     <col width="13" customWidth="1" min="116" max="116"/>
+    <col width="13" customWidth="1" min="117" max="117"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8105,6 +8151,11 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="DM1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8129,16 +8180,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.6679</v>
+        <v>57.4516</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64731.1797278</v>
+        <v>64488.3868712</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14731.1797278</v>
+        <v>14488.3868712</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.294623594556</v>
+        <v>0.2897677374239999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8460,6 +8511,9 @@
       </c>
       <c r="DL2" s="3" t="n">
         <v>57.6679</v>
+      </c>
+      <c r="DM2" s="3" t="n">
+        <v>57.4516</v>
       </c>
     </row>
     <row r="3">
@@ -8485,16 +8539,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.7769</v>
+        <v>26.814</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65742.99297970001</v>
+        <v>65834.081382</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5742.992979700008</v>
+        <v>5834.081382000004</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09571654966166679</v>
+        <v>0.09723468970000007</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8810,6 +8864,9 @@
       </c>
       <c r="DL3" s="3" t="n">
         <v>26.7769</v>
+      </c>
+      <c r="DM3" s="3" t="n">
+        <v>26.814</v>
       </c>
     </row>
     <row r="4">
@@ -8835,16 +8892,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.7</v>
+        <v>12.78</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>243917.3811</v>
+        <v>245453.86854</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>63917.3811</v>
+        <v>65453.86854</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3550965616666666</v>
+        <v>0.363632603</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9160,6 +9217,9 @@
       </c>
       <c r="DL4" s="3" t="n">
         <v>12.7</v>
+      </c>
+      <c r="DM4" s="3" t="n">
+        <v>12.78</v>
       </c>
     </row>
     <row r="5">
@@ -9185,16 +9245,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.998799999999999</v>
+        <v>9.01</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>165164.7670944</v>
+        <v>165370.33288</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-44835.23290560002</v>
+        <v>-44629.66712</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2135011090742858</v>
+        <v>-0.2125222243809524</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9510,6 +9570,9 @@
       </c>
       <c r="DL5" s="3" t="n">
         <v>8.998799999999999</v>
+      </c>
+      <c r="DM5" s="3" t="n">
+        <v>9.01</v>
       </c>
     </row>
     <row r="6">
@@ -9535,16 +9598,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.3464</v>
+        <v>11.3546</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>47983.66463279999</v>
+        <v>48018.34224419999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-2016.335367200008</v>
+        <v>-1981.657755800006</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.04032670734400017</v>
+        <v>-0.03963315511600012</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9866,6 +9929,9 @@
       </c>
       <c r="DL6" s="3" t="n">
         <v>11.3464</v>
+      </c>
+      <c r="DM6" s="3" t="n">
+        <v>11.3546</v>
       </c>
     </row>
     <row r="7">
@@ -9891,16 +9957,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.4078</v>
+        <v>34.2265</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75904.983112</v>
+        <v>75505.02806</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15904.983112</v>
+        <v>15505.02806</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2650830518666667</v>
+        <v>0.2584171343333333</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -10216,6 +10282,9 @@
       </c>
       <c r="DL7" s="3" t="n">
         <v>34.4078</v>
+      </c>
+      <c r="DM7" s="3" t="n">
+        <v>34.2265</v>
       </c>
     </row>
     <row r="8">
@@ -10241,16 +10310,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.5494</v>
+        <v>35.4815</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57042.3183942</v>
+        <v>56933.3665295</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7042.318394200003</v>
+        <v>6933.366529499996</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1408463678840001</v>
+        <v>0.1386673305899999</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -10572,6 +10641,9 @@
       </c>
       <c r="DL8" s="3" t="n">
         <v>35.5494</v>
+      </c>
+      <c r="DM8" s="3" t="n">
+        <v>35.4815</v>
       </c>
     </row>
     <row r="9">
@@ -10597,16 +10669,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.8901</v>
+        <v>42.322</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>134860.6947093</v>
+        <v>136251.150546</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>34860.69470930001</v>
+        <v>36251.15054600002</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3486069470930001</v>
+        <v>0.3625115054600002</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10922,6 +10994,9 @@
       </c>
       <c r="DL9" s="3" t="n">
         <v>41.8901</v>
+      </c>
+      <c r="DM9" s="3" t="n">
+        <v>42.322</v>
       </c>
     </row>
     <row r="10">
@@ -10947,16 +11022,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.3434</v>
+        <v>48.3981</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>137617.1747006</v>
+        <v>137772.8869479</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>37617.17470060001</v>
+        <v>37772.8869479</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3761717470060001</v>
+        <v>0.377728869479</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -11272,6 +11347,9 @@
       </c>
       <c r="DL10" s="3" t="n">
         <v>48.3434</v>
+      </c>
+      <c r="DM10" s="3" t="n">
+        <v>48.3981</v>
       </c>
     </row>
     <row r="11">
@@ -11297,16 +11375,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.326</v>
+        <v>107.1959</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32296.43259399999</v>
+        <v>32257.2830321</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2296.432593999994</v>
+        <v>2257.283032099996</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07654775313333315</v>
+        <v>0.07524276773666655</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -11622,6 +11700,9 @@
       </c>
       <c r="DL11" s="3" t="n">
         <v>107.326</v>
+      </c>
+      <c r="DM11" s="3" t="n">
+        <v>107.1959</v>
       </c>
     </row>
     <row r="12">
@@ -11647,16 +11728,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>221.354</v>
+        <v>220.579</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>103045.156788</v>
+        <v>102684.377238</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3045.156788000008</v>
+        <v>2684.377238000001</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.03045156788000008</v>
+        <v>0.02684377238000001</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -11978,6 +12059,9 @@
       </c>
       <c r="DL12" s="3" t="n">
         <v>221.354</v>
+      </c>
+      <c r="DM12" s="3" t="n">
+        <v>220.579</v>
       </c>
     </row>
     <row r="13">
@@ -12003,16 +12087,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22.392</v>
+        <v>21.944</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>259469.65116</v>
+        <v>254278.40412</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>59469.65115999998</v>
+        <v>54278.40411999999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2973482557999999</v>
+        <v>0.2713920206</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -12334,6 +12418,9 @@
       </c>
       <c r="DL13" s="3" t="n">
         <v>22.392</v>
+      </c>
+      <c r="DM13" s="3" t="n">
+        <v>21.944</v>
       </c>
     </row>
     <row r="14">
@@ -12359,16 +12446,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.8958</v>
+        <v>37.8428</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>136713.1154548</v>
+        <v>136521.9123368</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>36713.11545480002</v>
+        <v>36521.91233679999</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3671311545480002</v>
+        <v>0.3652191233679998</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -12684,6 +12771,9 @@
       </c>
       <c r="DL14" s="3" t="n">
         <v>37.8958</v>
+      </c>
+      <c r="DM14" s="3" t="n">
+        <v>37.8428</v>
       </c>
     </row>
     <row r="15">
@@ -13041,6 +13131,9 @@
       <c r="DL15" s="3" t="n">
         <v>11.51</v>
       </c>
+      <c r="DM15" s="3" t="n">
+        <v>11.51</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13065,16 +13158,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.3304</v>
+        <v>25.3753</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>144964.0554112</v>
+        <v>145221.0148784</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>44964.05541120001</v>
+        <v>45221.01487839999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4496405541120001</v>
+        <v>0.4522101487839999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -13390,6 +13483,9 @@
       </c>
       <c r="DL16" s="3" t="n">
         <v>25.3304</v>
+      </c>
+      <c r="DM16" s="3" t="n">
+        <v>25.3753</v>
       </c>
     </row>
     <row r="17">
@@ -13415,16 +13511,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6951</v>
+        <v>16.6963</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55194.9522207</v>
+        <v>55198.9194891</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5194.952220699997</v>
+        <v>5198.919489100001</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1038990444139999</v>
+        <v>0.103978389782</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -13740,6 +13836,9 @@
       </c>
       <c r="DL17" s="3" t="n">
         <v>16.6951</v>
+      </c>
+      <c r="DM17" s="3" t="n">
+        <v>16.6963</v>
       </c>
     </row>
     <row r="18">
@@ -13765,16 +13864,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.98</v>
+        <v>46.11</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>88624.76327999998</v>
+        <v>86983.56396</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8624.763279999985</v>
+        <v>6983.563959999999</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1078095409999998</v>
+        <v>0.0872945495</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -14096,6 +14195,9 @@
       </c>
       <c r="DL18" s="3" t="n">
         <v>46.98</v>
+      </c>
+      <c r="DM18" s="3" t="n">
+        <v>46.11</v>
       </c>
     </row>
     <row r="19">
@@ -14121,16 +14223,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>12.9141</v>
+        <v>13.1103</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>186825.2628006</v>
+        <v>189663.6422898</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>36825.2628006</v>
+        <v>39663.64228980002</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.245501752004</v>
+        <v>0.2644242819320001</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -14446,6 +14548,9 @@
       </c>
       <c r="DL19" s="3" t="n">
         <v>12.9141</v>
+      </c>
+      <c r="DM19" s="3" t="n">
+        <v>13.1103</v>
       </c>
     </row>
     <row r="20">
@@ -14471,16 +14576,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.59</v>
+        <v>9.58</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>251793.15077</v>
+        <v>251530.59274</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>1793.150770000007</v>
+        <v>1530.592739999993</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.00717260308000003</v>
+        <v>0.006122370959999971</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -14802,6 +14907,9 @@
       </c>
       <c r="DL20" s="3" t="n">
         <v>9.59</v>
+      </c>
+      <c r="DM20" s="3" t="n">
+        <v>9.58</v>
       </c>
     </row>
     <row r="21">
@@ -14827,16 +14935,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>112.015</v>
+        <v>111.9738</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>170179.796885</v>
+        <v>170117.2034142</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>179.7968849999888</v>
+        <v>117.2034141999902</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.001057628735294052</v>
+        <v>0.0006894318482352366</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -15158,6 +15266,9 @@
       </c>
       <c r="DL21" s="3" t="n">
         <v>112.015</v>
+      </c>
+      <c r="DM21" s="3" t="n">
+        <v>111.9738</v>
       </c>
     </row>
     <row r="22">
@@ -15183,16 +15294,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.607</v>
+        <v>43.599</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>66913.19722</v>
+        <v>66900.92154</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>6913.197220000002</v>
+        <v>6900.921539999996</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1152199536666667</v>
+        <v>0.1150153589999999</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -15508,6 +15619,9 @@
       </c>
       <c r="DL22" s="3" t="n">
         <v>43.607</v>
+      </c>
+      <c r="DM22" s="3" t="n">
+        <v>43.599</v>
       </c>
     </row>
     <row r="23">
@@ -15533,16 +15647,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.4269</v>
+        <v>62.3712</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>169580.6137623</v>
+        <v>169429.3065504</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>19580.61376230002</v>
+        <v>19429.30655040001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1305374250820002</v>
+        <v>0.1295287103360001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -15864,6 +15978,9 @@
       </c>
       <c r="DL23" s="3" t="n">
         <v>62.4269</v>
+      </c>
+      <c r="DM23" s="3" t="n">
+        <v>62.3712</v>
       </c>
     </row>
     <row r="24">
@@ -15889,16 +16006,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>26.117</v>
+        <v>26.1358</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>94893.142162</v>
+        <v>94961.4498188</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-5106.857837999996</v>
+        <v>-5038.5501812</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.05106857837999997</v>
+        <v>-0.050385501812</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -16214,6 +16331,9 @@
       </c>
       <c r="DL24" s="3" t="n">
         <v>26.117</v>
+      </c>
+      <c r="DM24" s="3" t="n">
+        <v>26.1358</v>
       </c>
     </row>
     <row r="25">
@@ -16239,16 +16359,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.6601</v>
+        <v>12.6132</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>207900.0350074</v>
+        <v>207129.8584968</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>7900.035007399973</v>
+        <v>7129.858496800007</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.03950017503699986</v>
+        <v>0.03564929248400003</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -16567,6 +16687,9 @@
       </c>
       <c r="DL25" s="3" t="n">
         <v>12.6601</v>
+      </c>
+      <c r="DM25" s="3" t="n">
+        <v>12.6132</v>
       </c>
     </row>
     <row r="26">
@@ -16592,16 +16715,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.8655</v>
+        <v>10.7949</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>129752.7043325</v>
+        <v>128909.6192535</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>19752.70433250001</v>
+        <v>18909.6192535</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1795700393863638</v>
+        <v>0.1719056295772727</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -16920,6 +17043,9 @@
       </c>
       <c r="DL26" s="3" t="n">
         <v>10.8655</v>
+      </c>
+      <c r="DM26" s="3" t="n">
+        <v>10.7949</v>
       </c>
     </row>
     <row r="27">
@@ -16945,16 +17071,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>68.7615</v>
+        <v>68.7773</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>110765.14989</v>
+        <v>110790.601478</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>765.149889999986</v>
+        <v>790.6014779999823</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.006955908090908964</v>
+        <v>0.007187286163636203</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -17276,6 +17402,9 @@
       </c>
       <c r="DL27" s="3" t="n">
         <v>68.7615</v>
+      </c>
+      <c r="DM27" s="3" t="n">
+        <v>68.7773</v>
       </c>
     </row>
     <row r="28">
@@ -17301,16 +17430,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>114.3124</v>
+        <v>114.3619</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>377991.8976468</v>
+        <v>378155.5771683</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-2008.102353199967</v>
+        <v>-1844.422831699951</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.005284479876842019</v>
+        <v>-0.004853744293947238</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -17632,6 +17761,9 @@
       </c>
       <c r="DL28" s="3" t="n">
         <v>114.3124</v>
+      </c>
+      <c r="DM28" s="3" t="n">
+        <v>114.3619</v>
       </c>
     </row>
     <row r="29">
@@ -17657,16 +17789,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.9835</v>
+        <v>12.1564</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>115085.9749005</v>
+        <v>116746.4551492</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>15085.97490049999</v>
+        <v>16746.45514919999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1508597490049999</v>
+        <v>0.1674645514919999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -17982,6 +18114,9 @@
       </c>
       <c r="DL29" s="3" t="n">
         <v>11.9835</v>
+      </c>
+      <c r="DM29" s="3" t="n">
+        <v>12.1564</v>
       </c>
     </row>
     <row r="30">
@@ -18007,16 +18142,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.2934</v>
+        <v>17.3415</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>127899.5826174</v>
+        <v>128255.3235315</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>27899.58261739998</v>
+        <v>28255.32353149999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2789958261739998</v>
+        <v>0.2825532353149999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -18332,6 +18467,9 @@
       </c>
       <c r="DL30" s="3" t="n">
         <v>17.2934</v>
+      </c>
+      <c r="DM30" s="3" t="n">
+        <v>17.3415</v>
       </c>
     </row>
     <row r="31">
@@ -18357,16 +18495,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>401.5127</v>
+        <v>402.9319</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>106834.499216</v>
+        <v>107212.119952</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>6834.499215999997</v>
+        <v>7212.119951999994</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.06834499215999996</v>
+        <v>0.07212119951999994</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -18685,6 +18823,9 @@
       </c>
       <c r="DL31" s="3" t="n">
         <v>401.5127</v>
+      </c>
+      <c r="DM31" s="3" t="n">
+        <v>402.9319</v>
       </c>
     </row>
     <row r="32">
@@ -19042,6 +19183,9 @@
       <c r="DL32" s="3" t="n">
         <v>10.69</v>
       </c>
+      <c r="DM32" s="3" t="n">
+        <v>10.69</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -19392,6 +19536,9 @@
       <c r="DL33" s="3" t="n">
         <v>19.8</v>
       </c>
+      <c r="DM33" s="3" t="n">
+        <v>19.8</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -19416,16 +19563,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>219.4698</v>
+        <v>219.0788</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>77150.4382638</v>
+        <v>77012.98964280001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-2849.561736200005</v>
+        <v>-2987.010357199993</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.03561952170250006</v>
+        <v>-0.03733762946499992</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -19744,6 +19891,9 @@
       </c>
       <c r="DL34" s="3" t="n">
         <v>219.4698</v>
+      </c>
+      <c r="DM34" s="3" t="n">
+        <v>219.0788</v>
       </c>
     </row>
     <row r="35">
@@ -19769,16 +19919,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.08</v>
+        <v>16.09</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>114737.60184</v>
+        <v>114808.95607</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>14737.60183999999</v>
+        <v>14808.95607</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1473760183999999</v>
+        <v>0.1480895607</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -20097,6 +20247,9 @@
       </c>
       <c r="DL35" s="3" t="n">
         <v>16.08</v>
+      </c>
+      <c r="DM35" s="3" t="n">
+        <v>16.09</v>
       </c>
     </row>
     <row r="36">
@@ -20122,16 +20275,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>388.3981</v>
+        <v>379.8786</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>180879.3255586</v>
+        <v>176911.7432916</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>30879.32555860002</v>
+        <v>26911.7432916</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.2058621703906668</v>
+        <v>0.179411621944</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -20450,6 +20603,9 @@
       </c>
       <c r="DL36" s="3" t="n">
         <v>388.3981</v>
+      </c>
+      <c r="DM36" s="3" t="n">
+        <v>379.8786</v>
       </c>
     </row>
     <row r="37">
@@ -20475,16 +20631,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.601</v>
+        <v>17.282</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>66230.609289</v>
+        <v>65030.247698</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>16230.609289</v>
+        <v>15030.247698</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.32461218578</v>
+        <v>0.30060495396</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -20803,6 +20959,9 @@
       </c>
       <c r="DL37" s="3" t="n">
         <v>17.601</v>
+      </c>
+      <c r="DM37" s="3" t="n">
+        <v>17.282</v>
       </c>
     </row>
     <row r="38">
@@ -20828,16 +20987,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.6809</v>
+        <v>13.6677</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>81818.3761938</v>
+        <v>81739.43383140001</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1818.376193799995</v>
+        <v>1739.433831400005</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.02272970242249994</v>
+        <v>0.02174292289250006</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -21153,6 +21312,9 @@
       </c>
       <c r="DL38" s="3" t="n">
         <v>13.6809</v>
+      </c>
+      <c r="DM38" s="3" t="n">
+        <v>13.6677</v>
       </c>
     </row>
     <row r="39">
@@ -21178,16 +21340,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.3573</v>
+        <v>1026.2097</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51145.84748129999</v>
+        <v>51188.36604570001</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1145.847481299992</v>
+        <v>1188.366045700008</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02291694962599984</v>
+        <v>0.02376732091400015</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -21503,6 +21665,9 @@
       </c>
       <c r="DL39" s="3" t="n">
         <v>1025.3573</v>
+      </c>
+      <c r="DM39" s="3" t="n">
+        <v>1026.2097</v>
       </c>
     </row>
     <row r="40">
@@ -21528,16 +21693,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.9922</v>
+        <v>20.8531</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>105822.2469894</v>
+        <v>105121.0401337</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>5822.24698940001</v>
+        <v>5121.040133700008</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.0582224698940001</v>
+        <v>0.05121040133700008</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -21856,6 +22021,9 @@
       </c>
       <c r="DL40" s="3" t="n">
         <v>20.9922</v>
+      </c>
+      <c r="DM40" s="3" t="n">
+        <v>20.8531</v>
       </c>
     </row>
     <row r="41">
@@ -21868,13 +22036,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5016567.8105559</v>
+        <v>5009483.4415209</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>546567.8105559</v>
+        <v>539483.4415209</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1222746779767114</v>
+        <v>0.1206898079465101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-02
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,9 +483,9 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-01 08:16 IST</t>
+          <t>Generated: 2026-10-02 07:54 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5009483.4415209</v>
+        <v>4984005.7749113</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>539483.4415208995</v>
+        <v>514005.7749113003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.12068980794651</v>
+        <v>0.1149901062441388</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>523712.0045166016</v>
+        <v>527793.0008010864</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-67070.01548339846</v>
+        <v>-62989.01919891359</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1135275164322002</v>
+        <v>-0.1066197295559428</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5533195.446037501</v>
+        <v>5511798.775712387</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>472413.4260375015</v>
+        <v>451016.7557123872</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09334791029736973</v>
+        <v>0.08911997274926835</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-01</t>
+          <t>Last snapshot: 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EQ19"/>
+  <dimension ref="A1:ER19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -766,6 +766,7 @@
     <col width="21" customWidth="1" min="145" max="145"/>
     <col width="21" customWidth="1" min="146" max="146"/>
     <col width="21" customWidth="1" min="147" max="147"/>
+    <col width="21" customWidth="1" min="148" max="148"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1504,6 +1505,11 @@
           <t>2026-10-01</t>
         </is>
       </c>
+      <c r="ER1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1523,13 +1529,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>580.7000122070312</v>
+        <v>586</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46456.0009765625</v>
+        <v>46880</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2638.490976562498</v>
+        <v>3062.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1947,6 +1953,9 @@
       </c>
       <c r="EQ2" s="3" t="n">
         <v>580.7000122070312</v>
+      </c>
+      <c r="ER2" s="3" t="n">
+        <v>586</v>
       </c>
     </row>
     <row r="3">
@@ -1994,13 +2003,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1321.800048828125</v>
+        <v>1344</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>26436.0009765625</v>
+        <v>26880</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5668.579023437502</v>
+        <v>-5224.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2421,6 +2430,9 @@
       </c>
       <c r="EQ4" s="3" t="n">
         <v>1321.800048828125</v>
+      </c>
+      <c r="ER4" s="3" t="n">
+        <v>1344</v>
       </c>
     </row>
     <row r="5">
@@ -2441,13 +2453,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>500.6000061035156</v>
+        <v>503.2999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>10012.00012207031</v>
+        <v>10065.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4201.099877929688</v>
+        <v>-4147.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2868,6 +2880,9 @@
       </c>
       <c r="EQ5" s="3" t="n">
         <v>500.6000061035156</v>
+      </c>
+      <c r="ER5" s="3" t="n">
+        <v>503.2999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -2888,13 +2903,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>315</v>
+        <v>326.7000122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12600</v>
+        <v>13068.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4902.240000000002</v>
+        <v>-4434.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3315,6 +3330,9 @@
       </c>
       <c r="EQ6" s="3" t="n">
         <v>315</v>
+      </c>
+      <c r="ER6" s="3" t="n">
+        <v>326.7000122070312</v>
       </c>
     </row>
     <row r="7">
@@ -3335,13 +3353,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>306.5499877929688</v>
+        <v>312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>30654.99877929688</v>
+        <v>31200</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4221.178779296875</v>
+        <v>4766.18</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3762,6 +3780,9 @@
       </c>
       <c r="EQ7" s="3" t="n">
         <v>306.5499877929688</v>
+      </c>
+      <c r="ER7" s="3" t="n">
+        <v>312</v>
       </c>
     </row>
     <row r="8">
@@ -3809,13 +3830,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.82999992370605</v>
+        <v>14.85000038146973</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22244.99988555908</v>
+        <v>22275.00057220459</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8805.170114440916</v>
+        <v>-8775.169427795408</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4236,6 +4257,9 @@
       </c>
       <c r="EQ9" s="3" t="n">
         <v>14.82999992370605</v>
+      </c>
+      <c r="ER9" s="3" t="n">
+        <v>14.85000038146973</v>
       </c>
     </row>
     <row r="10">
@@ -4256,13 +4280,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>437.2000122070312</v>
+        <v>444</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>43720.00122070312</v>
+        <v>44400</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-7778.478779296878</v>
+        <v>-7098.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4683,6 +4707,9 @@
       </c>
       <c r="EQ10" s="3" t="n">
         <v>437.2000122070312</v>
+      </c>
+      <c r="ER10" s="3" t="n">
+        <v>444</v>
       </c>
     </row>
     <row r="11">
@@ -4703,13 +4730,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12.69999980926514</v>
+        <v>12.92000007629395</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>12699.99980926514</v>
+        <v>12920.00007629395</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2858.789809265138</v>
+        <v>3078.790076293946</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5130,6 +5157,9 @@
       </c>
       <c r="EQ11" s="3" t="n">
         <v>12.69999980926514</v>
+      </c>
+      <c r="ER11" s="3" t="n">
+        <v>12.92000007629395</v>
       </c>
     </row>
     <row r="12">
@@ -5150,13 +5180,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2591</v>
+        <v>2620</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25910</v>
+        <v>26200</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1813.25</v>
+        <v>-1523.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5577,6 +5607,9 @@
       </c>
       <c r="EQ12" s="3" t="n">
         <v>2591</v>
+      </c>
+      <c r="ER12" s="3" t="n">
+        <v>2620</v>
       </c>
     </row>
     <row r="13">
@@ -5597,13 +5630,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>38.5</v>
+        <v>38.90999984741211</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23100</v>
+        <v>23345.99990844727</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11931.76</v>
+        <v>-11685.76009155274</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6024,6 +6057,9 @@
       </c>
       <c r="EQ13" s="3" t="n">
         <v>38.5</v>
+      </c>
+      <c r="ER13" s="3" t="n">
+        <v>38.90999984741211</v>
       </c>
     </row>
     <row r="14">
@@ -6044,13 +6080,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>602.4000244140625</v>
+        <v>608.4500122070312</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>30120.00122070312</v>
+        <v>30422.50061035156</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12342.50877929688</v>
+        <v>-12040.00938964844</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6471,6 +6507,9 @@
       </c>
       <c r="EQ14" s="3" t="n">
         <v>602.4000244140625</v>
+      </c>
+      <c r="ER14" s="3" t="n">
+        <v>608.4500122070312</v>
       </c>
     </row>
     <row r="15">
@@ -6545,13 +6584,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>464.3500061035156</v>
+        <v>467</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23217.50030517578</v>
+        <v>23350</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1462.970305175782</v>
+        <v>1595.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -6972,6 +7011,9 @@
       </c>
       <c r="EQ17" s="3" t="n">
         <v>464.3500061035156</v>
+      </c>
+      <c r="ER17" s="3" t="n">
+        <v>467</v>
       </c>
     </row>
     <row r="18">
@@ -6992,13 +7034,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>347.7000122070312</v>
+        <v>350.1499938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34770.00122070312</v>
+        <v>35014.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11870.81877929687</v>
+        <v>-11625.82061035156</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7419,6 +7461,9 @@
       </c>
       <c r="EQ18" s="3" t="n">
         <v>347.7000122070312</v>
+      </c>
+      <c r="ER18" s="3" t="n">
+        <v>350.1499938964844</v>
       </c>
     </row>
     <row r="19">
@@ -7431,10 +7476,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>523712.0045166016</v>
+        <v>527793.0008010864</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-67070.01548339844</v>
+        <v>-62989.01919891359</v>
       </c>
     </row>
   </sheetData>
@@ -7448,7 +7493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DM41"/>
+  <dimension ref="A1:DN41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7568,6 +7613,7 @@
     <col width="13" customWidth="1" min="115" max="115"/>
     <col width="13" customWidth="1" min="116" max="116"/>
     <col width="13" customWidth="1" min="117" max="117"/>
+    <col width="13" customWidth="1" min="118" max="118"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8156,6 +8202,11 @@
           <t>2026-10-01</t>
         </is>
       </c>
+      <c r="DN1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8180,16 +8231,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.4516</v>
+        <v>57.8202</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64488.3868712</v>
+        <v>64902.1337364</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14488.3868712</v>
+        <v>14902.1337364</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2897677374239999</v>
+        <v>0.298042674728</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8514,6 +8565,9 @@
       </c>
       <c r="DM2" s="3" t="n">
         <v>57.4516</v>
+      </c>
+      <c r="DN2" s="3" t="n">
+        <v>57.8202</v>
       </c>
     </row>
     <row r="3">
@@ -8539,16 +8593,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.814</v>
+        <v>26.6767</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65834.081382</v>
+        <v>65496.98063710001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5834.081382000004</v>
+        <v>5496.980637100009</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09723468970000007</v>
+        <v>0.0916163439516668</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -8867,6 +8921,9 @@
       </c>
       <c r="DM3" s="3" t="n">
         <v>26.814</v>
+      </c>
+      <c r="DN3" s="3" t="n">
+        <v>26.6767</v>
       </c>
     </row>
     <row r="4">
@@ -9221,6 +9278,9 @@
       <c r="DM4" s="3" t="n">
         <v>12.78</v>
       </c>
+      <c r="DN4" s="3" t="n">
+        <v>12.78</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9245,16 +9305,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.01</v>
+        <v>8.9436</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>165370.33288</v>
+        <v>164151.6214368</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-44629.66712</v>
+        <v>-45848.37856320001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2125222243809524</v>
+        <v>-0.2183256122057143</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9573,6 +9633,9 @@
       </c>
       <c r="DM5" s="3" t="n">
         <v>9.01</v>
+      </c>
+      <c r="DN5" s="3" t="n">
+        <v>8.9436</v>
       </c>
     </row>
     <row r="6">
@@ -9598,16 +9661,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.3546</v>
+        <v>11.2513</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>48018.34224419999</v>
+        <v>47581.4889201</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-1981.657755800006</v>
+        <v>-2418.511079899996</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.03963315511600012</v>
+        <v>-0.04837022159799992</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -9932,6 +9995,9 @@
       </c>
       <c r="DM6" s="3" t="n">
         <v>11.3546</v>
+      </c>
+      <c r="DN6" s="3" t="n">
+        <v>11.2513</v>
       </c>
     </row>
     <row r="7">
@@ -9957,16 +10023,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.2265</v>
+        <v>33.7773</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75505.02806</v>
+        <v>74514.07489199999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15505.02806</v>
+        <v>14514.07489199999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2584171343333333</v>
+        <v>0.2419012481999998</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -10285,6 +10351,9 @@
       </c>
       <c r="DM7" s="3" t="n">
         <v>34.2265</v>
+      </c>
+      <c r="DN7" s="3" t="n">
+        <v>33.7773</v>
       </c>
     </row>
     <row r="8">
@@ -10310,16 +10379,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.4815</v>
+        <v>35.2788</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>56933.3665295</v>
+        <v>56608.1155284</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6933.366529499996</v>
+        <v>6608.115528399998</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1386673305899999</v>
+        <v>0.132162310568</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -10644,6 +10713,9 @@
       </c>
       <c r="DM8" s="3" t="n">
         <v>35.4815</v>
+      </c>
+      <c r="DN8" s="3" t="n">
+        <v>35.2788</v>
       </c>
     </row>
     <row r="9">
@@ -10669,16 +10741,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.322</v>
+        <v>42.5363</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>136251.150546</v>
+        <v>136941.0664659</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>36251.15054600002</v>
+        <v>36941.06646589999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3625115054600002</v>
+        <v>0.3694106646589999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -10997,6 +11069,9 @@
       </c>
       <c r="DM9" s="3" t="n">
         <v>42.322</v>
+      </c>
+      <c r="DN9" s="3" t="n">
+        <v>42.5363</v>
       </c>
     </row>
     <row r="10">
@@ -11022,16 +11097,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.3981</v>
+        <v>47.8409</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>137772.8869479</v>
+        <v>136186.7285531</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>37772.8869479</v>
+        <v>36186.72855309999</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.377728869479</v>
+        <v>0.3618672855309999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -11350,6 +11425,9 @@
       </c>
       <c r="DM10" s="3" t="n">
         <v>48.3981</v>
+      </c>
+      <c r="DN10" s="3" t="n">
+        <v>47.8409</v>
       </c>
     </row>
     <row r="11">
@@ -11375,16 +11453,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.1959</v>
+        <v>108.1355</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32257.2830321</v>
+        <v>32540.0265245</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2257.283032099996</v>
+        <v>2540.026524499997</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07524276773666655</v>
+        <v>0.08466755081666658</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -11703,6 +11781,9 @@
       </c>
       <c r="DM11" s="3" t="n">
         <v>107.1959</v>
+      </c>
+      <c r="DN11" s="3" t="n">
+        <v>108.1355</v>
       </c>
     </row>
     <row r="12">
@@ -11728,16 +11809,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.579</v>
+        <v>219.441</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102684.377238</v>
+        <v>102154.613202</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2684.377238000001</v>
+        <v>2154.613201999993</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02684377238000001</v>
+        <v>0.02154613201999993</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -12062,6 +12143,9 @@
       </c>
       <c r="DM12" s="3" t="n">
         <v>220.579</v>
+      </c>
+      <c r="DN12" s="3" t="n">
+        <v>219.441</v>
       </c>
     </row>
     <row r="13">
@@ -12087,16 +12171,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.944</v>
+        <v>21.979</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>254278.40412</v>
+        <v>254683.970295</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>54278.40411999999</v>
+        <v>54683.97029499998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2713920206</v>
+        <v>0.2734198514749999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -12421,6 +12505,9 @@
       </c>
       <c r="DM13" s="3" t="n">
         <v>21.944</v>
+      </c>
+      <c r="DN13" s="3" t="n">
+        <v>21.979</v>
       </c>
     </row>
     <row r="14">
@@ -12775,6 +12862,9 @@
       <c r="DM14" s="3" t="n">
         <v>37.8428</v>
       </c>
+      <c r="DN14" s="3" t="n">
+        <v>37.8428</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12799,16 +12889,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.51</v>
+        <v>11.4</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>112152.82997</v>
+        <v>111080.9958</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>12152.82997000001</v>
+        <v>11080.9958</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1215282997000001</v>
+        <v>0.110809958</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -13133,6 +13223,9 @@
       </c>
       <c r="DM15" s="3" t="n">
         <v>11.51</v>
+      </c>
+      <c r="DN15" s="3" t="n">
+        <v>11.4</v>
       </c>
     </row>
     <row r="16">
@@ -13158,16 +13251,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.3753</v>
+        <v>25.455</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>145221.0148784</v>
+        <v>145677.13224</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>45221.01487839999</v>
+        <v>45677.13223999998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4522101487839999</v>
+        <v>0.4567713223999998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -13486,6 +13579,9 @@
       </c>
       <c r="DM16" s="3" t="n">
         <v>25.3753</v>
+      </c>
+      <c r="DN16" s="3" t="n">
+        <v>25.455</v>
       </c>
     </row>
     <row r="17">
@@ -13511,16 +13607,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6963</v>
+        <v>16.6081</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55198.9194891</v>
+        <v>54907.3252617</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5198.919489100001</v>
+        <v>4907.325261699996</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.103978389782</v>
+        <v>0.09814650523399993</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -13839,6 +13935,9 @@
       </c>
       <c r="DM17" s="3" t="n">
         <v>16.6963</v>
+      </c>
+      <c r="DN17" s="3" t="n">
+        <v>16.6081</v>
       </c>
     </row>
     <row r="18">
@@ -13864,16 +13963,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.11</v>
+        <v>45.92</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>86983.56396</v>
+        <v>86625.14112</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>6983.563959999999</v>
+        <v>6625.14112</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.0872945495</v>
+        <v>0.082814264</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -14198,6 +14297,9 @@
       </c>
       <c r="DM18" s="3" t="n">
         <v>46.11</v>
+      </c>
+      <c r="DN18" s="3" t="n">
+        <v>45.92</v>
       </c>
     </row>
     <row r="19">
@@ -14223,16 +14325,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.1103</v>
+        <v>13.3046</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>189663.6422898</v>
+        <v>192474.5349236</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>39663.64228980002</v>
+        <v>42474.5349236</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2644242819320001</v>
+        <v>0.2831635661573333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -14551,6 +14653,9 @@
       </c>
       <c r="DM19" s="3" t="n">
         <v>13.1103</v>
+      </c>
+      <c r="DN19" s="3" t="n">
+        <v>13.3046</v>
       </c>
     </row>
     <row r="20">
@@ -14911,6 +15016,9 @@
       <c r="DM20" s="3" t="n">
         <v>9.58</v>
       </c>
+      <c r="DN20" s="3" t="n">
+        <v>9.58</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -14935,16 +15043,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.9738</v>
+        <v>110.6902</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>170117.2034142</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>117.2034141999902</v>
-      </c>
-      <c r="I21" s="12" t="n">
-        <v>0.0006894318482352366</v>
+        <v>168167.0825618</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>-1832.917438200006</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>-0.01078186728352945</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -15269,6 +15377,9 @@
       </c>
       <c r="DM21" s="3" t="n">
         <v>111.9738</v>
+      </c>
+      <c r="DN21" s="3" t="n">
+        <v>110.6902</v>
       </c>
     </row>
     <row r="22">
@@ -15294,16 +15405,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.599</v>
+        <v>43.713</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>66900.92154</v>
+        <v>67075.84998</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>6900.921539999996</v>
+        <v>7075.849979999999</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1150153589999999</v>
+        <v>0.117930833</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -15622,6 +15733,9 @@
       </c>
       <c r="DM22" s="3" t="n">
         <v>43.599</v>
+      </c>
+      <c r="DN22" s="3" t="n">
+        <v>43.713</v>
       </c>
     </row>
     <row r="23">
@@ -15647,16 +15761,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.3712</v>
+        <v>61.8288</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>169429.3065504</v>
+        <v>167955.8948496</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>19429.30655040001</v>
+        <v>17955.89484960001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1295287103360001</v>
+        <v>0.1197059656640001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -15981,6 +16095,9 @@
       </c>
       <c r="DM23" s="3" t="n">
         <v>62.3712</v>
+      </c>
+      <c r="DN23" s="3" t="n">
+        <v>61.8288</v>
       </c>
     </row>
     <row r="24">
@@ -16006,16 +16123,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>26.1358</v>
+        <v>25.8135</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>94961.4498188</v>
+        <v>93790.40951100001</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-5038.5501812</v>
+        <v>-6209.590488999995</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.050385501812</v>
+        <v>-0.06209590488999995</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -16334,6 +16451,9 @@
       </c>
       <c r="DM24" s="3" t="n">
         <v>26.1358</v>
+      </c>
+      <c r="DN24" s="3" t="n">
+        <v>25.8135</v>
       </c>
     </row>
     <row r="25">
@@ -16359,16 +16479,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.6132</v>
+        <v>12.4714</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>207129.8584968</v>
+        <v>204801.2651236</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>7129.858496800007</v>
+        <v>4801.265123599966</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.03564929248400003</v>
+        <v>0.02400632561799983</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -16690,6 +16810,9 @@
       </c>
       <c r="DM25" s="3" t="n">
         <v>12.6132</v>
+      </c>
+      <c r="DN25" s="3" t="n">
+        <v>12.4714</v>
       </c>
     </row>
     <row r="26">
@@ -16715,16 +16838,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.7949</v>
+        <v>10.6149</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>128909.6192535</v>
+        <v>126760.1105535</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>18909.6192535</v>
+        <v>16760.11055350001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1719056295772727</v>
+        <v>0.1523646413954546</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -17046,6 +17169,9 @@
       </c>
       <c r="DM26" s="3" t="n">
         <v>10.7949</v>
+      </c>
+      <c r="DN26" s="3" t="n">
+        <v>10.6149</v>
       </c>
     </row>
     <row r="27">
@@ -17071,16 +17197,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>68.7773</v>
+        <v>68.3399</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>110790.601478</v>
+        <v>110086.011314</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>790.6014779999823</v>
+        <v>86.01131399998849</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.007187286163636203</v>
+        <v>0.0007819210363635317</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -17405,6 +17531,9 @@
       </c>
       <c r="DM27" s="3" t="n">
         <v>68.7773</v>
+      </c>
+      <c r="DN27" s="3" t="n">
+        <v>68.3399</v>
       </c>
     </row>
     <row r="28">
@@ -17430,16 +17559,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>114.3619</v>
+        <v>113.207</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>378155.5771683</v>
+        <v>374336.718999</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-1844.422831699951</v>
+        <v>-5663.281001000025</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.004853744293947238</v>
+        <v>-0.01490337105526322</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -17764,6 +17893,9 @@
       </c>
       <c r="DM28" s="3" t="n">
         <v>114.3619</v>
+      </c>
+      <c r="DN28" s="3" t="n">
+        <v>113.207</v>
       </c>
     </row>
     <row r="29">
@@ -17789,16 +17921,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.1564</v>
+        <v>11.9755</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>116746.4551492</v>
+        <v>115009.1452765</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>16746.45514919999</v>
+        <v>15009.1452765</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1674645514919999</v>
+        <v>0.150091452765</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -18117,6 +18249,9 @@
       </c>
       <c r="DM29" s="3" t="n">
         <v>12.1564</v>
+      </c>
+      <c r="DN29" s="3" t="n">
+        <v>11.9755</v>
       </c>
     </row>
     <row r="30">
@@ -18142,16 +18277,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.3415</v>
+        <v>17.1644</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>128255.3235315</v>
+        <v>126945.5165484</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>28255.32353149999</v>
+        <v>26945.5165484</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2825532353149999</v>
+        <v>0.269455165484</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -18470,6 +18605,9 @@
       </c>
       <c r="DM30" s="3" t="n">
         <v>17.3415</v>
+      </c>
+      <c r="DN30" s="3" t="n">
+        <v>17.1644</v>
       </c>
     </row>
     <row r="31">
@@ -18495,16 +18633,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>402.9319</v>
+        <v>397.4755</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>107212.119952</v>
+        <v>105760.28104</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>7212.119951999994</v>
+        <v>5760.281040000002</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.07212119951999994</v>
+        <v>0.05760281040000002</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -18826,6 +18964,9 @@
       </c>
       <c r="DM31" s="3" t="n">
         <v>402.9319</v>
+      </c>
+      <c r="DN31" s="3" t="n">
+        <v>397.4755</v>
       </c>
     </row>
     <row r="32">
@@ -18851,16 +18992,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.69</v>
+        <v>10.62</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>225986.1724</v>
+        <v>224506.3752</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>25986.17239999998</v>
+        <v>24506.37519999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1299308619999999</v>
+        <v>0.1225318759999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -19185,6 +19326,9 @@
       </c>
       <c r="DM32" s="3" t="n">
         <v>10.69</v>
+      </c>
+      <c r="DN32" s="3" t="n">
+        <v>10.62</v>
       </c>
     </row>
     <row r="33">
@@ -19210,16 +19354,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.8</v>
+        <v>19.62</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>70956.072</v>
+        <v>70311.0168</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>10956.072</v>
+        <v>10311.0168</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1826012</v>
+        <v>0.17185028</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -19538,6 +19682,9 @@
       </c>
       <c r="DM33" s="3" t="n">
         <v>19.8</v>
+      </c>
+      <c r="DN33" s="3" t="n">
+        <v>19.62</v>
       </c>
     </row>
     <row r="34">
@@ -19563,16 +19710,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>219.0788</v>
+        <v>219.7075</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>77012.98964280001</v>
+        <v>77233.99718250001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-2987.010357199993</v>
+        <v>-2766.00281749999</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.03733762946499992</v>
+        <v>-0.03457503521874987</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -19894,6 +20041,9 @@
       </c>
       <c r="DM34" s="3" t="n">
         <v>219.0788</v>
+      </c>
+      <c r="DN34" s="3" t="n">
+        <v>219.7075</v>
       </c>
     </row>
     <row r="35">
@@ -19919,16 +20069,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.09</v>
+        <v>16.01</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>114808.95607</v>
+        <v>114238.12223</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>14808.95607</v>
+        <v>14238.12223000001</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1480895607</v>
+        <v>0.1423812223000001</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -20250,6 +20400,9 @@
       </c>
       <c r="DM35" s="3" t="n">
         <v>16.09</v>
+      </c>
+      <c r="DN35" s="3" t="n">
+        <v>16.01</v>
       </c>
     </row>
     <row r="36">
@@ -20275,16 +20428,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>379.8786</v>
+        <v>378.6495</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>176911.7432916</v>
+        <v>176339.344047</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>26911.7432916</v>
+        <v>26339.34404699999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.179411621944</v>
+        <v>0.1755956269799999</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -20606,6 +20759,9 @@
       </c>
       <c r="DM36" s="3" t="n">
         <v>379.8786</v>
+      </c>
+      <c r="DN36" s="3" t="n">
+        <v>378.6495</v>
       </c>
     </row>
     <row r="37">
@@ -20631,16 +20787,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.282</v>
+        <v>17.22</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>65030.247698</v>
+        <v>64796.94858</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>15030.247698</v>
+        <v>14796.94858</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.30060495396</v>
+        <v>0.2959389715999999</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -20962,6 +21118,9 @@
       </c>
       <c r="DM37" s="3" t="n">
         <v>17.282</v>
+      </c>
+      <c r="DN37" s="3" t="n">
+        <v>17.22</v>
       </c>
     </row>
     <row r="38">
@@ -20987,16 +21146,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.6677</v>
+        <v>13.5352</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>81739.43383140001</v>
+        <v>80947.0199664</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1739.433831400005</v>
+        <v>947.0199663999956</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.02174292289250006</v>
+        <v>0.01183774957999995</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -21315,6 +21474,9 @@
       </c>
       <c r="DM38" s="3" t="n">
         <v>13.6677</v>
+      </c>
+      <c r="DN38" s="3" t="n">
+        <v>13.5352</v>
       </c>
     </row>
     <row r="39">
@@ -21340,16 +21502,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1026.2097</v>
+        <v>1025.5792</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51188.36604570001</v>
+        <v>51156.9160752</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1188.366045700008</v>
+        <v>1156.916075199995</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02376732091400015</v>
+        <v>0.0231383215039999</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -21668,6 +21830,9 @@
       </c>
       <c r="DM39" s="3" t="n">
         <v>1026.2097</v>
+      </c>
+      <c r="DN39" s="3" t="n">
+        <v>1025.5792</v>
       </c>
     </row>
     <row r="40">
@@ -21693,16 +21858,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.8531</v>
+        <v>20.5822</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>105121.0401337</v>
+        <v>103755.4259194</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>5121.040133700008</v>
+        <v>3755.425919400004</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.05121040133700008</v>
+        <v>0.03755425919400004</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -22024,6 +22189,9 @@
       </c>
       <c r="DM40" s="3" t="n">
         <v>20.8531</v>
+      </c>
+      <c r="DN40" s="3" t="n">
+        <v>20.5822</v>
       </c>
     </row>
     <row r="41">
@@ -22036,13 +22204,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5009483.4415209</v>
+        <v>4984005.7749113</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>539483.4415209</v>
+        <v>514005.7749112998</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1206898079465101</v>
+        <v>0.1149901062441387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-03
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-02 07:54 IST</t>
+          <t>Generated: 2026-10-03 07:32 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-02</t>
+          <t>Last snapshot: 2026-10-03</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:ER19"/>
+  <dimension ref="A1:ES19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -767,6 +767,7 @@
     <col width="21" customWidth="1" min="146" max="146"/>
     <col width="21" customWidth="1" min="147" max="147"/>
     <col width="21" customWidth="1" min="148" max="148"/>
+    <col width="21" customWidth="1" min="149" max="149"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1510,6 +1511,11 @@
           <t>2026-10-02</t>
         </is>
       </c>
+      <c r="ES1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1957,6 +1963,9 @@
       <c r="ER2" s="3" t="n">
         <v>586</v>
       </c>
+      <c r="ES2" s="3" t="n">
+        <v>586</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2434,6 +2443,9 @@
       <c r="ER4" s="3" t="n">
         <v>1344</v>
       </c>
+      <c r="ES4" s="3" t="n">
+        <v>1344</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2884,6 +2896,9 @@
       <c r="ER5" s="3" t="n">
         <v>503.2999877929688</v>
       </c>
+      <c r="ES5" s="3" t="n">
+        <v>503.2999877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3334,6 +3349,9 @@
       <c r="ER6" s="3" t="n">
         <v>326.7000122070312</v>
       </c>
+      <c r="ES6" s="3" t="n">
+        <v>326.7000122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3784,6 +3802,9 @@
       <c r="ER7" s="3" t="n">
         <v>312</v>
       </c>
+      <c r="ES7" s="3" t="n">
+        <v>312</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4261,6 +4282,9 @@
       <c r="ER9" s="3" t="n">
         <v>14.85000038146973</v>
       </c>
+      <c r="ES9" s="3" t="n">
+        <v>14.85000038146973</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4711,6 +4735,9 @@
       <c r="ER10" s="3" t="n">
         <v>444</v>
       </c>
+      <c r="ES10" s="3" t="n">
+        <v>444</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5161,6 +5188,9 @@
       <c r="ER11" s="3" t="n">
         <v>12.92000007629395</v>
       </c>
+      <c r="ES11" s="3" t="n">
+        <v>12.92000007629395</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5611,6 +5641,9 @@
       <c r="ER12" s="3" t="n">
         <v>2620</v>
       </c>
+      <c r="ES12" s="3" t="n">
+        <v>2620</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6061,6 +6094,9 @@
       <c r="ER13" s="3" t="n">
         <v>38.90999984741211</v>
       </c>
+      <c r="ES13" s="3" t="n">
+        <v>38.90999984741211</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6511,6 +6547,9 @@
       <c r="ER14" s="3" t="n">
         <v>608.4500122070312</v>
       </c>
+      <c r="ES14" s="3" t="n">
+        <v>608.4500122070312</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7015,6 +7054,9 @@
       <c r="ER17" s="3" t="n">
         <v>467</v>
       </c>
+      <c r="ES17" s="3" t="n">
+        <v>467</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7463,6 +7505,9 @@
         <v>347.7000122070312</v>
       </c>
       <c r="ER18" s="3" t="n">
+        <v>350.1499938964844</v>
+      </c>
+      <c r="ES18" s="3" t="n">
         <v>350.1499938964844</v>
       </c>
     </row>
@@ -7493,7 +7538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DN41"/>
+  <dimension ref="A1:DO41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7614,6 +7659,7 @@
     <col width="13" customWidth="1" min="116" max="116"/>
     <col width="13" customWidth="1" min="117" max="117"/>
     <col width="13" customWidth="1" min="118" max="118"/>
+    <col width="13" customWidth="1" min="119" max="119"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8207,6 +8253,11 @@
           <t>2026-10-02</t>
         </is>
       </c>
+      <c r="DO1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8569,6 +8620,9 @@
       <c r="DN2" s="3" t="n">
         <v>57.8202</v>
       </c>
+      <c r="DO2" s="3" t="n">
+        <v>57.8202</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8925,6 +8979,9 @@
       <c r="DN3" s="3" t="n">
         <v>26.6767</v>
       </c>
+      <c r="DO3" s="3" t="n">
+        <v>26.6767</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9281,6 +9338,9 @@
       <c r="DN4" s="3" t="n">
         <v>12.78</v>
       </c>
+      <c r="DO4" s="3" t="n">
+        <v>12.78</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9637,6 +9697,9 @@
       <c r="DN5" s="3" t="n">
         <v>8.9436</v>
       </c>
+      <c r="DO5" s="3" t="n">
+        <v>8.9436</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9999,6 +10062,9 @@
       <c r="DN6" s="3" t="n">
         <v>11.2513</v>
       </c>
+      <c r="DO6" s="3" t="n">
+        <v>11.2513</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10355,6 +10421,9 @@
       <c r="DN7" s="3" t="n">
         <v>33.7773</v>
       </c>
+      <c r="DO7" s="3" t="n">
+        <v>33.7773</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10717,6 +10786,9 @@
       <c r="DN8" s="3" t="n">
         <v>35.2788</v>
       </c>
+      <c r="DO8" s="3" t="n">
+        <v>35.2788</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11073,6 +11145,9 @@
       <c r="DN9" s="3" t="n">
         <v>42.5363</v>
       </c>
+      <c r="DO9" s="3" t="n">
+        <v>42.5363</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11429,6 +11504,9 @@
       <c r="DN10" s="3" t="n">
         <v>47.8409</v>
       </c>
+      <c r="DO10" s="3" t="n">
+        <v>47.8409</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11785,6 +11863,9 @@
       <c r="DN11" s="3" t="n">
         <v>108.1355</v>
       </c>
+      <c r="DO11" s="3" t="n">
+        <v>108.1355</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12147,6 +12228,9 @@
       <c r="DN12" s="3" t="n">
         <v>219.441</v>
       </c>
+      <c r="DO12" s="3" t="n">
+        <v>219.441</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12509,6 +12593,9 @@
       <c r="DN13" s="3" t="n">
         <v>21.979</v>
       </c>
+      <c r="DO13" s="3" t="n">
+        <v>21.979</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12865,6 +12952,9 @@
       <c r="DN14" s="3" t="n">
         <v>37.8428</v>
       </c>
+      <c r="DO14" s="3" t="n">
+        <v>37.8428</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13227,6 +13317,9 @@
       <c r="DN15" s="3" t="n">
         <v>11.4</v>
       </c>
+      <c r="DO15" s="3" t="n">
+        <v>11.4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13583,6 +13676,9 @@
       <c r="DN16" s="3" t="n">
         <v>25.455</v>
       </c>
+      <c r="DO16" s="3" t="n">
+        <v>25.455</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13939,6 +14035,9 @@
       <c r="DN17" s="3" t="n">
         <v>16.6081</v>
       </c>
+      <c r="DO17" s="3" t="n">
+        <v>16.6081</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14301,6 +14400,9 @@
       <c r="DN18" s="3" t="n">
         <v>45.92</v>
       </c>
+      <c r="DO18" s="3" t="n">
+        <v>45.92</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14657,6 +14759,9 @@
       <c r="DN19" s="3" t="n">
         <v>13.3046</v>
       </c>
+      <c r="DO19" s="3" t="n">
+        <v>13.3046</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15019,6 +15124,9 @@
       <c r="DN20" s="3" t="n">
         <v>9.58</v>
       </c>
+      <c r="DO20" s="3" t="n">
+        <v>9.58</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -15381,6 +15489,9 @@
       <c r="DN21" s="3" t="n">
         <v>110.6902</v>
       </c>
+      <c r="DO21" s="3" t="n">
+        <v>110.6902</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -15737,6 +15848,9 @@
       <c r="DN22" s="3" t="n">
         <v>43.713</v>
       </c>
+      <c r="DO22" s="3" t="n">
+        <v>43.713</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -16099,6 +16213,9 @@
       <c r="DN23" s="3" t="n">
         <v>61.8288</v>
       </c>
+      <c r="DO23" s="3" t="n">
+        <v>61.8288</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -16455,6 +16572,9 @@
       <c r="DN24" s="3" t="n">
         <v>25.8135</v>
       </c>
+      <c r="DO24" s="3" t="n">
+        <v>25.8135</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -16814,6 +16934,9 @@
       <c r="DN25" s="3" t="n">
         <v>12.4714</v>
       </c>
+      <c r="DO25" s="3" t="n">
+        <v>12.4714</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -17173,6 +17296,9 @@
       <c r="DN26" s="3" t="n">
         <v>10.6149</v>
       </c>
+      <c r="DO26" s="3" t="n">
+        <v>10.6149</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -17535,6 +17661,9 @@
       <c r="DN27" s="3" t="n">
         <v>68.3399</v>
       </c>
+      <c r="DO27" s="3" t="n">
+        <v>68.3399</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -17897,6 +18026,9 @@
       <c r="DN28" s="3" t="n">
         <v>113.207</v>
       </c>
+      <c r="DO28" s="3" t="n">
+        <v>113.207</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -18253,6 +18385,9 @@
       <c r="DN29" s="3" t="n">
         <v>11.9755</v>
       </c>
+      <c r="DO29" s="3" t="n">
+        <v>11.9755</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -18609,6 +18744,9 @@
       <c r="DN30" s="3" t="n">
         <v>17.1644</v>
       </c>
+      <c r="DO30" s="3" t="n">
+        <v>17.1644</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -18968,6 +19106,9 @@
       <c r="DN31" s="3" t="n">
         <v>397.4755</v>
       </c>
+      <c r="DO31" s="3" t="n">
+        <v>397.4755</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -19330,6 +19471,9 @@
       <c r="DN32" s="3" t="n">
         <v>10.62</v>
       </c>
+      <c r="DO32" s="3" t="n">
+        <v>10.62</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -19686,6 +19830,9 @@
       <c r="DN33" s="3" t="n">
         <v>19.62</v>
       </c>
+      <c r="DO33" s="3" t="n">
+        <v>19.62</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -20045,6 +20192,9 @@
       <c r="DN34" s="3" t="n">
         <v>219.7075</v>
       </c>
+      <c r="DO34" s="3" t="n">
+        <v>219.7075</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -20404,6 +20554,9 @@
       <c r="DN35" s="3" t="n">
         <v>16.01</v>
       </c>
+      <c r="DO35" s="3" t="n">
+        <v>16.01</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -20763,6 +20916,9 @@
       <c r="DN36" s="3" t="n">
         <v>378.6495</v>
       </c>
+      <c r="DO36" s="3" t="n">
+        <v>378.6495</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -21122,6 +21278,9 @@
       <c r="DN37" s="3" t="n">
         <v>17.22</v>
       </c>
+      <c r="DO37" s="3" t="n">
+        <v>17.22</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -21478,6 +21637,9 @@
       <c r="DN38" s="3" t="n">
         <v>13.5352</v>
       </c>
+      <c r="DO38" s="3" t="n">
+        <v>13.5352</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -21834,6 +21996,9 @@
       <c r="DN39" s="3" t="n">
         <v>1025.5792</v>
       </c>
+      <c r="DO39" s="3" t="n">
+        <v>1025.5792</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -22191,6 +22356,9 @@
         <v>20.8531</v>
       </c>
       <c r="DN40" s="3" t="n">
+        <v>20.5822</v>
+      </c>
+      <c r="DO40" s="3" t="n">
         <v>20.5822</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-04
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-03 07:32 IST</t>
+          <t>Generated: 2026-10-04 07:44 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-03</t>
+          <t>Last snapshot: 2026-10-04</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:ES19"/>
+  <dimension ref="A1:ET19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -768,6 +768,7 @@
     <col width="21" customWidth="1" min="147" max="147"/>
     <col width="21" customWidth="1" min="148" max="148"/>
     <col width="21" customWidth="1" min="149" max="149"/>
+    <col width="21" customWidth="1" min="150" max="150"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1516,6 +1517,11 @@
           <t>2026-10-03</t>
         </is>
       </c>
+      <c r="ET1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1966,6 +1972,9 @@
       <c r="ES2" s="3" t="n">
         <v>586</v>
       </c>
+      <c r="ET2" s="3" t="n">
+        <v>586</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2446,6 +2455,9 @@
       <c r="ES4" s="3" t="n">
         <v>1344</v>
       </c>
+      <c r="ET4" s="3" t="n">
+        <v>1344</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2899,6 +2911,9 @@
       <c r="ES5" s="3" t="n">
         <v>503.2999877929688</v>
       </c>
+      <c r="ET5" s="3" t="n">
+        <v>503.2999877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3352,6 +3367,9 @@
       <c r="ES6" s="3" t="n">
         <v>326.7000122070312</v>
       </c>
+      <c r="ET6" s="3" t="n">
+        <v>326.7000122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3805,6 +3823,9 @@
       <c r="ES7" s="3" t="n">
         <v>312</v>
       </c>
+      <c r="ET7" s="3" t="n">
+        <v>312</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4285,6 +4306,9 @@
       <c r="ES9" s="3" t="n">
         <v>14.85000038146973</v>
       </c>
+      <c r="ET9" s="3" t="n">
+        <v>14.85000038146973</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4738,6 +4762,9 @@
       <c r="ES10" s="3" t="n">
         <v>444</v>
       </c>
+      <c r="ET10" s="3" t="n">
+        <v>444</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5191,6 +5218,9 @@
       <c r="ES11" s="3" t="n">
         <v>12.92000007629395</v>
       </c>
+      <c r="ET11" s="3" t="n">
+        <v>12.92000007629395</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5644,6 +5674,9 @@
       <c r="ES12" s="3" t="n">
         <v>2620</v>
       </c>
+      <c r="ET12" s="3" t="n">
+        <v>2620</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6097,6 +6130,9 @@
       <c r="ES13" s="3" t="n">
         <v>38.90999984741211</v>
       </c>
+      <c r="ET13" s="3" t="n">
+        <v>38.90999984741211</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6550,6 +6586,9 @@
       <c r="ES14" s="3" t="n">
         <v>608.4500122070312</v>
       </c>
+      <c r="ET14" s="3" t="n">
+        <v>608.4500122070312</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7057,6 +7096,9 @@
       <c r="ES17" s="3" t="n">
         <v>467</v>
       </c>
+      <c r="ET17" s="3" t="n">
+        <v>467</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7508,6 +7550,9 @@
         <v>350.1499938964844</v>
       </c>
       <c r="ES18" s="3" t="n">
+        <v>350.1499938964844</v>
+      </c>
+      <c r="ET18" s="3" t="n">
         <v>350.1499938964844</v>
       </c>
     </row>
@@ -7538,7 +7583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DO41"/>
+  <dimension ref="A1:DP41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7660,6 +7705,7 @@
     <col width="13" customWidth="1" min="117" max="117"/>
     <col width="13" customWidth="1" min="118" max="118"/>
     <col width="13" customWidth="1" min="119" max="119"/>
+    <col width="13" customWidth="1" min="120" max="120"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8258,6 +8304,11 @@
           <t>2026-10-03</t>
         </is>
       </c>
+      <c r="DP1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8623,6 +8674,9 @@
       <c r="DO2" s="3" t="n">
         <v>57.8202</v>
       </c>
+      <c r="DP2" s="3" t="n">
+        <v>57.8202</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8982,6 +9036,9 @@
       <c r="DO3" s="3" t="n">
         <v>26.6767</v>
       </c>
+      <c r="DP3" s="3" t="n">
+        <v>26.6767</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9341,6 +9398,9 @@
       <c r="DO4" s="3" t="n">
         <v>12.78</v>
       </c>
+      <c r="DP4" s="3" t="n">
+        <v>12.78</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9700,6 +9760,9 @@
       <c r="DO5" s="3" t="n">
         <v>8.9436</v>
       </c>
+      <c r="DP5" s="3" t="n">
+        <v>8.9436</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10065,6 +10128,9 @@
       <c r="DO6" s="3" t="n">
         <v>11.2513</v>
       </c>
+      <c r="DP6" s="3" t="n">
+        <v>11.2513</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10424,6 +10490,9 @@
       <c r="DO7" s="3" t="n">
         <v>33.7773</v>
       </c>
+      <c r="DP7" s="3" t="n">
+        <v>33.7773</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10789,6 +10858,9 @@
       <c r="DO8" s="3" t="n">
         <v>35.2788</v>
       </c>
+      <c r="DP8" s="3" t="n">
+        <v>35.2788</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11148,6 +11220,9 @@
       <c r="DO9" s="3" t="n">
         <v>42.5363</v>
       </c>
+      <c r="DP9" s="3" t="n">
+        <v>42.5363</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11507,6 +11582,9 @@
       <c r="DO10" s="3" t="n">
         <v>47.8409</v>
       </c>
+      <c r="DP10" s="3" t="n">
+        <v>47.8409</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11866,6 +11944,9 @@
       <c r="DO11" s="3" t="n">
         <v>108.1355</v>
       </c>
+      <c r="DP11" s="3" t="n">
+        <v>108.1355</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12231,6 +12312,9 @@
       <c r="DO12" s="3" t="n">
         <v>219.441</v>
       </c>
+      <c r="DP12" s="3" t="n">
+        <v>219.441</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12596,6 +12680,9 @@
       <c r="DO13" s="3" t="n">
         <v>21.979</v>
       </c>
+      <c r="DP13" s="3" t="n">
+        <v>21.979</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12955,6 +13042,9 @@
       <c r="DO14" s="3" t="n">
         <v>37.8428</v>
       </c>
+      <c r="DP14" s="3" t="n">
+        <v>37.8428</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13320,6 +13410,9 @@
       <c r="DO15" s="3" t="n">
         <v>11.4</v>
       </c>
+      <c r="DP15" s="3" t="n">
+        <v>11.4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13679,6 +13772,9 @@
       <c r="DO16" s="3" t="n">
         <v>25.455</v>
       </c>
+      <c r="DP16" s="3" t="n">
+        <v>25.455</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14038,6 +14134,9 @@
       <c r="DO17" s="3" t="n">
         <v>16.6081</v>
       </c>
+      <c r="DP17" s="3" t="n">
+        <v>16.6081</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14403,6 +14502,9 @@
       <c r="DO18" s="3" t="n">
         <v>45.92</v>
       </c>
+      <c r="DP18" s="3" t="n">
+        <v>45.92</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14762,6 +14864,9 @@
       <c r="DO19" s="3" t="n">
         <v>13.3046</v>
       </c>
+      <c r="DP19" s="3" t="n">
+        <v>13.3046</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15127,6 +15232,9 @@
       <c r="DO20" s="3" t="n">
         <v>9.58</v>
       </c>
+      <c r="DP20" s="3" t="n">
+        <v>9.58</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -15492,6 +15600,9 @@
       <c r="DO21" s="3" t="n">
         <v>110.6902</v>
       </c>
+      <c r="DP21" s="3" t="n">
+        <v>110.6902</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -15851,6 +15962,9 @@
       <c r="DO22" s="3" t="n">
         <v>43.713</v>
       </c>
+      <c r="DP22" s="3" t="n">
+        <v>43.713</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -16216,6 +16330,9 @@
       <c r="DO23" s="3" t="n">
         <v>61.8288</v>
       </c>
+      <c r="DP23" s="3" t="n">
+        <v>61.8288</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -16575,6 +16692,9 @@
       <c r="DO24" s="3" t="n">
         <v>25.8135</v>
       </c>
+      <c r="DP24" s="3" t="n">
+        <v>25.8135</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -16937,6 +17057,9 @@
       <c r="DO25" s="3" t="n">
         <v>12.4714</v>
       </c>
+      <c r="DP25" s="3" t="n">
+        <v>12.4714</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -17299,6 +17422,9 @@
       <c r="DO26" s="3" t="n">
         <v>10.6149</v>
       </c>
+      <c r="DP26" s="3" t="n">
+        <v>10.6149</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -17664,6 +17790,9 @@
       <c r="DO27" s="3" t="n">
         <v>68.3399</v>
       </c>
+      <c r="DP27" s="3" t="n">
+        <v>68.3399</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -18029,6 +18158,9 @@
       <c r="DO28" s="3" t="n">
         <v>113.207</v>
       </c>
+      <c r="DP28" s="3" t="n">
+        <v>113.207</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -18388,6 +18520,9 @@
       <c r="DO29" s="3" t="n">
         <v>11.9755</v>
       </c>
+      <c r="DP29" s="3" t="n">
+        <v>11.9755</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -18747,6 +18882,9 @@
       <c r="DO30" s="3" t="n">
         <v>17.1644</v>
       </c>
+      <c r="DP30" s="3" t="n">
+        <v>17.1644</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -19109,6 +19247,9 @@
       <c r="DO31" s="3" t="n">
         <v>397.4755</v>
       </c>
+      <c r="DP31" s="3" t="n">
+        <v>397.4755</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -19474,6 +19615,9 @@
       <c r="DO32" s="3" t="n">
         <v>10.62</v>
       </c>
+      <c r="DP32" s="3" t="n">
+        <v>10.62</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -19833,6 +19977,9 @@
       <c r="DO33" s="3" t="n">
         <v>19.62</v>
       </c>
+      <c r="DP33" s="3" t="n">
+        <v>19.62</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -20195,6 +20342,9 @@
       <c r="DO34" s="3" t="n">
         <v>219.7075</v>
       </c>
+      <c r="DP34" s="3" t="n">
+        <v>219.7075</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -20557,6 +20707,9 @@
       <c r="DO35" s="3" t="n">
         <v>16.01</v>
       </c>
+      <c r="DP35" s="3" t="n">
+        <v>16.01</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -20919,6 +21072,9 @@
       <c r="DO36" s="3" t="n">
         <v>378.6495</v>
       </c>
+      <c r="DP36" s="3" t="n">
+        <v>378.6495</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -21281,6 +21437,9 @@
       <c r="DO37" s="3" t="n">
         <v>17.22</v>
       </c>
+      <c r="DP37" s="3" t="n">
+        <v>17.22</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -21640,6 +21799,9 @@
       <c r="DO38" s="3" t="n">
         <v>13.5352</v>
       </c>
+      <c r="DP38" s="3" t="n">
+        <v>13.5352</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -21999,6 +22161,9 @@
       <c r="DO39" s="3" t="n">
         <v>1025.5792</v>
       </c>
+      <c r="DP39" s="3" t="n">
+        <v>1025.5792</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -22359,6 +22524,9 @@
         <v>20.5822</v>
       </c>
       <c r="DO40" s="3" t="n">
+        <v>20.5822</v>
+      </c>
+      <c r="DP40" s="3" t="n">
         <v>20.5822</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-05
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-04 07:44 IST</t>
+          <t>Generated: 2026-10-05 08:14 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>527793.0008010864</v>
+        <v>530376.4993553162</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-62989.01919891359</v>
+        <v>-60405.52064468386</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1066197295559428</v>
+        <v>-0.1022467146929825</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5511798.775712387</v>
+        <v>5514382.274266616</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>451016.7557123872</v>
+        <v>453600.2542666169</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08911997274926835</v>
+        <v>0.08963046668953684</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-04</t>
+          <t>Last snapshot: 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:ET19"/>
+  <dimension ref="A1:EU19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -769,6 +769,7 @@
     <col width="21" customWidth="1" min="148" max="148"/>
     <col width="21" customWidth="1" min="149" max="149"/>
     <col width="21" customWidth="1" min="150" max="150"/>
+    <col width="21" customWidth="1" min="151" max="151"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1522,6 +1523,11 @@
           <t>2026-10-04</t>
         </is>
       </c>
+      <c r="EU1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1541,13 +1547,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>586</v>
+        <v>594.7999877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46880</v>
+        <v>47583.9990234375</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3062.489999999998</v>
+        <v>3766.489023437498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1974,6 +1980,9 @@
       </c>
       <c r="ET2" s="3" t="n">
         <v>586</v>
+      </c>
+      <c r="EU2" s="3" t="n">
+        <v>594.7999877929688</v>
       </c>
     </row>
     <row r="3">
@@ -2021,13 +2030,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1344</v>
+        <v>1356</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>26880</v>
+        <v>27120</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5224.580000000002</v>
+        <v>-4984.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2457,6 +2466,9 @@
       </c>
       <c r="ET4" s="3" t="n">
         <v>1344</v>
+      </c>
+      <c r="EU4" s="3" t="n">
+        <v>1356</v>
       </c>
     </row>
     <row r="5">
@@ -2477,13 +2489,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>503.2999877929688</v>
+        <v>492.1000061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>10065.99975585938</v>
+        <v>9842.000122070312</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4147.100244140625</v>
+        <v>-4371.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2913,6 +2925,9 @@
       </c>
       <c r="ET5" s="3" t="n">
         <v>503.2999877929688</v>
+      </c>
+      <c r="EU5" s="3" t="n">
+        <v>492.1000061035156</v>
       </c>
     </row>
     <row r="6">
@@ -2933,13 +2948,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>326.7000122070312</v>
+        <v>338</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13068.00048828125</v>
+        <v>13520</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4434.239511718752</v>
+        <v>-3982.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3369,6 +3384,9 @@
       </c>
       <c r="ET6" s="3" t="n">
         <v>326.7000122070312</v>
+      </c>
+      <c r="EU6" s="3" t="n">
+        <v>338</v>
       </c>
     </row>
     <row r="7">
@@ -3389,13 +3407,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>312</v>
+        <v>310.9500122070312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>31200</v>
+        <v>31095.00122070312</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4766.18</v>
+        <v>4661.181220703125</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3825,6 +3843,9 @@
       </c>
       <c r="ET7" s="3" t="n">
         <v>312</v>
+      </c>
+      <c r="EU7" s="3" t="n">
+        <v>310.9500122070312</v>
       </c>
     </row>
     <row r="8">
@@ -3872,13 +3893,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.85000038146973</v>
+        <v>15.02999973297119</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22275.00057220459</v>
+        <v>22544.99959945679</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8775.169427795408</v>
+        <v>-8505.170400543211</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4308,6 +4329,9 @@
       </c>
       <c r="ET9" s="3" t="n">
         <v>14.85000038146973</v>
+      </c>
+      <c r="EU9" s="3" t="n">
+        <v>15.02999973297119</v>
       </c>
     </row>
     <row r="10">
@@ -4328,13 +4352,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>444</v>
+        <v>447.25</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44400</v>
+        <v>44725</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-7098.480000000003</v>
+        <v>-6773.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4764,6 +4788,9 @@
       </c>
       <c r="ET10" s="3" t="n">
         <v>444</v>
+      </c>
+      <c r="EU10" s="3" t="n">
+        <v>447.25</v>
       </c>
     </row>
     <row r="11">
@@ -4784,13 +4811,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12.92000007629395</v>
+        <v>13.02000045776367</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>12920.00007629395</v>
+        <v>13020.00045776367</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3078.790076293946</v>
+        <v>3178.790457763673</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5220,6 +5247,9 @@
       </c>
       <c r="ET11" s="3" t="n">
         <v>12.92000007629395</v>
+      </c>
+      <c r="EU11" s="3" t="n">
+        <v>13.02000045776367</v>
       </c>
     </row>
     <row r="12">
@@ -5240,13 +5270,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2620</v>
+        <v>2588.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26200</v>
+        <v>25885</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1523.25</v>
+        <v>-1838.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5676,6 +5706,9 @@
       </c>
       <c r="ET12" s="3" t="n">
         <v>2620</v>
+      </c>
+      <c r="EU12" s="3" t="n">
+        <v>2588.5</v>
       </c>
     </row>
     <row r="13">
@@ -5696,13 +5729,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>38.90999984741211</v>
+        <v>39.29999923706055</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23345.99990844727</v>
+        <v>23579.99954223633</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11685.76009155274</v>
+        <v>-11451.76045776367</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6132,6 +6165,9 @@
       </c>
       <c r="ET13" s="3" t="n">
         <v>38.90999984741211</v>
+      </c>
+      <c r="EU13" s="3" t="n">
+        <v>39.29999923706055</v>
       </c>
     </row>
     <row r="14">
@@ -6152,13 +6188,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>608.4500122070312</v>
+        <v>624.5999755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>30422.50061035156</v>
+        <v>31229.99877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12040.00938964844</v>
+        <v>-11232.51122070313</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6588,6 +6624,9 @@
       </c>
       <c r="ET14" s="3" t="n">
         <v>608.4500122070312</v>
+      </c>
+      <c r="EU14" s="3" t="n">
+        <v>624.5999755859375</v>
       </c>
     </row>
     <row r="15">
@@ -6662,13 +6701,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>467</v>
+        <v>466.5</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23350</v>
+        <v>23325</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1595.470000000001</v>
+        <v>1570.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7098,6 +7137,9 @@
       </c>
       <c r="ET17" s="3" t="n">
         <v>467</v>
+      </c>
+      <c r="EU17" s="3" t="n">
+        <v>466.5</v>
       </c>
     </row>
     <row r="18">
@@ -7118,13 +7160,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>350.1499938964844</v>
+        <v>351.3500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35014.99938964844</v>
+        <v>35135.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11625.82061035156</v>
+        <v>-11505.81938964844</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7554,6 +7596,9 @@
       </c>
       <c r="ET18" s="3" t="n">
         <v>350.1499938964844</v>
+      </c>
+      <c r="EU18" s="3" t="n">
+        <v>351.3500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -7566,10 +7611,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>527793.0008010864</v>
+        <v>530376.4993553162</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-62989.01919891359</v>
+        <v>-60405.52064468385</v>
       </c>
     </row>
   </sheetData>
@@ -7583,7 +7628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DP41"/>
+  <dimension ref="A1:DQ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7706,6 +7751,7 @@
     <col width="13" customWidth="1" min="118" max="118"/>
     <col width="13" customWidth="1" min="119" max="119"/>
     <col width="13" customWidth="1" min="120" max="120"/>
+    <col width="13" customWidth="1" min="121" max="121"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8309,6 +8355,11 @@
           <t>2026-10-04</t>
         </is>
       </c>
+      <c r="DQ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8677,6 +8728,9 @@
       <c r="DP2" s="3" t="n">
         <v>57.8202</v>
       </c>
+      <c r="DQ2" s="3" t="n">
+        <v>57.8202</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9039,6 +9093,9 @@
       <c r="DP3" s="3" t="n">
         <v>26.6767</v>
       </c>
+      <c r="DQ3" s="3" t="n">
+        <v>26.6767</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9401,6 +9458,9 @@
       <c r="DP4" s="3" t="n">
         <v>12.78</v>
       </c>
+      <c r="DQ4" s="3" t="n">
+        <v>12.78</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9763,6 +9823,9 @@
       <c r="DP5" s="3" t="n">
         <v>8.9436</v>
       </c>
+      <c r="DQ5" s="3" t="n">
+        <v>8.9436</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10131,6 +10194,9 @@
       <c r="DP6" s="3" t="n">
         <v>11.2513</v>
       </c>
+      <c r="DQ6" s="3" t="n">
+        <v>11.2513</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10493,6 +10559,9 @@
       <c r="DP7" s="3" t="n">
         <v>33.7773</v>
       </c>
+      <c r="DQ7" s="3" t="n">
+        <v>33.7773</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10861,6 +10930,9 @@
       <c r="DP8" s="3" t="n">
         <v>35.2788</v>
       </c>
+      <c r="DQ8" s="3" t="n">
+        <v>35.2788</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11223,6 +11295,9 @@
       <c r="DP9" s="3" t="n">
         <v>42.5363</v>
       </c>
+      <c r="DQ9" s="3" t="n">
+        <v>42.5363</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11585,6 +11660,9 @@
       <c r="DP10" s="3" t="n">
         <v>47.8409</v>
       </c>
+      <c r="DQ10" s="3" t="n">
+        <v>47.8409</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11947,6 +12025,9 @@
       <c r="DP11" s="3" t="n">
         <v>108.1355</v>
       </c>
+      <c r="DQ11" s="3" t="n">
+        <v>108.1355</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12315,6 +12396,9 @@
       <c r="DP12" s="3" t="n">
         <v>219.441</v>
       </c>
+      <c r="DQ12" s="3" t="n">
+        <v>219.441</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12683,6 +12767,9 @@
       <c r="DP13" s="3" t="n">
         <v>21.979</v>
       </c>
+      <c r="DQ13" s="3" t="n">
+        <v>21.979</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13045,6 +13132,9 @@
       <c r="DP14" s="3" t="n">
         <v>37.8428</v>
       </c>
+      <c r="DQ14" s="3" t="n">
+        <v>37.8428</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13413,6 +13503,9 @@
       <c r="DP15" s="3" t="n">
         <v>11.4</v>
       </c>
+      <c r="DQ15" s="3" t="n">
+        <v>11.4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13775,6 +13868,9 @@
       <c r="DP16" s="3" t="n">
         <v>25.455</v>
       </c>
+      <c r="DQ16" s="3" t="n">
+        <v>25.455</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14137,6 +14233,9 @@
       <c r="DP17" s="3" t="n">
         <v>16.6081</v>
       </c>
+      <c r="DQ17" s="3" t="n">
+        <v>16.6081</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14505,6 +14604,9 @@
       <c r="DP18" s="3" t="n">
         <v>45.92</v>
       </c>
+      <c r="DQ18" s="3" t="n">
+        <v>45.92</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14867,6 +14969,9 @@
       <c r="DP19" s="3" t="n">
         <v>13.3046</v>
       </c>
+      <c r="DQ19" s="3" t="n">
+        <v>13.3046</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15235,6 +15340,9 @@
       <c r="DP20" s="3" t="n">
         <v>9.58</v>
       </c>
+      <c r="DQ20" s="3" t="n">
+        <v>9.58</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -15603,6 +15711,9 @@
       <c r="DP21" s="3" t="n">
         <v>110.6902</v>
       </c>
+      <c r="DQ21" s="3" t="n">
+        <v>110.6902</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -15965,6 +16076,9 @@
       <c r="DP22" s="3" t="n">
         <v>43.713</v>
       </c>
+      <c r="DQ22" s="3" t="n">
+        <v>43.713</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -16333,6 +16447,9 @@
       <c r="DP23" s="3" t="n">
         <v>61.8288</v>
       </c>
+      <c r="DQ23" s="3" t="n">
+        <v>61.8288</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -16695,6 +16812,9 @@
       <c r="DP24" s="3" t="n">
         <v>25.8135</v>
       </c>
+      <c r="DQ24" s="3" t="n">
+        <v>25.8135</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -17060,6 +17180,9 @@
       <c r="DP25" s="3" t="n">
         <v>12.4714</v>
       </c>
+      <c r="DQ25" s="3" t="n">
+        <v>12.4714</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -17425,6 +17548,9 @@
       <c r="DP26" s="3" t="n">
         <v>10.6149</v>
       </c>
+      <c r="DQ26" s="3" t="n">
+        <v>10.6149</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -17793,6 +17919,9 @@
       <c r="DP27" s="3" t="n">
         <v>68.3399</v>
       </c>
+      <c r="DQ27" s="3" t="n">
+        <v>68.3399</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -18161,6 +18290,9 @@
       <c r="DP28" s="3" t="n">
         <v>113.207</v>
       </c>
+      <c r="DQ28" s="3" t="n">
+        <v>113.207</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -18523,6 +18655,9 @@
       <c r="DP29" s="3" t="n">
         <v>11.9755</v>
       </c>
+      <c r="DQ29" s="3" t="n">
+        <v>11.9755</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -18885,6 +19020,9 @@
       <c r="DP30" s="3" t="n">
         <v>17.1644</v>
       </c>
+      <c r="DQ30" s="3" t="n">
+        <v>17.1644</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -19250,6 +19388,9 @@
       <c r="DP31" s="3" t="n">
         <v>397.4755</v>
       </c>
+      <c r="DQ31" s="3" t="n">
+        <v>397.4755</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -19618,6 +19759,9 @@
       <c r="DP32" s="3" t="n">
         <v>10.62</v>
       </c>
+      <c r="DQ32" s="3" t="n">
+        <v>10.62</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -19980,6 +20124,9 @@
       <c r="DP33" s="3" t="n">
         <v>19.62</v>
       </c>
+      <c r="DQ33" s="3" t="n">
+        <v>19.62</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -20345,6 +20492,9 @@
       <c r="DP34" s="3" t="n">
         <v>219.7075</v>
       </c>
+      <c r="DQ34" s="3" t="n">
+        <v>219.7075</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -20710,6 +20860,9 @@
       <c r="DP35" s="3" t="n">
         <v>16.01</v>
       </c>
+      <c r="DQ35" s="3" t="n">
+        <v>16.01</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -21075,6 +21228,9 @@
       <c r="DP36" s="3" t="n">
         <v>378.6495</v>
       </c>
+      <c r="DQ36" s="3" t="n">
+        <v>378.6495</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -21440,6 +21596,9 @@
       <c r="DP37" s="3" t="n">
         <v>17.22</v>
       </c>
+      <c r="DQ37" s="3" t="n">
+        <v>17.22</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -21802,6 +21961,9 @@
       <c r="DP38" s="3" t="n">
         <v>13.5352</v>
       </c>
+      <c r="DQ38" s="3" t="n">
+        <v>13.5352</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -22164,6 +22326,9 @@
       <c r="DP39" s="3" t="n">
         <v>1025.5792</v>
       </c>
+      <c r="DQ39" s="3" t="n">
+        <v>1025.5792</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -22527,6 +22692,9 @@
         <v>20.5822</v>
       </c>
       <c r="DP40" s="3" t="n">
+        <v>20.5822</v>
+      </c>
+      <c r="DQ40" s="3" t="n">
         <v>20.5822</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-06
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-05 08:14 IST</t>
+          <t>Generated: 2026-10-06 08:31 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4984005.7749113</v>
+        <v>5022377.6381402</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>514005.7749113003</v>
+        <v>552377.6381401997</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1149901062441388</v>
+        <v>0.1235744156913198</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>530376.4993553162</v>
+        <v>532575.9981613159</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-60405.52064468386</v>
+        <v>-58206.0218386841</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1022467146929825</v>
+        <v>-0.09852368533267837</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5514382.274266616</v>
+        <v>5554953.636301516</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>453600.2542666169</v>
+        <v>494171.6163015161</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08963046668953684</v>
+        <v>0.0976472834333845</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-05</t>
+          <t>Last snapshot: 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -616,14 +616,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EU19"/>
+  <dimension ref="A1:EV19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
@@ -770,6 +770,7 @@
     <col width="21" customWidth="1" min="149" max="149"/>
     <col width="21" customWidth="1" min="150" max="150"/>
     <col width="21" customWidth="1" min="151" max="151"/>
+    <col width="20" customWidth="1" min="152" max="152"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1528,6 +1529,11 @@
           <t>2026-10-05</t>
         </is>
       </c>
+      <c r="EV1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1547,13 +1553,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>594.7999877929688</v>
+        <v>586.7999877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47583.9990234375</v>
+        <v>46943.9990234375</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3766.489023437498</v>
+        <v>3126.489023437498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1983,6 +1989,9 @@
       </c>
       <c r="EU2" s="3" t="n">
         <v>594.7999877929688</v>
+      </c>
+      <c r="EV2" s="3" t="n">
+        <v>586.7999877929688</v>
       </c>
     </row>
     <row r="3">
@@ -2030,13 +2039,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1356</v>
+        <v>1396.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27120</v>
+        <v>27923.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4984.580000000002</v>
+        <v>-4180.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2469,6 +2478,9 @@
       </c>
       <c r="EU4" s="3" t="n">
         <v>1356</v>
+      </c>
+      <c r="EV4" s="3" t="n">
+        <v>1396.199951171875</v>
       </c>
     </row>
     <row r="5">
@@ -2489,13 +2501,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>492.1000061035156</v>
+        <v>480.1000061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9842.000122070312</v>
+        <v>9602.000122070312</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4371.099877929688</v>
+        <v>-4611.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2928,6 +2940,9 @@
       </c>
       <c r="EU5" s="3" t="n">
         <v>492.1000061035156</v>
+      </c>
+      <c r="EV5" s="3" t="n">
+        <v>480.1000061035156</v>
       </c>
     </row>
     <row r="6">
@@ -2948,13 +2963,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>338</v>
+        <v>379.5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13520</v>
+        <v>15180</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-3982.240000000002</v>
+        <v>-2322.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3387,6 +3402,9 @@
       </c>
       <c r="EU6" s="3" t="n">
         <v>338</v>
+      </c>
+      <c r="EV6" s="3" t="n">
+        <v>379.5</v>
       </c>
     </row>
     <row r="7">
@@ -3407,13 +3425,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>310.9500122070312</v>
+        <v>314.3500061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>31095.00122070312</v>
+        <v>31435.00061035156</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4661.181220703125</v>
+        <v>5001.180610351563</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3846,6 +3864,9 @@
       </c>
       <c r="EU7" s="3" t="n">
         <v>310.9500122070312</v>
+      </c>
+      <c r="EV7" s="3" t="n">
+        <v>314.3500061035156</v>
       </c>
     </row>
     <row r="8">
@@ -3893,13 +3914,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.02999973297119</v>
+        <v>15.09000015258789</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22544.99959945679</v>
+        <v>22635.00022888184</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8505.170400543211</v>
+        <v>-8415.169771118162</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4332,6 +4353,9 @@
       </c>
       <c r="EU9" s="3" t="n">
         <v>15.02999973297119</v>
+      </c>
+      <c r="EV9" s="3" t="n">
+        <v>15.09000015258789</v>
       </c>
     </row>
     <row r="10">
@@ -4352,13 +4376,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>447.25</v>
+        <v>446.1000061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44725</v>
+        <v>44610.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6773.480000000003</v>
+        <v>-6888.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4791,6 +4815,9 @@
       </c>
       <c r="EU10" s="3" t="n">
         <v>447.25</v>
+      </c>
+      <c r="EV10" s="3" t="n">
+        <v>446.1000061035156</v>
       </c>
     </row>
     <row r="11">
@@ -4811,13 +4838,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>13.02000045776367</v>
+        <v>12.9399995803833</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>13020.00045776367</v>
+        <v>12939.9995803833</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3178.790457763673</v>
+        <v>3098.789580383302</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5250,6 +5277,9 @@
       </c>
       <c r="EU11" s="3" t="n">
         <v>13.02000045776367</v>
+      </c>
+      <c r="EV11" s="3" t="n">
+        <v>12.9399995803833</v>
       </c>
     </row>
     <row r="12">
@@ -5270,13 +5300,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2588.5</v>
+        <v>2593.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25885</v>
+        <v>25935</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1838.25</v>
+        <v>-1788.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5709,6 +5739,9 @@
       </c>
       <c r="EU12" s="3" t="n">
         <v>2588.5</v>
+      </c>
+      <c r="EV12" s="3" t="n">
+        <v>2593.5</v>
       </c>
     </row>
     <row r="13">
@@ -5729,13 +5762,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>39.29999923706055</v>
+        <v>39.18000030517578</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23579.99954223633</v>
+        <v>23508.00018310547</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11451.76045776367</v>
+        <v>-11523.75981689453</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6168,6 +6201,9 @@
       </c>
       <c r="EU13" s="3" t="n">
         <v>39.29999923706055</v>
+      </c>
+      <c r="EV13" s="3" t="n">
+        <v>39.18000030517578</v>
       </c>
     </row>
     <row r="14">
@@ -6188,13 +6224,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>624.5999755859375</v>
+        <v>617.0499877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31229.99877929688</v>
+        <v>30852.49938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11232.51122070313</v>
+        <v>-11610.01061035156</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6627,6 +6663,9 @@
       </c>
       <c r="EU14" s="3" t="n">
         <v>624.5999755859375</v>
+      </c>
+      <c r="EV14" s="3" t="n">
+        <v>617.0499877929688</v>
       </c>
     </row>
     <row r="15">
@@ -6701,13 +6740,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>466.5</v>
+        <v>473.5</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23325</v>
+        <v>23675</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1570.470000000001</v>
+        <v>1920.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7140,6 +7179,9 @@
       </c>
       <c r="EU17" s="3" t="n">
         <v>466.5</v>
+      </c>
+      <c r="EV17" s="3" t="n">
+        <v>473.5</v>
       </c>
     </row>
     <row r="18">
@@ -7160,13 +7202,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>351.3500061035156</v>
+        <v>355.6499938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35135.00061035156</v>
+        <v>35564.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11505.81938964844</v>
+        <v>-11075.82061035156</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7599,6 +7641,9 @@
       </c>
       <c r="EU18" s="3" t="n">
         <v>351.3500061035156</v>
+      </c>
+      <c r="EV18" s="3" t="n">
+        <v>355.6499938964844</v>
       </c>
     </row>
     <row r="19">
@@ -7611,10 +7656,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>530376.4993553162</v>
+        <v>532575.9981613159</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-60405.52064468385</v>
+        <v>-58206.02183868409</v>
       </c>
     </row>
   </sheetData>
@@ -7628,7 +7673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DQ41"/>
+  <dimension ref="A1:DR41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7752,6 +7797,7 @@
     <col width="13" customWidth="1" min="119" max="119"/>
     <col width="13" customWidth="1" min="120" max="120"/>
     <col width="13" customWidth="1" min="121" max="121"/>
+    <col width="13" customWidth="1" min="122" max="122"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8360,6 +8406,11 @@
           <t>2026-10-05</t>
         </is>
       </c>
+      <c r="DR1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8384,16 +8435,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.8202</v>
+        <v>58.383</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64902.1337364</v>
+        <v>65533.866606</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14902.1337364</v>
+        <v>15533.866606</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.298042674728</v>
+        <v>0.31067733212</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8730,6 +8781,9 @@
       </c>
       <c r="DQ2" s="3" t="n">
         <v>57.8202</v>
+      </c>
+      <c r="DR2" s="3" t="n">
+        <v>58.383</v>
       </c>
     </row>
     <row r="3">
@@ -8755,16 +8809,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.6767</v>
+        <v>26.8342</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65496.98063710001</v>
+        <v>65883.67668460001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5496.980637100009</v>
+        <v>5883.67668460001</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.0916163439516668</v>
+        <v>0.09806127807666683</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9095,6 +9149,9 @@
       </c>
       <c r="DQ3" s="3" t="n">
         <v>26.6767</v>
+      </c>
+      <c r="DR3" s="3" t="n">
+        <v>26.8342</v>
       </c>
     </row>
     <row r="4">
@@ -9120,16 +9177,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.78</v>
+        <v>12.99</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>245453.86854</v>
+        <v>249487.14807</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>65453.86854</v>
+        <v>69487.14807000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.363632603</v>
+        <v>0.3860397115000002</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9460,6 +9517,9 @@
       </c>
       <c r="DQ4" s="3" t="n">
         <v>12.78</v>
+      </c>
+      <c r="DR4" s="3" t="n">
+        <v>12.99</v>
       </c>
     </row>
     <row r="5">
@@ -9485,16 +9545,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.9436</v>
+        <v>8.992100000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>164151.6214368</v>
+        <v>165041.7947048</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-45848.37856320001</v>
+        <v>-44958.20529519999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2183256122057143</v>
+        <v>-0.2140866918819047</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9825,6 +9885,9 @@
       </c>
       <c r="DQ5" s="3" t="n">
         <v>8.9436</v>
+      </c>
+      <c r="DR5" s="3" t="n">
+        <v>8.992100000000001</v>
       </c>
     </row>
     <row r="6">
@@ -9850,16 +9913,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.2513</v>
+        <v>11.3159</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>47581.4889201</v>
+        <v>47854.68083429999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-2418.511079899996</v>
+        <v>-2145.319165700006</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.04837022159799992</v>
+        <v>-0.04290638331400012</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -10196,6 +10259,9 @@
       </c>
       <c r="DQ6" s="3" t="n">
         <v>11.2513</v>
+      </c>
+      <c r="DR6" s="3" t="n">
+        <v>11.3159</v>
       </c>
     </row>
     <row r="7">
@@ -10221,16 +10287,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.7773</v>
+        <v>33.7456</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74514.07489199999</v>
+        <v>74444.14342400001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14514.07489199999</v>
+        <v>14444.14342400001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2419012481999998</v>
+        <v>0.2407357237333335</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -10561,6 +10627,9 @@
       </c>
       <c r="DQ7" s="3" t="n">
         <v>33.7773</v>
+      </c>
+      <c r="DR7" s="3" t="n">
+        <v>33.7456</v>
       </c>
     </row>
     <row r="8">
@@ -10586,16 +10655,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.2788</v>
+        <v>35.5881</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>56608.1155284</v>
+        <v>57104.4161433</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6608.115528399998</v>
+        <v>7104.416143299997</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.132162310568</v>
+        <v>0.142088322866</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -10932,6 +11001,9 @@
       </c>
       <c r="DQ8" s="3" t="n">
         <v>35.2788</v>
+      </c>
+      <c r="DR8" s="3" t="n">
+        <v>35.5881</v>
       </c>
     </row>
     <row r="9">
@@ -10957,16 +11029,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.5363</v>
+        <v>43.4029</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>136941.0664659</v>
+        <v>139730.9924397</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>36941.06646589999</v>
+        <v>39730.9924397</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3694106646589999</v>
+        <v>0.397309924397</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -11297,6 +11369,9 @@
       </c>
       <c r="DQ9" s="3" t="n">
         <v>42.5363</v>
+      </c>
+      <c r="DR9" s="3" t="n">
+        <v>43.4029</v>
       </c>
     </row>
     <row r="10">
@@ -11322,16 +11397,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.8409</v>
+        <v>48.2809</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>136186.7285531</v>
+        <v>137439.2585131</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>36186.72855309999</v>
+        <v>37439.25851310001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3618672855309999</v>
+        <v>0.3743925851310001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -11662,6 +11737,9 @@
       </c>
       <c r="DQ10" s="3" t="n">
         <v>47.8409</v>
+      </c>
+      <c r="DR10" s="3" t="n">
+        <v>48.2809</v>
       </c>
     </row>
     <row r="11">
@@ -11687,16 +11765,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>108.1355</v>
+        <v>110.7336</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32540.0265245</v>
+        <v>33321.8441784</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2540.026524499997</v>
+        <v>3321.844178399995</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.08466755081666658</v>
+        <v>0.1107281392799998</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -12027,6 +12105,9 @@
       </c>
       <c r="DQ11" s="3" t="n">
         <v>108.1355</v>
+      </c>
+      <c r="DR11" s="3" t="n">
+        <v>110.7336</v>
       </c>
     </row>
     <row r="12">
@@ -12052,16 +12133,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>219.441</v>
+        <v>220.493</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102154.613202</v>
+        <v>102644.342346</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2154.613201999993</v>
+        <v>2644.34234599999</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02154613201999993</v>
+        <v>0.0264434234599999</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -12398,6 +12479,9 @@
       </c>
       <c r="DQ12" s="3" t="n">
         <v>219.441</v>
+      </c>
+      <c r="DR12" s="3" t="n">
+        <v>220.493</v>
       </c>
     </row>
     <row r="13">
@@ -12423,16 +12507,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.979</v>
+        <v>21.777</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>254683.970295</v>
+        <v>252343.274085</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>54683.97029499998</v>
+        <v>52343.27408500001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2734198514749999</v>
+        <v>0.2617163704250001</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -12769,6 +12853,9 @@
       </c>
       <c r="DQ13" s="3" t="n">
         <v>21.979</v>
+      </c>
+      <c r="DR13" s="3" t="n">
+        <v>21.777</v>
       </c>
     </row>
     <row r="14">
@@ -12794,16 +12881,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.8428</v>
+        <v>39.0609</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>136521.9123368</v>
+        <v>140916.3372054</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>36521.91233679999</v>
+        <v>40916.33720539999</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3652191233679998</v>
+        <v>0.4091633720539999</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -13134,6 +13221,9 @@
       </c>
       <c r="DQ14" s="3" t="n">
         <v>37.8428</v>
+      </c>
+      <c r="DR14" s="3" t="n">
+        <v>39.0609</v>
       </c>
     </row>
     <row r="15">
@@ -13159,16 +13249,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.4</v>
+        <v>11.45</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>111080.9958</v>
+        <v>111568.19315</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>11080.9958</v>
+        <v>11568.19314999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.110809958</v>
+        <v>0.1156819314999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -13505,6 +13595,9 @@
       </c>
       <c r="DQ15" s="3" t="n">
         <v>11.4</v>
+      </c>
+      <c r="DR15" s="3" t="n">
+        <v>11.45</v>
       </c>
     </row>
     <row r="16">
@@ -13530,16 +13623,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.455</v>
+        <v>26.0122</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>145677.13224</v>
+        <v>148865.9477216</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>45677.13223999998</v>
+        <v>48865.94772160001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4567713223999998</v>
+        <v>0.4886594772160001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -13870,6 +13963,9 @@
       </c>
       <c r="DQ16" s="3" t="n">
         <v>25.455</v>
+      </c>
+      <c r="DR16" s="3" t="n">
+        <v>26.0122</v>
       </c>
     </row>
     <row r="17">
@@ -13895,16 +13991,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6081</v>
+        <v>16.7361</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54907.3252617</v>
+        <v>55330.5005577</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4907.325261699996</v>
+        <v>5330.500557699997</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.09814650523399993</v>
+        <v>0.1066100111539999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -14235,6 +14331,9 @@
       </c>
       <c r="DQ17" s="3" t="n">
         <v>16.6081</v>
+      </c>
+      <c r="DR17" s="3" t="n">
+        <v>16.7361</v>
       </c>
     </row>
     <row r="18">
@@ -14260,16 +14359,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.92</v>
+        <v>45.54</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>86625.14112</v>
+        <v>85908.29544</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>6625.14112</v>
+        <v>5908.295440000002</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.082814264</v>
+        <v>0.07385369300000003</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -14606,6 +14705,9 @@
       </c>
       <c r="DQ18" s="3" t="n">
         <v>45.92</v>
+      </c>
+      <c r="DR18" s="3" t="n">
+        <v>45.54</v>
       </c>
     </row>
     <row r="19">
@@ -14631,16 +14733,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.3046</v>
+        <v>13.5475</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>192474.5349236</v>
+        <v>195988.512385</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>42474.5349236</v>
+        <v>45988.51238499998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2831635661573333</v>
+        <v>0.3065900825666665</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -14971,6 +15073,9 @@
       </c>
       <c r="DQ19" s="3" t="n">
         <v>13.3046</v>
+      </c>
+      <c r="DR19" s="3" t="n">
+        <v>13.5475</v>
       </c>
     </row>
     <row r="20">
@@ -14996,16 +15101,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.58</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>251530.59274</v>
+        <v>255206.40516</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>1530.592739999993</v>
+        <v>5206.405160000024</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.006122370959999971</v>
+        <v>0.02082562064000009</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -15342,6 +15447,9 @@
       </c>
       <c r="DQ20" s="3" t="n">
         <v>9.58</v>
+      </c>
+      <c r="DR20" s="3" t="n">
+        <v>9.720000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -15367,16 +15475,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>110.6902</v>
+        <v>111.3786</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>168167.0825618</v>
+        <v>169212.9404574</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-1832.917438200006</v>
+        <v>-787.0595425999782</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.01078186728352945</v>
+        <v>-0.004629762015293989</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -15713,6 +15821,9 @@
       </c>
       <c r="DQ21" s="3" t="n">
         <v>110.6902</v>
+      </c>
+      <c r="DR21" s="3" t="n">
+        <v>111.3786</v>
       </c>
     </row>
     <row r="22">
@@ -15738,16 +15849,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.713</v>
+        <v>44.646</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67075.84998</v>
+        <v>68507.50116</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7075.849979999999</v>
+        <v>8507.50116</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.117930833</v>
+        <v>0.141791686</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -16078,6 +16189,9 @@
       </c>
       <c r="DQ22" s="3" t="n">
         <v>43.713</v>
+      </c>
+      <c r="DR22" s="3" t="n">
+        <v>44.646</v>
       </c>
     </row>
     <row r="23">
@@ -16103,16 +16217,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.8288</v>
+        <v>62.0073</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>167955.8948496</v>
+        <v>168440.7842091</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>17955.89484960001</v>
+        <v>18440.78420910001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1197059656640001</v>
+        <v>0.122938561394</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -16449,6 +16563,9 @@
       </c>
       <c r="DQ23" s="3" t="n">
         <v>61.8288</v>
+      </c>
+      <c r="DR23" s="3" t="n">
+        <v>62.0073</v>
       </c>
     </row>
     <row r="24">
@@ -16474,16 +16591,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.8135</v>
+        <v>25.8872</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>93790.40951100001</v>
+        <v>94058.1900592</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-6209.590488999995</v>
+        <v>-5941.809940799998</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.06209590488999995</v>
+        <v>-0.05941809940799998</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -16814,6 +16931,9 @@
       </c>
       <c r="DQ24" s="3" t="n">
         <v>25.8135</v>
+      </c>
+      <c r="DR24" s="3" t="n">
+        <v>25.8872</v>
       </c>
     </row>
     <row r="25">
@@ -16839,16 +16959,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.4714</v>
+        <v>12.549</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>204801.2651236</v>
+        <v>206075.587026</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>4801.265123599966</v>
+        <v>6075.587025999994</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.02400632561799983</v>
+        <v>0.03037793512999997</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -17182,6 +17302,9 @@
       </c>
       <c r="DQ25" s="3" t="n">
         <v>12.4714</v>
+      </c>
+      <c r="DR25" s="3" t="n">
+        <v>12.549</v>
       </c>
     </row>
     <row r="26">
@@ -17207,16 +17330,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.6149</v>
+        <v>10.6702</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>126760.1105535</v>
+        <v>127420.487393</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>16760.11055350001</v>
+        <v>17420.48739299999</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1523646413954546</v>
+        <v>0.1583680672090908</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -17550,6 +17673,9 @@
       </c>
       <c r="DQ26" s="3" t="n">
         <v>10.6149</v>
+      </c>
+      <c r="DR26" s="3" t="n">
+        <v>10.6702</v>
       </c>
     </row>
     <row r="27">
@@ -17575,16 +17701,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>68.3399</v>
+        <v>69.2222</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>110086.011314</v>
+        <v>111507.273092</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>86.01131399998849</v>
+        <v>1507.273091999989</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.0007819210363635317</v>
+        <v>0.01370248265454535</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -17921,6 +18047,9 @@
       </c>
       <c r="DQ27" s="3" t="n">
         <v>68.3399</v>
+      </c>
+      <c r="DR27" s="3" t="n">
+        <v>69.2222</v>
       </c>
     </row>
     <row r="28">
@@ -17946,16 +18075,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>113.207</v>
+        <v>115.0356</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>374336.718999</v>
-      </c>
-      <c r="H28" s="6" t="n">
-        <v>-5663.281001000025</v>
-      </c>
-      <c r="I28" s="13" t="n">
-        <v>-0.01490337105526322</v>
+        <v>380383.2719892</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>383.2719892000314</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>0.001008610497894819</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -18292,6 +18421,9 @@
       </c>
       <c r="DQ28" s="3" t="n">
         <v>113.207</v>
+      </c>
+      <c r="DR28" s="3" t="n">
+        <v>115.0356</v>
       </c>
     </row>
     <row r="29">
@@ -18317,16 +18449,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.9755</v>
+        <v>12.0227</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>115009.1452765</v>
+        <v>115462.4400581</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>15009.1452765</v>
+        <v>15462.44005809999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.150091452765</v>
+        <v>0.1546244005809999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -18657,6 +18789,9 @@
       </c>
       <c r="DQ29" s="3" t="n">
         <v>11.9755</v>
+      </c>
+      <c r="DR29" s="3" t="n">
+        <v>12.0227</v>
       </c>
     </row>
     <row r="30">
@@ -18682,16 +18817,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.1644</v>
+        <v>17.2023</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>126945.5165484</v>
+        <v>127225.8196803</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>26945.5165484</v>
+        <v>27225.8196803</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.269455165484</v>
+        <v>0.272258196803</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -19022,6 +19157,9 @@
       </c>
       <c r="DQ30" s="3" t="n">
         <v>17.1644</v>
+      </c>
+      <c r="DR30" s="3" t="n">
+        <v>17.2023</v>
       </c>
     </row>
     <row r="31">
@@ -19047,16 +19185,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>397.4755</v>
+        <v>400.5655</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>105760.28104</v>
+        <v>106582.46824</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>5760.281040000002</v>
+        <v>6582.468239999987</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.05760281040000002</v>
+        <v>0.06582468239999988</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -19390,6 +19528,9 @@
       </c>
       <c r="DQ31" s="3" t="n">
         <v>397.4755</v>
+      </c>
+      <c r="DR31" s="3" t="n">
+        <v>400.5655</v>
       </c>
     </row>
     <row r="32">
@@ -19415,16 +19556,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.62</v>
+        <v>10.65</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>224506.3752</v>
+        <v>225140.574</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>24506.37519999998</v>
+        <v>25140.57399999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1225318759999999</v>
+        <v>0.12570287</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -19761,6 +19902,9 @@
       </c>
       <c r="DQ32" s="3" t="n">
         <v>10.62</v>
+      </c>
+      <c r="DR32" s="3" t="n">
+        <v>10.65</v>
       </c>
     </row>
     <row r="33">
@@ -19786,16 +19930,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.62</v>
+        <v>19.59</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>70311.0168</v>
+        <v>70203.5076</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>10311.0168</v>
+        <v>10203.5076</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.17185028</v>
+        <v>0.17005846</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -20126,6 +20270,9 @@
       </c>
       <c r="DQ33" s="3" t="n">
         <v>19.62</v>
+      </c>
+      <c r="DR33" s="3" t="n">
+        <v>19.59</v>
       </c>
     </row>
     <row r="34">
@@ -20151,16 +20298,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>219.7075</v>
+        <v>221.5816</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>77233.99718250001</v>
+        <v>77892.8014296</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-2766.00281749999</v>
+        <v>-2107.198570399996</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.03457503521874987</v>
+        <v>-0.02633998212999995</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -20494,6 +20641,9 @@
       </c>
       <c r="DQ34" s="3" t="n">
         <v>219.7075</v>
+      </c>
+      <c r="DR34" s="3" t="n">
+        <v>221.5816</v>
       </c>
     </row>
     <row r="35">
@@ -20519,16 +20669,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.01</v>
+        <v>16.08</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>114238.12223</v>
+        <v>114737.60184</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>14238.12223000001</v>
+        <v>14737.60183999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1423812223000001</v>
+        <v>0.1473760183999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -20862,6 +21012,9 @@
       </c>
       <c r="DQ35" s="3" t="n">
         <v>16.01</v>
+      </c>
+      <c r="DR35" s="3" t="n">
+        <v>16.08</v>
       </c>
     </row>
     <row r="36">
@@ -20887,16 +21040,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>378.6495</v>
+        <v>374.9996</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>176339.344047</v>
+        <v>174639.5637176</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>26339.34404699999</v>
+        <v>24639.56371759999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1755956269799999</v>
+        <v>0.1642637581173332</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -21230,6 +21383,9 @@
       </c>
       <c r="DQ36" s="3" t="n">
         <v>378.6495</v>
+      </c>
+      <c r="DR36" s="3" t="n">
+        <v>374.9996</v>
       </c>
     </row>
     <row r="37">
@@ -21255,16 +21411,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.22</v>
+        <v>17.071</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>64796.94858</v>
+        <v>64236.27811900001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>14796.94858</v>
+        <v>14236.27811900001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2959389715999999</v>
+        <v>0.2847255623800002</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -21598,6 +21754,9 @@
       </c>
       <c r="DQ37" s="3" t="n">
         <v>17.22</v>
+      </c>
+      <c r="DR37" s="3" t="n">
+        <v>17.071</v>
       </c>
     </row>
     <row r="38">
@@ -21623,16 +21782,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.5352</v>
+        <v>13.6087</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>80947.0199664</v>
+        <v>81386.5853934</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>947.0199663999956</v>
+        <v>1386.585393400004</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.01183774957999995</v>
+        <v>0.01733231741750005</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -21963,6 +22122,9 @@
       </c>
       <c r="DQ38" s="3" t="n">
         <v>13.5352</v>
+      </c>
+      <c r="DR38" s="3" t="n">
+        <v>13.6087</v>
       </c>
     </row>
     <row r="39">
@@ -21988,16 +22150,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.5792</v>
+        <v>1026.087</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51156.9160752</v>
+        <v>51182.245647</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1156.916075199995</v>
+        <v>1182.245646999996</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.0231383215039999</v>
+        <v>0.02364491293999992</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -22328,6 +22490,9 @@
       </c>
       <c r="DQ39" s="3" t="n">
         <v>1025.5792</v>
+      </c>
+      <c r="DR39" s="3" t="n">
+        <v>1026.087</v>
       </c>
     </row>
     <row r="40">
@@ -22353,16 +22518,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.5822</v>
+        <v>20.5252</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>103755.4259194</v>
+        <v>103468.0873804</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>3755.425919400004</v>
+        <v>3468.087380400015</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.03755425919400004</v>
+        <v>0.03468087380400015</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -22696,6 +22861,9 @@
       </c>
       <c r="DQ40" s="3" t="n">
         <v>20.5822</v>
+      </c>
+      <c r="DR40" s="3" t="n">
+        <v>20.5252</v>
       </c>
     </row>
     <row r="41">
@@ -22708,13 +22876,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4984005.7749113</v>
+        <v>5022377.6381402</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>514005.7749112998</v>
+        <v>552377.6381402001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1149901062441387</v>
+        <v>0.1235744156913199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-07
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-06 08:31 IST</t>
+          <t>Generated: 2026-10-07 08:06 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5022377.6381402</v>
+        <v>5071456.2288884</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>552377.6381401997</v>
+        <v>601456.2288883999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1235744156913198</v>
+        <v>0.1345539661942729</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>532575.9981613159</v>
+        <v>530715.5012588501</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-58206.0218386841</v>
+        <v>-60066.51874114992</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.09852368533267837</v>
+        <v>-0.1016728957681378</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5554953.636301516</v>
+        <v>5602171.73014725</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>494171.6163015161</v>
+        <v>541389.7101472504</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.0976472834333845</v>
+        <v>0.1069774805568983</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-06</t>
+          <t>Last snapshot: 2026-10-07</t>
         </is>
       </c>
     </row>
@@ -616,14 +616,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EV19"/>
+  <dimension ref="A1:EW19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
@@ -771,6 +771,7 @@
     <col width="21" customWidth="1" min="150" max="150"/>
     <col width="21" customWidth="1" min="151" max="151"/>
     <col width="20" customWidth="1" min="152" max="152"/>
+    <col width="21" customWidth="1" min="153" max="153"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1534,6 +1535,11 @@
           <t>2026-10-06</t>
         </is>
       </c>
+      <c r="EW1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1553,13 +1559,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>586.7999877929688</v>
+        <v>581.2000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46943.9990234375</v>
+        <v>46496.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3126.489023437498</v>
+        <v>2678.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1992,6 +1998,9 @@
       </c>
       <c r="EV2" s="3" t="n">
         <v>586.7999877929688</v>
+      </c>
+      <c r="EW2" s="3" t="n">
+        <v>581.2000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -2039,13 +2048,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1396.199951171875</v>
+        <v>1436.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27923.9990234375</v>
+        <v>28723.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4180.580976562502</v>
+        <v>-3380.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2481,6 +2490,9 @@
       </c>
       <c r="EV4" s="3" t="n">
         <v>1396.199951171875</v>
+      </c>
+      <c r="EW4" s="3" t="n">
+        <v>1436.199951171875</v>
       </c>
     </row>
     <row r="5">
@@ -2501,13 +2513,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>480.1000061035156</v>
+        <v>484.7999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9602.000122070312</v>
+        <v>9695.999755859375</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4611.099877929688</v>
+        <v>-4517.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2943,6 +2955,9 @@
       </c>
       <c r="EV5" s="3" t="n">
         <v>480.1000061035156</v>
+      </c>
+      <c r="EW5" s="3" t="n">
+        <v>484.7999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -2963,13 +2978,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>379.5</v>
+        <v>393.7999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15180</v>
+        <v>15751.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2322.240000000002</v>
+        <v>-1750.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3405,6 +3420,9 @@
       </c>
       <c r="EV6" s="3" t="n">
         <v>379.5</v>
+      </c>
+      <c r="EW6" s="3" t="n">
+        <v>393.7999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -3425,13 +3443,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>314.3500061035156</v>
+        <v>309</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>31435.00061035156</v>
+        <v>30900</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>5001.180610351563</v>
+        <v>4466.18</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3867,6 +3885,9 @@
       </c>
       <c r="EV7" s="3" t="n">
         <v>314.3500061035156</v>
+      </c>
+      <c r="EW7" s="3" t="n">
+        <v>309</v>
       </c>
     </row>
     <row r="8">
@@ -3914,13 +3935,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.09000015258789</v>
+        <v>14.82999992370605</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22635.00022888184</v>
+        <v>22244.99988555908</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8415.169771118162</v>
+        <v>-8805.170114440916</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4356,6 +4377,9 @@
       </c>
       <c r="EV9" s="3" t="n">
         <v>15.09000015258789</v>
+      </c>
+      <c r="EW9" s="3" t="n">
+        <v>14.82999992370605</v>
       </c>
     </row>
     <row r="10">
@@ -4376,13 +4400,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>446.1000061035156</v>
+        <v>452.4500122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44610.00061035156</v>
+        <v>45245.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6888.479389648441</v>
+        <v>-6253.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4818,6 +4842,9 @@
       </c>
       <c r="EV10" s="3" t="n">
         <v>446.1000061035156</v>
+      </c>
+      <c r="EW10" s="3" t="n">
+        <v>452.4500122070312</v>
       </c>
     </row>
     <row r="11">
@@ -4838,13 +4865,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12.9399995803833</v>
+        <v>13</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>12939.9995803833</v>
+        <v>13000</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3098.789580383302</v>
+        <v>3158.790000000001</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5280,6 +5307,9 @@
       </c>
       <c r="EV11" s="3" t="n">
         <v>12.9399995803833</v>
+      </c>
+      <c r="EW11" s="3" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="12">
@@ -5300,13 +5330,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2593.5</v>
+        <v>2525.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25935</v>
+        <v>25253.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1788.25</v>
+        <v>-2470.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5742,6 +5772,9 @@
       </c>
       <c r="EV12" s="3" t="n">
         <v>2593.5</v>
+      </c>
+      <c r="EW12" s="3" t="n">
+        <v>2525.300048828125</v>
       </c>
     </row>
     <row r="13">
@@ -5762,13 +5795,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>39.18000030517578</v>
+        <v>38.59000015258789</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23508.00018310547</v>
+        <v>23154.00009155273</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11523.75981689453</v>
+        <v>-11877.75990844727</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6204,6 +6237,9 @@
       </c>
       <c r="EV13" s="3" t="n">
         <v>39.18000030517578</v>
+      </c>
+      <c r="EW13" s="3" t="n">
+        <v>38.59000015258789</v>
       </c>
     </row>
     <row r="14">
@@ -6224,13 +6260,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>617.0499877929688</v>
+        <v>611.75</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>30852.49938964844</v>
+        <v>30587.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11610.01061035156</v>
+        <v>-11875.01</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6666,6 +6702,9 @@
       </c>
       <c r="EV14" s="3" t="n">
         <v>617.0499877929688</v>
+      </c>
+      <c r="EW14" s="3" t="n">
+        <v>611.75</v>
       </c>
     </row>
     <row r="15">
@@ -6740,13 +6779,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>473.5</v>
+        <v>468.1499938964844</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23675</v>
+        <v>23407.49969482422</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1920.470000000001</v>
+        <v>1652.96969482422</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7182,6 +7221,9 @@
       </c>
       <c r="EV17" s="3" t="n">
         <v>473.5</v>
+      </c>
+      <c r="EW17" s="3" t="n">
+        <v>468.1499938964844</v>
       </c>
     </row>
     <row r="18">
@@ -7202,13 +7244,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>355.6499938964844</v>
+        <v>344.8500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35564.99938964844</v>
+        <v>34485.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11075.82061035156</v>
+        <v>-12155.81938964844</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7644,6 +7686,9 @@
       </c>
       <c r="EV18" s="3" t="n">
         <v>355.6499938964844</v>
+      </c>
+      <c r="EW18" s="3" t="n">
+        <v>344.8500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -7656,10 +7701,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>532575.9981613159</v>
+        <v>530715.5012588501</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-58206.02183868409</v>
+        <v>-60066.51874114991</v>
       </c>
     </row>
   </sheetData>
@@ -7673,7 +7718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DR41"/>
+  <dimension ref="A1:DS41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7798,6 +7843,7 @@
     <col width="13" customWidth="1" min="120" max="120"/>
     <col width="13" customWidth="1" min="121" max="121"/>
     <col width="13" customWidth="1" min="122" max="122"/>
+    <col width="13" customWidth="1" min="123" max="123"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8411,6 +8457,11 @@
           <t>2026-10-06</t>
         </is>
       </c>
+      <c r="DS1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8435,16 +8486,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>58.383</v>
+        <v>58.5201</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>65533.866606</v>
+        <v>65687.7588882</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>15533.866606</v>
+        <v>15687.7588882</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.31067733212</v>
+        <v>0.313755177764</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8784,6 +8835,9 @@
       </c>
       <c r="DR2" s="3" t="n">
         <v>58.383</v>
+      </c>
+      <c r="DS2" s="3" t="n">
+        <v>58.5201</v>
       </c>
     </row>
     <row r="3">
@@ -8809,16 +8863,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.8342</v>
+        <v>27.2216</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65883.67668460001</v>
+        <v>66834.8262008</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5883.67668460001</v>
+        <v>6834.826200800002</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09806127807666683</v>
+        <v>0.1139137700133334</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9152,6 +9206,9 @@
       </c>
       <c r="DR3" s="3" t="n">
         <v>26.8342</v>
+      </c>
+      <c r="DS3" s="3" t="n">
+        <v>27.2216</v>
       </c>
     </row>
     <row r="4">
@@ -9177,16 +9234,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.99</v>
+        <v>13.04</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>249487.14807</v>
+        <v>250447.45272</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>69487.14807000002</v>
+        <v>70447.45272</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3860397115000002</v>
+        <v>0.3913747373333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9520,6 +9577,9 @@
       </c>
       <c r="DR4" s="3" t="n">
         <v>12.99</v>
+      </c>
+      <c r="DS4" s="3" t="n">
+        <v>13.04</v>
       </c>
     </row>
     <row r="5">
@@ -9545,16 +9605,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.992100000000001</v>
+        <v>9.0642</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>165041.7947048</v>
+        <v>166365.1244496</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-44958.20529519999</v>
+        <v>-43634.8755504</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2140866918819047</v>
+        <v>-0.2077851216685714</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9888,6 +9948,9 @@
       </c>
       <c r="DR5" s="3" t="n">
         <v>8.992100000000001</v>
+      </c>
+      <c r="DS5" s="3" t="n">
+        <v>9.0642</v>
       </c>
     </row>
     <row r="6">
@@ -9913,16 +9976,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.3159</v>
+        <v>11.4421</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>47854.68083429999</v>
+        <v>48388.3777317</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-2145.319165700006</v>
+        <v>-1611.622268300001</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.04290638331400012</v>
+        <v>-0.03223244536600003</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -10262,6 +10325,9 @@
       </c>
       <c r="DR6" s="3" t="n">
         <v>11.3159</v>
+      </c>
+      <c r="DS6" s="3" t="n">
+        <v>11.4421</v>
       </c>
     </row>
     <row r="7">
@@ -10287,16 +10353,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.7456</v>
+        <v>34.0442</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74444.14342400001</v>
+        <v>75102.86696799999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14444.14342400001</v>
+        <v>15102.86696799999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2407357237333335</v>
+        <v>0.2517144494666664</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -10630,6 +10696,9 @@
       </c>
       <c r="DR7" s="3" t="n">
         <v>33.7456</v>
+      </c>
+      <c r="DS7" s="3" t="n">
+        <v>34.0442</v>
       </c>
     </row>
     <row r="8">
@@ -10655,16 +10724,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.5881</v>
+        <v>36.165</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57104.4161433</v>
+        <v>58030.105845</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7104.416143299997</v>
+        <v>8030.105844999998</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.142088322866</v>
+        <v>0.1606021169</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -11004,6 +11073,9 @@
       </c>
       <c r="DR8" s="3" t="n">
         <v>35.5881</v>
+      </c>
+      <c r="DS8" s="3" t="n">
+        <v>36.165</v>
       </c>
     </row>
     <row r="9">
@@ -11029,16 +11101,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.4029</v>
+        <v>44.2928</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>139730.9924397</v>
+        <v>142595.9302704</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>39730.9924397</v>
+        <v>42595.93027040001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.397309924397</v>
+        <v>0.4259593027040001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -11372,6 +11444,9 @@
       </c>
       <c r="DR9" s="3" t="n">
         <v>43.4029</v>
+      </c>
+      <c r="DS9" s="3" t="n">
+        <v>44.2928</v>
       </c>
     </row>
     <row r="10">
@@ -11397,16 +11472,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.2809</v>
+        <v>48.8744</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>137439.2585131</v>
+        <v>139128.7506296</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>37439.25851310001</v>
+        <v>39128.75062960002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3743925851310001</v>
+        <v>0.3912875062960002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -11740,6 +11815,9 @@
       </c>
       <c r="DR10" s="3" t="n">
         <v>48.2809</v>
+      </c>
+      <c r="DS10" s="3" t="n">
+        <v>48.8744</v>
       </c>
     </row>
     <row r="11">
@@ -11765,16 +11843,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>110.7336</v>
+        <v>111.4383</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>33321.8441784</v>
+        <v>33533.9017977</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>3321.844178399995</v>
+        <v>3533.901797699997</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.1107281392799998</v>
+        <v>0.1177967265899999</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -12108,6 +12186,9 @@
       </c>
       <c r="DR11" s="3" t="n">
         <v>110.7336</v>
+      </c>
+      <c r="DS11" s="3" t="n">
+        <v>111.4383</v>
       </c>
     </row>
     <row r="12">
@@ -12133,16 +12214,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.493</v>
+        <v>222.03</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102644.342346</v>
+        <v>103359.84966</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2644.34234599999</v>
+        <v>3359.849659999993</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.0264434234599999</v>
+        <v>0.03359849659999992</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -12482,6 +12563,9 @@
       </c>
       <c r="DR12" s="3" t="n">
         <v>220.493</v>
+      </c>
+      <c r="DS12" s="3" t="n">
+        <v>222.03</v>
       </c>
     </row>
     <row r="13">
@@ -12507,16 +12591,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.777</v>
+        <v>21.988</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>252343.274085</v>
+        <v>254788.25874</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>52343.27408500001</v>
+        <v>54788.25873999999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2617163704250001</v>
+        <v>0.2739412937</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -12856,6 +12940,9 @@
       </c>
       <c r="DR13" s="3" t="n">
         <v>21.777</v>
+      </c>
+      <c r="DS13" s="3" t="n">
+        <v>21.988</v>
       </c>
     </row>
     <row r="14">
@@ -12881,16 +12968,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.0609</v>
+        <v>39.1406</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>140916.3372054</v>
+        <v>141203.8634036</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>40916.33720539999</v>
+        <v>41203.8634036</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4091633720539999</v>
+        <v>0.412038634036</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -13224,6 +13311,9 @@
       </c>
       <c r="DR14" s="3" t="n">
         <v>39.0609</v>
+      </c>
+      <c r="DS14" s="3" t="n">
+        <v>39.1406</v>
       </c>
     </row>
     <row r="15">
@@ -13249,16 +13339,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.45</v>
+        <v>11.6</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>111568.19315</v>
+        <v>113029.7852</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>11568.19314999999</v>
+        <v>13029.7852</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1156819314999999</v>
+        <v>0.130297852</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -13598,6 +13688,9 @@
       </c>
       <c r="DR15" s="3" t="n">
         <v>11.45</v>
+      </c>
+      <c r="DS15" s="3" t="n">
+        <v>11.6</v>
       </c>
     </row>
     <row r="16">
@@ -13623,16 +13716,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>26.0122</v>
+        <v>26.1765</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>148865.9477216</v>
+        <v>149806.224792</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>48865.94772160001</v>
+        <v>49806.22479199999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4886594772160001</v>
+        <v>0.4980622479199999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -13966,6 +14059,9 @@
       </c>
       <c r="DR16" s="3" t="n">
         <v>26.0122</v>
+      </c>
+      <c r="DS16" s="3" t="n">
+        <v>26.1765</v>
       </c>
     </row>
     <row r="17">
@@ -13991,16 +14087,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7361</v>
+        <v>16.8148</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55330.5005577</v>
+        <v>55590.6872436</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5330.500557699997</v>
+        <v>5590.687243600005</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1066100111539999</v>
+        <v>0.1118137448720001</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -14334,6 +14430,9 @@
       </c>
       <c r="DR17" s="3" t="n">
         <v>16.7361</v>
+      </c>
+      <c r="DS17" s="3" t="n">
+        <v>16.8148</v>
       </c>
     </row>
     <row r="18">
@@ -14359,16 +14458,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.54</v>
+        <v>45.99</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85908.29544</v>
+        <v>86757.19164</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5908.295440000002</v>
+        <v>6757.191640000005</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.07385369300000003</v>
+        <v>0.08446489550000005</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -14708,6 +14807,9 @@
       </c>
       <c r="DR18" s="3" t="n">
         <v>45.54</v>
+      </c>
+      <c r="DS18" s="3" t="n">
+        <v>45.99</v>
       </c>
     </row>
     <row r="19">
@@ -14733,16 +14835,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.5475</v>
+        <v>13.7612</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>195988.512385</v>
+        <v>199080.0602792</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>45988.51238499998</v>
+        <v>49080.0602792</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3065900825666665</v>
+        <v>0.3272004018613333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -15076,6 +15178,9 @@
       </c>
       <c r="DR19" s="3" t="n">
         <v>13.5475</v>
+      </c>
+      <c r="DS19" s="3" t="n">
+        <v>13.7612</v>
       </c>
     </row>
     <row r="20">
@@ -15101,16 +15206,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.720000000000001</v>
+        <v>9.81</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>255206.40516</v>
+        <v>257569.42743</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>5206.405160000024</v>
+        <v>7569.427430000011</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.02082562064000009</v>
+        <v>0.03027770972000004</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -15450,6 +15555,9 @@
       </c>
       <c r="DR20" s="3" t="n">
         <v>9.720000000000001</v>
+      </c>
+      <c r="DS20" s="3" t="n">
+        <v>9.81</v>
       </c>
     </row>
     <row r="21">
@@ -15475,16 +15583,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.3786</v>
+        <v>112.803</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>169212.9404574</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>-787.0595425999782</v>
-      </c>
-      <c r="I21" s="13" t="n">
-        <v>-0.004629762015293989</v>
+        <v>171376.972977</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>1376.972976999998</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>0.008099841041176456</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -15824,6 +15932,9 @@
       </c>
       <c r="DR21" s="3" t="n">
         <v>111.3786</v>
+      </c>
+      <c r="DS21" s="3" t="n">
+        <v>112.803</v>
       </c>
     </row>
     <row r="22">
@@ -15849,16 +15960,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.646</v>
+        <v>44.791</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68507.50116</v>
+        <v>68729.99786</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8507.50116</v>
+        <v>8729.997860000003</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.141791686</v>
+        <v>0.1454999643333334</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -16192,6 +16303,9 @@
       </c>
       <c r="DR22" s="3" t="n">
         <v>44.646</v>
+      </c>
+      <c r="DS22" s="3" t="n">
+        <v>44.791</v>
       </c>
     </row>
     <row r="23">
@@ -16217,16 +16331,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.0073</v>
+        <v>62.4221</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>168440.7842091</v>
+        <v>169567.5747207</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>18440.78420910001</v>
+        <v>19567.57472070001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.122938561394</v>
+        <v>0.1304504981380001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -16566,6 +16680,9 @@
       </c>
       <c r="DR23" s="3" t="n">
         <v>62.0073</v>
+      </c>
+      <c r="DS23" s="3" t="n">
+        <v>62.4221</v>
       </c>
     </row>
     <row r="24">
@@ -16591,16 +16708,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.8872</v>
+        <v>25.9274</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>94058.1900592</v>
+        <v>94204.2521764</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-5941.809940799998</v>
+        <v>-5795.747823600002</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.05941809940799998</v>
+        <v>-0.05795747823600002</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -16934,6 +17051,9 @@
       </c>
       <c r="DR24" s="3" t="n">
         <v>25.8872</v>
+      </c>
+      <c r="DS24" s="3" t="n">
+        <v>25.9274</v>
       </c>
     </row>
     <row r="25">
@@ -16959,16 +17079,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.549</v>
+        <v>12.693</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>206075.587026</v>
+        <v>208440.308082</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>6075.587025999994</v>
+        <v>8440.308081999974</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.03037793512999997</v>
+        <v>0.04220154040999987</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -17305,6 +17425,9 @@
       </c>
       <c r="DR25" s="3" t="n">
         <v>12.549</v>
+      </c>
+      <c r="DS25" s="3" t="n">
+        <v>12.693</v>
       </c>
     </row>
     <row r="26">
@@ -17330,16 +17453,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.6702</v>
+        <v>10.7515</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>127420.487393</v>
+        <v>128391.3488225</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>17420.48739299999</v>
+        <v>18391.3488225</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1583680672090908</v>
+        <v>0.1671940802045455</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -17676,6 +17799,9 @@
       </c>
       <c r="DR26" s="3" t="n">
         <v>10.6702</v>
+      </c>
+      <c r="DS26" s="3" t="n">
+        <v>10.7515</v>
       </c>
     </row>
     <row r="27">
@@ -17701,16 +17827,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>69.2222</v>
+        <v>70.1572</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>111507.273092</v>
+        <v>113013.427192</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>1507.273091999989</v>
+        <v>3013.427192000003</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.01370248265454535</v>
+        <v>0.02739479265454548</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -18050,6 +18176,9 @@
       </c>
       <c r="DR27" s="3" t="n">
         <v>69.2222</v>
+      </c>
+      <c r="DS27" s="3" t="n">
+        <v>70.1572</v>
       </c>
     </row>
     <row r="28">
@@ -18075,16 +18204,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>115.0356</v>
+        <v>116.0388</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>380383.2719892</v>
+        <v>383700.5102916</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>383.2719892000314</v>
+        <v>3700.510291600018</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.001008610497894819</v>
+        <v>0.009738184977894783</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -18424,6 +18553,9 @@
       </c>
       <c r="DR28" s="3" t="n">
         <v>115.0356</v>
+      </c>
+      <c r="DS28" s="3" t="n">
+        <v>116.0388</v>
       </c>
     </row>
     <row r="29">
@@ -18449,16 +18581,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.0227</v>
+        <v>12.2413</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>115462.4400581</v>
+        <v>117561.8095339</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>15462.44005809999</v>
+        <v>17561.8095339</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1546244005809999</v>
+        <v>0.175618095339</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -18792,6 +18924,9 @@
       </c>
       <c r="DR29" s="3" t="n">
         <v>12.0227</v>
+      </c>
+      <c r="DS29" s="3" t="n">
+        <v>12.2413</v>
       </c>
     </row>
     <row r="30">
@@ -18817,16 +18952,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.2023</v>
+        <v>17.3478</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>127225.8196803</v>
+        <v>128301.9174558</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>27225.8196803</v>
+        <v>28301.91745579999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.272258196803</v>
+        <v>0.283019174558</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -19160,6 +19295,9 @@
       </c>
       <c r="DR30" s="3" t="n">
         <v>17.2023</v>
+      </c>
+      <c r="DS30" s="3" t="n">
+        <v>17.3478</v>
       </c>
     </row>
     <row r="31">
@@ -19185,16 +19323,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>400.5655</v>
+        <v>405.3828</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>106582.46824</v>
+        <v>107864.255424</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>6582.468239999987</v>
+        <v>7864.255423999988</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.06582468239999988</v>
+        <v>0.07864255423999988</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -19531,6 +19669,9 @@
       </c>
       <c r="DR31" s="3" t="n">
         <v>400.5655</v>
+      </c>
+      <c r="DS31" s="3" t="n">
+        <v>405.3828</v>
       </c>
     </row>
     <row r="32">
@@ -19556,16 +19697,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.65</v>
+        <v>10.77</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>225140.574</v>
+        <v>227677.3692</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>25140.57399999999</v>
+        <v>27677.36919999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.12570287</v>
+        <v>0.1383868459999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -19905,6 +20046,9 @@
       </c>
       <c r="DR32" s="3" t="n">
         <v>10.65</v>
+      </c>
+      <c r="DS32" s="3" t="n">
+        <v>10.77</v>
       </c>
     </row>
     <row r="33">
@@ -19930,16 +20074,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.59</v>
+        <v>19.83</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>70203.5076</v>
+        <v>71063.58119999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>10203.5076</v>
+        <v>11063.58119999999</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.17005846</v>
+        <v>0.1843930199999998</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -20273,6 +20417,9 @@
       </c>
       <c r="DR33" s="3" t="n">
         <v>19.59</v>
+      </c>
+      <c r="DS33" s="3" t="n">
+        <v>19.83</v>
       </c>
     </row>
     <row r="34">
@@ -20298,16 +20445,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>221.5816</v>
+        <v>222.9056</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>77892.8014296</v>
+        <v>78358.2284736</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-2107.198570399996</v>
+        <v>-1641.7715264</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.02633998212999995</v>
+        <v>-0.02052214408</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -20644,6 +20791,9 @@
       </c>
       <c r="DR34" s="3" t="n">
         <v>221.5816</v>
+      </c>
+      <c r="DS34" s="3" t="n">
+        <v>222.9056</v>
       </c>
     </row>
     <row r="35">
@@ -20669,16 +20819,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.08</v>
+        <v>16.38</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>114737.60184</v>
+        <v>116878.22874</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>14737.60183999999</v>
+        <v>16878.22873999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1473760183999999</v>
+        <v>0.1687822873999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -21015,6 +21165,9 @@
       </c>
       <c r="DR35" s="3" t="n">
         <v>16.08</v>
+      </c>
+      <c r="DS35" s="3" t="n">
+        <v>16.38</v>
       </c>
     </row>
     <row r="36">
@@ -21040,16 +21193,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>374.9996</v>
+        <v>378.523</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>174639.5637176</v>
+        <v>176280.432238</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>24639.56371759999</v>
+        <v>26280.43223800001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1642637581173332</v>
+        <v>0.1752028815866667</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -21386,6 +21539,9 @@
       </c>
       <c r="DR36" s="3" t="n">
         <v>374.9996</v>
+      </c>
+      <c r="DS36" s="3" t="n">
+        <v>378.523</v>
       </c>
     </row>
     <row r="37">
@@ -21411,16 +21567,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.071</v>
+        <v>17.297</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>64236.27811900001</v>
+        <v>65086.691033</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>14236.27811900001</v>
+        <v>15086.691033</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2847255623800002</v>
+        <v>0.30173382066</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -21757,6 +21913,9 @@
       </c>
       <c r="DR37" s="3" t="n">
         <v>17.071</v>
+      </c>
+      <c r="DS37" s="3" t="n">
+        <v>17.297</v>
       </c>
     </row>
     <row r="38">
@@ -21782,16 +21941,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.6087</v>
+        <v>13.7467</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>81386.5853934</v>
+        <v>82211.8919094</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1386.585393400004</v>
+        <v>2211.891909400001</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.01733231741750005</v>
+        <v>0.02764864886750001</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -22125,6 +22284,9 @@
       </c>
       <c r="DR38" s="3" t="n">
         <v>13.6087</v>
+      </c>
+      <c r="DS38" s="3" t="n">
+        <v>13.7467</v>
       </c>
     </row>
     <row r="39">
@@ -22150,16 +22312,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1026.087</v>
+        <v>1026.4947</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51182.245647</v>
+        <v>51202.5821307</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1182.245646999996</v>
+        <v>1202.582130700001</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02364491293999992</v>
+        <v>0.02405164261400001</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -22493,6 +22655,9 @@
       </c>
       <c r="DR39" s="3" t="n">
         <v>1026.087</v>
+      </c>
+      <c r="DS39" s="3" t="n">
+        <v>1026.4947</v>
       </c>
     </row>
     <row r="40">
@@ -22518,16 +22683,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.5252</v>
+        <v>20.6792</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>103468.0873804</v>
+        <v>104244.4055384</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>3468.087380400015</v>
+        <v>4244.405538400009</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.03468087380400015</v>
+        <v>0.0424440553840001</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -22864,6 +23029,9 @@
       </c>
       <c r="DR40" s="3" t="n">
         <v>20.5252</v>
+      </c>
+      <c r="DS40" s="3" t="n">
+        <v>20.6792</v>
       </c>
     </row>
     <row r="41">
@@ -22876,13 +23044,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5022377.6381402</v>
+        <v>5071456.2288884</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>552377.6381402001</v>
+        <v>601456.2288884</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1235744156913199</v>
+        <v>0.1345539661942729</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-08
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-07 08:06 IST</t>
+          <t>Generated: 2026-10-08 08:23 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5071456.2288884</v>
+        <v>5052720.4099612</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>601456.2288883999</v>
+        <v>582720.4099612003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1345539661942729</v>
+        <v>0.1303625078212976</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>530715.5012588501</v>
+        <v>522408.5021286011</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-60066.51874114992</v>
+        <v>-68373.51787139894</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1016728957681378</v>
+        <v>-0.1157339180217417</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5602171.73014725</v>
+        <v>5575128.912089801</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>541389.7101472504</v>
+        <v>514346.8920898018</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1069774805568983</v>
+        <v>0.1016338759616843</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-07</t>
+          <t>Last snapshot: 2026-10-08</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EW19"/>
+  <dimension ref="A1:EX19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -772,6 +772,7 @@
     <col width="21" customWidth="1" min="151" max="151"/>
     <col width="20" customWidth="1" min="152" max="152"/>
     <col width="21" customWidth="1" min="153" max="153"/>
+    <col width="21" customWidth="1" min="154" max="154"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1540,6 +1541,11 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="EX1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1559,13 +1565,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>581.2000122070312</v>
+        <v>570.6500244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46496.0009765625</v>
+        <v>45652.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2678.490976562498</v>
+        <v>1834.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2001,6 +2007,9 @@
       </c>
       <c r="EW2" s="3" t="n">
         <v>581.2000122070312</v>
+      </c>
+      <c r="EX2" s="3" t="n">
+        <v>570.6500244140625</v>
       </c>
     </row>
     <row r="3">
@@ -2048,13 +2057,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1436.199951171875</v>
+        <v>1421.900024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28723.9990234375</v>
+        <v>28438.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3380.580976562502</v>
+        <v>-3666.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2493,6 +2502,9 @@
       </c>
       <c r="EW4" s="3" t="n">
         <v>1436.199951171875</v>
+      </c>
+      <c r="EX4" s="3" t="n">
+        <v>1421.900024414062</v>
       </c>
     </row>
     <row r="5">
@@ -2513,13 +2525,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>484.7999877929688</v>
+        <v>471.9500122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9695.999755859375</v>
+        <v>9439.000244140625</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4517.100244140625</v>
+        <v>-4774.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2958,6 +2970,9 @@
       </c>
       <c r="EW5" s="3" t="n">
         <v>484.7999877929688</v>
+      </c>
+      <c r="EX5" s="3" t="n">
+        <v>471.9500122070312</v>
       </c>
     </row>
     <row r="6">
@@ -2978,13 +2993,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>393.7999877929688</v>
+        <v>377.5499877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15751.99951171875</v>
+        <v>15101.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1750.240488281252</v>
+        <v>-2400.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3423,6 +3438,9 @@
       </c>
       <c r="EW6" s="3" t="n">
         <v>393.7999877929688</v>
+      </c>
+      <c r="EX6" s="3" t="n">
+        <v>377.5499877929688</v>
       </c>
     </row>
     <row r="7">
@@ -3443,13 +3461,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>309</v>
+        <v>288.4500122070312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>30900</v>
+        <v>28845.00122070312</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4466.18</v>
+        <v>2411.181220703125</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3888,6 +3906,9 @@
       </c>
       <c r="EW7" s="3" t="n">
         <v>309</v>
+      </c>
+      <c r="EX7" s="3" t="n">
+        <v>288.4500122070312</v>
       </c>
     </row>
     <row r="8">
@@ -3935,13 +3956,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.82999992370605</v>
+        <v>14.40999984741211</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22244.99988555908</v>
+        <v>21614.99977111816</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8805.170114440916</v>
+        <v>-9435.170228881834</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4380,6 +4401,9 @@
       </c>
       <c r="EW9" s="3" t="n">
         <v>14.82999992370605</v>
+      </c>
+      <c r="EX9" s="3" t="n">
+        <v>14.40999984741211</v>
       </c>
     </row>
     <row r="10">
@@ -4400,13 +4424,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>452.4500122070312</v>
+        <v>445.4500122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45245.00122070312</v>
+        <v>44545.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6253.478779296878</v>
+        <v>-6953.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4845,6 +4869,9 @@
       </c>
       <c r="EW10" s="3" t="n">
         <v>452.4500122070312</v>
+      </c>
+      <c r="EX10" s="3" t="n">
+        <v>445.4500122070312</v>
       </c>
     </row>
     <row r="11">
@@ -4865,13 +4892,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>13</v>
+        <v>14.14000034332275</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>13000</v>
+        <v>14140.00034332275</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3158.790000000001</v>
+        <v>4298.790343322755</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5310,6 +5337,9 @@
       </c>
       <c r="EW11" s="3" t="n">
         <v>13</v>
+      </c>
+      <c r="EX11" s="3" t="n">
+        <v>14.14000034332275</v>
       </c>
     </row>
     <row r="12">
@@ -5330,13 +5360,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2525.300048828125</v>
+        <v>2497.199951171875</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25253.00048828125</v>
+        <v>24971.99951171875</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2470.24951171875</v>
+        <v>-2751.25048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5775,6 +5805,9 @@
       </c>
       <c r="EW12" s="3" t="n">
         <v>2525.300048828125</v>
+      </c>
+      <c r="EX12" s="3" t="n">
+        <v>2497.199951171875</v>
       </c>
     </row>
     <row r="13">
@@ -5795,13 +5828,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>38.59000015258789</v>
+        <v>36.59999847412109</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23154.00009155273</v>
+        <v>21959.99908447266</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11877.75990844727</v>
+        <v>-13071.76091552735</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6240,6 +6273,9 @@
       </c>
       <c r="EW13" s="3" t="n">
         <v>38.59000015258789</v>
+      </c>
+      <c r="EX13" s="3" t="n">
+        <v>36.59999847412109</v>
       </c>
     </row>
     <row r="14">
@@ -6260,13 +6296,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>611.75</v>
+        <v>595.5499877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>30587.5</v>
+        <v>29777.49938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11875.01</v>
+        <v>-12685.01061035156</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6705,6 +6741,9 @@
       </c>
       <c r="EW14" s="3" t="n">
         <v>611.75</v>
+      </c>
+      <c r="EX14" s="3" t="n">
+        <v>595.5499877929688</v>
       </c>
     </row>
     <row r="15">
@@ -6779,13 +6818,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>468.1499938964844</v>
+        <v>452.0499877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23407.49969482422</v>
+        <v>22602.49938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1652.96969482422</v>
+        <v>847.9693896484387</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7224,6 +7263,9 @@
       </c>
       <c r="EW17" s="3" t="n">
         <v>468.1499938964844</v>
+      </c>
+      <c r="EX17" s="3" t="n">
+        <v>452.0499877929688</v>
       </c>
     </row>
     <row r="18">
@@ -7244,13 +7286,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>344.8500061035156</v>
+        <v>335.5</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34485.00061035156</v>
+        <v>33550</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12155.81938964844</v>
+        <v>-13090.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7689,6 +7731,9 @@
       </c>
       <c r="EW18" s="3" t="n">
         <v>344.8500061035156</v>
+      </c>
+      <c r="EX18" s="3" t="n">
+        <v>335.5</v>
       </c>
     </row>
     <row r="19">
@@ -7701,10 +7746,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>530715.5012588501</v>
+        <v>522408.5021286011</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-60066.51874114991</v>
+        <v>-68373.51787139893</v>
       </c>
     </row>
   </sheetData>
@@ -7718,7 +7763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DS41"/>
+  <dimension ref="A1:DT41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7844,6 +7889,7 @@
     <col width="13" customWidth="1" min="121" max="121"/>
     <col width="13" customWidth="1" min="122" max="122"/>
     <col width="13" customWidth="1" min="123" max="123"/>
+    <col width="13" customWidth="1" min="124" max="124"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8462,6 +8508,11 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="DT1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8486,16 +8537,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>58.5201</v>
+        <v>58.2614</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>65687.7588882</v>
+        <v>65397.3727948</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>15687.7588882</v>
+        <v>15397.3727948</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.313755177764</v>
+        <v>0.307947455896</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8838,6 +8889,9 @@
       </c>
       <c r="DS2" s="3" t="n">
         <v>58.5201</v>
+      </c>
+      <c r="DT2" s="3" t="n">
+        <v>58.2614</v>
       </c>
     </row>
     <row r="3">
@@ -8863,16 +8917,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>27.2216</v>
+        <v>27.0825</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>66834.8262008</v>
+        <v>66493.30607250001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>6834.826200800002</v>
+        <v>6493.30607250001</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.1139137700133334</v>
+        <v>0.1082217678750002</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9209,6 +9263,9 @@
       </c>
       <c r="DS3" s="3" t="n">
         <v>27.2216</v>
+      </c>
+      <c r="DT3" s="3" t="n">
+        <v>27.0825</v>
       </c>
     </row>
     <row r="4">
@@ -9234,16 +9291,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>13.04</v>
+        <v>12.87</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>250447.45272</v>
+        <v>247182.41691</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>70447.45272</v>
+        <v>67182.41691</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3913747373333333</v>
+        <v>0.3732356495</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9580,6 +9637,9 @@
       </c>
       <c r="DS4" s="3" t="n">
         <v>13.04</v>
+      </c>
+      <c r="DT4" s="3" t="n">
+        <v>12.87</v>
       </c>
     </row>
     <row r="5">
@@ -9605,16 +9665,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.0642</v>
+        <v>8.9625</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>166365.1244496</v>
+        <v>164498.5137</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-43634.8755504</v>
+        <v>-45501.48629999999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2077851216685714</v>
+        <v>-0.2166737442857142</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -9951,6 +10011,9 @@
       </c>
       <c r="DS5" s="3" t="n">
         <v>9.0642</v>
+      </c>
+      <c r="DT5" s="3" t="n">
+        <v>8.9625</v>
       </c>
     </row>
     <row r="6">
@@ -9976,16 +10039,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.4421</v>
+        <v>11.388</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>48388.3777317</v>
+        <v>48159.590076</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-1611.622268300001</v>
+        <v>-1840.409924</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.03223244536600003</v>
+        <v>-0.03680819847999999</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -10328,6 +10391,9 @@
       </c>
       <c r="DS6" s="3" t="n">
         <v>11.4421</v>
+      </c>
+      <c r="DT6" s="3" t="n">
+        <v>11.388</v>
       </c>
     </row>
     <row r="7">
@@ -10353,16 +10419,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.0442</v>
+        <v>33.7253</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75102.86696799999</v>
+        <v>74399.360812</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15102.86696799999</v>
+        <v>14399.360812</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2517144494666664</v>
+        <v>0.2399893468666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -10699,6 +10765,9 @@
       </c>
       <c r="DS7" s="3" t="n">
         <v>34.0442</v>
+      </c>
+      <c r="DT7" s="3" t="n">
+        <v>33.7253</v>
       </c>
     </row>
     <row r="8">
@@ -10724,16 +10793,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>36.165</v>
+        <v>36.8714</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>58030.105845</v>
+        <v>59163.5903402</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>8030.105844999998</v>
+        <v>9163.590340200004</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1606021169</v>
+        <v>0.1832718068040001</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -11076,6 +11145,9 @@
       </c>
       <c r="DS8" s="3" t="n">
         <v>36.165</v>
+      </c>
+      <c r="DT8" s="3" t="n">
+        <v>36.8714</v>
       </c>
     </row>
     <row r="9">
@@ -11101,16 +11173,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>44.2928</v>
+        <v>43.2112</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>142595.9302704</v>
+        <v>139113.8348016</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>42595.93027040001</v>
+        <v>39113.83480159999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.4259593027040001</v>
+        <v>0.3911383480159999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -11447,6 +11519,9 @@
       </c>
       <c r="DS9" s="3" t="n">
         <v>44.2928</v>
+      </c>
+      <c r="DT9" s="3" t="n">
+        <v>43.2112</v>
       </c>
     </row>
     <row r="10">
@@ -11472,16 +11547,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.8744</v>
+        <v>48.6639</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>139128.7506296</v>
+        <v>138529.5289101</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>39128.75062960002</v>
+        <v>38529.52891009999</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3912875062960002</v>
+        <v>0.385295289101</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -11818,6 +11893,9 @@
       </c>
       <c r="DS10" s="3" t="n">
         <v>48.8744</v>
+      </c>
+      <c r="DT10" s="3" t="n">
+        <v>48.6639</v>
       </c>
     </row>
     <row r="11">
@@ -11843,16 +11921,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>111.4383</v>
+        <v>111.0866</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>33533.9017977</v>
+        <v>33428.0685854</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>3533.901797699997</v>
+        <v>3428.068585399997</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.1177967265899999</v>
+        <v>0.1142689528466665</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -12189,6 +12267,9 @@
       </c>
       <c r="DS11" s="3" t="n">
         <v>111.4383</v>
+      </c>
+      <c r="DT11" s="3" t="n">
+        <v>111.0866</v>
       </c>
     </row>
     <row r="12">
@@ -12214,16 +12295,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>222.03</v>
+        <v>220.873</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>103359.84966</v>
+        <v>102821.240706</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3359.849659999993</v>
+        <v>2821.240705999997</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.03359849659999992</v>
+        <v>0.02821240705999997</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -12566,6 +12647,9 @@
       </c>
       <c r="DS12" s="3" t="n">
         <v>222.03</v>
+      </c>
+      <c r="DT12" s="3" t="n">
+        <v>220.873</v>
       </c>
     </row>
     <row r="13">
@@ -12591,16 +12675,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.988</v>
+        <v>21.916</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>254788.25874</v>
+        <v>253953.95118</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>54788.25873999999</v>
+        <v>53953.95118</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2739412937</v>
+        <v>0.2697697559</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -12943,6 +13027,9 @@
       </c>
       <c r="DS13" s="3" t="n">
         <v>21.988</v>
+      </c>
+      <c r="DT13" s="3" t="n">
+        <v>21.916</v>
       </c>
     </row>
     <row r="14">
@@ -12968,16 +13055,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.1406</v>
+        <v>38.6251</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>141203.8634036</v>
+        <v>139344.1425106</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>41203.8634036</v>
+        <v>39344.14251060001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.412038634036</v>
+        <v>0.3934414251060001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -13314,6 +13401,9 @@
       </c>
       <c r="DS14" s="3" t="n">
         <v>39.1406</v>
+      </c>
+      <c r="DT14" s="3" t="n">
+        <v>38.6251</v>
       </c>
     </row>
     <row r="15">
@@ -13339,16 +13429,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.6</v>
+        <v>11.54</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>113029.7852</v>
+        <v>112445.14838</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>13029.7852</v>
+        <v>12445.14838</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.130297852</v>
+        <v>0.1244514838</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -13691,6 +13781,9 @@
       </c>
       <c r="DS15" s="3" t="n">
         <v>11.6</v>
+      </c>
+      <c r="DT15" s="3" t="n">
+        <v>11.54</v>
       </c>
     </row>
     <row r="16">
@@ -13716,16 +13809,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>26.1765</v>
+        <v>26.1743</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>149806.224792</v>
+        <v>149793.6343504</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>49806.22479199999</v>
+        <v>49793.63435039998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4980622479199999</v>
+        <v>0.4979363435039998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -14062,6 +14155,9 @@
       </c>
       <c r="DS16" s="3" t="n">
         <v>26.1765</v>
+      </c>
+      <c r="DT16" s="3" t="n">
+        <v>26.1743</v>
       </c>
     </row>
     <row r="17">
@@ -14087,16 +14183,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8148</v>
+        <v>16.7436</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55590.6872436</v>
+        <v>55355.2959852</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5590.687243600005</v>
+        <v>5355.295985199999</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1118137448720001</v>
+        <v>0.107105919704</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -14433,6 +14529,9 @@
       </c>
       <c r="DS17" s="3" t="n">
         <v>16.8148</v>
+      </c>
+      <c r="DT17" s="3" t="n">
+        <v>16.7436</v>
       </c>
     </row>
     <row r="18">
@@ -14458,16 +14557,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.99</v>
+        <v>45.83</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>86757.19164</v>
+        <v>86455.36188</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>6757.191640000005</v>
+        <v>6455.361879999997</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.08446489550000005</v>
+        <v>0.08069202349999996</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -14810,6 +14909,9 @@
       </c>
       <c r="DS18" s="3" t="n">
         <v>45.99</v>
+      </c>
+      <c r="DT18" s="3" t="n">
+        <v>45.83</v>
       </c>
     </row>
     <row r="19">
@@ -14835,16 +14937,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.7612</v>
+        <v>13.7599</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>199080.0602792</v>
+        <v>199061.2534834</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>49080.0602792</v>
+        <v>49061.25348339998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3272004018613333</v>
+        <v>0.3270750232226665</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -15181,6 +15283,9 @@
       </c>
       <c r="DS19" s="3" t="n">
         <v>13.7612</v>
+      </c>
+      <c r="DT19" s="3" t="n">
+        <v>13.7599</v>
       </c>
     </row>
     <row r="20">
@@ -15206,16 +15311,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.81</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>257569.42743</v>
+        <v>257044.31137</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>7569.427430000011</v>
+        <v>7044.311369999981</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.03027770972000004</v>
+        <v>0.02817724547999993</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -15558,6 +15663,9 @@
       </c>
       <c r="DS20" s="3" t="n">
         <v>9.81</v>
+      </c>
+      <c r="DT20" s="3" t="n">
+        <v>9.789999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -15583,16 +15691,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>112.803</v>
+        <v>112.5001</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>171376.972977</v>
+        <v>170916.7894259</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>1376.972976999998</v>
+        <v>916.7894259000022</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.008099841041176456</v>
+        <v>0.005392878975882366</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -15935,6 +16043,9 @@
       </c>
       <c r="DS21" s="3" t="n">
         <v>112.803</v>
+      </c>
+      <c r="DT21" s="3" t="n">
+        <v>112.5001</v>
       </c>
     </row>
     <row r="22">
@@ -15960,16 +16071,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.791</v>
+        <v>44.206</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68729.99786</v>
+        <v>67832.33876000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8729.997860000003</v>
+        <v>7832.338760000013</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1454999643333334</v>
+        <v>0.1305389793333336</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -16306,6 +16417,9 @@
       </c>
       <c r="DS22" s="3" t="n">
         <v>44.791</v>
+      </c>
+      <c r="DT22" s="3" t="n">
+        <v>44.206</v>
       </c>
     </row>
     <row r="23">
@@ -16331,16 +16445,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.4221</v>
+        <v>61.9087</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>169567.5747207</v>
+        <v>168172.9405629</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>19567.57472070001</v>
+        <v>18172.94056290001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1304504981380001</v>
+        <v>0.1211529370860001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -16683,6 +16797,9 @@
       </c>
       <c r="DS23" s="3" t="n">
         <v>62.4221</v>
+      </c>
+      <c r="DT23" s="3" t="n">
+        <v>61.9087</v>
       </c>
     </row>
     <row r="24">
@@ -16708,16 +16825,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.9274</v>
+        <v>25.8452</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>94204.2521764</v>
+        <v>93905.58784719999</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-5795.747823600002</v>
+        <v>-6094.412152800011</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.05795747823600002</v>
+        <v>-0.06094412152800011</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -17054,6 +17171,9 @@
       </c>
       <c r="DS24" s="3" t="n">
         <v>25.9274</v>
+      </c>
+      <c r="DT24" s="3" t="n">
+        <v>25.8452</v>
       </c>
     </row>
     <row r="25">
@@ -17079,16 +17199,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.693</v>
+        <v>12.7091</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>208440.308082</v>
+        <v>208704.6970334</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>8440.308081999974</v>
+        <v>8704.697033399978</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.04220154040999987</v>
+        <v>0.04352348516699989</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -17428,6 +17548,9 @@
       </c>
       <c r="DS25" s="3" t="n">
         <v>12.693</v>
+      </c>
+      <c r="DT25" s="3" t="n">
+        <v>12.7091</v>
       </c>
     </row>
     <row r="26">
@@ -17453,16 +17576,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.7515</v>
+        <v>10.8119</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>128391.3488225</v>
+        <v>129112.6284085</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>18391.3488225</v>
+        <v>19112.62840849999</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1671940802045455</v>
+        <v>0.1737511673499999</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -17802,6 +17925,9 @@
       </c>
       <c r="DS26" s="3" t="n">
         <v>10.7515</v>
+      </c>
+      <c r="DT26" s="3" t="n">
+        <v>10.8119</v>
       </c>
     </row>
     <row r="27">
@@ -17827,16 +17953,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>70.1572</v>
+        <v>69.9776</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>113013.427192</v>
+        <v>112724.116736</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>3013.427192000003</v>
+        <v>2724.116735999982</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.02739479265454548</v>
+        <v>0.02476469759999983</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -18179,6 +18305,9 @@
       </c>
       <c r="DS27" s="3" t="n">
         <v>70.1572</v>
+      </c>
+      <c r="DT27" s="3" t="n">
+        <v>69.9776</v>
       </c>
     </row>
     <row r="28">
@@ -18204,16 +18333,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>116.0388</v>
+        <v>116.4021</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>383700.5102916</v>
+        <v>384901.8187797</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>3700.510291600018</v>
+        <v>4901.818779700028</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.009738184977894783</v>
+        <v>0.01289952310447376</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -18556,6 +18685,9 @@
       </c>
       <c r="DS28" s="3" t="n">
         <v>116.0388</v>
+      </c>
+      <c r="DT28" s="3" t="n">
+        <v>116.4021</v>
       </c>
     </row>
     <row r="29">
@@ -18581,16 +18713,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.2413</v>
+        <v>12.0683</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>117561.8095339</v>
+        <v>115900.3689149</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>17561.8095339</v>
+        <v>15900.3689149</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.175618095339</v>
+        <v>0.159003689149</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -18927,6 +19059,9 @@
       </c>
       <c r="DS29" s="3" t="n">
         <v>12.2413</v>
+      </c>
+      <c r="DT29" s="3" t="n">
+        <v>12.0683</v>
       </c>
     </row>
     <row r="30">
@@ -18952,16 +19087,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.3478</v>
+        <v>17.4214</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>128301.9174558</v>
+        <v>128846.2528254</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>28301.91745579999</v>
+        <v>28846.25282539999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.283019174558</v>
+        <v>0.2884625282539999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -19298,6 +19433,9 @@
       </c>
       <c r="DS30" s="3" t="n">
         <v>17.3478</v>
+      </c>
+      <c r="DT30" s="3" t="n">
+        <v>17.4214</v>
       </c>
     </row>
     <row r="31">
@@ -19323,16 +19461,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>405.3828</v>
+        <v>402.799</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>107864.255424</v>
+        <v>107176.75792</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>7864.255423999988</v>
+        <v>7176.757919999989</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.07864255423999988</v>
+        <v>0.07176757919999989</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -19672,6 +19810,9 @@
       </c>
       <c r="DS31" s="3" t="n">
         <v>405.3828</v>
+      </c>
+      <c r="DT31" s="3" t="n">
+        <v>402.799</v>
       </c>
     </row>
     <row r="32">
@@ -19697,16 +19838,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.77</v>
+        <v>10.75</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>227677.3692</v>
+        <v>227254.57</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>27677.36919999999</v>
+        <v>27254.56999999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1383868459999999</v>
+        <v>0.1362728499999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -20049,6 +20190,9 @@
       </c>
       <c r="DS32" s="3" t="n">
         <v>10.77</v>
+      </c>
+      <c r="DT32" s="3" t="n">
+        <v>10.75</v>
       </c>
     </row>
     <row r="33">
@@ -20421,6 +20565,9 @@
       <c r="DS33" s="3" t="n">
         <v>19.83</v>
       </c>
+      <c r="DT33" s="3" t="n">
+        <v>19.83</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -20445,16 +20592,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>222.9056</v>
+        <v>222.7767</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>78358.2284736</v>
+        <v>78312.91612770001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-1641.7715264</v>
+        <v>-1687.083872299991</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.02052214408</v>
+        <v>-0.02108854840374988</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -20794,6 +20941,9 @@
       </c>
       <c r="DS34" s="3" t="n">
         <v>222.9056</v>
+      </c>
+      <c r="DT34" s="3" t="n">
+        <v>222.7767</v>
       </c>
     </row>
     <row r="35">
@@ -20819,16 +20969,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.38</v>
+        <v>16.45</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>116878.22874</v>
+        <v>117377.70835</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>16878.22873999999</v>
+        <v>17377.70834999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1687822873999999</v>
+        <v>0.1737770834999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -21168,6 +21318,9 @@
       </c>
       <c r="DS35" s="3" t="n">
         <v>16.38</v>
+      </c>
+      <c r="DT35" s="3" t="n">
+        <v>16.45</v>
       </c>
     </row>
     <row r="36">
@@ -21193,16 +21346,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>378.523</v>
+        <v>378.49</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>176280.432238</v>
+        <v>176265.06394</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>26280.43223800001</v>
+        <v>26265.06394000002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1752028815866667</v>
+        <v>0.1751004262666668</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -21542,6 +21695,9 @@
       </c>
       <c r="DS36" s="3" t="n">
         <v>378.523</v>
+      </c>
+      <c r="DT36" s="3" t="n">
+        <v>378.49</v>
       </c>
     </row>
     <row r="37">
@@ -21567,16 +21723,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.297</v>
+        <v>17.242</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>65086.691033</v>
+        <v>64879.73213800001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>15086.691033</v>
+        <v>14879.73213800001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.30173382066</v>
+        <v>0.2975946427600001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -21916,6 +22072,9 @@
       </c>
       <c r="DS37" s="3" t="n">
         <v>17.297</v>
+      </c>
+      <c r="DT37" s="3" t="n">
+        <v>17.242</v>
       </c>
     </row>
     <row r="38">
@@ -21941,16 +22100,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.7467</v>
+        <v>13.6496</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>82211.8919094</v>
+        <v>81631.18710719999</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>2211.891909400001</v>
+        <v>1631.187107199992</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.02764864886750001</v>
+        <v>0.0203898388399999</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -22287,6 +22446,9 @@
       </c>
       <c r="DS38" s="3" t="n">
         <v>13.7467</v>
+      </c>
+      <c r="DT38" s="3" t="n">
+        <v>13.6496</v>
       </c>
     </row>
     <row r="39">
@@ -22312,16 +22474,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1026.4947</v>
+        <v>1026.0552</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51202.5821307</v>
+        <v>51180.6594312</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1202.582130700001</v>
+        <v>1180.659431200002</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02405164261400001</v>
+        <v>0.02361318862400003</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -22658,6 +22820,9 @@
       </c>
       <c r="DS39" s="3" t="n">
         <v>1026.4947</v>
+      </c>
+      <c r="DT39" s="3" t="n">
+        <v>1026.0552</v>
       </c>
     </row>
     <row r="40">
@@ -22683,16 +22848,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.6792</v>
+        <v>20.615</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>104244.4055384</v>
+        <v>103920.771605</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>4244.405538400009</v>
+        <v>3920.771604999987</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.0424440553840001</v>
+        <v>0.03920771604999987</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -23032,6 +23197,9 @@
       </c>
       <c r="DS40" s="3" t="n">
         <v>20.6792</v>
+      </c>
+      <c r="DT40" s="3" t="n">
+        <v>20.615</v>
       </c>
     </row>
     <row r="41">
@@ -23044,13 +23212,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5071456.2288884</v>
+        <v>5052720.4099612</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>601456.2288884</v>
+        <v>582720.4099611999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1345539661942729</v>
+        <v>0.1303625078212975</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-10
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-08 08:23 IST</t>
+          <t>Generated: 2026-10-10 08:03 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5052720.4099612</v>
+        <v>5002638.7241529</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>582720.4099612003</v>
+        <v>532638.7241529003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1303625078212976</v>
+        <v>0.1191585512646309</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>522408.5021286011</v>
+        <v>523761.0038642883</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-68373.51787139894</v>
+        <v>-67021.01613571169</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1157339180217417</v>
+        <v>-0.1134445766235602</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5575128.912089801</v>
+        <v>5526399.728017189</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>514346.8920898018</v>
+        <v>465617.7080171891</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1016338759616843</v>
+        <v>0.09200509055262354</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-08</t>
+          <t>Last snapshot: 2026-10-10</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EX19"/>
+  <dimension ref="A1:EY19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -773,6 +773,7 @@
     <col width="20" customWidth="1" min="152" max="152"/>
     <col width="21" customWidth="1" min="153" max="153"/>
     <col width="21" customWidth="1" min="154" max="154"/>
+    <col width="21" customWidth="1" min="155" max="155"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1546,6 +1547,11 @@
           <t>2026-10-08</t>
         </is>
       </c>
+      <c r="EY1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1565,13 +1571,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>570.6500244140625</v>
+        <v>570.4000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45652.001953125</v>
+        <v>45632.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1834.491953124998</v>
+        <v>1814.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2010,6 +2016,9 @@
       </c>
       <c r="EX2" s="3" t="n">
         <v>570.6500244140625</v>
+      </c>
+      <c r="EY2" s="3" t="n">
+        <v>570.4000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -2057,13 +2066,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1421.900024414062</v>
+        <v>1409.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28438.00048828125</v>
+        <v>28196.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3666.579511718752</v>
+        <v>-3908.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2505,6 +2514,9 @@
       </c>
       <c r="EX4" s="3" t="n">
         <v>1421.900024414062</v>
+      </c>
+      <c r="EY4" s="3" t="n">
+        <v>1409.800048828125</v>
       </c>
     </row>
     <row r="5">
@@ -2525,13 +2537,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>471.9500122070312</v>
+        <v>472.0499877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9439.000244140625</v>
+        <v>9440.999755859375</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4774.099755859375</v>
+        <v>-4772.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -2973,6 +2985,9 @@
       </c>
       <c r="EX5" s="3" t="n">
         <v>471.9500122070312</v>
+      </c>
+      <c r="EY5" s="3" t="n">
+        <v>472.0499877929688</v>
       </c>
     </row>
     <row r="6">
@@ -2993,13 +3008,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>377.5499877929688</v>
+        <v>364.9500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15101.99951171875</v>
+        <v>14598.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2400.240488281252</v>
+        <v>-2904.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3441,6 +3456,9 @@
       </c>
       <c r="EX6" s="3" t="n">
         <v>377.5499877929688</v>
+      </c>
+      <c r="EY6" s="3" t="n">
+        <v>364.9500122070312</v>
       </c>
     </row>
     <row r="7">
@@ -3461,13 +3479,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>288.4500122070312</v>
+        <v>293.1000061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>28845.00122070312</v>
+        <v>29310.00061035156</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>2411.181220703125</v>
+        <v>2876.180610351563</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3909,6 +3927,9 @@
       </c>
       <c r="EX7" s="3" t="n">
         <v>288.4500122070312</v>
+      </c>
+      <c r="EY7" s="3" t="n">
+        <v>293.1000061035156</v>
       </c>
     </row>
     <row r="8">
@@ -3956,13 +3977,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.40999984741211</v>
+        <v>14.52999973297119</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>21614.99977111816</v>
+        <v>21794.99959945679</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-9435.170228881834</v>
+        <v>-9255.170400543211</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4404,6 +4425,9 @@
       </c>
       <c r="EX9" s="3" t="n">
         <v>14.40999984741211</v>
+      </c>
+      <c r="EY9" s="3" t="n">
+        <v>14.52999973297119</v>
       </c>
     </row>
     <row r="10">
@@ -4424,13 +4448,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>445.4500122070312</v>
+        <v>443.5</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44545.00122070312</v>
+        <v>44350</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6953.478779296878</v>
+        <v>-7148.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4872,6 +4896,9 @@
       </c>
       <c r="EX10" s="3" t="n">
         <v>445.4500122070312</v>
+      </c>
+      <c r="EY10" s="3" t="n">
+        <v>443.5</v>
       </c>
     </row>
     <row r="11">
@@ -4892,13 +4919,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>14.14000034332275</v>
+        <v>14.8100004196167</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14140.00034332275</v>
+        <v>14810.0004196167</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4298.790343322755</v>
+        <v>4968.7904196167</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5340,6 +5367,9 @@
       </c>
       <c r="EX11" s="3" t="n">
         <v>14.14000034332275</v>
+      </c>
+      <c r="EY11" s="3" t="n">
+        <v>14.8100004196167</v>
       </c>
     </row>
     <row r="12">
@@ -5360,13 +5390,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2497.199951171875</v>
+        <v>2523.60009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>24971.99951171875</v>
+        <v>25236.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2751.25048828125</v>
+        <v>-2487.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5808,6 +5838,9 @@
       </c>
       <c r="EX12" s="3" t="n">
         <v>2497.199951171875</v>
+      </c>
+      <c r="EY12" s="3" t="n">
+        <v>2523.60009765625</v>
       </c>
     </row>
     <row r="13">
@@ -5828,13 +5861,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>36.59999847412109</v>
+        <v>37.59999847412109</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21959.99908447266</v>
+        <v>22559.99908447266</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-13071.76091552735</v>
+        <v>-12471.76091552735</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6276,6 +6309,9 @@
       </c>
       <c r="EX13" s="3" t="n">
         <v>36.59999847412109</v>
+      </c>
+      <c r="EY13" s="3" t="n">
+        <v>37.59999847412109</v>
       </c>
     </row>
     <row r="14">
@@ -6296,13 +6332,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>595.5499877929688</v>
+        <v>589.75</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>29777.49938964844</v>
+        <v>29487.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12685.01061035156</v>
+        <v>-12975.01</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6744,6 +6780,9 @@
       </c>
       <c r="EX14" s="3" t="n">
         <v>595.5499877929688</v>
+      </c>
+      <c r="EY14" s="3" t="n">
+        <v>589.75</v>
       </c>
     </row>
     <row r="15">
@@ -6818,13 +6857,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>452.0499877929688</v>
+        <v>447.2000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>22602.49938964844</v>
+        <v>22360.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>847.9693896484387</v>
+        <v>605.4706103515637</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7266,6 +7305,9 @@
       </c>
       <c r="EX17" s="3" t="n">
         <v>452.0499877929688</v>
+      </c>
+      <c r="EY17" s="3" t="n">
+        <v>447.2000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -7286,13 +7328,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>335.5</v>
+        <v>342.1499938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>33550</v>
+        <v>34214.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-13090.82</v>
+        <v>-12425.82061035156</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7734,6 +7776,9 @@
       </c>
       <c r="EX18" s="3" t="n">
         <v>335.5</v>
+      </c>
+      <c r="EY18" s="3" t="n">
+        <v>342.1499938964844</v>
       </c>
     </row>
     <row r="19">
@@ -7746,10 +7791,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>522408.5021286011</v>
+        <v>523761.0038642883</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-68373.51787139893</v>
+        <v>-67021.01613571167</v>
       </c>
     </row>
   </sheetData>
@@ -7763,7 +7808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DT41"/>
+  <dimension ref="A1:DU41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7774,7 +7819,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -7890,6 +7935,7 @@
     <col width="13" customWidth="1" min="122" max="122"/>
     <col width="13" customWidth="1" min="123" max="123"/>
     <col width="13" customWidth="1" min="124" max="124"/>
+    <col width="13" customWidth="1" min="125" max="125"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8513,6 +8559,11 @@
           <t>2026-10-08</t>
         </is>
       </c>
+      <c r="DU1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8537,16 +8588,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>58.2614</v>
+        <v>58.3132</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>65397.3727948</v>
+        <v>65455.5173624</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>15397.3727948</v>
+        <v>15455.5173624</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.307947455896</v>
+        <v>0.309110347248</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -8892,6 +8943,9 @@
       </c>
       <c r="DT2" s="3" t="n">
         <v>58.2614</v>
+      </c>
+      <c r="DU2" s="3" t="n">
+        <v>58.3132</v>
       </c>
     </row>
     <row r="3">
@@ -8917,16 +8971,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>27.0825</v>
+        <v>27.0969</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>66493.30607250001</v>
+        <v>66528.66113970001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>6493.30607250001</v>
+        <v>6528.661139700009</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.1082217678750002</v>
+        <v>0.1088110189950001</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9266,6 +9320,9 @@
       </c>
       <c r="DT3" s="3" t="n">
         <v>27.0825</v>
+      </c>
+      <c r="DU3" s="3" t="n">
+        <v>27.0969</v>
       </c>
     </row>
     <row r="4">
@@ -9291,16 +9348,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.87</v>
+        <v>12.84</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>247182.41691</v>
+        <v>246606.23412</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>67182.41691</v>
+        <v>66606.23412000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3732356495</v>
+        <v>0.370034634</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9640,6 +9697,9 @@
       </c>
       <c r="DT4" s="3" t="n">
         <v>12.87</v>
+      </c>
+      <c r="DU4" s="3" t="n">
+        <v>12.84</v>
       </c>
     </row>
     <row r="5">
@@ -9665,16 +9725,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.9625</v>
+        <v>8.971500000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>164498.5137</v>
+        <v>164663.700492</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-45501.48629999999</v>
+        <v>-45336.299508</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2166737442857142</v>
+        <v>-0.2158871405142857</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10014,6 +10074,9 @@
       </c>
       <c r="DT5" s="3" t="n">
         <v>8.9625</v>
+      </c>
+      <c r="DU5" s="3" t="n">
+        <v>8.971500000000001</v>
       </c>
     </row>
     <row r="6">
@@ -10039,16 +10102,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.388</v>
+        <v>11.1444</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>48159.590076</v>
+        <v>47129.4112788</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-1840.409924</v>
+        <v>-2870.588721200002</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.03680819847999999</v>
+        <v>-0.05741177442400004</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -10394,6 +10457,9 @@
       </c>
       <c r="DT6" s="3" t="n">
         <v>11.388</v>
+      </c>
+      <c r="DU6" s="3" t="n">
+        <v>11.1444</v>
       </c>
     </row>
     <row r="7">
@@ -10419,16 +10485,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.7253</v>
+        <v>33.8842</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74399.360812</v>
+        <v>74749.900568</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14399.360812</v>
+        <v>14749.900568</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2399893468666666</v>
+        <v>0.2458316761333333</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -10768,6 +10834,9 @@
       </c>
       <c r="DT7" s="3" t="n">
         <v>33.7253</v>
+      </c>
+      <c r="DU7" s="3" t="n">
+        <v>33.8842</v>
       </c>
     </row>
     <row r="8">
@@ -10793,16 +10862,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>36.8714</v>
+        <v>35.8579</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>59163.5903402</v>
+        <v>57537.3353347</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>9163.590340200004</v>
+        <v>7537.335334700001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1832718068040001</v>
+        <v>0.150746706694</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -11148,6 +11217,9 @@
       </c>
       <c r="DT8" s="3" t="n">
         <v>36.8714</v>
+      </c>
+      <c r="DU8" s="3" t="n">
+        <v>35.8579</v>
       </c>
     </row>
     <row r="9">
@@ -11173,16 +11245,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.2112</v>
+        <v>43.1225</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>139113.8348016</v>
+        <v>138828.2746425</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>39113.83480159999</v>
+        <v>38828.27464250001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3911383480159999</v>
+        <v>0.3882827464250001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -11522,6 +11594,9 @@
       </c>
       <c r="DT9" s="3" t="n">
         <v>43.2112</v>
+      </c>
+      <c r="DU9" s="3" t="n">
+        <v>43.1225</v>
       </c>
     </row>
     <row r="10">
@@ -11547,16 +11622,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.6639</v>
+        <v>49.0718</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138529.5289101</v>
+        <v>139690.6811162</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38529.52891009999</v>
+        <v>39690.68111620002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.385295289101</v>
+        <v>0.3969068111620002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -11896,6 +11971,9 @@
       </c>
       <c r="DT10" s="3" t="n">
         <v>48.6639</v>
+      </c>
+      <c r="DU10" s="3" t="n">
+        <v>49.0718</v>
       </c>
     </row>
     <row r="11">
@@ -11921,16 +11999,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>111.0866</v>
+        <v>110.1877</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>33428.0685854</v>
+        <v>33157.5724963</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>3428.068585399997</v>
+        <v>3157.572496300003</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.1142689528466665</v>
+        <v>0.1052524165433334</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -12270,6 +12348,9 @@
       </c>
       <c r="DT11" s="3" t="n">
         <v>111.0866</v>
+      </c>
+      <c r="DU11" s="3" t="n">
+        <v>110.1877</v>
       </c>
     </row>
     <row r="12">
@@ -12295,16 +12376,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.873</v>
+        <v>219.816</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102821.240706</v>
+        <v>102329.183952</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2821.240705999997</v>
+        <v>2329.183951999992</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02821240705999997</v>
+        <v>0.02329183951999992</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -12650,6 +12731,9 @@
       </c>
       <c r="DT12" s="3" t="n">
         <v>220.873</v>
+      </c>
+      <c r="DU12" s="3" t="n">
+        <v>219.816</v>
       </c>
     </row>
     <row r="13">
@@ -12675,16 +12759,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.916</v>
+        <v>21.561</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>253953.95118</v>
+        <v>249840.351405</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>53953.95118</v>
+        <v>49840.35140499999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2697697559</v>
+        <v>0.249201757025</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -13030,6 +13114,9 @@
       </c>
       <c r="DT13" s="3" t="n">
         <v>21.916</v>
+      </c>
+      <c r="DU13" s="3" t="n">
+        <v>21.561</v>
       </c>
     </row>
     <row r="14">
@@ -13055,16 +13142,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.6251</v>
+        <v>38.3609</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>139344.1425106</v>
+        <v>138391.0130054</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>39344.14251060001</v>
+        <v>38391.01300540002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3934414251060001</v>
+        <v>0.3839101300540002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -13404,6 +13491,9 @@
       </c>
       <c r="DT14" s="3" t="n">
         <v>38.6251</v>
+      </c>
+      <c r="DU14" s="3" t="n">
+        <v>38.3609</v>
       </c>
     </row>
     <row r="15">
@@ -13429,16 +13519,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.54</v>
+        <v>11.29</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>112445.14838</v>
+        <v>110009.16163</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>12445.14838</v>
+        <v>10009.16162999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1244514838</v>
+        <v>0.1000916162999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -13784,6 +13874,9 @@
       </c>
       <c r="DT15" s="3" t="n">
         <v>11.54</v>
+      </c>
+      <c r="DU15" s="3" t="n">
+        <v>11.29</v>
       </c>
     </row>
     <row r="16">
@@ -13809,16 +13902,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>26.1743</v>
+        <v>25.939</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>149793.6343504</v>
+        <v>148447.029392</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>49793.63435039998</v>
+        <v>48447.029392</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4979363435039998</v>
+        <v>0.48447029392</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -14158,6 +14251,9 @@
       </c>
       <c r="DT16" s="3" t="n">
         <v>26.1743</v>
+      </c>
+      <c r="DU16" s="3" t="n">
+        <v>25.939</v>
       </c>
     </row>
     <row r="17">
@@ -14183,16 +14279,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7436</v>
+        <v>16.7599</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55355.2959852</v>
+        <v>55409.18471429999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5355.295985199999</v>
+        <v>5409.18471429999</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.107105919704</v>
+        <v>0.1081836942859998</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -14532,6 +14628,9 @@
       </c>
       <c r="DT17" s="3" t="n">
         <v>16.7436</v>
+      </c>
+      <c r="DU17" s="3" t="n">
+        <v>16.7599</v>
       </c>
     </row>
     <row r="18">
@@ -14557,16 +14656,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.83</v>
+        <v>44.81</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>86455.36188</v>
+        <v>84531.19716</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>6455.361879999997</v>
+        <v>4531.197159999996</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.08069202349999996</v>
+        <v>0.05663996449999995</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -14912,6 +15011,9 @@
       </c>
       <c r="DT18" s="3" t="n">
         <v>45.83</v>
+      </c>
+      <c r="DU18" s="3" t="n">
+        <v>44.81</v>
       </c>
     </row>
     <row r="19">
@@ -14937,16 +15039,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.7599</v>
+        <v>13.4251</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>199061.2534834</v>
+        <v>194217.7802266</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>49061.25348339998</v>
+        <v>44217.78022660001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3270750232226665</v>
+        <v>0.2947852015106667</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -15286,6 +15388,9 @@
       </c>
       <c r="DT19" s="3" t="n">
         <v>13.7599</v>
+      </c>
+      <c r="DU19" s="3" t="n">
+        <v>13.4251</v>
       </c>
     </row>
     <row r="20">
@@ -15311,16 +15416,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.789999999999999</v>
+        <v>9.83</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>257044.31137</v>
+        <v>258094.54349</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>7044.311369999981</v>
+        <v>8094.543490000011</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.02817724547999993</v>
+        <v>0.03237817396000004</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -15666,6 +15771,9 @@
       </c>
       <c r="DT20" s="3" t="n">
         <v>9.789999999999999</v>
+      </c>
+      <c r="DU20" s="3" t="n">
+        <v>9.83</v>
       </c>
     </row>
     <row r="21">
@@ -15691,16 +15799,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>112.5001</v>
+        <v>110.4929</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>170916.7894259</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>916.7894259000022</v>
-      </c>
-      <c r="I21" s="12" t="n">
-        <v>0.005392878975882366</v>
+        <v>167867.3327611</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>-2132.667238900001</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>-0.01254510140529413</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -16046,6 +16154,9 @@
       </c>
       <c r="DT21" s="3" t="n">
         <v>112.5001</v>
+      </c>
+      <c r="DU21" s="3" t="n">
+        <v>110.4929</v>
       </c>
     </row>
     <row r="22">
@@ -16071,16 +16182,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.206</v>
+        <v>43.729</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67832.33876000001</v>
+        <v>67100.40134</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7832.338760000013</v>
+        <v>7100.401339999997</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1305389793333336</v>
+        <v>0.1183400223333333</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -16420,6 +16531,9 @@
       </c>
       <c r="DT22" s="3" t="n">
         <v>44.206</v>
+      </c>
+      <c r="DU22" s="3" t="n">
+        <v>43.729</v>
       </c>
     </row>
     <row r="23">
@@ -16445,16 +16559,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.9087</v>
+        <v>60.7351</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>168172.9405629</v>
+        <v>164984.8948917</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>18172.94056290001</v>
+        <v>14984.89489170001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1211529370860001</v>
+        <v>0.09989929927800006</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -16800,6 +16914,9 @@
       </c>
       <c r="DT23" s="3" t="n">
         <v>61.9087</v>
+      </c>
+      <c r="DU23" s="3" t="n">
+        <v>60.7351</v>
       </c>
     </row>
     <row r="24">
@@ -16825,16 +16942,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.8452</v>
+        <v>25.617</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>93905.58784719999</v>
+        <v>93076.449162</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-6094.412152800011</v>
+        <v>-6923.550837999996</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.06094412152800011</v>
+        <v>-0.06923550837999995</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -17174,6 +17291,9 @@
       </c>
       <c r="DT24" s="3" t="n">
         <v>25.8452</v>
+      </c>
+      <c r="DU24" s="3" t="n">
+        <v>25.617</v>
       </c>
     </row>
     <row r="25">
@@ -17199,16 +17319,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.7091</v>
+        <v>12.558</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>208704.6970334</v>
+        <v>206223.382092</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>8704.697033399978</v>
+        <v>6223.382091999985</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.04352348516699989</v>
+        <v>0.03111691045999992</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -17551,6 +17671,9 @@
       </c>
       <c r="DT25" s="3" t="n">
         <v>12.7091</v>
+      </c>
+      <c r="DU25" s="3" t="n">
+        <v>12.558</v>
       </c>
     </row>
     <row r="26">
@@ -17576,16 +17699,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.8119</v>
+        <v>10.864</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>129112.6284085</v>
+        <v>129734.79176</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>19112.62840849999</v>
+        <v>19734.79176000001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1737511673499999</v>
+        <v>0.1794071978181819</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -17928,6 +18051,9 @@
       </c>
       <c r="DT26" s="3" t="n">
         <v>10.8119</v>
+      </c>
+      <c r="DU26" s="3" t="n">
+        <v>10.864</v>
       </c>
     </row>
     <row r="27">
@@ -17953,16 +18079,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>69.9776</v>
+        <v>69.2042</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>112724.116736</v>
+        <v>111478.277612</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>2724.116735999982</v>
+        <v>1478.277611999991</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.02476469759999983</v>
+        <v>0.0134388873818181</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -18308,6 +18434,9 @@
       </c>
       <c r="DT27" s="3" t="n">
         <v>69.9776</v>
+      </c>
+      <c r="DU27" s="3" t="n">
+        <v>69.2042</v>
       </c>
     </row>
     <row r="28">
@@ -18333,16 +18462,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>116.4021</v>
+        <v>114.9478</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>384901.8187797</v>
+        <v>380092.9475046</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>4901.818779700028</v>
+        <v>92.94750460004434</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.01289952310447376</v>
+        <v>0.0002445986963159061</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -18688,6 +18817,9 @@
       </c>
       <c r="DT28" s="3" t="n">
         <v>116.4021</v>
+      </c>
+      <c r="DU28" s="3" t="n">
+        <v>114.9478</v>
       </c>
     </row>
     <row r="29">
@@ -18713,16 +18845,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.0683</v>
+        <v>11.7946</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>115900.3689149</v>
+        <v>113271.8354038</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>15900.3689149</v>
+        <v>13271.8354038</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.159003689149</v>
+        <v>0.132718354038</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -19062,6 +19194,9 @@
       </c>
       <c r="DT29" s="3" t="n">
         <v>12.0683</v>
+      </c>
+      <c r="DU29" s="3" t="n">
+        <v>11.7946</v>
       </c>
     </row>
     <row r="30">
@@ -19087,16 +19222,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.4214</v>
+        <v>17.2014</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>128846.2528254</v>
+        <v>127219.1634054</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>28846.25282539999</v>
+        <v>27219.16340539999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2884625282539999</v>
+        <v>0.2721916340539999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -19436,6 +19571,9 @@
       </c>
       <c r="DT30" s="3" t="n">
         <v>17.4214</v>
+      </c>
+      <c r="DU30" s="3" t="n">
+        <v>17.2014</v>
       </c>
     </row>
     <row r="31">
@@ -19461,16 +19599,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>402.799</v>
+        <v>395.3733</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>107176.75792</v>
+        <v>105200.927664</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>7176.757919999989</v>
+        <v>5200.927663999988</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.07176757919999989</v>
+        <v>0.05200927663999988</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -19813,6 +19951,9 @@
       </c>
       <c r="DT31" s="3" t="n">
         <v>402.799</v>
+      </c>
+      <c r="DU31" s="3" t="n">
+        <v>395.3733</v>
       </c>
     </row>
     <row r="32">
@@ -19838,16 +19979,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.75</v>
+        <v>10.61</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>227254.57</v>
+        <v>224294.9756</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>27254.56999999998</v>
+        <v>24294.97559999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1362728499999999</v>
+        <v>0.1214748779999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -20193,6 +20334,9 @@
       </c>
       <c r="DT32" s="3" t="n">
         <v>10.75</v>
+      </c>
+      <c r="DU32" s="3" t="n">
+        <v>10.61</v>
       </c>
     </row>
     <row r="33">
@@ -20218,16 +20362,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.83</v>
+        <v>19.44</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>71063.58119999999</v>
+        <v>69665.9616</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>11063.58119999999</v>
+        <v>9665.961599999995</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1843930199999998</v>
+        <v>0.1610993599999999</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -20567,6 +20711,9 @@
       </c>
       <c r="DT33" s="3" t="n">
         <v>19.83</v>
+      </c>
+      <c r="DU33" s="3" t="n">
+        <v>19.44</v>
       </c>
     </row>
     <row r="34">
@@ -20592,16 +20739,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>222.7767</v>
+        <v>224.3834</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>78312.91612770001</v>
+        <v>78877.7209854</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-1687.083872299991</v>
+        <v>-1122.279014600004</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.02108854840374988</v>
+        <v>-0.01402848768250005</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -20944,6 +21091,9 @@
       </c>
       <c r="DT34" s="3" t="n">
         <v>222.7767</v>
+      </c>
+      <c r="DU34" s="3" t="n">
+        <v>224.3834</v>
       </c>
     </row>
     <row r="35">
@@ -20969,16 +21119,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.45</v>
+        <v>16.18</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>117377.70835</v>
+        <v>115451.14414</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>17377.70834999999</v>
+        <v>15451.14413999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1737770834999999</v>
+        <v>0.1545114413999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -21321,6 +21471,9 @@
       </c>
       <c r="DT35" s="3" t="n">
         <v>16.45</v>
+      </c>
+      <c r="DU35" s="3" t="n">
+        <v>16.18</v>
       </c>
     </row>
     <row r="36">
@@ -21346,16 +21499,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>378.49</v>
+        <v>371.1075</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>176265.06394</v>
+        <v>172826.989395</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>26265.06394000002</v>
+        <v>22826.98939500001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1751004262666668</v>
+        <v>0.1521799293000001</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -21698,6 +21851,9 @@
       </c>
       <c r="DT36" s="3" t="n">
         <v>378.49</v>
+      </c>
+      <c r="DU36" s="3" t="n">
+        <v>371.1075</v>
       </c>
     </row>
     <row r="37">
@@ -21723,16 +21879,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.242</v>
+        <v>16.922</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>64879.73213800001</v>
+        <v>63675.607658</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>14879.73213800001</v>
+        <v>13675.607658</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2975946427600001</v>
+        <v>0.27351215316</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -22075,6 +22231,9 @@
       </c>
       <c r="DT37" s="3" t="n">
         <v>17.242</v>
+      </c>
+      <c r="DU37" s="3" t="n">
+        <v>16.922</v>
       </c>
     </row>
     <row r="38">
@@ -22100,16 +22259,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.6496</v>
+        <v>13.5331</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>81631.18710719999</v>
+        <v>80934.4609542</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1631.187107199992</v>
+        <v>934.4609541999962</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.0203898388399999</v>
+        <v>0.01168076192749995</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -22449,6 +22608,9 @@
       </c>
       <c r="DT38" s="3" t="n">
         <v>13.6496</v>
+      </c>
+      <c r="DU38" s="3" t="n">
+        <v>13.5331</v>
       </c>
     </row>
     <row r="39">
@@ -22474,16 +22636,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1026.0552</v>
+        <v>1025.8987</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51180.6594312</v>
+        <v>51172.8530547</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1180.659431200002</v>
+        <v>1172.853054699997</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02361318862400003</v>
+        <v>0.02345706109399994</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -22823,6 +22985,9 @@
       </c>
       <c r="DT39" s="3" t="n">
         <v>1026.0552</v>
+      </c>
+      <c r="DU39" s="3" t="n">
+        <v>1025.8987</v>
       </c>
     </row>
     <row r="40">
@@ -22848,16 +23013,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.615</v>
+        <v>20.6053</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>103920.771605</v>
+        <v>103871.8736431</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>3920.771604999987</v>
+        <v>3871.8736431</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.03920771604999987</v>
+        <v>0.038718736431</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -23200,6 +23365,9 @@
       </c>
       <c r="DT40" s="3" t="n">
         <v>20.615</v>
+      </c>
+      <c r="DU40" s="3" t="n">
+        <v>20.6053</v>
       </c>
     </row>
     <row r="41">
@@ -23212,13 +23380,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5052720.4099612</v>
+        <v>5002638.7241529</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>582720.4099611999</v>
+        <v>532638.7241529</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1303625078212975</v>
+        <v>0.1191585512646309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-11
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-10 08:03 IST</t>
+          <t>Generated: 2026-10-11 08:15 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-10</t>
+          <t>Last snapshot: 2026-10-11</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EY19"/>
+  <dimension ref="A1:EZ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -774,6 +774,7 @@
     <col width="21" customWidth="1" min="153" max="153"/>
     <col width="21" customWidth="1" min="154" max="154"/>
     <col width="21" customWidth="1" min="155" max="155"/>
+    <col width="21" customWidth="1" min="156" max="156"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1552,6 +1553,11 @@
           <t>2026-10-10</t>
         </is>
       </c>
+      <c r="EZ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2020,6 +2026,9 @@
       <c r="EY2" s="3" t="n">
         <v>570.4000244140625</v>
       </c>
+      <c r="EZ2" s="3" t="n">
+        <v>570.4000244140625</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2518,6 +2527,9 @@
       <c r="EY4" s="3" t="n">
         <v>1409.800048828125</v>
       </c>
+      <c r="EZ4" s="3" t="n">
+        <v>1409.800048828125</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2989,6 +3001,9 @@
       <c r="EY5" s="3" t="n">
         <v>472.0499877929688</v>
       </c>
+      <c r="EZ5" s="3" t="n">
+        <v>472.0499877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3460,6 +3475,9 @@
       <c r="EY6" s="3" t="n">
         <v>364.9500122070312</v>
       </c>
+      <c r="EZ6" s="3" t="n">
+        <v>364.9500122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3931,6 +3949,9 @@
       <c r="EY7" s="3" t="n">
         <v>293.1000061035156</v>
       </c>
+      <c r="EZ7" s="3" t="n">
+        <v>293.1000061035156</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4429,6 +4450,9 @@
       <c r="EY9" s="3" t="n">
         <v>14.52999973297119</v>
       </c>
+      <c r="EZ9" s="3" t="n">
+        <v>14.52999973297119</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4900,6 +4924,9 @@
       <c r="EY10" s="3" t="n">
         <v>443.5</v>
       </c>
+      <c r="EZ10" s="3" t="n">
+        <v>443.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5371,6 +5398,9 @@
       <c r="EY11" s="3" t="n">
         <v>14.8100004196167</v>
       </c>
+      <c r="EZ11" s="3" t="n">
+        <v>14.8100004196167</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5842,6 +5872,9 @@
       <c r="EY12" s="3" t="n">
         <v>2523.60009765625</v>
       </c>
+      <c r="EZ12" s="3" t="n">
+        <v>2523.60009765625</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6313,6 +6346,9 @@
       <c r="EY13" s="3" t="n">
         <v>37.59999847412109</v>
       </c>
+      <c r="EZ13" s="3" t="n">
+        <v>37.59999847412109</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6784,6 +6820,9 @@
       <c r="EY14" s="3" t="n">
         <v>589.75</v>
       </c>
+      <c r="EZ14" s="3" t="n">
+        <v>589.75</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7309,6 +7348,9 @@
       <c r="EY17" s="3" t="n">
         <v>447.2000122070312</v>
       </c>
+      <c r="EZ17" s="3" t="n">
+        <v>447.2000122070312</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7778,6 +7820,9 @@
         <v>335.5</v>
       </c>
       <c r="EY18" s="3" t="n">
+        <v>342.1499938964844</v>
+      </c>
+      <c r="EZ18" s="3" t="n">
         <v>342.1499938964844</v>
       </c>
     </row>
@@ -7808,7 +7853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DU41"/>
+  <dimension ref="A1:DV41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7936,6 +7981,7 @@
     <col width="13" customWidth="1" min="123" max="123"/>
     <col width="13" customWidth="1" min="124" max="124"/>
     <col width="13" customWidth="1" min="125" max="125"/>
+    <col width="13" customWidth="1" min="126" max="126"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8564,6 +8610,11 @@
           <t>2026-10-10</t>
         </is>
       </c>
+      <c r="DV1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8947,6 +8998,9 @@
       <c r="DU2" s="3" t="n">
         <v>58.3132</v>
       </c>
+      <c r="DV2" s="3" t="n">
+        <v>58.3132</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9324,6 +9378,9 @@
       <c r="DU3" s="3" t="n">
         <v>27.0969</v>
       </c>
+      <c r="DV3" s="3" t="n">
+        <v>27.0969</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9701,6 +9758,9 @@
       <c r="DU4" s="3" t="n">
         <v>12.84</v>
       </c>
+      <c r="DV4" s="3" t="n">
+        <v>12.84</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10078,6 +10138,9 @@
       <c r="DU5" s="3" t="n">
         <v>8.971500000000001</v>
       </c>
+      <c r="DV5" s="3" t="n">
+        <v>8.971500000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10461,6 +10524,9 @@
       <c r="DU6" s="3" t="n">
         <v>11.1444</v>
       </c>
+      <c r="DV6" s="3" t="n">
+        <v>11.1444</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10838,6 +10904,9 @@
       <c r="DU7" s="3" t="n">
         <v>33.8842</v>
       </c>
+      <c r="DV7" s="3" t="n">
+        <v>33.8842</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11221,6 +11290,9 @@
       <c r="DU8" s="3" t="n">
         <v>35.8579</v>
       </c>
+      <c r="DV8" s="3" t="n">
+        <v>35.8579</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11598,6 +11670,9 @@
       <c r="DU9" s="3" t="n">
         <v>43.1225</v>
       </c>
+      <c r="DV9" s="3" t="n">
+        <v>43.1225</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11975,6 +12050,9 @@
       <c r="DU10" s="3" t="n">
         <v>49.0718</v>
       </c>
+      <c r="DV10" s="3" t="n">
+        <v>49.0718</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12352,6 +12430,9 @@
       <c r="DU11" s="3" t="n">
         <v>110.1877</v>
       </c>
+      <c r="DV11" s="3" t="n">
+        <v>110.1877</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12735,6 +12816,9 @@
       <c r="DU12" s="3" t="n">
         <v>219.816</v>
       </c>
+      <c r="DV12" s="3" t="n">
+        <v>219.816</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13118,6 +13202,9 @@
       <c r="DU13" s="3" t="n">
         <v>21.561</v>
       </c>
+      <c r="DV13" s="3" t="n">
+        <v>21.561</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13495,6 +13582,9 @@
       <c r="DU14" s="3" t="n">
         <v>38.3609</v>
       </c>
+      <c r="DV14" s="3" t="n">
+        <v>38.3609</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13878,6 +13968,9 @@
       <c r="DU15" s="3" t="n">
         <v>11.29</v>
       </c>
+      <c r="DV15" s="3" t="n">
+        <v>11.29</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -14255,6 +14348,9 @@
       <c r="DU16" s="3" t="n">
         <v>25.939</v>
       </c>
+      <c r="DV16" s="3" t="n">
+        <v>25.939</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14632,6 +14728,9 @@
       <c r="DU17" s="3" t="n">
         <v>16.7599</v>
       </c>
+      <c r="DV17" s="3" t="n">
+        <v>16.7599</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15015,6 +15114,9 @@
       <c r="DU18" s="3" t="n">
         <v>44.81</v>
       </c>
+      <c r="DV18" s="3" t="n">
+        <v>44.81</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -15392,6 +15494,9 @@
       <c r="DU19" s="3" t="n">
         <v>13.4251</v>
       </c>
+      <c r="DV19" s="3" t="n">
+        <v>13.4251</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15775,6 +15880,9 @@
       <c r="DU20" s="3" t="n">
         <v>9.83</v>
       </c>
+      <c r="DV20" s="3" t="n">
+        <v>9.83</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -16158,6 +16266,9 @@
       <c r="DU21" s="3" t="n">
         <v>110.4929</v>
       </c>
+      <c r="DV21" s="3" t="n">
+        <v>110.4929</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -16535,6 +16646,9 @@
       <c r="DU22" s="3" t="n">
         <v>43.729</v>
       </c>
+      <c r="DV22" s="3" t="n">
+        <v>43.729</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -16918,6 +17032,9 @@
       <c r="DU23" s="3" t="n">
         <v>60.7351</v>
       </c>
+      <c r="DV23" s="3" t="n">
+        <v>60.7351</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -17295,6 +17412,9 @@
       <c r="DU24" s="3" t="n">
         <v>25.617</v>
       </c>
+      <c r="DV24" s="3" t="n">
+        <v>25.617</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -17675,6 +17795,9 @@
       <c r="DU25" s="3" t="n">
         <v>12.558</v>
       </c>
+      <c r="DV25" s="3" t="n">
+        <v>12.558</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -18055,6 +18178,9 @@
       <c r="DU26" s="3" t="n">
         <v>10.864</v>
       </c>
+      <c r="DV26" s="3" t="n">
+        <v>10.864</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -18438,6 +18564,9 @@
       <c r="DU27" s="3" t="n">
         <v>69.2042</v>
       </c>
+      <c r="DV27" s="3" t="n">
+        <v>69.2042</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -18821,6 +18950,9 @@
       <c r="DU28" s="3" t="n">
         <v>114.9478</v>
       </c>
+      <c r="DV28" s="3" t="n">
+        <v>114.9478</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -19198,6 +19330,9 @@
       <c r="DU29" s="3" t="n">
         <v>11.7946</v>
       </c>
+      <c r="DV29" s="3" t="n">
+        <v>11.7946</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -19575,6 +19710,9 @@
       <c r="DU30" s="3" t="n">
         <v>17.2014</v>
       </c>
+      <c r="DV30" s="3" t="n">
+        <v>17.2014</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -19955,6 +20093,9 @@
       <c r="DU31" s="3" t="n">
         <v>395.3733</v>
       </c>
+      <c r="DV31" s="3" t="n">
+        <v>395.3733</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -20338,6 +20479,9 @@
       <c r="DU32" s="3" t="n">
         <v>10.61</v>
       </c>
+      <c r="DV32" s="3" t="n">
+        <v>10.61</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -20715,6 +20859,9 @@
       <c r="DU33" s="3" t="n">
         <v>19.44</v>
       </c>
+      <c r="DV33" s="3" t="n">
+        <v>19.44</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -21095,6 +21242,9 @@
       <c r="DU34" s="3" t="n">
         <v>224.3834</v>
       </c>
+      <c r="DV34" s="3" t="n">
+        <v>224.3834</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -21475,6 +21625,9 @@
       <c r="DU35" s="3" t="n">
         <v>16.18</v>
       </c>
+      <c r="DV35" s="3" t="n">
+        <v>16.18</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -21855,6 +22008,9 @@
       <c r="DU36" s="3" t="n">
         <v>371.1075</v>
       </c>
+      <c r="DV36" s="3" t="n">
+        <v>371.1075</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -22235,6 +22391,9 @@
       <c r="DU37" s="3" t="n">
         <v>16.922</v>
       </c>
+      <c r="DV37" s="3" t="n">
+        <v>16.922</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -22612,6 +22771,9 @@
       <c r="DU38" s="3" t="n">
         <v>13.5331</v>
       </c>
+      <c r="DV38" s="3" t="n">
+        <v>13.5331</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -22989,6 +23151,9 @@
       <c r="DU39" s="3" t="n">
         <v>1025.8987</v>
       </c>
+      <c r="DV39" s="3" t="n">
+        <v>1025.8987</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -23367,6 +23532,9 @@
         <v>20.615</v>
       </c>
       <c r="DU40" s="3" t="n">
+        <v>20.6053</v>
+      </c>
+      <c r="DV40" s="3" t="n">
         <v>20.6053</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-12
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-11 08:15 IST</t>
+          <t>Generated: 2026-10-12 08:32 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>523761.0038642883</v>
+        <v>529760.5015068054</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-67021.01613571169</v>
+        <v>-61021.5184931946</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1134445766235602</v>
+        <v>-0.1032893968120333</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5526399.728017189</v>
+        <v>5532399.225659706</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>465617.7080171891</v>
+        <v>471617.2056597061</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09200509055262354</v>
+        <v>0.09319057880696988</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-11</t>
+          <t>Last snapshot: 2026-10-12</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EZ19"/>
+  <dimension ref="A1:FA19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -775,6 +775,7 @@
     <col width="21" customWidth="1" min="154" max="154"/>
     <col width="21" customWidth="1" min="155" max="155"/>
     <col width="21" customWidth="1" min="156" max="156"/>
+    <col width="21" customWidth="1" min="157" max="157"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1558,6 +1559,11 @@
           <t>2026-10-11</t>
         </is>
       </c>
+      <c r="FA1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1577,13 +1583,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>570.4000244140625</v>
+        <v>571.2000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45632.001953125</v>
+        <v>45696.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1814.491953124998</v>
+        <v>1878.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2028,6 +2034,9 @@
       </c>
       <c r="EZ2" s="3" t="n">
         <v>570.4000244140625</v>
+      </c>
+      <c r="FA2" s="3" t="n">
+        <v>571.2000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -2075,13 +2084,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1409.800048828125</v>
+        <v>1432</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28196.0009765625</v>
+        <v>28640</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3908.579023437502</v>
+        <v>-3464.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2529,6 +2538,9 @@
       </c>
       <c r="EZ4" s="3" t="n">
         <v>1409.800048828125</v>
+      </c>
+      <c r="FA4" s="3" t="n">
+        <v>1432</v>
       </c>
     </row>
     <row r="5">
@@ -2549,13 +2561,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>472.0499877929688</v>
+        <v>475.2999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9440.999755859375</v>
+        <v>9505.999755859375</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4772.100244140625</v>
+        <v>-4707.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3003,6 +3015,9 @@
       </c>
       <c r="EZ5" s="3" t="n">
         <v>472.0499877929688</v>
+      </c>
+      <c r="FA5" s="3" t="n">
+        <v>475.2999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -3023,13 +3038,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>364.9500122070312</v>
+        <v>366.6499938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14598.00048828125</v>
+        <v>14665.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2904.239511718752</v>
+        <v>-2836.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3477,6 +3492,9 @@
       </c>
       <c r="EZ6" s="3" t="n">
         <v>364.9500122070312</v>
+      </c>
+      <c r="FA6" s="3" t="n">
+        <v>366.6499938964844</v>
       </c>
     </row>
     <row r="7">
@@ -3497,13 +3515,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>293.1000061035156</v>
+        <v>293.5</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>29310.00061035156</v>
+        <v>29350</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>2876.180610351563</v>
+        <v>2916.18</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3951,6 +3969,9 @@
       </c>
       <c r="EZ7" s="3" t="n">
         <v>293.1000061035156</v>
+      </c>
+      <c r="FA7" s="3" t="n">
+        <v>293.5</v>
       </c>
     </row>
     <row r="8">
@@ -3998,13 +4019,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.52999973297119</v>
+        <v>14.6899995803833</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>21794.99959945679</v>
+        <v>22034.99937057495</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-9255.170400543211</v>
+        <v>-9015.170629425047</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4452,6 +4473,9 @@
       </c>
       <c r="EZ9" s="3" t="n">
         <v>14.52999973297119</v>
+      </c>
+      <c r="FA9" s="3" t="n">
+        <v>14.6899995803833</v>
       </c>
     </row>
     <row r="10">
@@ -4472,13 +4496,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>443.5</v>
+        <v>445.2000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44350</v>
+        <v>44520.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-7148.480000000003</v>
+        <v>-6978.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4926,6 +4950,9 @@
       </c>
       <c r="EZ10" s="3" t="n">
         <v>443.5</v>
+      </c>
+      <c r="FA10" s="3" t="n">
+        <v>445.2000122070312</v>
       </c>
     </row>
     <row r="11">
@@ -4946,13 +4973,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>14.8100004196167</v>
+        <v>15.18000030517578</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14810.0004196167</v>
+        <v>15180.00030517578</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4968.7904196167</v>
+        <v>5338.790305175782</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5400,6 +5427,9 @@
       </c>
       <c r="EZ11" s="3" t="n">
         <v>14.8100004196167</v>
+      </c>
+      <c r="FA11" s="3" t="n">
+        <v>15.18000030517578</v>
       </c>
     </row>
     <row r="12">
@@ -5420,13 +5450,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2523.60009765625</v>
+        <v>2551.199951171875</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25236.0009765625</v>
+        <v>25511.99951171875</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2487.2490234375</v>
+        <v>-2211.25048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5874,6 +5904,9 @@
       </c>
       <c r="EZ12" s="3" t="n">
         <v>2523.60009765625</v>
+      </c>
+      <c r="FA12" s="3" t="n">
+        <v>2551.199951171875</v>
       </c>
     </row>
     <row r="13">
@@ -5894,13 +5927,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>37.59999847412109</v>
+        <v>39.75</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22559.99908447266</v>
+        <v>23850</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-12471.76091552735</v>
+        <v>-11181.76</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6348,6 +6381,9 @@
       </c>
       <c r="EZ13" s="3" t="n">
         <v>37.59999847412109</v>
+      </c>
+      <c r="FA13" s="3" t="n">
+        <v>39.75</v>
       </c>
     </row>
     <row r="14">
@@ -6368,13 +6404,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>589.75</v>
+        <v>631</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>29487.5</v>
+        <v>31550</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12975.01</v>
+        <v>-10912.51</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6822,6 +6858,9 @@
       </c>
       <c r="EZ14" s="3" t="n">
         <v>589.75</v>
+      </c>
+      <c r="FA14" s="3" t="n">
+        <v>631</v>
       </c>
     </row>
     <row r="15">
@@ -6896,13 +6935,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>447.2000122070312</v>
+        <v>462</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>22360.00061035156</v>
+        <v>23100</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>605.4706103515637</v>
+        <v>1345.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7350,6 +7389,9 @@
       </c>
       <c r="EZ17" s="3" t="n">
         <v>447.2000122070312</v>
+      </c>
+      <c r="FA17" s="3" t="n">
+        <v>462</v>
       </c>
     </row>
     <row r="18">
@@ -7370,13 +7412,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>342.1499938964844</v>
+        <v>343.8500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34214.99938964844</v>
+        <v>34385.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12425.82061035156</v>
+        <v>-12255.81938964844</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7824,6 +7866,9 @@
       </c>
       <c r="EZ18" s="3" t="n">
         <v>342.1499938964844</v>
+      </c>
+      <c r="FA18" s="3" t="n">
+        <v>343.8500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -7836,10 +7881,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>523761.0038642883</v>
+        <v>529760.5015068054</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-67021.01613571167</v>
+        <v>-61021.51849319459</v>
       </c>
     </row>
   </sheetData>
@@ -7853,7 +7898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DV41"/>
+  <dimension ref="A1:DW41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7982,6 +8027,7 @@
     <col width="13" customWidth="1" min="124" max="124"/>
     <col width="13" customWidth="1" min="125" max="125"/>
     <col width="13" customWidth="1" min="126" max="126"/>
+    <col width="13" customWidth="1" min="127" max="127"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8615,6 +8661,11 @@
           <t>2026-10-11</t>
         </is>
       </c>
+      <c r="DW1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9001,6 +9052,9 @@
       <c r="DV2" s="3" t="n">
         <v>58.3132</v>
       </c>
+      <c r="DW2" s="3" t="n">
+        <v>58.3132</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9381,6 +9435,9 @@
       <c r="DV3" s="3" t="n">
         <v>27.0969</v>
       </c>
+      <c r="DW3" s="3" t="n">
+        <v>27.0969</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9761,6 +9818,9 @@
       <c r="DV4" s="3" t="n">
         <v>12.84</v>
       </c>
+      <c r="DW4" s="3" t="n">
+        <v>12.84</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10141,6 +10201,9 @@
       <c r="DV5" s="3" t="n">
         <v>8.971500000000001</v>
       </c>
+      <c r="DW5" s="3" t="n">
+        <v>8.971500000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10527,6 +10590,9 @@
       <c r="DV6" s="3" t="n">
         <v>11.1444</v>
       </c>
+      <c r="DW6" s="3" t="n">
+        <v>11.1444</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10907,6 +10973,9 @@
       <c r="DV7" s="3" t="n">
         <v>33.8842</v>
       </c>
+      <c r="DW7" s="3" t="n">
+        <v>33.8842</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11293,6 +11362,9 @@
       <c r="DV8" s="3" t="n">
         <v>35.8579</v>
       </c>
+      <c r="DW8" s="3" t="n">
+        <v>35.8579</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11673,6 +11745,9 @@
       <c r="DV9" s="3" t="n">
         <v>43.1225</v>
       </c>
+      <c r="DW9" s="3" t="n">
+        <v>43.1225</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12053,6 +12128,9 @@
       <c r="DV10" s="3" t="n">
         <v>49.0718</v>
       </c>
+      <c r="DW10" s="3" t="n">
+        <v>49.0718</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12433,6 +12511,9 @@
       <c r="DV11" s="3" t="n">
         <v>110.1877</v>
       </c>
+      <c r="DW11" s="3" t="n">
+        <v>110.1877</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12819,6 +12900,9 @@
       <c r="DV12" s="3" t="n">
         <v>219.816</v>
       </c>
+      <c r="DW12" s="3" t="n">
+        <v>219.816</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13205,6 +13289,9 @@
       <c r="DV13" s="3" t="n">
         <v>21.561</v>
       </c>
+      <c r="DW13" s="3" t="n">
+        <v>21.561</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13585,6 +13672,9 @@
       <c r="DV14" s="3" t="n">
         <v>38.3609</v>
       </c>
+      <c r="DW14" s="3" t="n">
+        <v>38.3609</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13971,6 +14061,9 @@
       <c r="DV15" s="3" t="n">
         <v>11.29</v>
       </c>
+      <c r="DW15" s="3" t="n">
+        <v>11.29</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -14351,6 +14444,9 @@
       <c r="DV16" s="3" t="n">
         <v>25.939</v>
       </c>
+      <c r="DW16" s="3" t="n">
+        <v>25.939</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14731,6 +14827,9 @@
       <c r="DV17" s="3" t="n">
         <v>16.7599</v>
       </c>
+      <c r="DW17" s="3" t="n">
+        <v>16.7599</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15117,6 +15216,9 @@
       <c r="DV18" s="3" t="n">
         <v>44.81</v>
       </c>
+      <c r="DW18" s="3" t="n">
+        <v>44.81</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -15497,6 +15599,9 @@
       <c r="DV19" s="3" t="n">
         <v>13.4251</v>
       </c>
+      <c r="DW19" s="3" t="n">
+        <v>13.4251</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15883,6 +15988,9 @@
       <c r="DV20" s="3" t="n">
         <v>9.83</v>
       </c>
+      <c r="DW20" s="3" t="n">
+        <v>9.83</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -16269,6 +16377,9 @@
       <c r="DV21" s="3" t="n">
         <v>110.4929</v>
       </c>
+      <c r="DW21" s="3" t="n">
+        <v>110.4929</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -16649,6 +16760,9 @@
       <c r="DV22" s="3" t="n">
         <v>43.729</v>
       </c>
+      <c r="DW22" s="3" t="n">
+        <v>43.729</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -17035,6 +17149,9 @@
       <c r="DV23" s="3" t="n">
         <v>60.7351</v>
       </c>
+      <c r="DW23" s="3" t="n">
+        <v>60.7351</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -17415,6 +17532,9 @@
       <c r="DV24" s="3" t="n">
         <v>25.617</v>
       </c>
+      <c r="DW24" s="3" t="n">
+        <v>25.617</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -17798,6 +17918,9 @@
       <c r="DV25" s="3" t="n">
         <v>12.558</v>
       </c>
+      <c r="DW25" s="3" t="n">
+        <v>12.558</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -18181,6 +18304,9 @@
       <c r="DV26" s="3" t="n">
         <v>10.864</v>
       </c>
+      <c r="DW26" s="3" t="n">
+        <v>10.864</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -18567,6 +18693,9 @@
       <c r="DV27" s="3" t="n">
         <v>69.2042</v>
       </c>
+      <c r="DW27" s="3" t="n">
+        <v>69.2042</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -18953,6 +19082,9 @@
       <c r="DV28" s="3" t="n">
         <v>114.9478</v>
       </c>
+      <c r="DW28" s="3" t="n">
+        <v>114.9478</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -19333,6 +19465,9 @@
       <c r="DV29" s="3" t="n">
         <v>11.7946</v>
       </c>
+      <c r="DW29" s="3" t="n">
+        <v>11.7946</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -19713,6 +19848,9 @@
       <c r="DV30" s="3" t="n">
         <v>17.2014</v>
       </c>
+      <c r="DW30" s="3" t="n">
+        <v>17.2014</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -20096,6 +20234,9 @@
       <c r="DV31" s="3" t="n">
         <v>395.3733</v>
       </c>
+      <c r="DW31" s="3" t="n">
+        <v>395.3733</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -20482,6 +20623,9 @@
       <c r="DV32" s="3" t="n">
         <v>10.61</v>
       </c>
+      <c r="DW32" s="3" t="n">
+        <v>10.61</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -20862,6 +21006,9 @@
       <c r="DV33" s="3" t="n">
         <v>19.44</v>
       </c>
+      <c r="DW33" s="3" t="n">
+        <v>19.44</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -21245,6 +21392,9 @@
       <c r="DV34" s="3" t="n">
         <v>224.3834</v>
       </c>
+      <c r="DW34" s="3" t="n">
+        <v>224.3834</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -21628,6 +21778,9 @@
       <c r="DV35" s="3" t="n">
         <v>16.18</v>
       </c>
+      <c r="DW35" s="3" t="n">
+        <v>16.18</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -22011,6 +22164,9 @@
       <c r="DV36" s="3" t="n">
         <v>371.1075</v>
       </c>
+      <c r="DW36" s="3" t="n">
+        <v>371.1075</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -22394,6 +22550,9 @@
       <c r="DV37" s="3" t="n">
         <v>16.922</v>
       </c>
+      <c r="DW37" s="3" t="n">
+        <v>16.922</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -22774,6 +22933,9 @@
       <c r="DV38" s="3" t="n">
         <v>13.5331</v>
       </c>
+      <c r="DW38" s="3" t="n">
+        <v>13.5331</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -23154,6 +23316,9 @@
       <c r="DV39" s="3" t="n">
         <v>1025.8987</v>
       </c>
+      <c r="DW39" s="3" t="n">
+        <v>1025.8987</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -23535,6 +23700,9 @@
         <v>20.6053</v>
       </c>
       <c r="DV40" s="3" t="n">
+        <v>20.6053</v>
+      </c>
+      <c r="DW40" s="3" t="n">
         <v>20.6053</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-13
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-12 08:32 IST</t>
+          <t>Generated: 2026-10-13 08:54 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5002638.7241529</v>
+        <v>5000697.2565921</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>532638.7241529003</v>
+        <v>530697.2565920996</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1191585512646309</v>
+        <v>0.1187242184769798</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>529760.5015068054</v>
+        <v>527330.4982452393</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-61021.5184931946</v>
+        <v>-63451.52175476076</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1032893968120333</v>
+        <v>-0.1074025945386096</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5532399.225659706</v>
+        <v>5528027.754837339</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>471617.2056597061</v>
+        <v>467245.7348373393</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09319057880696988</v>
+        <v>0.09232678526575608</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-12</t>
+          <t>Last snapshot: 2026-10-13</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FA19"/>
+  <dimension ref="A1:FB19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -776,6 +776,7 @@
     <col width="21" customWidth="1" min="155" max="155"/>
     <col width="21" customWidth="1" min="156" max="156"/>
     <col width="21" customWidth="1" min="157" max="157"/>
+    <col width="21" customWidth="1" min="158" max="158"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1564,6 +1565,11 @@
           <t>2026-10-12</t>
         </is>
       </c>
+      <c r="FB1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1583,13 +1589,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>571.2000122070312</v>
+        <v>571.2999877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45696.0009765625</v>
+        <v>45703.9990234375</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1878.490976562498</v>
+        <v>1886.489023437498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2037,6 +2043,9 @@
       </c>
       <c r="FA2" s="3" t="n">
         <v>571.2000122070312</v>
+      </c>
+      <c r="FB2" s="3" t="n">
+        <v>571.2999877929688</v>
       </c>
     </row>
     <row r="3">
@@ -2084,13 +2093,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1432</v>
+        <v>1431</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28640</v>
+        <v>28620</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3464.580000000002</v>
+        <v>-3484.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2541,6 +2550,9 @@
       </c>
       <c r="FA4" s="3" t="n">
         <v>1432</v>
+      </c>
+      <c r="FB4" s="3" t="n">
+        <v>1431</v>
       </c>
     </row>
     <row r="5">
@@ -2561,13 +2573,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>475.2999877929688</v>
+        <v>469.7999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9505.999755859375</v>
+        <v>9395.999755859375</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4707.100244140625</v>
+        <v>-4817.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3018,6 +3030,9 @@
       </c>
       <c r="FA5" s="3" t="n">
         <v>475.2999877929688</v>
+      </c>
+      <c r="FB5" s="3" t="n">
+        <v>469.7999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -3038,13 +3053,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>366.6499938964844</v>
+        <v>362.7000122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14665.99975585938</v>
+        <v>14508.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2836.240244140627</v>
+        <v>-2994.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3495,6 +3510,9 @@
       </c>
       <c r="FA6" s="3" t="n">
         <v>366.6499938964844</v>
+      </c>
+      <c r="FB6" s="3" t="n">
+        <v>362.7000122070312</v>
       </c>
     </row>
     <row r="7">
@@ -3515,13 +3533,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>293.5</v>
+        <v>288.1499938964844</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>29350</v>
+        <v>28814.99938964844</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>2916.18</v>
+        <v>2381.179389648438</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3972,6 +3990,9 @@
       </c>
       <c r="FA7" s="3" t="n">
         <v>293.5</v>
+      </c>
+      <c r="FB7" s="3" t="n">
+        <v>288.1499938964844</v>
       </c>
     </row>
     <row r="8">
@@ -4019,13 +4040,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.6899995803833</v>
+        <v>14.97999954223633</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22034.99937057495</v>
+        <v>22469.99931335449</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-9015.170629425047</v>
+        <v>-8580.170686645506</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4476,6 +4497,9 @@
       </c>
       <c r="FA9" s="3" t="n">
         <v>14.6899995803833</v>
+      </c>
+      <c r="FB9" s="3" t="n">
+        <v>14.97999954223633</v>
       </c>
     </row>
     <row r="10">
@@ -4496,13 +4520,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>445.2000122070312</v>
+        <v>443.6499938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44520.00122070312</v>
+        <v>44364.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6978.478779296878</v>
+        <v>-7133.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4953,6 +4977,9 @@
       </c>
       <c r="FA10" s="3" t="n">
         <v>445.2000122070312</v>
+      </c>
+      <c r="FB10" s="3" t="n">
+        <v>443.6499938964844</v>
       </c>
     </row>
     <row r="11">
@@ -4973,13 +5000,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>15.18000030517578</v>
+        <v>14.09000015258789</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>15180.00030517578</v>
+        <v>14090.00015258789</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>5338.790305175782</v>
+        <v>4248.790152587891</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5430,6 +5457,9 @@
       </c>
       <c r="FA11" s="3" t="n">
         <v>15.18000030517578</v>
+      </c>
+      <c r="FB11" s="3" t="n">
+        <v>14.09000015258789</v>
       </c>
     </row>
     <row r="12">
@@ -5450,13 +5480,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2551.199951171875</v>
+        <v>2526</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25511.99951171875</v>
+        <v>25260</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2211.25048828125</v>
+        <v>-2463.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5907,6 +5937,9 @@
       </c>
       <c r="FA12" s="3" t="n">
         <v>2551.199951171875</v>
+      </c>
+      <c r="FB12" s="3" t="n">
+        <v>2526</v>
       </c>
     </row>
     <row r="13">
@@ -5927,13 +5960,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>39.75</v>
+        <v>39.66999816894531</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23850</v>
+        <v>23801.99890136719</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11181.76</v>
+        <v>-11229.76109863281</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6384,6 +6417,9 @@
       </c>
       <c r="FA13" s="3" t="n">
         <v>39.75</v>
+      </c>
+      <c r="FB13" s="3" t="n">
+        <v>39.66999816894531</v>
       </c>
     </row>
     <row r="14">
@@ -6404,13 +6440,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>631</v>
+        <v>627.5</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31550</v>
+        <v>31375</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-10912.51</v>
+        <v>-11087.51</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6861,6 +6897,9 @@
       </c>
       <c r="FA14" s="3" t="n">
         <v>631</v>
+      </c>
+      <c r="FB14" s="3" t="n">
+        <v>627.5</v>
       </c>
     </row>
     <row r="15">
@@ -6935,13 +6974,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>462</v>
+        <v>457.2000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23100</v>
+        <v>22860.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1345.470000000001</v>
+        <v>1105.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7392,6 +7431,9 @@
       </c>
       <c r="FA17" s="3" t="n">
         <v>462</v>
+      </c>
+      <c r="FB17" s="3" t="n">
+        <v>457.2000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -7412,13 +7454,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>343.8500061035156</v>
+        <v>342.9500122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34385.00061035156</v>
+        <v>34295.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12255.81938964844</v>
+        <v>-12345.81877929687</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7869,6 +7911,9 @@
       </c>
       <c r="FA18" s="3" t="n">
         <v>343.8500061035156</v>
+      </c>
+      <c r="FB18" s="3" t="n">
+        <v>342.9500122070312</v>
       </c>
     </row>
     <row r="19">
@@ -7881,10 +7926,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>529760.5015068054</v>
+        <v>527330.4982452393</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-61021.51849319459</v>
+        <v>-63451.52175476075</v>
       </c>
     </row>
   </sheetData>
@@ -7898,7 +7943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DW41"/>
+  <dimension ref="A1:DX41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7909,7 +7954,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -8028,6 +8073,7 @@
     <col width="13" customWidth="1" min="125" max="125"/>
     <col width="13" customWidth="1" min="126" max="126"/>
     <col width="13" customWidth="1" min="127" max="127"/>
+    <col width="13" customWidth="1" min="128" max="128"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8666,6 +8712,11 @@
           <t>2026-10-12</t>
         </is>
       </c>
+      <c r="DX1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8690,16 +8741,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>58.3132</v>
+        <v>57.6758</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>65455.5173624</v>
+        <v>64740.0473356</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>15455.5173624</v>
+        <v>14740.0473356</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.309110347248</v>
+        <v>0.294800946712</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9054,6 +9105,9 @@
       </c>
       <c r="DW2" s="3" t="n">
         <v>58.3132</v>
+      </c>
+      <c r="DX2" s="3" t="n">
+        <v>57.6758</v>
       </c>
     </row>
     <row r="3">
@@ -9079,16 +9133,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>27.0969</v>
+        <v>26.9597</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>66528.66113970001</v>
+        <v>66191.80591610001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>6528.661139700009</v>
+        <v>6191.805916100013</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.1088110189950001</v>
+        <v>0.1031967652683335</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9437,6 +9491,9 @@
       </c>
       <c r="DW3" s="3" t="n">
         <v>27.0969</v>
+      </c>
+      <c r="DX3" s="3" t="n">
+        <v>26.9597</v>
       </c>
     </row>
     <row r="4">
@@ -9462,16 +9519,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.84</v>
+        <v>12.71</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>246606.23412</v>
+        <v>244109.44203</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>66606.23412000001</v>
+        <v>64109.44203000003</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.370034634</v>
+        <v>0.3561635668333335</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9820,6 +9877,9 @@
       </c>
       <c r="DW4" s="3" t="n">
         <v>12.84</v>
+      </c>
+      <c r="DX4" s="3" t="n">
+        <v>12.71</v>
       </c>
     </row>
     <row r="5">
@@ -9845,16 +9905,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.971500000000001</v>
+        <v>8.959199999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>164663.700492</v>
+        <v>164437.9452096</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-45336.299508</v>
+        <v>-45562.05479040003</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2158871405142857</v>
+        <v>-0.2169621656685715</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10203,6 +10263,9 @@
       </c>
       <c r="DW5" s="3" t="n">
         <v>8.971500000000001</v>
+      </c>
+      <c r="DX5" s="3" t="n">
+        <v>8.959199999999999</v>
       </c>
     </row>
     <row r="6">
@@ -10228,16 +10291,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.1444</v>
+        <v>11.1372</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>47129.4112788</v>
+        <v>47098.9626444</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-2870.588721200002</v>
+        <v>-2901.037355600005</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.05741177442400004</v>
+        <v>-0.0580207471120001</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -10592,6 +10655,9 @@
       </c>
       <c r="DW6" s="3" t="n">
         <v>11.1444</v>
+      </c>
+      <c r="DX6" s="3" t="n">
+        <v>11.1372</v>
       </c>
     </row>
     <row r="7">
@@ -10617,16 +10683,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.8842</v>
+        <v>33.7421</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74749.900568</v>
+        <v>74436.422284</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14749.900568</v>
+        <v>14436.422284</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2458316761333333</v>
+        <v>0.2406070380666667</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -10975,6 +11041,9 @@
       </c>
       <c r="DW7" s="3" t="n">
         <v>33.8842</v>
+      </c>
+      <c r="DX7" s="3" t="n">
+        <v>33.7421</v>
       </c>
     </row>
     <row r="8">
@@ -11000,16 +11069,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.8579</v>
+        <v>35.8242</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57537.3353347</v>
+        <v>57483.2605506</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7537.335334700001</v>
+        <v>7483.260550599996</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.150746706694</v>
+        <v>0.1496652110119999</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -11364,6 +11433,9 @@
       </c>
       <c r="DW8" s="3" t="n">
         <v>35.8579</v>
+      </c>
+      <c r="DX8" s="3" t="n">
+        <v>35.8242</v>
       </c>
     </row>
     <row r="9">
@@ -11389,16 +11461,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.1225</v>
+        <v>42.6817</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>138828.2746425</v>
+        <v>137409.1662081</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>38828.27464250001</v>
+        <v>37409.16620810001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3882827464250001</v>
+        <v>0.3740916620810001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -11747,6 +11819,9 @@
       </c>
       <c r="DW9" s="3" t="n">
         <v>43.1225</v>
+      </c>
+      <c r="DX9" s="3" t="n">
+        <v>42.6817</v>
       </c>
     </row>
     <row r="10">
@@ -11772,16 +11847,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49.0718</v>
+        <v>48.9149</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>139690.6811162</v>
+        <v>139244.0403191</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>39690.68111620002</v>
+        <v>39244.04031910002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3969068111620002</v>
+        <v>0.3924404031910002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -12130,6 +12205,9 @@
       </c>
       <c r="DW10" s="3" t="n">
         <v>49.0718</v>
+      </c>
+      <c r="DX10" s="3" t="n">
+        <v>48.9149</v>
       </c>
     </row>
     <row r="11">
@@ -12155,16 +12233,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>110.1877</v>
+        <v>108.209</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>33157.5724963</v>
+        <v>32562.144071</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>3157.572496300003</v>
+        <v>2562.144070999999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.1052524165433334</v>
+        <v>0.08540480236666663</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -12513,6 +12591,9 @@
       </c>
       <c r="DW11" s="3" t="n">
         <v>110.1877</v>
+      </c>
+      <c r="DX11" s="3" t="n">
+        <v>108.209</v>
       </c>
     </row>
     <row r="12">
@@ -12538,16 +12619,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>219.816</v>
+        <v>219.3</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102329.183952</v>
+        <v>102088.9746</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2329.183951999992</v>
+        <v>2088.974600000001</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02329183951999992</v>
+        <v>0.02088974600000001</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -12902,6 +12983,9 @@
       </c>
       <c r="DW12" s="3" t="n">
         <v>219.816</v>
+      </c>
+      <c r="DX12" s="3" t="n">
+        <v>219.3</v>
       </c>
     </row>
     <row r="13">
@@ -12927,16 +13011,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.561</v>
+        <v>21.532</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>249840.351405</v>
+        <v>249504.31086</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>49840.35140499999</v>
+        <v>49504.31086</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.249201757025</v>
+        <v>0.2475215543</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -13291,6 +13375,9 @@
       </c>
       <c r="DW13" s="3" t="n">
         <v>21.561</v>
+      </c>
+      <c r="DX13" s="3" t="n">
+        <v>21.532</v>
       </c>
     </row>
     <row r="14">
@@ -13316,16 +13403,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.3609</v>
+        <v>37.7693</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>138391.0130054</v>
+        <v>136256.7532958</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>38391.01300540002</v>
+        <v>36256.75329580001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3839101300540002</v>
+        <v>0.3625675329580001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -13674,6 +13761,9 @@
       </c>
       <c r="DW14" s="3" t="n">
         <v>38.3609</v>
+      </c>
+      <c r="DX14" s="3" t="n">
+        <v>37.7693</v>
       </c>
     </row>
     <row r="15">
@@ -13699,16 +13789,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.29</v>
+        <v>11.3</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>110009.16163</v>
+        <v>110106.6011</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>10009.16162999999</v>
+        <v>10106.60110000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1000916162999999</v>
+        <v>0.1010660110000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -14063,6 +14153,9 @@
       </c>
       <c r="DW15" s="3" t="n">
         <v>11.29</v>
+      </c>
+      <c r="DX15" s="3" t="n">
+        <v>11.3</v>
       </c>
     </row>
     <row r="16">
@@ -14088,16 +14181,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.939</v>
+        <v>25.5233</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>148447.029392</v>
+        <v>146068.0082224</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>48447.029392</v>
+        <v>46068.00822239998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.48447029392</v>
+        <v>0.4606800822239998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -14446,6 +14539,9 @@
       </c>
       <c r="DW16" s="3" t="n">
         <v>25.939</v>
+      </c>
+      <c r="DX16" s="3" t="n">
+        <v>25.5233</v>
       </c>
     </row>
     <row r="17">
@@ -14471,16 +14567,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7599</v>
+        <v>16.6548</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55409.18471429999</v>
+        <v>55061.7181236</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5409.18471429999</v>
+        <v>5061.718123600003</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1081836942859998</v>
+        <v>0.1012343624720001</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -14829,6 +14925,9 @@
       </c>
       <c r="DW17" s="3" t="n">
         <v>16.7599</v>
+      </c>
+      <c r="DX17" s="3" t="n">
+        <v>16.6548</v>
       </c>
     </row>
     <row r="18">
@@ -14854,16 +14953,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.81</v>
+        <v>45.01</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84531.19716</v>
+        <v>84908.48435999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4531.197159999996</v>
+        <v>4908.484359999988</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.05663996449999995</v>
+        <v>0.06135605449999985</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -15218,6 +15317,9 @@
       </c>
       <c r="DW18" s="3" t="n">
         <v>44.81</v>
+      </c>
+      <c r="DX18" s="3" t="n">
+        <v>45.01</v>
       </c>
     </row>
     <row r="19">
@@ -15602,6 +15704,9 @@
       <c r="DW19" s="3" t="n">
         <v>13.4251</v>
       </c>
+      <c r="DX19" s="3" t="n">
+        <v>13.4251</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15626,16 +15731,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.83</v>
+        <v>9.84</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>258094.54349</v>
+        <v>258357.10152</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>8094.543490000011</v>
+        <v>8357.101519999997</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.03237817396000004</v>
+        <v>0.03342840607999999</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -15990,6 +16095,9 @@
       </c>
       <c r="DW20" s="3" t="n">
         <v>9.83</v>
+      </c>
+      <c r="DX20" s="3" t="n">
+        <v>9.84</v>
       </c>
     </row>
     <row r="21">
@@ -16015,16 +16123,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>110.4929</v>
+        <v>110.6126</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>167867.3327611</v>
+        <v>168049.1880634</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-2132.667238900001</v>
+        <v>-1950.811936599988</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.01254510140529413</v>
+        <v>-0.01147536433294111</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -16379,6 +16487,9 @@
       </c>
       <c r="DW21" s="3" t="n">
         <v>110.4929</v>
+      </c>
+      <c r="DX21" s="3" t="n">
+        <v>110.6126</v>
       </c>
     </row>
     <row r="22">
@@ -16763,6 +16874,9 @@
       <c r="DW22" s="3" t="n">
         <v>43.729</v>
       </c>
+      <c r="DX22" s="3" t="n">
+        <v>43.729</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -16787,16 +16901,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.7351</v>
+        <v>60.8089</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>164984.8948917</v>
+        <v>165185.3701563</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>14984.89489170001</v>
+        <v>15185.37015630002</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.09989929927800006</v>
+        <v>0.1012358010420001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -17151,6 +17265,9 @@
       </c>
       <c r="DW23" s="3" t="n">
         <v>60.7351</v>
+      </c>
+      <c r="DX23" s="3" t="n">
+        <v>60.8089</v>
       </c>
     </row>
     <row r="24">
@@ -17176,16 +17293,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.617</v>
+        <v>25.5508</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>93076.449162</v>
+        <v>92835.91900879999</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-6923.550837999996</v>
+        <v>-7164.080991200011</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.06923550837999995</v>
+        <v>-0.07164080991200011</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -17534,6 +17651,9 @@
       </c>
       <c r="DW24" s="3" t="n">
         <v>25.617</v>
+      </c>
+      <c r="DX24" s="3" t="n">
+        <v>25.5508</v>
       </c>
     </row>
     <row r="25">
@@ -17559,16 +17679,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.558</v>
+        <v>12.6429</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>206223.382092</v>
+        <v>207617.5822146</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>6223.382091999985</v>
+        <v>7617.58221459997</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.03111691045999992</v>
+        <v>0.03808791107299985</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -17920,6 +18040,9 @@
       </c>
       <c r="DW25" s="3" t="n">
         <v>12.558</v>
+      </c>
+      <c r="DX25" s="3" t="n">
+        <v>12.6429</v>
       </c>
     </row>
     <row r="26">
@@ -17945,16 +18068,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.864</v>
+        <v>10.9552</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>129734.79176</v>
+        <v>130823.876168</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>19734.79176000001</v>
+        <v>20823.876168</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1794071978181819</v>
+        <v>0.1893079651636364</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -18306,6 +18429,9 @@
       </c>
       <c r="DW26" s="3" t="n">
         <v>10.864</v>
+      </c>
+      <c r="DX26" s="3" t="n">
+        <v>10.9552</v>
       </c>
     </row>
     <row r="27">
@@ -18331,16 +18457,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>69.2042</v>
+        <v>69.56189999999999</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>111478.277612</v>
+        <v>112054.482234</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>1478.277611999991</v>
+        <v>2054.482233999981</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.0134388873818181</v>
+        <v>0.01867711121818165</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -18695,6 +18821,9 @@
       </c>
       <c r="DW27" s="3" t="n">
         <v>69.2042</v>
+      </c>
+      <c r="DX27" s="3" t="n">
+        <v>69.56189999999999</v>
       </c>
     </row>
     <row r="28">
@@ -18720,16 +18849,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>114.9478</v>
+        <v>115.5924</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>380092.9475046</v>
+        <v>382224.4186068</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>92.94750460004434</v>
+        <v>2224.418606800027</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.0002445986963159061</v>
+        <v>0.005853733175789545</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -19084,6 +19213,9 @@
       </c>
       <c r="DW28" s="3" t="n">
         <v>114.9478</v>
+      </c>
+      <c r="DX28" s="3" t="n">
+        <v>115.5924</v>
       </c>
     </row>
     <row r="29">
@@ -19109,16 +19241,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.7946</v>
+        <v>11.9453</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>113271.8354038</v>
+        <v>114719.1134459</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>13271.8354038</v>
+        <v>14719.11344589999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.132718354038</v>
+        <v>0.1471911344589999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -19467,6 +19599,9 @@
       </c>
       <c r="DW29" s="3" t="n">
         <v>11.7946</v>
+      </c>
+      <c r="DX29" s="3" t="n">
+        <v>11.9453</v>
       </c>
     </row>
     <row r="30">
@@ -19492,16 +19627,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.2014</v>
+        <v>17.2823</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>127219.1634054</v>
+        <v>127817.4885603</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>27219.16340539999</v>
+        <v>27817.48856029999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2721916340539999</v>
+        <v>0.2781748856029999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -19850,6 +19985,9 @@
       </c>
       <c r="DW30" s="3" t="n">
         <v>17.2014</v>
+      </c>
+      <c r="DX30" s="3" t="n">
+        <v>17.2823</v>
       </c>
     </row>
     <row r="31">
@@ -19875,16 +20013,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>395.3733</v>
+        <v>396.8772</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>105200.927664</v>
+        <v>105601.085376</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>5200.927663999988</v>
+        <v>5601.085376000003</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.05200927663999988</v>
+        <v>0.05601085376000003</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -20236,6 +20374,9 @@
       </c>
       <c r="DW31" s="3" t="n">
         <v>395.3733</v>
+      </c>
+      <c r="DX31" s="3" t="n">
+        <v>396.8772</v>
       </c>
     </row>
     <row r="32">
@@ -20261,16 +20402,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.61</v>
+        <v>10.6</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>224294.9756</v>
+        <v>224083.576</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>24294.97559999998</v>
+        <v>24083.57599999997</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1214748779999999</v>
+        <v>0.1204178799999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -20625,6 +20766,9 @@
       </c>
       <c r="DW32" s="3" t="n">
         <v>10.61</v>
+      </c>
+      <c r="DX32" s="3" t="n">
+        <v>10.6</v>
       </c>
     </row>
     <row r="33">
@@ -20650,16 +20794,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.44</v>
+        <v>19.53</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>69665.9616</v>
+        <v>69988.4892</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>9665.961599999995</v>
+        <v>9988.489199999996</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1610993599999999</v>
+        <v>0.1664748199999999</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -21008,6 +21152,9 @@
       </c>
       <c r="DW33" s="3" t="n">
         <v>19.44</v>
+      </c>
+      <c r="DX33" s="3" t="n">
+        <v>19.53</v>
       </c>
     </row>
     <row r="34">
@@ -21033,16 +21180,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>224.3834</v>
+        <v>223.3608</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>78877.7209854</v>
+        <v>78518.2453848</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-1122.279014600004</v>
+        <v>-1481.7546152</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.01402848768250005</v>
+        <v>-0.01852193268999999</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -21394,6 +21541,9 @@
       </c>
       <c r="DW34" s="3" t="n">
         <v>224.3834</v>
+      </c>
+      <c r="DX34" s="3" t="n">
+        <v>223.3608</v>
       </c>
     </row>
     <row r="35">
@@ -21419,16 +21569,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.18</v>
+        <v>16.37</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>115451.14414</v>
+        <v>116806.87451</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>15451.14413999999</v>
+        <v>16806.87451000001</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1545114413999999</v>
+        <v>0.1680687451000001</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -21780,6 +21930,9 @@
       </c>
       <c r="DW35" s="3" t="n">
         <v>16.18</v>
+      </c>
+      <c r="DX35" s="3" t="n">
+        <v>16.37</v>
       </c>
     </row>
     <row r="36">
@@ -21805,16 +21958,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>371.1075</v>
+        <v>370.6817</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>172826.989395</v>
+        <v>172628.6917802</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>22826.98939500001</v>
+        <v>22628.6917802</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1521799293000001</v>
+        <v>0.1508579452013333</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -22166,6 +22319,9 @@
       </c>
       <c r="DW36" s="3" t="n">
         <v>371.1075</v>
+      </c>
+      <c r="DX36" s="3" t="n">
+        <v>370.6817</v>
       </c>
     </row>
     <row r="37">
@@ -22191,16 +22347,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.922</v>
+        <v>16.976</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>63675.607658</v>
+        <v>63878.803664</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>13675.607658</v>
+        <v>13878.803664</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.27351215316</v>
+        <v>0.27757607328</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -22552,6 +22708,9 @@
       </c>
       <c r="DW37" s="3" t="n">
         <v>16.922</v>
+      </c>
+      <c r="DX37" s="3" t="n">
+        <v>16.976</v>
       </c>
     </row>
     <row r="38">
@@ -22577,16 +22736,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.5331</v>
+        <v>13.5033</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>80934.4609542</v>
+        <v>80756.2425906</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>934.4609541999962</v>
+        <v>756.2425905999989</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.01168076192749995</v>
+        <v>0.009453032382499987</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -22935,6 +23094,9 @@
       </c>
       <c r="DW38" s="3" t="n">
         <v>13.5331</v>
+      </c>
+      <c r="DX38" s="3" t="n">
+        <v>13.5033</v>
       </c>
     </row>
     <row r="39">
@@ -22960,16 +23122,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.8987</v>
+        <v>1025.3162</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51172.8530547</v>
+        <v>51143.7973722</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1172.853054699997</v>
+        <v>1143.797372200002</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02345706109399994</v>
+        <v>0.02287594744400005</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -23318,6 +23480,9 @@
       </c>
       <c r="DW39" s="3" t="n">
         <v>1025.8987</v>
+      </c>
+      <c r="DX39" s="3" t="n">
+        <v>1025.3162</v>
       </c>
     </row>
     <row r="40">
@@ -23343,16 +23508,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.6053</v>
+        <v>20.7459</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>103871.8736431</v>
+        <v>104580.6420393</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>3871.8736431</v>
+        <v>4580.642039300001</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.038718736431</v>
+        <v>0.04580642039300001</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -23704,6 +23869,9 @@
       </c>
       <c r="DW40" s="3" t="n">
         <v>20.6053</v>
+      </c>
+      <c r="DX40" s="3" t="n">
+        <v>20.7459</v>
       </c>
     </row>
     <row r="41">
@@ -23716,13 +23884,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5002638.7241529</v>
+        <v>5000697.2565921</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>532638.7241529</v>
+        <v>530697.2565921</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1191585512646309</v>
+        <v>0.1187242184769799</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-14
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-13 08:54 IST</t>
+          <t>Generated: 2026-10-14 07:04 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5000697.2565921</v>
+        <v>5003786.9415251</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>530697.2565920996</v>
+        <v>533786.9415250998</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1187242184769798</v>
+        <v>0.1194154231599776</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>527330.4982452393</v>
+        <v>531360.0041847229</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-63451.52175476076</v>
+        <v>-59422.01581527712</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1074025945386096</v>
+        <v>-0.1005819639116253</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5528027.754837339</v>
+        <v>5535146.945709823</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>467245.7348373393</v>
+        <v>474364.9257098231</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09232678526575608</v>
+        <v>0.09373352257322144</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-13</t>
+          <t>Last snapshot: 2026-10-14</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FB19"/>
+  <dimension ref="A1:FC19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -777,6 +777,7 @@
     <col width="21" customWidth="1" min="156" max="156"/>
     <col width="21" customWidth="1" min="157" max="157"/>
     <col width="21" customWidth="1" min="158" max="158"/>
+    <col width="21" customWidth="1" min="159" max="159"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1570,6 +1571,11 @@
           <t>2026-10-13</t>
         </is>
       </c>
+      <c r="FC1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1589,13 +1595,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>571.2999877929688</v>
+        <v>569.9000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45703.9990234375</v>
+        <v>45592.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1886.489023437498</v>
+        <v>1774.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2046,6 +2052,9 @@
       </c>
       <c r="FB2" s="3" t="n">
         <v>571.2999877929688</v>
+      </c>
+      <c r="FC2" s="3" t="n">
+        <v>569.9000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -2093,13 +2102,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1431</v>
+        <v>1447.900024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28620</v>
+        <v>28958.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3484.580000000002</v>
+        <v>-3146.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2553,6 +2562,9 @@
       </c>
       <c r="FB4" s="3" t="n">
         <v>1431</v>
+      </c>
+      <c r="FC4" s="3" t="n">
+        <v>1447.900024414062</v>
       </c>
     </row>
     <row r="5">
@@ -2573,13 +2585,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>469.7999877929688</v>
+        <v>475</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9395.999755859375</v>
+        <v>9500</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4817.100244140625</v>
+        <v>-4713.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3033,6 +3045,9 @@
       </c>
       <c r="FB5" s="3" t="n">
         <v>469.7999877929688</v>
+      </c>
+      <c r="FC5" s="3" t="n">
+        <v>475</v>
       </c>
     </row>
     <row r="6">
@@ -3053,13 +3068,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>362.7000122070312</v>
+        <v>376.5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14508.00048828125</v>
+        <v>15060</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2994.239511718752</v>
+        <v>-2442.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3513,6 +3528,9 @@
       </c>
       <c r="FB6" s="3" t="n">
         <v>362.7000122070312</v>
+      </c>
+      <c r="FC6" s="3" t="n">
+        <v>376.5</v>
       </c>
     </row>
     <row r="7">
@@ -3533,13 +3551,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>288.1499938964844</v>
+        <v>288.8500061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>28814.99938964844</v>
+        <v>28885.00061035156</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>2381.179389648438</v>
+        <v>2451.180610351563</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -3993,6 +4011,9 @@
       </c>
       <c r="FB7" s="3" t="n">
         <v>288.1499938964844</v>
+      </c>
+      <c r="FC7" s="3" t="n">
+        <v>288.8500061035156</v>
       </c>
     </row>
     <row r="8">
@@ -4040,13 +4061,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.97999954223633</v>
+        <v>15.30000019073486</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22469.99931335449</v>
+        <v>22950.00028610229</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8580.170686645506</v>
+        <v>-8100.169713897703</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4500,6 +4521,9 @@
       </c>
       <c r="FB9" s="3" t="n">
         <v>14.97999954223633</v>
+      </c>
+      <c r="FC9" s="3" t="n">
+        <v>15.30000019073486</v>
       </c>
     </row>
     <row r="10">
@@ -4520,13 +4544,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>443.6499938964844</v>
+        <v>449.75</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44364.99938964844</v>
+        <v>44975</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-7133.480610351566</v>
+        <v>-6523.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -4980,6 +5004,9 @@
       </c>
       <c r="FB10" s="3" t="n">
         <v>443.6499938964844</v>
+      </c>
+      <c r="FC10" s="3" t="n">
+        <v>449.75</v>
       </c>
     </row>
     <row r="11">
@@ -5000,13 +5027,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>14.09000015258789</v>
+        <v>14.03999996185303</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14090.00015258789</v>
+        <v>14039.99996185303</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4248.790152587891</v>
+        <v>4198.789961853028</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5460,6 +5487,9 @@
       </c>
       <c r="FB11" s="3" t="n">
         <v>14.09000015258789</v>
+      </c>
+      <c r="FC11" s="3" t="n">
+        <v>14.03999996185303</v>
       </c>
     </row>
     <row r="12">
@@ -5480,13 +5510,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2526</v>
+        <v>2556.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25260</v>
+        <v>25568.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2463.25</v>
+        <v>-2154.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5940,6 +5970,9 @@
       </c>
       <c r="FB12" s="3" t="n">
         <v>2526</v>
+      </c>
+      <c r="FC12" s="3" t="n">
+        <v>2556.89990234375</v>
       </c>
     </row>
     <row r="13">
@@ -5960,13 +5993,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>39.66999816894531</v>
+        <v>40.47999954223633</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23801.99890136719</v>
+        <v>24287.9997253418</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11229.76109863281</v>
+        <v>-10743.76027465821</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6420,6 +6453,9 @@
       </c>
       <c r="FB13" s="3" t="n">
         <v>39.66999816894531</v>
+      </c>
+      <c r="FC13" s="3" t="n">
+        <v>40.47999954223633</v>
       </c>
     </row>
     <row r="14">
@@ -6440,13 +6476,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>627.5</v>
+        <v>631.6500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31375</v>
+        <v>31582.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11087.51</v>
+        <v>-10880.00877929688</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6900,6 +6936,9 @@
       </c>
       <c r="FB14" s="3" t="n">
         <v>627.5</v>
+      </c>
+      <c r="FC14" s="3" t="n">
+        <v>631.6500244140625</v>
       </c>
     </row>
     <row r="15">
@@ -6974,13 +7013,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>457.2000122070312</v>
+        <v>462.1000061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>22860.00061035156</v>
+        <v>23105.00030517578</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1105.470610351564</v>
+        <v>1350.470305175782</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7434,6 +7473,9 @@
       </c>
       <c r="FB17" s="3" t="n">
         <v>457.2000122070312</v>
+      </c>
+      <c r="FC17" s="3" t="n">
+        <v>462.1000061035156</v>
       </c>
     </row>
     <row r="18">
@@ -7454,13 +7496,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>342.9500122070312</v>
+        <v>350.8500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34295.00122070312</v>
+        <v>35085.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12345.81877929687</v>
+        <v>-11555.81938964844</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7914,6 +7956,9 @@
       </c>
       <c r="FB18" s="3" t="n">
         <v>342.9500122070312</v>
+      </c>
+      <c r="FC18" s="3" t="n">
+        <v>350.8500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -7926,10 +7971,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>527330.4982452393</v>
+        <v>531360.0041847229</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-63451.52175476075</v>
+        <v>-59422.01581527711</v>
       </c>
     </row>
   </sheetData>
@@ -7943,7 +7988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DX41"/>
+  <dimension ref="A1:DY41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7954,7 +7999,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -8074,6 +8119,7 @@
     <col width="13" customWidth="1" min="126" max="126"/>
     <col width="13" customWidth="1" min="127" max="127"/>
     <col width="13" customWidth="1" min="128" max="128"/>
+    <col width="13" customWidth="1" min="129" max="129"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8717,6 +8763,11 @@
           <t>2026-10-13</t>
         </is>
       </c>
+      <c r="DY1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8741,16 +8792,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.6758</v>
+        <v>57.2884</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64740.0473356</v>
+        <v>64305.1978088</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14740.0473356</v>
+        <v>14305.1978088</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.294800946712</v>
+        <v>0.286103956176</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9108,6 +9159,9 @@
       </c>
       <c r="DX2" s="3" t="n">
         <v>57.6758</v>
+      </c>
+      <c r="DY2" s="3" t="n">
+        <v>57.2884</v>
       </c>
     </row>
     <row r="3">
@@ -9133,16 +9187,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.9597</v>
+        <v>26.7507</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>66191.80591610001</v>
+        <v>65678.6663991</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>6191.805916100013</v>
+        <v>5678.666399099995</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.1031967652683335</v>
+        <v>0.09464443998499991</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9494,6 +9548,9 @@
       </c>
       <c r="DX3" s="3" t="n">
         <v>26.9597</v>
+      </c>
+      <c r="DY3" s="3" t="n">
+        <v>26.7507</v>
       </c>
     </row>
     <row r="4">
@@ -9519,16 +9576,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.71</v>
+        <v>12.45</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>244109.44203</v>
+        <v>239115.85785</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>64109.44203000003</v>
+        <v>59115.85785</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3561635668333335</v>
+        <v>0.3284214325</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9880,6 +9937,9 @@
       </c>
       <c r="DX4" s="3" t="n">
         <v>12.71</v>
+      </c>
+      <c r="DY4" s="3" t="n">
+        <v>12.45</v>
       </c>
     </row>
     <row r="5">
@@ -9905,16 +9965,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.959199999999999</v>
+        <v>9.1648</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>164437.9452096</v>
+        <v>168211.5457024</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-45562.05479040003</v>
+        <v>-41788.45429760002</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2169621656685715</v>
+        <v>-0.1989926395123811</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10266,6 +10326,9 @@
       </c>
       <c r="DX5" s="3" t="n">
         <v>8.959199999999999</v>
+      </c>
+      <c r="DY5" s="3" t="n">
+        <v>9.1648</v>
       </c>
     </row>
     <row r="6">
@@ -10291,16 +10354,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.1372</v>
+        <v>11.1627</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>47098.9626444</v>
+        <v>47206.8015579</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-2901.037355600005</v>
+        <v>-2793.198442100002</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.0580207471120001</v>
+        <v>-0.05586396884200003</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -10658,6 +10721,9 @@
       </c>
       <c r="DX6" s="3" t="n">
         <v>11.1372</v>
+      </c>
+      <c r="DY6" s="3" t="n">
+        <v>11.1627</v>
       </c>
     </row>
     <row r="7">
@@ -10683,16 +10749,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.7421</v>
+        <v>33.4936</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74436.422284</v>
+        <v>73888.22134400001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14436.422284</v>
+        <v>13888.22134400001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2406070380666667</v>
+        <v>0.2314703557333334</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -11044,6 +11110,9 @@
       </c>
       <c r="DX7" s="3" t="n">
         <v>33.7421</v>
+      </c>
+      <c r="DY7" s="3" t="n">
+        <v>33.4936</v>
       </c>
     </row>
     <row r="8">
@@ -11069,16 +11138,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.8242</v>
+        <v>35.8444</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57483.2605506</v>
+        <v>57515.67332920001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7483.260550599996</v>
+        <v>7515.673329200006</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1496652110119999</v>
+        <v>0.1503134665840001</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -11436,6 +11505,9 @@
       </c>
       <c r="DX8" s="3" t="n">
         <v>35.8242</v>
+      </c>
+      <c r="DY8" s="3" t="n">
+        <v>35.8444</v>
       </c>
     </row>
     <row r="9">
@@ -11461,16 +11533,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.6817</v>
+        <v>42.1279</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>137409.1662081</v>
+        <v>135626.2663647</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>37409.16620810001</v>
+        <v>35626.26636469999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3740916620810001</v>
+        <v>0.3562626636469999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -11822,6 +11894,9 @@
       </c>
       <c r="DX9" s="3" t="n">
         <v>42.6817</v>
+      </c>
+      <c r="DY9" s="3" t="n">
+        <v>42.1279</v>
       </c>
     </row>
     <row r="10">
@@ -11847,16 +11922,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.9149</v>
+        <v>48.7339</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>139244.0403191</v>
+        <v>138728.7950401</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>39244.04031910002</v>
+        <v>38728.7950401</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3924404031910002</v>
+        <v>0.387287950401</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -12208,6 +12283,9 @@
       </c>
       <c r="DX10" s="3" t="n">
         <v>48.9149</v>
+      </c>
+      <c r="DY10" s="3" t="n">
+        <v>48.7339</v>
       </c>
     </row>
     <row r="11">
@@ -12233,16 +12311,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>108.209</v>
+        <v>107.5504</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32562.144071</v>
+        <v>32363.9588176</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2562.144070999999</v>
+        <v>2363.958817599996</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.08540480236666663</v>
+        <v>0.0787986272533332</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -12594,6 +12672,9 @@
       </c>
       <c r="DX11" s="3" t="n">
         <v>108.209</v>
+      </c>
+      <c r="DY11" s="3" t="n">
+        <v>107.5504</v>
       </c>
     </row>
     <row r="12">
@@ -12619,16 +12700,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>219.3</v>
+        <v>221.294</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102088.9746</v>
+        <v>103017.225468</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2088.974600000001</v>
+        <v>3017.225468000004</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02088974600000001</v>
+        <v>0.03017225468000004</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -12986,6 +13067,9 @@
       </c>
       <c r="DX12" s="3" t="n">
         <v>219.3</v>
+      </c>
+      <c r="DY12" s="3" t="n">
+        <v>221.294</v>
       </c>
     </row>
     <row r="13">
@@ -13011,16 +13095,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.532</v>
+        <v>21.498</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>249504.31086</v>
+        <v>249110.33229</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>49504.31086</v>
+        <v>49110.33228999999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2475215543</v>
+        <v>0.24555166145</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -13378,6 +13462,9 @@
       </c>
       <c r="DX13" s="3" t="n">
         <v>21.532</v>
+      </c>
+      <c r="DY13" s="3" t="n">
+        <v>21.498</v>
       </c>
     </row>
     <row r="14">
@@ -13403,16 +13490,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.7693</v>
+        <v>36.7233</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>136256.7532958</v>
+        <v>132483.1974198</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>36256.75329580001</v>
+        <v>32483.19741980001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3625675329580001</v>
+        <v>0.3248319741980001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -13764,6 +13851,9 @@
       </c>
       <c r="DX14" s="3" t="n">
         <v>37.7693</v>
+      </c>
+      <c r="DY14" s="3" t="n">
+        <v>36.7233</v>
       </c>
     </row>
     <row r="15">
@@ -13789,16 +13879,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.3</v>
+        <v>11.32</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>110106.6011</v>
+        <v>110301.48004</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>10106.60110000001</v>
+        <v>10301.48004000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1010660110000001</v>
+        <v>0.1030148004000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -14156,6 +14246,9 @@
       </c>
       <c r="DX15" s="3" t="n">
         <v>11.3</v>
+      </c>
+      <c r="DY15" s="3" t="n">
+        <v>11.32</v>
       </c>
     </row>
     <row r="16">
@@ -14181,16 +14274,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.5233</v>
+        <v>25.3108</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>146068.0082224</v>
+        <v>144851.8860224</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>46068.00822239998</v>
+        <v>44851.88602239999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4606800822239998</v>
+        <v>0.4485188602239999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -14542,6 +14635,9 @@
       </c>
       <c r="DX16" s="3" t="n">
         <v>25.5233</v>
+      </c>
+      <c r="DY16" s="3" t="n">
+        <v>25.3108</v>
       </c>
     </row>
     <row r="17">
@@ -14567,16 +14663,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6548</v>
+        <v>16.7115</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55061.7181236</v>
+        <v>55249.1715555</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5061.718123600003</v>
+        <v>5249.171555499997</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1012343624720001</v>
+        <v>0.1049834311099999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -14928,6 +15024,9 @@
       </c>
       <c r="DX17" s="3" t="n">
         <v>16.6548</v>
+      </c>
+      <c r="DY17" s="3" t="n">
+        <v>16.7115</v>
       </c>
     </row>
     <row r="18">
@@ -14953,16 +15052,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.01</v>
+        <v>45.12</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84908.48435999999</v>
+        <v>85115.99231999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4908.484359999988</v>
+        <v>5115.99231999999</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06135605449999985</v>
+        <v>0.06394990399999988</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -15320,6 +15419,9 @@
       </c>
       <c r="DX18" s="3" t="n">
         <v>45.01</v>
+      </c>
+      <c r="DY18" s="3" t="n">
+        <v>45.12</v>
       </c>
     </row>
     <row r="19">
@@ -15345,16 +15447,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.4251</v>
+        <v>12.7797</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>194217.7802266</v>
+        <v>184880.9294502</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>44217.78022660001</v>
+        <v>34880.9294502</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2947852015106667</v>
+        <v>0.232539529668</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -15706,6 +15808,9 @@
       </c>
       <c r="DX19" s="3" t="n">
         <v>13.4251</v>
+      </c>
+      <c r="DY19" s="3" t="n">
+        <v>12.7797</v>
       </c>
     </row>
     <row r="20">
@@ -15731,16 +15836,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.84</v>
+        <v>10.05</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>258357.10152</v>
+        <v>263870.82015</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>8357.101519999997</v>
+        <v>13870.82015000004</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.03342840607999999</v>
+        <v>0.05548328060000017</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -16098,6 +16203,9 @@
       </c>
       <c r="DX20" s="3" t="n">
         <v>9.84</v>
+      </c>
+      <c r="DY20" s="3" t="n">
+        <v>10.05</v>
       </c>
     </row>
     <row r="21">
@@ -16123,16 +16231,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>110.6126</v>
+        <v>111.8284</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>168049.1880634</v>
+        <v>169896.3031556</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-1950.811936599988</v>
+        <v>-103.696844399994</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.01147536433294111</v>
+        <v>-0.0006099814376470235</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -16490,6 +16598,9 @@
       </c>
       <c r="DX21" s="3" t="n">
         <v>110.6126</v>
+      </c>
+      <c r="DY21" s="3" t="n">
+        <v>111.8284</v>
       </c>
     </row>
     <row r="22">
@@ -16515,16 +16626,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.729</v>
+        <v>41.783</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67100.40134</v>
+        <v>64114.34218000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7100.401339999997</v>
+        <v>4114.342180000007</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1183400223333333</v>
+        <v>0.06857236966666679</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -16876,6 +16987,9 @@
       </c>
       <c r="DX22" s="3" t="n">
         <v>43.729</v>
+      </c>
+      <c r="DY22" s="3" t="n">
+        <v>41.783</v>
       </c>
     </row>
     <row r="23">
@@ -16901,16 +17015,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.8089</v>
+        <v>61.149</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>165185.3701563</v>
+        <v>166109.240583</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>15185.37015630002</v>
+        <v>16109.24058300001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1012358010420001</v>
+        <v>0.10739493722</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -17268,6 +17382,9 @@
       </c>
       <c r="DX23" s="3" t="n">
         <v>60.8089</v>
+      </c>
+      <c r="DY23" s="3" t="n">
+        <v>61.149</v>
       </c>
     </row>
     <row r="24">
@@ -17293,16 +17410,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.5508</v>
+        <v>25.8095</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>92835.91900879999</v>
+        <v>93775.875967</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-7164.080991200011</v>
+        <v>-6224.124033</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.07164080991200011</v>
+        <v>-0.06224124033</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -17654,6 +17771,9 @@
       </c>
       <c r="DX24" s="3" t="n">
         <v>25.5508</v>
+      </c>
+      <c r="DY24" s="3" t="n">
+        <v>25.8095</v>
       </c>
     </row>
     <row r="25">
@@ -17679,16 +17799,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.6429</v>
+        <v>12.7551</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>207617.5822146</v>
+        <v>209460.0940374</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>7617.58221459997</v>
+        <v>9460.094037400006</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.03808791107299985</v>
+        <v>0.04730047018700003</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -18043,6 +18163,9 @@
       </c>
       <c r="DX25" s="3" t="n">
         <v>12.6429</v>
+      </c>
+      <c r="DY25" s="3" t="n">
+        <v>12.7551</v>
       </c>
     </row>
     <row r="26">
@@ -18068,16 +18191,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.9552</v>
+        <v>11.1636</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>130823.876168</v>
+        <v>133312.529574</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>20823.876168</v>
+        <v>23312.52957400001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1893079651636364</v>
+        <v>0.2119320870363638</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -18432,6 +18555,9 @@
       </c>
       <c r="DX26" s="3" t="n">
         <v>10.9552</v>
+      </c>
+      <c r="DY26" s="3" t="n">
+        <v>11.1636</v>
       </c>
     </row>
     <row r="27">
@@ -18457,16 +18583,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>69.56189999999999</v>
+        <v>69.9344</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>112054.482234</v>
+        <v>112654.527584</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>2054.482233999981</v>
+        <v>2654.527583999981</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.01867711121818165</v>
+        <v>0.02413206894545437</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -18824,6 +18950,9 @@
       </c>
       <c r="DX27" s="3" t="n">
         <v>69.56189999999999</v>
+      </c>
+      <c r="DY27" s="3" t="n">
+        <v>69.9344</v>
       </c>
     </row>
     <row r="28">
@@ -18849,16 +18978,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>115.5924</v>
+        <v>116.6107</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>382224.4186068</v>
+        <v>385591.5874299</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>2224.418606800027</v>
+        <v>5591.587429900013</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.005853733175789545</v>
+        <v>0.01471470376289477</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -19216,6 +19345,9 @@
       </c>
       <c r="DX28" s="3" t="n">
         <v>115.5924</v>
+      </c>
+      <c r="DY28" s="3" t="n">
+        <v>116.6107</v>
       </c>
     </row>
     <row r="29">
@@ -19241,16 +19373,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.9453</v>
+        <v>12.1132</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114719.1134459</v>
+        <v>116331.5751796</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14719.11344589999</v>
+        <v>16331.5751796</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1471911344589999</v>
+        <v>0.163315751796</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -19602,6 +19734,9 @@
       </c>
       <c r="DX29" s="3" t="n">
         <v>11.9453</v>
+      </c>
+      <c r="DY29" s="3" t="n">
+        <v>12.1132</v>
       </c>
     </row>
     <row r="30">
@@ -19627,16 +19762,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.2823</v>
+        <v>17.3778</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>127817.4885603</v>
+        <v>128523.7932858</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>27817.48856029999</v>
+        <v>28523.7932858</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2781748856029999</v>
+        <v>0.285237932858</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -19988,6 +20123,9 @@
       </c>
       <c r="DX30" s="3" t="n">
         <v>17.2823</v>
+      </c>
+      <c r="DY30" s="3" t="n">
+        <v>17.3778</v>
       </c>
     </row>
     <row r="31">
@@ -20013,16 +20151,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>396.8772</v>
+        <v>399.3015</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>105601.085376</v>
+        <v>106246.14312</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>5601.085376000003</v>
+        <v>6246.143119999993</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.05601085376000003</v>
+        <v>0.06246143119999993</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -20377,6 +20515,9 @@
       </c>
       <c r="DX31" s="3" t="n">
         <v>396.8772</v>
+      </c>
+      <c r="DY31" s="3" t="n">
+        <v>399.3015</v>
       </c>
     </row>
     <row r="32">
@@ -20402,16 +20543,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.6</v>
+        <v>10.68</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>224083.576</v>
+        <v>225774.7728</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>24083.57599999997</v>
+        <v>25774.77279999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1204178799999999</v>
+        <v>0.1288738639999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -20769,6 +20910,9 @@
       </c>
       <c r="DX32" s="3" t="n">
         <v>10.6</v>
+      </c>
+      <c r="DY32" s="3" t="n">
+        <v>10.68</v>
       </c>
     </row>
     <row r="33">
@@ -20794,16 +20938,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.53</v>
+        <v>19.61</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>69988.4892</v>
+        <v>70275.1804</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>9988.489199999996</v>
+        <v>10275.1804</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1664748199999999</v>
+        <v>0.1712530066666666</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -21155,6 +21299,9 @@
       </c>
       <c r="DX33" s="3" t="n">
         <v>19.53</v>
+      </c>
+      <c r="DY33" s="3" t="n">
+        <v>19.61</v>
       </c>
     </row>
     <row r="34">
@@ -21180,16 +21327,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>223.3608</v>
+        <v>228.6134</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>78518.2453848</v>
-      </c>
-      <c r="H34" s="6" t="n">
-        <v>-1481.7546152</v>
-      </c>
-      <c r="I34" s="13" t="n">
-        <v>-0.01852193268999999</v>
+        <v>80364.69711540001</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>364.6971154000057</v>
+      </c>
+      <c r="I34" s="12" t="n">
+        <v>0.004558713942500072</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -21544,6 +21691,9 @@
       </c>
       <c r="DX34" s="3" t="n">
         <v>223.3608</v>
+      </c>
+      <c r="DY34" s="3" t="n">
+        <v>228.6134</v>
       </c>
     </row>
     <row r="35">
@@ -21569,16 +21719,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.37</v>
+        <v>16.27</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>116806.87451</v>
+        <v>116093.33221</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>16806.87451000001</v>
+        <v>16093.33220999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1680687451000001</v>
+        <v>0.1609333220999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -21933,6 +22083,9 @@
       </c>
       <c r="DX35" s="3" t="n">
         <v>16.37</v>
+      </c>
+      <c r="DY35" s="3" t="n">
+        <v>16.27</v>
       </c>
     </row>
     <row r="36">
@@ -21958,16 +22111,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>370.6817</v>
+        <v>369.2882</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>172628.6917802</v>
+        <v>171979.7304692</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>22628.6917802</v>
+        <v>21979.7304692</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1508579452013333</v>
+        <v>0.1465315364613334</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -22322,6 +22475,9 @@
       </c>
       <c r="DX36" s="3" t="n">
         <v>370.6817</v>
+      </c>
+      <c r="DY36" s="3" t="n">
+        <v>369.2882</v>
       </c>
     </row>
     <row r="37">
@@ -22347,16 +22503,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.976</v>
+        <v>16.894</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>63878.803664</v>
+        <v>63570.246766</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>13878.803664</v>
+        <v>13570.246766</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.27757607328</v>
+        <v>0.2714049353199999</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -22711,6 +22867,9 @@
       </c>
       <c r="DX37" s="3" t="n">
         <v>16.976</v>
+      </c>
+      <c r="DY37" s="3" t="n">
+        <v>16.894</v>
       </c>
     </row>
     <row r="38">
@@ -22736,16 +22895,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.5033</v>
+        <v>13.6672</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>80756.2425906</v>
+        <v>81736.4435904</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>756.2425905999989</v>
+        <v>1736.443590399998</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.009453032382499987</v>
+        <v>0.02170554487999998</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -23097,6 +23256,9 @@
       </c>
       <c r="DX38" s="3" t="n">
         <v>13.5033</v>
+      </c>
+      <c r="DY38" s="3" t="n">
+        <v>13.6672</v>
       </c>
     </row>
     <row r="39">
@@ -23122,16 +23284,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.3162</v>
+        <v>1026.4001</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51143.7973722</v>
+        <v>51197.86338810001</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1143.797372200002</v>
+        <v>1197.863388100006</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02287594744400005</v>
+        <v>0.02395726776200012</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -23483,6 +23645,9 @@
       </c>
       <c r="DX39" s="3" t="n">
         <v>1025.3162</v>
+      </c>
+      <c r="DY39" s="3" t="n">
+        <v>1026.4001</v>
       </c>
     </row>
     <row r="40">
@@ -23508,16 +23673,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.7459</v>
+        <v>20.88</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>104580.6420393</v>
+        <v>105256.64376</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>4580.642039300001</v>
+        <v>5256.643759999992</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.04580642039300001</v>
+        <v>0.05256643759999992</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -23872,6 +24037,9 @@
       </c>
       <c r="DX40" s="3" t="n">
         <v>20.7459</v>
+      </c>
+      <c r="DY40" s="3" t="n">
+        <v>20.88</v>
       </c>
     </row>
     <row r="41">
@@ -23884,13 +24052,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5000697.2565921</v>
+        <v>5003786.9415251</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>530697.2565921</v>
+        <v>533786.9415251</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1187242184769799</v>
+        <v>0.1194154231599776</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-15
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-14 07:04 IST</t>
+          <t>Generated: 2026-10-15 06:55 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5003786.9415251</v>
+        <v>4983781.1649683</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>533786.9415250998</v>
+        <v>513781.1649682997</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1194154231599776</v>
+        <v>0.1149398579347427</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>531360.0041847229</v>
+        <v>530049.4978981018</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-59422.01581527712</v>
+        <v>-60732.52210189821</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1005819639116253</v>
+        <v>-0.1028002208020789</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5535146.945709823</v>
+        <v>5513830.662866401</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>474364.9257098231</v>
+        <v>453048.6428664019</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09373352257322144</v>
+        <v>0.08952146942428514</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-14</t>
+          <t>Last snapshot: 2026-10-15</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FC19"/>
+  <dimension ref="A1:FD19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -778,6 +778,7 @@
     <col width="21" customWidth="1" min="157" max="157"/>
     <col width="21" customWidth="1" min="158" max="158"/>
     <col width="21" customWidth="1" min="159" max="159"/>
+    <col width="21" customWidth="1" min="160" max="160"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1576,6 +1577,11 @@
           <t>2026-10-14</t>
         </is>
       </c>
+      <c r="FD1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1595,13 +1601,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>569.9000244140625</v>
+        <v>567.8499755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45592.001953125</v>
+        <v>45427.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1774.491953124998</v>
+        <v>1610.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2055,6 +2061,9 @@
       </c>
       <c r="FC2" s="3" t="n">
         <v>569.9000244140625</v>
+      </c>
+      <c r="FD2" s="3" t="n">
+        <v>567.8499755859375</v>
       </c>
     </row>
     <row r="3">
@@ -2102,13 +2111,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1447.900024414062</v>
+        <v>1452.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28958.00048828125</v>
+        <v>29056.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3146.579511718752</v>
+        <v>-3048.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2565,6 +2574,9 @@
       </c>
       <c r="FC4" s="3" t="n">
         <v>1447.900024414062</v>
+      </c>
+      <c r="FD4" s="3" t="n">
+        <v>1452.800048828125</v>
       </c>
     </row>
     <row r="5">
@@ -2585,13 +2597,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>475</v>
+        <v>469.6000061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9500</v>
+        <v>9392.000122070312</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4713.1</v>
+        <v>-4821.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3048,6 +3060,9 @@
       </c>
       <c r="FC5" s="3" t="n">
         <v>475</v>
+      </c>
+      <c r="FD5" s="3" t="n">
+        <v>469.6000061035156</v>
       </c>
     </row>
     <row r="6">
@@ -3068,13 +3083,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>376.5</v>
+        <v>363.8999938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15060</v>
+        <v>14555.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2442.240000000002</v>
+        <v>-2946.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3531,6 +3546,9 @@
       </c>
       <c r="FC6" s="3" t="n">
         <v>376.5</v>
+      </c>
+      <c r="FD6" s="3" t="n">
+        <v>363.8999938964844</v>
       </c>
     </row>
     <row r="7">
@@ -3551,13 +3569,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>288.8500061035156</v>
+        <v>280</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>28885.00061035156</v>
+        <v>28000</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>2451.180610351563</v>
+        <v>1566.18</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4014,6 +4032,9 @@
       </c>
       <c r="FC7" s="3" t="n">
         <v>288.8500061035156</v>
+      </c>
+      <c r="FD7" s="3" t="n">
+        <v>280</v>
       </c>
     </row>
     <row r="8">
@@ -4061,13 +4082,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.30000019073486</v>
+        <v>15.35999965667725</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22950.00028610229</v>
+        <v>23039.99948501587</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8100.169713897703</v>
+        <v>-8010.170514984129</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4524,6 +4545,9 @@
       </c>
       <c r="FC9" s="3" t="n">
         <v>15.30000019073486</v>
+      </c>
+      <c r="FD9" s="3" t="n">
+        <v>15.35999965667725</v>
       </c>
     </row>
     <row r="10">
@@ -4544,13 +4568,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>449.75</v>
+        <v>447.3500061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44975</v>
+        <v>44735.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6523.480000000003</v>
+        <v>-6763.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5007,6 +5031,9 @@
       </c>
       <c r="FC10" s="3" t="n">
         <v>449.75</v>
+      </c>
+      <c r="FD10" s="3" t="n">
+        <v>447.3500061035156</v>
       </c>
     </row>
     <row r="11">
@@ -5027,13 +5054,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>14.03999996185303</v>
+        <v>14.40999984741211</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14039.99996185303</v>
+        <v>14409.99984741211</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4198.789961853028</v>
+        <v>4568.78984741211</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5490,6 +5517,9 @@
       </c>
       <c r="FC11" s="3" t="n">
         <v>14.03999996185303</v>
+      </c>
+      <c r="FD11" s="3" t="n">
+        <v>14.40999984741211</v>
       </c>
     </row>
     <row r="12">
@@ -5510,13 +5540,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2556.89990234375</v>
+        <v>2564.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25568.9990234375</v>
+        <v>25645</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2154.2509765625</v>
+        <v>-2078.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -5973,6 +6003,9 @@
       </c>
       <c r="FC12" s="3" t="n">
         <v>2556.89990234375</v>
+      </c>
+      <c r="FD12" s="3" t="n">
+        <v>2564.5</v>
       </c>
     </row>
     <row r="13">
@@ -5993,13 +6026,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>40.47999954223633</v>
+        <v>41.11999893188477</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>24287.9997253418</v>
+        <v>24671.99935913086</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-10743.76027465821</v>
+        <v>-10359.76064086914</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6456,6 +6489,9 @@
       </c>
       <c r="FC13" s="3" t="n">
         <v>40.47999954223633</v>
+      </c>
+      <c r="FD13" s="3" t="n">
+        <v>41.11999893188477</v>
       </c>
     </row>
     <row r="14">
@@ -6476,13 +6512,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>631.6500244140625</v>
+        <v>627</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31582.50122070312</v>
+        <v>31350</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-10880.00877929688</v>
+        <v>-11112.51</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6939,6 +6975,9 @@
       </c>
       <c r="FC14" s="3" t="n">
         <v>631.6500244140625</v>
+      </c>
+      <c r="FD14" s="3" t="n">
+        <v>627</v>
       </c>
     </row>
     <row r="15">
@@ -7013,13 +7052,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>462.1000061035156</v>
+        <v>460.1000061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23105.00030517578</v>
+        <v>23005.00030517578</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1350.470305175782</v>
+        <v>1250.470305175782</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7476,6 +7515,9 @@
       </c>
       <c r="FC17" s="3" t="n">
         <v>462.1000061035156</v>
+      </c>
+      <c r="FD17" s="3" t="n">
+        <v>460.1000061035156</v>
       </c>
     </row>
     <row r="18">
@@ -7496,13 +7538,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>350.8500061035156</v>
+        <v>349.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35085.00061035156</v>
+        <v>34989.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11555.81938964844</v>
+        <v>-11650.82061035156</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -7959,6 +8001,9 @@
       </c>
       <c r="FC18" s="3" t="n">
         <v>350.8500061035156</v>
+      </c>
+      <c r="FD18" s="3" t="n">
+        <v>349.8999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -7971,10 +8016,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>531360.0041847229</v>
+        <v>530049.4978981018</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-59422.01581527711</v>
+        <v>-60732.5221018982</v>
       </c>
     </row>
   </sheetData>
@@ -7988,7 +8033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DY41"/>
+  <dimension ref="A1:DZ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8120,6 +8165,7 @@
     <col width="13" customWidth="1" min="127" max="127"/>
     <col width="13" customWidth="1" min="128" max="128"/>
     <col width="13" customWidth="1" min="129" max="129"/>
+    <col width="13" customWidth="1" min="130" max="130"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8768,6 +8814,11 @@
           <t>2026-10-14</t>
         </is>
       </c>
+      <c r="DZ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8792,16 +8843,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.2884</v>
+        <v>56.7451</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64305.1978088</v>
+        <v>63695.3533382</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14305.1978088</v>
+        <v>13695.3533382</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.286103956176</v>
+        <v>0.2739070667640001</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9162,6 +9213,9 @@
       </c>
       <c r="DY2" s="3" t="n">
         <v>57.2884</v>
+      </c>
+      <c r="DZ2" s="3" t="n">
+        <v>56.7451</v>
       </c>
     </row>
     <row r="3">
@@ -9187,16 +9241,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.7507</v>
+        <v>26.6112</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65678.6663991</v>
+        <v>65336.16418560001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5678.666399099995</v>
+        <v>5336.164185600006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09464443998499991</v>
+        <v>0.0889360697600001</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9551,6 +9605,9 @@
       </c>
       <c r="DY3" s="3" t="n">
         <v>26.7507</v>
+      </c>
+      <c r="DZ3" s="3" t="n">
+        <v>26.6112</v>
       </c>
     </row>
     <row r="4">
@@ -9576,16 +9633,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.45</v>
+        <v>12.37</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>239115.85785</v>
+        <v>237579.37041</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>59115.85785</v>
+        <v>57579.37041</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3284214325</v>
+        <v>0.3198853911666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -9940,6 +9997,9 @@
       </c>
       <c r="DY4" s="3" t="n">
         <v>12.45</v>
+      </c>
+      <c r="DZ4" s="3" t="n">
+        <v>12.37</v>
       </c>
     </row>
     <row r="5">
@@ -9965,16 +10025,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.1648</v>
+        <v>9.233000000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>168211.5457024</v>
+        <v>169463.294504</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-41788.45429760002</v>
+        <v>-40536.70549599998</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1989926395123811</v>
+        <v>-0.1930319309333332</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10329,6 +10389,9 @@
       </c>
       <c r="DY5" s="3" t="n">
         <v>9.1648</v>
+      </c>
+      <c r="DZ5" s="3" t="n">
+        <v>9.233000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -10354,16 +10417,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.1627</v>
+        <v>11.2744</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>47206.8015579</v>
+        <v>47679.1782888</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-2793.198442100002</v>
+        <v>-2320.821711199998</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.05586396884200003</v>
+        <v>-0.04641643422399997</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -10724,6 +10787,9 @@
       </c>
       <c r="DY6" s="3" t="n">
         <v>11.1627</v>
+      </c>
+      <c r="DZ6" s="3" t="n">
+        <v>11.2744</v>
       </c>
     </row>
     <row r="7">
@@ -10749,16 +10815,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.4936</v>
+        <v>33.5161</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73888.22134400001</v>
+        <v>73937.857244</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13888.22134400001</v>
+        <v>13937.857244</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2314703557333334</v>
+        <v>0.2322976207333333</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -11113,6 +11179,9 @@
       </c>
       <c r="DY7" s="3" t="n">
         <v>33.4936</v>
+      </c>
+      <c r="DZ7" s="3" t="n">
+        <v>33.5161</v>
       </c>
     </row>
     <row r="8">
@@ -11138,16 +11207,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.8444</v>
+        <v>35.7205</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57515.67332920001</v>
+        <v>57316.8642565</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7515.673329200006</v>
+        <v>7316.864256500005</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1503134665840001</v>
+        <v>0.1463372851300001</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -11508,6 +11577,9 @@
       </c>
       <c r="DY8" s="3" t="n">
         <v>35.8444</v>
+      </c>
+      <c r="DZ8" s="3" t="n">
+        <v>35.7205</v>
       </c>
     </row>
     <row r="9">
@@ -11533,16 +11605,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.1279</v>
+        <v>41.2063</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>135626.2663647</v>
+        <v>132659.2737759</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>35626.26636469999</v>
+        <v>32659.27377589999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3562626636469999</v>
+        <v>0.3265927377589999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -11897,6 +11969,9 @@
       </c>
       <c r="DY9" s="3" t="n">
         <v>42.1279</v>
+      </c>
+      <c r="DZ9" s="3" t="n">
+        <v>41.2063</v>
       </c>
     </row>
     <row r="10">
@@ -11922,16 +11997,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.7339</v>
+        <v>48.3515</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138728.7950401</v>
+        <v>137640.2326385</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38728.7950401</v>
+        <v>37640.23263850002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.387287950401</v>
+        <v>0.3764023263850002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -12286,6 +12361,9 @@
       </c>
       <c r="DY10" s="3" t="n">
         <v>48.7339</v>
+      </c>
+      <c r="DZ10" s="3" t="n">
+        <v>48.3515</v>
       </c>
     </row>
     <row r="11">
@@ -12311,16 +12389,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.5504</v>
+        <v>104.9217</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32363.9588176</v>
+        <v>31572.9330423</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2363.958817599996</v>
+        <v>1572.933042299999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.0787986272533332</v>
+        <v>0.05243110140999997</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -12675,6 +12753,9 @@
       </c>
       <c r="DY11" s="3" t="n">
         <v>107.5504</v>
+      </c>
+      <c r="DZ11" s="3" t="n">
+        <v>104.9217</v>
       </c>
     </row>
     <row r="12">
@@ -12700,16 +12781,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>221.294</v>
+        <v>220.903</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>103017.225468</v>
+        <v>102835.206366</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3017.225468000004</v>
+        <v>2835.206365999999</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.03017225468000004</v>
+        <v>0.02835206365999999</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -13070,6 +13151,9 @@
       </c>
       <c r="DY12" s="3" t="n">
         <v>221.294</v>
+      </c>
+      <c r="DZ12" s="3" t="n">
+        <v>220.903</v>
       </c>
     </row>
     <row r="13">
@@ -13095,16 +13179,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.498</v>
+        <v>21.275</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>249110.33229</v>
+        <v>246526.296375</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>49110.33228999999</v>
+        <v>46526.29637499998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.24555166145</v>
+        <v>0.2326314818749999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -13465,6 +13549,9 @@
       </c>
       <c r="DY13" s="3" t="n">
         <v>21.498</v>
+      </c>
+      <c r="DZ13" s="3" t="n">
+        <v>21.275</v>
       </c>
     </row>
     <row r="14">
@@ -13490,16 +13577,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36.7233</v>
+        <v>36.4753</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>132483.1974198</v>
+        <v>131588.5111318</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>32483.19741980001</v>
+        <v>31588.51113179998</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3248319741980001</v>
+        <v>0.3158851113179998</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -13854,6 +13941,9 @@
       </c>
       <c r="DY14" s="3" t="n">
         <v>36.7233</v>
+      </c>
+      <c r="DZ14" s="3" t="n">
+        <v>36.4753</v>
       </c>
     </row>
     <row r="15">
@@ -13879,16 +13969,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.32</v>
+        <v>11.42</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>110301.48004</v>
+        <v>111275.87474</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>10301.48004000001</v>
+        <v>11275.87474</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1030148004000001</v>
+        <v>0.1127587474</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -14249,6 +14339,9 @@
       </c>
       <c r="DY15" s="3" t="n">
         <v>11.32</v>
+      </c>
+      <c r="DZ15" s="3" t="n">
+        <v>11.42</v>
       </c>
     </row>
     <row r="16">
@@ -14274,16 +14367,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.3108</v>
+        <v>24.7424</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>144851.8860224</v>
+        <v>141598.9737472</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>44851.88602239999</v>
+        <v>41598.97374719998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4485188602239999</v>
+        <v>0.4159897374719999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -14638,6 +14731,9 @@
       </c>
       <c r="DY16" s="3" t="n">
         <v>25.3108</v>
+      </c>
+      <c r="DZ16" s="3" t="n">
+        <v>24.7424</v>
       </c>
     </row>
     <row r="17">
@@ -14663,16 +14759,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7115</v>
+        <v>16.686</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55249.1715555</v>
+        <v>55164.867102</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5249.171555499997</v>
+        <v>5164.867101999997</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1049834311099999</v>
+        <v>0.1032973420399999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -15027,6 +15123,9 @@
       </c>
       <c r="DY17" s="3" t="n">
         <v>16.7115</v>
+      </c>
+      <c r="DZ17" s="3" t="n">
+        <v>16.686</v>
       </c>
     </row>
     <row r="18">
@@ -15052,16 +15151,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.12</v>
+        <v>44.88</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85115.99231999999</v>
+        <v>84663.24768</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5115.99231999999</v>
+        <v>4663.24768</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06394990399999988</v>
+        <v>0.05829059600000001</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -15422,6 +15521,9 @@
       </c>
       <c r="DY18" s="3" t="n">
         <v>45.12</v>
+      </c>
+      <c r="DZ18" s="3" t="n">
+        <v>44.88</v>
       </c>
     </row>
     <row r="19">
@@ -15447,16 +15549,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>12.7797</v>
+        <v>12.8126</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>184880.9294502</v>
+        <v>185356.8860516</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>34880.9294502</v>
+        <v>35356.88605159998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.232539529668</v>
+        <v>0.2357125736773332</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -15811,6 +15913,9 @@
       </c>
       <c r="DY19" s="3" t="n">
         <v>12.7797</v>
+      </c>
+      <c r="DZ19" s="3" t="n">
+        <v>12.8126</v>
       </c>
     </row>
     <row r="20">
@@ -16207,6 +16312,9 @@
       <c r="DY20" s="3" t="n">
         <v>10.05</v>
       </c>
+      <c r="DZ20" s="3" t="n">
+        <v>10.05</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -16231,16 +16339,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.8284</v>
+        <v>111.7202</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>169896.3031556</v>
+        <v>169731.9193318</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-103.696844399994</v>
+        <v>-268.080668199982</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.0006099814376470235</v>
+        <v>-0.001576945107058718</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -16601,6 +16709,9 @@
       </c>
       <c r="DY21" s="3" t="n">
         <v>111.8284</v>
+      </c>
+      <c r="DZ21" s="3" t="n">
+        <v>111.7202</v>
       </c>
     </row>
     <row r="22">
@@ -16626,16 +16737,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>41.783</v>
+        <v>41.551</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>64114.34218000001</v>
+        <v>63758.34746</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>4114.342180000007</v>
+        <v>3758.347460000005</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.06857236966666679</v>
+        <v>0.06263912433333341</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -16990,6 +17101,9 @@
       </c>
       <c r="DY22" s="3" t="n">
         <v>41.783</v>
+      </c>
+      <c r="DZ22" s="3" t="n">
+        <v>41.551</v>
       </c>
     </row>
     <row r="23">
@@ -17015,16 +17129,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.149</v>
+        <v>61.0749</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>166109.240583</v>
+        <v>165907.9503783</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>16109.24058300001</v>
+        <v>15907.95037830001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.10739493722</v>
+        <v>0.1060530025220001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -17385,6 +17499,9 @@
       </c>
       <c r="DY23" s="3" t="n">
         <v>61.149</v>
+      </c>
+      <c r="DZ23" s="3" t="n">
+        <v>61.0749</v>
       </c>
     </row>
     <row r="24">
@@ -17410,16 +17527,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.8095</v>
+        <v>25.8735</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>93775.875967</v>
+        <v>94008.412671</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-6224.124033</v>
+        <v>-5991.587329000002</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.06224124033</v>
+        <v>-0.05991587329000002</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -17774,6 +17891,9 @@
       </c>
       <c r="DY24" s="3" t="n">
         <v>25.8095</v>
+      </c>
+      <c r="DZ24" s="3" t="n">
+        <v>25.8735</v>
       </c>
     </row>
     <row r="25">
@@ -17799,16 +17919,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.7551</v>
+        <v>12.6752</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>209460.0940374</v>
+        <v>208148.0022848</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>9460.094037400006</v>
+        <v>8148.002284799994</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.04730047018700003</v>
+        <v>0.04074001142399997</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -18166,6 +18286,9 @@
       </c>
       <c r="DY25" s="3" t="n">
         <v>12.7551</v>
+      </c>
+      <c r="DZ25" s="3" t="n">
+        <v>12.6752</v>
       </c>
     </row>
     <row r="26">
@@ -18191,16 +18314,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.1636</v>
+        <v>11.1993</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>133312.529574</v>
+        <v>133738.8487995</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>23312.52957400001</v>
+        <v>23738.8487995</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.2119320870363638</v>
+        <v>0.2158077163590909</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -18558,6 +18681,9 @@
       </c>
       <c r="DY26" s="3" t="n">
         <v>11.1636</v>
+      </c>
+      <c r="DZ26" s="3" t="n">
+        <v>11.1993</v>
       </c>
     </row>
     <row r="27">
@@ -18583,16 +18709,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>69.9344</v>
+        <v>69.4941</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>112654.527584</v>
+        <v>111945.265926</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>2654.527583999981</v>
+        <v>1945.265925999993</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.02413206894545437</v>
+        <v>0.01768423569090902</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -18953,6 +19079,9 @@
       </c>
       <c r="DY27" s="3" t="n">
         <v>69.9344</v>
+      </c>
+      <c r="DZ27" s="3" t="n">
+        <v>69.4941</v>
       </c>
     </row>
     <row r="28">
@@ -18978,16 +19107,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>116.6107</v>
+        <v>115.7297</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>385591.5874299</v>
+        <v>382678.4226129</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>5591.587429900013</v>
+        <v>2678.422612899973</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.01471470376289477</v>
+        <v>0.007048480560263086</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -19348,6 +19477,9 @@
       </c>
       <c r="DY28" s="3" t="n">
         <v>116.6107</v>
+      </c>
+      <c r="DZ28" s="3" t="n">
+        <v>115.7297</v>
       </c>
     </row>
     <row r="29">
@@ -19373,16 +19505,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.1132</v>
+        <v>12.1702</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>116331.5751796</v>
+        <v>116878.9862506</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>16331.5751796</v>
+        <v>16878.98625059999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.163315751796</v>
+        <v>0.1687898625059999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -19737,6 +19869,9 @@
       </c>
       <c r="DY29" s="3" t="n">
         <v>12.1132</v>
+      </c>
+      <c r="DZ29" s="3" t="n">
+        <v>12.1702</v>
       </c>
     </row>
     <row r="30">
@@ -19762,16 +19897,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.3778</v>
+        <v>17.4109</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>128523.7932858</v>
+        <v>128768.5962849</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>28523.7932858</v>
+        <v>28768.59628490001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.285237932858</v>
+        <v>0.2876859628490001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -20126,6 +20261,9 @@
       </c>
       <c r="DY30" s="3" t="n">
         <v>17.3778</v>
+      </c>
+      <c r="DZ30" s="3" t="n">
+        <v>17.4109</v>
       </c>
     </row>
     <row r="31">
@@ -20151,16 +20289,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>399.3015</v>
+        <v>400.4653</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>106246.14312</v>
+        <v>106555.807024</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>6246.143119999993</v>
+        <v>6555.807023999994</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.06246143119999993</v>
+        <v>0.06555807023999995</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -20518,6 +20656,9 @@
       </c>
       <c r="DY31" s="3" t="n">
         <v>399.3015</v>
+      </c>
+      <c r="DZ31" s="3" t="n">
+        <v>400.4653</v>
       </c>
     </row>
     <row r="32">
@@ -20543,16 +20684,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.68</v>
+        <v>10.64</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>225774.7728</v>
+        <v>224929.1744</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>25774.77279999998</v>
+        <v>24929.17439999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1288738639999999</v>
+        <v>0.1246458719999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -20913,6 +21054,9 @@
       </c>
       <c r="DY32" s="3" t="n">
         <v>10.68</v>
+      </c>
+      <c r="DZ32" s="3" t="n">
+        <v>10.64</v>
       </c>
     </row>
     <row r="33">
@@ -20938,16 +21082,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.61</v>
+        <v>19.55</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>70275.1804</v>
+        <v>70060.162</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>10275.1804</v>
+        <v>10060.162</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1712530066666666</v>
+        <v>0.1676693666666666</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -21302,6 +21446,9 @@
       </c>
       <c r="DY33" s="3" t="n">
         <v>19.61</v>
+      </c>
+      <c r="DZ33" s="3" t="n">
+        <v>19.55</v>
       </c>
     </row>
     <row r="34">
@@ -21327,16 +21474,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>228.6134</v>
+        <v>229.2419</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>80364.69711540001</v>
+        <v>80585.6343489</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>364.6971154000057</v>
+        <v>585.6343488999992</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.004558713942500072</v>
+        <v>0.00732042936124999</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -21694,6 +21841,9 @@
       </c>
       <c r="DY34" s="3" t="n">
         <v>228.6134</v>
+      </c>
+      <c r="DZ34" s="3" t="n">
+        <v>229.2419</v>
       </c>
     </row>
     <row r="35">
@@ -21719,16 +21869,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.27</v>
+        <v>16.2</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>116093.33221</v>
+        <v>115593.8526</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>16093.33220999999</v>
+        <v>15593.8526</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1609333220999999</v>
+        <v>0.155938526</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -22086,6 +22236,9 @@
       </c>
       <c r="DY35" s="3" t="n">
         <v>16.27</v>
+      </c>
+      <c r="DZ35" s="3" t="n">
+        <v>16.2</v>
       </c>
     </row>
     <row r="36">
@@ -22111,16 +22264,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>369.2882</v>
+        <v>366.3425</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>171979.7304692</v>
+        <v>170607.900305</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>21979.7304692</v>
+        <v>20607.90030499999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1465315364613334</v>
+        <v>0.1373860020333333</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -22478,6 +22631,9 @@
       </c>
       <c r="DY36" s="3" t="n">
         <v>369.2882</v>
+      </c>
+      <c r="DZ36" s="3" t="n">
+        <v>366.3425</v>
       </c>
     </row>
     <row r="37">
@@ -22503,16 +22659,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.894</v>
+        <v>16.722</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>63570.246766</v>
+        <v>62923.02985800001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>13570.246766</v>
+        <v>12923.02985800001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2714049353199999</v>
+        <v>0.2584605971600002</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -22870,6 +23026,9 @@
       </c>
       <c r="DY37" s="3" t="n">
         <v>16.894</v>
+      </c>
+      <c r="DZ37" s="3" t="n">
+        <v>16.722</v>
       </c>
     </row>
     <row r="38">
@@ -22895,16 +23054,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.6672</v>
+        <v>13.6425</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>81736.4435904</v>
+        <v>81588.725685</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1736.443590399998</v>
+        <v>1588.725684999998</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.02170554487999998</v>
+        <v>0.01985907106249997</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -23259,6 +23418,9 @@
       </c>
       <c r="DY38" s="3" t="n">
         <v>13.6672</v>
+      </c>
+      <c r="DZ38" s="3" t="n">
+        <v>13.6425</v>
       </c>
     </row>
     <row r="39">
@@ -23284,16 +23446,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1026.4001</v>
+        <v>1025.1425</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51197.86338810001</v>
+        <v>51135.1330425</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1197.863388100006</v>
+        <v>1135.133042499998</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02395726776200012</v>
+        <v>0.02270266084999996</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -23648,6 +23810,9 @@
       </c>
       <c r="DY39" s="3" t="n">
         <v>1026.4001</v>
+      </c>
+      <c r="DZ39" s="3" t="n">
+        <v>1025.1425</v>
       </c>
     </row>
     <row r="40">
@@ -23673,16 +23838,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.88</v>
+        <v>20.7251</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>105256.64376</v>
+        <v>104475.7886777</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>5256.643759999992</v>
+        <v>4475.788677700009</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.05256643759999992</v>
+        <v>0.04475788677700009</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -24040,6 +24205,9 @@
       </c>
       <c r="DY40" s="3" t="n">
         <v>20.88</v>
+      </c>
+      <c r="DZ40" s="3" t="n">
+        <v>20.7251</v>
       </c>
     </row>
     <row r="41">
@@ -24052,13 +24220,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5003786.9415251</v>
+        <v>4983781.1649683</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>533786.9415251</v>
+        <v>513781.1649683</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1194154231599776</v>
+        <v>0.1149398579347427</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-16
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-15 06:55 IST</t>
+          <t>Generated: 2026-10-16 06:42 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4983781.1649683</v>
+        <v>4939033.6657246</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>513781.1649682997</v>
+        <v>469033.6657245997</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1149398579347427</v>
+        <v>0.104929231705727</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>530049.4978981018</v>
+        <v>532062.4985771179</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-60732.52210189821</v>
+        <v>-58719.5214228821</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1028002208020789</v>
+        <v>-0.09939287154149021</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5513830.662866401</v>
+        <v>5471096.164301718</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>453048.6428664019</v>
+        <v>410314.1443017181</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08952146942428514</v>
+        <v>0.08107722140178607</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-15</t>
+          <t>Last snapshot: 2026-10-16</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FD19"/>
+  <dimension ref="A1:FE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -779,6 +779,7 @@
     <col width="21" customWidth="1" min="158" max="158"/>
     <col width="21" customWidth="1" min="159" max="159"/>
     <col width="21" customWidth="1" min="160" max="160"/>
+    <col width="21" customWidth="1" min="161" max="161"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1582,6 +1583,11 @@
           <t>2026-10-15</t>
         </is>
       </c>
+      <c r="FE1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1601,13 +1607,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>567.8499755859375</v>
+        <v>566.2000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45427.998046875</v>
+        <v>45296.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1610.488046874998</v>
+        <v>1478.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2064,6 +2070,9 @@
       </c>
       <c r="FD2" s="3" t="n">
         <v>567.8499755859375</v>
+      </c>
+      <c r="FE2" s="3" t="n">
+        <v>566.2000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -2111,13 +2120,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1452.800048828125</v>
+        <v>1435.900024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>29056.0009765625</v>
+        <v>28718.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3048.579023437502</v>
+        <v>-3386.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2577,6 +2586,9 @@
       </c>
       <c r="FD4" s="3" t="n">
         <v>1452.800048828125</v>
+      </c>
+      <c r="FE4" s="3" t="n">
+        <v>1435.900024414062</v>
       </c>
     </row>
     <row r="5">
@@ -2597,13 +2609,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>469.6000061035156</v>
+        <v>468.25</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9392.000122070312</v>
+        <v>9365</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4821.099877929688</v>
+        <v>-4848.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3063,6 +3075,9 @@
       </c>
       <c r="FD5" s="3" t="n">
         <v>469.6000061035156</v>
+      </c>
+      <c r="FE5" s="3" t="n">
+        <v>468.25</v>
       </c>
     </row>
     <row r="6">
@@ -3083,13 +3098,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>363.8999938964844</v>
+        <v>374.5499877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14555.99975585938</v>
+        <v>14981.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2946.240244140627</v>
+        <v>-2520.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3549,6 +3564,9 @@
       </c>
       <c r="FD6" s="3" t="n">
         <v>363.8999938964844</v>
+      </c>
+      <c r="FE6" s="3" t="n">
+        <v>374.5499877929688</v>
       </c>
     </row>
     <row r="7">
@@ -3569,13 +3587,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>280</v>
+        <v>276.3500061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>28000</v>
+        <v>27635.00061035156</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1566.18</v>
+        <v>1201.180610351563</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4035,6 +4053,9 @@
       </c>
       <c r="FD7" s="3" t="n">
         <v>280</v>
+      </c>
+      <c r="FE7" s="3" t="n">
+        <v>276.3500061035156</v>
       </c>
     </row>
     <row r="8">
@@ -4082,13 +4103,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>15.35999965667725</v>
+        <v>14.9399995803833</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>23039.99948501587</v>
+        <v>22409.99937057495</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8010.170514984129</v>
+        <v>-8640.170629425047</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4548,6 +4569,9 @@
       </c>
       <c r="FD9" s="3" t="n">
         <v>15.35999965667725</v>
+      </c>
+      <c r="FE9" s="3" t="n">
+        <v>14.9399995803833</v>
       </c>
     </row>
     <row r="10">
@@ -4568,13 +4592,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>447.3500061035156</v>
+        <v>447</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44735.00061035156</v>
+        <v>44700</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6763.479389648441</v>
+        <v>-6798.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5034,6 +5058,9 @@
       </c>
       <c r="FD10" s="3" t="n">
         <v>447.3500061035156</v>
+      </c>
+      <c r="FE10" s="3" t="n">
+        <v>447</v>
       </c>
     </row>
     <row r="11">
@@ -5054,13 +5081,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>14.40999984741211</v>
+        <v>16.79999923706055</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14409.99984741211</v>
+        <v>16799.99923706055</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4568.78984741211</v>
+        <v>6958.789237060548</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5520,6 +5547,9 @@
       </c>
       <c r="FD11" s="3" t="n">
         <v>14.40999984741211</v>
+      </c>
+      <c r="FE11" s="3" t="n">
+        <v>16.79999923706055</v>
       </c>
     </row>
     <row r="12">
@@ -5540,13 +5570,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2564.5</v>
+        <v>2514</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25645</v>
+        <v>25140</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2078.25</v>
+        <v>-2583.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6006,6 +6036,9 @@
       </c>
       <c r="FD12" s="3" t="n">
         <v>2564.5</v>
+      </c>
+      <c r="FE12" s="3" t="n">
+        <v>2514</v>
       </c>
     </row>
     <row r="13">
@@ -6026,13 +6059,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>41.11999893188477</v>
+        <v>41.0099983215332</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>24671.99935913086</v>
+        <v>24605.99899291992</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-10359.76064086914</v>
+        <v>-10425.76100708008</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6492,6 +6525,9 @@
       </c>
       <c r="FD13" s="3" t="n">
         <v>41.11999893188477</v>
+      </c>
+      <c r="FE13" s="3" t="n">
+        <v>41.0099983215332</v>
       </c>
     </row>
     <row r="14">
@@ -6512,13 +6548,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>627</v>
+        <v>630.5499877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31350</v>
+        <v>31527.49938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11112.51</v>
+        <v>-10935.01061035156</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -6978,6 +7014,9 @@
       </c>
       <c r="FD14" s="3" t="n">
         <v>627</v>
+      </c>
+      <c r="FE14" s="3" t="n">
+        <v>630.5499877929688</v>
       </c>
     </row>
     <row r="15">
@@ -7052,13 +7091,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>460.1000061035156</v>
+        <v>476.25</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23005.00030517578</v>
+        <v>23812.5</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1250.470305175782</v>
+        <v>2057.970000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7518,6 +7557,9 @@
       </c>
       <c r="FD17" s="3" t="n">
         <v>460.1000061035156</v>
+      </c>
+      <c r="FE17" s="3" t="n">
+        <v>476.25</v>
       </c>
     </row>
     <row r="18">
@@ -7538,13 +7580,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>349.8999938964844</v>
+        <v>353</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34989.99938964844</v>
+        <v>35300</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11650.82061035156</v>
+        <v>-11340.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8004,6 +8046,9 @@
       </c>
       <c r="FD18" s="3" t="n">
         <v>349.8999938964844</v>
+      </c>
+      <c r="FE18" s="3" t="n">
+        <v>353</v>
       </c>
     </row>
     <row r="19">
@@ -8016,10 +8061,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>530049.4978981018</v>
+        <v>532062.4985771179</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-60732.5221018982</v>
+        <v>-58719.52142288209</v>
       </c>
     </row>
   </sheetData>
@@ -8033,7 +8078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DZ41"/>
+  <dimension ref="A1:EA41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8043,8 +8088,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -8166,6 +8211,7 @@
     <col width="13" customWidth="1" min="128" max="128"/>
     <col width="13" customWidth="1" min="129" max="129"/>
     <col width="13" customWidth="1" min="130" max="130"/>
+    <col width="13" customWidth="1" min="131" max="131"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8819,6 +8865,11 @@
           <t>2026-10-15</t>
         </is>
       </c>
+      <c r="EA1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8843,16 +8894,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.7451</v>
+        <v>56.793</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63695.3533382</v>
+        <v>63749.120226</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13695.3533382</v>
+        <v>13749.120226</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2739070667640001</v>
+        <v>0.27498240452</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9216,6 +9267,9 @@
       </c>
       <c r="DZ2" s="3" t="n">
         <v>56.7451</v>
+      </c>
+      <c r="EA2" s="3" t="n">
+        <v>56.793</v>
       </c>
     </row>
     <row r="3">
@@ -9241,16 +9295,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.6112</v>
+        <v>26.4287</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65336.16418560001</v>
+        <v>64888.08781310001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5336.164185600006</v>
+        <v>4888.087813100006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.0889360697600001</v>
+        <v>0.08146813021833343</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9608,6 +9662,9 @@
       </c>
       <c r="DZ3" s="3" t="n">
         <v>26.6112</v>
+      </c>
+      <c r="EA3" s="3" t="n">
+        <v>26.4287</v>
       </c>
     </row>
     <row r="4">
@@ -9633,16 +9690,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.37</v>
+        <v>12.02</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>237579.37041</v>
+        <v>230857.23786</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>57579.37041</v>
+        <v>50857.23785999999</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3198853911666667</v>
+        <v>0.2825402103333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -10000,6 +10057,9 @@
       </c>
       <c r="DZ4" s="3" t="n">
         <v>12.37</v>
+      </c>
+      <c r="EA4" s="3" t="n">
+        <v>12.02</v>
       </c>
     </row>
     <row r="5">
@@ -10025,16 +10085,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.233000000000001</v>
+        <v>9.214399999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>169463.294504</v>
+        <v>169121.9084672</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-40536.70549599998</v>
+        <v>-40878.09153280003</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1930319309333332</v>
+        <v>-0.1946575787276192</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10392,6 +10452,9 @@
       </c>
       <c r="DZ5" s="3" t="n">
         <v>9.233000000000001</v>
+      </c>
+      <c r="EA5" s="3" t="n">
+        <v>9.214399999999999</v>
       </c>
     </row>
     <row r="6">
@@ -10417,16 +10480,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.2744</v>
+        <v>11.1733</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>47679.1782888</v>
+        <v>47251.62871409999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-2320.821711199998</v>
+        <v>-2748.371285900008</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.04641643422399997</v>
+        <v>-0.05496742571800016</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -10790,6 +10853,9 @@
       </c>
       <c r="DZ6" s="3" t="n">
         <v>11.2744</v>
+      </c>
+      <c r="EA6" s="3" t="n">
+        <v>11.1733</v>
       </c>
     </row>
     <row r="7">
@@ -10815,16 +10881,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.5161</v>
+        <v>33.2567</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73937.857244</v>
+        <v>73365.610468</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13937.857244</v>
+        <v>13365.610468</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2322976207333333</v>
+        <v>0.2227601744666667</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -11182,6 +11248,9 @@
       </c>
       <c r="DZ7" s="3" t="n">
         <v>33.5161</v>
+      </c>
+      <c r="EA7" s="3" t="n">
+        <v>33.2567</v>
       </c>
     </row>
     <row r="8">
@@ -11207,16 +11276,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.7205</v>
+        <v>34.9524</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57316.8642565</v>
+        <v>56084.3763732</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7316.864256500005</v>
+        <v>6084.376373200001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.1463372851300001</v>
+        <v>0.121687527464</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -11580,6 +11649,9 @@
       </c>
       <c r="DZ8" s="3" t="n">
         <v>35.7205</v>
+      </c>
+      <c r="EA8" s="3" t="n">
+        <v>34.9524</v>
       </c>
     </row>
     <row r="9">
@@ -11605,16 +11677,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.2063</v>
+        <v>39.4148</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>132659.2737759</v>
+        <v>126891.7312164</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>32659.27377589999</v>
+        <v>26891.7312164</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3265927377589999</v>
+        <v>0.2689173121640001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -11972,6 +12044,9 @@
       </c>
       <c r="DZ9" s="3" t="n">
         <v>41.2063</v>
+      </c>
+      <c r="EA9" s="3" t="n">
+        <v>39.4148</v>
       </c>
     </row>
     <row r="10">
@@ -11997,16 +12072,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.3515</v>
+        <v>48.6546</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>137640.2326385</v>
+        <v>138503.0549814</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>37640.23263850002</v>
+        <v>38503.0549814</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3764023263850002</v>
+        <v>0.385030549814</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -12364,6 +12439,9 @@
       </c>
       <c r="DZ10" s="3" t="n">
         <v>48.3515</v>
+      </c>
+      <c r="EA10" s="3" t="n">
+        <v>48.6546</v>
       </c>
     </row>
     <row r="11">
@@ -12389,16 +12467,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.9217</v>
+        <v>104.5643</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31572.9330423</v>
+        <v>31465.3845917</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1572.933042299999</v>
+        <v>1465.3845917</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.05243110140999997</v>
+        <v>0.04884615305666666</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -12756,6 +12834,9 @@
       </c>
       <c r="DZ11" s="3" t="n">
         <v>104.9217</v>
+      </c>
+      <c r="EA11" s="3" t="n">
+        <v>104.5643</v>
       </c>
     </row>
     <row r="12">
@@ -12781,16 +12862,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.903</v>
+        <v>221.574</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102835.206366</v>
+        <v>103147.571628</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2835.206365999999</v>
+        <v>3147.571628000005</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02835206365999999</v>
+        <v>0.03147571628000005</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -13154,6 +13235,9 @@
       </c>
       <c r="DZ12" s="3" t="n">
         <v>220.903</v>
+      </c>
+      <c r="EA12" s="3" t="n">
+        <v>221.574</v>
       </c>
     </row>
     <row r="13">
@@ -13179,16 +13263,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.275</v>
+        <v>21.224</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>246526.296375</v>
+        <v>245935.32852</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>46526.29637499998</v>
+        <v>45935.32851999998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2326314818749999</v>
+        <v>0.2296766425999999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -13552,6 +13636,9 @@
       </c>
       <c r="DZ13" s="3" t="n">
         <v>21.275</v>
+      </c>
+      <c r="EA13" s="3" t="n">
+        <v>21.224</v>
       </c>
     </row>
     <row r="14">
@@ -13577,16 +13664,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36.4753</v>
+        <v>35.4841</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>131588.5111318</v>
+        <v>128012.6520646</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>31588.51113179998</v>
+        <v>28012.6520646</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3158851113179998</v>
+        <v>0.280126520646</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -13944,6 +14031,9 @@
       </c>
       <c r="DZ14" s="3" t="n">
         <v>36.4753</v>
+      </c>
+      <c r="EA14" s="3" t="n">
+        <v>35.4841</v>
       </c>
     </row>
     <row r="15">
@@ -13969,16 +14059,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.42</v>
+        <v>11.3</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>111275.87474</v>
+        <v>110106.6011</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>11275.87474</v>
+        <v>10106.60110000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1127587474</v>
+        <v>0.1010660110000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -14342,6 +14432,9 @@
       </c>
       <c r="DZ15" s="3" t="n">
         <v>11.42</v>
+      </c>
+      <c r="EA15" s="3" t="n">
+        <v>11.3</v>
       </c>
     </row>
     <row r="16">
@@ -14367,16 +14460,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.7424</v>
+        <v>24.7391</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>141598.9737472</v>
+        <v>141580.0880848</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>41598.97374719998</v>
+        <v>41580.08808479999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4159897374719999</v>
+        <v>0.4158008808479999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -14734,6 +14827,9 @@
       </c>
       <c r="DZ16" s="3" t="n">
         <v>24.7424</v>
+      </c>
+      <c r="EA16" s="3" t="n">
+        <v>24.7391</v>
       </c>
     </row>
     <row r="17">
@@ -14759,16 +14855,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.686</v>
+        <v>16.7782</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55164.867102</v>
+        <v>55469.68555739999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5164.867101999997</v>
+        <v>5469.685557399993</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1032973420399999</v>
+        <v>0.1093937111479999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -15126,6 +15222,9 @@
       </c>
       <c r="DZ17" s="3" t="n">
         <v>16.686</v>
+      </c>
+      <c r="EA17" s="3" t="n">
+        <v>16.7782</v>
       </c>
     </row>
     <row r="18">
@@ -15151,16 +15250,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.88</v>
+        <v>44.92</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84663.24768</v>
+        <v>84738.70512</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4663.24768</v>
+        <v>4738.705119999999</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.05829059600000001</v>
+        <v>0.05923381399999998</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -15524,6 +15623,9 @@
       </c>
       <c r="DZ18" s="3" t="n">
         <v>44.88</v>
+      </c>
+      <c r="EA18" s="3" t="n">
+        <v>44.92</v>
       </c>
     </row>
     <row r="19">
@@ -15549,16 +15651,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>12.8126</v>
+        <v>11.8753</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>185356.8860516</v>
+        <v>171797.1862798</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>35356.88605159998</v>
+        <v>21797.18627979999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2357125736773332</v>
+        <v>0.1453145751986666</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -15916,6 +16018,9 @@
       </c>
       <c r="DZ19" s="3" t="n">
         <v>12.8126</v>
+      </c>
+      <c r="EA19" s="3" t="n">
+        <v>11.8753</v>
       </c>
     </row>
     <row r="20">
@@ -15941,16 +16046,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.05</v>
+        <v>10.09</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>263870.82015</v>
+        <v>264921.05227</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>13870.82015000004</v>
+        <v>14921.05226999999</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.05548328060000017</v>
+        <v>0.05968420907999994</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -16314,6 +16419,9 @@
       </c>
       <c r="DZ20" s="3" t="n">
         <v>10.05</v>
+      </c>
+      <c r="EA20" s="3" t="n">
+        <v>10.09</v>
       </c>
     </row>
     <row r="21">
@@ -16339,16 +16447,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.7202</v>
+        <v>111.4945</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>169731.9193318</v>
+        <v>169389.0225755</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-268.080668199982</v>
+        <v>-610.9774244999862</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.001576945107058718</v>
+        <v>-0.003593984849999919</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -16712,6 +16820,9 @@
       </c>
       <c r="DZ21" s="3" t="n">
         <v>111.7202</v>
+      </c>
+      <c r="EA21" s="3" t="n">
+        <v>111.4945</v>
       </c>
     </row>
     <row r="22">
@@ -16737,16 +16848,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>41.551</v>
+        <v>40.316</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>63758.34746</v>
+        <v>61863.28936</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>3758.347460000005</v>
+        <v>1863.289360000002</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.06263912433333341</v>
+        <v>0.03105482266666671</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -17104,6 +17215,9 @@
       </c>
       <c r="DZ22" s="3" t="n">
         <v>41.551</v>
+      </c>
+      <c r="EA22" s="3" t="n">
+        <v>40.316</v>
       </c>
     </row>
     <row r="23">
@@ -17129,16 +17243,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.0749</v>
+        <v>60.84</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>165907.9503783</v>
+        <v>165269.85228</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>15907.95037830001</v>
+        <v>15269.85228000002</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1060530025220001</v>
+        <v>0.1017990152000001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -17502,6 +17616,9 @@
       </c>
       <c r="DZ23" s="3" t="n">
         <v>61.0749</v>
+      </c>
+      <c r="EA23" s="3" t="n">
+        <v>60.84</v>
       </c>
     </row>
     <row r="24">
@@ -17527,16 +17644,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.8735</v>
+        <v>25.8919</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>94008.412671</v>
+        <v>94075.26697339999</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-5991.587329000002</v>
+        <v>-5924.733026600006</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.05991587329000002</v>
+        <v>-0.05924733026600006</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -17894,6 +18011,9 @@
       </c>
       <c r="DZ24" s="3" t="n">
         <v>25.8735</v>
+      </c>
+      <c r="EA24" s="3" t="n">
+        <v>25.8919</v>
       </c>
     </row>
     <row r="25">
@@ -17919,16 +18039,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.6752</v>
+        <v>12.581</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>208148.0022848</v>
+        <v>206601.080594</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>8148.002284799994</v>
+        <v>6601.08059399997</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.04074001142399997</v>
+        <v>0.03300540296999985</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -18289,6 +18409,9 @@
       </c>
       <c r="DZ25" s="3" t="n">
         <v>12.6752</v>
+      </c>
+      <c r="EA25" s="3" t="n">
+        <v>12.581</v>
       </c>
     </row>
     <row r="26">
@@ -18314,16 +18437,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.1993</v>
+        <v>11.1228</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>133738.8487995</v>
+        <v>132825.307602</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>23738.8487995</v>
+        <v>22825.30760199999</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.2158077163590909</v>
+        <v>0.2075027963818181</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -18684,6 +18807,9 @@
       </c>
       <c r="DZ26" s="3" t="n">
         <v>11.1993</v>
+      </c>
+      <c r="EA26" s="3" t="n">
+        <v>11.1228</v>
       </c>
     </row>
     <row r="27">
@@ -18709,16 +18835,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>69.4941</v>
+        <v>68.7634</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>111945.265926</v>
+        <v>110768.210524</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>1945.265925999993</v>
+        <v>768.2105239999946</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.01768423569090902</v>
+        <v>0.006983732036363588</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -19082,6 +19208,9 @@
       </c>
       <c r="DZ27" s="3" t="n">
         <v>69.4941</v>
+      </c>
+      <c r="EA27" s="3" t="n">
+        <v>68.7634</v>
       </c>
     </row>
     <row r="28">
@@ -19107,16 +19236,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>115.7297</v>
+        <v>115.6012</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>382678.4226129</v>
+        <v>382253.5171884</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>2678.422612899973</v>
+        <v>2253.51718840003</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.007048480560263086</v>
+        <v>0.005930308390526395</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -19480,6 +19609,9 @@
       </c>
       <c r="DZ28" s="3" t="n">
         <v>115.7297</v>
+      </c>
+      <c r="EA28" s="3" t="n">
+        <v>115.6012</v>
       </c>
     </row>
     <row r="29">
@@ -19505,16 +19637,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.1702</v>
+        <v>12.0418</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>116878.9862506</v>
+        <v>115645.8707854</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>16878.98625059999</v>
+        <v>15645.87078539999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1687898625059999</v>
+        <v>0.156458707854</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -19872,6 +20004,9 @@
       </c>
       <c r="DZ29" s="3" t="n">
         <v>12.1702</v>
+      </c>
+      <c r="EA29" s="3" t="n">
+        <v>12.0418</v>
       </c>
     </row>
     <row r="30">
@@ -19897,16 +20032,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.4109</v>
+        <v>17.2457</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>128768.5962849</v>
+        <v>127546.8000477</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>28768.59628490001</v>
+        <v>27546.80004769999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2876859628490001</v>
+        <v>0.2754680004769999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -20264,6 +20399,9 @@
       </c>
       <c r="DZ30" s="3" t="n">
         <v>17.4109</v>
+      </c>
+      <c r="EA30" s="3" t="n">
+        <v>17.2457</v>
       </c>
     </row>
     <row r="31">
@@ -20289,16 +20427,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>400.4653</v>
+        <v>396.7333</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>106555.807024</v>
+        <v>105562.796464</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>6555.807023999994</v>
+        <v>5562.796463999985</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.06555807023999995</v>
+        <v>0.05562796463999985</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -20659,6 +20797,9 @@
       </c>
       <c r="DZ31" s="3" t="n">
         <v>400.4653</v>
+      </c>
+      <c r="EA31" s="3" t="n">
+        <v>396.7333</v>
       </c>
     </row>
     <row r="32">
@@ -20684,16 +20825,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.64</v>
+        <v>10.63</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>224929.1744</v>
+        <v>224717.7748</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>24929.17439999999</v>
+        <v>24717.77480000001</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1246458719999999</v>
+        <v>0.1235888740000001</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -21057,6 +21198,9 @@
       </c>
       <c r="DZ32" s="3" t="n">
         <v>10.64</v>
+      </c>
+      <c r="EA32" s="3" t="n">
+        <v>10.63</v>
       </c>
     </row>
     <row r="33">
@@ -21082,16 +21226,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.55</v>
+        <v>19.36</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>70060.162</v>
+        <v>69379.27039999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>10060.162</v>
+        <v>9379.270399999994</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1676693666666666</v>
+        <v>0.1563211733333332</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -21449,6 +21593,9 @@
       </c>
       <c r="DZ33" s="3" t="n">
         <v>19.55</v>
+      </c>
+      <c r="EA33" s="3" t="n">
+        <v>19.36</v>
       </c>
     </row>
     <row r="34">
@@ -21474,16 +21621,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>229.2419</v>
+        <v>232.5041</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>80585.6343489</v>
+        <v>81732.3987771</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>585.6343488999992</v>
+        <v>1732.398777099996</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.00732042936124999</v>
+        <v>0.02165498471374995</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -21844,6 +21991,9 @@
       </c>
       <c r="DZ34" s="3" t="n">
         <v>229.2419</v>
+      </c>
+      <c r="EA34" s="3" t="n">
+        <v>232.5041</v>
       </c>
     </row>
     <row r="35">
@@ -21869,16 +22019,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>16.2</v>
+        <v>15.82</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>115593.8526</v>
+        <v>112882.39186</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>15593.8526</v>
+        <v>12882.39186</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.155938526</v>
+        <v>0.1288239186</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -22239,6 +22389,9 @@
       </c>
       <c r="DZ35" s="3" t="n">
         <v>16.2</v>
+      </c>
+      <c r="EA35" s="3" t="n">
+        <v>15.82</v>
       </c>
     </row>
     <row r="36">
@@ -22264,16 +22417,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>366.3425</v>
+        <v>365.9877</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>170607.900305</v>
+        <v>170442.6678162</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>20607.90030499999</v>
+        <v>20442.6678162</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1373860020333333</v>
+        <v>0.136284452108</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -22634,6 +22787,9 @@
       </c>
       <c r="DZ36" s="3" t="n">
         <v>366.3425</v>
+      </c>
+      <c r="EA36" s="3" t="n">
+        <v>365.9877</v>
       </c>
     </row>
     <row r="37">
@@ -22659,16 +22815,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.722</v>
+        <v>16.675</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62923.02985800001</v>
+        <v>62746.174075</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12923.02985800001</v>
+        <v>12746.174075</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2584605971600002</v>
+        <v>0.2549234815</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -23029,6 +23185,9 @@
       </c>
       <c r="DZ37" s="3" t="n">
         <v>16.722</v>
+      </c>
+      <c r="EA37" s="3" t="n">
+        <v>16.675</v>
       </c>
     </row>
     <row r="38">
@@ -23054,16 +23213,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.6425</v>
+        <v>13.7084</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>81588.725685</v>
+        <v>81982.83944879999</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1588.725684999998</v>
+        <v>1982.83944879999</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.01985907106249997</v>
+        <v>0.02478549310999988</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -23421,6 +23580,9 @@
       </c>
       <c r="DZ38" s="3" t="n">
         <v>13.6425</v>
+      </c>
+      <c r="EA38" s="3" t="n">
+        <v>13.7084</v>
       </c>
     </row>
     <row r="39">
@@ -23446,16 +23608,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.1425</v>
+        <v>1024.6051</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51135.1330425</v>
+        <v>51108.3269931</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1135.133042499998</v>
+        <v>1108.326993100003</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02270266084999996</v>
+        <v>0.02216653986200006</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -23813,6 +23975,9 @@
       </c>
       <c r="DZ39" s="3" t="n">
         <v>1025.1425</v>
+      </c>
+      <c r="EA39" s="3" t="n">
+        <v>1024.6051</v>
       </c>
     </row>
     <row r="40">
@@ -23838,16 +24003,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.7251</v>
+        <v>20.7009</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>104475.7886777</v>
+        <v>104353.7958243</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>4475.788677700009</v>
+        <v>4353.795824300003</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.04475788677700009</v>
+        <v>0.04353795824300003</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -24208,6 +24373,9 @@
       </c>
       <c r="DZ40" s="3" t="n">
         <v>20.7251</v>
+      </c>
+      <c r="EA40" s="3" t="n">
+        <v>20.7009</v>
       </c>
     </row>
     <row r="41">
@@ -24220,13 +24388,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4983781.1649683</v>
+        <v>4939033.6657246</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>513781.1649683</v>
+        <v>469033.6657245999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1149398579347427</v>
+        <v>0.104929231705727</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-17
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-16 06:42 IST</t>
+          <t>Generated: 2026-10-17 06:31 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4939033.6657246</v>
+        <v>4947987.3039979</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>469033.6657245997</v>
+        <v>477987.3039979003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.104929231705727</v>
+        <v>0.1069322827735795</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>532062.4985771179</v>
+        <v>531440.5047492981</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-58719.5214228821</v>
+        <v>-59341.51525070192</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.09939287154149021</v>
+        <v>-0.1004457028849692</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5471096.164301718</v>
+        <v>5479427.808747198</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>410314.1443017181</v>
+        <v>418645.7887471989</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08107722140178607</v>
+        <v>0.08272353701319839</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-16</t>
+          <t>Last snapshot: 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FE19"/>
+  <dimension ref="A1:FF19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -780,6 +780,7 @@
     <col width="21" customWidth="1" min="159" max="159"/>
     <col width="21" customWidth="1" min="160" max="160"/>
     <col width="21" customWidth="1" min="161" max="161"/>
+    <col width="21" customWidth="1" min="162" max="162"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1588,6 +1589,11 @@
           <t>2026-10-16</t>
         </is>
       </c>
+      <c r="FF1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1607,13 +1613,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>566.2000122070312</v>
+        <v>559.7000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45296.0009765625</v>
+        <v>44776.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1478.490976562498</v>
+        <v>958.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2073,6 +2079,9 @@
       </c>
       <c r="FE2" s="3" t="n">
         <v>566.2000122070312</v>
+      </c>
+      <c r="FF2" s="3" t="n">
+        <v>559.7000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -2120,13 +2129,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1435.900024414062</v>
+        <v>1427.400024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28718.00048828125</v>
+        <v>28548.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3386.579511718752</v>
+        <v>-3556.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2589,6 +2598,9 @@
       </c>
       <c r="FE4" s="3" t="n">
         <v>1435.900024414062</v>
+      </c>
+      <c r="FF4" s="3" t="n">
+        <v>1427.400024414062</v>
       </c>
     </row>
     <row r="5">
@@ -2609,13 +2621,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>468.25</v>
+        <v>474.1499938964844</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9365</v>
+        <v>9482.999877929688</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4848.1</v>
+        <v>-4730.100122070313</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3078,6 +3090,9 @@
       </c>
       <c r="FE5" s="3" t="n">
         <v>468.25</v>
+      </c>
+      <c r="FF5" s="3" t="n">
+        <v>474.1499938964844</v>
       </c>
     </row>
     <row r="6">
@@ -3098,13 +3113,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>374.5499877929688</v>
+        <v>376.6000061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14981.99951171875</v>
+        <v>15064.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2520.240488281252</v>
+        <v>-2438.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3567,6 +3582,9 @@
       </c>
       <c r="FE6" s="3" t="n">
         <v>374.5499877929688</v>
+      </c>
+      <c r="FF6" s="3" t="n">
+        <v>376.6000061035156</v>
       </c>
     </row>
     <row r="7">
@@ -3587,13 +3605,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>276.3500061035156</v>
+        <v>273.4500122070312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>27635.00061035156</v>
+        <v>27345.00122070312</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1201.180610351563</v>
+        <v>911.1812207031253</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4056,6 +4074,9 @@
       </c>
       <c r="FE7" s="3" t="n">
         <v>276.3500061035156</v>
+      </c>
+      <c r="FF7" s="3" t="n">
+        <v>273.4500122070312</v>
       </c>
     </row>
     <row r="8">
@@ -4103,13 +4124,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.9399995803833</v>
+        <v>14.97000026702881</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22409.99937057495</v>
+        <v>22455.00040054321</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8640.170629425047</v>
+        <v>-8595.169599456785</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4572,6 +4593,9 @@
       </c>
       <c r="FE9" s="3" t="n">
         <v>14.9399995803833</v>
+      </c>
+      <c r="FF9" s="3" t="n">
+        <v>14.97000026702881</v>
       </c>
     </row>
     <row r="10">
@@ -4592,13 +4616,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44700</v>
+        <v>44500</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6798.480000000003</v>
+        <v>-6998.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5061,6 +5085,9 @@
       </c>
       <c r="FE10" s="3" t="n">
         <v>447</v>
+      </c>
+      <c r="FF10" s="3" t="n">
+        <v>445</v>
       </c>
     </row>
     <row r="11">
@@ -5081,13 +5108,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>16.79999923706055</v>
+        <v>16.28000068664551</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>16799.99923706055</v>
+        <v>16280.00068664551</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>6958.789237060548</v>
+        <v>6438.790686645509</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5550,6 +5577,9 @@
       </c>
       <c r="FE11" s="3" t="n">
         <v>16.79999923706055</v>
+      </c>
+      <c r="FF11" s="3" t="n">
+        <v>16.28000068664551</v>
       </c>
     </row>
     <row r="12">
@@ -5570,13 +5600,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2514</v>
+        <v>2523.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25140</v>
+        <v>25238.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2583.25</v>
+        <v>-2484.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6039,6 +6069,9 @@
       </c>
       <c r="FE12" s="3" t="n">
         <v>2514</v>
+      </c>
+      <c r="FF12" s="3" t="n">
+        <v>2523.89990234375</v>
       </c>
     </row>
     <row r="13">
@@ -6059,13 +6092,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>41.0099983215332</v>
+        <v>42</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>24605.99899291992</v>
+        <v>25200</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-10425.76100708008</v>
+        <v>-9831.760000000002</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6528,6 +6561,9 @@
       </c>
       <c r="FE13" s="3" t="n">
         <v>41.0099983215332</v>
+      </c>
+      <c r="FF13" s="3" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="14">
@@ -6548,13 +6584,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>630.5499877929688</v>
+        <v>633.1500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31527.49938964844</v>
+        <v>31657.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-10935.01061035156</v>
+        <v>-10805.00877929688</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7017,6 +7053,9 @@
       </c>
       <c r="FE14" s="3" t="n">
         <v>630.5499877929688</v>
+      </c>
+      <c r="FF14" s="3" t="n">
+        <v>633.1500244140625</v>
       </c>
     </row>
     <row r="15">
@@ -7091,13 +7130,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>476.25</v>
+        <v>474.75</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23812.5</v>
+        <v>23737.5</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>2057.970000000001</v>
+        <v>1982.970000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7560,6 +7599,9 @@
       </c>
       <c r="FE17" s="3" t="n">
         <v>476.25</v>
+      </c>
+      <c r="FF17" s="3" t="n">
+        <v>474.75</v>
       </c>
     </row>
     <row r="18">
@@ -7580,13 +7622,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>353</v>
+        <v>353.8500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35300</v>
+        <v>35385.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11340.82</v>
+        <v>-11255.81938964844</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8049,6 +8091,9 @@
       </c>
       <c r="FE18" s="3" t="n">
         <v>353</v>
+      </c>
+      <c r="FF18" s="3" t="n">
+        <v>353.8500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -8061,10 +8106,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>532062.4985771179</v>
+        <v>531440.5047492981</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-58719.52142288209</v>
+        <v>-59341.51525070192</v>
       </c>
     </row>
   </sheetData>
@@ -8078,7 +8123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EA41"/>
+  <dimension ref="A1:EB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8088,7 +8133,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
@@ -8212,6 +8257,7 @@
     <col width="13" customWidth="1" min="129" max="129"/>
     <col width="13" customWidth="1" min="130" max="130"/>
     <col width="13" customWidth="1" min="131" max="131"/>
+    <col width="13" customWidth="1" min="132" max="132"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8870,6 +8916,11 @@
           <t>2026-10-16</t>
         </is>
       </c>
+      <c r="EB1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8894,16 +8945,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.793</v>
+        <v>56.2538</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63749.120226</v>
+        <v>63143.8779316</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13749.120226</v>
+        <v>13143.8779316</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.27498240452</v>
+        <v>0.262877558632</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9270,6 +9321,9 @@
       </c>
       <c r="EA2" s="3" t="n">
         <v>56.793</v>
+      </c>
+      <c r="EB2" s="3" t="n">
+        <v>56.2538</v>
       </c>
     </row>
     <row r="3">
@@ -9295,16 +9349,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.4287</v>
+        <v>26.7682</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>64888.08781310001</v>
+        <v>65721.63262660001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4888.087813100006</v>
+        <v>5721.632626600011</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.08146813021833343</v>
+        <v>0.09536054377666685</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9665,6 +9719,9 @@
       </c>
       <c r="EA3" s="3" t="n">
         <v>26.4287</v>
+      </c>
+      <c r="EB3" s="3" t="n">
+        <v>26.7682</v>
       </c>
     </row>
     <row r="4">
@@ -9690,16 +9747,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.02</v>
+        <v>12.08</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>230857.23786</v>
+        <v>232009.60344</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>50857.23785999999</v>
+        <v>52009.60344000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2825402103333333</v>
+        <v>0.2889422413333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -10060,6 +10117,9 @@
       </c>
       <c r="EA4" s="3" t="n">
         <v>12.02</v>
+      </c>
+      <c r="EB4" s="3" t="n">
+        <v>12.08</v>
       </c>
     </row>
     <row r="5">
@@ -10085,16 +10145,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.214399999999999</v>
+        <v>9.2668</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>169121.9084672</v>
+        <v>170083.6626784</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-40878.09153280003</v>
+        <v>-39916.3373216</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1946575787276192</v>
+        <v>-0.1900777967695238</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10455,6 +10515,9 @@
       </c>
       <c r="EA5" s="3" t="n">
         <v>9.214399999999999</v>
+      </c>
+      <c r="EB5" s="3" t="n">
+        <v>9.2668</v>
       </c>
     </row>
     <row r="6">
@@ -10480,16 +10543,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.1733</v>
+        <v>11.1632</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>47251.62871409999</v>
+        <v>47208.91604639999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-2748.371285900008</v>
+        <v>-2791.083953600006</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.05496742571800016</v>
+        <v>-0.05582167907200011</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -10856,6 +10919,9 @@
       </c>
       <c r="EA6" s="3" t="n">
         <v>11.1733</v>
+      </c>
+      <c r="EB6" s="3" t="n">
+        <v>11.1632</v>
       </c>
     </row>
     <row r="7">
@@ -10881,16 +10947,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.2567</v>
+        <v>33.7586</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73365.610468</v>
+        <v>74472.821944</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13365.610468</v>
+        <v>14472.821944</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2227601744666667</v>
+        <v>0.2412136990666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -11251,6 +11317,9 @@
       </c>
       <c r="EA7" s="3" t="n">
         <v>33.2567</v>
+      </c>
+      <c r="EB7" s="3" t="n">
+        <v>33.7586</v>
       </c>
     </row>
     <row r="8">
@@ -11276,16 +11345,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>34.9524</v>
+        <v>35.1128</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>56084.3763732</v>
+        <v>56341.7530904</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6084.376373200001</v>
+        <v>6341.753090400001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.121687527464</v>
+        <v>0.126835061808</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -11652,6 +11721,9 @@
       </c>
       <c r="EA8" s="3" t="n">
         <v>34.9524</v>
+      </c>
+      <c r="EB8" s="3" t="n">
+        <v>35.1128</v>
       </c>
     </row>
     <row r="9">
@@ -11677,16 +11749,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>39.4148</v>
+        <v>39.6566</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>126891.7312164</v>
+        <v>127670.1804438</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>26891.7312164</v>
+        <v>27670.1804438</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.2689173121640001</v>
+        <v>0.276701804438</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -12047,6 +12119,9 @@
       </c>
       <c r="EA9" s="3" t="n">
         <v>39.4148</v>
+      </c>
+      <c r="EB9" s="3" t="n">
+        <v>39.6566</v>
       </c>
     </row>
     <row r="10">
@@ -12072,16 +12147,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.6546</v>
+        <v>49.1177</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138503.0549814</v>
+        <v>139821.3427643</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38503.0549814</v>
+        <v>39821.3427643</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.385030549814</v>
+        <v>0.3982134276430001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -12442,6 +12517,9 @@
       </c>
       <c r="EA10" s="3" t="n">
         <v>48.6546</v>
+      </c>
+      <c r="EB10" s="3" t="n">
+        <v>49.1177</v>
       </c>
     </row>
     <row r="11">
@@ -12467,16 +12545,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.5643</v>
+        <v>102.269</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31465.3845917</v>
+        <v>30774.685211</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1465.3845917</v>
+        <v>774.685211</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04884615305666666</v>
+        <v>0.02582284036666667</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -12837,6 +12915,9 @@
       </c>
       <c r="EA11" s="3" t="n">
         <v>104.5643</v>
+      </c>
+      <c r="EB11" s="3" t="n">
+        <v>102.269</v>
       </c>
     </row>
     <row r="12">
@@ -12862,16 +12943,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>221.574</v>
+        <v>221.058</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>103147.571628</v>
+        <v>102907.362276</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3147.571628000005</v>
+        <v>2907.362276</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.03147571628000005</v>
+        <v>0.02907362276</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -13238,6 +13319,9 @@
       </c>
       <c r="EA12" s="3" t="n">
         <v>221.574</v>
+      </c>
+      <c r="EB12" s="3" t="n">
+        <v>221.058</v>
       </c>
     </row>
     <row r="13">
@@ -13263,16 +13347,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.224</v>
+        <v>21.23</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>245935.32852</v>
+        <v>246004.85415</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>45935.32851999998</v>
+        <v>46004.85415</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2296766425999999</v>
+        <v>0.23002427075</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -13639,6 +13723,9 @@
       </c>
       <c r="EA13" s="3" t="n">
         <v>21.224</v>
+      </c>
+      <c r="EB13" s="3" t="n">
+        <v>21.23</v>
       </c>
     </row>
     <row r="14">
@@ -13664,16 +13751,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35.4841</v>
+        <v>35.7137</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>128012.6520646</v>
+        <v>128840.9584022</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>28012.6520646</v>
+        <v>28840.95840220002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.280126520646</v>
+        <v>0.2884095840220002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -14034,6 +14121,9 @@
       </c>
       <c r="EA14" s="3" t="n">
         <v>35.4841</v>
+      </c>
+      <c r="EB14" s="3" t="n">
+        <v>35.7137</v>
       </c>
     </row>
     <row r="15">
@@ -14059,16 +14149,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.3</v>
+        <v>11.25</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>110106.6011</v>
+        <v>109619.40375</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>10106.60110000001</v>
+        <v>9619.403749999998</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1010660110000001</v>
+        <v>0.09619403749999998</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -14435,6 +14525,9 @@
       </c>
       <c r="EA15" s="3" t="n">
         <v>11.3</v>
+      </c>
+      <c r="EB15" s="3" t="n">
+        <v>11.25</v>
       </c>
     </row>
     <row r="16">
@@ -14460,16 +14553,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.7391</v>
+        <v>24.1085</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>141580.0880848</v>
+        <v>137971.209688</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>41580.08808479999</v>
+        <v>37971.209688</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4158008808479999</v>
+        <v>0.37971209688</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -14830,6 +14923,9 @@
       </c>
       <c r="EA16" s="3" t="n">
         <v>24.7391</v>
+      </c>
+      <c r="EB16" s="3" t="n">
+        <v>24.1085</v>
       </c>
     </row>
     <row r="17">
@@ -14855,16 +14951,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7782</v>
+        <v>16.8084</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55469.68555739999</v>
+        <v>55569.52847879999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5469.685557399993</v>
+        <v>5569.528478799992</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1093937111479999</v>
+        <v>0.1113905695759998</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -15225,6 +15321,9 @@
       </c>
       <c r="EA17" s="3" t="n">
         <v>16.7782</v>
+      </c>
+      <c r="EB17" s="3" t="n">
+        <v>16.8084</v>
       </c>
     </row>
     <row r="18">
@@ -15250,16 +15349,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.92</v>
+        <v>44.81</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84738.70512</v>
+        <v>84531.19716</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4738.705119999999</v>
+        <v>4531.197159999996</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.05923381399999998</v>
+        <v>0.05663996449999995</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -15626,6 +15725,9 @@
       </c>
       <c r="EA18" s="3" t="n">
         <v>44.92</v>
+      </c>
+      <c r="EB18" s="3" t="n">
+        <v>44.81</v>
       </c>
     </row>
     <row r="19">
@@ -15651,16 +15753,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.8753</v>
+        <v>12.1823</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>171797.1862798</v>
+        <v>176238.4834418</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>21797.18627979999</v>
+        <v>26238.4834418</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.1453145751986666</v>
+        <v>0.1749232229453333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -16021,6 +16123,9 @@
       </c>
       <c r="EA19" s="3" t="n">
         <v>11.8753</v>
+      </c>
+      <c r="EB19" s="3" t="n">
+        <v>12.1823</v>
       </c>
     </row>
     <row r="20">
@@ -16046,16 +16151,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.09</v>
+        <v>10.24</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>264921.05227</v>
+        <v>268859.42272</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>14921.05226999999</v>
+        <v>18859.42272000003</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.05968420907999994</v>
+        <v>0.07543769088000013</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -16422,6 +16527,9 @@
       </c>
       <c r="EA20" s="3" t="n">
         <v>10.09</v>
+      </c>
+      <c r="EB20" s="3" t="n">
+        <v>10.24</v>
       </c>
     </row>
     <row r="21">
@@ -16447,16 +16555,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.4945</v>
+        <v>111.6656</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>169389.0225755</v>
+        <v>169648.9677904</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-610.9774244999862</v>
+        <v>-351.0322096000018</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.003593984849999919</v>
+        <v>-0.002064895350588246</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -16823,6 +16931,9 @@
       </c>
       <c r="EA21" s="3" t="n">
         <v>111.4945</v>
+      </c>
+      <c r="EB21" s="3" t="n">
+        <v>111.6656</v>
       </c>
     </row>
     <row r="22">
@@ -17219,6 +17330,9 @@
       <c r="EA22" s="3" t="n">
         <v>40.316</v>
       </c>
+      <c r="EB22" s="3" t="n">
+        <v>40.316</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -17243,16 +17357,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.84</v>
+        <v>60.8286</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>165269.85228</v>
+        <v>165238.8845562</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>15269.85228000002</v>
+        <v>15238.88455620001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1017990152000001</v>
+        <v>0.101592563708</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -17619,6 +17733,9 @@
       </c>
       <c r="EA23" s="3" t="n">
         <v>60.84</v>
+      </c>
+      <c r="EB23" s="3" t="n">
+        <v>60.8286</v>
       </c>
     </row>
     <row r="24">
@@ -17644,16 +17761,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.8919</v>
+        <v>25.9235</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>94075.26697339999</v>
+        <v>94190.08197100001</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-5924.733026600006</v>
+        <v>-5809.918028999993</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.05924733026600006</v>
+        <v>-0.05809918028999993</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -18014,6 +18131,9 @@
       </c>
       <c r="EA24" s="3" t="n">
         <v>25.8919</v>
+      </c>
+      <c r="EB24" s="3" t="n">
+        <v>25.9235</v>
       </c>
     </row>
     <row r="25">
@@ -18437,16 +18557,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.1228</v>
+        <v>11.1334</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>132825.307602</v>
+        <v>132951.889781</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>22825.30760199999</v>
+        <v>22951.88978100001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.2075027963818181</v>
+        <v>0.2086535434636364</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -18810,6 +18930,9 @@
       </c>
       <c r="EA26" s="3" t="n">
         <v>11.1228</v>
+      </c>
+      <c r="EB26" s="3" t="n">
+        <v>11.1334</v>
       </c>
     </row>
     <row r="27">
@@ -19236,16 +19359,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>115.6012</v>
+        <v>114.9642</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>382253.5171884</v>
+        <v>380147.1766794</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>2253.51718840003</v>
+        <v>147.1766794000287</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>0.005930308390526395</v>
+        <v>0.000387307051052707</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -19612,6 +19735,9 @@
       </c>
       <c r="EA28" s="3" t="n">
         <v>115.6012</v>
+      </c>
+      <c r="EB28" s="3" t="n">
+        <v>114.9642</v>
       </c>
     </row>
     <row r="29">
@@ -19637,16 +19763,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.0418</v>
+        <v>12.0605</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>115645.8707854</v>
+        <v>115825.4600315</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>15645.87078539999</v>
+        <v>15825.46003149998</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.156458707854</v>
+        <v>0.1582546003149999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -20007,6 +20133,9 @@
       </c>
       <c r="EA29" s="3" t="n">
         <v>12.0418</v>
+      </c>
+      <c r="EB29" s="3" t="n">
+        <v>12.0605</v>
       </c>
     </row>
     <row r="30">
@@ -20032,16 +20161,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.2457</v>
+        <v>17.2022</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>127546.8000477</v>
+        <v>127225.0800942</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>27546.80004769999</v>
+        <v>27225.08009420001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2754680004769999</v>
+        <v>0.272250800942</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -20402,6 +20531,9 @@
       </c>
       <c r="EA30" s="3" t="n">
         <v>17.2457</v>
+      </c>
+      <c r="EB30" s="3" t="n">
+        <v>17.2022</v>
       </c>
     </row>
     <row r="31">
@@ -20427,16 +20559,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>396.7333</v>
+        <v>395.4481</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>105562.796464</v>
+        <v>105220.830448</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>5562.796463999985</v>
+        <v>5220.830447999993</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.05562796463999985</v>
+        <v>0.05220830447999993</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -20800,6 +20932,9 @@
       </c>
       <c r="EA31" s="3" t="n">
         <v>396.7333</v>
+      </c>
+      <c r="EB31" s="3" t="n">
+        <v>395.4481</v>
       </c>
     </row>
     <row r="32">
@@ -20825,16 +20960,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.63</v>
+        <v>10.66</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>224717.7748</v>
+        <v>225351.9736</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>24717.77480000001</v>
+        <v>25351.9736</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1235888740000001</v>
+        <v>0.126759868</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -21201,6 +21336,9 @@
       </c>
       <c r="EA32" s="3" t="n">
         <v>10.63</v>
+      </c>
+      <c r="EB32" s="3" t="n">
+        <v>10.66</v>
       </c>
     </row>
     <row r="33">
@@ -21226,16 +21364,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.36</v>
+        <v>19.43</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>69379.27039999999</v>
+        <v>69630.12519999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>9379.270399999994</v>
+        <v>9630.125199999995</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1563211733333332</v>
+        <v>0.1605020866666666</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -21596,6 +21734,9 @@
       </c>
       <c r="EA33" s="3" t="n">
         <v>19.36</v>
+      </c>
+      <c r="EB33" s="3" t="n">
+        <v>19.43</v>
       </c>
     </row>
     <row r="34">
@@ -21621,16 +21762,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>232.5041</v>
+        <v>236.6514</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>81732.3987771</v>
+        <v>83190.30329339999</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>1732.398777099996</v>
+        <v>3190.303293399993</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.02165498471374995</v>
+        <v>0.03987879116749991</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -21994,6 +22135,9 @@
       </c>
       <c r="EA34" s="3" t="n">
         <v>232.5041</v>
+      </c>
+      <c r="EB34" s="3" t="n">
+        <v>236.6514</v>
       </c>
     </row>
     <row r="35">
@@ -22019,16 +22163,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.82</v>
+        <v>15.84</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>112882.39186</v>
+        <v>113025.10032</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>12882.39186</v>
+        <v>13025.10032</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1288239186</v>
+        <v>0.1302510032</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -22392,6 +22536,9 @@
       </c>
       <c r="EA35" s="3" t="n">
         <v>15.82</v>
+      </c>
+      <c r="EB35" s="3" t="n">
+        <v>15.84</v>
       </c>
     </row>
     <row r="36">
@@ -22417,16 +22564,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>365.9877</v>
+        <v>364.6221</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>170442.6678162</v>
+        <v>169806.6997026</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>20442.6678162</v>
+        <v>19806.69970259999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.136284452108</v>
+        <v>0.1320446646839999</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -22790,6 +22937,9 @@
       </c>
       <c r="EA36" s="3" t="n">
         <v>365.9877</v>
+      </c>
+      <c r="EB36" s="3" t="n">
+        <v>364.6221</v>
       </c>
     </row>
     <row r="37">
@@ -22815,16 +22965,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.675</v>
+        <v>16.628</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62746.174075</v>
+        <v>62569.318292</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12746.174075</v>
+        <v>12569.318292</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2549234815</v>
+        <v>0.2513863658400001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -23188,6 +23338,9 @@
       </c>
       <c r="EA37" s="3" t="n">
         <v>16.675</v>
+      </c>
+      <c r="EB37" s="3" t="n">
+        <v>16.628</v>
       </c>
     </row>
     <row r="38">
@@ -23213,16 +23366,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.7084</v>
+        <v>13.7453</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>81982.83944879999</v>
+        <v>82203.5192346</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1982.83944879999</v>
+        <v>2203.519234599997</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.02478549310999988</v>
+        <v>0.02754399043249996</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -23583,6 +23736,9 @@
       </c>
       <c r="EA38" s="3" t="n">
         <v>13.7084</v>
+      </c>
+      <c r="EB38" s="3" t="n">
+        <v>13.7453</v>
       </c>
     </row>
     <row r="39">
@@ -23608,16 +23764,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1024.6051</v>
+        <v>1025.5891</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51108.3269931</v>
+        <v>51157.4098971</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1108.326993100003</v>
+        <v>1157.409897099998</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02216653986200006</v>
+        <v>0.02314819794199997</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -23978,6 +24134,9 @@
       </c>
       <c r="EA39" s="3" t="n">
         <v>1024.6051</v>
+      </c>
+      <c r="EB39" s="3" t="n">
+        <v>1025.5891</v>
       </c>
     </row>
     <row r="40">
@@ -24003,16 +24162,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.7009</v>
+        <v>20.5476</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>104353.7958243</v>
+        <v>103581.0063852</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>4353.795824300003</v>
+        <v>3581.006385200002</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.04353795824300003</v>
+        <v>0.03581006385200002</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -24376,6 +24535,9 @@
       </c>
       <c r="EA40" s="3" t="n">
         <v>20.7009</v>
+      </c>
+      <c r="EB40" s="3" t="n">
+        <v>20.5476</v>
       </c>
     </row>
     <row r="41">
@@ -24388,13 +24550,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4939033.6657246</v>
+        <v>4947987.3039979</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>469033.6657245999</v>
+        <v>477987.3039979</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.104929231705727</v>
+        <v>0.1069322827735794</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-18
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-17 06:31 IST</t>
+          <t>Generated: 2026-10-18 06:56 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4947987.3039979</v>
+        <v>4948355.3351537</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>477987.3039979003</v>
+        <v>478355.3351536999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1069322827735795</v>
+        <v>0.107014616365481</v>
       </c>
     </row>
     <row r="6">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5479427.808747198</v>
+        <v>5479795.839902998</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>418645.7887471989</v>
+        <v>419013.8199029984</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08272353701319839</v>
+        <v>0.08279625920402682</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-17</t>
+          <t>Last snapshot: 2026-10-18</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FF19"/>
+  <dimension ref="A1:FG19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -781,6 +781,7 @@
     <col width="21" customWidth="1" min="160" max="160"/>
     <col width="21" customWidth="1" min="161" max="161"/>
     <col width="21" customWidth="1" min="162" max="162"/>
+    <col width="21" customWidth="1" min="163" max="163"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1594,6 +1595,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
+      <c r="FG1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2083,6 +2089,9 @@
       <c r="FF2" s="3" t="n">
         <v>559.7000122070312</v>
       </c>
+      <c r="FG2" s="3" t="n">
+        <v>559.7000122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2602,6 +2611,9 @@
       <c r="FF4" s="3" t="n">
         <v>1427.400024414062</v>
       </c>
+      <c r="FG4" s="3" t="n">
+        <v>1427.400024414062</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3094,6 +3106,9 @@
       <c r="FF5" s="3" t="n">
         <v>474.1499938964844</v>
       </c>
+      <c r="FG5" s="3" t="n">
+        <v>474.1499938964844</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3586,6 +3601,9 @@
       <c r="FF6" s="3" t="n">
         <v>376.6000061035156</v>
       </c>
+      <c r="FG6" s="3" t="n">
+        <v>376.6000061035156</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4078,6 +4096,9 @@
       <c r="FF7" s="3" t="n">
         <v>273.4500122070312</v>
       </c>
+      <c r="FG7" s="3" t="n">
+        <v>273.4500122070312</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4597,6 +4618,9 @@
       <c r="FF9" s="3" t="n">
         <v>14.97000026702881</v>
       </c>
+      <c r="FG9" s="3" t="n">
+        <v>14.97000026702881</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5089,6 +5113,9 @@
       <c r="FF10" s="3" t="n">
         <v>445</v>
       </c>
+      <c r="FG10" s="3" t="n">
+        <v>445</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5581,6 +5608,9 @@
       <c r="FF11" s="3" t="n">
         <v>16.28000068664551</v>
       </c>
+      <c r="FG11" s="3" t="n">
+        <v>16.28000068664551</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6073,6 +6103,9 @@
       <c r="FF12" s="3" t="n">
         <v>2523.89990234375</v>
       </c>
+      <c r="FG12" s="3" t="n">
+        <v>2523.89990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6565,6 +6598,9 @@
       <c r="FF13" s="3" t="n">
         <v>42</v>
       </c>
+      <c r="FG13" s="3" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7057,6 +7093,9 @@
       <c r="FF14" s="3" t="n">
         <v>633.1500244140625</v>
       </c>
+      <c r="FG14" s="3" t="n">
+        <v>633.1500244140625</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7603,6 +7642,9 @@
       <c r="FF17" s="3" t="n">
         <v>474.75</v>
       </c>
+      <c r="FG17" s="3" t="n">
+        <v>474.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8093,6 +8135,9 @@
         <v>353</v>
       </c>
       <c r="FF18" s="3" t="n">
+        <v>353.8500061035156</v>
+      </c>
+      <c r="FG18" s="3" t="n">
         <v>353.8500061035156</v>
       </c>
     </row>
@@ -8123,7 +8168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EB41"/>
+  <dimension ref="A1:EC41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8258,6 +8303,7 @@
     <col width="13" customWidth="1" min="130" max="130"/>
     <col width="13" customWidth="1" min="131" max="131"/>
     <col width="13" customWidth="1" min="132" max="132"/>
+    <col width="13" customWidth="1" min="133" max="133"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8921,6 +8967,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
+      <c r="EC1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9325,6 +9376,9 @@
       <c r="EB2" s="3" t="n">
         <v>56.2538</v>
       </c>
+      <c r="EC2" s="3" t="n">
+        <v>56.2538</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9723,6 +9777,9 @@
       <c r="EB3" s="3" t="n">
         <v>26.7682</v>
       </c>
+      <c r="EC3" s="3" t="n">
+        <v>26.7682</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10121,6 +10178,9 @@
       <c r="EB4" s="3" t="n">
         <v>12.08</v>
       </c>
+      <c r="EC4" s="3" t="n">
+        <v>12.08</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10519,6 +10579,9 @@
       <c r="EB5" s="3" t="n">
         <v>9.2668</v>
       </c>
+      <c r="EC5" s="3" t="n">
+        <v>9.2668</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10923,6 +10986,9 @@
       <c r="EB6" s="3" t="n">
         <v>11.1632</v>
       </c>
+      <c r="EC6" s="3" t="n">
+        <v>11.1632</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11321,6 +11387,9 @@
       <c r="EB7" s="3" t="n">
         <v>33.7586</v>
       </c>
+      <c r="EC7" s="3" t="n">
+        <v>33.7586</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11725,6 +11794,9 @@
       <c r="EB8" s="3" t="n">
         <v>35.1128</v>
       </c>
+      <c r="EC8" s="3" t="n">
+        <v>35.1128</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12123,6 +12195,9 @@
       <c r="EB9" s="3" t="n">
         <v>39.6566</v>
       </c>
+      <c r="EC9" s="3" t="n">
+        <v>39.6566</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12521,6 +12596,9 @@
       <c r="EB10" s="3" t="n">
         <v>49.1177</v>
       </c>
+      <c r="EC10" s="3" t="n">
+        <v>49.1177</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12919,6 +12997,9 @@
       <c r="EB11" s="3" t="n">
         <v>102.269</v>
       </c>
+      <c r="EC11" s="3" t="n">
+        <v>102.269</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13323,6 +13404,9 @@
       <c r="EB12" s="3" t="n">
         <v>221.058</v>
       </c>
+      <c r="EC12" s="3" t="n">
+        <v>221.058</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13727,6 +13811,9 @@
       <c r="EB13" s="3" t="n">
         <v>21.23</v>
       </c>
+      <c r="EC13" s="3" t="n">
+        <v>21.23</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14125,6 +14212,9 @@
       <c r="EB14" s="3" t="n">
         <v>35.7137</v>
       </c>
+      <c r="EC14" s="3" t="n">
+        <v>35.7137</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14529,6 +14619,9 @@
       <c r="EB15" s="3" t="n">
         <v>11.25</v>
       </c>
+      <c r="EC15" s="3" t="n">
+        <v>11.25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -14927,6 +15020,9 @@
       <c r="EB16" s="3" t="n">
         <v>24.1085</v>
       </c>
+      <c r="EC16" s="3" t="n">
+        <v>24.1085</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -15325,6 +15421,9 @@
       <c r="EB17" s="3" t="n">
         <v>16.8084</v>
       </c>
+      <c r="EC17" s="3" t="n">
+        <v>16.8084</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15729,6 +15828,9 @@
       <c r="EB18" s="3" t="n">
         <v>44.81</v>
       </c>
+      <c r="EC18" s="3" t="n">
+        <v>44.81</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -16127,6 +16229,9 @@
       <c r="EB19" s="3" t="n">
         <v>12.1823</v>
       </c>
+      <c r="EC19" s="3" t="n">
+        <v>12.1823</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -16531,6 +16636,9 @@
       <c r="EB20" s="3" t="n">
         <v>10.24</v>
       </c>
+      <c r="EC20" s="3" t="n">
+        <v>10.24</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -16935,6 +17043,9 @@
       <c r="EB21" s="3" t="n">
         <v>111.6656</v>
       </c>
+      <c r="EC21" s="3" t="n">
+        <v>111.6656</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -16959,16 +17070,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>40.316</v>
+        <v>40.62</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>61863.28936</v>
+        <v>62329.76519999999</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>1863.289360000002</v>
+        <v>2329.765199999994</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.03105482266666671</v>
+        <v>0.03882941999999991</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -17332,6 +17443,9 @@
       </c>
       <c r="EB22" s="3" t="n">
         <v>40.316</v>
+      </c>
+      <c r="EC22" s="3" t="n">
+        <v>40.62</v>
       </c>
     </row>
     <row r="23">
@@ -17737,6 +17851,9 @@
       <c r="EB23" s="3" t="n">
         <v>60.8286</v>
       </c>
+      <c r="EC23" s="3" t="n">
+        <v>60.8286</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -18135,6 +18252,9 @@
       <c r="EB24" s="3" t="n">
         <v>25.9235</v>
       </c>
+      <c r="EC24" s="3" t="n">
+        <v>25.9235</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -18159,16 +18279,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.581</v>
+        <v>12.5727</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>206601.080594</v>
+        <v>206464.7806998</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>6601.08059399997</v>
+        <v>6464.780699799972</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.03300540296999985</v>
+        <v>0.03232390349899986</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -18532,6 +18652,9 @@
       </c>
       <c r="EA25" s="3" t="n">
         <v>12.581</v>
+      </c>
+      <c r="EC25" s="3" t="n">
+        <v>12.5727</v>
       </c>
     </row>
     <row r="26">
@@ -18934,6 +19057,9 @@
       <c r="EB26" s="3" t="n">
         <v>11.1334</v>
       </c>
+      <c r="EC26" s="3" t="n">
+        <v>11.1334</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -18958,16 +19084,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>68.7634</v>
+        <v>68.7869</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>110768.210524</v>
+        <v>110806.065734</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>768.2105239999946</v>
+        <v>806.0657340000034</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>0.006983732036363588</v>
+        <v>0.007327870309090941</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -19334,6 +19460,9 @@
       </c>
       <c r="EA27" s="3" t="n">
         <v>68.7634</v>
+      </c>
+      <c r="EC27" s="3" t="n">
+        <v>68.7869</v>
       </c>
     </row>
     <row r="28">
@@ -19739,6 +19868,9 @@
       <c r="EB28" s="3" t="n">
         <v>114.9642</v>
       </c>
+      <c r="EC28" s="3" t="n">
+        <v>114.9642</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -20137,6 +20269,9 @@
       <c r="EB29" s="3" t="n">
         <v>12.0605</v>
       </c>
+      <c r="EC29" s="3" t="n">
+        <v>12.0605</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -20535,6 +20670,9 @@
       <c r="EB30" s="3" t="n">
         <v>17.2022</v>
       </c>
+      <c r="EC30" s="3" t="n">
+        <v>17.2022</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -20936,6 +21074,9 @@
       <c r="EB31" s="3" t="n">
         <v>395.4481</v>
       </c>
+      <c r="EC31" s="3" t="n">
+        <v>395.4481</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -21340,6 +21481,9 @@
       <c r="EB32" s="3" t="n">
         <v>10.66</v>
       </c>
+      <c r="EC32" s="3" t="n">
+        <v>10.66</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -21738,6 +21882,9 @@
       <c r="EB33" s="3" t="n">
         <v>19.43</v>
       </c>
+      <c r="EC33" s="3" t="n">
+        <v>19.43</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -22139,6 +22286,9 @@
       <c r="EB34" s="3" t="n">
         <v>236.6514</v>
       </c>
+      <c r="EC34" s="3" t="n">
+        <v>236.6514</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -22540,6 +22690,9 @@
       <c r="EB35" s="3" t="n">
         <v>15.84</v>
       </c>
+      <c r="EC35" s="3" t="n">
+        <v>15.84</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -22941,6 +23094,9 @@
       <c r="EB36" s="3" t="n">
         <v>364.6221</v>
       </c>
+      <c r="EC36" s="3" t="n">
+        <v>364.6221</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -23342,6 +23498,9 @@
       <c r="EB37" s="3" t="n">
         <v>16.628</v>
       </c>
+      <c r="EC37" s="3" t="n">
+        <v>16.628</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -23740,6 +23899,9 @@
       <c r="EB38" s="3" t="n">
         <v>13.7453</v>
       </c>
+      <c r="EC38" s="3" t="n">
+        <v>13.7453</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -24138,6 +24300,9 @@
       <c r="EB39" s="3" t="n">
         <v>1025.5891</v>
       </c>
+      <c r="EC39" s="3" t="n">
+        <v>1025.5891</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -24539,6 +24704,9 @@
       <c r="EB40" s="3" t="n">
         <v>20.5476</v>
       </c>
+      <c r="EC40" s="3" t="n">
+        <v>20.5476</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -24550,13 +24718,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4947987.3039979</v>
+        <v>4948355.3351537</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>477987.3039979</v>
+        <v>478355.3351537</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1069322827735794</v>
+        <v>0.107014616365481</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-19
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-18 06:56 IST</t>
+          <t>Generated: 2026-10-19 07:16 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>531440.5047492981</v>
+        <v>530627.9961853027</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-59341.51525070192</v>
+        <v>-60154.02381469728</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1004457028849692</v>
+        <v>-0.101821013128831</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5479795.839902998</v>
+        <v>5478983.331339003</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>419013.8199029984</v>
+        <v>418201.311339003</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08279625920402682</v>
+        <v>0.08263570920191561</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-18</t>
+          <t>Last snapshot: 2026-10-19</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FG19"/>
+  <dimension ref="A1:FH19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -782,6 +782,7 @@
     <col width="21" customWidth="1" min="161" max="161"/>
     <col width="21" customWidth="1" min="162" max="162"/>
     <col width="21" customWidth="1" min="163" max="163"/>
+    <col width="21" customWidth="1" min="164" max="164"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1600,6 +1601,11 @@
           <t>2026-10-18</t>
         </is>
       </c>
+      <c r="FH1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1619,13 +1625,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>559.7000122070312</v>
+        <v>562.2999877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44776.0009765625</v>
+        <v>44983.9990234375</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>958.490976562498</v>
+        <v>1166.489023437498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2091,6 +2097,9 @@
       </c>
       <c r="FG2" s="3" t="n">
         <v>559.7000122070312</v>
+      </c>
+      <c r="FH2" s="3" t="n">
+        <v>562.2999877929688</v>
       </c>
     </row>
     <row r="3">
@@ -2138,13 +2147,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1427.400024414062</v>
+        <v>1430</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28548.00048828125</v>
+        <v>28600</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3556.579511718752</v>
+        <v>-3504.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2613,6 +2622,9 @@
       </c>
       <c r="FG4" s="3" t="n">
         <v>1427.400024414062</v>
+      </c>
+      <c r="FH4" s="3" t="n">
+        <v>1430</v>
       </c>
     </row>
     <row r="5">
@@ -2633,13 +2645,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>474.1499938964844</v>
+        <v>464.2000122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9482.999877929688</v>
+        <v>9284.000244140625</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4730.100122070313</v>
+        <v>-4929.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3108,6 +3120,9 @@
       </c>
       <c r="FG5" s="3" t="n">
         <v>474.1499938964844</v>
+      </c>
+      <c r="FH5" s="3" t="n">
+        <v>464.2000122070312</v>
       </c>
     </row>
     <row r="6">
@@ -3128,13 +3143,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>376.6000061035156</v>
+        <v>369.8999938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15064.00024414062</v>
+        <v>14795.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2438.239755859377</v>
+        <v>-2706.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3603,6 +3618,9 @@
       </c>
       <c r="FG6" s="3" t="n">
         <v>376.6000061035156</v>
+      </c>
+      <c r="FH6" s="3" t="n">
+        <v>369.8999938964844</v>
       </c>
     </row>
     <row r="7">
@@ -3623,13 +3641,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>273.4500122070312</v>
+        <v>270.75</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>27345.00122070312</v>
+        <v>27075</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>911.1812207031253</v>
+        <v>641.1800000000003</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4098,6 +4116,9 @@
       </c>
       <c r="FG7" s="3" t="n">
         <v>273.4500122070312</v>
+      </c>
+      <c r="FH7" s="3" t="n">
+        <v>270.75</v>
       </c>
     </row>
     <row r="8">
@@ -4145,13 +4166,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.97000026702881</v>
+        <v>14.72999954223633</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22455.00040054321</v>
+        <v>22094.99931335449</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8595.169599456785</v>
+        <v>-8955.170686645506</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4620,6 +4641,9 @@
       </c>
       <c r="FG9" s="3" t="n">
         <v>14.97000026702881</v>
+      </c>
+      <c r="FH9" s="3" t="n">
+        <v>14.72999954223633</v>
       </c>
     </row>
     <row r="10">
@@ -4640,13 +4664,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>445</v>
+        <v>446.2999877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44500</v>
+        <v>44629.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6998.480000000003</v>
+        <v>-6868.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5115,6 +5139,9 @@
       </c>
       <c r="FG10" s="3" t="n">
         <v>445</v>
+      </c>
+      <c r="FH10" s="3" t="n">
+        <v>446.2999877929688</v>
       </c>
     </row>
     <row r="11">
@@ -5135,13 +5162,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>16.28000068664551</v>
+        <v>18.42000007629395</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>16280.00068664551</v>
+        <v>18420.00007629395</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>6438.790686645509</v>
+        <v>8578.790076293946</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5610,6 +5637,9 @@
       </c>
       <c r="FG11" s="3" t="n">
         <v>16.28000068664551</v>
+      </c>
+      <c r="FH11" s="3" t="n">
+        <v>18.42000007629395</v>
       </c>
     </row>
     <row r="12">
@@ -5630,13 +5660,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2523.89990234375</v>
+        <v>2504.199951171875</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25238.9990234375</v>
+        <v>25041.99951171875</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2484.2509765625</v>
+        <v>-2681.25048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6105,6 +6135,9 @@
       </c>
       <c r="FG12" s="3" t="n">
         <v>2523.89990234375</v>
+      </c>
+      <c r="FH12" s="3" t="n">
+        <v>2504.199951171875</v>
       </c>
     </row>
     <row r="13">
@@ -6125,13 +6158,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>42</v>
+        <v>40.84000015258789</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>25200</v>
+        <v>24504.00009155273</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-9831.760000000002</v>
+        <v>-10527.75990844727</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6600,6 +6633,9 @@
       </c>
       <c r="FG13" s="3" t="n">
         <v>42</v>
+      </c>
+      <c r="FH13" s="3" t="n">
+        <v>40.84000015258789</v>
       </c>
     </row>
     <row r="14">
@@ -6620,13 +6656,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>633.1500244140625</v>
+        <v>624.5</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31657.50122070312</v>
+        <v>31225</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-10805.00877929688</v>
+        <v>-11237.51</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7095,6 +7131,9 @@
       </c>
       <c r="FG14" s="3" t="n">
         <v>633.1500244140625</v>
+      </c>
+      <c r="FH14" s="3" t="n">
+        <v>624.5</v>
       </c>
     </row>
     <row r="15">
@@ -7169,13 +7208,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>474.75</v>
+        <v>460.4500122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23737.5</v>
+        <v>23022.50061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1982.970000000001</v>
+        <v>1267.970610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7644,6 +7683,9 @@
       </c>
       <c r="FG17" s="3" t="n">
         <v>474.75</v>
+      </c>
+      <c r="FH17" s="3" t="n">
+        <v>460.4500122070312</v>
       </c>
     </row>
     <row r="18">
@@ -7664,13 +7706,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>353.8500061035156</v>
+        <v>351.7999877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35385.00061035156</v>
+        <v>35179.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11255.81938964844</v>
+        <v>-11460.82122070312</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8139,6 +8181,9 @@
       </c>
       <c r="FG18" s="3" t="n">
         <v>353.8500061035156</v>
+      </c>
+      <c r="FH18" s="3" t="n">
+        <v>351.7999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -8151,10 +8196,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>531440.5047492981</v>
+        <v>530627.9961853027</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-59341.51525070192</v>
+        <v>-60154.02381469728</v>
       </c>
     </row>
   </sheetData>
@@ -8168,7 +8213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EC41"/>
+  <dimension ref="A1:ED41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8304,6 +8349,7 @@
     <col width="13" customWidth="1" min="131" max="131"/>
     <col width="13" customWidth="1" min="132" max="132"/>
     <col width="13" customWidth="1" min="133" max="133"/>
+    <col width="13" customWidth="1" min="134" max="134"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8972,6 +9018,11 @@
           <t>2026-10-18</t>
         </is>
       </c>
+      <c r="ED1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9379,6 +9430,9 @@
       <c r="EC2" s="3" t="n">
         <v>56.2538</v>
       </c>
+      <c r="ED2" s="3" t="n">
+        <v>56.2538</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9780,6 +9834,9 @@
       <c r="EC3" s="3" t="n">
         <v>26.7682</v>
       </c>
+      <c r="ED3" s="3" t="n">
+        <v>26.7682</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10181,6 +10238,9 @@
       <c r="EC4" s="3" t="n">
         <v>12.08</v>
       </c>
+      <c r="ED4" s="3" t="n">
+        <v>12.08</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10582,6 +10642,9 @@
       <c r="EC5" s="3" t="n">
         <v>9.2668</v>
       </c>
+      <c r="ED5" s="3" t="n">
+        <v>9.2668</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10989,6 +11052,9 @@
       <c r="EC6" s="3" t="n">
         <v>11.1632</v>
       </c>
+      <c r="ED6" s="3" t="n">
+        <v>11.1632</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11390,6 +11456,9 @@
       <c r="EC7" s="3" t="n">
         <v>33.7586</v>
       </c>
+      <c r="ED7" s="3" t="n">
+        <v>33.7586</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11797,6 +11866,9 @@
       <c r="EC8" s="3" t="n">
         <v>35.1128</v>
       </c>
+      <c r="ED8" s="3" t="n">
+        <v>35.1128</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12198,6 +12270,9 @@
       <c r="EC9" s="3" t="n">
         <v>39.6566</v>
       </c>
+      <c r="ED9" s="3" t="n">
+        <v>39.6566</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12599,6 +12674,9 @@
       <c r="EC10" s="3" t="n">
         <v>49.1177</v>
       </c>
+      <c r="ED10" s="3" t="n">
+        <v>49.1177</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13000,6 +13078,9 @@
       <c r="EC11" s="3" t="n">
         <v>102.269</v>
       </c>
+      <c r="ED11" s="3" t="n">
+        <v>102.269</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13407,6 +13488,9 @@
       <c r="EC12" s="3" t="n">
         <v>221.058</v>
       </c>
+      <c r="ED12" s="3" t="n">
+        <v>221.058</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13814,6 +13898,9 @@
       <c r="EC13" s="3" t="n">
         <v>21.23</v>
       </c>
+      <c r="ED13" s="3" t="n">
+        <v>21.23</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14215,6 +14302,9 @@
       <c r="EC14" s="3" t="n">
         <v>35.7137</v>
       </c>
+      <c r="ED14" s="3" t="n">
+        <v>35.7137</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14622,6 +14712,9 @@
       <c r="EC15" s="3" t="n">
         <v>11.25</v>
       </c>
+      <c r="ED15" s="3" t="n">
+        <v>11.25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15023,6 +15116,9 @@
       <c r="EC16" s="3" t="n">
         <v>24.1085</v>
       </c>
+      <c r="ED16" s="3" t="n">
+        <v>24.1085</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -15424,6 +15520,9 @@
       <c r="EC17" s="3" t="n">
         <v>16.8084</v>
       </c>
+      <c r="ED17" s="3" t="n">
+        <v>16.8084</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15831,6 +15930,9 @@
       <c r="EC18" s="3" t="n">
         <v>44.81</v>
       </c>
+      <c r="ED18" s="3" t="n">
+        <v>44.81</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -16232,6 +16334,9 @@
       <c r="EC19" s="3" t="n">
         <v>12.1823</v>
       </c>
+      <c r="ED19" s="3" t="n">
+        <v>12.1823</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -16639,6 +16744,9 @@
       <c r="EC20" s="3" t="n">
         <v>10.24</v>
       </c>
+      <c r="ED20" s="3" t="n">
+        <v>10.24</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -17046,6 +17154,9 @@
       <c r="EC21" s="3" t="n">
         <v>111.6656</v>
       </c>
+      <c r="ED21" s="3" t="n">
+        <v>111.6656</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -17447,6 +17558,9 @@
       <c r="EC22" s="3" t="n">
         <v>40.62</v>
       </c>
+      <c r="ED22" s="3" t="n">
+        <v>40.62</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -17854,6 +17968,9 @@
       <c r="EC23" s="3" t="n">
         <v>60.8286</v>
       </c>
+      <c r="ED23" s="3" t="n">
+        <v>60.8286</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -18255,6 +18372,9 @@
       <c r="EC24" s="3" t="n">
         <v>25.9235</v>
       </c>
+      <c r="ED24" s="3" t="n">
+        <v>25.9235</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -18656,6 +18776,9 @@
       <c r="EC25" s="3" t="n">
         <v>12.5727</v>
       </c>
+      <c r="ED25" s="3" t="n">
+        <v>12.5727</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -19060,6 +19183,9 @@
       <c r="EC26" s="3" t="n">
         <v>11.1334</v>
       </c>
+      <c r="ED26" s="3" t="n">
+        <v>11.1334</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -19464,6 +19590,9 @@
       <c r="EC27" s="3" t="n">
         <v>68.7869</v>
       </c>
+      <c r="ED27" s="3" t="n">
+        <v>68.7869</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -19871,6 +20000,9 @@
       <c r="EC28" s="3" t="n">
         <v>114.9642</v>
       </c>
+      <c r="ED28" s="3" t="n">
+        <v>114.9642</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -20272,6 +20404,9 @@
       <c r="EC29" s="3" t="n">
         <v>12.0605</v>
       </c>
+      <c r="ED29" s="3" t="n">
+        <v>12.0605</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -20673,6 +20808,9 @@
       <c r="EC30" s="3" t="n">
         <v>17.2022</v>
       </c>
+      <c r="ED30" s="3" t="n">
+        <v>17.2022</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -21077,6 +21215,9 @@
       <c r="EC31" s="3" t="n">
         <v>395.4481</v>
       </c>
+      <c r="ED31" s="3" t="n">
+        <v>395.4481</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -21484,6 +21625,9 @@
       <c r="EC32" s="3" t="n">
         <v>10.66</v>
       </c>
+      <c r="ED32" s="3" t="n">
+        <v>10.66</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -21885,6 +22029,9 @@
       <c r="EC33" s="3" t="n">
         <v>19.43</v>
       </c>
+      <c r="ED33" s="3" t="n">
+        <v>19.43</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -22289,6 +22436,9 @@
       <c r="EC34" s="3" t="n">
         <v>236.6514</v>
       </c>
+      <c r="ED34" s="3" t="n">
+        <v>236.6514</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -22693,6 +22843,9 @@
       <c r="EC35" s="3" t="n">
         <v>15.84</v>
       </c>
+      <c r="ED35" s="3" t="n">
+        <v>15.84</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -23097,6 +23250,9 @@
       <c r="EC36" s="3" t="n">
         <v>364.6221</v>
       </c>
+      <c r="ED36" s="3" t="n">
+        <v>364.6221</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -23501,6 +23657,9 @@
       <c r="EC37" s="3" t="n">
         <v>16.628</v>
       </c>
+      <c r="ED37" s="3" t="n">
+        <v>16.628</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -23902,6 +24061,9 @@
       <c r="EC38" s="3" t="n">
         <v>13.7453</v>
       </c>
+      <c r="ED38" s="3" t="n">
+        <v>13.7453</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -24303,6 +24465,9 @@
       <c r="EC39" s="3" t="n">
         <v>1025.5891</v>
       </c>
+      <c r="ED39" s="3" t="n">
+        <v>1025.5891</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -24705,6 +24870,9 @@
         <v>20.5476</v>
       </c>
       <c r="EC40" s="3" t="n">
+        <v>20.5476</v>
+      </c>
+      <c r="ED40" s="3" t="n">
         <v>20.5476</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-20
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,8 +483,8 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-19 07:16 IST</t>
+          <t>Generated: 2026-10-20 07:06 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4948355.3351537</v>
+        <v>4900391.678336699</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>478355.3351536999</v>
+        <v>430391.6783366995</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.107014616365481</v>
+        <v>0.09628449179791936</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>530627.9961853027</v>
+        <v>530933.5044555664</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-60154.02381469728</v>
+        <v>-59848.51554443361</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.101821013128831</v>
+        <v>-0.101303887928806</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5478983.331339003</v>
+        <v>5431325.182792266</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>418201.311339003</v>
+        <v>370543.1627922663</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08263570920191561</v>
+        <v>0.0732185581848606</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-19</t>
+          <t>Last snapshot: 2026-10-20</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FH19"/>
+  <dimension ref="A1:FI19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -783,6 +783,7 @@
     <col width="21" customWidth="1" min="162" max="162"/>
     <col width="21" customWidth="1" min="163" max="163"/>
     <col width="21" customWidth="1" min="164" max="164"/>
+    <col width="21" customWidth="1" min="165" max="165"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1606,6 +1607,11 @@
           <t>2026-10-19</t>
         </is>
       </c>
+      <c r="FI1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1625,13 +1631,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>562.2999877929688</v>
+        <v>563.9000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44983.9990234375</v>
+        <v>45112.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1166.489023437498</v>
+        <v>1294.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2100,6 +2106,9 @@
       </c>
       <c r="FH2" s="3" t="n">
         <v>562.2999877929688</v>
+      </c>
+      <c r="FI2" s="3" t="n">
+        <v>563.9000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -2147,13 +2156,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1430</v>
+        <v>1428</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28600</v>
+        <v>28560</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3504.580000000002</v>
+        <v>-3544.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2625,6 +2634,9 @@
       </c>
       <c r="FH4" s="3" t="n">
         <v>1430</v>
+      </c>
+      <c r="FI4" s="3" t="n">
+        <v>1428</v>
       </c>
     </row>
     <row r="5">
@@ -2645,13 +2657,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>464.2000122070312</v>
+        <v>466.3999938964844</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9284.000244140625</v>
+        <v>9327.999877929688</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4929.099755859375</v>
+        <v>-4885.100122070313</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3123,6 +3135,9 @@
       </c>
       <c r="FH5" s="3" t="n">
         <v>464.2000122070312</v>
+      </c>
+      <c r="FI5" s="3" t="n">
+        <v>466.3999938964844</v>
       </c>
     </row>
     <row r="6">
@@ -3143,13 +3158,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>369.8999938964844</v>
+        <v>368.3500061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14795.99975585938</v>
+        <v>14734.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2706.240244140627</v>
+        <v>-2768.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3621,6 +3636,9 @@
       </c>
       <c r="FH6" s="3" t="n">
         <v>369.8999938964844</v>
+      </c>
+      <c r="FI6" s="3" t="n">
+        <v>368.3500061035156</v>
       </c>
     </row>
     <row r="7">
@@ -3641,13 +3659,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>270.75</v>
+        <v>269.8500061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>27075</v>
+        <v>26985.00061035156</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>641.1800000000003</v>
+        <v>551.1806103515628</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4119,6 +4137,9 @@
       </c>
       <c r="FH7" s="3" t="n">
         <v>270.75</v>
+      </c>
+      <c r="FI7" s="3" t="n">
+        <v>269.8500061035156</v>
       </c>
     </row>
     <row r="8">
@@ -4166,13 +4187,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.72999954223633</v>
+        <v>14.90999984741211</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22094.99931335449</v>
+        <v>22364.99977111816</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8955.170686645506</v>
+        <v>-8685.170228881834</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4644,6 +4665,9 @@
       </c>
       <c r="FH9" s="3" t="n">
         <v>14.72999954223633</v>
+      </c>
+      <c r="FI9" s="3" t="n">
+        <v>14.90999984741211</v>
       </c>
     </row>
     <row r="10">
@@ -4664,13 +4688,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>446.2999877929688</v>
+        <v>449</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44629.99877929688</v>
+        <v>44900</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6868.481220703128</v>
+        <v>-6598.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5142,6 +5166,9 @@
       </c>
       <c r="FH10" s="3" t="n">
         <v>446.2999877929688</v>
+      </c>
+      <c r="FI10" s="3" t="n">
+        <v>449</v>
       </c>
     </row>
     <row r="11">
@@ -5162,13 +5189,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>18.42000007629395</v>
+        <v>18.1299991607666</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>18420.00007629395</v>
+        <v>18129.9991607666</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>8578.790076293946</v>
+        <v>8288.789160766602</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5640,6 +5667,9 @@
       </c>
       <c r="FH11" s="3" t="n">
         <v>18.42000007629395</v>
+      </c>
+      <c r="FI11" s="3" t="n">
+        <v>18.1299991607666</v>
       </c>
     </row>
     <row r="12">
@@ -5660,13 +5690,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2504.199951171875</v>
+        <v>2505.10009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25041.99951171875</v>
+        <v>25051.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2681.25048828125</v>
+        <v>-2672.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6138,6 +6168,9 @@
       </c>
       <c r="FH12" s="3" t="n">
         <v>2504.199951171875</v>
+      </c>
+      <c r="FI12" s="3" t="n">
+        <v>2505.10009765625</v>
       </c>
     </row>
     <row r="13">
@@ -6158,13 +6191,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>40.84000015258789</v>
+        <v>40.38000106811523</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>24504.00009155273</v>
+        <v>24228.00064086914</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-10527.75990844727</v>
+        <v>-10803.75935913086</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6636,6 +6669,9 @@
       </c>
       <c r="FH13" s="3" t="n">
         <v>40.84000015258789</v>
+      </c>
+      <c r="FI13" s="3" t="n">
+        <v>40.38000106811523</v>
       </c>
     </row>
     <row r="14">
@@ -6656,13 +6692,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>624.5</v>
+        <v>637.6500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31225</v>
+        <v>31882.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11237.51</v>
+        <v>-10580.00877929688</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7134,6 +7170,9 @@
       </c>
       <c r="FH14" s="3" t="n">
         <v>624.5</v>
+      </c>
+      <c r="FI14" s="3" t="n">
+        <v>637.6500244140625</v>
       </c>
     </row>
     <row r="15">
@@ -7208,13 +7247,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>460.4500122070312</v>
+        <v>453.25</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23022.50061035156</v>
+        <v>22662.5</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1267.970610351564</v>
+        <v>907.9700000000012</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7686,6 +7725,9 @@
       </c>
       <c r="FH17" s="3" t="n">
         <v>460.4500122070312</v>
+      </c>
+      <c r="FI17" s="3" t="n">
+        <v>453.25</v>
       </c>
     </row>
     <row r="18">
@@ -7706,13 +7748,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>351.7999877929688</v>
+        <v>352.25</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35179.99877929688</v>
+        <v>35225</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11460.82122070312</v>
+        <v>-11415.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8184,6 +8226,9 @@
       </c>
       <c r="FH18" s="3" t="n">
         <v>351.7999877929688</v>
+      </c>
+      <c r="FI18" s="3" t="n">
+        <v>352.25</v>
       </c>
     </row>
     <row r="19">
@@ -8196,10 +8241,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>530627.9961853027</v>
+        <v>530933.5044555664</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-60154.02381469728</v>
+        <v>-59848.51554443361</v>
       </c>
     </row>
   </sheetData>
@@ -8213,7 +8258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:ED41"/>
+  <dimension ref="A1:EE41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8224,7 +8269,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -8350,6 +8395,7 @@
     <col width="13" customWidth="1" min="132" max="132"/>
     <col width="13" customWidth="1" min="133" max="133"/>
     <col width="13" customWidth="1" min="134" max="134"/>
+    <col width="13" customWidth="1" min="135" max="135"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9023,6 +9069,11 @@
           <t>2026-10-19</t>
         </is>
       </c>
+      <c r="EE1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9047,16 +9098,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.2538</v>
+        <v>56.3747</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63143.8779316</v>
+        <v>63279.58600539999</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13143.8779316</v>
+        <v>13279.58600539999</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.262877558632</v>
+        <v>0.2655917201079999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9432,6 +9483,9 @@
       </c>
       <c r="ED2" s="3" t="n">
         <v>56.2538</v>
+      </c>
+      <c r="EE2" s="3" t="n">
+        <v>56.3747</v>
       </c>
     </row>
     <row r="3">
@@ -9457,16 +9511,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.7682</v>
+        <v>26.4406</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65721.63262660001</v>
+        <v>64917.30484780001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5721.632626600011</v>
+        <v>4917.304847800006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.09536054377666685</v>
+        <v>0.08195508079666676</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9836,6 +9890,9 @@
       </c>
       <c r="ED3" s="3" t="n">
         <v>26.7682</v>
+      </c>
+      <c r="EE3" s="3" t="n">
+        <v>26.4406</v>
       </c>
     </row>
     <row r="4">
@@ -10241,6 +10298,9 @@
       <c r="ED4" s="3" t="n">
         <v>12.08</v>
       </c>
+      <c r="EE4" s="3" t="n">
+        <v>12.08</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10265,16 +10325,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.2668</v>
+        <v>9.1593</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>170083.6626784</v>
+        <v>168110.5982184</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-39916.3373216</v>
+        <v>-41889.4017816</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1900777967695238</v>
+        <v>-0.1994733418171429</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10644,6 +10704,9 @@
       </c>
       <c r="ED5" s="3" t="n">
         <v>9.2668</v>
+      </c>
+      <c r="EE5" s="3" t="n">
+        <v>9.1593</v>
       </c>
     </row>
     <row r="6">
@@ -10669,16 +10732,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.1632</v>
+        <v>11.0962</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>47208.91604639999</v>
+        <v>46925.5745874</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-2791.083953600006</v>
+        <v>-3074.425412600001</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.05582167907200011</v>
+        <v>-0.06148850825200003</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -11054,6 +11117,9 @@
       </c>
       <c r="ED6" s="3" t="n">
         <v>11.1632</v>
+      </c>
+      <c r="EE6" s="3" t="n">
+        <v>11.0962</v>
       </c>
     </row>
     <row r="7">
@@ -11079,16 +11145,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.7586</v>
+        <v>33.3041</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74472.821944</v>
+        <v>73470.17676399999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14472.821944</v>
+        <v>13470.17676399999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2412136990666666</v>
+        <v>0.2245029460666665</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -11458,6 +11524,9 @@
       </c>
       <c r="ED7" s="3" t="n">
         <v>33.7586</v>
+      </c>
+      <c r="EE7" s="3" t="n">
+        <v>33.3041</v>
       </c>
     </row>
     <row r="8">
@@ -11483,16 +11552,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>35.1128</v>
+        <v>34.4229</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>56341.7530904</v>
+        <v>55234.7443797</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6341.753090400001</v>
+        <v>5234.744379700001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.126835061808</v>
+        <v>0.104694887594</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -11868,6 +11937,9 @@
       </c>
       <c r="ED8" s="3" t="n">
         <v>35.1128</v>
+      </c>
+      <c r="EE8" s="3" t="n">
+        <v>34.4229</v>
       </c>
     </row>
     <row r="9">
@@ -11893,16 +11965,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>39.6566</v>
+        <v>39.0912</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>127670.1804438</v>
+        <v>125849.9356416</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>27670.1804438</v>
+        <v>25849.93564160001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.276701804438</v>
+        <v>0.2584993564160001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -12272,6 +12344,9 @@
       </c>
       <c r="ED9" s="3" t="n">
         <v>39.6566</v>
+      </c>
+      <c r="EE9" s="3" t="n">
+        <v>39.0912</v>
       </c>
     </row>
     <row r="10">
@@ -12297,16 +12372,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49.1177</v>
+        <v>48.6714</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>139821.3427643</v>
+        <v>138550.8788526</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>39821.3427643</v>
+        <v>38550.8788526</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3982134276430001</v>
+        <v>0.385508788526</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -12676,6 +12751,9 @@
       </c>
       <c r="ED10" s="3" t="n">
         <v>49.1177</v>
+      </c>
+      <c r="EE10" s="3" t="n">
+        <v>48.6714</v>
       </c>
     </row>
     <row r="11">
@@ -12701,16 +12779,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>102.269</v>
+        <v>103.2508</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30774.685211</v>
+        <v>31070.1274852</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>774.685211</v>
+        <v>1070.127485199999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.02582284036666667</v>
+        <v>0.03567091617333329</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -13080,6 +13158,9 @@
       </c>
       <c r="ED11" s="3" t="n">
         <v>102.269</v>
+      </c>
+      <c r="EE11" s="3" t="n">
+        <v>103.2508</v>
       </c>
     </row>
     <row r="12">
@@ -13105,16 +13186,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>221.058</v>
+        <v>219.784</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102907.362276</v>
+        <v>102314.287248</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2907.362276</v>
+        <v>2314.287247999993</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02907362276</v>
+        <v>0.02314287247999993</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -13490,6 +13571,9 @@
       </c>
       <c r="ED12" s="3" t="n">
         <v>221.058</v>
+      </c>
+      <c r="EE12" s="3" t="n">
+        <v>219.784</v>
       </c>
     </row>
     <row r="13">
@@ -13515,16 +13599,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.23</v>
+        <v>20.956</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>246004.85415</v>
+        <v>242829.85038</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>46004.85415</v>
+        <v>42829.85037999999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.23002427075</v>
+        <v>0.2141492518999999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -13900,6 +13984,9 @@
       </c>
       <c r="ED13" s="3" t="n">
         <v>21.23</v>
+      </c>
+      <c r="EE13" s="3" t="n">
+        <v>20.956</v>
       </c>
     </row>
     <row r="14">
@@ -14305,6 +14392,9 @@
       <c r="ED14" s="3" t="n">
         <v>35.7137</v>
       </c>
+      <c r="EE14" s="3" t="n">
+        <v>35.7137</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14329,16 +14419,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.25</v>
+        <v>11.16</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>109619.40375</v>
+        <v>108742.44852</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>9619.403749999998</v>
+        <v>8742.448520000005</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.09619403749999998</v>
+        <v>0.08742448520000005</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -14714,6 +14804,9 @@
       </c>
       <c r="ED15" s="3" t="n">
         <v>11.25</v>
+      </c>
+      <c r="EE15" s="3" t="n">
+        <v>11.16</v>
       </c>
     </row>
     <row r="16">
@@ -14739,16 +14832,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.1085</v>
+        <v>24.3251</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>137971.209688</v>
+        <v>139210.7958928</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>37971.209688</v>
+        <v>39210.7958928</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.37971209688</v>
+        <v>0.392107958928</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -15118,6 +15211,9 @@
       </c>
       <c r="ED16" s="3" t="n">
         <v>24.1085</v>
+      </c>
+      <c r="EE16" s="3" t="n">
+        <v>24.3251</v>
       </c>
     </row>
     <row r="17">
@@ -15143,16 +15239,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8084</v>
+        <v>16.6996</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55569.52847879999</v>
+        <v>55209.8294772</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5569.528478799992</v>
+        <v>5209.829477200001</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1113905695759998</v>
+        <v>0.104196589544</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -15522,6 +15618,9 @@
       </c>
       <c r="ED17" s="3" t="n">
         <v>16.8084</v>
+      </c>
+      <c r="EE17" s="3" t="n">
+        <v>16.6996</v>
       </c>
     </row>
     <row r="18">
@@ -15547,16 +15646,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.81</v>
+        <v>44.43</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84531.19716</v>
+        <v>83814.35148</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4531.197159999996</v>
+        <v>3814.351479999998</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.05663996449999995</v>
+        <v>0.04767939349999997</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -15932,6 +16031,9 @@
       </c>
       <c r="ED18" s="3" t="n">
         <v>44.81</v>
+      </c>
+      <c r="EE18" s="3" t="n">
+        <v>44.43</v>
       </c>
     </row>
     <row r="19">
@@ -15957,16 +16059,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>12.1823</v>
+        <v>11.8479</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>176238.4834418</v>
+        <v>171400.7968914</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>26238.4834418</v>
+        <v>21400.79689139998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.1749232229453333</v>
+        <v>0.1426719792759999</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -16336,6 +16438,9 @@
       </c>
       <c r="ED19" s="3" t="n">
         <v>12.1823</v>
+      </c>
+      <c r="EE19" s="3" t="n">
+        <v>11.8479</v>
       </c>
     </row>
     <row r="20">
@@ -16361,16 +16466,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.24</v>
+        <v>10.11</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>268859.42272</v>
+        <v>265446.16833</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>18859.42272000003</v>
+        <v>15446.16832999996</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.07543769088000013</v>
+        <v>0.06178467331999983</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -16746,6 +16851,9 @@
       </c>
       <c r="ED20" s="3" t="n">
         <v>10.24</v>
+      </c>
+      <c r="EE20" s="3" t="n">
+        <v>10.11</v>
       </c>
     </row>
     <row r="21">
@@ -16771,16 +16879,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.6656</v>
+        <v>110.2491</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>169648.9677904</v>
+        <v>167496.9374169</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-351.0322096000018</v>
+        <v>-2503.062583099992</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.002064895350588246</v>
+        <v>-0.01472389754764701</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -17156,6 +17264,9 @@
       </c>
       <c r="ED21" s="3" t="n">
         <v>111.6656</v>
+      </c>
+      <c r="EE21" s="3" t="n">
+        <v>110.2491</v>
       </c>
     </row>
     <row r="22">
@@ -17181,16 +17292,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>40.62</v>
+        <v>40.368</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>62329.76519999999</v>
+        <v>61943.08128000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>2329.765199999994</v>
+        <v>1943.081280000006</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.03882941999999991</v>
+        <v>0.0323846880000001</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -17560,6 +17671,9 @@
       </c>
       <c r="ED22" s="3" t="n">
         <v>40.62</v>
+      </c>
+      <c r="EE22" s="3" t="n">
+        <v>40.368</v>
       </c>
     </row>
     <row r="23">
@@ -17585,16 +17699,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.8286</v>
+        <v>60.1458</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>165238.8845562</v>
+        <v>163384.0808886</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>15238.88455620001</v>
+        <v>13384.0808886</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.101592563708</v>
+        <v>0.08922720592400001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -17970,6 +18084,9 @@
       </c>
       <c r="ED23" s="3" t="n">
         <v>60.8286</v>
+      </c>
+      <c r="EE23" s="3" t="n">
+        <v>60.1458</v>
       </c>
     </row>
     <row r="24">
@@ -17995,16 +18112,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.9235</v>
+        <v>25.9424</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>94190.08197100001</v>
+        <v>94258.7529664</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-5809.918028999993</v>
+        <v>-5741.247033599997</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.05809918028999993</v>
+        <v>-0.05741247033599997</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -18374,6 +18491,9 @@
       </c>
       <c r="ED24" s="3" t="n">
         <v>25.9235</v>
+      </c>
+      <c r="EE24" s="3" t="n">
+        <v>25.9424</v>
       </c>
     </row>
     <row r="25">
@@ -18399,16 +18519,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.5727</v>
+        <v>12.3748</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>206464.7806998</v>
+        <v>203214.9314152</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>6464.780699799972</v>
+        <v>3214.931415200001</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0.03232390349899986</v>
+        <v>0.016074657076</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -18778,6 +18898,9 @@
       </c>
       <c r="ED25" s="3" t="n">
         <v>12.5727</v>
+      </c>
+      <c r="EE25" s="3" t="n">
+        <v>12.3748</v>
       </c>
     </row>
     <row r="26">
@@ -18803,16 +18926,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.1334</v>
+        <v>10.9554</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>132951.889781</v>
+        <v>130826.264511</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>22951.88978100001</v>
+        <v>20826.26451099999</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.2086535434636364</v>
+        <v>0.1893296773727272</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -19185,6 +19308,9 @@
       </c>
       <c r="ED26" s="3" t="n">
         <v>11.1334</v>
+      </c>
+      <c r="EE26" s="3" t="n">
+        <v>10.9554</v>
       </c>
     </row>
     <row r="27">
@@ -19210,16 +19336,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>68.7869</v>
+        <v>68.0258</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>110806.065734</v>
-      </c>
-      <c r="H27" s="4" t="n">
-        <v>806.0657340000034</v>
-      </c>
-      <c r="I27" s="12" t="n">
-        <v>0.007327870309090941</v>
+        <v>109580.040188</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>-419.959812000001</v>
+      </c>
+      <c r="I27" s="13" t="n">
+        <v>-0.003817816472727282</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -19592,6 +19718,9 @@
       </c>
       <c r="ED27" s="3" t="n">
         <v>68.7869</v>
+      </c>
+      <c r="EE27" s="3" t="n">
+        <v>68.0258</v>
       </c>
     </row>
     <row r="28">
@@ -19617,16 +19746,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>114.9642</v>
+        <v>113.9108</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>380147.1766794</v>
-      </c>
-      <c r="H28" s="4" t="n">
-        <v>147.1766794000287</v>
-      </c>
-      <c r="I28" s="12" t="n">
-        <v>0.000387307051052707</v>
+        <v>376663.9441956</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>-3336.055804400006</v>
+      </c>
+      <c r="I28" s="13" t="n">
+        <v>-0.00877909422210528</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -20002,6 +20131,9 @@
       </c>
       <c r="ED28" s="3" t="n">
         <v>114.9642</v>
+      </c>
+      <c r="EE28" s="3" t="n">
+        <v>113.9108</v>
       </c>
     </row>
     <row r="29">
@@ -20027,16 +20159,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.0605</v>
+        <v>11.947</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>115825.4600315</v>
+        <v>114735.439741</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>15825.46003149998</v>
+        <v>14735.43974099998</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1582546003149999</v>
+        <v>0.1473543974099998</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -20406,6 +20538,9 @@
       </c>
       <c r="ED29" s="3" t="n">
         <v>12.0605</v>
+      </c>
+      <c r="EE29" s="3" t="n">
+        <v>11.947</v>
       </c>
     </row>
     <row r="30">
@@ -20431,16 +20566,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.2022</v>
+        <v>17.0271</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>127225.0800942</v>
+        <v>125930.0648331</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>27225.08009420001</v>
+        <v>25930.0648331</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.272250800942</v>
+        <v>0.259300648331</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -20810,6 +20945,9 @@
       </c>
       <c r="ED30" s="3" t="n">
         <v>17.2022</v>
+      </c>
+      <c r="EE30" s="3" t="n">
+        <v>17.0271</v>
       </c>
     </row>
     <row r="31">
@@ -20835,16 +20973,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>395.4481</v>
+        <v>390.3477</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>105220.830448</v>
+        <v>103863.716016</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>5220.830447999993</v>
+        <v>3863.716015999991</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.05220830447999993</v>
+        <v>0.03863716015999991</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -21217,6 +21355,9 @@
       </c>
       <c r="ED31" s="3" t="n">
         <v>395.4481</v>
+      </c>
+      <c r="EE31" s="3" t="n">
+        <v>390.3477</v>
       </c>
     </row>
     <row r="32">
@@ -21242,16 +21383,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.66</v>
+        <v>10.56</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>225351.9736</v>
+        <v>223237.9776</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>25351.9736</v>
+        <v>23237.97760000001</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.126759868</v>
+        <v>0.1161898880000001</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -21627,6 +21768,9 @@
       </c>
       <c r="ED32" s="3" t="n">
         <v>10.66</v>
+      </c>
+      <c r="EE32" s="3" t="n">
+        <v>10.56</v>
       </c>
     </row>
     <row r="33">
@@ -21652,16 +21796,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.43</v>
+        <v>19.24</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>69630.12519999999</v>
+        <v>68949.23359999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>9630.125199999995</v>
+        <v>8949.233599999992</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1605020866666666</v>
+        <v>0.1491538933333332</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -22031,6 +22175,9 @@
       </c>
       <c r="ED33" s="3" t="n">
         <v>19.43</v>
+      </c>
+      <c r="EE33" s="3" t="n">
+        <v>19.24</v>
       </c>
     </row>
     <row r="34">
@@ -22056,16 +22203,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>236.6514</v>
+        <v>233.693</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>83190.30329339999</v>
+        <v>82150.333983</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>3190.303293399993</v>
+        <v>2150.333983000004</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.03987879116749991</v>
+        <v>0.02687917478750005</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -22438,6 +22585,9 @@
       </c>
       <c r="ED34" s="3" t="n">
         <v>236.6514</v>
+      </c>
+      <c r="EE34" s="3" t="n">
+        <v>233.693</v>
       </c>
     </row>
     <row r="35">
@@ -22463,16 +22613,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.84</v>
+        <v>15.72</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>113025.10032</v>
+        <v>112168.84956</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>13025.10032</v>
+        <v>12168.84956</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1302510032</v>
+        <v>0.1216884956</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -22845,6 +22995,9 @@
       </c>
       <c r="ED35" s="3" t="n">
         <v>15.84</v>
+      </c>
+      <c r="EE35" s="3" t="n">
+        <v>15.72</v>
       </c>
     </row>
     <row r="36">
@@ -22870,16 +23023,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>364.6221</v>
+        <v>360.8055</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>169806.6997026</v>
+        <v>168029.286183</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>19806.69970259999</v>
+        <v>18029.28618300002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1320446646839999</v>
+        <v>0.1201952412200001</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -23252,6 +23405,9 @@
       </c>
       <c r="ED36" s="3" t="n">
         <v>364.6221</v>
+      </c>
+      <c r="EE36" s="3" t="n">
+        <v>360.8055</v>
       </c>
     </row>
     <row r="37">
@@ -23277,16 +23433,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.628</v>
+        <v>16.477</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62569.318292</v>
+        <v>62001.12205300001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12569.318292</v>
+        <v>12001.12205300001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2513863658400001</v>
+        <v>0.2400224410600001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -23659,6 +23815,9 @@
       </c>
       <c r="ED37" s="3" t="n">
         <v>16.628</v>
+      </c>
+      <c r="EE37" s="3" t="n">
+        <v>16.477</v>
       </c>
     </row>
     <row r="38">
@@ -23684,16 +23843,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.7453</v>
+        <v>13.6028</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>82203.5192346</v>
+        <v>81351.3005496</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>2203.519234599997</v>
+        <v>1351.300549599997</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.02754399043249996</v>
+        <v>0.01689125686999996</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -24063,6 +24222,9 @@
       </c>
       <c r="ED38" s="3" t="n">
         <v>13.7453</v>
+      </c>
+      <c r="EE38" s="3" t="n">
+        <v>13.6028</v>
       </c>
     </row>
     <row r="39">
@@ -24088,16 +24250,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.5891</v>
+        <v>1025.184</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51157.4098971</v>
+        <v>51137.203104</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1157.409897099998</v>
+        <v>1137.203104</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02314819794199997</v>
+        <v>0.02274406208</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -24467,6 +24629,9 @@
       </c>
       <c r="ED39" s="3" t="n">
         <v>1025.5891</v>
+      </c>
+      <c r="EE39" s="3" t="n">
+        <v>1025.184</v>
       </c>
     </row>
     <row r="40">
@@ -24492,16 +24657,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.5476</v>
+        <v>20.2818</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>103581.0063852</v>
+        <v>102241.1014086</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>3581.006385200002</v>
+        <v>2241.101408600007</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.03581006385200002</v>
+        <v>0.02241101408600007</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -24874,6 +25039,9 @@
       </c>
       <c r="ED40" s="3" t="n">
         <v>20.5476</v>
+      </c>
+      <c r="EE40" s="3" t="n">
+        <v>20.2818</v>
       </c>
     </row>
     <row r="41">
@@ -24886,13 +25054,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4948355.3351537</v>
+        <v>4900391.678336699</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>478355.3351537</v>
+        <v>430391.6783367</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.107014616365481</v>
+        <v>0.09628449179791945</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-21
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-20 07:06 IST</t>
+          <t>Generated: 2026-10-21 06:59 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>530933.5044555664</v>
+        <v>522320.0019340515</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-59848.51554443361</v>
+        <v>-68462.0180659485</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.101303887928806</v>
+        <v>-0.115883719795583</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5431325.182792266</v>
+        <v>5422711.680270751</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>370543.1627922663</v>
+        <v>361929.6602707515</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.0732185581848606</v>
+        <v>0.07151654800392913</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-20</t>
+          <t>Last snapshot: 2026-10-21</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FI19"/>
+  <dimension ref="A1:FJ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -784,6 +784,7 @@
     <col width="21" customWidth="1" min="163" max="163"/>
     <col width="21" customWidth="1" min="164" max="164"/>
     <col width="21" customWidth="1" min="165" max="165"/>
+    <col width="21" customWidth="1" min="166" max="166"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1612,6 +1613,11 @@
           <t>2026-10-20</t>
         </is>
       </c>
+      <c r="FJ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1631,13 +1637,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>563.9000244140625</v>
+        <v>550</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45112.001953125</v>
+        <v>44000</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1294.491953124998</v>
+        <v>182.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2109,6 +2115,9 @@
       </c>
       <c r="FI2" s="3" t="n">
         <v>563.9000244140625</v>
+      </c>
+      <c r="FJ2" s="3" t="n">
+        <v>550</v>
       </c>
     </row>
     <row r="3">
@@ -2156,13 +2165,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1428</v>
+        <v>1393.699951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28560</v>
+        <v>27873.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3544.580000000002</v>
+        <v>-4230.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2637,6 +2646,9 @@
       </c>
       <c r="FI4" s="3" t="n">
         <v>1428</v>
+      </c>
+      <c r="FJ4" s="3" t="n">
+        <v>1393.699951171875</v>
       </c>
     </row>
     <row r="5">
@@ -2657,13 +2669,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>466.3999938964844</v>
+        <v>466.5</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9327.999877929688</v>
+        <v>9330</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4885.100122070313</v>
+        <v>-4883.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3138,6 +3150,9 @@
       </c>
       <c r="FI5" s="3" t="n">
         <v>466.3999938964844</v>
+      </c>
+      <c r="FJ5" s="3" t="n">
+        <v>466.5</v>
       </c>
     </row>
     <row r="6">
@@ -3158,13 +3173,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>368.3500061035156</v>
+        <v>365.2999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14734.00024414062</v>
+        <v>14611.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2768.239755859377</v>
+        <v>-2890.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3639,6 +3654,9 @@
       </c>
       <c r="FI6" s="3" t="n">
         <v>368.3500061035156</v>
+      </c>
+      <c r="FJ6" s="3" t="n">
+        <v>365.2999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -3659,13 +3677,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>269.8500061035156</v>
+        <v>258.9500122070312</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>26985.00061035156</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>551.1806103515628</v>
+        <v>25895.00122070312</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>-538.8187792968747</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4140,6 +4158,9 @@
       </c>
       <c r="FI7" s="3" t="n">
         <v>269.8500061035156</v>
+      </c>
+      <c r="FJ7" s="3" t="n">
+        <v>258.9500122070312</v>
       </c>
     </row>
     <row r="8">
@@ -4187,13 +4208,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14.90999984741211</v>
+        <v>13.89000034332275</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>22364.99977111816</v>
+        <v>20835.00051498413</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-8685.170228881834</v>
+        <v>-10215.16948501587</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4668,6 +4689,9 @@
       </c>
       <c r="FI9" s="3" t="n">
         <v>14.90999984741211</v>
+      </c>
+      <c r="FJ9" s="3" t="n">
+        <v>13.89000034332275</v>
       </c>
     </row>
     <row r="10">
@@ -4688,13 +4712,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>449</v>
+        <v>449.4500122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44900</v>
+        <v>44945.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6598.480000000003</v>
+        <v>-6553.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5169,6 +5193,9 @@
       </c>
       <c r="FI10" s="3" t="n">
         <v>449</v>
+      </c>
+      <c r="FJ10" s="3" t="n">
+        <v>449.4500122070312</v>
       </c>
     </row>
     <row r="11">
@@ -5189,13 +5216,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>18.1299991607666</v>
+        <v>18.51000022888184</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>18129.9991607666</v>
+        <v>18510.00022888184</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>8288.789160766602</v>
+        <v>8668.790228881837</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5670,6 +5697,9 @@
       </c>
       <c r="FI11" s="3" t="n">
         <v>18.1299991607666</v>
+      </c>
+      <c r="FJ11" s="3" t="n">
+        <v>18.51000022888184</v>
       </c>
     </row>
     <row r="12">
@@ -5690,13 +5720,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2505.10009765625</v>
+        <v>2408.60009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25051.0009765625</v>
+        <v>24086.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2672.2490234375</v>
+        <v>-3637.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6171,6 +6201,9 @@
       </c>
       <c r="FI12" s="3" t="n">
         <v>2505.10009765625</v>
+      </c>
+      <c r="FJ12" s="3" t="n">
+        <v>2408.60009765625</v>
       </c>
     </row>
     <row r="13">
@@ -6191,13 +6224,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>40.38000106811523</v>
+        <v>39.04999923706055</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>24228.00064086914</v>
+        <v>23429.99954223633</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-10803.75935913086</v>
+        <v>-11601.76045776367</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6672,6 +6705,9 @@
       </c>
       <c r="FI13" s="3" t="n">
         <v>40.38000106811523</v>
+      </c>
+      <c r="FJ13" s="3" t="n">
+        <v>39.04999923706055</v>
       </c>
     </row>
     <row r="14">
@@ -6692,13 +6728,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>637.6500244140625</v>
+        <v>616.3499755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>31882.50122070312</v>
+        <v>30817.49877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-10580.00877929688</v>
+        <v>-11645.01122070313</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7173,6 +7209,9 @@
       </c>
       <c r="FI14" s="3" t="n">
         <v>637.6500244140625</v>
+      </c>
+      <c r="FJ14" s="3" t="n">
+        <v>616.3499755859375</v>
       </c>
     </row>
     <row r="15">
@@ -7247,13 +7286,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>453.25</v>
+        <v>428.3999938964844</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>22662.5</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>907.9700000000012</v>
+        <v>21419.99969482422</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>-334.5303051757801</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7728,6 +7767,9 @@
       </c>
       <c r="FI17" s="3" t="n">
         <v>453.25</v>
+      </c>
+      <c r="FJ17" s="3" t="n">
+        <v>428.3999938964844</v>
       </c>
     </row>
     <row r="18">
@@ -7748,13 +7790,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>352.25</v>
+        <v>347.9500122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35225</v>
+        <v>34795.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11415.82</v>
+        <v>-11845.81877929687</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8229,6 +8271,9 @@
       </c>
       <c r="FI18" s="3" t="n">
         <v>352.25</v>
+      </c>
+      <c r="FJ18" s="3" t="n">
+        <v>347.9500122070312</v>
       </c>
     </row>
     <row r="19">
@@ -8241,10 +8286,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>530933.5044555664</v>
+        <v>522320.0019340515</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-59848.51554443361</v>
+        <v>-68462.01806594849</v>
       </c>
     </row>
   </sheetData>
@@ -8258,7 +8303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EE41"/>
+  <dimension ref="A1:EF41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8396,6 +8441,7 @@
     <col width="13" customWidth="1" min="133" max="133"/>
     <col width="13" customWidth="1" min="134" max="134"/>
     <col width="13" customWidth="1" min="135" max="135"/>
+    <col width="13" customWidth="1" min="136" max="136"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9074,6 +9120,11 @@
           <t>2026-10-20</t>
         </is>
       </c>
+      <c r="EF1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9487,6 +9538,9 @@
       <c r="EE2" s="3" t="n">
         <v>56.3747</v>
       </c>
+      <c r="EF2" s="3" t="n">
+        <v>56.3747</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9894,6 +9948,9 @@
       <c r="EE3" s="3" t="n">
         <v>26.4406</v>
       </c>
+      <c r="EF3" s="3" t="n">
+        <v>26.4406</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10301,6 +10358,9 @@
       <c r="EE4" s="3" t="n">
         <v>12.08</v>
       </c>
+      <c r="EF4" s="3" t="n">
+        <v>12.08</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10708,6 +10768,9 @@
       <c r="EE5" s="3" t="n">
         <v>9.1593</v>
       </c>
+      <c r="EF5" s="3" t="n">
+        <v>9.1593</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11121,6 +11184,9 @@
       <c r="EE6" s="3" t="n">
         <v>11.0962</v>
       </c>
+      <c r="EF6" s="3" t="n">
+        <v>11.0962</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11528,6 +11594,9 @@
       <c r="EE7" s="3" t="n">
         <v>33.3041</v>
       </c>
+      <c r="EF7" s="3" t="n">
+        <v>33.3041</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11941,6 +12010,9 @@
       <c r="EE8" s="3" t="n">
         <v>34.4229</v>
       </c>
+      <c r="EF8" s="3" t="n">
+        <v>34.4229</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12348,6 +12420,9 @@
       <c r="EE9" s="3" t="n">
         <v>39.0912</v>
       </c>
+      <c r="EF9" s="3" t="n">
+        <v>39.0912</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12755,6 +12830,9 @@
       <c r="EE10" s="3" t="n">
         <v>48.6714</v>
       </c>
+      <c r="EF10" s="3" t="n">
+        <v>48.6714</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13162,6 +13240,9 @@
       <c r="EE11" s="3" t="n">
         <v>103.2508</v>
       </c>
+      <c r="EF11" s="3" t="n">
+        <v>103.2508</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13575,6 +13656,9 @@
       <c r="EE12" s="3" t="n">
         <v>219.784</v>
       </c>
+      <c r="EF12" s="3" t="n">
+        <v>219.784</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13988,6 +14072,9 @@
       <c r="EE13" s="3" t="n">
         <v>20.956</v>
       </c>
+      <c r="EF13" s="3" t="n">
+        <v>20.956</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14395,6 +14482,9 @@
       <c r="EE14" s="3" t="n">
         <v>35.7137</v>
       </c>
+      <c r="EF14" s="3" t="n">
+        <v>35.7137</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14808,6 +14898,9 @@
       <c r="EE15" s="3" t="n">
         <v>11.16</v>
       </c>
+      <c r="EF15" s="3" t="n">
+        <v>11.16</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15215,6 +15308,9 @@
       <c r="EE16" s="3" t="n">
         <v>24.3251</v>
       </c>
+      <c r="EF16" s="3" t="n">
+        <v>24.3251</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -15622,6 +15718,9 @@
       <c r="EE17" s="3" t="n">
         <v>16.6996</v>
       </c>
+      <c r="EF17" s="3" t="n">
+        <v>16.6996</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -16035,6 +16134,9 @@
       <c r="EE18" s="3" t="n">
         <v>44.43</v>
       </c>
+      <c r="EF18" s="3" t="n">
+        <v>44.43</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -16442,6 +16544,9 @@
       <c r="EE19" s="3" t="n">
         <v>11.8479</v>
       </c>
+      <c r="EF19" s="3" t="n">
+        <v>11.8479</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -16855,6 +16960,9 @@
       <c r="EE20" s="3" t="n">
         <v>10.11</v>
       </c>
+      <c r="EF20" s="3" t="n">
+        <v>10.11</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -17268,6 +17376,9 @@
       <c r="EE21" s="3" t="n">
         <v>110.2491</v>
       </c>
+      <c r="EF21" s="3" t="n">
+        <v>110.2491</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -17675,6 +17786,9 @@
       <c r="EE22" s="3" t="n">
         <v>40.368</v>
       </c>
+      <c r="EF22" s="3" t="n">
+        <v>40.368</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -18088,6 +18202,9 @@
       <c r="EE23" s="3" t="n">
         <v>60.1458</v>
       </c>
+      <c r="EF23" s="3" t="n">
+        <v>60.1458</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -18495,6 +18612,9 @@
       <c r="EE24" s="3" t="n">
         <v>25.9424</v>
       </c>
+      <c r="EF24" s="3" t="n">
+        <v>25.9424</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -18902,6 +19022,9 @@
       <c r="EE25" s="3" t="n">
         <v>12.3748</v>
       </c>
+      <c r="EF25" s="3" t="n">
+        <v>12.3748</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -19312,6 +19435,9 @@
       <c r="EE26" s="3" t="n">
         <v>10.9554</v>
       </c>
+      <c r="EF26" s="3" t="n">
+        <v>10.9554</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -19722,6 +19848,9 @@
       <c r="EE27" s="3" t="n">
         <v>68.0258</v>
       </c>
+      <c r="EF27" s="3" t="n">
+        <v>68.0258</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -20135,6 +20264,9 @@
       <c r="EE28" s="3" t="n">
         <v>113.9108</v>
       </c>
+      <c r="EF28" s="3" t="n">
+        <v>113.9108</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -20542,6 +20674,9 @@
       <c r="EE29" s="3" t="n">
         <v>11.947</v>
       </c>
+      <c r="EF29" s="3" t="n">
+        <v>11.947</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -20949,6 +21084,9 @@
       <c r="EE30" s="3" t="n">
         <v>17.0271</v>
       </c>
+      <c r="EF30" s="3" t="n">
+        <v>17.0271</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -21359,6 +21497,9 @@
       <c r="EE31" s="3" t="n">
         <v>390.3477</v>
       </c>
+      <c r="EF31" s="3" t="n">
+        <v>390.3477</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -21772,6 +21913,9 @@
       <c r="EE32" s="3" t="n">
         <v>10.56</v>
       </c>
+      <c r="EF32" s="3" t="n">
+        <v>10.56</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -22179,6 +22323,9 @@
       <c r="EE33" s="3" t="n">
         <v>19.24</v>
       </c>
+      <c r="EF33" s="3" t="n">
+        <v>19.24</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -22589,6 +22736,9 @@
       <c r="EE34" s="3" t="n">
         <v>233.693</v>
       </c>
+      <c r="EF34" s="3" t="n">
+        <v>233.693</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -22999,6 +23149,9 @@
       <c r="EE35" s="3" t="n">
         <v>15.72</v>
       </c>
+      <c r="EF35" s="3" t="n">
+        <v>15.72</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -23409,6 +23562,9 @@
       <c r="EE36" s="3" t="n">
         <v>360.8055</v>
       </c>
+      <c r="EF36" s="3" t="n">
+        <v>360.8055</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -23819,6 +23975,9 @@
       <c r="EE37" s="3" t="n">
         <v>16.477</v>
       </c>
+      <c r="EF37" s="3" t="n">
+        <v>16.477</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -24226,6 +24385,9 @@
       <c r="EE38" s="3" t="n">
         <v>13.6028</v>
       </c>
+      <c r="EF38" s="3" t="n">
+        <v>13.6028</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -24633,6 +24795,9 @@
       <c r="EE39" s="3" t="n">
         <v>1025.184</v>
       </c>
+      <c r="EF39" s="3" t="n">
+        <v>1025.184</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -25041,6 +25206,9 @@
         <v>20.5476</v>
       </c>
       <c r="EE40" s="3" t="n">
+        <v>20.2818</v>
+      </c>
+      <c r="EF40" s="3" t="n">
         <v>20.2818</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-22
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-21 06:59 IST</t>
+          <t>Generated: 2026-10-22 07:02 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4900391.678336699</v>
+        <v>4861736.8311561</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>430391.6783366995</v>
+        <v>391736.8311561001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09628449179791936</v>
+        <v>0.08763687497899332</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>522320.0019340515</v>
+        <v>520045.0019340515</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-68462.0180659485</v>
+        <v>-70737.0180659485</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.115883719795583</v>
+        <v>-0.119734547889505</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5422711.680270751</v>
+        <v>5381781.833090152</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>361929.6602707515</v>
+        <v>320999.8130901521</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07151654800392913</v>
+        <v>0.06342889534099161</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-21</t>
+          <t>Last snapshot: 2026-10-22</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FJ19"/>
+  <dimension ref="A1:FK19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -785,6 +785,7 @@
     <col width="21" customWidth="1" min="164" max="164"/>
     <col width="21" customWidth="1" min="165" max="165"/>
     <col width="21" customWidth="1" min="166" max="166"/>
+    <col width="21" customWidth="1" min="167" max="167"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1618,6 +1619,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="FK1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1637,13 +1643,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>550</v>
+        <v>566.7000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44000</v>
+        <v>45336.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>182.489999999998</v>
+        <v>1518.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2118,6 +2124,9 @@
       </c>
       <c r="FJ2" s="3" t="n">
         <v>550</v>
+      </c>
+      <c r="FK2" s="3" t="n">
+        <v>566.7000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -2165,13 +2174,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1393.699951171875</v>
+        <v>1367.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27873.9990234375</v>
+        <v>27356.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4230.580976562502</v>
+        <v>-4748.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2649,6 +2658,9 @@
       </c>
       <c r="FJ4" s="3" t="n">
         <v>1393.699951171875</v>
+      </c>
+      <c r="FK4" s="3" t="n">
+        <v>1367.800048828125</v>
       </c>
     </row>
     <row r="5">
@@ -2669,13 +2681,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>466.5</v>
+        <v>462.3500061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9330</v>
+        <v>9247.000122070312</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4883.1</v>
+        <v>-4966.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3153,6 +3165,9 @@
       </c>
       <c r="FJ5" s="3" t="n">
         <v>466.5</v>
+      </c>
+      <c r="FK5" s="3" t="n">
+        <v>462.3500061035156</v>
       </c>
     </row>
     <row r="6">
@@ -3173,13 +3188,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>365.2999877929688</v>
+        <v>365.1499938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14611.99951171875</v>
+        <v>14605.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2890.240488281252</v>
+        <v>-2896.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3657,6 +3672,9 @@
       </c>
       <c r="FJ6" s="3" t="n">
         <v>365.2999877929688</v>
+      </c>
+      <c r="FK6" s="3" t="n">
+        <v>365.1499938964844</v>
       </c>
     </row>
     <row r="7">
@@ -3677,13 +3695,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>258.9500122070312</v>
+        <v>252.75</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25895.00122070312</v>
+        <v>25275</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-538.8187792968747</v>
+        <v>-1158.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4161,6 +4179,9 @@
       </c>
       <c r="FJ7" s="3" t="n">
         <v>258.9500122070312</v>
+      </c>
+      <c r="FK7" s="3" t="n">
+        <v>252.75</v>
       </c>
     </row>
     <row r="8">
@@ -4208,13 +4229,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>13.89000034332275</v>
+        <v>13.64000034332275</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>20835.00051498413</v>
+        <v>20460.00051498413</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-10215.16948501587</v>
+        <v>-10590.16948501587</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4692,6 +4713,9 @@
       </c>
       <c r="FJ9" s="3" t="n">
         <v>13.89000034332275</v>
+      </c>
+      <c r="FK9" s="3" t="n">
+        <v>13.64000034332275</v>
       </c>
     </row>
     <row r="10">
@@ -4712,13 +4736,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>449.4500122070312</v>
+        <v>451.4500122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44945.00122070312</v>
+        <v>45145.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6553.478779296878</v>
+        <v>-6353.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5196,6 +5220,9 @@
       </c>
       <c r="FJ10" s="3" t="n">
         <v>449.4500122070312</v>
+      </c>
+      <c r="FK10" s="3" t="n">
+        <v>451.4500122070312</v>
       </c>
     </row>
     <row r="11">
@@ -5216,13 +5243,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>18.51000022888184</v>
+        <v>17.78000068664551</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>18510.00022888184</v>
+        <v>17780.00068664551</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>8668.790228881837</v>
+        <v>7938.790686645509</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5700,6 +5727,9 @@
       </c>
       <c r="FJ11" s="3" t="n">
         <v>18.51000022888184</v>
+      </c>
+      <c r="FK11" s="3" t="n">
+        <v>17.78000068664551</v>
       </c>
     </row>
     <row r="12">
@@ -5720,13 +5750,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2408.60009765625</v>
+        <v>2378.699951171875</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>24086.0009765625</v>
+        <v>23786.99951171875</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-3637.2490234375</v>
+        <v>-3936.25048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6204,6 +6234,9 @@
       </c>
       <c r="FJ12" s="3" t="n">
         <v>2408.60009765625</v>
+      </c>
+      <c r="FK12" s="3" t="n">
+        <v>2378.699951171875</v>
       </c>
     </row>
     <row r="13">
@@ -6224,13 +6257,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>39.04999923706055</v>
+        <v>38.59999847412109</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23429.99954223633</v>
+        <v>23159.99908447266</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11601.76045776367</v>
+        <v>-11871.76091552735</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6708,6 +6741,9 @@
       </c>
       <c r="FJ13" s="3" t="n">
         <v>39.04999923706055</v>
+      </c>
+      <c r="FK13" s="3" t="n">
+        <v>38.59999847412109</v>
       </c>
     </row>
     <row r="14">
@@ -6728,13 +6764,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>616.3499755859375</v>
+        <v>594.7000122070312</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>30817.49877929688</v>
+        <v>29735.00061035156</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-11645.01122070313</v>
+        <v>-12727.50938964844</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7212,6 +7248,9 @@
       </c>
       <c r="FJ14" s="3" t="n">
         <v>616.3499755859375</v>
+      </c>
+      <c r="FK14" s="3" t="n">
+        <v>594.7000122070312</v>
       </c>
     </row>
     <row r="15">
@@ -7286,13 +7325,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>428.3999938964844</v>
+        <v>425.1499938964844</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>21419.99969482422</v>
+        <v>21257.49969482422</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-334.5303051757801</v>
+        <v>-497.0303051757801</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7770,6 +7809,9 @@
       </c>
       <c r="FJ17" s="3" t="n">
         <v>428.3999938964844</v>
+      </c>
+      <c r="FK17" s="3" t="n">
+        <v>425.1499938964844</v>
       </c>
     </row>
     <row r="18">
@@ -7790,13 +7832,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>347.9500122070312</v>
+        <v>351.2999877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34795.00122070312</v>
+        <v>35129.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11845.81877929687</v>
+        <v>-11510.82122070312</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8274,6 +8316,9 @@
       </c>
       <c r="FJ18" s="3" t="n">
         <v>347.9500122070312</v>
+      </c>
+      <c r="FK18" s="3" t="n">
+        <v>351.2999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -8286,10 +8331,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>522320.0019340515</v>
+        <v>520045.0019340515</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-68462.01806594849</v>
+        <v>-70737.01806594849</v>
       </c>
     </row>
   </sheetData>
@@ -8303,7 +8348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EF41"/>
+  <dimension ref="A1:EG41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8442,6 +8487,7 @@
     <col width="13" customWidth="1" min="134" max="134"/>
     <col width="13" customWidth="1" min="135" max="135"/>
     <col width="13" customWidth="1" min="136" max="136"/>
+    <col width="13" customWidth="1" min="137" max="137"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9125,6 +9171,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
+      <c r="EG1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9149,16 +9200,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.3747</v>
+        <v>56.6826</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63279.58600539999</v>
+        <v>63625.1982132</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13279.58600539999</v>
+        <v>13625.1982132</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2655917201079999</v>
+        <v>0.272503964264</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9540,6 +9591,9 @@
       </c>
       <c r="EF2" s="3" t="n">
         <v>56.3747</v>
+      </c>
+      <c r="EG2" s="3" t="n">
+        <v>56.6826</v>
       </c>
     </row>
     <row r="3">
@@ -9565,16 +9619,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.4406</v>
+        <v>26.5873</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>64917.30484780001</v>
+        <v>65277.4845949</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4917.304847800006</v>
+        <v>5277.484594900001</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.08195508079666676</v>
+        <v>0.08795807658166668</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -9950,6 +10004,9 @@
       </c>
       <c r="EF3" s="3" t="n">
         <v>26.4406</v>
+      </c>
+      <c r="EG3" s="3" t="n">
+        <v>26.5873</v>
       </c>
     </row>
     <row r="4">
@@ -9975,16 +10032,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.08</v>
+        <v>11.9</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>232009.60344</v>
+        <v>228552.5067</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>52009.60344000001</v>
+        <v>48552.50670000003</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2889422413333333</v>
+        <v>0.2697361483333335</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -10360,6 +10417,9 @@
       </c>
       <c r="EF4" s="3" t="n">
         <v>12.08</v>
+      </c>
+      <c r="EG4" s="3" t="n">
+        <v>11.9</v>
       </c>
     </row>
     <row r="5">
@@ -10385,16 +10445,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.1593</v>
+        <v>9.1172</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>168110.5982184</v>
+        <v>167337.8911136</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-41889.4017816</v>
+        <v>-42662.1088864</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1994733418171429</v>
+        <v>-0.2031528994590476</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10770,6 +10830,9 @@
       </c>
       <c r="EF5" s="3" t="n">
         <v>9.1593</v>
+      </c>
+      <c r="EG5" s="3" t="n">
+        <v>9.1172</v>
       </c>
     </row>
     <row r="6">
@@ -10795,16 +10858,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.0962</v>
+        <v>10.9827</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>46925.5745874</v>
+        <v>46445.58569789999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-3074.425412600001</v>
+        <v>-3554.414302100005</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.06148850825200003</v>
+        <v>-0.07108828604200011</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -11186,6 +11249,9 @@
       </c>
       <c r="EF6" s="3" t="n">
         <v>11.0962</v>
+      </c>
+      <c r="EG6" s="3" t="n">
+        <v>10.9827</v>
       </c>
     </row>
     <row r="7">
@@ -11211,16 +11277,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.3041</v>
+        <v>33.5796</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73470.17676399999</v>
+        <v>74077.94078399999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13470.17676399999</v>
+        <v>14077.94078399999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2245029460666665</v>
+        <v>0.2346323463999999</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -11596,6 +11662,9 @@
       </c>
       <c r="EF7" s="3" t="n">
         <v>33.3041</v>
+      </c>
+      <c r="EG7" s="3" t="n">
+        <v>33.5796</v>
       </c>
     </row>
     <row r="8">
@@ -11621,16 +11690,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>34.4229</v>
+        <v>33.4912</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>55234.7443797</v>
+        <v>53739.7450816</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5234.744379700001</v>
+        <v>3739.745081599998</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.104694887594</v>
+        <v>0.07479490163199996</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -12012,6 +12081,9 @@
       </c>
       <c r="EF8" s="3" t="n">
         <v>34.4229</v>
+      </c>
+      <c r="EG8" s="3" t="n">
+        <v>33.4912</v>
       </c>
     </row>
     <row r="9">
@@ -12037,16 +12109,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>39.0912</v>
+        <v>39.9284</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>125849.9356416</v>
+        <v>128545.2114612</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>25849.93564160001</v>
+        <v>28545.21146120002</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.2584993564160001</v>
+        <v>0.2854521146120002</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -12422,6 +12494,9 @@
       </c>
       <c r="EF9" s="3" t="n">
         <v>39.0912</v>
+      </c>
+      <c r="EG9" s="3" t="n">
+        <v>39.9284</v>
       </c>
     </row>
     <row r="10">
@@ -12447,16 +12522,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.6714</v>
+        <v>49.0611</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138550.8788526</v>
+        <v>139660.2218649</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38550.8788526</v>
+        <v>39660.22186490003</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.385508788526</v>
+        <v>0.3966022186490003</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -12832,6 +12907,9 @@
       </c>
       <c r="EF10" s="3" t="n">
         <v>48.6714</v>
+      </c>
+      <c r="EG10" s="3" t="n">
+        <v>49.0611</v>
       </c>
     </row>
     <row r="11">
@@ -12857,16 +12935,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>103.2508</v>
+        <v>103.6975</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31070.1274852</v>
+        <v>31204.5480025</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1070.127485199999</v>
+        <v>1204.5480025</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.03567091617333329</v>
+        <v>0.04015160008333332</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -13242,6 +13320,9 @@
       </c>
       <c r="EF11" s="3" t="n">
         <v>103.2508</v>
+      </c>
+      <c r="EG11" s="3" t="n">
+        <v>103.6975</v>
       </c>
     </row>
     <row r="12">
@@ -13267,16 +13348,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>219.784</v>
+        <v>217.782</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102314.287248</v>
+        <v>101382.312204</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2314.287247999993</v>
+        <v>1382.312204000002</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02314287247999993</v>
+        <v>0.01382312204000002</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -13658,6 +13739,9 @@
       </c>
       <c r="EF12" s="3" t="n">
         <v>219.784</v>
+      </c>
+      <c r="EG12" s="3" t="n">
+        <v>217.782</v>
       </c>
     </row>
     <row r="13">
@@ -13683,16 +13767,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.956</v>
+        <v>20.819</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>242829.85038</v>
+        <v>241242.348495</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>42829.85037999999</v>
+        <v>41242.34849499998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2141492518999999</v>
+        <v>0.2062117424749999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -14074,6 +14158,9 @@
       </c>
       <c r="EF13" s="3" t="n">
         <v>20.956</v>
+      </c>
+      <c r="EG13" s="3" t="n">
+        <v>20.819</v>
       </c>
     </row>
     <row r="14">
@@ -14099,16 +14186,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35.7137</v>
+        <v>35.499</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>128840.9584022</v>
+        <v>128066.405394</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>28840.95840220002</v>
+        <v>28066.40539400002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.2884095840220002</v>
+        <v>0.2806640539400002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -14484,6 +14571,9 @@
       </c>
       <c r="EF14" s="3" t="n">
         <v>35.7137</v>
+      </c>
+      <c r="EG14" s="3" t="n">
+        <v>35.499</v>
       </c>
     </row>
     <row r="15">
@@ -14509,16 +14599,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.16</v>
+        <v>10.95</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>108742.44852</v>
+        <v>106696.21965</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>8742.448520000005</v>
+        <v>6696.219649999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.08742448520000005</v>
+        <v>0.06696219649999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -14900,6 +14990,9 @@
       </c>
       <c r="EF15" s="3" t="n">
         <v>11.16</v>
+      </c>
+      <c r="EG15" s="3" t="n">
+        <v>10.95</v>
       </c>
     </row>
     <row r="16">
@@ -14925,16 +15018,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.3251</v>
+        <v>24.5514</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>139210.7958928</v>
+        <v>140505.8944992</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>39210.7958928</v>
+        <v>40505.89449919999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.392107958928</v>
+        <v>0.4050589449919999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -15310,6 +15403,9 @@
       </c>
       <c r="EF16" s="3" t="n">
         <v>24.3251</v>
+      </c>
+      <c r="EG16" s="3" t="n">
+        <v>24.5514</v>
       </c>
     </row>
     <row r="17">
@@ -15335,16 +15431,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6996</v>
+        <v>16.6436</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55209.8294772</v>
+        <v>55024.69028519999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5209.829477200001</v>
+        <v>5024.690285199991</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.104196589544</v>
+        <v>0.1004938057039998</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -15720,6 +15816,9 @@
       </c>
       <c r="EF17" s="3" t="n">
         <v>16.6996</v>
+      </c>
+      <c r="EG17" s="3" t="n">
+        <v>16.6436</v>
       </c>
     </row>
     <row r="18">
@@ -15745,16 +15844,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.43</v>
+        <v>44.12</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>83814.35148</v>
+        <v>83229.55631999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3814.351479999998</v>
+        <v>3229.556319999989</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.04767939349999997</v>
+        <v>0.04036945399999986</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -16136,6 +16235,9 @@
       </c>
       <c r="EF18" s="3" t="n">
         <v>44.43</v>
+      </c>
+      <c r="EG18" s="3" t="n">
+        <v>44.12</v>
       </c>
     </row>
     <row r="19">
@@ -16161,16 +16263,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.8479</v>
+        <v>11.9506</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>171400.7968914</v>
+        <v>172886.5337596</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>21400.79689139998</v>
+        <v>22886.53375959999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.1426719792759999</v>
+        <v>0.1525768917306666</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -16546,6 +16648,9 @@
       </c>
       <c r="EF19" s="3" t="n">
         <v>11.8479</v>
+      </c>
+      <c r="EG19" s="3" t="n">
+        <v>11.9506</v>
       </c>
     </row>
     <row r="20">
@@ -16571,16 +16676,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.11</v>
+        <v>10.17</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>265446.16833</v>
+        <v>267021.51651</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>15446.16832999996</v>
+        <v>17021.51650999999</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.06178467331999983</v>
+        <v>0.06808606603999995</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -16962,6 +17067,9 @@
       </c>
       <c r="EF20" s="3" t="n">
         <v>10.11</v>
+      </c>
+      <c r="EG20" s="3" t="n">
+        <v>10.17</v>
       </c>
     </row>
     <row r="21">
@@ -16987,16 +17095,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>110.2491</v>
+        <v>108.5689</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>167496.9374169</v>
+        <v>164944.2784451</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-2503.062583099992</v>
+        <v>-5055.721554899996</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.01472389754764701</v>
+        <v>-0.02973953855823527</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -17378,6 +17486,9 @@
       </c>
       <c r="EF21" s="3" t="n">
         <v>110.2491</v>
+      </c>
+      <c r="EG21" s="3" t="n">
+        <v>108.5689</v>
       </c>
     </row>
     <row r="22">
@@ -17403,16 +17514,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>40.368</v>
+        <v>40.388</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>61943.08128000001</v>
+        <v>61973.77048</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>1943.081280000006</v>
+        <v>1973.770479999999</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.0323846880000001</v>
+        <v>0.03289617466666665</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -17788,6 +17899,9 @@
       </c>
       <c r="EF22" s="3" t="n">
         <v>40.368</v>
+      </c>
+      <c r="EG22" s="3" t="n">
+        <v>40.388</v>
       </c>
     </row>
     <row r="23">
@@ -17813,16 +17927,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.1458</v>
+        <v>59.227</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>163384.0808886</v>
+        <v>160888.191009</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>13384.0808886</v>
+        <v>10888.191009</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.08922720592400001</v>
+        <v>0.07258794006000001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -18204,6 +18318,9 @@
       </c>
       <c r="EF23" s="3" t="n">
         <v>60.1458</v>
+      </c>
+      <c r="EG23" s="3" t="n">
+        <v>59.227</v>
       </c>
     </row>
     <row r="24">
@@ -18229,16 +18346,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.9424</v>
+        <v>25.7931</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>94258.7529664</v>
+        <v>93716.28843659999</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-5741.247033599997</v>
+        <v>-6283.711563400007</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.05741247033599997</v>
+        <v>-0.06283711563400007</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -18614,6 +18731,9 @@
       </c>
       <c r="EF24" s="3" t="n">
         <v>25.9424</v>
+      </c>
+      <c r="EG24" s="3" t="n">
+        <v>25.7931</v>
       </c>
     </row>
     <row r="25">
@@ -18639,16 +18759,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.3748</v>
+        <v>12.1453</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>203214.9314152</v>
-      </c>
-      <c r="H25" s="4" t="n">
-        <v>3214.931415200001</v>
-      </c>
-      <c r="I25" s="12" t="n">
-        <v>0.016074657076</v>
+        <v>199446.1572322</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>-553.8427678000007</v>
+      </c>
+      <c r="I25" s="13" t="n">
+        <v>-0.002769213839000004</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -19024,6 +19144,9 @@
       </c>
       <c r="EF25" s="3" t="n">
         <v>12.3748</v>
+      </c>
+      <c r="EG25" s="3" t="n">
+        <v>12.1453</v>
       </c>
     </row>
     <row r="26">
@@ -19049,16 +19172,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.9554</v>
+        <v>10.8427</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>130826.264511</v>
+        <v>129480.4332305</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>20826.26451099999</v>
+        <v>19480.43323050001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1893296773727272</v>
+        <v>0.1770948475500001</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -19437,6 +19560,9 @@
       </c>
       <c r="EF26" s="3" t="n">
         <v>10.9554</v>
+      </c>
+      <c r="EG26" s="3" t="n">
+        <v>10.8427</v>
       </c>
     </row>
     <row r="27">
@@ -19462,16 +19588,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>68.0258</v>
+        <v>66.8815</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>109580.040188</v>
+        <v>107736.73309</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-419.959812000001</v>
+        <v>-2263.266910000006</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.003817816472727282</v>
+        <v>-0.02057515372727278</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -19850,6 +19976,9 @@
       </c>
       <c r="EF27" s="3" t="n">
         <v>68.0258</v>
+      </c>
+      <c r="EG27" s="3" t="n">
+        <v>66.8815</v>
       </c>
     </row>
     <row r="28">
@@ -19875,16 +20004,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>113.9108</v>
+        <v>112.2117</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>376663.9441956</v>
+        <v>371045.6032869</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-3336.055804400006</v>
+        <v>-8954.396713100024</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.00877909422210528</v>
+        <v>-0.02356420187657901</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -20266,6 +20395,9 @@
       </c>
       <c r="EF28" s="3" t="n">
         <v>113.9108</v>
+      </c>
+      <c r="EG28" s="3" t="n">
+        <v>112.2117</v>
       </c>
     </row>
     <row r="29">
@@ -20291,16 +20423,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.947</v>
+        <v>11.6492</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114735.439741</v>
+        <v>111875.4569876</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14735.43974099998</v>
+        <v>11875.4569876</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1473543974099998</v>
+        <v>0.118754569876</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -20676,6 +20808,9 @@
       </c>
       <c r="EF29" s="3" t="n">
         <v>11.947</v>
+      </c>
+      <c r="EG29" s="3" t="n">
+        <v>11.6492</v>
       </c>
     </row>
     <row r="30">
@@ -20701,16 +20836,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>17.0271</v>
+        <v>16.6407</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>125930.0648331</v>
+        <v>123072.3041427</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>25930.0648331</v>
+        <v>23072.30414269998</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.259300648331</v>
+        <v>0.2307230414269998</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -21086,6 +21221,9 @@
       </c>
       <c r="EF30" s="3" t="n">
         <v>17.0271</v>
+      </c>
+      <c r="EG30" s="3" t="n">
+        <v>16.6407</v>
       </c>
     </row>
     <row r="31">
@@ -21111,16 +21249,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>390.3477</v>
+        <v>382.9721</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>103863.716016</v>
+        <v>101901.216368</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>3863.716015999991</v>
+        <v>1901.216367999994</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.03863716015999991</v>
+        <v>0.01901216367999994</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -21499,6 +21637,9 @@
       </c>
       <c r="EF31" s="3" t="n">
         <v>390.3477</v>
+      </c>
+      <c r="EG31" s="3" t="n">
+        <v>382.9721</v>
       </c>
     </row>
     <row r="32">
@@ -21524,16 +21665,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.56</v>
+        <v>10.4</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>223237.9776</v>
+        <v>219855.584</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>23237.97760000001</v>
+        <v>19855.584</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1161898880000001</v>
+        <v>0.09927792000000002</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -21915,6 +22056,9 @@
       </c>
       <c r="EF32" s="3" t="n">
         <v>10.56</v>
+      </c>
+      <c r="EG32" s="3" t="n">
+        <v>10.4</v>
       </c>
     </row>
     <row r="33">
@@ -21940,16 +22084,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.24</v>
+        <v>18.88</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>68949.23359999999</v>
+        <v>67659.12319999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>8949.233599999992</v>
+        <v>7659.123199999987</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1491538933333332</v>
+        <v>0.1276520533333331</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -22325,6 +22469,9 @@
       </c>
       <c r="EF33" s="3" t="n">
         <v>19.24</v>
+      </c>
+      <c r="EG33" s="3" t="n">
+        <v>18.88</v>
       </c>
     </row>
     <row r="34">
@@ -22350,16 +22497,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>233.693</v>
+        <v>236.296</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>82150.333983</v>
+        <v>83065.36917599999</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>2150.333983000004</v>
+        <v>3065.369175999993</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.02687917478750005</v>
+        <v>0.03831711469999991</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -22738,6 +22885,9 @@
       </c>
       <c r="EF34" s="3" t="n">
         <v>233.693</v>
+      </c>
+      <c r="EG34" s="3" t="n">
+        <v>236.296</v>
       </c>
     </row>
     <row r="35">
@@ -22763,16 +22913,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.72</v>
+        <v>15.39</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>112168.84956</v>
+        <v>109814.15997</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>12168.84956</v>
+        <v>9814.159969999993</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1216884956</v>
+        <v>0.09814159969999993</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -23151,6 +23301,9 @@
       </c>
       <c r="EF35" s="3" t="n">
         <v>15.72</v>
+      </c>
+      <c r="EG35" s="3" t="n">
+        <v>15.39</v>
       </c>
     </row>
     <row r="36">
@@ -23176,16 +23329,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>360.8055</v>
+        <v>358.9447</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>168029.286183</v>
+        <v>167162.7004582</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>18029.28618300002</v>
+        <v>17162.70045820001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1201952412200001</v>
+        <v>0.1144180030546667</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -23564,6 +23717,9 @@
       </c>
       <c r="EF36" s="3" t="n">
         <v>360.8055</v>
+      </c>
+      <c r="EG36" s="3" t="n">
+        <v>358.9447</v>
       </c>
     </row>
     <row r="37">
@@ -23589,16 +23745,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.477</v>
+        <v>16.35</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62001.12205300001</v>
+        <v>61523.23515000001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12001.12205300001</v>
+        <v>11523.23515000001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2400224410600001</v>
+        <v>0.2304647030000002</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -23977,6 +24133,9 @@
       </c>
       <c r="EF37" s="3" t="n">
         <v>16.477</v>
+      </c>
+      <c r="EG37" s="3" t="n">
+        <v>16.35</v>
       </c>
     </row>
     <row r="38">
@@ -24002,16 +24161,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.6028</v>
+        <v>13.4716</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>81351.3005496</v>
+        <v>80566.66131120001</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1351.300549599997</v>
+        <v>566.661311200005</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.01689125686999996</v>
+        <v>0.007083266390000062</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -24387,6 +24546,9 @@
       </c>
       <c r="EF38" s="3" t="n">
         <v>13.6028</v>
+      </c>
+      <c r="EG38" s="3" t="n">
+        <v>13.4716</v>
       </c>
     </row>
     <row r="39">
@@ -24412,16 +24574,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.184</v>
+        <v>1024.8573</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51137.203104</v>
+        <v>51120.9069813</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1137.203104</v>
+        <v>1120.906981299995</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02274406208</v>
+        <v>0.0224181396259999</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -24797,6 +24959,9 @@
       </c>
       <c r="EF39" s="3" t="n">
         <v>1025.184</v>
+      </c>
+      <c r="EG39" s="3" t="n">
+        <v>1024.8573</v>
       </c>
     </row>
     <row r="40">
@@ -24822,16 +24987,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.2818</v>
+        <v>19.91</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>102241.1014086</v>
+        <v>100366.84757</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>2241.101408600007</v>
+        <v>366.8475699999981</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.02241101408600007</v>
+        <v>0.003668475699999981</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -25210,6 +25375,9 @@
       </c>
       <c r="EF40" s="3" t="n">
         <v>20.2818</v>
+      </c>
+      <c r="EG40" s="3" t="n">
+        <v>19.91</v>
       </c>
     </row>
     <row r="41">
@@ -25222,13 +25390,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4900391.678336699</v>
+        <v>4861736.8311561</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>430391.6783367</v>
+        <v>391736.8311560999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09628449179791945</v>
+        <v>0.08763687497899326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-23
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-22 07:02 IST</t>
+          <t>Generated: 2026-10-23 06:55 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4861736.8311561</v>
+        <v>4804113.3060405</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>391736.8311561001</v>
+        <v>334113.3060405003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.08763687497899332</v>
+        <v>0.07474570604932892</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>520045.0019340515</v>
+        <v>510128.0028610229</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-70737.0180659485</v>
+        <v>-80654.01713897707</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.119734547889505</v>
+        <v>-0.1365207714665674</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5381781.833090152</v>
+        <v>5314241.308901523</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>320999.8130901521</v>
+        <v>253459.2889015237</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06342889534099161</v>
+        <v>0.05008302825529002</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-22</t>
+          <t>Last snapshot: 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FK19"/>
+  <dimension ref="A1:FL19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -786,6 +786,7 @@
     <col width="21" customWidth="1" min="165" max="165"/>
     <col width="21" customWidth="1" min="166" max="166"/>
     <col width="21" customWidth="1" min="167" max="167"/>
+    <col width="21" customWidth="1" min="168" max="168"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1624,6 +1625,11 @@
           <t>2026-10-22</t>
         </is>
       </c>
+      <c r="FL1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1643,13 +1649,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>566.7000122070312</v>
+        <v>551.7000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45336.0009765625</v>
+        <v>44136.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1518.490976562498</v>
+        <v>318.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2127,6 +2133,9 @@
       </c>
       <c r="FK2" s="3" t="n">
         <v>566.7000122070312</v>
+      </c>
+      <c r="FL2" s="3" t="n">
+        <v>551.7000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -2174,13 +2183,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1367.800048828125</v>
+        <v>1365</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27356.0009765625</v>
+        <v>27300</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4748.579023437502</v>
+        <v>-4804.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2661,6 +2670,9 @@
       </c>
       <c r="FK4" s="3" t="n">
         <v>1367.800048828125</v>
+      </c>
+      <c r="FL4" s="3" t="n">
+        <v>1365</v>
       </c>
     </row>
     <row r="5">
@@ -2681,13 +2693,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>462.3500061035156</v>
+        <v>449.3500061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9247.000122070312</v>
+        <v>8987.000122070312</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4966.099877929688</v>
+        <v>-5226.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3168,6 +3180,9 @@
       </c>
       <c r="FK5" s="3" t="n">
         <v>462.3500061035156</v>
+      </c>
+      <c r="FL5" s="3" t="n">
+        <v>449.3500061035156</v>
       </c>
     </row>
     <row r="6">
@@ -3188,13 +3203,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>365.1499938964844</v>
+        <v>356.6000061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14605.99975585938</v>
+        <v>14264.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2896.240244140627</v>
+        <v>-3238.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3675,6 +3690,9 @@
       </c>
       <c r="FK6" s="3" t="n">
         <v>365.1499938964844</v>
+      </c>
+      <c r="FL6" s="3" t="n">
+        <v>356.6000061035156</v>
       </c>
     </row>
     <row r="7">
@@ -3695,13 +3713,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>252.75</v>
+        <v>238.8500061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25275</v>
+        <v>23885.00061035156</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1158.82</v>
+        <v>-2548.819389648437</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4182,6 +4200,9 @@
       </c>
       <c r="FK7" s="3" t="n">
         <v>252.75</v>
+      </c>
+      <c r="FL7" s="3" t="n">
+        <v>238.8500061035156</v>
       </c>
     </row>
     <row r="8">
@@ -4229,13 +4250,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>13.64000034332275</v>
+        <v>12.85000038146973</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>20460.00051498413</v>
+        <v>19275.00057220459</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-10590.16948501587</v>
+        <v>-11775.16942779541</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4716,6 +4737,9 @@
       </c>
       <c r="FK9" s="3" t="n">
         <v>13.64000034332275</v>
+      </c>
+      <c r="FL9" s="3" t="n">
+        <v>12.85000038146973</v>
       </c>
     </row>
     <row r="10">
@@ -4736,13 +4760,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>451.4500122070312</v>
+        <v>447</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45145.00122070312</v>
+        <v>44700</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6353.478779296878</v>
+        <v>-6798.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5223,6 +5247,9 @@
       </c>
       <c r="FK10" s="3" t="n">
         <v>451.4500122070312</v>
+      </c>
+      <c r="FL10" s="3" t="n">
+        <v>447</v>
       </c>
     </row>
     <row r="11">
@@ -5243,13 +5270,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>17.78000068664551</v>
+        <v>17.27000045776367</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>17780.00068664551</v>
+        <v>17270.00045776367</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>7938.790686645509</v>
+        <v>7428.790457763673</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5730,6 +5757,9 @@
       </c>
       <c r="FK11" s="3" t="n">
         <v>17.78000068664551</v>
+      </c>
+      <c r="FL11" s="3" t="n">
+        <v>17.27000045776367</v>
       </c>
     </row>
     <row r="12">
@@ -5750,13 +5780,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2378.699951171875</v>
+        <v>2295</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>23786.99951171875</v>
+        <v>22950</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-3936.25048828125</v>
+        <v>-4773.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6237,6 +6267,9 @@
       </c>
       <c r="FK12" s="3" t="n">
         <v>2378.699951171875</v>
+      </c>
+      <c r="FL12" s="3" t="n">
+        <v>2295</v>
       </c>
     </row>
     <row r="13">
@@ -6257,13 +6290,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>38.59999847412109</v>
+        <v>37.27999877929688</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>23159.99908447266</v>
+        <v>22367.99926757812</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-11871.76091552735</v>
+        <v>-12663.76073242188</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6744,6 +6777,9 @@
       </c>
       <c r="FK13" s="3" t="n">
         <v>38.59999847412109</v>
+      </c>
+      <c r="FL13" s="3" t="n">
+        <v>37.27999877929688</v>
       </c>
     </row>
     <row r="14">
@@ -6764,13 +6800,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>594.7000122070312</v>
+        <v>574.2999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>29735.00061035156</v>
+        <v>28714.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12727.50938964844</v>
+        <v>-13747.51061035156</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7251,6 +7287,9 @@
       </c>
       <c r="FK14" s="3" t="n">
         <v>594.7000122070312</v>
+      </c>
+      <c r="FL14" s="3" t="n">
+        <v>574.2999877929688</v>
       </c>
     </row>
     <row r="15">
@@ -7325,13 +7364,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>425.1499938964844</v>
+        <v>405.75</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>21257.49969482422</v>
+        <v>20287.5</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-497.0303051757801</v>
+        <v>-1467.029999999999</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7812,6 +7851,9 @@
       </c>
       <c r="FK17" s="3" t="n">
         <v>425.1499938964844</v>
+      </c>
+      <c r="FL17" s="3" t="n">
+        <v>405.75</v>
       </c>
     </row>
     <row r="18">
@@ -7832,13 +7874,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>351.2999877929688</v>
+        <v>342.2000122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>35129.99877929688</v>
+        <v>34220.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11510.82122070312</v>
+        <v>-12420.81877929687</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8319,6 +8361,9 @@
       </c>
       <c r="FK18" s="3" t="n">
         <v>351.2999877929688</v>
+      </c>
+      <c r="FL18" s="3" t="n">
+        <v>342.2000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -8331,10 +8376,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>520045.0019340515</v>
+        <v>510128.0028610229</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-70737.01806594849</v>
+        <v>-80654.01713897705</v>
       </c>
     </row>
   </sheetData>
@@ -8348,7 +8393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EG41"/>
+  <dimension ref="A1:EH41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8359,7 +8404,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -8488,6 +8533,7 @@
     <col width="13" customWidth="1" min="135" max="135"/>
     <col width="13" customWidth="1" min="136" max="136"/>
     <col width="13" customWidth="1" min="137" max="137"/>
+    <col width="13" customWidth="1" min="138" max="138"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9176,6 +9222,11 @@
           <t>2026-10-22</t>
         </is>
       </c>
+      <c r="EH1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9200,16 +9251,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.6826</v>
+        <v>56.0146</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63625.1982132</v>
+        <v>62875.3802372</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13625.1982132</v>
+        <v>12875.3802372</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.272503964264</v>
+        <v>0.257507604744</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9594,6 +9645,9 @@
       </c>
       <c r="EG2" s="3" t="n">
         <v>56.6826</v>
+      </c>
+      <c r="EH2" s="3" t="n">
+        <v>56.0146</v>
       </c>
     </row>
     <row r="3">
@@ -9619,16 +9673,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.5873</v>
+        <v>26.2773</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>65277.4845949</v>
+        <v>64516.3685649</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>5277.484594900001</v>
+        <v>4516.368564900004</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.08795807658166668</v>
+        <v>0.07527280941500006</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -10007,6 +10061,9 @@
       </c>
       <c r="EG3" s="3" t="n">
         <v>26.5873</v>
+      </c>
+      <c r="EH3" s="3" t="n">
+        <v>26.2773</v>
       </c>
     </row>
     <row r="4">
@@ -10032,16 +10089,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>11.9</v>
+        <v>11.45</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>228552.5067</v>
+        <v>219909.76485</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>48552.50670000003</v>
+        <v>39909.76485000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2697361483333335</v>
+        <v>0.2217209158333334</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -10420,6 +10477,9 @@
       </c>
       <c r="EG4" s="3" t="n">
         <v>11.9</v>
+      </c>
+      <c r="EH4" s="3" t="n">
+        <v>11.45</v>
       </c>
     </row>
     <row r="5">
@@ -10445,16 +10505,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.1172</v>
+        <v>9.018800000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>167337.8911136</v>
+        <v>165531.8488544</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-42662.1088864</v>
+        <v>-44468.15114559999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2031528994590476</v>
+        <v>-0.2117531006933333</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10833,6 +10893,9 @@
       </c>
       <c r="EG5" s="3" t="n">
         <v>9.1172</v>
+      </c>
+      <c r="EH5" s="3" t="n">
+        <v>9.018800000000001</v>
       </c>
     </row>
     <row r="6">
@@ -10858,16 +10921,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.9827</v>
+        <v>10.8625</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>46445.58569789999</v>
+        <v>45937.2626625</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-3554.414302100005</v>
+        <v>-4062.737337499995</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.07108828604200011</v>
+        <v>-0.0812547467499999</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -11252,6 +11315,9 @@
       </c>
       <c r="EG6" s="3" t="n">
         <v>10.9827</v>
+      </c>
+      <c r="EH6" s="3" t="n">
+        <v>10.8625</v>
       </c>
     </row>
     <row r="7">
@@ -11277,16 +11343,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.5796</v>
+        <v>33.4498</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74077.94078399999</v>
+        <v>73791.59679200001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14077.94078399999</v>
+        <v>13791.59679200001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2346323463999999</v>
+        <v>0.2298599465333335</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -11665,6 +11731,9 @@
       </c>
       <c r="EG7" s="3" t="n">
         <v>33.5796</v>
+      </c>
+      <c r="EH7" s="3" t="n">
+        <v>33.4498</v>
       </c>
     </row>
     <row r="8">
@@ -11690,16 +11759,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.4912</v>
+        <v>33.2025</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53739.7450816</v>
+        <v>53276.49908250001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3739.745081599998</v>
+        <v>3276.499082500006</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.07479490163199996</v>
+        <v>0.06552998165000012</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -12084,6 +12153,9 @@
       </c>
       <c r="EG8" s="3" t="n">
         <v>33.4912</v>
+      </c>
+      <c r="EH8" s="3" t="n">
+        <v>33.2025</v>
       </c>
     </row>
     <row r="9">
@@ -12109,16 +12181,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>39.9284</v>
+        <v>39.3891</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>128545.2114612</v>
+        <v>126808.9928163</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>28545.21146120002</v>
+        <v>26808.9928163</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.2854521146120002</v>
+        <v>0.268089928163</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -12497,6 +12569,9 @@
       </c>
       <c r="EG9" s="3" t="n">
         <v>39.9284</v>
+      </c>
+      <c r="EH9" s="3" t="n">
+        <v>39.3891</v>
       </c>
     </row>
     <row r="10">
@@ -12522,16 +12597,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49.0611</v>
+        <v>49.1299</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>139660.2218649</v>
+        <v>139856.0720041</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>39660.22186490003</v>
+        <v>39856.07200410002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3966022186490003</v>
+        <v>0.3985607200410002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -12910,6 +12985,9 @@
       </c>
       <c r="EG10" s="3" t="n">
         <v>49.0611</v>
+      </c>
+      <c r="EH10" s="3" t="n">
+        <v>49.1299</v>
       </c>
     </row>
     <row r="11">
@@ -12935,16 +13013,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>103.6975</v>
+        <v>100.3557</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31204.5480025</v>
+        <v>30198.9368883</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1204.5480025</v>
+        <v>198.9368882999988</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04015160008333332</v>
+        <v>0.006631229609999961</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -13323,6 +13401,9 @@
       </c>
       <c r="EG11" s="3" t="n">
         <v>103.6975</v>
+      </c>
+      <c r="EH11" s="3" t="n">
+        <v>100.3557</v>
       </c>
     </row>
     <row r="12">
@@ -13348,16 +13429,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>217.782</v>
+        <v>216.493</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>101382.312204</v>
+        <v>100782.254346</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1382.312204000002</v>
+        <v>782.2543460000015</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.01382312204000002</v>
+        <v>0.007822543460000015</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -13742,6 +13823,9 @@
       </c>
       <c r="EG12" s="3" t="n">
         <v>217.782</v>
+      </c>
+      <c r="EH12" s="3" t="n">
+        <v>216.493</v>
       </c>
     </row>
     <row r="13">
@@ -13767,16 +13851,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.819</v>
+        <v>20.797</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>241242.348495</v>
+        <v>240987.421185</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>41242.34849499998</v>
+        <v>40987.42118499998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2062117424749999</v>
+        <v>0.2049371059249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -14161,6 +14245,9 @@
       </c>
       <c r="EG13" s="3" t="n">
         <v>20.819</v>
+      </c>
+      <c r="EH13" s="3" t="n">
+        <v>20.797</v>
       </c>
     </row>
     <row r="14">
@@ -14186,16 +14273,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35.499</v>
+        <v>34.4964</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>128066.405394</v>
+        <v>124449.4196184</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>28066.40539400002</v>
+        <v>24449.41961840002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.2806640539400002</v>
+        <v>0.2444941961840002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -14574,6 +14661,9 @@
       </c>
       <c r="EG14" s="3" t="n">
         <v>35.499</v>
+      </c>
+      <c r="EH14" s="3" t="n">
+        <v>34.4964</v>
       </c>
     </row>
     <row r="15">
@@ -14599,16 +14689,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>10.95</v>
+        <v>10.83</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>106696.21965</v>
+        <v>105526.94601</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>6696.219649999999</v>
+        <v>5526.94601</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.06696219649999999</v>
+        <v>0.05526946009999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -14993,6 +15083,9 @@
       </c>
       <c r="EG15" s="3" t="n">
         <v>10.95</v>
+      </c>
+      <c r="EH15" s="3" t="n">
+        <v>10.83</v>
       </c>
     </row>
     <row r="16">
@@ -15018,16 +15111,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.5514</v>
+        <v>23.8364</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>140505.8944992</v>
+        <v>136414.0009792</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>40505.89449919999</v>
+        <v>36414.00097920001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4050589449919999</v>
+        <v>0.3641400097920001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -15406,6 +15499,9 @@
       </c>
       <c r="EG16" s="3" t="n">
         <v>24.5514</v>
+      </c>
+      <c r="EH16" s="3" t="n">
+        <v>23.8364</v>
       </c>
     </row>
     <row r="17">
@@ -15431,16 +15527,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6436</v>
+        <v>16.5872</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55024.69028519999</v>
+        <v>54838.22867039999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5024.690285199991</v>
+        <v>4838.228670399993</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1004938057039998</v>
+        <v>0.09676457340799985</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -15819,6 +15915,9 @@
       </c>
       <c r="EG17" s="3" t="n">
         <v>16.6436</v>
+      </c>
+      <c r="EH17" s="3" t="n">
+        <v>16.5872</v>
       </c>
     </row>
     <row r="18">
@@ -15844,16 +15943,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.12</v>
+        <v>43.93</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>83229.55631999999</v>
+        <v>82871.13347999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3229.556319999989</v>
+        <v>2871.13347999999</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.04036945399999986</v>
+        <v>0.03588916849999987</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -16238,6 +16337,9 @@
       </c>
       <c r="EG18" s="3" t="n">
         <v>44.12</v>
+      </c>
+      <c r="EH18" s="3" t="n">
+        <v>43.93</v>
       </c>
     </row>
     <row r="19">
@@ -16263,16 +16365,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.9506</v>
+        <v>11.615</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>172886.5337596</v>
+        <v>168031.48709</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>22886.53375959999</v>
+        <v>18031.48709000001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.1525768917306666</v>
+        <v>0.1202099139333334</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -16651,6 +16753,9 @@
       </c>
       <c r="EG19" s="3" t="n">
         <v>11.9506</v>
+      </c>
+      <c r="EH19" s="3" t="n">
+        <v>11.615</v>
       </c>
     </row>
     <row r="20">
@@ -16676,16 +16781,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.17</v>
+        <v>10.06</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>267021.51651</v>
+        <v>264133.37818</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>17021.51650999999</v>
+        <v>14133.37818</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.06808606603999995</v>
+        <v>0.05653351272</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -17070,6 +17175,9 @@
       </c>
       <c r="EG20" s="3" t="n">
         <v>10.17</v>
+      </c>
+      <c r="EH20" s="3" t="n">
+        <v>10.06</v>
       </c>
     </row>
     <row r="21">
@@ -17095,16 +17203,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>108.5689</v>
+        <v>107.7842</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>164944.2784451</v>
+        <v>163752.1159078</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-5055.721554899996</v>
+        <v>-6247.884092199994</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.02973953855823527</v>
+        <v>-0.03675225936588232</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -17489,6 +17597,9 @@
       </c>
       <c r="EG21" s="3" t="n">
         <v>108.5689</v>
+      </c>
+      <c r="EH21" s="3" t="n">
+        <v>107.7842</v>
       </c>
     </row>
     <row r="22">
@@ -17514,16 +17625,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>40.388</v>
+        <v>39.378</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>61973.77048</v>
+        <v>60423.96588</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>1973.770479999999</v>
+        <v>423.9658800000034</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.03289617466666665</v>
+        <v>0.007066098000000056</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -17902,6 +18013,9 @@
       </c>
       <c r="EG22" s="3" t="n">
         <v>40.388</v>
+      </c>
+      <c r="EH22" s="3" t="n">
+        <v>39.378</v>
       </c>
     </row>
     <row r="23">
@@ -17927,16 +18041,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>59.227</v>
+        <v>59.0253</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>160888.191009</v>
+        <v>160340.2796151</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>10888.191009</v>
+        <v>10340.27961510001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.07258794006000001</v>
+        <v>0.06893519743400005</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -18321,6 +18435,9 @@
       </c>
       <c r="EG23" s="3" t="n">
         <v>59.227</v>
+      </c>
+      <c r="EH23" s="3" t="n">
+        <v>59.0253</v>
       </c>
     </row>
     <row r="24">
@@ -18346,16 +18463,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.7931</v>
+        <v>25.6827</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>93716.28843659999</v>
+        <v>93315.1626222</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-6283.711563400007</v>
+        <v>-6684.837377799995</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.06283711563400007</v>
+        <v>-0.06684837377799994</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -18734,6 +18851,9 @@
       </c>
       <c r="EG24" s="3" t="n">
         <v>25.7931</v>
+      </c>
+      <c r="EH24" s="3" t="n">
+        <v>25.6827</v>
       </c>
     </row>
     <row r="25">
@@ -18759,16 +18879,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.1453</v>
+        <v>12.0312</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>199446.1572322</v>
+        <v>197572.4442288</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-553.8427678000007</v>
+        <v>-2427.555771200015</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.002769213839000004</v>
+        <v>-0.01213777885600008</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -19147,6 +19267,9 @@
       </c>
       <c r="EG25" s="3" t="n">
         <v>12.1453</v>
+      </c>
+      <c r="EH25" s="3" t="n">
+        <v>12.0312</v>
       </c>
     </row>
     <row r="26">
@@ -19172,16 +19295,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.8427</v>
+        <v>10.7477</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>129480.4332305</v>
+        <v>128345.9703055</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>19480.43323050001</v>
+        <v>18345.9703055</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1770948475500001</v>
+        <v>0.1667815482318182</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -19563,6 +19686,9 @@
       </c>
       <c r="EG26" s="3" t="n">
         <v>10.8427</v>
+      </c>
+      <c r="EH26" s="3" t="n">
+        <v>10.7477</v>
       </c>
     </row>
     <row r="27">
@@ -19588,16 +19714,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>66.8815</v>
+        <v>65.7362</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>107736.73309</v>
+        <v>105891.815132</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-2263.266910000006</v>
+        <v>-4108.184868000011</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.02057515372727278</v>
+        <v>-0.03734713516363646</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -19979,6 +20105,9 @@
       </c>
       <c r="EG27" s="3" t="n">
         <v>66.8815</v>
+      </c>
+      <c r="EH27" s="3" t="n">
+        <v>65.7362</v>
       </c>
     </row>
     <row r="28">
@@ -20004,16 +20133,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>112.2117</v>
+        <v>110.2021</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>371045.6032869</v>
+        <v>364400.5453797</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-8954.396713100024</v>
+        <v>-15599.45462029998</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.02356420187657901</v>
+        <v>-0.04105119636921047</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -20398,6 +20527,9 @@
       </c>
       <c r="EG28" s="3" t="n">
         <v>112.2117</v>
+      </c>
+      <c r="EH28" s="3" t="n">
+        <v>110.2021</v>
       </c>
     </row>
     <row r="29">
@@ -20423,16 +20555,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.6492</v>
+        <v>11.5083</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>111875.4569876</v>
+        <v>110522.2952349</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>11875.4569876</v>
+        <v>10522.2952349</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.118754569876</v>
+        <v>0.105222952349</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -20811,6 +20943,9 @@
       </c>
       <c r="EG29" s="3" t="n">
         <v>11.6492</v>
+      </c>
+      <c r="EH29" s="3" t="n">
+        <v>11.5083</v>
       </c>
     </row>
     <row r="30">
@@ -20836,16 +20971,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.6407</v>
+        <v>16.5408</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>123072.3041427</v>
+        <v>122333.4576288</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>23072.30414269998</v>
+        <v>22333.45762880001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2307230414269998</v>
+        <v>0.2233345762880001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -21224,6 +21359,9 @@
       </c>
       <c r="EG30" s="3" t="n">
         <v>16.6407</v>
+      </c>
+      <c r="EH30" s="3" t="n">
+        <v>16.5408</v>
       </c>
     </row>
     <row r="31">
@@ -21249,16 +21387,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>382.9721</v>
+        <v>380.5353</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>101901.216368</v>
+        <v>101252.832624</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>1901.216367999994</v>
+        <v>1252.832624000002</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.01901216367999994</v>
+        <v>0.01252832624000002</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -21640,6 +21778,9 @@
       </c>
       <c r="EG31" s="3" t="n">
         <v>382.9721</v>
+      </c>
+      <c r="EH31" s="3" t="n">
+        <v>380.5353</v>
       </c>
     </row>
     <row r="32">
@@ -21665,16 +21806,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.4</v>
+        <v>10.32</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>219855.584</v>
+        <v>218164.3872</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>19855.584</v>
+        <v>18164.3872</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.09927792000000002</v>
+        <v>0.09082193599999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -22059,6 +22200,9 @@
       </c>
       <c r="EG32" s="3" t="n">
         <v>10.4</v>
+      </c>
+      <c r="EH32" s="3" t="n">
+        <v>10.32</v>
       </c>
     </row>
     <row r="33">
@@ -22084,16 +22228,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.88</v>
+        <v>18.69</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67659.12319999999</v>
+        <v>66978.2316</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7659.123199999987</v>
+        <v>6978.231599999999</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1276520533333331</v>
+        <v>0.11630386</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -22472,6 +22616,9 @@
       </c>
       <c r="EG33" s="3" t="n">
         <v>18.88</v>
+      </c>
+      <c r="EH33" s="3" t="n">
+        <v>18.69</v>
       </c>
     </row>
     <row r="34">
@@ -22497,16 +22644,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>236.296</v>
+        <v>234.8558</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>83065.36917599999</v>
+        <v>82559.0942298</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>3065.369175999993</v>
+        <v>2559.094229800001</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.03831711469999991</v>
+        <v>0.03198867787250001</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -22888,6 +23035,9 @@
       </c>
       <c r="EG34" s="3" t="n">
         <v>236.296</v>
+      </c>
+      <c r="EH34" s="3" t="n">
+        <v>234.8558</v>
       </c>
     </row>
     <row r="35">
@@ -22913,16 +23063,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.39</v>
+        <v>15.25</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>109814.15997</v>
+        <v>108815.20075</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>9814.159969999993</v>
+        <v>8815.200750000004</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.09814159969999993</v>
+        <v>0.08815200750000003</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -23304,6 +23454,9 @@
       </c>
       <c r="EG35" s="3" t="n">
         <v>15.39</v>
+      </c>
+      <c r="EH35" s="3" t="n">
+        <v>15.25</v>
       </c>
     </row>
     <row r="36">
@@ -23329,16 +23482,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>358.9447</v>
+        <v>357.3916</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>167162.7004582</v>
+        <v>166439.4124696</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>17162.70045820001</v>
+        <v>16439.41246960001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1144180030546667</v>
+        <v>0.1095960831306667</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -23720,6 +23873,9 @@
       </c>
       <c r="EG36" s="3" t="n">
         <v>358.9447</v>
+      </c>
+      <c r="EH36" s="3" t="n">
+        <v>357.3916</v>
       </c>
     </row>
     <row r="37">
@@ -23745,16 +23901,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.35</v>
+        <v>16.369</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>61523.23515000001</v>
+        <v>61594.730041</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>11523.23515000001</v>
+        <v>11594.730041</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2304647030000002</v>
+        <v>0.23189460082</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -24136,6 +24292,9 @@
       </c>
       <c r="EG37" s="3" t="n">
         <v>16.35</v>
+      </c>
+      <c r="EH37" s="3" t="n">
+        <v>16.369</v>
       </c>
     </row>
     <row r="38">
@@ -24161,16 +24320,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.4716</v>
+        <v>13.3821</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>80566.66131120001</v>
+        <v>80031.4081722</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>566.661311200005</v>
+        <v>31.40817219999735</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.007083266390000062</v>
+        <v>0.0003926021524999669</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -24549,6 +24708,9 @@
       </c>
       <c r="EG38" s="3" t="n">
         <v>13.4716</v>
+      </c>
+      <c r="EH38" s="3" t="n">
+        <v>13.3821</v>
       </c>
     </row>
     <row r="39">
@@ -24574,16 +24736,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1024.8573</v>
+        <v>1024.3133</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51120.9069813</v>
+        <v>51093.7717173</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1120.906981299995</v>
+        <v>1093.771717299998</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.0224181396259999</v>
+        <v>0.02187543434599996</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -24962,6 +25124,9 @@
       </c>
       <c r="EG39" s="3" t="n">
         <v>1024.8573</v>
+      </c>
+      <c r="EH39" s="3" t="n">
+        <v>1024.3133</v>
       </c>
     </row>
     <row r="40">
@@ -24987,16 +25152,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.91</v>
+        <v>19.7478</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>100366.84757</v>
-      </c>
-      <c r="H40" s="4" t="n">
-        <v>366.8475699999981</v>
-      </c>
-      <c r="I40" s="12" t="n">
-        <v>0.003668475699999981</v>
+        <v>99549.19299060002</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>-450.807009399985</v>
+      </c>
+      <c r="I40" s="13" t="n">
+        <v>-0.00450807009399985</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -25378,6 +25543,9 @@
       </c>
       <c r="EG40" s="3" t="n">
         <v>19.91</v>
+      </c>
+      <c r="EH40" s="3" t="n">
+        <v>19.7478</v>
       </c>
     </row>
     <row r="41">
@@ -25390,13 +25558,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4861736.8311561</v>
+        <v>4804113.3060405</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>391736.8311560999</v>
+        <v>334113.3060405001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.08763687497899326</v>
+        <v>0.07474570604932888</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-24
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-23 06:55 IST</t>
+          <t>Generated: 2026-10-24 06:51 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4804113.3060405</v>
+        <v>4742003.478038399</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>334113.3060405003</v>
+        <v>272003.4780383995</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07474570604932892</v>
+        <v>0.0608508899414764</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>510128.0028610229</v>
+        <v>512060.5043869019</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-80654.01713897707</v>
+        <v>-78721.51561309816</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1365207714665674</v>
+        <v>-0.1332496808435337</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5314241.308901523</v>
+        <v>5254063.982425301</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>253459.2889015237</v>
+        <v>193281.9624253018</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.05008302825529002</v>
+        <v>0.03819211372105329</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-23</t>
+          <t>Last snapshot: 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FL19"/>
+  <dimension ref="A1:FM19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -787,6 +787,7 @@
     <col width="21" customWidth="1" min="166" max="166"/>
     <col width="21" customWidth="1" min="167" max="167"/>
     <col width="21" customWidth="1" min="168" max="168"/>
+    <col width="21" customWidth="1" min="169" max="169"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1630,6 +1631,11 @@
           <t>2026-10-23</t>
         </is>
       </c>
+      <c r="FM1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1649,13 +1655,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>551.7000122070312</v>
+        <v>550.9000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44136.0009765625</v>
+        <v>44072.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>318.490976562498</v>
+        <v>254.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2136,6 +2142,9 @@
       </c>
       <c r="FL2" s="3" t="n">
         <v>551.7000122070312</v>
+      </c>
+      <c r="FM2" s="3" t="n">
+        <v>550.9000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -2183,13 +2192,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1365</v>
+        <v>1357</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27300</v>
+        <v>27140</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4804.580000000002</v>
+        <v>-4964.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2673,6 +2682,9 @@
       </c>
       <c r="FL4" s="3" t="n">
         <v>1365</v>
+      </c>
+      <c r="FM4" s="3" t="n">
+        <v>1357</v>
       </c>
     </row>
     <row r="5">
@@ -2693,13 +2705,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>449.3500061035156</v>
+        <v>462.75</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8987.000122070312</v>
+        <v>9255</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-5226.099877929688</v>
+        <v>-4958.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3183,6 +3195,9 @@
       </c>
       <c r="FL5" s="3" t="n">
         <v>449.3500061035156</v>
+      </c>
+      <c r="FM5" s="3" t="n">
+        <v>462.75</v>
       </c>
     </row>
     <row r="6">
@@ -3203,13 +3218,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>356.6000061035156</v>
+        <v>354</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14264.00024414062</v>
+        <v>14160</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-3238.239755859377</v>
+        <v>-3342.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3693,6 +3708,9 @@
       </c>
       <c r="FL6" s="3" t="n">
         <v>356.6000061035156</v>
+      </c>
+      <c r="FM6" s="3" t="n">
+        <v>354</v>
       </c>
     </row>
     <row r="7">
@@ -3713,13 +3731,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>238.8500061035156</v>
+        <v>242.5</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23885.00061035156</v>
+        <v>24250</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2548.819389648437</v>
+        <v>-2183.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4203,6 +4221,9 @@
       </c>
       <c r="FL7" s="3" t="n">
         <v>238.8500061035156</v>
+      </c>
+      <c r="FM7" s="3" t="n">
+        <v>242.5</v>
       </c>
     </row>
     <row r="8">
@@ -4250,13 +4271,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>12.85000038146973</v>
+        <v>12.67000007629395</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>19275.00057220459</v>
+        <v>19005.00011444092</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-11775.16942779541</v>
+        <v>-12045.16988555908</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4740,6 +4761,9 @@
       </c>
       <c r="FL9" s="3" t="n">
         <v>12.85000038146973</v>
+      </c>
+      <c r="FM9" s="3" t="n">
+        <v>12.67000007629395</v>
       </c>
     </row>
     <row r="10">
@@ -4760,13 +4784,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>447</v>
+        <v>447.8500061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44700</v>
+        <v>44785.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6798.480000000003</v>
+        <v>-6713.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5250,6 +5274,9 @@
       </c>
       <c r="FL10" s="3" t="n">
         <v>447</v>
+      </c>
+      <c r="FM10" s="3" t="n">
+        <v>447.8500061035156</v>
       </c>
     </row>
     <row r="11">
@@ -5270,13 +5297,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>17.27000045776367</v>
+        <v>18.04000091552734</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>17270.00045776367</v>
+        <v>18040.00091552734</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>7428.790457763673</v>
+        <v>8198.790915527345</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5760,6 +5787,9 @@
       </c>
       <c r="FL11" s="3" t="n">
         <v>17.27000045776367</v>
+      </c>
+      <c r="FM11" s="3" t="n">
+        <v>18.04000091552734</v>
       </c>
     </row>
     <row r="12">
@@ -5780,13 +5810,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2295</v>
+        <v>2312.800048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>22950</v>
+        <v>23128.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-4773.25</v>
+        <v>-4595.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6270,6 +6300,9 @@
       </c>
       <c r="FL12" s="3" t="n">
         <v>2295</v>
+      </c>
+      <c r="FM12" s="3" t="n">
+        <v>2312.800048828125</v>
       </c>
     </row>
     <row r="13">
@@ -6290,13 +6323,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>37.27999877929688</v>
+        <v>37.40000152587891</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22367.99926757812</v>
+        <v>22440.00091552734</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-12663.76073242188</v>
+        <v>-12591.75908447266</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6780,6 +6813,9 @@
       </c>
       <c r="FL13" s="3" t="n">
         <v>37.27999877929688</v>
+      </c>
+      <c r="FM13" s="3" t="n">
+        <v>37.40000152587891</v>
       </c>
     </row>
     <row r="14">
@@ -6800,13 +6836,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>574.2999877929688</v>
+        <v>576.7999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>28714.99938964844</v>
+        <v>28839.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-13747.51061035156</v>
+        <v>-13622.51061035156</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7290,6 +7326,9 @@
       </c>
       <c r="FL14" s="3" t="n">
         <v>574.2999877929688</v>
+      </c>
+      <c r="FM14" s="3" t="n">
+        <v>576.7999877929688</v>
       </c>
     </row>
     <row r="15">
@@ -7364,13 +7403,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>405.75</v>
+        <v>407.2999877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>20287.5</v>
+        <v>20364.99938964844</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-1467.029999999999</v>
+        <v>-1389.530610351561</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7854,6 +7893,9 @@
       </c>
       <c r="FL17" s="3" t="n">
         <v>405.75</v>
+      </c>
+      <c r="FM17" s="3" t="n">
+        <v>407.2999877929688</v>
       </c>
     </row>
     <row r="18">
@@ -7874,13 +7916,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>342.2000122070312</v>
+        <v>348.1000061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34220.00122070312</v>
+        <v>34810.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12420.81877929687</v>
+        <v>-11830.81938964844</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8364,6 +8406,9 @@
       </c>
       <c r="FL18" s="3" t="n">
         <v>342.2000122070312</v>
+      </c>
+      <c r="FM18" s="3" t="n">
+        <v>348.1000061035156</v>
       </c>
     </row>
     <row r="19">
@@ -8376,10 +8421,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>510128.0028610229</v>
+        <v>512060.5043869019</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-80654.01713897705</v>
+        <v>-78721.51561309815</v>
       </c>
     </row>
   </sheetData>
@@ -8393,7 +8438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EH41"/>
+  <dimension ref="A1:EI41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8534,6 +8579,7 @@
     <col width="13" customWidth="1" min="136" max="136"/>
     <col width="13" customWidth="1" min="137" max="137"/>
     <col width="13" customWidth="1" min="138" max="138"/>
+    <col width="13" customWidth="1" min="139" max="139"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9227,6 +9273,11 @@
           <t>2026-10-23</t>
         </is>
       </c>
+      <c r="EI1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9251,16 +9302,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.0146</v>
+        <v>55.8014</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>62875.3802372</v>
+        <v>62636.0670748</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>12875.3802372</v>
+        <v>12636.0670748</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.257507604744</v>
+        <v>0.252721341496</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9648,6 +9699,9 @@
       </c>
       <c r="EH2" s="3" t="n">
         <v>56.0146</v>
+      </c>
+      <c r="EI2" s="3" t="n">
+        <v>55.8014</v>
       </c>
     </row>
     <row r="3">
@@ -9673,16 +9727,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.2773</v>
+        <v>26.1132</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>64516.3685649</v>
+        <v>64113.4681116</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4516.368564900004</v>
+        <v>4113.468111599999</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.07527280941500006</v>
+        <v>0.06855780185999999</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -10064,6 +10118,9 @@
       </c>
       <c r="EH3" s="3" t="n">
         <v>26.2773</v>
+      </c>
+      <c r="EI3" s="3" t="n">
+        <v>26.1132</v>
       </c>
     </row>
     <row r="4">
@@ -10481,6 +10538,9 @@
       <c r="EH4" s="3" t="n">
         <v>11.45</v>
       </c>
+      <c r="EI4" s="3" t="n">
+        <v>11.45</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10505,16 +10565,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.018800000000001</v>
+        <v>8.8916</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>165531.8488544</v>
+        <v>163197.2088608</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-44468.15114559999</v>
+        <v>-46802.79113920001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2117531006933333</v>
+        <v>-0.2228704339961905</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -10896,6 +10956,9 @@
       </c>
       <c r="EH5" s="3" t="n">
         <v>9.018800000000001</v>
+      </c>
+      <c r="EI5" s="3" t="n">
+        <v>8.8916</v>
       </c>
     </row>
     <row r="6">
@@ -10921,16 +10984,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.8625</v>
+        <v>10.6973</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>45937.2626625</v>
+        <v>45238.6356621</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-4062.737337499995</v>
+        <v>-4761.364337899999</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.0812547467499999</v>
+        <v>-0.09522728675799998</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -11318,6 +11381,9 @@
       </c>
       <c r="EH6" s="3" t="n">
         <v>10.8625</v>
+      </c>
+      <c r="EI6" s="3" t="n">
+        <v>10.6973</v>
       </c>
     </row>
     <row r="7">
@@ -11343,16 +11409,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.4498</v>
+        <v>32.7421</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73791.59679200001</v>
+        <v>72230.38228400001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13791.59679200001</v>
+        <v>12230.38228400001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2298599465333335</v>
+        <v>0.2038397047333334</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -11734,6 +11800,9 @@
       </c>
       <c r="EH7" s="3" t="n">
         <v>33.4498</v>
+      </c>
+      <c r="EI7" s="3" t="n">
+        <v>32.7421</v>
       </c>
     </row>
     <row r="8">
@@ -11759,16 +11828,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.2025</v>
+        <v>32.3871</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53276.49908250001</v>
+        <v>51968.11395029999</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3276.499082500006</v>
+        <v>1968.113950299994</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.06552998165000012</v>
+        <v>0.03936227900599988</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -12156,6 +12225,9 @@
       </c>
       <c r="EH8" s="3" t="n">
         <v>33.2025</v>
+      </c>
+      <c r="EI8" s="3" t="n">
+        <v>32.3871</v>
       </c>
     </row>
     <row r="9">
@@ -12181,16 +12253,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>39.3891</v>
+        <v>38.8661</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>126808.9928163</v>
+        <v>125125.2502773</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>26808.9928163</v>
+        <v>25125.25027730002</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.268089928163</v>
+        <v>0.2512525027730002</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -12572,6 +12644,9 @@
       </c>
       <c r="EH9" s="3" t="n">
         <v>39.3891</v>
+      </c>
+      <c r="EI9" s="3" t="n">
+        <v>38.8661</v>
       </c>
     </row>
     <row r="10">
@@ -12597,16 +12672,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49.1299</v>
+        <v>49.0519</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>139856.0720041</v>
+        <v>139634.0326021</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>39856.07200410002</v>
+        <v>39634.03260210002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3985607200410002</v>
+        <v>0.3963403260210002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -12988,6 +13063,9 @@
       </c>
       <c r="EH10" s="3" t="n">
         <v>49.1299</v>
+      </c>
+      <c r="EI10" s="3" t="n">
+        <v>49.0519</v>
       </c>
     </row>
     <row r="11">
@@ -13013,16 +13091,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>100.3557</v>
+        <v>100.2279</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30198.9368883</v>
+        <v>30160.4794401</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>198.9368882999988</v>
+        <v>160.4794400999999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.006631229609999961</v>
+        <v>0.005349314669999997</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -13404,6 +13482,9 @@
       </c>
       <c r="EH11" s="3" t="n">
         <v>100.3557</v>
+      </c>
+      <c r="EI11" s="3" t="n">
+        <v>100.2279</v>
       </c>
     </row>
     <row r="12">
@@ -13429,16 +13510,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>216.493</v>
+        <v>213.423</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>100782.254346</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>782.2543460000015</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>0.007822543460000015</v>
+        <v>99353.10180600001</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>-646.898193999994</v>
+      </c>
+      <c r="I12" s="13" t="n">
+        <v>-0.006468981939999939</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -13826,6 +13907,9 @@
       </c>
       <c r="EH12" s="3" t="n">
         <v>216.493</v>
+      </c>
+      <c r="EI12" s="3" t="n">
+        <v>213.423</v>
       </c>
     </row>
     <row r="13">
@@ -13851,16 +13935,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.797</v>
+        <v>20.656</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>240987.421185</v>
+        <v>239353.56888</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>40987.42118499998</v>
+        <v>39353.56887999998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2049371059249999</v>
+        <v>0.1967678443999999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -14248,6 +14332,9 @@
       </c>
       <c r="EH13" s="3" t="n">
         <v>20.797</v>
+      </c>
+      <c r="EI13" s="3" t="n">
+        <v>20.656</v>
       </c>
     </row>
     <row r="14">
@@ -14273,16 +14360,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34.4964</v>
+        <v>34.7483</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>124449.4196184</v>
+        <v>125358.1755698</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>24449.41961840002</v>
+        <v>25358.17556980001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.2444941961840002</v>
+        <v>0.2535817556980001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -14664,6 +14751,9 @@
       </c>
       <c r="EH14" s="3" t="n">
         <v>34.4964</v>
+      </c>
+      <c r="EI14" s="3" t="n">
+        <v>34.7483</v>
       </c>
     </row>
     <row r="15">
@@ -14689,16 +14779,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>10.83</v>
+        <v>10.61</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>105526.94601</v>
+        <v>103383.27767</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>5526.94601</v>
+        <v>3383.277669999996</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.05526946009999999</v>
+        <v>0.03383277669999996</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -15086,6 +15176,9 @@
       </c>
       <c r="EH15" s="3" t="n">
         <v>10.83</v>
+      </c>
+      <c r="EI15" s="3" t="n">
+        <v>10.61</v>
       </c>
     </row>
     <row r="16">
@@ -15111,16 +15204,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>23.8364</v>
+        <v>23.8966</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>136414.0009792</v>
+        <v>136758.5212448</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>36414.00097920001</v>
+        <v>36758.52124479998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3641400097920001</v>
+        <v>0.3675852124479998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -15502,6 +15595,9 @@
       </c>
       <c r="EH16" s="3" t="n">
         <v>23.8364</v>
+      </c>
+      <c r="EI16" s="3" t="n">
+        <v>23.8966</v>
       </c>
     </row>
     <row r="17">
@@ -15527,16 +15623,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.5872</v>
+        <v>16.5054</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54838.22867039999</v>
+        <v>54567.7932078</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4838.228670399993</v>
+        <v>4567.793207800001</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.09676457340799985</v>
+        <v>0.09135586415600003</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -15918,6 +16014,9 @@
       </c>
       <c r="EH17" s="3" t="n">
         <v>16.5872</v>
+      </c>
+      <c r="EI17" s="3" t="n">
+        <v>16.5054</v>
       </c>
     </row>
     <row r="18">
@@ -15943,16 +16042,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>43.93</v>
+        <v>43.47</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>82871.13347999999</v>
+        <v>82003.37291999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>2871.13347999999</v>
+        <v>2003.372919999994</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.03588916849999987</v>
+        <v>0.02504216149999993</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -16340,6 +16439,9 @@
       </c>
       <c r="EH18" s="3" t="n">
         <v>43.93</v>
+      </c>
+      <c r="EI18" s="3" t="n">
+        <v>43.47</v>
       </c>
     </row>
     <row r="19">
@@ -16365,16 +16467,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.615</v>
+        <v>11.3218</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>168031.48709</v>
+        <v>163789.8312988</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>18031.48709000001</v>
+        <v>13789.83129879998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.1202099139333334</v>
+        <v>0.09193220865866654</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -16756,6 +16858,9 @@
       </c>
       <c r="EH19" s="3" t="n">
         <v>11.615</v>
+      </c>
+      <c r="EI19" s="3" t="n">
+        <v>11.3218</v>
       </c>
     </row>
     <row r="20">
@@ -16781,16 +16886,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.06</v>
+        <v>9.93</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>264133.37818</v>
+        <v>260720.12379</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>14133.37818</v>
+        <v>10720.12378999998</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.05653351272</v>
+        <v>0.04288049515999993</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -17178,6 +17283,9 @@
       </c>
       <c r="EH20" s="3" t="n">
         <v>10.06</v>
+      </c>
+      <c r="EI20" s="3" t="n">
+        <v>9.93</v>
       </c>
     </row>
     <row r="21">
@@ -17203,16 +17311,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.7842</v>
+        <v>105.9959</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163752.1159078</v>
+        <v>161035.2250381</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6247.884092199994</v>
+        <v>-8964.774961899995</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03675225936588232</v>
+        <v>-0.05273397036411762</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -17600,6 +17708,9 @@
       </c>
       <c r="EH21" s="3" t="n">
         <v>107.7842</v>
+      </c>
+      <c r="EI21" s="3" t="n">
+        <v>105.9959</v>
       </c>
     </row>
     <row r="22">
@@ -17625,16 +17736,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>39.378</v>
+        <v>39.638</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>60423.96588</v>
+        <v>60822.92548</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>423.9658800000034</v>
+        <v>822.9254799999981</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.007066098000000056</v>
+        <v>0.01371542466666663</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -18016,6 +18127,9 @@
       </c>
       <c r="EH22" s="3" t="n">
         <v>39.378</v>
+      </c>
+      <c r="EI22" s="3" t="n">
+        <v>39.638</v>
       </c>
     </row>
     <row r="23">
@@ -18041,16 +18155,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>59.0253</v>
+        <v>58.115</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>160340.2796151</v>
+        <v>157867.479705</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>10340.27961510001</v>
+        <v>7867.479705000005</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.06893519743400005</v>
+        <v>0.05244986470000004</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -18438,6 +18552,9 @@
       </c>
       <c r="EH23" s="3" t="n">
         <v>59.0253</v>
+      </c>
+      <c r="EI23" s="3" t="n">
+        <v>58.115</v>
       </c>
     </row>
     <row r="24">
@@ -18463,16 +18580,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.6827</v>
+        <v>25.213</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>93315.1626222</v>
+        <v>91608.561218</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-6684.837377799995</v>
+        <v>-8391.438781999997</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.06684837377799994</v>
+        <v>-0.08391438781999998</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -18854,6 +18971,9 @@
       </c>
       <c r="EH24" s="3" t="n">
         <v>25.6827</v>
+      </c>
+      <c r="EI24" s="3" t="n">
+        <v>25.213</v>
       </c>
     </row>
     <row r="25">
@@ -18879,16 +18999,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.0312</v>
+        <v>11.7845</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>197572.4442288</v>
+        <v>193521.217253</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-2427.555771200015</v>
+        <v>-6478.782747000019</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.01213777885600008</v>
+        <v>-0.0323939137350001</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -19270,6 +19390,9 @@
       </c>
       <c r="EH25" s="3" t="n">
         <v>12.0312</v>
+      </c>
+      <c r="EI25" s="3" t="n">
+        <v>11.7845</v>
       </c>
     </row>
     <row r="26">
@@ -19295,16 +19418,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.7477</v>
+        <v>10.5186</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>128345.9703055</v>
+        <v>125610.123399</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>18345.9703055</v>
+        <v>15610.12339899999</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1667815482318182</v>
+        <v>0.1419102127181817</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -19689,6 +19812,9 @@
       </c>
       <c r="EH26" s="3" t="n">
         <v>10.7477</v>
+      </c>
+      <c r="EI26" s="3" t="n">
+        <v>10.5186</v>
       </c>
     </row>
     <row r="27">
@@ -19714,16 +19840,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.7362</v>
+        <v>64.6493</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>105891.815132</v>
+        <v>104140.971398</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-4108.184868000011</v>
+        <v>-5859.028602000006</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.03734713516363646</v>
+        <v>-0.05326389638181823</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -20108,6 +20234,9 @@
       </c>
       <c r="EH27" s="3" t="n">
         <v>65.7362</v>
+      </c>
+      <c r="EI27" s="3" t="n">
+        <v>64.6493</v>
       </c>
     </row>
     <row r="28">
@@ -20133,16 +20262,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>110.2021</v>
+        <v>108.6049</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>364400.5453797</v>
+        <v>359119.1528193</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-15599.45462029998</v>
+        <v>-20880.84718069999</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.04105119636921047</v>
+        <v>-0.05494959784394734</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -20530,6 +20659,9 @@
       </c>
       <c r="EH28" s="3" t="n">
         <v>110.2021</v>
+      </c>
+      <c r="EI28" s="3" t="n">
+        <v>108.6049</v>
       </c>
     </row>
     <row r="29">
@@ -20555,16 +20687,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.5083</v>
+        <v>11.209</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>110522.2952349</v>
+        <v>107647.906927</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>10522.2952349</v>
+        <v>7647.906926999989</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.105222952349</v>
+        <v>0.07647906926999989</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -20946,6 +21078,9 @@
       </c>
       <c r="EH29" s="3" t="n">
         <v>11.5083</v>
+      </c>
+      <c r="EI29" s="3" t="n">
+        <v>11.209</v>
       </c>
     </row>
     <row r="30">
@@ -20971,16 +21106,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.5408</v>
+        <v>16.1908</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>122333.4576288</v>
+        <v>119744.9062788</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>22333.45762880001</v>
+        <v>19744.90627879999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2233345762880001</v>
+        <v>0.1974490627879999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -21362,6 +21497,9 @@
       </c>
       <c r="EH30" s="3" t="n">
         <v>16.5408</v>
+      </c>
+      <c r="EI30" s="3" t="n">
+        <v>16.1908</v>
       </c>
     </row>
     <row r="31">
@@ -21387,16 +21525,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>380.5353</v>
+        <v>373.1721</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>101252.832624</v>
-      </c>
-      <c r="H31" s="4" t="n">
-        <v>1252.832624000002</v>
-      </c>
-      <c r="I31" s="12" t="n">
-        <v>0.01252832624000002</v>
+        <v>99293.63236799999</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>-706.3676320000086</v>
+      </c>
+      <c r="I31" s="13" t="n">
+        <v>-0.007063676320000086</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -21781,6 +21919,9 @@
       </c>
       <c r="EH31" s="3" t="n">
         <v>380.5353</v>
+      </c>
+      <c r="EI31" s="3" t="n">
+        <v>373.1721</v>
       </c>
     </row>
     <row r="32">
@@ -21806,16 +21947,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.32</v>
+        <v>10.18</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>218164.3872</v>
+        <v>215204.7928</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>18164.3872</v>
+        <v>15204.7928</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.09082193599999999</v>
+        <v>0.07602396399999997</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -22203,6 +22344,9 @@
       </c>
       <c r="EH32" s="3" t="n">
         <v>10.32</v>
+      </c>
+      <c r="EI32" s="3" t="n">
+        <v>10.18</v>
       </c>
     </row>
     <row r="33">
@@ -22228,16 +22372,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.69</v>
+        <v>18.3</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>66978.2316</v>
+        <v>65580.61199999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>6978.231599999999</v>
+        <v>5580.611999999994</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.11630386</v>
+        <v>0.09301019999999989</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -22619,6 +22763,9 @@
       </c>
       <c r="EH33" s="3" t="n">
         <v>18.69</v>
+      </c>
+      <c r="EI33" s="3" t="n">
+        <v>18.3</v>
       </c>
     </row>
     <row r="34">
@@ -22644,16 +22791,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>234.8558</v>
+        <v>232.9044</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>82559.0942298</v>
+        <v>81873.11663640001</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>2559.094229800001</v>
+        <v>1873.116636400009</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.03198867787250001</v>
+        <v>0.02341395795500011</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -23038,6 +23185,9 @@
       </c>
       <c r="EH34" s="3" t="n">
         <v>234.8558</v>
+      </c>
+      <c r="EI34" s="3" t="n">
+        <v>232.9044</v>
       </c>
     </row>
     <row r="35">
@@ -23063,16 +23213,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.25</v>
+        <v>14.96</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>108815.20075</v>
+        <v>106745.92808</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>8815.200750000004</v>
+        <v>6745.928079999998</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.08815200750000003</v>
+        <v>0.06745928079999998</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -23457,6 +23607,9 @@
       </c>
       <c r="EH35" s="3" t="n">
         <v>15.25</v>
+      </c>
+      <c r="EI35" s="3" t="n">
+        <v>14.96</v>
       </c>
     </row>
     <row r="36">
@@ -23482,16 +23635,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>357.3916</v>
+        <v>354.6417</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>166439.4124696</v>
+        <v>165158.7675402</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>16439.41246960001</v>
+        <v>15158.7675402</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1095960831306667</v>
+        <v>0.101058450268</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -23876,6 +24029,9 @@
       </c>
       <c r="EH36" s="3" t="n">
         <v>357.3916</v>
+      </c>
+      <c r="EI36" s="3" t="n">
+        <v>354.6417</v>
       </c>
     </row>
     <row r="37">
@@ -23901,16 +24057,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.369</v>
+        <v>16.219</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>61594.730041</v>
+        <v>61030.296691</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>11594.730041</v>
+        <v>11030.296691</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.23189460082</v>
+        <v>0.2206059338200001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -24295,6 +24451,9 @@
       </c>
       <c r="EH37" s="3" t="n">
         <v>16.369</v>
+      </c>
+      <c r="EI37" s="3" t="n">
+        <v>16.219</v>
       </c>
     </row>
     <row r="38">
@@ -24320,16 +24479,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.3821</v>
+        <v>13.1979</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>80031.4081722</v>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>31.40817219999735</v>
-      </c>
-      <c r="I38" s="12" t="n">
-        <v>0.0003926021524999669</v>
+        <v>78929.8033878</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>-1070.196612200001</v>
+      </c>
+      <c r="I38" s="13" t="n">
+        <v>-0.01337745765250002</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -24711,6 +24870,9 @@
       </c>
       <c r="EH38" s="3" t="n">
         <v>13.3821</v>
+      </c>
+      <c r="EI38" s="3" t="n">
+        <v>13.1979</v>
       </c>
     </row>
     <row r="39">
@@ -24736,16 +24898,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1024.3133</v>
+        <v>1024.3327</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51093.7717173</v>
+        <v>51094.7394087</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1093.771717299998</v>
+        <v>1094.739408699999</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02187543434599996</v>
+        <v>0.02189478817399999</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -25127,6 +25289,9 @@
       </c>
       <c r="EH39" s="3" t="n">
         <v>1024.3133</v>
+      </c>
+      <c r="EI39" s="3" t="n">
+        <v>1024.3327</v>
       </c>
     </row>
     <row r="40">
@@ -25152,16 +25317,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.7478</v>
+        <v>19.1374</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>99549.19299060002</v>
+        <v>96472.1501098</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>-450.807009399985</v>
+        <v>-3527.849890199999</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>-0.00450807009399985</v>
+        <v>-0.03527849890199999</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -25546,6 +25711,9 @@
       </c>
       <c r="EH40" s="3" t="n">
         <v>19.7478</v>
+      </c>
+      <c r="EI40" s="3" t="n">
+        <v>19.1374</v>
       </c>
     </row>
     <row r="41">
@@ -25558,13 +25726,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4804113.3060405</v>
+        <v>4742003.478038399</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>334113.3060405001</v>
+        <v>272003.4780383999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07474570604932888</v>
+        <v>0.06085088994147649</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-25
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-24 06:51 IST</t>
+          <t>Generated: 2026-10-25 07:14 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-24</t>
+          <t>Last snapshot: 2026-10-25</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FM19"/>
+  <dimension ref="A1:FN19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -788,6 +788,7 @@
     <col width="21" customWidth="1" min="167" max="167"/>
     <col width="21" customWidth="1" min="168" max="168"/>
     <col width="21" customWidth="1" min="169" max="169"/>
+    <col width="21" customWidth="1" min="170" max="170"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1636,6 +1637,11 @@
           <t>2026-10-24</t>
         </is>
       </c>
+      <c r="FN1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2146,6 +2152,9 @@
       <c r="FM2" s="3" t="n">
         <v>550.9000244140625</v>
       </c>
+      <c r="FN2" s="3" t="n">
+        <v>550.9000244140625</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2686,6 +2695,9 @@
       <c r="FM4" s="3" t="n">
         <v>1357</v>
       </c>
+      <c r="FN4" s="3" t="n">
+        <v>1357</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3199,6 +3211,9 @@
       <c r="FM5" s="3" t="n">
         <v>462.75</v>
       </c>
+      <c r="FN5" s="3" t="n">
+        <v>462.75</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3712,6 +3727,9 @@
       <c r="FM6" s="3" t="n">
         <v>354</v>
       </c>
+      <c r="FN6" s="3" t="n">
+        <v>354</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4225,6 +4243,9 @@
       <c r="FM7" s="3" t="n">
         <v>242.5</v>
       </c>
+      <c r="FN7" s="3" t="n">
+        <v>242.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4765,6 +4786,9 @@
       <c r="FM9" s="3" t="n">
         <v>12.67000007629395</v>
       </c>
+      <c r="FN9" s="3" t="n">
+        <v>12.67000007629395</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5278,6 +5302,9 @@
       <c r="FM10" s="3" t="n">
         <v>447.8500061035156</v>
       </c>
+      <c r="FN10" s="3" t="n">
+        <v>447.8500061035156</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5791,6 +5818,9 @@
       <c r="FM11" s="3" t="n">
         <v>18.04000091552734</v>
       </c>
+      <c r="FN11" s="3" t="n">
+        <v>18.04000091552734</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6304,6 +6334,9 @@
       <c r="FM12" s="3" t="n">
         <v>2312.800048828125</v>
       </c>
+      <c r="FN12" s="3" t="n">
+        <v>2312.800048828125</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6817,6 +6850,9 @@
       <c r="FM13" s="3" t="n">
         <v>37.40000152587891</v>
       </c>
+      <c r="FN13" s="3" t="n">
+        <v>37.40000152587891</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7330,6 +7366,9 @@
       <c r="FM14" s="3" t="n">
         <v>576.7999877929688</v>
       </c>
+      <c r="FN14" s="3" t="n">
+        <v>576.7999877929688</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7897,6 +7936,9 @@
       <c r="FM17" s="3" t="n">
         <v>407.2999877929688</v>
       </c>
+      <c r="FN17" s="3" t="n">
+        <v>407.2999877929688</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8408,6 +8450,9 @@
         <v>342.2000122070312</v>
       </c>
       <c r="FM18" s="3" t="n">
+        <v>348.1000061035156</v>
+      </c>
+      <c r="FN18" s="3" t="n">
         <v>348.1000061035156</v>
       </c>
     </row>
@@ -8438,7 +8483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EI41"/>
+  <dimension ref="A1:EJ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8580,6 +8625,7 @@
     <col width="13" customWidth="1" min="137" max="137"/>
     <col width="13" customWidth="1" min="138" max="138"/>
     <col width="13" customWidth="1" min="139" max="139"/>
+    <col width="13" customWidth="1" min="140" max="140"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9278,6 +9324,11 @@
           <t>2026-10-24</t>
         </is>
       </c>
+      <c r="EJ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9703,6 +9754,9 @@
       <c r="EI2" s="3" t="n">
         <v>55.8014</v>
       </c>
+      <c r="EJ2" s="3" t="n">
+        <v>55.8014</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10122,6 +10176,9 @@
       <c r="EI3" s="3" t="n">
         <v>26.1132</v>
       </c>
+      <c r="EJ3" s="3" t="n">
+        <v>26.1132</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10541,6 +10598,9 @@
       <c r="EI4" s="3" t="n">
         <v>11.45</v>
       </c>
+      <c r="EJ4" s="3" t="n">
+        <v>11.45</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10960,6 +11020,9 @@
       <c r="EI5" s="3" t="n">
         <v>8.8916</v>
       </c>
+      <c r="EJ5" s="3" t="n">
+        <v>8.8916</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11385,6 +11448,9 @@
       <c r="EI6" s="3" t="n">
         <v>10.6973</v>
       </c>
+      <c r="EJ6" s="3" t="n">
+        <v>10.6973</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11804,6 +11870,9 @@
       <c r="EI7" s="3" t="n">
         <v>32.7421</v>
       </c>
+      <c r="EJ7" s="3" t="n">
+        <v>32.7421</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12229,6 +12298,9 @@
       <c r="EI8" s="3" t="n">
         <v>32.3871</v>
       </c>
+      <c r="EJ8" s="3" t="n">
+        <v>32.3871</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12648,6 +12720,9 @@
       <c r="EI9" s="3" t="n">
         <v>38.8661</v>
       </c>
+      <c r="EJ9" s="3" t="n">
+        <v>38.8661</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -13067,6 +13142,9 @@
       <c r="EI10" s="3" t="n">
         <v>49.0519</v>
       </c>
+      <c r="EJ10" s="3" t="n">
+        <v>49.0519</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13486,6 +13564,9 @@
       <c r="EI11" s="3" t="n">
         <v>100.2279</v>
       </c>
+      <c r="EJ11" s="3" t="n">
+        <v>100.2279</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13911,6 +13992,9 @@
       <c r="EI12" s="3" t="n">
         <v>213.423</v>
       </c>
+      <c r="EJ12" s="3" t="n">
+        <v>213.423</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14336,6 +14420,9 @@
       <c r="EI13" s="3" t="n">
         <v>20.656</v>
       </c>
+      <c r="EJ13" s="3" t="n">
+        <v>20.656</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14755,6 +14842,9 @@
       <c r="EI14" s="3" t="n">
         <v>34.7483</v>
       </c>
+      <c r="EJ14" s="3" t="n">
+        <v>34.7483</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -15180,6 +15270,9 @@
       <c r="EI15" s="3" t="n">
         <v>10.61</v>
       </c>
+      <c r="EJ15" s="3" t="n">
+        <v>10.61</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15599,6 +15692,9 @@
       <c r="EI16" s="3" t="n">
         <v>23.8966</v>
       </c>
+      <c r="EJ16" s="3" t="n">
+        <v>23.8966</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -16018,6 +16114,9 @@
       <c r="EI17" s="3" t="n">
         <v>16.5054</v>
       </c>
+      <c r="EJ17" s="3" t="n">
+        <v>16.5054</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -16443,6 +16542,9 @@
       <c r="EI18" s="3" t="n">
         <v>43.47</v>
       </c>
+      <c r="EJ18" s="3" t="n">
+        <v>43.47</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -16862,6 +16964,9 @@
       <c r="EI19" s="3" t="n">
         <v>11.3218</v>
       </c>
+      <c r="EJ19" s="3" t="n">
+        <v>11.3218</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -17287,6 +17392,9 @@
       <c r="EI20" s="3" t="n">
         <v>9.93</v>
       </c>
+      <c r="EJ20" s="3" t="n">
+        <v>9.93</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -17712,6 +17820,9 @@
       <c r="EI21" s="3" t="n">
         <v>105.9959</v>
       </c>
+      <c r="EJ21" s="3" t="n">
+        <v>105.9959</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -18131,6 +18242,9 @@
       <c r="EI22" s="3" t="n">
         <v>39.638</v>
       </c>
+      <c r="EJ22" s="3" t="n">
+        <v>39.638</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -18556,6 +18670,9 @@
       <c r="EI23" s="3" t="n">
         <v>58.115</v>
       </c>
+      <c r="EJ23" s="3" t="n">
+        <v>58.115</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -18975,6 +19092,9 @@
       <c r="EI24" s="3" t="n">
         <v>25.213</v>
       </c>
+      <c r="EJ24" s="3" t="n">
+        <v>25.213</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -19394,6 +19514,9 @@
       <c r="EI25" s="3" t="n">
         <v>11.7845</v>
       </c>
+      <c r="EJ25" s="3" t="n">
+        <v>11.7845</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -19816,6 +19939,9 @@
       <c r="EI26" s="3" t="n">
         <v>10.5186</v>
       </c>
+      <c r="EJ26" s="3" t="n">
+        <v>10.5186</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -20238,6 +20364,9 @@
       <c r="EI27" s="3" t="n">
         <v>64.6493</v>
       </c>
+      <c r="EJ27" s="3" t="n">
+        <v>64.6493</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -20663,6 +20792,9 @@
       <c r="EI28" s="3" t="n">
         <v>108.6049</v>
       </c>
+      <c r="EJ28" s="3" t="n">
+        <v>108.6049</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -21082,6 +21214,9 @@
       <c r="EI29" s="3" t="n">
         <v>11.209</v>
       </c>
+      <c r="EJ29" s="3" t="n">
+        <v>11.209</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -21501,6 +21636,9 @@
       <c r="EI30" s="3" t="n">
         <v>16.1908</v>
       </c>
+      <c r="EJ30" s="3" t="n">
+        <v>16.1908</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -21923,6 +22061,9 @@
       <c r="EI31" s="3" t="n">
         <v>373.1721</v>
       </c>
+      <c r="EJ31" s="3" t="n">
+        <v>373.1721</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -22348,6 +22489,9 @@
       <c r="EI32" s="3" t="n">
         <v>10.18</v>
       </c>
+      <c r="EJ32" s="3" t="n">
+        <v>10.18</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -22767,6 +22911,9 @@
       <c r="EI33" s="3" t="n">
         <v>18.3</v>
       </c>
+      <c r="EJ33" s="3" t="n">
+        <v>18.3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -23189,6 +23336,9 @@
       <c r="EI34" s="3" t="n">
         <v>232.9044</v>
       </c>
+      <c r="EJ34" s="3" t="n">
+        <v>232.9044</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -23611,6 +23761,9 @@
       <c r="EI35" s="3" t="n">
         <v>14.96</v>
       </c>
+      <c r="EJ35" s="3" t="n">
+        <v>14.96</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -24033,6 +24186,9 @@
       <c r="EI36" s="3" t="n">
         <v>354.6417</v>
       </c>
+      <c r="EJ36" s="3" t="n">
+        <v>354.6417</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -24455,6 +24611,9 @@
       <c r="EI37" s="3" t="n">
         <v>16.219</v>
       </c>
+      <c r="EJ37" s="3" t="n">
+        <v>16.219</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -24874,6 +25033,9 @@
       <c r="EI38" s="3" t="n">
         <v>13.1979</v>
       </c>
+      <c r="EJ38" s="3" t="n">
+        <v>13.1979</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -25293,6 +25455,9 @@
       <c r="EI39" s="3" t="n">
         <v>1024.3327</v>
       </c>
+      <c r="EJ39" s="3" t="n">
+        <v>1024.3327</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -25713,6 +25878,9 @@
         <v>19.7478</v>
       </c>
       <c r="EI40" s="3" t="n">
+        <v>19.1374</v>
+      </c>
+      <c r="EJ40" s="3" t="n">
         <v>19.1374</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-26
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -39,10 +39,10 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="00006100"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
-      <color rgb="009C0006"/>
+      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
@@ -97,9 +97,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -109,8 +109,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-25 07:14 IST</t>
+          <t>Generated: 2026-10-26 07:23 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>512060.5043869019</v>
+        <v>511065.9990386963</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-78721.51561309816</v>
+        <v>-79716.02096130373</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1332496808435337</v>
+        <v>-0.1349330518916329</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5254063.982425301</v>
+        <v>5253069.477077096</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>193281.9624253018</v>
+        <v>192287.4570770962</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.03819211372105329</v>
+        <v>0.03799560153296155</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-25</t>
+          <t>Last snapshot: 2026-10-26</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FN19"/>
+  <dimension ref="A1:FO19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -789,6 +789,7 @@
     <col width="21" customWidth="1" min="168" max="168"/>
     <col width="21" customWidth="1" min="169" max="169"/>
     <col width="21" customWidth="1" min="170" max="170"/>
+    <col width="21" customWidth="1" min="171" max="171"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1642,6 +1643,11 @@
           <t>2026-10-25</t>
         </is>
       </c>
+      <c r="FO1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1661,13 +1667,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>550.9000244140625</v>
+        <v>529.0499877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44072.001953125</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>254.491953124998</v>
+        <v>42323.9990234375</v>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>-1493.510976562502</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2154,6 +2160,9 @@
       </c>
       <c r="FN2" s="3" t="n">
         <v>550.9000244140625</v>
+      </c>
+      <c r="FO2" s="3" t="n">
+        <v>529.0499877929688</v>
       </c>
     </row>
     <row r="3">
@@ -2201,13 +2210,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1357</v>
+        <v>1381.099975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27140</v>
+        <v>27621.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4964.580000000002</v>
+        <v>-4482.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2697,6 +2706,9 @@
       </c>
       <c r="FN4" s="3" t="n">
         <v>1357</v>
+      </c>
+      <c r="FO4" s="3" t="n">
+        <v>1381.099975585938</v>
       </c>
     </row>
     <row r="5">
@@ -2717,13 +2729,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>462.75</v>
+        <v>467.25</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9255</v>
+        <v>9345</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4958.1</v>
+        <v>-4868.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3213,6 +3225,9 @@
       </c>
       <c r="FN5" s="3" t="n">
         <v>462.75</v>
+      </c>
+      <c r="FO5" s="3" t="n">
+        <v>467.25</v>
       </c>
     </row>
     <row r="6">
@@ -3233,13 +3248,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>354</v>
+        <v>353.2999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14160</v>
+        <v>14131.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-3342.240000000002</v>
+        <v>-3370.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3729,6 +3744,9 @@
       </c>
       <c r="FN6" s="3" t="n">
         <v>354</v>
+      </c>
+      <c r="FO6" s="3" t="n">
+        <v>353.2999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -3749,13 +3767,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>242.5</v>
+        <v>243.8000030517578</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24250</v>
+        <v>24380.00030517578</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2183.82</v>
+        <v>-2053.819694824218</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4245,6 +4263,9 @@
       </c>
       <c r="FN7" s="3" t="n">
         <v>242.5</v>
+      </c>
+      <c r="FO7" s="3" t="n">
+        <v>243.8000030517578</v>
       </c>
     </row>
     <row r="8">
@@ -4292,13 +4313,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>12.67000007629395</v>
+        <v>13</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>19005.00011444092</v>
+        <v>19500</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-12045.16988555908</v>
+        <v>-11550.17</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4788,6 +4809,9 @@
       </c>
       <c r="FN9" s="3" t="n">
         <v>12.67000007629395</v>
+      </c>
+      <c r="FO9" s="3" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="10">
@@ -4808,13 +4832,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>447.8500061035156</v>
+        <v>451.8999938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44785.00061035156</v>
+        <v>45189.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6713.479389648441</v>
+        <v>-6308.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5304,6 +5328,9 @@
       </c>
       <c r="FN10" s="3" t="n">
         <v>447.8500061035156</v>
+      </c>
+      <c r="FO10" s="3" t="n">
+        <v>451.8999938964844</v>
       </c>
     </row>
     <row r="11">
@@ -5324,13 +5351,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>18.04000091552734</v>
+        <v>17.64999961853027</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>18040.00091552734</v>
+        <v>17649.99961853027</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>8198.790915527345</v>
+        <v>7808.789618530274</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5820,6 +5847,9 @@
       </c>
       <c r="FN11" s="3" t="n">
         <v>18.04000091552734</v>
+      </c>
+      <c r="FO11" s="3" t="n">
+        <v>17.64999961853027</v>
       </c>
     </row>
     <row r="12">
@@ -5840,13 +5870,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2312.800048828125</v>
+        <v>2303.800048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>23128.00048828125</v>
+        <v>23038.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-4595.24951171875</v>
+        <v>-4685.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6336,6 +6366,9 @@
       </c>
       <c r="FN12" s="3" t="n">
         <v>2312.800048828125</v>
+      </c>
+      <c r="FO12" s="3" t="n">
+        <v>2303.800048828125</v>
       </c>
     </row>
     <row r="13">
@@ -6356,13 +6389,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>37.40000152587891</v>
+        <v>36.77000045776367</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22440.00091552734</v>
+        <v>22062.0002746582</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-12591.75908447266</v>
+        <v>-12969.7597253418</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6852,6 +6885,9 @@
       </c>
       <c r="FN13" s="3" t="n">
         <v>37.40000152587891</v>
+      </c>
+      <c r="FO13" s="3" t="n">
+        <v>36.77000045776367</v>
       </c>
     </row>
     <row r="14">
@@ -6872,13 +6908,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>576.7999877929688</v>
+        <v>602.6500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>28839.99938964844</v>
+        <v>30132.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-13622.51061035156</v>
+        <v>-12330.00877929688</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7368,6 +7404,9 @@
       </c>
       <c r="FN14" s="3" t="n">
         <v>576.7999877929688</v>
+      </c>
+      <c r="FO14" s="3" t="n">
+        <v>602.6500244140625</v>
       </c>
     </row>
     <row r="15">
@@ -7442,13 +7481,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>407.2999877929688</v>
+        <v>404.6000061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>20364.99938964844</v>
+        <v>20230.00030517578</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-1389.530610351561</v>
+        <v>-1524.529694824218</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7938,6 +7977,9 @@
       </c>
       <c r="FN17" s="3" t="n">
         <v>407.2999877929688</v>
+      </c>
+      <c r="FO17" s="3" t="n">
+        <v>404.6000061035156</v>
       </c>
     </row>
     <row r="18">
@@ -7958,13 +8000,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>348.1000061035156</v>
+        <v>336.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34810.00061035156</v>
+        <v>33689.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-11830.81938964844</v>
+        <v>-12950.82061035156</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8454,6 +8496,9 @@
       </c>
       <c r="FN18" s="3" t="n">
         <v>348.1000061035156</v>
+      </c>
+      <c r="FO18" s="3" t="n">
+        <v>336.8999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -8466,10 +8511,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>512060.5043869019</v>
+        <v>511065.9990386963</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-78721.51561309815</v>
+        <v>-79716.02096130372</v>
       </c>
     </row>
   </sheetData>
@@ -8483,7 +8528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EJ41"/>
+  <dimension ref="A1:EK41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8626,6 +8671,7 @@
     <col width="13" customWidth="1" min="138" max="138"/>
     <col width="13" customWidth="1" min="139" max="139"/>
     <col width="13" customWidth="1" min="140" max="140"/>
+    <col width="13" customWidth="1" min="141" max="141"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9329,6 +9375,11 @@
           <t>2026-10-25</t>
         </is>
       </c>
+      <c r="EK1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9757,6 +9808,9 @@
       <c r="EJ2" s="3" t="n">
         <v>55.8014</v>
       </c>
+      <c r="EK2" s="3" t="n">
+        <v>55.8014</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10179,6 +10233,9 @@
       <c r="EJ3" s="3" t="n">
         <v>26.1132</v>
       </c>
+      <c r="EK3" s="3" t="n">
+        <v>26.1132</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10601,6 +10658,9 @@
       <c r="EJ4" s="3" t="n">
         <v>11.45</v>
       </c>
+      <c r="EK4" s="3" t="n">
+        <v>11.45</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -11023,6 +11083,9 @@
       <c r="EJ5" s="3" t="n">
         <v>8.8916</v>
       </c>
+      <c r="EK5" s="3" t="n">
+        <v>8.8916</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11451,6 +11514,9 @@
       <c r="EJ6" s="3" t="n">
         <v>10.6973</v>
       </c>
+      <c r="EK6" s="3" t="n">
+        <v>10.6973</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11873,6 +11939,9 @@
       <c r="EJ7" s="3" t="n">
         <v>32.7421</v>
       </c>
+      <c r="EK7" s="3" t="n">
+        <v>32.7421</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12301,6 +12370,9 @@
       <c r="EJ8" s="3" t="n">
         <v>32.3871</v>
       </c>
+      <c r="EK8" s="3" t="n">
+        <v>32.3871</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12723,6 +12795,9 @@
       <c r="EJ9" s="3" t="n">
         <v>38.8661</v>
       </c>
+      <c r="EK9" s="3" t="n">
+        <v>38.8661</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -13145,6 +13220,9 @@
       <c r="EJ10" s="3" t="n">
         <v>49.0519</v>
       </c>
+      <c r="EK10" s="3" t="n">
+        <v>49.0519</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13567,6 +13645,9 @@
       <c r="EJ11" s="3" t="n">
         <v>100.2279</v>
       </c>
+      <c r="EK11" s="3" t="n">
+        <v>100.2279</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13995,6 +14076,9 @@
       <c r="EJ12" s="3" t="n">
         <v>213.423</v>
       </c>
+      <c r="EK12" s="3" t="n">
+        <v>213.423</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14423,6 +14507,9 @@
       <c r="EJ13" s="3" t="n">
         <v>20.656</v>
       </c>
+      <c r="EK13" s="3" t="n">
+        <v>20.656</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14845,6 +14932,9 @@
       <c r="EJ14" s="3" t="n">
         <v>34.7483</v>
       </c>
+      <c r="EK14" s="3" t="n">
+        <v>34.7483</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -15273,6 +15363,9 @@
       <c r="EJ15" s="3" t="n">
         <v>10.61</v>
       </c>
+      <c r="EK15" s="3" t="n">
+        <v>10.61</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15695,6 +15788,9 @@
       <c r="EJ16" s="3" t="n">
         <v>23.8966</v>
       </c>
+      <c r="EK16" s="3" t="n">
+        <v>23.8966</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -16117,6 +16213,9 @@
       <c r="EJ17" s="3" t="n">
         <v>16.5054</v>
       </c>
+      <c r="EK17" s="3" t="n">
+        <v>16.5054</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -16545,6 +16644,9 @@
       <c r="EJ18" s="3" t="n">
         <v>43.47</v>
       </c>
+      <c r="EK18" s="3" t="n">
+        <v>43.47</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -16967,6 +17069,9 @@
       <c r="EJ19" s="3" t="n">
         <v>11.3218</v>
       </c>
+      <c r="EK19" s="3" t="n">
+        <v>11.3218</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -17395,6 +17500,9 @@
       <c r="EJ20" s="3" t="n">
         <v>9.93</v>
       </c>
+      <c r="EK20" s="3" t="n">
+        <v>9.93</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -17823,6 +17931,9 @@
       <c r="EJ21" s="3" t="n">
         <v>105.9959</v>
       </c>
+      <c r="EK21" s="3" t="n">
+        <v>105.9959</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -18245,6 +18356,9 @@
       <c r="EJ22" s="3" t="n">
         <v>39.638</v>
       </c>
+      <c r="EK22" s="3" t="n">
+        <v>39.638</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -18673,6 +18787,9 @@
       <c r="EJ23" s="3" t="n">
         <v>58.115</v>
       </c>
+      <c r="EK23" s="3" t="n">
+        <v>58.115</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -19095,6 +19212,9 @@
       <c r="EJ24" s="3" t="n">
         <v>25.213</v>
       </c>
+      <c r="EK24" s="3" t="n">
+        <v>25.213</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -19517,6 +19637,9 @@
       <c r="EJ25" s="3" t="n">
         <v>11.7845</v>
       </c>
+      <c r="EK25" s="3" t="n">
+        <v>11.7845</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -19942,6 +20065,9 @@
       <c r="EJ26" s="3" t="n">
         <v>10.5186</v>
       </c>
+      <c r="EK26" s="3" t="n">
+        <v>10.5186</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -20367,6 +20493,9 @@
       <c r="EJ27" s="3" t="n">
         <v>64.6493</v>
       </c>
+      <c r="EK27" s="3" t="n">
+        <v>64.6493</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -20795,6 +20924,9 @@
       <c r="EJ28" s="3" t="n">
         <v>108.6049</v>
       </c>
+      <c r="EK28" s="3" t="n">
+        <v>108.6049</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -21217,6 +21349,9 @@
       <c r="EJ29" s="3" t="n">
         <v>11.209</v>
       </c>
+      <c r="EK29" s="3" t="n">
+        <v>11.209</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -21639,6 +21774,9 @@
       <c r="EJ30" s="3" t="n">
         <v>16.1908</v>
       </c>
+      <c r="EK30" s="3" t="n">
+        <v>16.1908</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -22064,6 +22202,9 @@
       <c r="EJ31" s="3" t="n">
         <v>373.1721</v>
       </c>
+      <c r="EK31" s="3" t="n">
+        <v>373.1721</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -22492,6 +22633,9 @@
       <c r="EJ32" s="3" t="n">
         <v>10.18</v>
       </c>
+      <c r="EK32" s="3" t="n">
+        <v>10.18</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -22914,6 +23058,9 @@
       <c r="EJ33" s="3" t="n">
         <v>18.3</v>
       </c>
+      <c r="EK33" s="3" t="n">
+        <v>18.3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -23339,6 +23486,9 @@
       <c r="EJ34" s="3" t="n">
         <v>232.9044</v>
       </c>
+      <c r="EK34" s="3" t="n">
+        <v>232.9044</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -23764,6 +23914,9 @@
       <c r="EJ35" s="3" t="n">
         <v>14.96</v>
       </c>
+      <c r="EK35" s="3" t="n">
+        <v>14.96</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -24189,6 +24342,9 @@
       <c r="EJ36" s="3" t="n">
         <v>354.6417</v>
       </c>
+      <c r="EK36" s="3" t="n">
+        <v>354.6417</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -24614,6 +24770,9 @@
       <c r="EJ37" s="3" t="n">
         <v>16.219</v>
       </c>
+      <c r="EK37" s="3" t="n">
+        <v>16.219</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -25036,6 +25195,9 @@
       <c r="EJ38" s="3" t="n">
         <v>13.1979</v>
       </c>
+      <c r="EK38" s="3" t="n">
+        <v>13.1979</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -25458,6 +25620,9 @@
       <c r="EJ39" s="3" t="n">
         <v>1024.3327</v>
       </c>
+      <c r="EK39" s="3" t="n">
+        <v>1024.3327</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -25881,6 +26046,9 @@
         <v>19.1374</v>
       </c>
       <c r="EJ40" s="3" t="n">
+        <v>19.1374</v>
+      </c>
+      <c r="EK40" s="3" t="n">
         <v>19.1374</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-27
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-26 07:23 IST</t>
+          <t>Generated: 2026-10-27 07:14 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4742003.478038399</v>
+        <v>4792053.5972701</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>272003.4780383995</v>
+        <v>322053.5972701004</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.0608508899414764</v>
+        <v>0.07204778462418353</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>511065.9990386963</v>
+        <v>512825.4987983704</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-79716.02096130373</v>
+        <v>-77956.52120162966</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1349330518916329</v>
+        <v>-0.1319547964605112</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5253069.477077096</v>
+        <v>5304879.096068471</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>192287.4570770962</v>
+        <v>244097.0760684712</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.03799560153296155</v>
+        <v>0.04823307447422349</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-26</t>
+          <t>Last snapshot: 2026-10-27</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FO19"/>
+  <dimension ref="A1:FP19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -790,6 +790,7 @@
     <col width="21" customWidth="1" min="169" max="169"/>
     <col width="21" customWidth="1" min="170" max="170"/>
     <col width="21" customWidth="1" min="171" max="171"/>
+    <col width="21" customWidth="1" min="172" max="172"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1648,6 +1649,11 @@
           <t>2026-10-26</t>
         </is>
       </c>
+      <c r="FP1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1667,13 +1673,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>529.0499877929688</v>
+        <v>534.9500122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42323.9990234375</v>
+        <v>42796.0009765625</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-1493.510976562502</v>
+        <v>-1021.509023437502</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2163,6 +2169,9 @@
       </c>
       <c r="FO2" s="3" t="n">
         <v>529.0499877929688</v>
+      </c>
+      <c r="FP2" s="3" t="n">
+        <v>534.9500122070312</v>
       </c>
     </row>
     <row r="3">
@@ -2210,13 +2219,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1381.099975585938</v>
+        <v>1361.099975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27621.99951171875</v>
+        <v>27221.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4482.580488281252</v>
+        <v>-4882.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2709,6 +2718,9 @@
       </c>
       <c r="FO4" s="3" t="n">
         <v>1381.099975585938</v>
+      </c>
+      <c r="FP4" s="3" t="n">
+        <v>1361.099975585938</v>
       </c>
     </row>
     <row r="5">
@@ -2729,13 +2741,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>467.25</v>
+        <v>465.8500061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9345</v>
+        <v>9317.000122070312</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4868.1</v>
+        <v>-4896.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3228,6 +3240,9 @@
       </c>
       <c r="FO5" s="3" t="n">
         <v>467.25</v>
+      </c>
+      <c r="FP5" s="3" t="n">
+        <v>465.8500061035156</v>
       </c>
     </row>
     <row r="6">
@@ -3248,13 +3263,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>353.2999877929688</v>
+        <v>339.4500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14131.99951171875</v>
+        <v>13578.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-3370.240488281252</v>
+        <v>-3924.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3747,6 +3762,9 @@
       </c>
       <c r="FO6" s="3" t="n">
         <v>353.2999877929688</v>
+      </c>
+      <c r="FP6" s="3" t="n">
+        <v>339.4500122070312</v>
       </c>
     </row>
     <row r="7">
@@ -3767,13 +3785,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>243.8000030517578</v>
+        <v>254.4499969482422</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24380.00030517578</v>
+        <v>25444.99969482422</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2053.819694824218</v>
+        <v>-988.820305175781</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4266,6 +4284,9 @@
       </c>
       <c r="FO7" s="3" t="n">
         <v>243.8000030517578</v>
+      </c>
+      <c r="FP7" s="3" t="n">
+        <v>254.4499969482422</v>
       </c>
     </row>
     <row r="8">
@@ -4313,13 +4334,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>13</v>
+        <v>13.19999980926514</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>19500</v>
+        <v>19799.99971389771</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-11550.17</v>
+        <v>-11250.17028610229</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4812,6 +4833,9 @@
       </c>
       <c r="FO9" s="3" t="n">
         <v>13</v>
+      </c>
+      <c r="FP9" s="3" t="n">
+        <v>13.19999980926514</v>
       </c>
     </row>
     <row r="10">
@@ -4832,13 +4856,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>451.8999938964844</v>
+        <v>451.7000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45189.99938964844</v>
+        <v>45170.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6308.480610351566</v>
+        <v>-6328.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5331,6 +5355,9 @@
       </c>
       <c r="FO10" s="3" t="n">
         <v>451.8999938964844</v>
+      </c>
+      <c r="FP10" s="3" t="n">
+        <v>451.7000122070312</v>
       </c>
     </row>
     <row r="11">
@@ -5351,13 +5378,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>17.64999961853027</v>
+        <v>17.06999969482422</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>17649.99961853027</v>
+        <v>17069.99969482422</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>7808.789618530274</v>
+        <v>7228.78969482422</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5850,6 +5877,9 @@
       </c>
       <c r="FO11" s="3" t="n">
         <v>17.64999961853027</v>
+      </c>
+      <c r="FP11" s="3" t="n">
+        <v>17.06999969482422</v>
       </c>
     </row>
     <row r="12">
@@ -5870,13 +5900,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2303.800048828125</v>
+        <v>2334.199951171875</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>23038.00048828125</v>
+        <v>23341.99951171875</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-4685.24951171875</v>
+        <v>-4381.25048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6369,6 +6399,9 @@
       </c>
       <c r="FO12" s="3" t="n">
         <v>2303.800048828125</v>
+      </c>
+      <c r="FP12" s="3" t="n">
+        <v>2334.199951171875</v>
       </c>
     </row>
     <row r="13">
@@ -6389,13 +6422,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>36.77000045776367</v>
+        <v>37.34999847412109</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22062.0002746582</v>
+        <v>22409.99908447266</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-12969.7597253418</v>
+        <v>-12621.76091552735</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6888,6 +6921,9 @@
       </c>
       <c r="FO13" s="3" t="n">
         <v>36.77000045776367</v>
+      </c>
+      <c r="FP13" s="3" t="n">
+        <v>37.34999847412109</v>
       </c>
     </row>
     <row r="14">
@@ -6908,13 +6944,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>602.6500244140625</v>
+        <v>601.8499755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>30132.50122070312</v>
+        <v>30092.49877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12330.00877929688</v>
+        <v>-12370.01122070313</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7407,6 +7443,9 @@
       </c>
       <c r="FO14" s="3" t="n">
         <v>602.6500244140625</v>
+      </c>
+      <c r="FP14" s="3" t="n">
+        <v>601.8499755859375</v>
       </c>
     </row>
     <row r="15">
@@ -7481,13 +7520,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>404.6000061035156</v>
+        <v>415.5499877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>20230.00030517578</v>
+        <v>20777.49938964844</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-1524.529694824218</v>
+        <v>-977.0306103515613</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -7980,6 +8019,9 @@
       </c>
       <c r="FO17" s="3" t="n">
         <v>404.6000061035156</v>
+      </c>
+      <c r="FP17" s="3" t="n">
+        <v>415.5499877929688</v>
       </c>
     </row>
     <row r="18">
@@ -8000,13 +8042,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>336.8999938964844</v>
+        <v>340.3500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>33689.99938964844</v>
+        <v>34035.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12950.82061035156</v>
+        <v>-12605.81938964844</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8499,6 +8541,9 @@
       </c>
       <c r="FO18" s="3" t="n">
         <v>336.8999938964844</v>
+      </c>
+      <c r="FP18" s="3" t="n">
+        <v>340.3500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -8511,10 +8556,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>511065.9990386963</v>
+        <v>512825.4987983704</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-79716.02096130372</v>
+        <v>-77956.52120162964</v>
       </c>
     </row>
   </sheetData>
@@ -8528,7 +8573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EK41"/>
+  <dimension ref="A1:EL41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8539,7 +8584,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -8672,6 +8717,7 @@
     <col width="13" customWidth="1" min="139" max="139"/>
     <col width="13" customWidth="1" min="140" max="140"/>
     <col width="13" customWidth="1" min="141" max="141"/>
+    <col width="13" customWidth="1" min="142" max="142"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9380,6 +9426,11 @@
           <t>2026-10-26</t>
         </is>
       </c>
+      <c r="EL1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9404,16 +9455,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>55.8014</v>
+        <v>56.2595</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>62636.0670748</v>
+        <v>63150.276079</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>12636.0670748</v>
+        <v>13150.276079</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.252721341496</v>
+        <v>0.2630055215800001</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9810,6 +9861,9 @@
       </c>
       <c r="EK2" s="3" t="n">
         <v>55.8014</v>
+      </c>
+      <c r="EL2" s="3" t="n">
+        <v>56.2595</v>
       </c>
     </row>
     <row r="3">
@@ -9835,16 +9889,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.1132</v>
+        <v>26.1714</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>64113.4681116</v>
+        <v>64256.3615082</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4113.468111599999</v>
+        <v>4256.361508200003</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.06855780185999999</v>
+        <v>0.07093935847000006</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -10235,6 +10289,9 @@
       </c>
       <c r="EK3" s="3" t="n">
         <v>26.1132</v>
+      </c>
+      <c r="EL3" s="3" t="n">
+        <v>26.1714</v>
       </c>
     </row>
     <row r="4">
@@ -10260,16 +10317,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>11.45</v>
+        <v>11.51</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>219909.76485</v>
+        <v>221062.13043</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>39909.76485000001</v>
+        <v>41062.13042999999</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2217209158333334</v>
+        <v>0.2281229468333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -10660,6 +10717,9 @@
       </c>
       <c r="EK4" s="3" t="n">
         <v>11.45</v>
+      </c>
+      <c r="EL4" s="3" t="n">
+        <v>11.51</v>
       </c>
     </row>
     <row r="5">
@@ -10685,16 +10745,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.8916</v>
+        <v>8.952500000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>163197.2088608</v>
+        <v>164314.97282</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-46802.79113920001</v>
+        <v>-45685.02718</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2228704339961905</v>
+        <v>-0.2175477484761905</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -11085,6 +11145,9 @@
       </c>
       <c r="EK5" s="3" t="n">
         <v>8.8916</v>
+      </c>
+      <c r="EL5" s="3" t="n">
+        <v>8.952500000000001</v>
       </c>
     </row>
     <row r="6">
@@ -11110,16 +11173,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.6973</v>
+        <v>10.8084</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>45238.6356621</v>
+        <v>45708.4750068</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-4761.364337899999</v>
+        <v>-4291.524993200001</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.09522728675799998</v>
+        <v>-0.08583049986400001</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -11516,6 +11579,9 @@
       </c>
       <c r="EK6" s="3" t="n">
         <v>10.6973</v>
+      </c>
+      <c r="EL6" s="3" t="n">
+        <v>10.8084</v>
       </c>
     </row>
     <row r="7">
@@ -11541,16 +11607,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>32.7421</v>
+        <v>33.214</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>72230.38228400001</v>
+        <v>73271.41256</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>12230.38228400001</v>
+        <v>13271.41256</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2038397047333334</v>
+        <v>0.2211902093333333</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -11941,6 +12007,9 @@
       </c>
       <c r="EK7" s="3" t="n">
         <v>32.7421</v>
+      </c>
+      <c r="EL7" s="3" t="n">
+        <v>33.214</v>
       </c>
     </row>
     <row r="8">
@@ -11966,16 +12035,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>32.3871</v>
+        <v>33.0075</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>51968.11395029999</v>
+        <v>52963.60344750001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1968.113950299994</v>
+        <v>2963.603447500005</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.03936227900599988</v>
+        <v>0.0592720689500001</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -12372,6 +12441,9 @@
       </c>
       <c r="EK8" s="3" t="n">
         <v>32.3871</v>
+      </c>
+      <c r="EL8" s="3" t="n">
+        <v>33.0075</v>
       </c>
     </row>
     <row r="9">
@@ -12397,16 +12469,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>38.8661</v>
+        <v>39.8397</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>125125.2502773</v>
+        <v>128259.6513021</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>25125.25027730002</v>
+        <v>28259.6513021</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.2512525027730002</v>
+        <v>0.282596513021</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -12797,6 +12869,9 @@
       </c>
       <c r="EK9" s="3" t="n">
         <v>38.8661</v>
+      </c>
+      <c r="EL9" s="3" t="n">
+        <v>39.8397</v>
       </c>
     </row>
     <row r="10">
@@ -12822,16 +12897,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49.0519</v>
+        <v>49.4232</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>139634.0326021</v>
+        <v>140690.9970888</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>39634.03260210002</v>
+        <v>40690.99708880001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3963403260210002</v>
+        <v>0.4069099708880001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -13222,6 +13297,9 @@
       </c>
       <c r="EK10" s="3" t="n">
         <v>49.0519</v>
+      </c>
+      <c r="EL10" s="3" t="n">
+        <v>49.4232</v>
       </c>
     </row>
     <row r="11">
@@ -13247,16 +13325,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>100.2279</v>
+        <v>101.374</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30160.4794401</v>
+        <v>30505.362706</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>160.4794400999999</v>
+        <v>505.3627059999963</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.005349314669999997</v>
+        <v>0.01684542353333321</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -13647,6 +13725,9 @@
       </c>
       <c r="EK11" s="3" t="n">
         <v>100.2279</v>
+      </c>
+      <c r="EL11" s="3" t="n">
+        <v>101.374</v>
       </c>
     </row>
     <row r="12">
@@ -13672,16 +13753,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>213.423</v>
+        <v>214.641</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>99353.10180600001</v>
+        <v>99920.10760199999</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>-646.898193999994</v>
+        <v>-79.89239800001087</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>-0.006468981939999939</v>
+        <v>-0.0007989239800001087</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -14078,6 +14159,9 @@
       </c>
       <c r="EK12" s="3" t="n">
         <v>213.423</v>
+      </c>
+      <c r="EL12" s="3" t="n">
+        <v>214.641</v>
       </c>
     </row>
     <row r="13">
@@ -14103,16 +14187,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.656</v>
+        <v>21.039</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>239353.56888</v>
+        <v>243791.621595</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>39353.56887999998</v>
+        <v>43791.621595</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1967678443999999</v>
+        <v>0.218958107975</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -14509,6 +14593,9 @@
       </c>
       <c r="EK13" s="3" t="n">
         <v>20.656</v>
+      </c>
+      <c r="EL13" s="3" t="n">
+        <v>21.039</v>
       </c>
     </row>
     <row r="14">
@@ -14534,16 +14621,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34.7483</v>
+        <v>34.1472</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>125358.1755698</v>
+        <v>123189.6436032</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>25358.17556980001</v>
+        <v>23189.64360320001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.2535817556980001</v>
+        <v>0.2318964360320001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -14934,6 +15021,9 @@
       </c>
       <c r="EK14" s="3" t="n">
         <v>34.7483</v>
+      </c>
+      <c r="EL14" s="3" t="n">
+        <v>34.1472</v>
       </c>
     </row>
     <row r="15">
@@ -14959,16 +15049,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>10.61</v>
+        <v>10.74</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>103383.27767</v>
+        <v>104649.99078</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>3383.277669999996</v>
+        <v>4649.990780000007</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.03383277669999996</v>
+        <v>0.04649990780000007</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -15365,6 +15455,9 @@
       </c>
       <c r="EK15" s="3" t="n">
         <v>10.61</v>
+      </c>
+      <c r="EL15" s="3" t="n">
+        <v>10.74</v>
       </c>
     </row>
     <row r="16">
@@ -15390,16 +15483,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>23.8966</v>
+        <v>24.21</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>136758.5212448</v>
+        <v>138552.08688</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>36758.52124479998</v>
+        <v>38552.08687999999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3675852124479998</v>
+        <v>0.3855208687999999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -15790,6 +15883,9 @@
       </c>
       <c r="EK16" s="3" t="n">
         <v>23.8966</v>
+      </c>
+      <c r="EL16" s="3" t="n">
+        <v>24.21</v>
       </c>
     </row>
     <row r="17">
@@ -15815,16 +15911,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.5054</v>
+        <v>16.5285</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54567.7932078</v>
+        <v>54644.1631245</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4567.793207800001</v>
+        <v>4644.163124500003</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.09135586415600003</v>
+        <v>0.09288326249000005</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -16215,6 +16311,9 @@
       </c>
       <c r="EK17" s="3" t="n">
         <v>16.5054</v>
+      </c>
+      <c r="EL17" s="3" t="n">
+        <v>16.5285</v>
       </c>
     </row>
     <row r="18">
@@ -16240,16 +16339,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>43.47</v>
+        <v>44.24</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>82003.37291999999</v>
+        <v>83455.92864</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>2003.372919999994</v>
+        <v>3455.928639999998</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.02504216149999993</v>
+        <v>0.04319910799999998</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -16646,6 +16745,9 @@
       </c>
       <c r="EK18" s="3" t="n">
         <v>43.47</v>
+      </c>
+      <c r="EL18" s="3" t="n">
+        <v>44.24</v>
       </c>
     </row>
     <row r="19">
@@ -16671,16 +16773,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.3218</v>
+        <v>11.3718</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>163789.8312988</v>
+        <v>164513.1695988</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>13789.83129879998</v>
+        <v>14513.16959880001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.09193220865866654</v>
+        <v>0.09675446399200009</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -17071,6 +17173,9 @@
       </c>
       <c r="EK19" s="3" t="n">
         <v>11.3218</v>
+      </c>
+      <c r="EL19" s="3" t="n">
+        <v>11.3718</v>
       </c>
     </row>
     <row r="20">
@@ -17096,16 +17201,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.93</v>
+        <v>10.13</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>260720.12379</v>
+        <v>265971.28439</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>10720.12378999998</v>
+        <v>15971.28439000004</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.04288049515999993</v>
+        <v>0.06388513756000018</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -17502,6 +17607,9 @@
       </c>
       <c r="EK20" s="3" t="n">
         <v>9.93</v>
+      </c>
+      <c r="EL20" s="3" t="n">
+        <v>10.13</v>
       </c>
     </row>
     <row r="21">
@@ -17527,16 +17635,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>105.9959</v>
+        <v>106.7684</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>161035.2250381</v>
+        <v>162208.8526156</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-8964.774961899995</v>
+        <v>-7791.147384399985</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.05273397036411762</v>
+        <v>-0.04583027873176462</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -17933,6 +18041,9 @@
       </c>
       <c r="EK21" s="3" t="n">
         <v>105.9959</v>
+      </c>
+      <c r="EL21" s="3" t="n">
+        <v>106.7684</v>
       </c>
     </row>
     <row r="22">
@@ -17958,16 +18069,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>39.638</v>
+        <v>39.265</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>60822.92548</v>
+        <v>60250.5719</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>822.9254799999981</v>
+        <v>250.5719000000026</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.01371542466666663</v>
+        <v>0.004176198333333377</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -18358,6 +18469,9 @@
       </c>
       <c r="EK22" s="3" t="n">
         <v>39.638</v>
+      </c>
+      <c r="EL22" s="3" t="n">
+        <v>39.265</v>
       </c>
     </row>
     <row r="23">
@@ -18383,16 +18497,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>58.115</v>
+        <v>58.2708</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>157867.479705</v>
+        <v>158290.7052636</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>7867.479705000005</v>
+        <v>8290.705263600015</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.05244986470000004</v>
+        <v>0.0552713684240001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -18789,6 +18903,9 @@
       </c>
       <c r="EK23" s="3" t="n">
         <v>58.115</v>
+      </c>
+      <c r="EL23" s="3" t="n">
+        <v>58.2708</v>
       </c>
     </row>
     <row r="24">
@@ -18814,16 +18931,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.213</v>
+        <v>25.5055</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>91608.561218</v>
+        <v>92671.326623</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-8391.438781999997</v>
+        <v>-7328.673376999999</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.08391438781999998</v>
+        <v>-0.07328673376999999</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -19214,6 +19331,9 @@
       </c>
       <c r="EK24" s="3" t="n">
         <v>25.213</v>
+      </c>
+      <c r="EL24" s="3" t="n">
+        <v>25.5055</v>
       </c>
     </row>
     <row r="25">
@@ -19239,16 +19359,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.7845</v>
+        <v>11.9355</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>193521.217253</v>
+        <v>196000.890027</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-6478.782747000019</v>
+        <v>-3999.109973000013</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.0323939137350001</v>
+        <v>-0.01999554986500007</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -19639,6 +19759,9 @@
       </c>
       <c r="EK25" s="3" t="n">
         <v>11.7845</v>
+      </c>
+      <c r="EL25" s="3" t="n">
+        <v>11.9355</v>
       </c>
     </row>
     <row r="26">
@@ -19664,16 +19787,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.5186</v>
+        <v>10.6609</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>125610.123399</v>
+        <v>127309.4294435</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>15610.12339899999</v>
+        <v>17309.4294435</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1419102127181817</v>
+        <v>0.1573584494863637</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -20067,6 +20190,9 @@
       </c>
       <c r="EK26" s="3" t="n">
         <v>10.5186</v>
+      </c>
+      <c r="EL26" s="3" t="n">
+        <v>10.6609</v>
       </c>
     </row>
     <row r="27">
@@ -20092,16 +20218,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.6493</v>
+        <v>65.8095</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>104140.971398</v>
+        <v>106009.89117</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-5859.028602000006</v>
+        <v>-3990.108830000012</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.05326389638181823</v>
+        <v>-0.03627371663636374</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -20495,6 +20621,9 @@
       </c>
       <c r="EK27" s="3" t="n">
         <v>64.6493</v>
+      </c>
+      <c r="EL27" s="3" t="n">
+        <v>65.8095</v>
       </c>
     </row>
     <row r="28">
@@ -20520,16 +20649,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>108.6049</v>
+        <v>110.2374</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>359119.1528193</v>
+        <v>364517.2703718</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-20880.84718069999</v>
+        <v>-15482.7296282</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.05494959784394734</v>
+        <v>-0.04074402533736843</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -20926,6 +21055,9 @@
       </c>
       <c r="EK28" s="3" t="n">
         <v>108.6049</v>
+      </c>
+      <c r="EL28" s="3" t="n">
+        <v>110.2374</v>
       </c>
     </row>
     <row r="29">
@@ -20951,16 +21083,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.209</v>
+        <v>11.3405</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>107647.906927</v>
+        <v>108910.7938715</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>7647.906926999989</v>
+        <v>8910.793871500005</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.07647906926999989</v>
+        <v>0.08910793871500006</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -21351,6 +21483,9 @@
       </c>
       <c r="EK29" s="3" t="n">
         <v>11.209</v>
+      </c>
+      <c r="EL29" s="3" t="n">
+        <v>11.3405</v>
       </c>
     </row>
     <row r="30">
@@ -21376,16 +21511,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.1908</v>
+        <v>16.2077</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>119744.9062788</v>
+        <v>119869.8963297</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>19744.90627879999</v>
+        <v>19869.89632969999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1974490627879999</v>
+        <v>0.1986989632969999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -21776,6 +21911,9 @@
       </c>
       <c r="EK30" s="3" t="n">
         <v>16.1908</v>
+      </c>
+      <c r="EL30" s="3" t="n">
+        <v>16.2077</v>
       </c>
     </row>
     <row r="31">
@@ -21801,16 +21939,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>373.1721</v>
+        <v>378.2158</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>99293.63236799999</v>
-      </c>
-      <c r="H31" s="6" t="n">
-        <v>-706.3676320000086</v>
-      </c>
-      <c r="I31" s="13" t="n">
-        <v>-0.007063676320000086</v>
+        <v>100635.660064</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>635.6600639999961</v>
+      </c>
+      <c r="I31" s="12" t="n">
+        <v>0.006356600639999961</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -22204,6 +22342,9 @@
       </c>
       <c r="EK31" s="3" t="n">
         <v>373.1721</v>
+      </c>
+      <c r="EL31" s="3" t="n">
+        <v>378.2158</v>
       </c>
     </row>
     <row r="32">
@@ -22229,16 +22370,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.18</v>
+        <v>10.28</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>215204.7928</v>
+        <v>217318.7888</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>15204.7928</v>
+        <v>17318.78879999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.07602396399999997</v>
+        <v>0.0865939439999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -22635,6 +22776,9 @@
       </c>
       <c r="EK32" s="3" t="n">
         <v>10.18</v>
+      </c>
+      <c r="EL32" s="3" t="n">
+        <v>10.28</v>
       </c>
     </row>
     <row r="33">
@@ -22660,16 +22804,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>65580.61199999999</v>
+        <v>65938.976</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>5580.611999999994</v>
+        <v>5938.975999999995</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.09301019999999989</v>
+        <v>0.09898293333333325</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -23060,6 +23204,9 @@
       </c>
       <c r="EK33" s="3" t="n">
         <v>18.3</v>
+      </c>
+      <c r="EL33" s="3" t="n">
+        <v>18.4</v>
       </c>
     </row>
     <row r="34">
@@ -23085,16 +23232,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>232.9044</v>
+        <v>235.1814</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>81873.11663640001</v>
+        <v>82673.5527234</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>1873.116636400009</v>
+        <v>2673.552723400004</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.02341395795500011</v>
+        <v>0.03341940904250005</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -23488,6 +23635,9 @@
       </c>
       <c r="EK34" s="3" t="n">
         <v>232.9044</v>
+      </c>
+      <c r="EL34" s="3" t="n">
+        <v>235.1814</v>
       </c>
     </row>
     <row r="35">
@@ -23513,16 +23663,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.96</v>
+        <v>15.19</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>106745.92808</v>
+        <v>108387.07537</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>6745.928079999998</v>
+        <v>8387.075369999991</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.06745928079999998</v>
+        <v>0.08387075369999991</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -23916,6 +24066,9 @@
       </c>
       <c r="EK35" s="3" t="n">
         <v>14.96</v>
+      </c>
+      <c r="EL35" s="3" t="n">
+        <v>15.19</v>
       </c>
     </row>
     <row r="36">
@@ -23941,16 +24094,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>354.6417</v>
+        <v>360.9395</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>165158.7675402</v>
+        <v>168091.690787</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>15158.7675402</v>
+        <v>18091.690787</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.101058450268</v>
+        <v>0.1206112719133333</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -24344,6 +24497,9 @@
       </c>
       <c r="EK36" s="3" t="n">
         <v>354.6417</v>
+      </c>
+      <c r="EL36" s="3" t="n">
+        <v>360.9395</v>
       </c>
     </row>
     <row r="37">
@@ -24369,16 +24525,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.219</v>
+        <v>16.508</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>61030.296691</v>
+        <v>62117.771612</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>11030.296691</v>
+        <v>12117.771612</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2206059338200001</v>
+        <v>0.2423554322399999</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -24772,6 +24928,9 @@
       </c>
       <c r="EK37" s="3" t="n">
         <v>16.219</v>
+      </c>
+      <c r="EL37" s="3" t="n">
+        <v>16.508</v>
       </c>
     </row>
     <row r="38">
@@ -24797,16 +24956,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.1979</v>
+        <v>13.3168</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>78929.8033878</v>
+        <v>79640.8826976</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>-1070.196612200001</v>
+        <v>-359.1173024000018</v>
       </c>
       <c r="I38" s="13" t="n">
-        <v>-0.01337745765250002</v>
+        <v>-0.004488966280000023</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -25197,6 +25356,9 @@
       </c>
       <c r="EK38" s="3" t="n">
         <v>13.1979</v>
+      </c>
+      <c r="EL38" s="3" t="n">
+        <v>13.3168</v>
       </c>
     </row>
     <row r="39">
@@ -25222,16 +25384,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1024.3327</v>
+        <v>1025.1243</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51094.7394087</v>
+        <v>51134.2252083</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1094.739408699999</v>
+        <v>1134.225208299998</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02189478817399999</v>
+        <v>0.02268450416599997</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -25622,6 +25784,9 @@
       </c>
       <c r="EK39" s="3" t="n">
         <v>1024.3327</v>
+      </c>
+      <c r="EL39" s="3" t="n">
+        <v>1025.1243</v>
       </c>
     </row>
     <row r="40">
@@ -25647,16 +25812,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.1374</v>
+        <v>19.2826</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>96472.1501098</v>
+        <v>97204.1072302</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>-3527.849890199999</v>
+        <v>-2795.892769800004</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>-0.03527849890199999</v>
+        <v>-0.02795892769800004</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -26050,6 +26215,9 @@
       </c>
       <c r="EK40" s="3" t="n">
         <v>19.1374</v>
+      </c>
+      <c r="EL40" s="3" t="n">
+        <v>19.2826</v>
       </c>
     </row>
     <row r="41">
@@ -26062,13 +26230,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4742003.478038399</v>
+        <v>4792053.5972701</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>272003.4780383999</v>
+        <v>322053.5972701</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.06085088994147649</v>
+        <v>0.07204778462418344</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-28
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -39,10 +39,10 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="009C0006"/>
+      <color rgb="00006100"/>
     </font>
     <font>
-      <color rgb="00006100"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
@@ -97,9 +97,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -109,8 +109,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -483,9 +483,9 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-27 07:14 IST</t>
+          <t>Generated: 2026-10-28 07:53 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4792053.5972701</v>
+        <v>4843567.5879383</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>322053.5972701004</v>
+        <v>373567.5879383003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07204778462418353</v>
+        <v>0.08357216732400455</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>512825.4987983704</v>
+        <v>512216.5001373291</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-77956.52120162966</v>
+        <v>-78565.51986267092</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1319547964605112</v>
+        <v>-0.132985631253082</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5304879.096068471</v>
+        <v>5355784.088075629</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>244097.0760684712</v>
+        <v>295002.0680756299</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.04823307447422349</v>
+        <v>0.0582917950051581</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-27</t>
+          <t>Last snapshot: 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FP19"/>
+  <dimension ref="A1:FQ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -791,6 +791,7 @@
     <col width="21" customWidth="1" min="170" max="170"/>
     <col width="21" customWidth="1" min="171" max="171"/>
     <col width="21" customWidth="1" min="172" max="172"/>
+    <col width="21" customWidth="1" min="173" max="173"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1654,6 +1655,11 @@
           <t>2026-10-27</t>
         </is>
       </c>
+      <c r="FQ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1673,13 +1679,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>534.9500122070312</v>
+        <v>555</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42796.0009765625</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>-1021.509023437502</v>
+        <v>44400</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>582.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2172,6 +2178,9 @@
       </c>
       <c r="FP2" s="3" t="n">
         <v>534.9500122070312</v>
+      </c>
+      <c r="FQ2" s="3" t="n">
+        <v>555</v>
       </c>
     </row>
     <row r="3">
@@ -2219,13 +2228,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1361.099975585938</v>
+        <v>1363.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27221.99951171875</v>
+        <v>27276.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4882.580488281252</v>
+        <v>-4828.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2721,6 +2730,9 @@
       </c>
       <c r="FP4" s="3" t="n">
         <v>1361.099975585938</v>
+      </c>
+      <c r="FQ4" s="3" t="n">
+        <v>1363.800048828125</v>
       </c>
     </row>
     <row r="5">
@@ -2741,13 +2753,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>465.8500061035156</v>
+        <v>464.1000061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9317.000122070312</v>
+        <v>9282.000122070312</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4896.099877929688</v>
+        <v>-4931.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3243,6 +3255,9 @@
       </c>
       <c r="FP5" s="3" t="n">
         <v>465.8500061035156</v>
+      </c>
+      <c r="FQ5" s="3" t="n">
+        <v>464.1000061035156</v>
       </c>
     </row>
     <row r="6">
@@ -3263,13 +3278,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>339.4500122070312</v>
+        <v>333.2999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13578.00048828125</v>
+        <v>13331.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-3924.239511718752</v>
+        <v>-4170.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3765,6 +3780,9 @@
       </c>
       <c r="FP6" s="3" t="n">
         <v>339.4500122070312</v>
+      </c>
+      <c r="FQ6" s="3" t="n">
+        <v>333.2999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -3785,13 +3803,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>254.4499969482422</v>
+        <v>254.9499969482422</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25444.99969482422</v>
+        <v>25494.99969482422</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-988.820305175781</v>
+        <v>-938.820305175781</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4287,6 +4305,9 @@
       </c>
       <c r="FP7" s="3" t="n">
         <v>254.4499969482422</v>
+      </c>
+      <c r="FQ7" s="3" t="n">
+        <v>254.9499969482422</v>
       </c>
     </row>
     <row r="8">
@@ -4334,13 +4355,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>13.19999980926514</v>
+        <v>13.09000015258789</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>19799.99971389771</v>
+        <v>19635.00022888184</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-11250.17028610229</v>
+        <v>-11415.16977111816</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4836,6 +4857,9 @@
       </c>
       <c r="FP9" s="3" t="n">
         <v>13.19999980926514</v>
+      </c>
+      <c r="FQ9" s="3" t="n">
+        <v>13.09000015258789</v>
       </c>
     </row>
     <row r="10">
@@ -4856,13 +4880,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>451.7000122070312</v>
+        <v>447.3500061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45170.00122070312</v>
+        <v>44735.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6328.478779296878</v>
+        <v>-6763.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5358,6 +5382,9 @@
       </c>
       <c r="FP10" s="3" t="n">
         <v>451.7000122070312</v>
+      </c>
+      <c r="FQ10" s="3" t="n">
+        <v>447.3500061035156</v>
       </c>
     </row>
     <row r="11">
@@ -5378,13 +5405,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>17.06999969482422</v>
+        <v>15.97999954223633</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>17069.99969482422</v>
+        <v>15979.99954223633</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>7228.78969482422</v>
+        <v>6138.789542236329</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5880,6 +5907,9 @@
       </c>
       <c r="FP11" s="3" t="n">
         <v>17.06999969482422</v>
+      </c>
+      <c r="FQ11" s="3" t="n">
+        <v>15.97999954223633</v>
       </c>
     </row>
     <row r="12">
@@ -5900,13 +5930,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2334.199951171875</v>
+        <v>2322.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>23341.99951171875</v>
+        <v>23223.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-4381.25048828125</v>
+        <v>-4500.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6402,6 +6432,9 @@
       </c>
       <c r="FP12" s="3" t="n">
         <v>2334.199951171875</v>
+      </c>
+      <c r="FQ12" s="3" t="n">
+        <v>2322.300048828125</v>
       </c>
     </row>
     <row r="13">
@@ -6422,13 +6455,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>37.34999847412109</v>
+        <v>37.43000030517578</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22409.99908447266</v>
+        <v>22458.00018310547</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-12621.76091552735</v>
+        <v>-12573.75981689453</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6924,6 +6957,9 @@
       </c>
       <c r="FP13" s="3" t="n">
         <v>37.34999847412109</v>
+      </c>
+      <c r="FQ13" s="3" t="n">
+        <v>37.43000030517578</v>
       </c>
     </row>
     <row r="14">
@@ -6944,13 +6980,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>601.8499755859375</v>
+        <v>599.2999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>30092.49877929688</v>
+        <v>29964.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12370.01122070313</v>
+        <v>-12497.51061035156</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7446,6 +7482,9 @@
       </c>
       <c r="FP14" s="3" t="n">
         <v>601.8499755859375</v>
+      </c>
+      <c r="FQ14" s="3" t="n">
+        <v>599.2999877929688</v>
       </c>
     </row>
     <row r="15">
@@ -7520,13 +7559,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>415.5499877929688</v>
+        <v>415.7999877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>20777.49938964844</v>
+        <v>20789.99938964844</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-977.0306103515613</v>
+        <v>-964.5306103515613</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -8022,6 +8061,9 @@
       </c>
       <c r="FP17" s="3" t="n">
         <v>415.5499877929688</v>
+      </c>
+      <c r="FQ17" s="3" t="n">
+        <v>415.7999877929688</v>
       </c>
     </row>
     <row r="18">
@@ -8042,13 +8084,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>340.3500061035156</v>
+        <v>338.75</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34035.00061035156</v>
+        <v>33875</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12605.81938964844</v>
+        <v>-12765.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8544,6 +8586,9 @@
       </c>
       <c r="FP18" s="3" t="n">
         <v>340.3500061035156</v>
+      </c>
+      <c r="FQ18" s="3" t="n">
+        <v>338.75</v>
       </c>
     </row>
     <row r="19">
@@ -8556,10 +8601,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>512825.4987983704</v>
+        <v>512216.5001373291</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-77956.52120162964</v>
+        <v>-78565.5198626709</v>
       </c>
     </row>
   </sheetData>
@@ -8573,7 +8618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL41"/>
+  <dimension ref="A1:EM41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8584,7 +8629,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -8718,6 +8763,7 @@
     <col width="13" customWidth="1" min="140" max="140"/>
     <col width="13" customWidth="1" min="141" max="141"/>
     <col width="13" customWidth="1" min="142" max="142"/>
+    <col width="13" customWidth="1" min="143" max="143"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9431,6 +9477,11 @@
           <t>2026-10-27</t>
         </is>
       </c>
+      <c r="EM1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9455,16 +9506,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.2595</v>
+        <v>56.628</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63150.276079</v>
+        <v>63563.910696</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13150.276079</v>
+        <v>13563.910696</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2630055215800001</v>
+        <v>0.27127821392</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9864,6 +9915,9 @@
       </c>
       <c r="EL2" s="3" t="n">
         <v>56.2595</v>
+      </c>
+      <c r="EM2" s="3" t="n">
+        <v>56.628</v>
       </c>
     </row>
     <row r="3">
@@ -9889,16 +9943,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.1714</v>
+        <v>26.2197</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>64256.3615082</v>
+        <v>64374.9482961</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4256.361508200003</v>
+        <v>4374.948296100003</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.07093935847000006</v>
+        <v>0.07291580493500005</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -10292,6 +10346,9 @@
       </c>
       <c r="EL3" s="3" t="n">
         <v>26.1714</v>
+      </c>
+      <c r="EM3" s="3" t="n">
+        <v>26.2197</v>
       </c>
     </row>
     <row r="4">
@@ -10317,16 +10374,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>11.51</v>
+        <v>11.54</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>221062.13043</v>
+        <v>221638.31322</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>41062.13042999999</v>
+        <v>41638.31321999998</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2281229468333333</v>
+        <v>0.2313239623333332</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -10720,6 +10777,9 @@
       </c>
       <c r="EL4" s="3" t="n">
         <v>11.51</v>
+      </c>
+      <c r="EM4" s="3" t="n">
+        <v>11.54</v>
       </c>
     </row>
     <row r="5">
@@ -10745,16 +10805,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.952500000000001</v>
+        <v>8.9582</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>164314.97282</v>
+        <v>164419.5911216</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-45685.02718</v>
+        <v>-45580.40887840002</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2175477484761905</v>
+        <v>-0.2170495660876191</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -11148,6 +11208,9 @@
       </c>
       <c r="EL5" s="3" t="n">
         <v>8.952500000000001</v>
+      </c>
+      <c r="EM5" s="3" t="n">
+        <v>8.9582</v>
       </c>
     </row>
     <row r="6">
@@ -11173,16 +11236,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.8084</v>
+        <v>10.9409</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>45708.4750068</v>
+        <v>46268.8144593</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-4291.524993200001</v>
+        <v>-3731.185540700004</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.08583049986400001</v>
+        <v>-0.07462371081400007</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -11582,6 +11645,9 @@
       </c>
       <c r="EL6" s="3" t="n">
         <v>10.8084</v>
+      </c>
+      <c r="EM6" s="3" t="n">
+        <v>10.9409</v>
       </c>
     </row>
     <row r="7">
@@ -11607,16 +11673,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.214</v>
+        <v>33.2013</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73271.41256</v>
+        <v>73243.395852</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13271.41256</v>
+        <v>13243.395852</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2211902093333333</v>
+        <v>0.2207232642</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -12010,6 +12076,9 @@
       </c>
       <c r="EL7" s="3" t="n">
         <v>33.214</v>
+      </c>
+      <c r="EM7" s="3" t="n">
+        <v>33.2013</v>
       </c>
     </row>
     <row r="8">
@@ -12035,16 +12104,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.0075</v>
+        <v>33.8477</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>52963.60344750001</v>
+        <v>54311.7824861</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2963.603447500005</v>
+        <v>4311.782486100004</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.0592720689500001</v>
+        <v>0.0862356497220001</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -12444,6 +12513,9 @@
       </c>
       <c r="EL8" s="3" t="n">
         <v>33.0075</v>
+      </c>
+      <c r="EM8" s="3" t="n">
+        <v>33.8477</v>
       </c>
     </row>
     <row r="9">
@@ -12469,16 +12541,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>39.8397</v>
+        <v>40.1163</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>128259.6513021</v>
+        <v>129150.1354059</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>28259.6513021</v>
+        <v>29150.13540590002</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.282596513021</v>
+        <v>0.2915013540590001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -12872,6 +12944,9 @@
       </c>
       <c r="EL9" s="3" t="n">
         <v>39.8397</v>
+      </c>
+      <c r="EM9" s="3" t="n">
+        <v>40.1163</v>
       </c>
     </row>
     <row r="10">
@@ -12897,16 +12972,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49.4232</v>
+        <v>49.3794</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>140690.9970888</v>
+        <v>140566.3134246</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>40690.99708880001</v>
+        <v>40566.3134246</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.4069099708880001</v>
+        <v>0.405663134246</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -13300,6 +13375,9 @@
       </c>
       <c r="EL10" s="3" t="n">
         <v>49.4232</v>
+      </c>
+      <c r="EM10" s="3" t="n">
+        <v>49.3794</v>
       </c>
     </row>
     <row r="11">
@@ -13325,16 +13403,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>101.374</v>
+        <v>102.7339</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30505.362706</v>
+        <v>30914.5824541</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>505.3627059999963</v>
+        <v>914.5824541000002</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.01684542353333321</v>
+        <v>0.03048608180333334</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -13728,6 +13806,9 @@
       </c>
       <c r="EL11" s="3" t="n">
         <v>101.374</v>
+      </c>
+      <c r="EM11" s="3" t="n">
+        <v>102.7339</v>
       </c>
     </row>
     <row r="12">
@@ -13753,16 +13834,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>214.641</v>
+        <v>216.123</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>99920.10760199999</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>-79.89239800001087</v>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>-0.0007989239800001087</v>
+        <v>100610.011206</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>610.0112059999956</v>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>0.006100112059999956</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -14162,6 +14243,9 @@
       </c>
       <c r="EL12" s="3" t="n">
         <v>214.641</v>
+      </c>
+      <c r="EM12" s="3" t="n">
+        <v>216.123</v>
       </c>
     </row>
     <row r="13">
@@ -14187,16 +14271,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.039</v>
+        <v>21.496</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>243791.621595</v>
+        <v>249087.15708</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>43791.621595</v>
+        <v>49087.15707999998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.218958107975</v>
+        <v>0.2454357853999999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -14596,6 +14680,9 @@
       </c>
       <c r="EL13" s="3" t="n">
         <v>21.039</v>
+      </c>
+      <c r="EM13" s="3" t="n">
+        <v>21.496</v>
       </c>
     </row>
     <row r="14">
@@ -14621,16 +14708,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34.1472</v>
+        <v>34.317</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>123189.6436032</v>
+        <v>123802.215102</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>23189.64360320001</v>
+        <v>23802.215102</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.2318964360320001</v>
+        <v>0.23802215102</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -15024,6 +15111,9 @@
       </c>
       <c r="EL14" s="3" t="n">
         <v>34.1472</v>
+      </c>
+      <c r="EM14" s="3" t="n">
+        <v>34.317</v>
       </c>
     </row>
     <row r="15">
@@ -15049,16 +15139,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>10.74</v>
+        <v>10.87</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>104649.99078</v>
+        <v>105916.70389</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>4649.990780000007</v>
+        <v>5916.70388999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.04649990780000007</v>
+        <v>0.0591670388999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -15458,6 +15548,9 @@
       </c>
       <c r="EL15" s="3" t="n">
         <v>10.74</v>
+      </c>
+      <c r="EM15" s="3" t="n">
+        <v>10.87</v>
       </c>
     </row>
     <row r="16">
@@ -15483,16 +15576,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.21</v>
+        <v>24.524</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>138552.08688</v>
+        <v>140349.086272</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>38552.08687999999</v>
+        <v>40349.08627200002</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3855208687999999</v>
+        <v>0.4034908627200002</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -15886,6 +15979,9 @@
       </c>
       <c r="EL16" s="3" t="n">
         <v>24.21</v>
+      </c>
+      <c r="EM16" s="3" t="n">
+        <v>24.524</v>
       </c>
     </row>
     <row r="17">
@@ -15911,16 +16007,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.5285</v>
+        <v>16.5548</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54644.1631245</v>
+        <v>54731.1124236</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4644.163124500003</v>
+        <v>4731.112423599996</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.09288326249000005</v>
+        <v>0.09462224847199992</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -16314,6 +16410,9 @@
       </c>
       <c r="EL17" s="3" t="n">
         <v>16.5285</v>
+      </c>
+      <c r="EM17" s="3" t="n">
+        <v>16.5548</v>
       </c>
     </row>
     <row r="18">
@@ -16339,16 +16438,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.24</v>
+        <v>45</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>83455.92864</v>
+        <v>84889.62</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3455.928639999998</v>
+        <v>4889.619999999995</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.04319910799999998</v>
+        <v>0.06112024999999994</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -16748,6 +16847,9 @@
       </c>
       <c r="EL18" s="3" t="n">
         <v>44.24</v>
+      </c>
+      <c r="EM18" s="3" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="19">
@@ -16773,16 +16875,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.3718</v>
+        <v>11.4998</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>164513.1695988</v>
+        <v>166364.9156468</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>14513.16959880001</v>
+        <v>16364.91564680001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.09675446399200009</v>
+        <v>0.1090994376453334</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -17176,6 +17278,9 @@
       </c>
       <c r="EL19" s="3" t="n">
         <v>11.3718</v>
+      </c>
+      <c r="EM19" s="3" t="n">
+        <v>11.4998</v>
       </c>
     </row>
     <row r="20">
@@ -17201,16 +17306,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.13</v>
+        <v>10.25</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>265971.28439</v>
+        <v>269121.98075</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>15971.28439000004</v>
+        <v>19121.98074999999</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.06388513756000018</v>
+        <v>0.07648792299999996</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -17610,6 +17715,9 @@
       </c>
       <c r="EL20" s="3" t="n">
         <v>10.13</v>
+      </c>
+      <c r="EM20" s="3" t="n">
+        <v>10.25</v>
       </c>
     </row>
     <row r="21">
@@ -17635,16 +17743,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>106.7684</v>
+        <v>107.9072</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>162208.8526156</v>
+        <v>163938.9847648</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-7791.147384399985</v>
+        <v>-6061.0152352</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.04583027873176462</v>
+        <v>-0.03565303079529412</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -18044,6 +18152,9 @@
       </c>
       <c r="EL21" s="3" t="n">
         <v>106.7684</v>
+      </c>
+      <c r="EM21" s="3" t="n">
+        <v>107.9072</v>
       </c>
     </row>
     <row r="22">
@@ -18069,16 +18180,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>39.265</v>
+        <v>39.573</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>60250.5719</v>
+        <v>60723.18558</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>250.5719000000026</v>
+        <v>723.1855800000048</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.004176198333333377</v>
+        <v>0.01205309300000008</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -18472,6 +18583,9 @@
       </c>
       <c r="EL22" s="3" t="n">
         <v>39.265</v>
+      </c>
+      <c r="EM22" s="3" t="n">
+        <v>39.573</v>
       </c>
     </row>
     <row r="23">
@@ -18497,16 +18611,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>58.2708</v>
+        <v>59.0255</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>158290.7052636</v>
+        <v>160340.8229085</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>8290.705263600015</v>
+        <v>10340.82290850001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.0552713684240001</v>
+        <v>0.06893881939000004</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -18906,6 +19020,9 @@
       </c>
       <c r="EL23" s="3" t="n">
         <v>58.2708</v>
+      </c>
+      <c r="EM23" s="3" t="n">
+        <v>59.0255</v>
       </c>
     </row>
     <row r="24">
@@ -18931,16 +19048,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.5055</v>
+        <v>25.575</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>92671.326623</v>
+        <v>92923.84694999999</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-7328.673376999999</v>
+        <v>-7076.153050000008</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.07328673376999999</v>
+        <v>-0.07076153050000009</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -19334,6 +19451,9 @@
       </c>
       <c r="EL24" s="3" t="n">
         <v>25.5055</v>
+      </c>
+      <c r="EM24" s="3" t="n">
+        <v>25.575</v>
       </c>
     </row>
     <row r="25">
@@ -19359,16 +19479,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.9355</v>
+        <v>12.0442</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>196000.890027</v>
+        <v>197785.9259908</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-3999.109973000013</v>
+        <v>-2214.074009200005</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.01999554986500007</v>
+        <v>-0.01107037004600003</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -19762,6 +19882,9 @@
       </c>
       <c r="EL25" s="3" t="n">
         <v>11.9355</v>
+      </c>
+      <c r="EM25" s="3" t="n">
+        <v>12.0442</v>
       </c>
     </row>
     <row r="26">
@@ -19787,16 +19910,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.6609</v>
+        <v>10.7007</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>127309.4294435</v>
+        <v>127784.7097005</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>17309.4294435</v>
+        <v>17784.7097005</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1573584494863637</v>
+        <v>0.1616791790954545</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -20193,6 +20316,9 @@
       </c>
       <c r="EL26" s="3" t="n">
         <v>10.6609</v>
+      </c>
+      <c r="EM26" s="3" t="n">
+        <v>10.7007</v>
       </c>
     </row>
     <row r="27">
@@ -20218,16 +20344,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.8095</v>
+        <v>67.2077</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>106009.89117</v>
+        <v>108262.195622</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-3990.108830000012</v>
+        <v>-1737.804378000001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.03627371663636374</v>
+        <v>-0.01579822161818183</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -20624,6 +20750,9 @@
       </c>
       <c r="EL27" s="3" t="n">
         <v>65.8095</v>
+      </c>
+      <c r="EM27" s="3" t="n">
+        <v>67.2077</v>
       </c>
     </row>
     <row r="28">
@@ -20649,16 +20778,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>110.2374</v>
+        <v>110.8049</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>364517.2703718</v>
+        <v>366393.7982193</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-15482.7296282</v>
+        <v>-13606.20178069995</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.04074402533736843</v>
+        <v>-0.03580579415973671</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -21058,6 +21187,9 @@
       </c>
       <c r="EL28" s="3" t="n">
         <v>110.2374</v>
+      </c>
+      <c r="EM28" s="3" t="n">
+        <v>110.8049</v>
       </c>
     </row>
     <row r="29">
@@ -21083,16 +21215,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.3405</v>
+        <v>11.5473</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>108910.7938715</v>
+        <v>110896.8396519</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>8910.793871500005</v>
+        <v>10896.83965189999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.08910793871500006</v>
+        <v>0.1089683965189999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -21486,6 +21618,9 @@
       </c>
       <c r="EL29" s="3" t="n">
         <v>11.3405</v>
+      </c>
+      <c r="EM29" s="3" t="n">
+        <v>11.5473</v>
       </c>
     </row>
     <row r="30">
@@ -21511,16 +21646,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.2077</v>
+        <v>16.535</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>119869.8963297</v>
+        <v>122290.561635</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>19869.89632969999</v>
+        <v>22290.56163500001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1986989632969999</v>
+        <v>0.2229056163500001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -21914,6 +22049,9 @@
       </c>
       <c r="EL30" s="3" t="n">
         <v>16.2077</v>
+      </c>
+      <c r="EM30" s="3" t="n">
+        <v>16.535</v>
       </c>
     </row>
     <row r="31">
@@ -21939,16 +22077,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>378.2158</v>
+        <v>382.0159</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>100635.660064</v>
+        <v>101646.790672</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>635.6600639999961</v>
+        <v>1646.790671999988</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.006356600639999961</v>
+        <v>0.01646790671999988</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -22345,6 +22483,9 @@
       </c>
       <c r="EL31" s="3" t="n">
         <v>378.2158</v>
+      </c>
+      <c r="EM31" s="3" t="n">
+        <v>382.0159</v>
       </c>
     </row>
     <row r="32">
@@ -22370,16 +22511,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.28</v>
+        <v>10.42</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>217318.7888</v>
+        <v>220278.3832</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>17318.78879999998</v>
+        <v>20278.38319999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.0865939439999999</v>
+        <v>0.1013919159999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -22779,6 +22920,9 @@
       </c>
       <c r="EL32" s="3" t="n">
         <v>10.28</v>
+      </c>
+      <c r="EM32" s="3" t="n">
+        <v>10.42</v>
       </c>
     </row>
     <row r="33">
@@ -22804,16 +22948,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.4</v>
+        <v>18.78</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>65938.976</v>
+        <v>67300.7592</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>5938.975999999995</v>
+        <v>7300.7592</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.09898293333333325</v>
+        <v>0.12167932</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -23207,6 +23351,9 @@
       </c>
       <c r="EL33" s="3" t="n">
         <v>18.4</v>
+      </c>
+      <c r="EM33" s="3" t="n">
+        <v>18.78</v>
       </c>
     </row>
     <row r="34">
@@ -23232,16 +23379,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>235.1814</v>
+        <v>237.0089</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>82673.5527234</v>
+        <v>83315.9756259</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>2673.552723400004</v>
+        <v>3315.975625899999</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.03341940904250005</v>
+        <v>0.04144969532374999</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -23638,6 +23785,9 @@
       </c>
       <c r="EL34" s="3" t="n">
         <v>235.1814</v>
+      </c>
+      <c r="EM34" s="3" t="n">
+        <v>237.0089</v>
       </c>
     </row>
     <row r="35">
@@ -23663,16 +23813,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.19</v>
+        <v>15.57</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>108387.07537</v>
+        <v>111098.53611</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>8387.075369999991</v>
+        <v>11098.53611</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.08387075369999991</v>
+        <v>0.1109853611</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -24069,6 +24219,9 @@
       </c>
       <c r="EL35" s="3" t="n">
         <v>15.19</v>
+      </c>
+      <c r="EM35" s="3" t="n">
+        <v>15.57</v>
       </c>
     </row>
     <row r="36">
@@ -24094,16 +24247,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>360.9395</v>
+        <v>369.0319</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>168091.690787</v>
+        <v>171860.3700214</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>18091.690787</v>
+        <v>21860.37002140001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1206112719133333</v>
+        <v>0.1457358001426667</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -24500,6 +24653,9 @@
       </c>
       <c r="EL36" s="3" t="n">
         <v>360.9395</v>
+      </c>
+      <c r="EM36" s="3" t="n">
+        <v>369.0319</v>
       </c>
     </row>
     <row r="37">
@@ -24525,16 +24681,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.508</v>
+        <v>17.013</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62117.771612</v>
+        <v>64018.03055700001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12117.771612</v>
+        <v>14018.03055700001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2423554322399999</v>
+        <v>0.2803606111400001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -24931,6 +25087,9 @@
       </c>
       <c r="EL37" s="3" t="n">
         <v>16.508</v>
+      </c>
+      <c r="EM37" s="3" t="n">
+        <v>17.013</v>
       </c>
     </row>
     <row r="38">
@@ -24956,16 +25115,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.3168</v>
+        <v>13.3918</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>79640.8826976</v>
-      </c>
-      <c r="H38" s="6" t="n">
-        <v>-359.1173024000018</v>
-      </c>
-      <c r="I38" s="13" t="n">
-        <v>-0.004488966280000023</v>
+        <v>80089.4188476</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>89.41884759999812</v>
+      </c>
+      <c r="I38" s="12" t="n">
+        <v>0.001117735594999976</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -25359,6 +25518,9 @@
       </c>
       <c r="EL38" s="3" t="n">
         <v>13.3168</v>
+      </c>
+      <c r="EM38" s="3" t="n">
+        <v>13.3918</v>
       </c>
     </row>
     <row r="39">
@@ -25384,16 +25546,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.1243</v>
+        <v>1025.4124</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51134.2252083</v>
+        <v>51148.5959244</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1134.225208299998</v>
+        <v>1148.595924399997</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02268450416599997</v>
+        <v>0.02297191848799994</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -25787,6 +25949,9 @@
       </c>
       <c r="EL39" s="3" t="n">
         <v>1025.1243</v>
+      </c>
+      <c r="EM39" s="3" t="n">
+        <v>1025.4124</v>
       </c>
     </row>
     <row r="40">
@@ -25812,16 +25977,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.2826</v>
+        <v>19.4693</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>97204.1072302</v>
+        <v>98145.26697110001</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>-2795.892769800004</v>
+        <v>-1854.733028899995</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>-0.02795892769800004</v>
+        <v>-0.01854733028899995</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -26218,6 +26383,9 @@
       </c>
       <c r="EL40" s="3" t="n">
         <v>19.2826</v>
+      </c>
+      <c r="EM40" s="3" t="n">
+        <v>19.4693</v>
       </c>
     </row>
     <row r="41">
@@ -26230,13 +26398,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4792053.5972701</v>
+        <v>4843567.5879383</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>322053.5972701</v>
+        <v>373567.5879383</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07204778462418344</v>
+        <v>0.08357216732400446</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-29
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-28 07:53 IST</t>
+          <t>Generated: 2026-10-29 07:58 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4843567.5879383</v>
+        <v>4864403.6752617</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>373567.5879383003</v>
+        <v>394403.6752616996</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.08357216732400455</v>
+        <v>0.08823348439859051</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>512216.5001373291</v>
+        <v>512525.5005912781</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-78565.51986267092</v>
+        <v>-78256.51940872194</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.132985631253082</v>
+        <v>-0.1324625949325979</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5355784.088075629</v>
+        <v>5376929.175852978</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>295002.0680756299</v>
+        <v>316147.1558529781</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.0582917950051581</v>
+        <v>0.06247002036514866</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-28</t>
+          <t>Last snapshot: 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FQ19"/>
+  <dimension ref="A1:FR19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -792,6 +792,7 @@
     <col width="21" customWidth="1" min="171" max="171"/>
     <col width="21" customWidth="1" min="172" max="172"/>
     <col width="21" customWidth="1" min="173" max="173"/>
+    <col width="21" customWidth="1" min="174" max="174"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1660,6 +1661,11 @@
           <t>2026-10-28</t>
         </is>
       </c>
+      <c r="FR1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1679,13 +1685,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>555</v>
+        <v>551.7000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44400</v>
+        <v>44136.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>582.489999999998</v>
+        <v>318.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2181,6 +2187,9 @@
       </c>
       <c r="FQ2" s="3" t="n">
         <v>555</v>
+      </c>
+      <c r="FR2" s="3" t="n">
+        <v>551.7000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -2228,13 +2237,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1363.800048828125</v>
+        <v>1351.900024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27276.0009765625</v>
+        <v>27038.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4828.579023437502</v>
+        <v>-5066.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2733,6 +2742,9 @@
       </c>
       <c r="FQ4" s="3" t="n">
         <v>1363.800048828125</v>
+      </c>
+      <c r="FR4" s="3" t="n">
+        <v>1351.900024414062</v>
       </c>
     </row>
     <row r="5">
@@ -2753,13 +2765,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>464.1000061035156</v>
+        <v>460.0499877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9282.000122070312</v>
+        <v>9200.999755859375</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-4931.099877929688</v>
+        <v>-5012.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3258,6 +3270,9 @@
       </c>
       <c r="FQ5" s="3" t="n">
         <v>464.1000061035156</v>
+      </c>
+      <c r="FR5" s="3" t="n">
+        <v>460.0499877929688</v>
       </c>
     </row>
     <row r="6">
@@ -3278,13 +3293,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>333.2999877929688</v>
+        <v>336.1499938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13331.99951171875</v>
+        <v>13445.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4170.240488281252</v>
+        <v>-4056.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3783,6 +3798,9 @@
       </c>
       <c r="FQ6" s="3" t="n">
         <v>333.2999877929688</v>
+      </c>
+      <c r="FR6" s="3" t="n">
+        <v>336.1499938964844</v>
       </c>
     </row>
     <row r="7">
@@ -3803,13 +3821,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>254.9499969482422</v>
+        <v>262.6000061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25494.99969482422</v>
+        <v>26260.00061035156</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-938.820305175781</v>
+        <v>-173.8193896484372</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4308,6 +4326,9 @@
       </c>
       <c r="FQ7" s="3" t="n">
         <v>254.9499969482422</v>
+      </c>
+      <c r="FR7" s="3" t="n">
+        <v>262.6000061035156</v>
       </c>
     </row>
     <row r="8">
@@ -4355,13 +4376,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>13.09000015258789</v>
+        <v>13.03999996185303</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>19635.00022888184</v>
+        <v>19559.99994277954</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-11415.16977111816</v>
+        <v>-11490.17005722046</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4860,6 +4881,9 @@
       </c>
       <c r="FQ9" s="3" t="n">
         <v>13.09000015258789</v>
+      </c>
+      <c r="FR9" s="3" t="n">
+        <v>13.03999996185303</v>
       </c>
     </row>
     <row r="10">
@@ -4880,13 +4904,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>447.3500061035156</v>
+        <v>449.8500061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44735.00061035156</v>
+        <v>44985.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6763.479389648441</v>
+        <v>-6513.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5385,6 +5409,9 @@
       </c>
       <c r="FQ10" s="3" t="n">
         <v>447.3500061035156</v>
+      </c>
+      <c r="FR10" s="3" t="n">
+        <v>449.8500061035156</v>
       </c>
     </row>
     <row r="11">
@@ -5405,13 +5432,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>15.97999954223633</v>
+        <v>15.96000003814697</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>15979.99954223633</v>
+        <v>15960.00003814697</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>6138.789542236329</v>
+        <v>6118.790038146974</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5910,6 +5937,9 @@
       </c>
       <c r="FQ11" s="3" t="n">
         <v>15.97999954223633</v>
+      </c>
+      <c r="FR11" s="3" t="n">
+        <v>15.96000003814697</v>
       </c>
     </row>
     <row r="12">
@@ -5930,13 +5960,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2322.300048828125</v>
+        <v>2315.39990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>23223.00048828125</v>
+        <v>23153.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-4500.24951171875</v>
+        <v>-4569.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6435,6 +6465,9 @@
       </c>
       <c r="FQ12" s="3" t="n">
         <v>2322.300048828125</v>
+      </c>
+      <c r="FR12" s="3" t="n">
+        <v>2315.39990234375</v>
       </c>
     </row>
     <row r="13">
@@ -6455,13 +6488,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>37.43000030517578</v>
+        <v>36.75</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22458.00018310547</v>
+        <v>22050</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-12573.75981689453</v>
+        <v>-12981.76</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6960,6 +6993,9 @@
       </c>
       <c r="FQ13" s="3" t="n">
         <v>37.43000030517578</v>
+      </c>
+      <c r="FR13" s="3" t="n">
+        <v>36.75</v>
       </c>
     </row>
     <row r="14">
@@ -6980,13 +7016,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>599.2999877929688</v>
+        <v>599.7999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>29964.99938964844</v>
+        <v>29989.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12497.51061035156</v>
+        <v>-12472.51061035156</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7485,6 +7521,9 @@
       </c>
       <c r="FQ14" s="3" t="n">
         <v>599.2999877929688</v>
+      </c>
+      <c r="FR14" s="3" t="n">
+        <v>599.7999877929688</v>
       </c>
     </row>
     <row r="15">
@@ -7559,13 +7598,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>415.7999877929688</v>
+        <v>411.7000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>20789.99938964844</v>
+        <v>20585.00061035156</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-964.5306103515613</v>
+        <v>-1169.529389648436</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -8064,6 +8103,9 @@
       </c>
       <c r="FQ17" s="3" t="n">
         <v>415.7999877929688</v>
+      </c>
+      <c r="FR17" s="3" t="n">
+        <v>411.7000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -8084,13 +8126,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>338.75</v>
+        <v>343.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>33875</v>
+        <v>34389.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12765.82</v>
+        <v>-12250.82061035156</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8589,6 +8631,9 @@
       </c>
       <c r="FQ18" s="3" t="n">
         <v>338.75</v>
+      </c>
+      <c r="FR18" s="3" t="n">
+        <v>343.8999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -8601,10 +8646,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>512216.5001373291</v>
+        <v>512525.5005912781</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-78565.5198626709</v>
+        <v>-78256.51940872193</v>
       </c>
     </row>
   </sheetData>
@@ -8618,7 +8663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EM41"/>
+  <dimension ref="A1:EN41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8629,7 +8674,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -8764,6 +8809,7 @@
     <col width="13" customWidth="1" min="141" max="141"/>
     <col width="13" customWidth="1" min="142" max="142"/>
     <col width="13" customWidth="1" min="143" max="143"/>
+    <col width="13" customWidth="1" min="144" max="144"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9482,6 +9528,11 @@
           <t>2026-10-28</t>
         </is>
       </c>
+      <c r="EN1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9506,16 +9557,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.628</v>
+        <v>56.823</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63563.910696</v>
+        <v>63782.794686</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13563.910696</v>
+        <v>13782.794686</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.27127821392</v>
+        <v>0.27565589372</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9918,6 +9969,9 @@
       </c>
       <c r="EM2" s="3" t="n">
         <v>56.628</v>
+      </c>
+      <c r="EN2" s="3" t="n">
+        <v>56.823</v>
       </c>
     </row>
     <row r="3">
@@ -9943,16 +9997,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.2197</v>
+        <v>26.3515</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>64374.9482961</v>
+        <v>64698.54536950001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4374.948296100003</v>
+        <v>4698.545369500011</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.07291580493500005</v>
+        <v>0.07830908949166684</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -10349,6 +10403,9 @@
       </c>
       <c r="EM3" s="3" t="n">
         <v>26.2197</v>
+      </c>
+      <c r="EN3" s="3" t="n">
+        <v>26.3515</v>
       </c>
     </row>
     <row r="4">
@@ -10374,16 +10431,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>11.54</v>
+        <v>11.68</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>221638.31322</v>
+        <v>224327.16624</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>41638.31321999998</v>
+        <v>44327.16623999999</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2313239623333332</v>
+        <v>0.2462620346666666</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -10780,6 +10837,9 @@
       </c>
       <c r="EM4" s="3" t="n">
         <v>11.54</v>
+      </c>
+      <c r="EN4" s="3" t="n">
+        <v>11.68</v>
       </c>
     </row>
     <row r="5">
@@ -10805,16 +10865,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.9582</v>
+        <v>8.932399999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>164419.5911216</v>
+        <v>163946.0556512</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-45580.40887840002</v>
+        <v>-46053.94434880003</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2170495660876191</v>
+        <v>-0.2193044968990477</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -11211,6 +11271,9 @@
       </c>
       <c r="EM5" s="3" t="n">
         <v>8.9582</v>
+      </c>
+      <c r="EN5" s="3" t="n">
+        <v>8.932399999999999</v>
       </c>
     </row>
     <row r="6">
@@ -11236,16 +11299,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.9409</v>
+        <v>10.889</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>46268.8144593</v>
+        <v>46049.33055299999</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-3731.185540700004</v>
+        <v>-3950.669447000007</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.07462371081400007</v>
+        <v>-0.07901338894000015</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -11648,6 +11711,9 @@
       </c>
       <c r="EM6" s="3" t="n">
         <v>10.9409</v>
+      </c>
+      <c r="EN6" s="3" t="n">
+        <v>10.889</v>
       </c>
     </row>
     <row r="7">
@@ -11673,16 +11739,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.2013</v>
+        <v>33.114</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73243.395852</v>
+        <v>73050.80855999999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13243.395852</v>
+        <v>13050.80855999999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2207232642</v>
+        <v>0.2175134759999998</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -12079,6 +12145,9 @@
       </c>
       <c r="EM7" s="3" t="n">
         <v>33.2013</v>
+      </c>
+      <c r="EN7" s="3" t="n">
+        <v>33.114</v>
       </c>
     </row>
     <row r="8">
@@ -12104,16 +12173,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.8477</v>
+        <v>34.1148</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>54311.7824861</v>
+        <v>54740.36927640001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4311.782486100004</v>
+        <v>4740.369276400008</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.0862356497220001</v>
+        <v>0.09480738552800017</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -12516,6 +12585,9 @@
       </c>
       <c r="EM8" s="3" t="n">
         <v>33.8477</v>
+      </c>
+      <c r="EN8" s="3" t="n">
+        <v>34.1148</v>
       </c>
     </row>
     <row r="9">
@@ -12541,16 +12613,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.1163</v>
+        <v>40.3679</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>129150.1354059</v>
+        <v>129960.1346847</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>29150.13540590002</v>
+        <v>29960.13468469999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.2915013540590001</v>
+        <v>0.299601346847</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -12947,6 +13019,9 @@
       </c>
       <c r="EM9" s="3" t="n">
         <v>40.1163</v>
+      </c>
+      <c r="EN9" s="3" t="n">
+        <v>40.3679</v>
       </c>
     </row>
     <row r="10">
@@ -12972,16 +13047,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49.3794</v>
+        <v>49.4973</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>140566.3134246</v>
+        <v>140901.9345207</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>40566.3134246</v>
+        <v>40901.93452070002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.405663134246</v>
+        <v>0.4090193452070002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -13378,6 +13453,9 @@
       </c>
       <c r="EM10" s="3" t="n">
         <v>49.3794</v>
+      </c>
+      <c r="EN10" s="3" t="n">
+        <v>49.4973</v>
       </c>
     </row>
     <row r="11">
@@ -13403,16 +13481,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>102.7339</v>
+        <v>103.3369</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30914.5824541</v>
+        <v>31096.0366111</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>914.5824541000002</v>
+        <v>1096.036611099997</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.03048608180333334</v>
+        <v>0.03653455370333322</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -13809,6 +13887,9 @@
       </c>
       <c r="EM11" s="3" t="n">
         <v>102.7339</v>
+      </c>
+      <c r="EN11" s="3" t="n">
+        <v>103.3369</v>
       </c>
     </row>
     <row r="12">
@@ -13834,16 +13915,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>216.123</v>
+        <v>216.183</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>100610.011206</v>
+        <v>100637.942526</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>610.0112059999956</v>
+        <v>637.9425259999989</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.006100112059999956</v>
+        <v>0.006379425259999989</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -14246,6 +14327,9 @@
       </c>
       <c r="EM12" s="3" t="n">
         <v>216.123</v>
+      </c>
+      <c r="EN12" s="3" t="n">
+        <v>216.183</v>
       </c>
     </row>
     <row r="13">
@@ -14271,16 +14355,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.496</v>
+        <v>21.715</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>249087.15708</v>
+        <v>251624.842575</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>49087.15707999998</v>
+        <v>51624.84257499999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2454357853999999</v>
+        <v>0.2581242128749999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -14683,6 +14767,9 @@
       </c>
       <c r="EM13" s="3" t="n">
         <v>21.496</v>
+      </c>
+      <c r="EN13" s="3" t="n">
+        <v>21.715</v>
       </c>
     </row>
     <row r="14">
@@ -14708,16 +14795,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34.317</v>
+        <v>34.8352</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>123802.215102</v>
+        <v>125671.6765312</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>23802.215102</v>
+        <v>25671.67653120001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.23802215102</v>
+        <v>0.2567167653120001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -15114,6 +15201,9 @@
       </c>
       <c r="EM14" s="3" t="n">
         <v>34.317</v>
+      </c>
+      <c r="EN14" s="3" t="n">
+        <v>34.8352</v>
       </c>
     </row>
     <row r="15">
@@ -15139,16 +15229,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>10.87</v>
+        <v>10.83</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>105916.70389</v>
+        <v>105526.94601</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>5916.70388999999</v>
+        <v>5526.94601</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.0591670388999999</v>
+        <v>0.05526946009999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -15551,6 +15641,9 @@
       </c>
       <c r="EM15" s="3" t="n">
         <v>10.87</v>
+      </c>
+      <c r="EN15" s="3" t="n">
+        <v>10.83</v>
       </c>
     </row>
     <row r="16">
@@ -15576,16 +15669,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.524</v>
+        <v>24.6745</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>140349.086272</v>
+        <v>141210.386936</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>40349.08627200002</v>
+        <v>41210.386936</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4034908627200002</v>
+        <v>0.4121038693599999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -15982,6 +16075,9 @@
       </c>
       <c r="EM16" s="3" t="n">
         <v>24.524</v>
+      </c>
+      <c r="EN16" s="3" t="n">
+        <v>24.6745</v>
       </c>
     </row>
     <row r="17">
@@ -16007,16 +16103,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.5548</v>
+        <v>16.5511</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54731.1124236</v>
+        <v>54718.8800127</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4731.112423599996</v>
+        <v>4718.880012699999</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.09462224847199992</v>
+        <v>0.09437760025399999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -16413,6 +16509,9 @@
       </c>
       <c r="EM17" s="3" t="n">
         <v>16.5548</v>
+      </c>
+      <c r="EN17" s="3" t="n">
+        <v>16.5511</v>
       </c>
     </row>
     <row r="18">
@@ -16438,16 +16537,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45</v>
+        <v>45.75</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84889.62</v>
+        <v>86304.447</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4889.619999999995</v>
+        <v>6304.447</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06112024999999994</v>
+        <v>0.0788055875</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -16850,6 +16949,9 @@
       </c>
       <c r="EM18" s="3" t="n">
         <v>45</v>
+      </c>
+      <c r="EN18" s="3" t="n">
+        <v>45.75</v>
       </c>
     </row>
     <row r="19">
@@ -16875,16 +16977,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.4998</v>
+        <v>11.8215</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>166364.9156468</v>
+        <v>171018.874269</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>16364.91564680001</v>
+        <v>21018.87426899999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.1090994376453334</v>
+        <v>0.14012582846</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -17281,6 +17383,9 @@
       </c>
       <c r="EM19" s="3" t="n">
         <v>11.4998</v>
+      </c>
+      <c r="EN19" s="3" t="n">
+        <v>11.8215</v>
       </c>
     </row>
     <row r="20">
@@ -17306,16 +17411,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.25</v>
+        <v>10.17</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>269121.98075</v>
+        <v>267021.51651</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>19121.98074999999</v>
+        <v>17021.51650999999</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.07648792299999996</v>
+        <v>0.06808606603999995</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -17718,6 +17823,9 @@
       </c>
       <c r="EM20" s="3" t="n">
         <v>10.25</v>
+      </c>
+      <c r="EN20" s="3" t="n">
+        <v>10.17</v>
       </c>
     </row>
     <row r="21">
@@ -17743,16 +17851,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.9072</v>
+        <v>108.5534</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163938.9847648</v>
+        <v>164920.7299306</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6061.0152352</v>
+        <v>-5079.270069399994</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03565303079529412</v>
+        <v>-0.02987805923176467</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -18155,6 +18263,9 @@
       </c>
       <c r="EM21" s="3" t="n">
         <v>107.9072</v>
+      </c>
+      <c r="EN21" s="3" t="n">
+        <v>108.5534</v>
       </c>
     </row>
     <row r="22">
@@ -18180,16 +18291,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>39.573</v>
+        <v>40.366</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>60723.18558</v>
+        <v>61940.01236</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>723.1855800000048</v>
+        <v>1940.012360000001</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.01205309300000008</v>
+        <v>0.03233353933333334</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -18586,6 +18697,9 @@
       </c>
       <c r="EM22" s="3" t="n">
         <v>39.573</v>
+      </c>
+      <c r="EN22" s="3" t="n">
+        <v>40.366</v>
       </c>
     </row>
     <row r="23">
@@ -18611,16 +18725,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>59.0255</v>
+        <v>59.1519</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>160340.8229085</v>
+        <v>160684.1843373</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>10340.82290850001</v>
+        <v>10684.18433729999</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.06893881939000004</v>
+        <v>0.07122789558199991</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -19023,6 +19137,9 @@
       </c>
       <c r="EM23" s="3" t="n">
         <v>59.0255</v>
+      </c>
+      <c r="EN23" s="3" t="n">
+        <v>59.1519</v>
       </c>
     </row>
     <row r="24">
@@ -19048,16 +19165,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.575</v>
+        <v>25.3562</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>92923.84694999999</v>
+        <v>92128.8620932</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-7076.153050000008</v>
+        <v>-7871.137906799995</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.07076153050000009</v>
+        <v>-0.07871137906799995</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -19454,6 +19571,9 @@
       </c>
       <c r="EM24" s="3" t="n">
         <v>25.575</v>
+      </c>
+      <c r="EN24" s="3" t="n">
+        <v>25.3562</v>
       </c>
     </row>
     <row r="25">
@@ -19479,16 +19599,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.0442</v>
+        <v>12.1503</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>197785.9259908</v>
+        <v>199528.2656022</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-2214.074009200005</v>
+        <v>-471.7343978000281</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.01107037004600003</v>
+        <v>-0.002358671989000141</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -19885,6 +20005,9 @@
       </c>
       <c r="EM25" s="3" t="n">
         <v>12.0442</v>
+      </c>
+      <c r="EN25" s="3" t="n">
+        <v>12.1503</v>
       </c>
     </row>
     <row r="26">
@@ -19910,16 +20033,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.7007</v>
+        <v>10.6767</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>127784.7097005</v>
+        <v>127498.1085405</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>17784.7097005</v>
+        <v>17498.1085405</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1616791790954545</v>
+        <v>0.1590737140045455</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -20319,6 +20442,9 @@
       </c>
       <c r="EM26" s="3" t="n">
         <v>10.7007</v>
+      </c>
+      <c r="EN26" s="3" t="n">
+        <v>10.6767</v>
       </c>
     </row>
     <row r="27">
@@ -20344,16 +20470,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>67.2077</v>
+        <v>67.2714</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>108262.195622</v>
+        <v>108364.807404</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-1737.804378000001</v>
+        <v>-1635.192596000008</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.01579822161818183</v>
+        <v>-0.01486538723636371</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -20753,6 +20879,9 @@
       </c>
       <c r="EM27" s="3" t="n">
         <v>67.2077</v>
+      </c>
+      <c r="EN27" s="3" t="n">
+        <v>67.2714</v>
       </c>
     </row>
     <row r="28">
@@ -20778,16 +20907,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>110.8049</v>
+        <v>111.1353</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>366393.7982193</v>
+        <v>367486.3176921</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-13606.20178069995</v>
+        <v>-12513.68230789999</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.03580579415973671</v>
+        <v>-0.03293074291552629</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -21190,6 +21319,9 @@
       </c>
       <c r="EM28" s="3" t="n">
         <v>110.8049</v>
+      </c>
+      <c r="EN28" s="3" t="n">
+        <v>111.1353</v>
       </c>
     </row>
     <row r="29">
@@ -21215,16 +21347,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.5473</v>
+        <v>11.4984</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>110896.8396519</v>
+        <v>110427.2185752</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>10896.83965189999</v>
+        <v>10427.21857519999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1089683965189999</v>
+        <v>0.1042721857519999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -21621,6 +21753,9 @@
       </c>
       <c r="EM29" s="3" t="n">
         <v>11.5473</v>
+      </c>
+      <c r="EN29" s="3" t="n">
+        <v>11.4984</v>
       </c>
     </row>
     <row r="30">
@@ -21646,16 +21781,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.535</v>
+        <v>16.5695</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>122290.561635</v>
+        <v>122545.7188395</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>22290.56163500001</v>
+        <v>22545.71883950001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2229056163500001</v>
+        <v>0.2254571883950001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -22052,6 +22187,9 @@
       </c>
       <c r="EM30" s="3" t="n">
         <v>16.535</v>
+      </c>
+      <c r="EN30" s="3" t="n">
+        <v>16.5695</v>
       </c>
     </row>
     <row r="31">
@@ -22077,16 +22215,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>382.0159</v>
+        <v>382.3478</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>101646.790672</v>
+        <v>101735.102624</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>1646.790671999988</v>
+        <v>1735.102623999992</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.01646790671999988</v>
+        <v>0.01735102623999992</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -22486,6 +22624,9 @@
       </c>
       <c r="EM31" s="3" t="n">
         <v>382.0159</v>
+      </c>
+      <c r="EN31" s="3" t="n">
+        <v>382.3478</v>
       </c>
     </row>
     <row r="32">
@@ -22511,16 +22652,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.42</v>
+        <v>10.45</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>220278.3832</v>
+        <v>220912.582</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>20278.38319999998</v>
+        <v>20912.58199999997</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1013919159999999</v>
+        <v>0.1045629099999998</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -22923,6 +23064,9 @@
       </c>
       <c r="EM32" s="3" t="n">
         <v>10.42</v>
+      </c>
+      <c r="EN32" s="3" t="n">
+        <v>10.45</v>
       </c>
     </row>
     <row r="33">
@@ -22948,16 +23092,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.78</v>
+        <v>18.9</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67300.7592</v>
+        <v>67730.79599999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7300.7592</v>
+        <v>7730.795999999988</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.12167932</v>
+        <v>0.1288465999999998</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -23354,6 +23498,9 @@
       </c>
       <c r="EM33" s="3" t="n">
         <v>18.78</v>
+      </c>
+      <c r="EN33" s="3" t="n">
+        <v>18.9</v>
       </c>
     </row>
     <row r="34">
@@ -23379,16 +23526,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>237.0089</v>
+        <v>235.2384</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>83315.9756259</v>
+        <v>82693.58999040001</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>3315.975625899999</v>
+        <v>2693.589990400011</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.04144969532374999</v>
+        <v>0.03366987488000013</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -23788,6 +23935,9 @@
       </c>
       <c r="EM34" s="3" t="n">
         <v>237.0089</v>
+      </c>
+      <c r="EN34" s="3" t="n">
+        <v>235.2384</v>
       </c>
     </row>
     <row r="35">
@@ -23813,16 +23963,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.57</v>
+        <v>15.64</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>111098.53611</v>
+        <v>111598.01572</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>11098.53611</v>
+        <v>11598.01572</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1109853611</v>
+        <v>0.1159801572</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -24222,6 +24372,9 @@
       </c>
       <c r="EM35" s="3" t="n">
         <v>15.57</v>
+      </c>
+      <c r="EN35" s="3" t="n">
+        <v>15.64</v>
       </c>
     </row>
     <row r="36">
@@ -24247,16 +24400,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>369.0319</v>
+        <v>373.3714</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>171860.3700214</v>
+        <v>173881.3012084</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>21860.37002140001</v>
+        <v>23881.30120839999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1457358001426667</v>
+        <v>0.1592086747226666</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -24656,6 +24809,9 @@
       </c>
       <c r="EM36" s="3" t="n">
         <v>369.0319</v>
+      </c>
+      <c r="EN36" s="3" t="n">
+        <v>373.3714</v>
       </c>
     </row>
     <row r="37">
@@ -24681,16 +24837,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.013</v>
+        <v>17.185</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>64018.03055700001</v>
+        <v>64665.247465</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>14018.03055700001</v>
+        <v>14665.247465</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2803606111400001</v>
+        <v>0.2933049493</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -25090,6 +25246,9 @@
       </c>
       <c r="EM37" s="3" t="n">
         <v>17.013</v>
+      </c>
+      <c r="EN37" s="3" t="n">
+        <v>17.185</v>
       </c>
     </row>
     <row r="38">
@@ -25115,16 +25274,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.3918</v>
+        <v>13.3982</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>80089.4188476</v>
+        <v>80127.6939324</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>89.41884759999812</v>
+        <v>127.6939323999977</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.001117735594999976</v>
+        <v>0.001596174154999972</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -25521,6 +25680,9 @@
       </c>
       <c r="EM38" s="3" t="n">
         <v>13.3918</v>
+      </c>
+      <c r="EN38" s="3" t="n">
+        <v>13.3982</v>
       </c>
     </row>
     <row r="39">
@@ -25546,16 +25708,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.4124</v>
+        <v>1025.078</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51148.5959244</v>
+        <v>51131.915718</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1148.595924399997</v>
+        <v>1131.915717999997</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02297191848799994</v>
+        <v>0.02263831435999993</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -25952,6 +26114,9 @@
       </c>
       <c r="EM39" s="3" t="n">
         <v>1025.4124</v>
+      </c>
+      <c r="EN39" s="3" t="n">
+        <v>1025.078</v>
       </c>
     </row>
     <row r="40">
@@ -25977,16 +26142,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.4693</v>
+        <v>19.4632</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>98145.26697110001</v>
+        <v>98114.5167064</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>-1854.733028899995</v>
+        <v>-1885.483293600002</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>-0.01854733028899995</v>
+        <v>-0.01885483293600002</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -26386,6 +26551,9 @@
       </c>
       <c r="EM40" s="3" t="n">
         <v>19.4693</v>
+      </c>
+      <c r="EN40" s="3" t="n">
+        <v>19.4632</v>
       </c>
     </row>
     <row r="41">
@@ -26398,13 +26566,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4843567.5879383</v>
+        <v>4864403.6752617</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>373567.5879383</v>
+        <v>394403.6752616999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.08357216732400446</v>
+        <v>0.08823348439859058</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-30
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -39,10 +39,10 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="00006100"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
-      <color rgb="009C0006"/>
+      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
@@ -97,9 +97,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -109,8 +109,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-29 07:58 IST</t>
+          <t>Generated: 2026-10-30 08:01 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4864403.6752617</v>
+        <v>4882996.2213227</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>394403.6752616996</v>
+        <v>412996.2213227004</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.08823348439859051</v>
+        <v>0.09239289067621932</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>512525.5005912781</v>
+        <v>506758.4968643188</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-78256.51940872194</v>
+        <v>-84023.52313568117</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1324625949325979</v>
+        <v>-0.1422242388752474</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5376929.175852978</v>
+        <v>5389754.718187019</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>316147.1558529781</v>
+        <v>328972.6981870197</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06247002036514866</v>
+        <v>0.06500432085138884</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-29</t>
+          <t>Last snapshot: 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FR19"/>
+  <dimension ref="A1:FS19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -793,6 +793,7 @@
     <col width="21" customWidth="1" min="172" max="172"/>
     <col width="21" customWidth="1" min="173" max="173"/>
     <col width="21" customWidth="1" min="174" max="174"/>
+    <col width="21" customWidth="1" min="175" max="175"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1666,6 +1667,11 @@
           <t>2026-10-29</t>
         </is>
       </c>
+      <c r="FS1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1685,13 +1691,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>551.7000122070312</v>
+        <v>538</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44136.0009765625</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>318.490976562498</v>
+        <v>43040</v>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>-777.510000000002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2190,6 +2196,9 @@
       </c>
       <c r="FR2" s="3" t="n">
         <v>551.7000122070312</v>
+      </c>
+      <c r="FS2" s="3" t="n">
+        <v>538</v>
       </c>
     </row>
     <row r="3">
@@ -2237,13 +2246,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1351.900024414062</v>
+        <v>1335</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27038.00048828125</v>
+        <v>26700</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5066.579511718752</v>
+        <v>-5404.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2745,6 +2754,9 @@
       </c>
       <c r="FR4" s="3" t="n">
         <v>1351.900024414062</v>
+      </c>
+      <c r="FS4" s="3" t="n">
+        <v>1335</v>
       </c>
     </row>
     <row r="5">
@@ -2765,13 +2777,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>460.0499877929688</v>
+        <v>454.3500061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9200.999755859375</v>
+        <v>9087.000122070312</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-5012.100244140625</v>
+        <v>-5126.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3273,6 +3285,9 @@
       </c>
       <c r="FR5" s="3" t="n">
         <v>460.0499877929688</v>
+      </c>
+      <c r="FS5" s="3" t="n">
+        <v>454.3500061035156</v>
       </c>
     </row>
     <row r="6">
@@ -3293,13 +3308,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>336.1499938964844</v>
+        <v>329.3999938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13445.99975585938</v>
+        <v>13175.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4056.240244140627</v>
+        <v>-4326.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3801,6 +3816,9 @@
       </c>
       <c r="FR6" s="3" t="n">
         <v>336.1499938964844</v>
+      </c>
+      <c r="FS6" s="3" t="n">
+        <v>329.3999938964844</v>
       </c>
     </row>
     <row r="7">
@@ -3821,13 +3839,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>262.6000061035156</v>
+        <v>253.4499969482422</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>26260.00061035156</v>
+        <v>25344.99969482422</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-173.8193896484372</v>
+        <v>-1088.820305175781</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4329,6 +4347,9 @@
       </c>
       <c r="FR7" s="3" t="n">
         <v>262.6000061035156</v>
+      </c>
+      <c r="FS7" s="3" t="n">
+        <v>253.4499969482422</v>
       </c>
     </row>
     <row r="8">
@@ -4376,13 +4397,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>13.03999996185303</v>
+        <v>12.73999977111816</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>19559.99994277954</v>
+        <v>19109.99965667725</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-11490.17005722046</v>
+        <v>-11940.17034332275</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4884,6 +4905,9 @@
       </c>
       <c r="FR9" s="3" t="n">
         <v>13.03999996185303</v>
+      </c>
+      <c r="FS9" s="3" t="n">
+        <v>12.73999977111816</v>
       </c>
     </row>
     <row r="10">
@@ -4904,13 +4928,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>449.8500061035156</v>
+        <v>449.8999938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44985.00061035156</v>
+        <v>44989.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6513.479389648441</v>
+        <v>-6508.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5412,6 +5436,9 @@
       </c>
       <c r="FR10" s="3" t="n">
         <v>449.8500061035156</v>
+      </c>
+      <c r="FS10" s="3" t="n">
+        <v>449.8999938964844</v>
       </c>
     </row>
     <row r="11">
@@ -5432,13 +5459,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>15.96000003814697</v>
+        <v>15.64999961853027</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>15960.00003814697</v>
+        <v>15649.99961853027</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>6118.790038146974</v>
+        <v>5808.789618530274</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5940,6 +5967,9 @@
       </c>
       <c r="FR11" s="3" t="n">
         <v>15.96000003814697</v>
+      </c>
+      <c r="FS11" s="3" t="n">
+        <v>15.64999961853027</v>
       </c>
     </row>
     <row r="12">
@@ -5960,13 +5990,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2315.39990234375</v>
+        <v>2321.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>23153.9990234375</v>
+        <v>23213.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-4569.2509765625</v>
+        <v>-4510.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6468,6 +6498,9 @@
       </c>
       <c r="FR12" s="3" t="n">
         <v>2315.39990234375</v>
+      </c>
+      <c r="FS12" s="3" t="n">
+        <v>2321.300048828125</v>
       </c>
     </row>
     <row r="13">
@@ -6488,13 +6521,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>36.75</v>
+        <v>33.61999893188477</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>22050</v>
+        <v>20171.99935913086</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-12981.76</v>
+        <v>-14859.76064086914</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -6996,6 +7029,9 @@
       </c>
       <c r="FR13" s="3" t="n">
         <v>36.75</v>
+      </c>
+      <c r="FS13" s="3" t="n">
+        <v>33.61999893188477</v>
       </c>
     </row>
     <row r="14">
@@ -7016,13 +7052,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>599.7999877929688</v>
+        <v>594.75</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>29989.99938964844</v>
+        <v>29737.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12472.51061035156</v>
+        <v>-12725.01</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7524,6 +7560,9 @@
       </c>
       <c r="FR14" s="3" t="n">
         <v>599.7999877929688</v>
+      </c>
+      <c r="FS14" s="3" t="n">
+        <v>594.75</v>
       </c>
     </row>
     <row r="15">
@@ -7598,13 +7637,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>411.7000122070312</v>
+        <v>403.25</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>20585.00061035156</v>
+        <v>20162.5</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-1169.529389648436</v>
+        <v>-1592.029999999999</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -8106,6 +8145,9 @@
       </c>
       <c r="FR17" s="3" t="n">
         <v>411.7000122070312</v>
+      </c>
+      <c r="FS17" s="3" t="n">
+        <v>403.25</v>
       </c>
     </row>
     <row r="18">
@@ -8126,13 +8168,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>343.8999938964844</v>
+        <v>346.0499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34389.99938964844</v>
+        <v>34604.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12250.82061035156</v>
+        <v>-12035.82122070312</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8634,6 +8676,9 @@
       </c>
       <c r="FR18" s="3" t="n">
         <v>343.8999938964844</v>
+      </c>
+      <c r="FS18" s="3" t="n">
+        <v>346.0499877929688</v>
       </c>
     </row>
     <row r="19">
@@ -8646,10 +8691,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>512525.5005912781</v>
+        <v>506758.4968643188</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-78256.51940872193</v>
+        <v>-84023.52313568116</v>
       </c>
     </row>
   </sheetData>
@@ -8663,7 +8708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EN41"/>
+  <dimension ref="A1:EO41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8810,6 +8855,7 @@
     <col width="13" customWidth="1" min="142" max="142"/>
     <col width="13" customWidth="1" min="143" max="143"/>
     <col width="13" customWidth="1" min="144" max="144"/>
+    <col width="13" customWidth="1" min="145" max="145"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9533,6 +9579,11 @@
           <t>2026-10-29</t>
         </is>
       </c>
+      <c r="EO1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9557,16 +9608,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.823</v>
+        <v>56.749</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63782.794686</v>
+        <v>63699.731018</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13782.794686</v>
+        <v>13699.731018</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.27565589372</v>
+        <v>0.27399462036</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -9972,6 +10023,9 @@
       </c>
       <c r="EN2" s="3" t="n">
         <v>56.823</v>
+      </c>
+      <c r="EO2" s="3" t="n">
+        <v>56.749</v>
       </c>
     </row>
     <row r="3">
@@ -9997,16 +10051,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.3515</v>
+        <v>26.2575</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>64698.54536950001</v>
+        <v>64467.7553475</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4698.545369500011</v>
+        <v>4467.755347500002</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.07830908949166684</v>
+        <v>0.07446258912500003</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -10406,6 +10460,9 @@
       </c>
       <c r="EN3" s="3" t="n">
         <v>26.3515</v>
+      </c>
+      <c r="EO3" s="3" t="n">
+        <v>26.2575</v>
       </c>
     </row>
     <row r="4">
@@ -10431,16 +10488,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>11.68</v>
+        <v>11.52</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>224327.16624</v>
+        <v>221254.19136</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>44327.16623999999</v>
+        <v>41254.19136</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2462620346666666</v>
+        <v>0.229189952</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -10840,6 +10897,9 @@
       </c>
       <c r="EN4" s="3" t="n">
         <v>11.68</v>
+      </c>
+      <c r="EO4" s="3" t="n">
+        <v>11.52</v>
       </c>
     </row>
     <row r="5">
@@ -10865,16 +10925,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>8.932399999999999</v>
+        <v>9.008599999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>163946.0556512</v>
+        <v>165344.6371568</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-46053.94434880003</v>
+        <v>-44655.36284320001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2193044968990477</v>
+        <v>-0.2126445849676191</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -11274,6 +11334,9 @@
       </c>
       <c r="EN5" s="3" t="n">
         <v>8.932399999999999</v>
+      </c>
+      <c r="EO5" s="3" t="n">
+        <v>9.008599999999999</v>
       </c>
     </row>
     <row r="6">
@@ -11299,16 +11362,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.889</v>
+        <v>10.9809</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>46049.33055299999</v>
+        <v>46437.9735393</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-3950.669447000007</v>
+        <v>-3562.026460699999</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.07901338894000015</v>
+        <v>-0.07124052921399998</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -11714,6 +11777,9 @@
       </c>
       <c r="EN6" s="3" t="n">
         <v>10.889</v>
+      </c>
+      <c r="EO6" s="3" t="n">
+        <v>10.9809</v>
       </c>
     </row>
     <row r="7">
@@ -11739,16 +11805,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.114</v>
+        <v>33.4758</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73050.80855999999</v>
+        <v>73848.953832</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13050.80855999999</v>
+        <v>13848.953832</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2175134759999998</v>
+        <v>0.2308158972</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -12148,6 +12214,9 @@
       </c>
       <c r="EN7" s="3" t="n">
         <v>33.114</v>
+      </c>
+      <c r="EO7" s="3" t="n">
+        <v>33.4758</v>
       </c>
     </row>
     <row r="8">
@@ -12173,16 +12242,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>34.1148</v>
+        <v>34.637</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>54740.36927640001</v>
+        <v>55578.287741</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4740.369276400008</v>
+        <v>5578.287741</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.09480738552800017</v>
+        <v>0.11156575482</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -12588,6 +12657,9 @@
       </c>
       <c r="EN8" s="3" t="n">
         <v>34.1148</v>
+      </c>
+      <c r="EO8" s="3" t="n">
+        <v>34.637</v>
       </c>
     </row>
     <row r="9">
@@ -12613,16 +12685,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.3679</v>
+        <v>39.5494</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>129960.1346847</v>
+        <v>127325.0615142</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>29960.13468469999</v>
+        <v>27325.0615142</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.299601346847</v>
+        <v>0.273250615142</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -13022,6 +13094,9 @@
       </c>
       <c r="EN9" s="3" t="n">
         <v>40.3679</v>
+      </c>
+      <c r="EO9" s="3" t="n">
+        <v>39.5494</v>
       </c>
     </row>
     <row r="10">
@@ -13047,16 +13122,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49.4973</v>
+        <v>49.9171</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>140901.9345207</v>
+        <v>142096.9619689</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>40901.93452070002</v>
+        <v>42096.9619689</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.4090193452070002</v>
+        <v>0.4209696196889999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -13456,6 +13531,9 @@
       </c>
       <c r="EN10" s="3" t="n">
         <v>49.4973</v>
+      </c>
+      <c r="EO10" s="3" t="n">
+        <v>49.9171</v>
       </c>
     </row>
     <row r="11">
@@ -13481,16 +13559,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>103.3369</v>
+        <v>102.4307</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31096.0366111</v>
+        <v>30823.3438133</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1096.036611099997</v>
+        <v>823.3438132999981</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.03653455370333322</v>
+        <v>0.0274447937766666</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -13890,6 +13968,9 @@
       </c>
       <c r="EN11" s="3" t="n">
         <v>103.3369</v>
+      </c>
+      <c r="EO11" s="3" t="n">
+        <v>102.4307</v>
       </c>
     </row>
     <row r="12">
@@ -13915,16 +13996,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>216.183</v>
+        <v>217.641</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>100637.942526</v>
+        <v>101316.673602</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>637.9425259999989</v>
+        <v>1316.673601999995</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.006379425259999989</v>
+        <v>0.01316673601999995</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -14330,6 +14411,9 @@
       </c>
       <c r="EN12" s="3" t="n">
         <v>216.183</v>
+      </c>
+      <c r="EO12" s="3" t="n">
+        <v>217.641</v>
       </c>
     </row>
     <row r="13">
@@ -14355,16 +14439,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.715</v>
+        <v>21.862</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>251624.842575</v>
+        <v>253328.22051</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>51624.84257499999</v>
+        <v>53328.22050999998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2581242128749999</v>
+        <v>0.2666411025499999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -14770,6 +14854,9 @@
       </c>
       <c r="EN13" s="3" t="n">
         <v>21.715</v>
+      </c>
+      <c r="EO13" s="3" t="n">
+        <v>21.862</v>
       </c>
     </row>
     <row r="14">
@@ -14795,16 +14882,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34.8352</v>
+        <v>34.5554</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>125671.6765312</v>
+        <v>124662.2683724</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>25671.67653120001</v>
+        <v>24662.26837240001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.2567167653120001</v>
+        <v>0.2466226837240001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -15204,6 +15291,9 @@
       </c>
       <c r="EN14" s="3" t="n">
         <v>34.8352</v>
+      </c>
+      <c r="EO14" s="3" t="n">
+        <v>34.5554</v>
       </c>
     </row>
     <row r="15">
@@ -15229,16 +15319,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>10.83</v>
+        <v>10.92</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>105526.94601</v>
+        <v>106403.90124</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>5526.94601</v>
+        <v>6403.901240000007</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.05526946009999999</v>
+        <v>0.06403901240000007</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -15644,6 +15734,9 @@
       </c>
       <c r="EN15" s="3" t="n">
         <v>10.83</v>
+      </c>
+      <c r="EO15" s="3" t="n">
+        <v>10.92</v>
       </c>
     </row>
     <row r="16">
@@ -15669,16 +15762,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.6745</v>
+        <v>24.3705</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>141210.386936</v>
+        <v>139470.616824</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>41210.386936</v>
+        <v>39470.616824</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4121038693599999</v>
+        <v>0.39470616824</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -16078,6 +16171,9 @@
       </c>
       <c r="EN16" s="3" t="n">
         <v>24.6745</v>
+      </c>
+      <c r="EO16" s="3" t="n">
+        <v>24.3705</v>
       </c>
     </row>
     <row r="17">
@@ -16103,16 +16199,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.5511</v>
+        <v>16.6511</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54718.8800127</v>
+        <v>55049.48571269999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4718.880012699999</v>
+        <v>5049.485712699992</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.09437760025399999</v>
+        <v>0.1009897142539998</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -16512,6 +16608,9 @@
       </c>
       <c r="EN17" s="3" t="n">
         <v>16.5511</v>
+      </c>
+      <c r="EO17" s="3" t="n">
+        <v>16.6511</v>
       </c>
     </row>
     <row r="18">
@@ -16537,16 +16636,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.75</v>
+        <v>45.84</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>86304.447</v>
+        <v>86474.22624</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>6304.447</v>
+        <v>6474.226240000004</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.0788055875</v>
+        <v>0.08092782800000005</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -16952,6 +17051,9 @@
       </c>
       <c r="EN18" s="3" t="n">
         <v>45.75</v>
+      </c>
+      <c r="EO18" s="3" t="n">
+        <v>45.84</v>
       </c>
     </row>
     <row r="19">
@@ -16977,16 +17079,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.8215</v>
+        <v>11.8047</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>171018.874269</v>
+        <v>170775.8326002</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>21018.87426899999</v>
+        <v>20775.8326002</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.14012582846</v>
+        <v>0.138505550668</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -17386,6 +17488,9 @@
       </c>
       <c r="EN19" s="3" t="n">
         <v>11.8215</v>
+      </c>
+      <c r="EO19" s="3" t="n">
+        <v>11.8047</v>
       </c>
     </row>
     <row r="20">
@@ -17411,16 +17516,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.17</v>
+        <v>10.23</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>267021.51651</v>
+        <v>268596.86469</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>17021.51650999999</v>
+        <v>18596.86469000002</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.06808606603999995</v>
+        <v>0.07438745876000007</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -17826,6 +17931,9 @@
       </c>
       <c r="EN20" s="3" t="n">
         <v>10.17</v>
+      </c>
+      <c r="EO20" s="3" t="n">
+        <v>10.23</v>
       </c>
     </row>
     <row r="21">
@@ -17851,16 +17959,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>108.5534</v>
+        <v>109.2624</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>164920.7299306</v>
+        <v>165997.8845616</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-5079.270069399994</v>
+        <v>-4002.115438400011</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.02987805923176467</v>
+        <v>-0.02354185552000006</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -18266,6 +18374,9 @@
       </c>
       <c r="EN21" s="3" t="n">
         <v>108.5534</v>
+      </c>
+      <c r="EO21" s="3" t="n">
+        <v>109.2624</v>
       </c>
     </row>
     <row r="22">
@@ -18291,16 +18402,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>40.366</v>
+        <v>40.038</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>61940.01236</v>
+        <v>61436.70948</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>1940.012360000001</v>
+        <v>1436.709479999998</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.03233353933333334</v>
+        <v>0.02394515799999996</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -18700,6 +18811,9 @@
       </c>
       <c r="EN22" s="3" t="n">
         <v>40.366</v>
+      </c>
+      <c r="EO22" s="3" t="n">
+        <v>40.038</v>
       </c>
     </row>
     <row r="23">
@@ -18725,16 +18839,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>59.1519</v>
+        <v>59.5056</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>160684.1843373</v>
+        <v>161644.9987152</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>10684.18433729999</v>
+        <v>11644.9987152</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.07122789558199991</v>
+        <v>0.07763332476799997</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -19140,6 +19254,9 @@
       </c>
       <c r="EN23" s="3" t="n">
         <v>59.1519</v>
+      </c>
+      <c r="EO23" s="3" t="n">
+        <v>59.5056</v>
       </c>
     </row>
     <row r="24">
@@ -19165,16 +19282,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.3562</v>
+        <v>25.6058</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>92128.8620932</v>
+        <v>93035.75523879999</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-7871.137906799995</v>
+        <v>-6964.244761200011</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.07871137906799995</v>
+        <v>-0.0696424476120001</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -19574,6 +19691,9 @@
       </c>
       <c r="EN24" s="3" t="n">
         <v>25.3562</v>
+      </c>
+      <c r="EO24" s="3" t="n">
+        <v>25.6058</v>
       </c>
     </row>
     <row r="25">
@@ -19599,16 +19719,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.1503</v>
+        <v>12.2221</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>199528.2656022</v>
-      </c>
-      <c r="H25" s="6" t="n">
-        <v>-471.7343978000281</v>
-      </c>
-      <c r="I25" s="13" t="n">
-        <v>-0.002358671989000141</v>
+        <v>200707.3417954</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>707.3417953999888</v>
+      </c>
+      <c r="I25" s="12" t="n">
+        <v>0.003536708976999944</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -20008,6 +20128,9 @@
       </c>
       <c r="EN25" s="3" t="n">
         <v>12.1503</v>
+      </c>
+      <c r="EO25" s="3" t="n">
+        <v>12.2221</v>
       </c>
     </row>
     <row r="26">
@@ -20033,16 +20156,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.6767</v>
+        <v>10.6887</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>127498.1085405</v>
+        <v>127641.4091205</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>17498.1085405</v>
+        <v>17641.40912050001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1590737140045455</v>
+        <v>0.1603764465500001</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -20445,6 +20568,9 @@
       </c>
       <c r="EN26" s="3" t="n">
         <v>10.6767</v>
+      </c>
+      <c r="EO26" s="3" t="n">
+        <v>10.6887</v>
       </c>
     </row>
     <row r="27">
@@ -20470,16 +20596,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>67.2714</v>
+        <v>68.1534</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>108364.807404</v>
+        <v>109785.585924</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-1635.192596000008</v>
+        <v>-214.4140760000009</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.01486538723636371</v>
+        <v>-0.001949218872727281</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -20882,6 +21008,9 @@
       </c>
       <c r="EN27" s="3" t="n">
         <v>67.2714</v>
+      </c>
+      <c r="EO27" s="3" t="n">
+        <v>68.1534</v>
       </c>
     </row>
     <row r="28">
@@ -20907,16 +21036,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>111.1353</v>
+        <v>112.2349</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>367486.3176921</v>
+        <v>371122.3177293</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-12513.68230789999</v>
+        <v>-8877.682270699996</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.03293074291552629</v>
+        <v>-0.02336232176499999</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -21322,6 +21451,9 @@
       </c>
       <c r="EN28" s="3" t="n">
         <v>111.1353</v>
+      </c>
+      <c r="EO28" s="3" t="n">
+        <v>112.2349</v>
       </c>
     </row>
     <row r="29">
@@ -21347,16 +21479,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.4984</v>
+        <v>11.6296</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>110427.2185752</v>
+        <v>111687.2244088</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>10427.21857519999</v>
+        <v>11687.2244088</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1042721857519999</v>
+        <v>0.116872244088</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -21756,6 +21888,9 @@
       </c>
       <c r="EN29" s="3" t="n">
         <v>11.4984</v>
+      </c>
+      <c r="EO29" s="3" t="n">
+        <v>11.6296</v>
       </c>
     </row>
     <row r="30">
@@ -21781,16 +21916,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.5695</v>
+        <v>16.735</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>122545.7188395</v>
+        <v>123769.733835</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>22545.71883950001</v>
+        <v>23769.73383499999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2254571883950001</v>
+        <v>0.2376973383499999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -22190,6 +22325,9 @@
       </c>
       <c r="EN30" s="3" t="n">
         <v>16.5695</v>
+      </c>
+      <c r="EO30" s="3" t="n">
+        <v>16.735</v>
       </c>
     </row>
     <row r="31">
@@ -22215,16 +22353,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>382.3478</v>
+        <v>386.4542</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>101735.102624</v>
+        <v>102827.733536</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>1735.102623999992</v>
+        <v>2827.733536</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.01735102623999992</v>
+        <v>0.02827733536</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -22627,6 +22765,9 @@
       </c>
       <c r="EN31" s="3" t="n">
         <v>382.3478</v>
+      </c>
+      <c r="EO31" s="3" t="n">
+        <v>386.4542</v>
       </c>
     </row>
     <row r="32">
@@ -22652,16 +22793,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.45</v>
+        <v>10.51</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>220912.582</v>
+        <v>222180.9796</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>20912.58199999997</v>
+        <v>22180.97959999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1045629099999998</v>
+        <v>0.110904898</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -23067,6 +23208,9 @@
       </c>
       <c r="EN32" s="3" t="n">
         <v>10.45</v>
+      </c>
+      <c r="EO32" s="3" t="n">
+        <v>10.51</v>
       </c>
     </row>
     <row r="33">
@@ -23092,16 +23236,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.9</v>
+        <v>19.05</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67730.79599999999</v>
+        <v>68268.342</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7730.795999999988</v>
+        <v>8268.342000000004</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1288465999999998</v>
+        <v>0.1378057000000001</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -23501,6 +23645,9 @@
       </c>
       <c r="EN33" s="3" t="n">
         <v>18.9</v>
+      </c>
+      <c r="EO33" s="3" t="n">
+        <v>19.05</v>
       </c>
     </row>
     <row r="34">
@@ -23526,16 +23673,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>235.2384</v>
+        <v>234.9943</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>82693.58999040001</v>
+        <v>82607.7812733</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>2693.589990400011</v>
+        <v>2607.781273300003</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.03366987488000013</v>
+        <v>0.03259726591625003</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -23938,6 +24085,9 @@
       </c>
       <c r="EN34" s="3" t="n">
         <v>235.2384</v>
+      </c>
+      <c r="EO34" s="3" t="n">
+        <v>234.9943</v>
       </c>
     </row>
     <row r="35">
@@ -23963,16 +24113,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.64</v>
+        <v>15.73</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>111598.01572</v>
+        <v>112240.20379</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>11598.01572</v>
+        <v>12240.20379</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1159801572</v>
+        <v>0.1224020379</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -24375,6 +24525,9 @@
       </c>
       <c r="EN35" s="3" t="n">
         <v>15.64</v>
+      </c>
+      <c r="EO35" s="3" t="n">
+        <v>15.73</v>
       </c>
     </row>
     <row r="36">
@@ -24400,16 +24553,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>373.3714</v>
+        <v>375.5926</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>173881.3012084</v>
+        <v>174915.7273756</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>23881.30120839999</v>
+        <v>24915.72737560002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1592086747226666</v>
+        <v>0.1661048491706668</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -24812,6 +24965,9 @@
       </c>
       <c r="EN36" s="3" t="n">
         <v>373.3714</v>
+      </c>
+      <c r="EO36" s="3" t="n">
+        <v>375.5926</v>
       </c>
     </row>
     <row r="37">
@@ -24837,16 +24993,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>17.185</v>
+        <v>17.292</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>64665.247465</v>
+        <v>65067.87658800001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>14665.247465</v>
+        <v>15067.87658800001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2933049493</v>
+        <v>0.3013575317600001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -25249,6 +25405,9 @@
       </c>
       <c r="EN37" s="3" t="n">
         <v>17.185</v>
+      </c>
+      <c r="EO37" s="3" t="n">
+        <v>17.292</v>
       </c>
     </row>
     <row r="38">
@@ -25274,16 +25433,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.3982</v>
+        <v>13.5288</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>80127.6939324</v>
+        <v>80908.7448816</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>127.6939323999977</v>
+        <v>908.744881599996</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.001596174154999972</v>
+        <v>0.01135931101999995</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -25683,6 +25842,9 @@
       </c>
       <c r="EN38" s="3" t="n">
         <v>13.3982</v>
+      </c>
+      <c r="EO38" s="3" t="n">
+        <v>13.5288</v>
       </c>
     </row>
     <row r="39">
@@ -25708,16 +25870,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.078</v>
+        <v>1025.5678</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51131.915718</v>
+        <v>51156.3474318</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1131.915717999997</v>
+        <v>1156.347431800001</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02263831435999993</v>
+        <v>0.02312694863600001</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -26117,6 +26279,9 @@
       </c>
       <c r="EN39" s="3" t="n">
         <v>1025.078</v>
+      </c>
+      <c r="EO39" s="3" t="n">
+        <v>1025.5678</v>
       </c>
     </row>
     <row r="40">
@@ -26142,16 +26307,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.4632</v>
+        <v>19.6465</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>98114.5167064</v>
+        <v>99038.53695549999</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>-1885.483293600002</v>
+        <v>-961.4630445000075</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>-0.01885483293600002</v>
+        <v>-0.009614630445000076</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -26554,6 +26719,9 @@
       </c>
       <c r="EN40" s="3" t="n">
         <v>19.4632</v>
+      </c>
+      <c r="EO40" s="3" t="n">
+        <v>19.6465</v>
       </c>
     </row>
     <row r="41">
@@ -26566,13 +26734,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4864403.6752617</v>
+        <v>4882996.2213227</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>394403.6752616999</v>
+        <v>412996.2213227</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.08823348439859058</v>
+        <v>0.09239289067621924</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-10-31
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-30 08:01 IST</t>
+          <t>Generated: 2026-10-31 07:58 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4882996.2213227</v>
+        <v>4827872.1436361</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>412996.2213227004</v>
+        <v>357872.1436361</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09239289067621932</v>
+        <v>0.08006088224521253</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>506758.4968643188</v>
+        <v>506694.0012245178</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-84023.52313568117</v>
+        <v>-84088.0187754822</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.1422242388752474</v>
+        <v>-0.1423334088188435</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5389754.718187019</v>
+        <v>5334566.144860618</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>328972.6981870197</v>
+        <v>273784.1248606183</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06500432085138884</v>
+        <v>0.05409917356223501</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-10-30</t>
+          <t>Last snapshot: 2026-10-31</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FS19"/>
+  <dimension ref="A1:FT19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -794,6 +794,7 @@
     <col width="21" customWidth="1" min="173" max="173"/>
     <col width="21" customWidth="1" min="174" max="174"/>
     <col width="21" customWidth="1" min="175" max="175"/>
+    <col width="21" customWidth="1" min="176" max="176"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1672,6 +1673,11 @@
           <t>2026-10-30</t>
         </is>
       </c>
+      <c r="FT1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1691,13 +1697,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>538</v>
+        <v>535.5</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43040</v>
+        <v>42840</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-777.510000000002</v>
+        <v>-977.510000000002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -2199,6 +2205,9 @@
       </c>
       <c r="FS2" s="3" t="n">
         <v>538</v>
+      </c>
+      <c r="FT2" s="3" t="n">
+        <v>535.5</v>
       </c>
     </row>
     <row r="3">
@@ -2246,13 +2255,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1335</v>
+        <v>1341.900024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>26700</v>
+        <v>26838.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5404.580000000002</v>
+        <v>-5266.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -2757,6 +2766,9 @@
       </c>
       <c r="FS4" s="3" t="n">
         <v>1335</v>
+      </c>
+      <c r="FT4" s="3" t="n">
+        <v>1341.900024414062</v>
       </c>
     </row>
     <row r="5">
@@ -2777,13 +2789,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>454.3500061035156</v>
+        <v>451.3500061035156</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9087.000122070312</v>
+        <v>9027.000122070312</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-5126.099877929688</v>
+        <v>-5186.099877929688</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -3288,6 +3300,9 @@
       </c>
       <c r="FS5" s="3" t="n">
         <v>454.3500061035156</v>
+      </c>
+      <c r="FT5" s="3" t="n">
+        <v>451.3500061035156</v>
       </c>
     </row>
     <row r="6">
@@ -3308,13 +3323,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>329.3999938964844</v>
+        <v>327.7000122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>13175.99975585938</v>
+        <v>13108.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-4326.240244140627</v>
+        <v>-4394.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -3819,6 +3834,9 @@
       </c>
       <c r="FS6" s="3" t="n">
         <v>329.3999938964844</v>
+      </c>
+      <c r="FT6" s="3" t="n">
+        <v>327.7000122070312</v>
       </c>
     </row>
     <row r="7">
@@ -3839,13 +3857,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>253.4499969482422</v>
+        <v>251.8500061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25344.99969482422</v>
+        <v>25185.00061035156</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1088.820305175781</v>
+        <v>-1248.819389648437</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -4350,6 +4368,9 @@
       </c>
       <c r="FS7" s="3" t="n">
         <v>253.4499969482422</v>
+      </c>
+      <c r="FT7" s="3" t="n">
+        <v>251.8500061035156</v>
       </c>
     </row>
     <row r="8">
@@ -4397,13 +4418,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>12.73999977111816</v>
+        <v>12.72000026702881</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>19109.99965667725</v>
+        <v>19080.00040054321</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-11940.17034332275</v>
+        <v>-11970.16959945679</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -4908,6 +4929,9 @@
       </c>
       <c r="FS9" s="3" t="n">
         <v>12.73999977111816</v>
+      </c>
+      <c r="FT9" s="3" t="n">
+        <v>12.72000026702881</v>
       </c>
     </row>
     <row r="10">
@@ -4928,13 +4952,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>449.8999938964844</v>
+        <v>454</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44989.99938964844</v>
+        <v>45400</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-6508.480610351566</v>
+        <v>-6098.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -5439,6 +5463,9 @@
       </c>
       <c r="FS10" s="3" t="n">
         <v>449.8999938964844</v>
+      </c>
+      <c r="FT10" s="3" t="n">
+        <v>454</v>
       </c>
     </row>
     <row r="11">
@@ -5459,13 +5486,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>15.64999961853027</v>
+        <v>15.47999954223633</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>15649.99961853027</v>
+        <v>15479.99954223633</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>5808.789618530274</v>
+        <v>5638.789542236329</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -5970,6 +5997,9 @@
       </c>
       <c r="FS11" s="3" t="n">
         <v>15.64999961853027</v>
+      </c>
+      <c r="FT11" s="3" t="n">
+        <v>15.47999954223633</v>
       </c>
     </row>
     <row r="12">
@@ -5990,13 +6020,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2321.300048828125</v>
+        <v>2319.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>23213.00048828125</v>
+        <v>23193.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-4510.24951171875</v>
+        <v>-4530.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -6501,6 +6531,9 @@
       </c>
       <c r="FS12" s="3" t="n">
         <v>2321.300048828125</v>
+      </c>
+      <c r="FT12" s="3" t="n">
+        <v>2319.300048828125</v>
       </c>
     </row>
     <row r="13">
@@ -6521,13 +6554,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>33.61999893188477</v>
+        <v>33.90000152587891</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20171.99935913086</v>
+        <v>20340.00091552734</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-14859.76064086914</v>
+        <v>-14691.75908447266</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -7032,6 +7065,9 @@
       </c>
       <c r="FS13" s="3" t="n">
         <v>33.61999893188477</v>
+      </c>
+      <c r="FT13" s="3" t="n">
+        <v>33.90000152587891</v>
       </c>
     </row>
     <row r="14">
@@ -7052,13 +7088,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>594.75</v>
+        <v>595.5999755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>29737.5</v>
+        <v>29779.99877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-12725.01</v>
+        <v>-12682.51122070313</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -7563,6 +7599,9 @@
       </c>
       <c r="FS14" s="3" t="n">
         <v>594.75</v>
+      </c>
+      <c r="FT14" s="3" t="n">
+        <v>595.5999755859375</v>
       </c>
     </row>
     <row r="15">
@@ -7637,13 +7676,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>403.25</v>
+        <v>402.9500122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>20162.5</v>
+        <v>20147.50061035156</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-1592.029999999999</v>
+        <v>-1607.029389648436</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -8148,6 +8187,9 @@
       </c>
       <c r="FS17" s="3" t="n">
         <v>403.25</v>
+      </c>
+      <c r="FT17" s="3" t="n">
+        <v>402.9500122070312</v>
       </c>
     </row>
     <row r="18">
@@ -8168,13 +8210,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>346.0499877929688</v>
+        <v>345.0499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34604.99877929688</v>
+        <v>34504.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-12035.82122070312</v>
+        <v>-12135.82122070312</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -8679,6 +8721,9 @@
       </c>
       <c r="FS18" s="3" t="n">
         <v>346.0499877929688</v>
+      </c>
+      <c r="FT18" s="3" t="n">
+        <v>345.0499877929688</v>
       </c>
     </row>
     <row r="19">
@@ -8691,10 +8736,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>506758.4968643188</v>
+        <v>506694.0012245178</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-84023.52313568116</v>
+        <v>-84088.01877548218</v>
       </c>
     </row>
   </sheetData>
@@ -8708,7 +8753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EO41"/>
+  <dimension ref="A1:EP41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8719,7 +8764,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -8856,6 +8901,7 @@
     <col width="13" customWidth="1" min="143" max="143"/>
     <col width="13" customWidth="1" min="144" max="144"/>
     <col width="13" customWidth="1" min="145" max="145"/>
+    <col width="13" customWidth="1" min="146" max="146"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9584,6 +9630,11 @@
           <t>2026-10-30</t>
         </is>
       </c>
+      <c r="EP1" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9608,16 +9659,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.749</v>
+        <v>55.5747</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63699.731018</v>
+        <v>62381.6004054</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13699.731018</v>
+        <v>12381.6004054</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.27399462036</v>
+        <v>0.247632008108</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -10026,6 +10077,9 @@
       </c>
       <c r="EO2" s="3" t="n">
         <v>56.749</v>
+      </c>
+      <c r="EP2" s="3" t="n">
+        <v>55.5747</v>
       </c>
     </row>
     <row r="3">
@@ -10051,16 +10105,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.2575</v>
+        <v>26.1019</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>64467.7553475</v>
+        <v>64085.7242047</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4467.755347500002</v>
+        <v>4085.724204700004</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.07446258912500003</v>
+        <v>0.06809540341166673</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -10463,6 +10517,9 @@
       </c>
       <c r="EO3" s="3" t="n">
         <v>26.2575</v>
+      </c>
+      <c r="EP3" s="3" t="n">
+        <v>26.1019</v>
       </c>
     </row>
     <row r="4">
@@ -10488,16 +10545,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>11.52</v>
+        <v>11.31</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>221254.19136</v>
+        <v>217220.91183</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>41254.19136</v>
+        <v>37220.91183000003</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.229189952</v>
+        <v>0.2067828435000001</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -10900,6 +10957,9 @@
       </c>
       <c r="EO4" s="3" t="n">
         <v>11.52</v>
+      </c>
+      <c r="EP4" s="3" t="n">
+        <v>11.31</v>
       </c>
     </row>
     <row r="5">
@@ -10925,16 +10985,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.008599999999999</v>
+        <v>9.011799999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>165344.6371568</v>
+        <v>165403.3702384</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-44655.36284320001</v>
+        <v>-44596.62976160002</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.2126445849676191</v>
+        <v>-0.2123649036266668</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -11337,6 +11397,9 @@
       </c>
       <c r="EO5" s="3" t="n">
         <v>9.008599999999999</v>
+      </c>
+      <c r="EP5" s="3" t="n">
+        <v>9.011799999999999</v>
       </c>
     </row>
     <row r="6">
@@ -11362,16 +11425,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.9809</v>
+        <v>10.9248</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>46437.9735393</v>
+        <v>46200.7279296</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>-3562.026460699999</v>
+        <v>-3799.272070400002</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>-0.07124052921399998</v>
+        <v>-0.07598544140800004</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -11780,6 +11843,9 @@
       </c>
       <c r="EO6" s="3" t="n">
         <v>10.9809</v>
+      </c>
+      <c r="EP6" s="3" t="n">
+        <v>10.9248</v>
       </c>
     </row>
     <row r="7">
@@ -11805,16 +11871,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.4758</v>
+        <v>33.536</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73848.953832</v>
+        <v>73981.75744</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13848.953832</v>
+        <v>13981.75744</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2308158972</v>
+        <v>0.2330292906666667</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -12217,6 +12283,9 @@
       </c>
       <c r="EO7" s="3" t="n">
         <v>33.4758</v>
+      </c>
+      <c r="EP7" s="3" t="n">
+        <v>33.536</v>
       </c>
     </row>
     <row r="8">
@@ -12242,16 +12311,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>34.637</v>
+        <v>34.1356</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>55578.287741</v>
+        <v>54773.7448108</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5578.287741</v>
+        <v>4773.744810799995</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.11156575482</v>
+        <v>0.0954748962159999</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -12660,6 +12729,9 @@
       </c>
       <c r="EO8" s="3" t="n">
         <v>34.637</v>
+      </c>
+      <c r="EP8" s="3" t="n">
+        <v>34.1356</v>
       </c>
     </row>
     <row r="9">
@@ -12685,16 +12757,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>39.5494</v>
+        <v>37.7995</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>127325.0615142</v>
+        <v>121691.4457035</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>27325.0615142</v>
+        <v>21691.44570350001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.273250615142</v>
+        <v>0.2169144570350001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -13097,6 +13169,9 @@
       </c>
       <c r="EO9" s="3" t="n">
         <v>39.5494</v>
+      </c>
+      <c r="EP9" s="3" t="n">
+        <v>37.7995</v>
       </c>
     </row>
     <row r="10">
@@ -13122,16 +13197,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49.9171</v>
+        <v>49.7922</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>142096.9619689</v>
+        <v>141741.4142598</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>42096.9619689</v>
+        <v>41741.41425980002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.4209696196889999</v>
+        <v>0.4174141425980002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -13534,6 +13609,9 @@
       </c>
       <c r="EO10" s="3" t="n">
         <v>49.9171</v>
+      </c>
+      <c r="EP10" s="3" t="n">
+        <v>49.7922</v>
       </c>
     </row>
     <row r="11">
@@ -13559,16 +13637,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>102.4307</v>
+        <v>99.0941</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30823.3438133</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>823.3438132999981</v>
-      </c>
-      <c r="I11" s="12" t="n">
-        <v>0.0274447937766666</v>
+        <v>29819.2974779</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>-180.702522100004</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>-0.006023417403333466</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -13971,6 +14049,9 @@
       </c>
       <c r="EO11" s="3" t="n">
         <v>102.4307</v>
+      </c>
+      <c r="EP11" s="3" t="n">
+        <v>99.0941</v>
       </c>
     </row>
     <row r="12">
@@ -13996,16 +14077,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>217.641</v>
+        <v>215.986</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>101316.673602</v>
+        <v>100546.234692</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1316.673601999995</v>
+        <v>546.2346919999982</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.01316673601999995</v>
+        <v>0.005462346919999981</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -14414,6 +14495,9 @@
       </c>
       <c r="EO12" s="3" t="n">
         <v>217.641</v>
+      </c>
+      <c r="EP12" s="3" t="n">
+        <v>215.986</v>
       </c>
     </row>
     <row r="13">
@@ -14439,16 +14523,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.862</v>
+        <v>21.952</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>253328.22051</v>
+        <v>254371.10496</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>53328.22050999998</v>
+        <v>54371.10496</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2666411025499999</v>
+        <v>0.2718555248</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -14857,6 +14941,9 @@
       </c>
       <c r="EO13" s="3" t="n">
         <v>21.862</v>
+      </c>
+      <c r="EP13" s="3" t="n">
+        <v>21.952</v>
       </c>
     </row>
     <row r="14">
@@ -14882,16 +14969,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34.5554</v>
+        <v>33.9474</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>124662.2683724</v>
+        <v>122468.8439244</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>24662.26837240001</v>
+        <v>22468.84392440002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.2466226837240001</v>
+        <v>0.2246884392440002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -15294,6 +15381,9 @@
       </c>
       <c r="EO14" s="3" t="n">
         <v>34.5554</v>
+      </c>
+      <c r="EP14" s="3" t="n">
+        <v>33.9474</v>
       </c>
     </row>
     <row r="15">
@@ -15319,16 +15409,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>10.92</v>
+        <v>10.81</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>106403.90124</v>
+        <v>105332.06707</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>6403.901240000007</v>
+        <v>5332.067070000005</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.06403901240000007</v>
+        <v>0.05332067070000004</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -15737,6 +15827,9 @@
       </c>
       <c r="EO15" s="3" t="n">
         <v>10.92</v>
+      </c>
+      <c r="EP15" s="3" t="n">
+        <v>10.81</v>
       </c>
     </row>
     <row r="16">
@@ -15762,16 +15855,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.3705</v>
+        <v>23.4994</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>139470.616824</v>
+        <v>134485.3742432</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>39470.616824</v>
+        <v>34485.3742432</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.39470616824</v>
+        <v>0.344853742432</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -16174,6 +16267,9 @@
       </c>
       <c r="EO16" s="3" t="n">
         <v>24.3705</v>
+      </c>
+      <c r="EP16" s="3" t="n">
+        <v>23.4994</v>
       </c>
     </row>
     <row r="17">
@@ -16199,16 +16295,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6511</v>
+        <v>16.5777</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55049.48571269999</v>
+        <v>54806.8211289</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5049.485712699992</v>
+        <v>4806.821128899996</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1009897142539998</v>
+        <v>0.09613642257799991</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -16611,6 +16707,9 @@
       </c>
       <c r="EO17" s="3" t="n">
         <v>16.6511</v>
+      </c>
+      <c r="EP17" s="3" t="n">
+        <v>16.5777</v>
       </c>
     </row>
     <row r="18">
@@ -17079,16 +17178,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>11.8047</v>
+        <v>11.2577</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>170775.8326002</v>
+        <v>162862.5115982</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>20775.8326002</v>
+        <v>12862.51159819998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.138505550668</v>
+        <v>0.08575007732133323</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -17491,6 +17590,9 @@
       </c>
       <c r="EO19" s="3" t="n">
         <v>11.8047</v>
+      </c>
+      <c r="EP19" s="3" t="n">
+        <v>11.2577</v>
       </c>
     </row>
     <row r="20">
@@ -17516,16 +17618,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>10.23</v>
+        <v>10.22</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>268596.86469</v>
+        <v>268334.30666</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>18596.86469000002</v>
+        <v>18334.30666</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0.07438745876000007</v>
+        <v>0.07333722664</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -17934,6 +18036,9 @@
       </c>
       <c r="EO20" s="3" t="n">
         <v>10.23</v>
+      </c>
+      <c r="EP20" s="3" t="n">
+        <v>10.22</v>
       </c>
     </row>
     <row r="21">
@@ -17959,16 +18064,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>109.2624</v>
+        <v>108.0429</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>165997.8845616</v>
+        <v>164145.1482111</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-4002.115438400011</v>
+        <v>-5854.851788900007</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.02354185552000006</v>
+        <v>-0.03444030464058827</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -18377,6 +18482,9 @@
       </c>
       <c r="EO21" s="3" t="n">
         <v>109.2624</v>
+      </c>
+      <c r="EP21" s="3" t="n">
+        <v>108.0429</v>
       </c>
     </row>
     <row r="22">
@@ -18402,16 +18510,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>40.038</v>
+        <v>39.14</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>61436.70948</v>
+        <v>60058.7644</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>1436.709479999998</v>
+        <v>58.76440000000002</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.02394515799999996</v>
+        <v>0.0009794066666666671</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -18814,6 +18922,9 @@
       </c>
       <c r="EO22" s="3" t="n">
         <v>40.038</v>
+      </c>
+      <c r="EP22" s="3" t="n">
+        <v>39.14</v>
       </c>
     </row>
     <row r="23">
@@ -18839,16 +18950,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>59.5056</v>
+        <v>58.9684</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>161644.9987152</v>
+        <v>160185.7126428</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>11644.9987152</v>
+        <v>10185.7126428</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.07763332476799997</v>
+        <v>0.06790475095200003</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -19257,6 +19368,9 @@
       </c>
       <c r="EO23" s="3" t="n">
         <v>59.5056</v>
+      </c>
+      <c r="EP23" s="3" t="n">
+        <v>58.9684</v>
       </c>
     </row>
     <row r="24">
@@ -19282,16 +19396,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>25.6058</v>
+        <v>25.3775</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>93035.75523879999</v>
+        <v>92206.253215</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-6964.244761200011</v>
+        <v>-7793.746784999996</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.0696424476120001</v>
+        <v>-0.07793746784999996</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -19694,6 +19808,9 @@
       </c>
       <c r="EO24" s="3" t="n">
         <v>25.6058</v>
+      </c>
+      <c r="EP24" s="3" t="n">
+        <v>25.3775</v>
       </c>
     </row>
     <row r="25">
@@ -19719,16 +19836,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.2221</v>
+        <v>12.0939</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>200707.3417954</v>
-      </c>
-      <c r="H25" s="4" t="n">
-        <v>707.3417953999888</v>
-      </c>
-      <c r="I25" s="12" t="n">
-        <v>0.003536708976999944</v>
+        <v>198602.0831886</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>-1397.916811400006</v>
+      </c>
+      <c r="I25" s="13" t="n">
+        <v>-0.006989584057000029</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -20131,6 +20248,9 @@
       </c>
       <c r="EO25" s="3" t="n">
         <v>12.2221</v>
+      </c>
+      <c r="EP25" s="3" t="n">
+        <v>12.0939</v>
       </c>
     </row>
     <row r="26">
@@ -20156,16 +20276,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>10.6887</v>
+        <v>10.501</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>127641.4091205</v>
+        <v>125399.949215</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>17641.40912050001</v>
+        <v>15399.949215</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.1603764465500001</v>
+        <v>0.1399995383181818</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -20571,6 +20691,9 @@
       </c>
       <c r="EO26" s="3" t="n">
         <v>10.6887</v>
+      </c>
+      <c r="EP26" s="3" t="n">
+        <v>10.501</v>
       </c>
     </row>
     <row r="27">
@@ -20596,16 +20719,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>68.1534</v>
+        <v>67.6101</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>109785.585924</v>
+        <v>108910.405686</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-214.4140760000009</v>
+        <v>-1089.594314000002</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.001949218872727281</v>
+        <v>-0.00990540285454547</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -21011,6 +21134,9 @@
       </c>
       <c r="EO27" s="3" t="n">
         <v>68.1534</v>
+      </c>
+      <c r="EP27" s="3" t="n">
+        <v>67.6101</v>
       </c>
     </row>
     <row r="28">
@@ -21036,16 +21162,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>112.2349</v>
+        <v>111.4372</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>371122.3177293</v>
+        <v>368484.5974404</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-8877.682270699996</v>
+        <v>-11515.40255959996</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.02336232176499999</v>
+        <v>-0.03030369094631567</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -21454,6 +21580,9 @@
       </c>
       <c r="EO28" s="3" t="n">
         <v>112.2349</v>
+      </c>
+      <c r="EP28" s="3" t="n">
+        <v>111.4372</v>
       </c>
     </row>
     <row r="29">
@@ -21479,16 +21608,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.6296</v>
+        <v>11.3957</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>111687.2244088</v>
+        <v>109440.9182771</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>11687.2244088</v>
+        <v>9440.918277099991</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.116872244088</v>
+        <v>0.09440918277099991</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -21891,6 +22020,9 @@
       </c>
       <c r="EO29" s="3" t="n">
         <v>11.6296</v>
+      </c>
+      <c r="EP29" s="3" t="n">
+        <v>11.3957</v>
       </c>
     </row>
     <row r="30">
@@ -21916,16 +22048,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.735</v>
+        <v>16.4684</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>123769.733835</v>
+        <v>121797.9972924</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>23769.73383499999</v>
+        <v>21797.99729239999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2376973383499999</v>
+        <v>0.2179799729239999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -22328,6 +22460,9 @@
       </c>
       <c r="EO30" s="3" t="n">
         <v>16.735</v>
+      </c>
+      <c r="EP30" s="3" t="n">
+        <v>16.4684</v>
       </c>
     </row>
     <row r="31">
@@ -22353,16 +22488,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>386.4542</v>
+        <v>381.7153</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>102827.733536</v>
+        <v>101566.807024</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>2827.733536</v>
+        <v>1566.807023999994</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.02827733536</v>
+        <v>0.01566807023999994</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -22768,6 +22903,9 @@
       </c>
       <c r="EO31" s="3" t="n">
         <v>386.4542</v>
+      </c>
+      <c r="EP31" s="3" t="n">
+        <v>381.7153</v>
       </c>
     </row>
     <row r="32">
@@ -22793,16 +22931,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.51</v>
+        <v>10.45</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>222180.9796</v>
+        <v>220912.582</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>22180.97959999999</v>
+        <v>20912.58199999997</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.110904898</v>
+        <v>0.1045629099999998</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -23211,6 +23349,9 @@
       </c>
       <c r="EO32" s="3" t="n">
         <v>10.51</v>
+      </c>
+      <c r="EP32" s="3" t="n">
+        <v>10.45</v>
       </c>
     </row>
     <row r="33">
@@ -23236,16 +23377,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.05</v>
+        <v>18.81</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>68268.342</v>
+        <v>67408.26839999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>8268.342000000004</v>
+        <v>7408.268399999986</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1378057000000001</v>
+        <v>0.1234711399999998</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -23648,6 +23789,9 @@
       </c>
       <c r="EO33" s="3" t="n">
         <v>19.05</v>
+      </c>
+      <c r="EP33" s="3" t="n">
+        <v>18.81</v>
       </c>
     </row>
     <row r="34">
@@ -23673,16 +23817,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>234.9943</v>
+        <v>236.4025</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>82607.7812733</v>
+        <v>83102.8072275</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>2607.781273300003</v>
+        <v>3102.807227500001</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0.03259726591625003</v>
+        <v>0.03878509034375002</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -24088,6 +24232,9 @@
       </c>
       <c r="EO34" s="3" t="n">
         <v>234.9943</v>
+      </c>
+      <c r="EP34" s="3" t="n">
+        <v>236.4025</v>
       </c>
     </row>
     <row r="35">
@@ -24113,16 +24260,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.73</v>
+        <v>15.5</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>112240.20379</v>
+        <v>110599.0565</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>12240.20379</v>
+        <v>10599.05649999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.1224020379</v>
+        <v>0.1059905649999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -24528,6 +24675,9 @@
       </c>
       <c r="EO35" s="3" t="n">
         <v>15.73</v>
+      </c>
+      <c r="EP35" s="3" t="n">
+        <v>15.5</v>
       </c>
     </row>
     <row r="36">
@@ -24553,16 +24703,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>375.5926</v>
+        <v>375.0929</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>174915.7273756</v>
+        <v>174683.0140874</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>24915.72737560002</v>
+        <v>24683.01408739999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1661048491706668</v>
+        <v>0.1645534272493333</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -24968,6 +25118,9 @@
       </c>
       <c r="EO36" s="3" t="n">
         <v>375.5926</v>
+      </c>
+      <c r="EP36" s="3" t="n">
+        <v>375.0929</v>
       </c>
     </row>
     <row r="37">
@@ -25433,16 +25586,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.5288</v>
+        <v>13.49</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>80908.7448816</v>
+        <v>80676.70218000001</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>908.744881599996</v>
+        <v>676.7021800000075</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.01135931101999995</v>
+        <v>0.008458777250000094</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -25845,6 +25998,9 @@
       </c>
       <c r="EO38" s="3" t="n">
         <v>13.5288</v>
+      </c>
+      <c r="EP38" s="3" t="n">
+        <v>13.49</v>
       </c>
     </row>
     <row r="39">
@@ -25870,16 +26026,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1025.5678</v>
+        <v>1025.1961</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51156.3474318</v>
+        <v>51137.8066641</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1156.347431800001</v>
+        <v>1137.806664099997</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02312694863600001</v>
+        <v>0.02275613328199994</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -26282,6 +26438,9 @@
       </c>
       <c r="EO39" s="3" t="n">
         <v>1025.5678</v>
+      </c>
+      <c r="EP39" s="3" t="n">
+        <v>1025.1961</v>
       </c>
     </row>
     <row r="40">
@@ -26307,16 +26466,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.6465</v>
+        <v>19.1437</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>99038.53695549999</v>
+        <v>96503.9085799</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>-961.4630445000075</v>
+        <v>-3496.091420099998</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>-0.009614630445000076</v>
+        <v>-0.03496091420099998</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -26722,6 +26881,9 @@
       </c>
       <c r="EO40" s="3" t="n">
         <v>19.6465</v>
+      </c>
+      <c r="EP40" s="3" t="n">
+        <v>19.1437</v>
       </c>
     </row>
     <row r="41">
@@ -26734,13 +26896,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4882996.2213227</v>
+        <v>4827872.1436361</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>412996.2213227</v>
+        <v>357872.1436361</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09239289067621924</v>
+        <v>0.08006088224521253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>